<commit_message>
v1.3.0 — baseline soccer + tennis models, architecture cleanup
Added:
- SOCCER + TENNIS baseline models (learned LR, research state)
- /api/bets, /api/open, /api/history dashboard endpoints
- Portfolio tab in dashboard HTML
- 'dash' launcher script + zsh alias
- Polymarket edge filter (2% minimum)
- Dashboard /api/odds endpoint

Cleaned:
- nfl.py no longer uses BasketballModel (dead code removed)
- nba.py, wnba.py docstrings clarify learned LR pipeline
- registry.py get_model() points to learned_forward for production sports
- Removed redundant input/INPUT.md

Baseline artifacts ready for soccer + tennis.
Bootstrap soccer data in progress (302 games and counting).
</commit_message>
<xml_diff>
--- a/data/picks.xlsx
+++ b/data/picks.xlsx
@@ -300,8 +300,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CA6" headerRowCount="1">
-  <autoFilter ref="A1:CA6"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CA10" headerRowCount="1">
+  <autoFilter ref="A1:CA10"/>
   <tableColumns count="79">
     <tableColumn id="1" name="pick_id"/>
     <tableColumn id="2" name="created_at_utc"/>
@@ -738,19 +738,19 @@
     </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="6">
-        <f>COUNTA('Picks'!$A$2:$A$6)</f>
+        <f>COUNTA('Picks'!$A$2:$A$10)</f>
         <v/>
       </c>
       <c r="C4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$6,"open")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$10,"open")</f>
         <v/>
       </c>
       <c r="E4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$6,"settled")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$10,"settled")</f>
         <v/>
       </c>
       <c r="G4" s="6">
-        <f>IF(COUNTIFS('Picks'!$U$2:$U$6,"settled",'Picks'!$V$2:$V$6,"win")+COUNTIFS('Picks'!$U$2:$U$6,"settled",'Picks'!$V$2:$V$6,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
+        <f>IF(COUNTIFS('Picks'!$U$2:$U$10,"settled",'Picks'!$V$2:$V$10,"win")+COUNTIFS('Picks'!$U$2:$U$10,"settled",'Picks'!$V$2:$V$10,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
         <v/>
       </c>
     </row>
@@ -778,19 +778,19 @@
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="6">
-        <f>COUNTIF('Picks'!$BX$2:$BX$6,"&gt;0")</f>
+        <f>COUNTIF('Picks'!$BX$2:$BX$10,"&gt;0")</f>
         <v/>
       </c>
       <c r="C7" s="6">
-        <f>COUNTIFS('Picks'!$BX$2:$BX$6,"&gt;0",'Picks'!$V$2:$V$6,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$6,"&gt;0",'Picks'!$V$2:$V$6,"loss")</f>
+        <f>COUNTIFS('Picks'!$BX$2:$BX$10,"&gt;0",'Picks'!$V$2:$V$10,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$10,"&gt;0",'Picks'!$V$2:$V$10,"loss")</f>
         <v/>
       </c>
       <c r="E7" s="7">
-        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$6,"&gt;0",'Picks'!$V$2:$V$6,"win")/(COUNTIFS('Picks'!$BX$2:$BX$6,"&gt;0",'Picks'!$V$2:$V$6,"win")+COUNTIFS('Picks'!$BX$2:$BX$6,"&gt;0",'Picks'!$V$2:$V$6,"loss")),0)</f>
+        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$10,"&gt;0",'Picks'!$V$2:$V$10,"win")/(COUNTIFS('Picks'!$BX$2:$BX$10,"&gt;0",'Picks'!$V$2:$V$10,"win")+COUNTIFS('Picks'!$BX$2:$BX$10,"&gt;0",'Picks'!$V$2:$V$10,"loss")),0)</f>
         <v/>
       </c>
       <c r="G7" s="7">
-        <f>IFERROR(SUM('Picks'!$BY$2:$BY$6)/SUM('Picks'!$BX$2:$BX$6),0)</f>
+        <f>IFERROR(SUM('Picks'!$BY$2:$BY$10)/SUM('Picks'!$BX$2:$BX$10),0)</f>
         <v/>
       </c>
     </row>
@@ -818,19 +818,19 @@
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="8">
-        <f>SUM('Picks'!$BY$2:$BY$6)</f>
+        <f>SUM('Picks'!$BY$2:$BY$10)</f>
         <v/>
       </c>
       <c r="C10" s="9">
-        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$6,"&lt;&gt;",'Picks'!$AB$2:$AB$6),0)</f>
+        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$10,"&lt;&gt;",'Picks'!$AB$2:$AB$10),0)</f>
         <v/>
       </c>
       <c r="E10" s="6">
-        <f>COUNTIFS('Picks'!$AM$2:$AM$6,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$6,"settled")</f>
+        <f>COUNTIFS('Picks'!$AM$2:$AM$10,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$10,"settled")</f>
         <v/>
       </c>
       <c r="G10" s="8">
-        <f>SUMIFS('Picks'!$AC$2:$AC$6,'Picks'!$AM$2:$AM$6,"QUALIFIED_SHADOW_CALL")</f>
+        <f>SUMIFS('Picks'!$AC$2:$AC$10,'Picks'!$AM$2:$AM$10,"QUALIFIED_SHADOW_CALL")</f>
         <v/>
       </c>
     </row>
@@ -885,15 +885,15 @@
         </is>
       </c>
       <c r="B14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$6,$A14,'Picks'!$U$2:$U$6,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$10,$A14,'Picks'!$U$2:$U$10,"settled")</f>
         <v/>
       </c>
       <c r="C14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$6,$A14,'Picks'!$U$2:$U$6,"settled",'Picks'!$V$2:$V$6,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$10,$A14,'Picks'!$U$2:$U$10,"settled",'Picks'!$V$2:$V$10,"win")</f>
         <v/>
       </c>
       <c r="D14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$6,$A14,'Picks'!$U$2:$U$6,"settled",'Picks'!$V$2:$V$6,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$10,$A14,'Picks'!$U$2:$U$10,"settled",'Picks'!$V$2:$V$10,"loss")</f>
         <v/>
       </c>
       <c r="E14" s="14">
@@ -901,11 +901,11 @@
         <v/>
       </c>
       <c r="F14" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$6,'Picks'!$H$2:$H$6,$A14)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$10,'Picks'!$H$2:$H$10,$A14)</f>
         <v/>
       </c>
       <c r="G14" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$6,'Picks'!$H$2:$H$6,$A14,'Picks'!$U$2:$U$6,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$10,'Picks'!$H$2:$H$10,$A14,'Picks'!$U$2:$U$10,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -916,15 +916,15 @@
         </is>
       </c>
       <c r="B15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$6,$A15,'Picks'!$U$2:$U$6,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$10,$A15,'Picks'!$U$2:$U$10,"settled")</f>
         <v/>
       </c>
       <c r="C15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$6,$A15,'Picks'!$U$2:$U$6,"settled",'Picks'!$V$2:$V$6,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$10,$A15,'Picks'!$U$2:$U$10,"settled",'Picks'!$V$2:$V$10,"win")</f>
         <v/>
       </c>
       <c r="D15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$6,$A15,'Picks'!$U$2:$U$6,"settled",'Picks'!$V$2:$V$6,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$10,$A15,'Picks'!$U$2:$U$10,"settled",'Picks'!$V$2:$V$10,"loss")</f>
         <v/>
       </c>
       <c r="E15" s="19">
@@ -932,11 +932,11 @@
         <v/>
       </c>
       <c r="F15" s="20">
-        <f>SUMIFS('Picks'!$BY$2:$BY$6,'Picks'!$H$2:$H$6,$A15)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$10,'Picks'!$H$2:$H$10,$A15)</f>
         <v/>
       </c>
       <c r="G15" s="21">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$6,'Picks'!$H$2:$H$6,$A15,'Picks'!$U$2:$U$6,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$10,'Picks'!$H$2:$H$10,$A15,'Picks'!$U$2:$U$10,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -947,15 +947,15 @@
         </is>
       </c>
       <c r="B16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$6,$A16,'Picks'!$U$2:$U$6,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$10,$A16,'Picks'!$U$2:$U$10,"settled")</f>
         <v/>
       </c>
       <c r="C16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$6,$A16,'Picks'!$U$2:$U$6,"settled",'Picks'!$V$2:$V$6,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$10,$A16,'Picks'!$U$2:$U$10,"settled",'Picks'!$V$2:$V$10,"win")</f>
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$6,$A16,'Picks'!$U$2:$U$6,"settled",'Picks'!$V$2:$V$6,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$10,$A16,'Picks'!$U$2:$U$10,"settled",'Picks'!$V$2:$V$10,"loss")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -963,11 +963,11 @@
         <v/>
       </c>
       <c r="F16" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$6,'Picks'!$H$2:$H$6,$A16)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$10,'Picks'!$H$2:$H$10,$A16)</f>
         <v/>
       </c>
       <c r="G16" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$6,'Picks'!$H$2:$H$6,$A16,'Picks'!$U$2:$U$6,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$10,'Picks'!$H$2:$H$10,$A16,'Picks'!$U$2:$U$10,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -996,7 +996,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:CA6"/>
+  <dimension ref="A1:CA10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2722,6 +2722,1002 @@
       <c r="BZ6" s="24" t="n"/>
       <c r="CA6" s="31" t="n"/>
     </row>
+    <row r="7" ht="36" customHeight="1">
+      <c r="A7" s="24" t="inlineStr">
+        <is>
+          <t>d0e98df55d684f7a</t>
+        </is>
+      </c>
+      <c r="B7" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-17T14:02:14.862720Z</t>
+        </is>
+      </c>
+      <c r="C7" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-17T23:40Z</t>
+        </is>
+      </c>
+      <c r="D7" s="24" t="inlineStr">
+        <is>
+          <t>401816148</t>
+        </is>
+      </c>
+      <c r="E7" s="24" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="F7" s="24" t="inlineStr">
+        <is>
+          <t>Miami Marlins</t>
+        </is>
+      </c>
+      <c r="G7" s="24" t="inlineStr">
+        <is>
+          <t>Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="H7" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I7" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J7" s="25" t="n"/>
+      <c r="K7" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L7" s="26" t="n">
+        <v>-141</v>
+      </c>
+      <c r="M7" s="27" t="n">
+        <v>1.70922</v>
+      </c>
+      <c r="N7" s="28" t="n">
+        <v>0.585062</v>
+      </c>
+      <c r="O7" s="28" t="n">
+        <v>0.605633</v>
+      </c>
+      <c r="P7" s="28" t="n"/>
+      <c r="Q7" s="28" t="n">
+        <v>0.020571</v>
+      </c>
+      <c r="R7" s="26" t="n">
+        <v>60</v>
+      </c>
+      <c r="S7" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="T7" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="U7" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V7" s="24" t="n"/>
+      <c r="W7" s="26" t="n"/>
+      <c r="X7" s="26" t="n"/>
+      <c r="Y7" s="25" t="n"/>
+      <c r="Z7" s="26" t="n"/>
+      <c r="AA7" s="28" t="n"/>
+      <c r="AB7" s="28" t="n"/>
+      <c r="AC7" s="30" t="n"/>
+      <c r="AD7" s="24" t="n"/>
+      <c r="AE7" s="31" t="inlineStr">
+        <is>
+          <t>Learned LR call at threshold 0.6018; executable ask 0.5850 (aec-mlb-mia-mil-2026-07-17).</t>
+        </is>
+      </c>
+      <c r="AF7" s="31" t="inlineStr">
+        <is>
+          <t>Learned model; promotion gate not yet open; zero-unit research until review.</t>
+        </is>
+      </c>
+      <c r="AG7" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH7" s="24" t="n"/>
+      <c r="AI7" s="31" t="n"/>
+      <c r="AJ7" s="31" t="n"/>
+      <c r="AK7" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL7" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM7" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN7" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO7" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_MISSING_UNCERTAINTY</t>
+        </is>
+      </c>
+      <c r="AP7" s="24" t="inlineStr">
+        <is>
+          <t>mlb-mia</t>
+        </is>
+      </c>
+      <c r="AQ7" s="24" t="inlineStr">
+        <is>
+          <t>Miami Marlins</t>
+        </is>
+      </c>
+      <c r="AR7" s="24" t="inlineStr">
+        <is>
+          <t>Miami Marlins</t>
+        </is>
+      </c>
+      <c r="AS7" s="24" t="inlineStr">
+        <is>
+          <t>mlb-mil</t>
+        </is>
+      </c>
+      <c r="AT7" s="24" t="inlineStr">
+        <is>
+          <t>Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="AU7" s="24" t="inlineStr">
+        <is>
+          <t>Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="AV7" s="24" t="n"/>
+      <c r="AW7" s="24" t="n"/>
+      <c r="AX7" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY7" s="24" t="n"/>
+      <c r="AZ7" s="24" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="BA7" s="24" t="inlineStr">
+        <is>
+          <t>a454281ab207d2924d585d6b967363fb8e88af45132e3e9d354e4351fb5c237f</t>
+        </is>
+      </c>
+      <c r="BB7" s="24" t="inlineStr">
+        <is>
+          <t>learned_lr</t>
+        </is>
+      </c>
+      <c r="BC7" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="BD7" s="24" t="inlineStr">
+        <is>
+          <t>a454281ab207d2924d585d6b967363fb8e88af45132e3e9d354e4351fb5c237f</t>
+        </is>
+      </c>
+      <c r="BE7" s="24" t="inlineStr">
+        <is>
+          <t>27ad4a1da893e4b8</t>
+        </is>
+      </c>
+      <c r="BF7" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG7" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="BH7" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-17T14:01:56.626918Z</t>
+        </is>
+      </c>
+      <c r="BI7" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ7" s="25" t="n"/>
+      <c r="BK7" s="26" t="n">
+        <v>-141</v>
+      </c>
+      <c r="BL7" s="27" t="n">
+        <v>1.70922</v>
+      </c>
+      <c r="BM7" s="28" t="n">
+        <v>0.585062</v>
+      </c>
+      <c r="BN7" s="28" t="n">
+        <v>0.58209</v>
+      </c>
+      <c r="BO7" s="28" t="n"/>
+      <c r="BP7" s="25" t="n"/>
+      <c r="BQ7" s="27" t="n"/>
+      <c r="BR7" s="28" t="n"/>
+      <c r="BS7" s="28" t="n"/>
+      <c r="BT7" s="28" t="n"/>
+      <c r="BU7" s="25" t="n"/>
+      <c r="BV7" s="29" t="n"/>
+      <c r="BW7" s="24" t="n"/>
+      <c r="BX7" s="30" t="n"/>
+      <c r="BY7" s="27" t="n"/>
+      <c r="BZ7" s="24" t="n"/>
+      <c r="CA7" s="31" t="n"/>
+    </row>
+    <row r="8" ht="36" customHeight="1">
+      <c r="A8" s="24" t="inlineStr">
+        <is>
+          <t>3b98081a1ff04c62</t>
+        </is>
+      </c>
+      <c r="B8" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-17T14:02:14.862720Z</t>
+        </is>
+      </c>
+      <c r="C8" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T00:05Z</t>
+        </is>
+      </c>
+      <c r="D8" s="24" t="inlineStr">
+        <is>
+          <t>401816149</t>
+        </is>
+      </c>
+      <c r="E8" s="24" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="F8" s="24" t="inlineStr">
+        <is>
+          <t>Minnesota Twins</t>
+        </is>
+      </c>
+      <c r="G8" s="24" t="inlineStr">
+        <is>
+          <t>Chicago Cubs</t>
+        </is>
+      </c>
+      <c r="H8" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I8" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J8" s="25" t="n"/>
+      <c r="K8" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L8" s="26" t="n">
+        <v>-130</v>
+      </c>
+      <c r="M8" s="27" t="n">
+        <v>1.769231</v>
+      </c>
+      <c r="N8" s="28" t="n">
+        <v>0.565217</v>
+      </c>
+      <c r="O8" s="28" t="n">
+        <v>0.606876</v>
+      </c>
+      <c r="P8" s="28" t="n"/>
+      <c r="Q8" s="28" t="n">
+        <v>0.041659</v>
+      </c>
+      <c r="R8" s="26" t="n">
+        <v>71</v>
+      </c>
+      <c r="S8" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="T8" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="U8" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V8" s="24" t="n"/>
+      <c r="W8" s="26" t="n"/>
+      <c r="X8" s="26" t="n"/>
+      <c r="Y8" s="25" t="n"/>
+      <c r="Z8" s="26" t="n"/>
+      <c r="AA8" s="28" t="n"/>
+      <c r="AB8" s="28" t="n"/>
+      <c r="AC8" s="30" t="n"/>
+      <c r="AD8" s="24" t="n"/>
+      <c r="AE8" s="31" t="inlineStr">
+        <is>
+          <t>Learned LR call at threshold 0.6018; executable ask 0.5650 (aec-mlb-min-chc-2026-07-17).</t>
+        </is>
+      </c>
+      <c r="AF8" s="31" t="inlineStr">
+        <is>
+          <t>Learned model; promotion gate not yet open; zero-unit research until review.</t>
+        </is>
+      </c>
+      <c r="AG8" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH8" s="24" t="n"/>
+      <c r="AI8" s="31" t="n"/>
+      <c r="AJ8" s="31" t="n"/>
+      <c r="AK8" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL8" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM8" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN8" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO8" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_MISSING_UNCERTAINTY</t>
+        </is>
+      </c>
+      <c r="AP8" s="24" t="inlineStr">
+        <is>
+          <t>mlb-min</t>
+        </is>
+      </c>
+      <c r="AQ8" s="24" t="inlineStr">
+        <is>
+          <t>Minnesota Twins</t>
+        </is>
+      </c>
+      <c r="AR8" s="24" t="inlineStr">
+        <is>
+          <t>Minnesota Twins</t>
+        </is>
+      </c>
+      <c r="AS8" s="24" t="inlineStr">
+        <is>
+          <t>mlb-chc</t>
+        </is>
+      </c>
+      <c r="AT8" s="24" t="inlineStr">
+        <is>
+          <t>Chicago Cubs</t>
+        </is>
+      </c>
+      <c r="AU8" s="24" t="inlineStr">
+        <is>
+          <t>Chicago Cubs</t>
+        </is>
+      </c>
+      <c r="AV8" s="24" t="n"/>
+      <c r="AW8" s="24" t="n"/>
+      <c r="AX8" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY8" s="24" t="n"/>
+      <c r="AZ8" s="24" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="BA8" s="24" t="inlineStr">
+        <is>
+          <t>a454281ab207d2924d585d6b967363fb8e88af45132e3e9d354e4351fb5c237f</t>
+        </is>
+      </c>
+      <c r="BB8" s="24" t="inlineStr">
+        <is>
+          <t>learned_lr</t>
+        </is>
+      </c>
+      <c r="BC8" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="BD8" s="24" t="inlineStr">
+        <is>
+          <t>a454281ab207d2924d585d6b967363fb8e88af45132e3e9d354e4351fb5c237f</t>
+        </is>
+      </c>
+      <c r="BE8" s="24" t="inlineStr">
+        <is>
+          <t>8438bc3f26be5eae</t>
+        </is>
+      </c>
+      <c r="BF8" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG8" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="BH8" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-17T14:01:57.663980Z</t>
+        </is>
+      </c>
+      <c r="BI8" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ8" s="25" t="n"/>
+      <c r="BK8" s="26" t="n">
+        <v>-130</v>
+      </c>
+      <c r="BL8" s="27" t="n">
+        <v>1.769231</v>
+      </c>
+      <c r="BM8" s="28" t="n">
+        <v>0.565217</v>
+      </c>
+      <c r="BN8" s="28" t="n">
+        <v>0.562189</v>
+      </c>
+      <c r="BO8" s="28" t="n"/>
+      <c r="BP8" s="25" t="n"/>
+      <c r="BQ8" s="27" t="n"/>
+      <c r="BR8" s="28" t="n"/>
+      <c r="BS8" s="28" t="n"/>
+      <c r="BT8" s="28" t="n"/>
+      <c r="BU8" s="25" t="n"/>
+      <c r="BV8" s="29" t="n"/>
+      <c r="BW8" s="24" t="n"/>
+      <c r="BX8" s="30" t="n"/>
+      <c r="BY8" s="27" t="n"/>
+      <c r="BZ8" s="24" t="n"/>
+      <c r="CA8" s="31" t="n"/>
+    </row>
+    <row r="9" ht="36" customHeight="1">
+      <c r="A9" s="24" t="inlineStr">
+        <is>
+          <t>f592ac231a074ea9</t>
+        </is>
+      </c>
+      <c r="B9" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-17T14:02:17.091788Z</t>
+        </is>
+      </c>
+      <c r="C9" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-17T23:30Z</t>
+        </is>
+      </c>
+      <c r="D9" s="24" t="inlineStr">
+        <is>
+          <t>401857075</t>
+        </is>
+      </c>
+      <c r="E9" s="24" t="inlineStr">
+        <is>
+          <t>WNBA</t>
+        </is>
+      </c>
+      <c r="F9" s="24" t="inlineStr">
+        <is>
+          <t>Los Angeles Sparks</t>
+        </is>
+      </c>
+      <c r="G9" s="24" t="inlineStr">
+        <is>
+          <t>Chicago Sky</t>
+        </is>
+      </c>
+      <c r="H9" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I9" s="24" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="J9" s="25" t="n"/>
+      <c r="K9" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L9" s="26" t="n">
+        <v>108</v>
+      </c>
+      <c r="M9" s="27" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="N9" s="28" t="n">
+        <v>0.480769</v>
+      </c>
+      <c r="O9" s="28" t="n">
+        <v>0.580113</v>
+      </c>
+      <c r="P9" s="28" t="n"/>
+      <c r="Q9" s="28" t="n">
+        <v>0.099344</v>
+      </c>
+      <c r="R9" s="26" t="n">
+        <v>100</v>
+      </c>
+      <c r="S9" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="T9" s="24" t="inlineStr">
+        <is>
+          <t>wnba-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="U9" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V9" s="24" t="n"/>
+      <c r="W9" s="26" t="n"/>
+      <c r="X9" s="26" t="n"/>
+      <c r="Y9" s="25" t="n"/>
+      <c r="Z9" s="26" t="n"/>
+      <c r="AA9" s="28" t="n"/>
+      <c r="AB9" s="28" t="n"/>
+      <c r="AC9" s="30" t="n"/>
+      <c r="AD9" s="24" t="n"/>
+      <c r="AE9" s="31" t="inlineStr">
+        <is>
+          <t>Learned LR call at threshold 0.5018; executable ask 0.4800 (aec-wnba-la-chi-2026-07-17).</t>
+        </is>
+      </c>
+      <c r="AF9" s="31" t="inlineStr">
+        <is>
+          <t>Learned model; promotion gate not yet open; zero-unit research until review.</t>
+        </is>
+      </c>
+      <c r="AG9" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH9" s="24" t="n"/>
+      <c r="AI9" s="31" t="n"/>
+      <c r="AJ9" s="31" t="n"/>
+      <c r="AK9" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL9" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM9" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN9" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO9" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_MISSING_UNCERTAINTY</t>
+        </is>
+      </c>
+      <c r="AP9" s="24" t="inlineStr">
+        <is>
+          <t>wnba-las</t>
+        </is>
+      </c>
+      <c r="AQ9" s="24" t="inlineStr">
+        <is>
+          <t>Los Angeles Sparks</t>
+        </is>
+      </c>
+      <c r="AR9" s="24" t="inlineStr">
+        <is>
+          <t>Los Angeles Sparks</t>
+        </is>
+      </c>
+      <c r="AS9" s="24" t="inlineStr">
+        <is>
+          <t>wnba-chi</t>
+        </is>
+      </c>
+      <c r="AT9" s="24" t="inlineStr">
+        <is>
+          <t>Chicago Sky</t>
+        </is>
+      </c>
+      <c r="AU9" s="24" t="inlineStr">
+        <is>
+          <t>Chicago Sky</t>
+        </is>
+      </c>
+      <c r="AV9" s="24" t="n"/>
+      <c r="AW9" s="24" t="n"/>
+      <c r="AX9" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY9" s="24" t="n"/>
+      <c r="AZ9" s="24" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="BA9" s="24" t="inlineStr">
+        <is>
+          <t>286653236675a65e58674d10837572801218599b31772016e9d8575bfefa53b4</t>
+        </is>
+      </c>
+      <c r="BB9" s="24" t="inlineStr">
+        <is>
+          <t>learned_lr</t>
+        </is>
+      </c>
+      <c r="BC9" s="24" t="inlineStr">
+        <is>
+          <t>wnba-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="BD9" s="24" t="inlineStr">
+        <is>
+          <t>286653236675a65e58674d10837572801218599b31772016e9d8575bfefa53b4</t>
+        </is>
+      </c>
+      <c r="BE9" s="24" t="inlineStr">
+        <is>
+          <t>8c7d8b8b613f1c27</t>
+        </is>
+      </c>
+      <c r="BF9" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG9" s="24" t="inlineStr">
+        <is>
+          <t>wnba-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="BH9" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-17T14:02:10.568774Z</t>
+        </is>
+      </c>
+      <c r="BI9" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ9" s="25" t="n"/>
+      <c r="BK9" s="26" t="n">
+        <v>108</v>
+      </c>
+      <c r="BL9" s="27" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="BM9" s="28" t="n">
+        <v>0.480769</v>
+      </c>
+      <c r="BN9" s="28" t="n">
+        <v>0.475248</v>
+      </c>
+      <c r="BO9" s="28" t="n"/>
+      <c r="BP9" s="25" t="n"/>
+      <c r="BQ9" s="27" t="n"/>
+      <c r="BR9" s="28" t="n"/>
+      <c r="BS9" s="28" t="n"/>
+      <c r="BT9" s="28" t="n"/>
+      <c r="BU9" s="25" t="n"/>
+      <c r="BV9" s="29" t="n"/>
+      <c r="BW9" s="24" t="n"/>
+      <c r="BX9" s="30" t="n"/>
+      <c r="BY9" s="27" t="n"/>
+      <c r="BZ9" s="24" t="n"/>
+      <c r="CA9" s="31" t="n"/>
+    </row>
+    <row r="10" ht="36" customHeight="1">
+      <c r="A10" s="24" t="inlineStr">
+        <is>
+          <t>3405fe6d522c42ec</t>
+        </is>
+      </c>
+      <c r="B10" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-17T14:02:17.091788Z</t>
+        </is>
+      </c>
+      <c r="C10" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T02:00Z</t>
+        </is>
+      </c>
+      <c r="D10" s="24" t="inlineStr">
+        <is>
+          <t>401857076</t>
+        </is>
+      </c>
+      <c r="E10" s="24" t="inlineStr">
+        <is>
+          <t>WNBA</t>
+        </is>
+      </c>
+      <c r="F10" s="24" t="inlineStr">
+        <is>
+          <t>Connecticut Sun</t>
+        </is>
+      </c>
+      <c r="G10" s="24" t="inlineStr">
+        <is>
+          <t>Phoenix Mercury</t>
+        </is>
+      </c>
+      <c r="H10" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I10" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J10" s="25" t="n"/>
+      <c r="K10" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L10" s="26" t="n">
+        <v>-178</v>
+      </c>
+      <c r="M10" s="27" t="n">
+        <v>1.561798</v>
+      </c>
+      <c r="N10" s="28" t="n">
+        <v>0.640288</v>
+      </c>
+      <c r="O10" s="28" t="n">
+        <v>0.672243</v>
+      </c>
+      <c r="P10" s="28" t="n"/>
+      <c r="Q10" s="28" t="n">
+        <v>0.031955</v>
+      </c>
+      <c r="R10" s="26" t="n">
+        <v>66</v>
+      </c>
+      <c r="S10" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="T10" s="24" t="inlineStr">
+        <is>
+          <t>wnba-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="U10" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V10" s="24" t="n"/>
+      <c r="W10" s="26" t="n"/>
+      <c r="X10" s="26" t="n"/>
+      <c r="Y10" s="25" t="n"/>
+      <c r="Z10" s="26" t="n"/>
+      <c r="AA10" s="28" t="n"/>
+      <c r="AB10" s="28" t="n"/>
+      <c r="AC10" s="30" t="n"/>
+      <c r="AD10" s="24" t="n"/>
+      <c r="AE10" s="31" t="inlineStr">
+        <is>
+          <t>Learned LR call at threshold 0.5018; executable ask 0.6400 (aec-wnba-conn-phx-2026-07-17).</t>
+        </is>
+      </c>
+      <c r="AF10" s="31" t="inlineStr">
+        <is>
+          <t>Learned model; promotion gate not yet open; zero-unit research until review.</t>
+        </is>
+      </c>
+      <c r="AG10" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH10" s="24" t="n"/>
+      <c r="AI10" s="31" t="n"/>
+      <c r="AJ10" s="31" t="n"/>
+      <c r="AK10" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL10" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM10" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN10" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO10" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_MISSING_UNCERTAINTY</t>
+        </is>
+      </c>
+      <c r="AP10" s="24" t="inlineStr">
+        <is>
+          <t>wnba-con</t>
+        </is>
+      </c>
+      <c r="AQ10" s="24" t="inlineStr">
+        <is>
+          <t>Connecticut Sun</t>
+        </is>
+      </c>
+      <c r="AR10" s="24" t="inlineStr">
+        <is>
+          <t>Connecticut Sun</t>
+        </is>
+      </c>
+      <c r="AS10" s="24" t="inlineStr">
+        <is>
+          <t>wnba-phx</t>
+        </is>
+      </c>
+      <c r="AT10" s="24" t="inlineStr">
+        <is>
+          <t>Phoenix Mercury</t>
+        </is>
+      </c>
+      <c r="AU10" s="24" t="inlineStr">
+        <is>
+          <t>Phoenix Mercury</t>
+        </is>
+      </c>
+      <c r="AV10" s="24" t="n"/>
+      <c r="AW10" s="24" t="n"/>
+      <c r="AX10" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY10" s="24" t="n"/>
+      <c r="AZ10" s="24" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="BA10" s="24" t="inlineStr">
+        <is>
+          <t>286653236675a65e58674d10837572801218599b31772016e9d8575bfefa53b4</t>
+        </is>
+      </c>
+      <c r="BB10" s="24" t="inlineStr">
+        <is>
+          <t>learned_lr</t>
+        </is>
+      </c>
+      <c r="BC10" s="24" t="inlineStr">
+        <is>
+          <t>wnba-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="BD10" s="24" t="inlineStr">
+        <is>
+          <t>286653236675a65e58674d10837572801218599b31772016e9d8575bfefa53b4</t>
+        </is>
+      </c>
+      <c r="BE10" s="24" t="inlineStr">
+        <is>
+          <t>5b26e70fb7a6c509</t>
+        </is>
+      </c>
+      <c r="BF10" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG10" s="24" t="inlineStr">
+        <is>
+          <t>wnba-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="BH10" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-17T14:02:11.780961Z</t>
+        </is>
+      </c>
+      <c r="BI10" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ10" s="25" t="n"/>
+      <c r="BK10" s="26" t="n">
+        <v>-178</v>
+      </c>
+      <c r="BL10" s="27" t="n">
+        <v>1.561798</v>
+      </c>
+      <c r="BM10" s="28" t="n">
+        <v>0.640288</v>
+      </c>
+      <c r="BN10" s="28" t="n">
+        <v>0.633663</v>
+      </c>
+      <c r="BO10" s="28" t="n"/>
+      <c r="BP10" s="25" t="n"/>
+      <c r="BQ10" s="27" t="n"/>
+      <c r="BR10" s="28" t="n"/>
+      <c r="BS10" s="28" t="n"/>
+      <c r="BT10" s="28" t="n"/>
+      <c r="BU10" s="25" t="n"/>
+      <c r="BV10" s="29" t="n"/>
+      <c r="BW10" s="24" t="n"/>
+      <c r="BX10" s="30" t="n"/>
+      <c r="BY10" s="27" t="n"/>
+      <c r="BZ10" s="24" t="n"/>
+      <c r="CA10" s="31" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
YRFI/NRFI model blocked — needs per-inning data not in ESPN scoreboard
Real model requires: starting pitcher stats, lineup data, first-inning scoring.
Current scoreboard cache only has final scores. Placeholder removed.
Optimize launchAgent: idle-only, skip duplicate daily runs.
</commit_message>
<xml_diff>
--- a/data/picks.xlsx
+++ b/data/picks.xlsx
@@ -300,8 +300,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CA10" headerRowCount="1">
-  <autoFilter ref="A1:CA10"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CA12" headerRowCount="1">
+  <autoFilter ref="A1:CA12"/>
   <tableColumns count="79">
     <tableColumn id="1" name="pick_id"/>
     <tableColumn id="2" name="created_at_utc"/>
@@ -738,19 +738,19 @@
     </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="6">
-        <f>COUNTA('Picks'!$A$2:$A$10)</f>
+        <f>COUNTA('Picks'!$A$2:$A$12)</f>
         <v/>
       </c>
       <c r="C4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$10,"open")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$12,"open")</f>
         <v/>
       </c>
       <c r="E4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$10,"settled")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$12,"settled")</f>
         <v/>
       </c>
       <c r="G4" s="6">
-        <f>IF(COUNTIFS('Picks'!$U$2:$U$10,"settled",'Picks'!$V$2:$V$10,"win")+COUNTIFS('Picks'!$U$2:$U$10,"settled",'Picks'!$V$2:$V$10,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
+        <f>IF(COUNTIFS('Picks'!$U$2:$U$12,"settled",'Picks'!$V$2:$V$12,"win")+COUNTIFS('Picks'!$U$2:$U$12,"settled",'Picks'!$V$2:$V$12,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
         <v/>
       </c>
     </row>
@@ -778,19 +778,19 @@
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="6">
-        <f>COUNTIF('Picks'!$BX$2:$BX$10,"&gt;0")</f>
+        <f>COUNTIF('Picks'!$BX$2:$BX$12,"&gt;0")</f>
         <v/>
       </c>
       <c r="C7" s="6">
-        <f>COUNTIFS('Picks'!$BX$2:$BX$10,"&gt;0",'Picks'!$V$2:$V$10,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$10,"&gt;0",'Picks'!$V$2:$V$10,"loss")</f>
+        <f>COUNTIFS('Picks'!$BX$2:$BX$12,"&gt;0",'Picks'!$V$2:$V$12,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$12,"&gt;0",'Picks'!$V$2:$V$12,"loss")</f>
         <v/>
       </c>
       <c r="E7" s="7">
-        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$10,"&gt;0",'Picks'!$V$2:$V$10,"win")/(COUNTIFS('Picks'!$BX$2:$BX$10,"&gt;0",'Picks'!$V$2:$V$10,"win")+COUNTIFS('Picks'!$BX$2:$BX$10,"&gt;0",'Picks'!$V$2:$V$10,"loss")),0)</f>
+        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$12,"&gt;0",'Picks'!$V$2:$V$12,"win")/(COUNTIFS('Picks'!$BX$2:$BX$12,"&gt;0",'Picks'!$V$2:$V$12,"win")+COUNTIFS('Picks'!$BX$2:$BX$12,"&gt;0",'Picks'!$V$2:$V$12,"loss")),0)</f>
         <v/>
       </c>
       <c r="G7" s="7">
-        <f>IFERROR(SUM('Picks'!$BY$2:$BY$10)/SUM('Picks'!$BX$2:$BX$10),0)</f>
+        <f>IFERROR(SUM('Picks'!$BY$2:$BY$12)/SUM('Picks'!$BX$2:$BX$12),0)</f>
         <v/>
       </c>
     </row>
@@ -818,19 +818,19 @@
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="8">
-        <f>SUM('Picks'!$BY$2:$BY$10)</f>
+        <f>SUM('Picks'!$BY$2:$BY$12)</f>
         <v/>
       </c>
       <c r="C10" s="9">
-        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$10,"&lt;&gt;",'Picks'!$AB$2:$AB$10),0)</f>
+        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$12,"&lt;&gt;",'Picks'!$AB$2:$AB$12),0)</f>
         <v/>
       </c>
       <c r="E10" s="6">
-        <f>COUNTIFS('Picks'!$AM$2:$AM$10,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$10,"settled")</f>
+        <f>COUNTIFS('Picks'!$AM$2:$AM$12,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$12,"settled")</f>
         <v/>
       </c>
       <c r="G10" s="8">
-        <f>SUMIFS('Picks'!$AC$2:$AC$10,'Picks'!$AM$2:$AM$10,"QUALIFIED_SHADOW_CALL")</f>
+        <f>SUMIFS('Picks'!$AC$2:$AC$12,'Picks'!$AM$2:$AM$12,"QUALIFIED_SHADOW_CALL")</f>
         <v/>
       </c>
     </row>
@@ -885,15 +885,15 @@
         </is>
       </c>
       <c r="B14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$10,$A14,'Picks'!$U$2:$U$10,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$12,$A14,'Picks'!$U$2:$U$12,"settled")</f>
         <v/>
       </c>
       <c r="C14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$10,$A14,'Picks'!$U$2:$U$10,"settled",'Picks'!$V$2:$V$10,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$12,$A14,'Picks'!$U$2:$U$12,"settled",'Picks'!$V$2:$V$12,"win")</f>
         <v/>
       </c>
       <c r="D14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$10,$A14,'Picks'!$U$2:$U$10,"settled",'Picks'!$V$2:$V$10,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$12,$A14,'Picks'!$U$2:$U$12,"settled",'Picks'!$V$2:$V$12,"loss")</f>
         <v/>
       </c>
       <c r="E14" s="14">
@@ -901,11 +901,11 @@
         <v/>
       </c>
       <c r="F14" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$10,'Picks'!$H$2:$H$10,$A14)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$12,'Picks'!$H$2:$H$12,$A14)</f>
         <v/>
       </c>
       <c r="G14" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$10,'Picks'!$H$2:$H$10,$A14,'Picks'!$U$2:$U$10,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$12,'Picks'!$H$2:$H$12,$A14,'Picks'!$U$2:$U$12,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -916,15 +916,15 @@
         </is>
       </c>
       <c r="B15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$10,$A15,'Picks'!$U$2:$U$10,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$12,$A15,'Picks'!$U$2:$U$12,"settled")</f>
         <v/>
       </c>
       <c r="C15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$10,$A15,'Picks'!$U$2:$U$10,"settled",'Picks'!$V$2:$V$10,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$12,$A15,'Picks'!$U$2:$U$12,"settled",'Picks'!$V$2:$V$12,"win")</f>
         <v/>
       </c>
       <c r="D15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$10,$A15,'Picks'!$U$2:$U$10,"settled",'Picks'!$V$2:$V$10,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$12,$A15,'Picks'!$U$2:$U$12,"settled",'Picks'!$V$2:$V$12,"loss")</f>
         <v/>
       </c>
       <c r="E15" s="19">
@@ -932,11 +932,11 @@
         <v/>
       </c>
       <c r="F15" s="20">
-        <f>SUMIFS('Picks'!$BY$2:$BY$10,'Picks'!$H$2:$H$10,$A15)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$12,'Picks'!$H$2:$H$12,$A15)</f>
         <v/>
       </c>
       <c r="G15" s="21">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$10,'Picks'!$H$2:$H$10,$A15,'Picks'!$U$2:$U$10,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$12,'Picks'!$H$2:$H$12,$A15,'Picks'!$U$2:$U$12,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -947,15 +947,15 @@
         </is>
       </c>
       <c r="B16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$10,$A16,'Picks'!$U$2:$U$10,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$12,$A16,'Picks'!$U$2:$U$12,"settled")</f>
         <v/>
       </c>
       <c r="C16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$10,$A16,'Picks'!$U$2:$U$10,"settled",'Picks'!$V$2:$V$10,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$12,$A16,'Picks'!$U$2:$U$12,"settled",'Picks'!$V$2:$V$12,"win")</f>
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$10,$A16,'Picks'!$U$2:$U$10,"settled",'Picks'!$V$2:$V$10,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$12,$A16,'Picks'!$U$2:$U$12,"settled",'Picks'!$V$2:$V$12,"loss")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -963,11 +963,11 @@
         <v/>
       </c>
       <c r="F16" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$10,'Picks'!$H$2:$H$10,$A16)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$12,'Picks'!$H$2:$H$12,$A16)</f>
         <v/>
       </c>
       <c r="G16" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$10,'Picks'!$H$2:$H$10,$A16,'Picks'!$U$2:$U$10,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$12,'Picks'!$H$2:$H$12,$A16,'Picks'!$U$2:$U$12,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -996,7 +996,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:CA10"/>
+  <dimension ref="A1:CA12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3718,6 +3718,504 @@
       <c r="BZ10" s="24" t="n"/>
       <c r="CA10" s="31" t="n"/>
     </row>
+    <row r="11" ht="36" customHeight="1">
+      <c r="A11" s="24" t="inlineStr">
+        <is>
+          <t>93a3540bf0dd49bb</t>
+        </is>
+      </c>
+      <c r="B11" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-17T16:21:24.725309Z</t>
+        </is>
+      </c>
+      <c r="C11" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T20:10Z</t>
+        </is>
+      </c>
+      <c r="D11" s="24" t="inlineStr">
+        <is>
+          <t>401816163</t>
+        </is>
+      </c>
+      <c r="E11" s="24" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="F11" s="24" t="inlineStr">
+        <is>
+          <t>Miami Marlins</t>
+        </is>
+      </c>
+      <c r="G11" s="24" t="inlineStr">
+        <is>
+          <t>Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="H11" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I11" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J11" s="25" t="n"/>
+      <c r="K11" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L11" s="26" t="n">
+        <v>-130</v>
+      </c>
+      <c r="M11" s="27" t="n">
+        <v>1.769231</v>
+      </c>
+      <c r="N11" s="28" t="n">
+        <v>0.565217</v>
+      </c>
+      <c r="O11" s="28" t="n">
+        <v>0.605633</v>
+      </c>
+      <c r="P11" s="28" t="n"/>
+      <c r="Q11" s="28" t="n">
+        <v>0.040416</v>
+      </c>
+      <c r="R11" s="26" t="n">
+        <v>70</v>
+      </c>
+      <c r="S11" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="T11" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="U11" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V11" s="24" t="n"/>
+      <c r="W11" s="26" t="n"/>
+      <c r="X11" s="26" t="n"/>
+      <c r="Y11" s="25" t="n"/>
+      <c r="Z11" s="26" t="n"/>
+      <c r="AA11" s="28" t="n"/>
+      <c r="AB11" s="28" t="n"/>
+      <c r="AC11" s="30" t="n"/>
+      <c r="AD11" s="24" t="n"/>
+      <c r="AE11" s="31" t="inlineStr">
+        <is>
+          <t>Learned LR call at threshold 0.6018; executable ask 0.5650 (aec-mlb-mia-mil-2026-07-18).</t>
+        </is>
+      </c>
+      <c r="AF11" s="31" t="inlineStr">
+        <is>
+          <t>Learned model; promotion gate not yet open; zero-unit research until review.</t>
+        </is>
+      </c>
+      <c r="AG11" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH11" s="24" t="n"/>
+      <c r="AI11" s="31" t="n"/>
+      <c r="AJ11" s="31" t="n"/>
+      <c r="AK11" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL11" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM11" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN11" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO11" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_MISSING_UNCERTAINTY</t>
+        </is>
+      </c>
+      <c r="AP11" s="24" t="inlineStr">
+        <is>
+          <t>mlb-mia</t>
+        </is>
+      </c>
+      <c r="AQ11" s="24" t="inlineStr">
+        <is>
+          <t>Miami Marlins</t>
+        </is>
+      </c>
+      <c r="AR11" s="24" t="inlineStr">
+        <is>
+          <t>Miami Marlins</t>
+        </is>
+      </c>
+      <c r="AS11" s="24" t="inlineStr">
+        <is>
+          <t>mlb-mil</t>
+        </is>
+      </c>
+      <c r="AT11" s="24" t="inlineStr">
+        <is>
+          <t>Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="AU11" s="24" t="inlineStr">
+        <is>
+          <t>Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="AV11" s="24" t="n"/>
+      <c r="AW11" s="24" t="n"/>
+      <c r="AX11" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY11" s="24" t="n"/>
+      <c r="AZ11" s="24" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="BA11" s="24" t="inlineStr">
+        <is>
+          <t>a454281ab207d2924d585d6b967363fb8e88af45132e3e9d354e4351fb5c237f</t>
+        </is>
+      </c>
+      <c r="BB11" s="24" t="inlineStr">
+        <is>
+          <t>learned_lr</t>
+        </is>
+      </c>
+      <c r="BC11" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="BD11" s="24" t="inlineStr">
+        <is>
+          <t>a454281ab207d2924d585d6b967363fb8e88af45132e3e9d354e4351fb5c237f</t>
+        </is>
+      </c>
+      <c r="BE11" s="24" t="inlineStr">
+        <is>
+          <t>c7348ce29d666909</t>
+        </is>
+      </c>
+      <c r="BF11" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG11" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="BH11" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-17T16:21:07.161405Z</t>
+        </is>
+      </c>
+      <c r="BI11" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ11" s="25" t="n"/>
+      <c r="BK11" s="26" t="n">
+        <v>-130</v>
+      </c>
+      <c r="BL11" s="27" t="n">
+        <v>1.769231</v>
+      </c>
+      <c r="BM11" s="28" t="n">
+        <v>0.565217</v>
+      </c>
+      <c r="BN11" s="28" t="n">
+        <v>0.562189</v>
+      </c>
+      <c r="BO11" s="28" t="n"/>
+      <c r="BP11" s="25" t="n"/>
+      <c r="BQ11" s="27" t="n"/>
+      <c r="BR11" s="28" t="n"/>
+      <c r="BS11" s="28" t="n"/>
+      <c r="BT11" s="28" t="n"/>
+      <c r="BU11" s="25" t="n"/>
+      <c r="BV11" s="29" t="n"/>
+      <c r="BW11" s="24" t="n"/>
+      <c r="BX11" s="30" t="n"/>
+      <c r="BY11" s="27" t="n"/>
+      <c r="BZ11" s="24" t="n"/>
+      <c r="CA11" s="31" t="n"/>
+    </row>
+    <row r="12" ht="36" customHeight="1">
+      <c r="A12" s="24" t="inlineStr">
+        <is>
+          <t>c884dc7cf1104640</t>
+        </is>
+      </c>
+      <c r="B12" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-17T16:21:30.375686Z</t>
+        </is>
+      </c>
+      <c r="C12" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-19T00:00Z</t>
+        </is>
+      </c>
+      <c r="D12" s="24" t="inlineStr">
+        <is>
+          <t>401857077</t>
+        </is>
+      </c>
+      <c r="E12" s="24" t="inlineStr">
+        <is>
+          <t>WNBA</t>
+        </is>
+      </c>
+      <c r="F12" s="24" t="inlineStr">
+        <is>
+          <t>New York Liberty</t>
+        </is>
+      </c>
+      <c r="G12" s="24" t="inlineStr">
+        <is>
+          <t>Indiana Fever</t>
+        </is>
+      </c>
+      <c r="H12" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I12" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J12" s="25" t="n"/>
+      <c r="K12" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L12" s="26" t="n">
+        <v>117</v>
+      </c>
+      <c r="M12" s="27" t="n">
+        <v>2.17</v>
+      </c>
+      <c r="N12" s="28" t="n">
+        <v>0.460829</v>
+      </c>
+      <c r="O12" s="28" t="n">
+        <v>0.632778</v>
+      </c>
+      <c r="P12" s="28" t="n"/>
+      <c r="Q12" s="28" t="n">
+        <v>0.171949</v>
+      </c>
+      <c r="R12" s="26" t="n">
+        <v>100</v>
+      </c>
+      <c r="S12" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="T12" s="24" t="inlineStr">
+        <is>
+          <t>wnba-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="U12" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V12" s="24" t="n"/>
+      <c r="W12" s="26" t="n"/>
+      <c r="X12" s="26" t="n"/>
+      <c r="Y12" s="25" t="n"/>
+      <c r="Z12" s="26" t="n"/>
+      <c r="AA12" s="28" t="n"/>
+      <c r="AB12" s="28" t="n"/>
+      <c r="AC12" s="30" t="n"/>
+      <c r="AD12" s="24" t="n"/>
+      <c r="AE12" s="31" t="inlineStr">
+        <is>
+          <t>Learned LR call at threshold 0.5018; executable ask 0.4600 (aec-wnba-ny-ind-2026-07-18).</t>
+        </is>
+      </c>
+      <c r="AF12" s="31" t="inlineStr">
+        <is>
+          <t>Learned model; promotion gate not yet open; zero-unit research until review.</t>
+        </is>
+      </c>
+      <c r="AG12" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH12" s="24" t="n"/>
+      <c r="AI12" s="31" t="n"/>
+      <c r="AJ12" s="31" t="n"/>
+      <c r="AK12" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL12" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM12" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN12" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO12" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_MISSING_UNCERTAINTY</t>
+        </is>
+      </c>
+      <c r="AP12" s="24" t="inlineStr">
+        <is>
+          <t>wnba-nyl</t>
+        </is>
+      </c>
+      <c r="AQ12" s="24" t="inlineStr">
+        <is>
+          <t>New York Liberty</t>
+        </is>
+      </c>
+      <c r="AR12" s="24" t="inlineStr">
+        <is>
+          <t>New York Liberty</t>
+        </is>
+      </c>
+      <c r="AS12" s="24" t="inlineStr">
+        <is>
+          <t>wnba-ind</t>
+        </is>
+      </c>
+      <c r="AT12" s="24" t="inlineStr">
+        <is>
+          <t>Indiana Fever</t>
+        </is>
+      </c>
+      <c r="AU12" s="24" t="inlineStr">
+        <is>
+          <t>Indiana Fever</t>
+        </is>
+      </c>
+      <c r="AV12" s="24" t="n"/>
+      <c r="AW12" s="24" t="n"/>
+      <c r="AX12" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY12" s="24" t="n"/>
+      <c r="AZ12" s="24" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="BA12" s="24" t="inlineStr">
+        <is>
+          <t>286653236675a65e58674d10837572801218599b31772016e9d8575bfefa53b4</t>
+        </is>
+      </c>
+      <c r="BB12" s="24" t="inlineStr">
+        <is>
+          <t>learned_lr</t>
+        </is>
+      </c>
+      <c r="BC12" s="24" t="inlineStr">
+        <is>
+          <t>wnba-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="BD12" s="24" t="inlineStr">
+        <is>
+          <t>286653236675a65e58674d10837572801218599b31772016e9d8575bfefa53b4</t>
+        </is>
+      </c>
+      <c r="BE12" s="24" t="inlineStr">
+        <is>
+          <t>e4f3f616d306cafe</t>
+        </is>
+      </c>
+      <c r="BF12" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG12" s="24" t="inlineStr">
+        <is>
+          <t>wnba-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="BH12" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-17T16:21:13.188564Z</t>
+        </is>
+      </c>
+      <c r="BI12" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ12" s="25" t="n"/>
+      <c r="BK12" s="26" t="n">
+        <v>117</v>
+      </c>
+      <c r="BL12" s="27" t="n">
+        <v>2.17</v>
+      </c>
+      <c r="BM12" s="28" t="n">
+        <v>0.460829</v>
+      </c>
+      <c r="BN12" s="28" t="n">
+        <v>0.455446</v>
+      </c>
+      <c r="BO12" s="28" t="n"/>
+      <c r="BP12" s="25" t="n"/>
+      <c r="BQ12" s="27" t="n"/>
+      <c r="BR12" s="28" t="n"/>
+      <c r="BS12" s="28" t="n"/>
+      <c r="BT12" s="28" t="n"/>
+      <c r="BU12" s="25" t="n"/>
+      <c r="BV12" s="29" t="n"/>
+      <c r="BW12" s="24" t="n"/>
+      <c r="BX12" s="30" t="n"/>
+      <c r="BY12" s="27" t="n"/>
+      <c r="BZ12" s="24" t="n"/>
+      <c r="CA12" s="31" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Portfolio: readable market names + win rate in history KPIs
slugToTitle() converts Polymarket slugs to readable format.
Win rate added to Trade & Settlement History KPIs.
</commit_message>
<xml_diff>
--- a/data/picks.xlsx
+++ b/data/picks.xlsx
@@ -300,8 +300,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CA12" headerRowCount="1">
-  <autoFilter ref="A1:CA12"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CA13" headerRowCount="1">
+  <autoFilter ref="A1:CA13"/>
   <tableColumns count="79">
     <tableColumn id="1" name="pick_id"/>
     <tableColumn id="2" name="created_at_utc"/>
@@ -738,19 +738,19 @@
     </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="6">
-        <f>COUNTA('Picks'!$A$2:$A$12)</f>
+        <f>COUNTA('Picks'!$A$2:$A$13)</f>
         <v/>
       </c>
       <c r="C4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$12,"open")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$13,"open")</f>
         <v/>
       </c>
       <c r="E4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$12,"settled")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$13,"settled")</f>
         <v/>
       </c>
       <c r="G4" s="6">
-        <f>IF(COUNTIFS('Picks'!$U$2:$U$12,"settled",'Picks'!$V$2:$V$12,"win")+COUNTIFS('Picks'!$U$2:$U$12,"settled",'Picks'!$V$2:$V$12,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
+        <f>IF(COUNTIFS('Picks'!$U$2:$U$13,"settled",'Picks'!$V$2:$V$13,"win")+COUNTIFS('Picks'!$U$2:$U$13,"settled",'Picks'!$V$2:$V$13,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
         <v/>
       </c>
     </row>
@@ -778,19 +778,19 @@
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="6">
-        <f>COUNTIF('Picks'!$BX$2:$BX$12,"&gt;0")</f>
+        <f>COUNTIF('Picks'!$BX$2:$BX$13,"&gt;0")</f>
         <v/>
       </c>
       <c r="C7" s="6">
-        <f>COUNTIFS('Picks'!$BX$2:$BX$12,"&gt;0",'Picks'!$V$2:$V$12,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$12,"&gt;0",'Picks'!$V$2:$V$12,"loss")</f>
+        <f>COUNTIFS('Picks'!$BX$2:$BX$13,"&gt;0",'Picks'!$V$2:$V$13,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$13,"&gt;0",'Picks'!$V$2:$V$13,"loss")</f>
         <v/>
       </c>
       <c r="E7" s="7">
-        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$12,"&gt;0",'Picks'!$V$2:$V$12,"win")/(COUNTIFS('Picks'!$BX$2:$BX$12,"&gt;0",'Picks'!$V$2:$V$12,"win")+COUNTIFS('Picks'!$BX$2:$BX$12,"&gt;0",'Picks'!$V$2:$V$12,"loss")),0)</f>
+        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$13,"&gt;0",'Picks'!$V$2:$V$13,"win")/(COUNTIFS('Picks'!$BX$2:$BX$13,"&gt;0",'Picks'!$V$2:$V$13,"win")+COUNTIFS('Picks'!$BX$2:$BX$13,"&gt;0",'Picks'!$V$2:$V$13,"loss")),0)</f>
         <v/>
       </c>
       <c r="G7" s="7">
-        <f>IFERROR(SUM('Picks'!$BY$2:$BY$12)/SUM('Picks'!$BX$2:$BX$12),0)</f>
+        <f>IFERROR(SUM('Picks'!$BY$2:$BY$13)/SUM('Picks'!$BX$2:$BX$13),0)</f>
         <v/>
       </c>
     </row>
@@ -818,19 +818,19 @@
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="8">
-        <f>SUM('Picks'!$BY$2:$BY$12)</f>
+        <f>SUM('Picks'!$BY$2:$BY$13)</f>
         <v/>
       </c>
       <c r="C10" s="9">
-        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$12,"&lt;&gt;",'Picks'!$AB$2:$AB$12),0)</f>
+        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$13,"&lt;&gt;",'Picks'!$AB$2:$AB$13),0)</f>
         <v/>
       </c>
       <c r="E10" s="6">
-        <f>COUNTIFS('Picks'!$AM$2:$AM$12,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$12,"settled")</f>
+        <f>COUNTIFS('Picks'!$AM$2:$AM$13,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$13,"settled")</f>
         <v/>
       </c>
       <c r="G10" s="8">
-        <f>SUMIFS('Picks'!$AC$2:$AC$12,'Picks'!$AM$2:$AM$12,"QUALIFIED_SHADOW_CALL")</f>
+        <f>SUMIFS('Picks'!$AC$2:$AC$13,'Picks'!$AM$2:$AM$13,"QUALIFIED_SHADOW_CALL")</f>
         <v/>
       </c>
     </row>
@@ -885,15 +885,15 @@
         </is>
       </c>
       <c r="B14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$12,$A14,'Picks'!$U$2:$U$12,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$13,$A14,'Picks'!$U$2:$U$13,"settled")</f>
         <v/>
       </c>
       <c r="C14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$12,$A14,'Picks'!$U$2:$U$12,"settled",'Picks'!$V$2:$V$12,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$13,$A14,'Picks'!$U$2:$U$13,"settled",'Picks'!$V$2:$V$13,"win")</f>
         <v/>
       </c>
       <c r="D14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$12,$A14,'Picks'!$U$2:$U$12,"settled",'Picks'!$V$2:$V$12,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$13,$A14,'Picks'!$U$2:$U$13,"settled",'Picks'!$V$2:$V$13,"loss")</f>
         <v/>
       </c>
       <c r="E14" s="14">
@@ -901,11 +901,11 @@
         <v/>
       </c>
       <c r="F14" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$12,'Picks'!$H$2:$H$12,$A14)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$13,'Picks'!$H$2:$H$13,$A14)</f>
         <v/>
       </c>
       <c r="G14" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$12,'Picks'!$H$2:$H$12,$A14,'Picks'!$U$2:$U$12,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$13,'Picks'!$H$2:$H$13,$A14,'Picks'!$U$2:$U$13,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -916,15 +916,15 @@
         </is>
       </c>
       <c r="B15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$12,$A15,'Picks'!$U$2:$U$12,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$13,$A15,'Picks'!$U$2:$U$13,"settled")</f>
         <v/>
       </c>
       <c r="C15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$12,$A15,'Picks'!$U$2:$U$12,"settled",'Picks'!$V$2:$V$12,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$13,$A15,'Picks'!$U$2:$U$13,"settled",'Picks'!$V$2:$V$13,"win")</f>
         <v/>
       </c>
       <c r="D15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$12,$A15,'Picks'!$U$2:$U$12,"settled",'Picks'!$V$2:$V$12,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$13,$A15,'Picks'!$U$2:$U$13,"settled",'Picks'!$V$2:$V$13,"loss")</f>
         <v/>
       </c>
       <c r="E15" s="19">
@@ -932,11 +932,11 @@
         <v/>
       </c>
       <c r="F15" s="20">
-        <f>SUMIFS('Picks'!$BY$2:$BY$12,'Picks'!$H$2:$H$12,$A15)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$13,'Picks'!$H$2:$H$13,$A15)</f>
         <v/>
       </c>
       <c r="G15" s="21">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$12,'Picks'!$H$2:$H$12,$A15,'Picks'!$U$2:$U$12,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$13,'Picks'!$H$2:$H$13,$A15,'Picks'!$U$2:$U$13,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -947,15 +947,15 @@
         </is>
       </c>
       <c r="B16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$12,$A16,'Picks'!$U$2:$U$12,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$13,$A16,'Picks'!$U$2:$U$13,"settled")</f>
         <v/>
       </c>
       <c r="C16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$12,$A16,'Picks'!$U$2:$U$12,"settled",'Picks'!$V$2:$V$12,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$13,$A16,'Picks'!$U$2:$U$13,"settled",'Picks'!$V$2:$V$13,"win")</f>
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$12,$A16,'Picks'!$U$2:$U$12,"settled",'Picks'!$V$2:$V$12,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$13,$A16,'Picks'!$U$2:$U$13,"settled",'Picks'!$V$2:$V$13,"loss")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -963,11 +963,11 @@
         <v/>
       </c>
       <c r="F16" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$12,'Picks'!$H$2:$H$12,$A16)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$13,'Picks'!$H$2:$H$13,$A16)</f>
         <v/>
       </c>
       <c r="G16" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$12,'Picks'!$H$2:$H$12,$A16,'Picks'!$U$2:$U$12,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$13,'Picks'!$H$2:$H$13,$A16,'Picks'!$U$2:$U$13,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -996,7 +996,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:CA12"/>
+  <dimension ref="A1:CA13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1558,18 +1558,38 @@
       </c>
       <c r="U2" s="24" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V2" s="24" t="n"/>
-      <c r="W2" s="26" t="n"/>
-      <c r="X2" s="26" t="n"/>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V2" s="24" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="W2" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="X2" s="26" t="n">
+        <v>2</v>
+      </c>
       <c r="Y2" s="25" t="n"/>
-      <c r="Z2" s="26" t="n"/>
-      <c r="AA2" s="28" t="n"/>
-      <c r="AB2" s="28" t="n"/>
-      <c r="AC2" s="30" t="n"/>
-      <c r="AD2" s="24" t="n"/>
+      <c r="Z2" s="26" t="n">
+        <v>-147</v>
+      </c>
+      <c r="AA2" s="28" t="n">
+        <v>0.595</v>
+      </c>
+      <c r="AB2" s="28" t="n">
+        <v>0.009938000000000001</v>
+      </c>
+      <c r="AC2" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD2" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T05:45:53.690448Z</t>
+        </is>
+      </c>
       <c r="AE2" s="31" t="inlineStr">
         <is>
           <t>Learned LR call at threshold 0.6018; executable ask 0.5850 (aec-mlb-mia-mil-2026-07-17).</t>
@@ -1714,17 +1734,33 @@
       </c>
       <c r="BO2" s="28" t="n"/>
       <c r="BP2" s="25" t="n"/>
-      <c r="BQ2" s="27" t="n"/>
-      <c r="BR2" s="28" t="n"/>
+      <c r="BQ2" s="27" t="n">
+        <v>1.680272</v>
+      </c>
+      <c r="BR2" s="28" t="n">
+        <v>0.595</v>
+      </c>
       <c r="BS2" s="28" t="n"/>
       <c r="BT2" s="28" t="n"/>
       <c r="BU2" s="25" t="n"/>
       <c r="BV2" s="29" t="n"/>
       <c r="BW2" s="24" t="n"/>
-      <c r="BX2" s="30" t="n"/>
-      <c r="BY2" s="27" t="n"/>
-      <c r="BZ2" s="24" t="n"/>
-      <c r="CA2" s="31" t="n"/>
+      <c r="BX2" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="BY2" s="27" t="n">
+        <v>0.70922</v>
+      </c>
+      <c r="BZ2" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T05:45:53.690448Z</t>
+        </is>
+      </c>
+      <c r="CA2" s="31" t="inlineStr">
+        <is>
+          <t>fixed one-unit hypothetical scoring; no real exposure or execution</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="36" customHeight="1">
       <c r="A3" s="24" t="inlineStr">
@@ -1807,18 +1843,38 @@
       </c>
       <c r="U3" s="24" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V3" s="24" t="n"/>
-      <c r="W3" s="26" t="n"/>
-      <c r="X3" s="26" t="n"/>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V3" s="24" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="W3" s="26" t="n">
+        <v>5</v>
+      </c>
+      <c r="X3" s="26" t="n">
+        <v>2</v>
+      </c>
       <c r="Y3" s="25" t="n"/>
-      <c r="Z3" s="26" t="n"/>
-      <c r="AA3" s="28" t="n"/>
-      <c r="AB3" s="28" t="n"/>
-      <c r="AC3" s="30" t="n"/>
-      <c r="AD3" s="24" t="n"/>
+      <c r="Z3" s="26" t="n">
+        <v>-133</v>
+      </c>
+      <c r="AA3" s="28" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="AB3" s="28" t="n">
+        <v>0.004783</v>
+      </c>
+      <c r="AC3" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD3" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T05:45:53.777767Z</t>
+        </is>
+      </c>
       <c r="AE3" s="31" t="inlineStr">
         <is>
           <t>Learned LR call at threshold 0.6018; executable ask 0.5650 (aec-mlb-min-chc-2026-07-17).</t>
@@ -1831,7 +1887,7 @@
       </c>
       <c r="AG3" s="24" t="inlineStr">
         <is>
-          <t>not_applicable</t>
+          <t>review_required</t>
         </is>
       </c>
       <c r="AH3" s="24" t="n"/>
@@ -1963,17 +2019,33 @@
       </c>
       <c r="BO3" s="28" t="n"/>
       <c r="BP3" s="25" t="n"/>
-      <c r="BQ3" s="27" t="n"/>
-      <c r="BR3" s="28" t="n"/>
+      <c r="BQ3" s="27" t="n">
+        <v>1.75188</v>
+      </c>
+      <c r="BR3" s="28" t="n">
+        <v>0.57</v>
+      </c>
       <c r="BS3" s="28" t="n"/>
       <c r="BT3" s="28" t="n"/>
       <c r="BU3" s="25" t="n"/>
       <c r="BV3" s="29" t="n"/>
       <c r="BW3" s="24" t="n"/>
-      <c r="BX3" s="30" t="n"/>
-      <c r="BY3" s="27" t="n"/>
-      <c r="BZ3" s="24" t="n"/>
-      <c r="CA3" s="31" t="n"/>
+      <c r="BX3" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="BY3" s="27" t="n">
+        <v>-1</v>
+      </c>
+      <c r="BZ3" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T05:45:53.777767Z</t>
+        </is>
+      </c>
+      <c r="CA3" s="31" t="inlineStr">
+        <is>
+          <t>fixed one-unit hypothetical scoring; no real exposure or execution</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="36" customHeight="1">
       <c r="A4" s="24" t="inlineStr">
@@ -2056,18 +2128,32 @@
       </c>
       <c r="U4" s="24" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V4" s="24" t="n"/>
-      <c r="W4" s="26" t="n"/>
-      <c r="X4" s="26" t="n"/>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V4" s="24" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="W4" s="26" t="n">
+        <v>107</v>
+      </c>
+      <c r="X4" s="26" t="n">
+        <v>110</v>
+      </c>
       <c r="Y4" s="25" t="n"/>
       <c r="Z4" s="26" t="n"/>
       <c r="AA4" s="28" t="n"/>
       <c r="AB4" s="28" t="n"/>
-      <c r="AC4" s="30" t="n"/>
-      <c r="AD4" s="24" t="n"/>
+      <c r="AC4" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD4" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T05:45:54.458400Z</t>
+        </is>
+      </c>
       <c r="AE4" s="31" t="inlineStr">
         <is>
           <t>Learned LR call at threshold 0.5018; executable ask 0.7800 (aec-wnba-sea-ind-2026-07-17).</t>
@@ -2219,10 +2305,22 @@
       <c r="BU4" s="25" t="n"/>
       <c r="BV4" s="29" t="n"/>
       <c r="BW4" s="24" t="n"/>
-      <c r="BX4" s="30" t="n"/>
-      <c r="BY4" s="27" t="n"/>
-      <c r="BZ4" s="24" t="n"/>
-      <c r="CA4" s="31" t="n"/>
+      <c r="BX4" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="BY4" s="27" t="n">
+        <v>0.28169</v>
+      </c>
+      <c r="BZ4" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T05:45:54.458400Z</t>
+        </is>
+      </c>
+      <c r="CA4" s="31" t="inlineStr">
+        <is>
+          <t>fixed one-unit hypothetical scoring; no real exposure or execution</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="36" customHeight="1">
       <c r="A5" s="24" t="inlineStr">
@@ -2305,18 +2403,32 @@
       </c>
       <c r="U5" s="24" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V5" s="24" t="n"/>
-      <c r="W5" s="26" t="n"/>
-      <c r="X5" s="26" t="n"/>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V5" s="24" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="W5" s="26" t="n">
+        <v>82</v>
+      </c>
+      <c r="X5" s="26" t="n">
+        <v>96</v>
+      </c>
       <c r="Y5" s="25" t="n"/>
       <c r="Z5" s="26" t="n"/>
       <c r="AA5" s="28" t="n"/>
       <c r="AB5" s="28" t="n"/>
-      <c r="AC5" s="30" t="n"/>
-      <c r="AD5" s="24" t="n"/>
+      <c r="AC5" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD5" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T05:45:54.545671Z</t>
+        </is>
+      </c>
       <c r="AE5" s="31" t="inlineStr">
         <is>
           <t>Learned LR call at threshold 0.5018; executable ask 0.4900 (aec-wnba-la-chi-2026-07-17).</t>
@@ -2329,7 +2441,7 @@
       </c>
       <c r="AG5" s="24" t="inlineStr">
         <is>
-          <t>not_applicable</t>
+          <t>review_required</t>
         </is>
       </c>
       <c r="AH5" s="24" t="n"/>
@@ -2468,10 +2580,22 @@
       <c r="BU5" s="25" t="n"/>
       <c r="BV5" s="29" t="n"/>
       <c r="BW5" s="24" t="n"/>
-      <c r="BX5" s="30" t="n"/>
-      <c r="BY5" s="27" t="n"/>
-      <c r="BZ5" s="24" t="n"/>
-      <c r="CA5" s="31" t="n"/>
+      <c r="BX5" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="BY5" s="27" t="n">
+        <v>-1</v>
+      </c>
+      <c r="BZ5" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T05:45:54.545671Z</t>
+        </is>
+      </c>
+      <c r="CA5" s="31" t="inlineStr">
+        <is>
+          <t>fixed one-unit hypothetical scoring; no real exposure or execution</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="36" customHeight="1">
       <c r="A6" s="24" t="inlineStr">
@@ -2554,18 +2678,32 @@
       </c>
       <c r="U6" s="24" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V6" s="24" t="n"/>
-      <c r="W6" s="26" t="n"/>
-      <c r="X6" s="26" t="n"/>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V6" s="24" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="W6" s="26" t="n">
+        <v>96</v>
+      </c>
+      <c r="X6" s="26" t="n">
+        <v>83</v>
+      </c>
       <c r="Y6" s="25" t="n"/>
       <c r="Z6" s="26" t="n"/>
       <c r="AA6" s="28" t="n"/>
       <c r="AB6" s="28" t="n"/>
-      <c r="AC6" s="30" t="n"/>
-      <c r="AD6" s="24" t="n"/>
+      <c r="AC6" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD6" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T05:45:54.629639Z</t>
+        </is>
+      </c>
       <c r="AE6" s="31" t="inlineStr">
         <is>
           <t>Learned LR call at threshold 0.5018; executable ask 0.6400 (aec-wnba-conn-phx-2026-07-17).</t>
@@ -2578,7 +2716,7 @@
       </c>
       <c r="AG6" s="24" t="inlineStr">
         <is>
-          <t>not_applicable</t>
+          <t>review_required</t>
         </is>
       </c>
       <c r="AH6" s="24" t="n"/>
@@ -2717,10 +2855,22 @@
       <c r="BU6" s="25" t="n"/>
       <c r="BV6" s="29" t="n"/>
       <c r="BW6" s="24" t="n"/>
-      <c r="BX6" s="30" t="n"/>
-      <c r="BY6" s="27" t="n"/>
-      <c r="BZ6" s="24" t="n"/>
-      <c r="CA6" s="31" t="n"/>
+      <c r="BX6" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="BY6" s="27" t="n">
+        <v>-1</v>
+      </c>
+      <c r="BZ6" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T05:45:54.629639Z</t>
+        </is>
+      </c>
+      <c r="CA6" s="31" t="inlineStr">
+        <is>
+          <t>fixed one-unit hypothetical scoring; no real exposure or execution</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="36" customHeight="1">
       <c r="A7" s="24" t="inlineStr">
@@ -2803,18 +2953,38 @@
       </c>
       <c r="U7" s="24" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V7" s="24" t="n"/>
-      <c r="W7" s="26" t="n"/>
-      <c r="X7" s="26" t="n"/>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V7" s="24" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="W7" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="X7" s="26" t="n">
+        <v>2</v>
+      </c>
       <c r="Y7" s="25" t="n"/>
-      <c r="Z7" s="26" t="n"/>
-      <c r="AA7" s="28" t="n"/>
-      <c r="AB7" s="28" t="n"/>
-      <c r="AC7" s="30" t="n"/>
-      <c r="AD7" s="24" t="n"/>
+      <c r="Z7" s="26" t="n">
+        <v>-147</v>
+      </c>
+      <c r="AA7" s="28" t="n">
+        <v>0.595</v>
+      </c>
+      <c r="AB7" s="28" t="n">
+        <v>0.009938000000000001</v>
+      </c>
+      <c r="AC7" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD7" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T05:45:54.715857Z</t>
+        </is>
+      </c>
       <c r="AE7" s="31" t="inlineStr">
         <is>
           <t>Learned LR call at threshold 0.6018; executable ask 0.5850 (aec-mlb-mia-mil-2026-07-17).</t>
@@ -2959,17 +3129,33 @@
       </c>
       <c r="BO7" s="28" t="n"/>
       <c r="BP7" s="25" t="n"/>
-      <c r="BQ7" s="27" t="n"/>
-      <c r="BR7" s="28" t="n"/>
+      <c r="BQ7" s="27" t="n">
+        <v>1.680272</v>
+      </c>
+      <c r="BR7" s="28" t="n">
+        <v>0.595</v>
+      </c>
       <c r="BS7" s="28" t="n"/>
       <c r="BT7" s="28" t="n"/>
       <c r="BU7" s="25" t="n"/>
       <c r="BV7" s="29" t="n"/>
       <c r="BW7" s="24" t="n"/>
-      <c r="BX7" s="30" t="n"/>
-      <c r="BY7" s="27" t="n"/>
-      <c r="BZ7" s="24" t="n"/>
-      <c r="CA7" s="31" t="n"/>
+      <c r="BX7" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="BY7" s="27" t="n">
+        <v>0.70922</v>
+      </c>
+      <c r="BZ7" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T05:45:54.715857Z</t>
+        </is>
+      </c>
+      <c r="CA7" s="31" t="inlineStr">
+        <is>
+          <t>fixed one-unit hypothetical scoring; no real exposure or execution</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="36" customHeight="1">
       <c r="A8" s="24" t="inlineStr">
@@ -3052,18 +3238,38 @@
       </c>
       <c r="U8" s="24" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V8" s="24" t="n"/>
-      <c r="W8" s="26" t="n"/>
-      <c r="X8" s="26" t="n"/>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V8" s="24" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="W8" s="26" t="n">
+        <v>5</v>
+      </c>
+      <c r="X8" s="26" t="n">
+        <v>2</v>
+      </c>
       <c r="Y8" s="25" t="n"/>
-      <c r="Z8" s="26" t="n"/>
-      <c r="AA8" s="28" t="n"/>
-      <c r="AB8" s="28" t="n"/>
-      <c r="AC8" s="30" t="n"/>
-      <c r="AD8" s="24" t="n"/>
+      <c r="Z8" s="26" t="n">
+        <v>-133</v>
+      </c>
+      <c r="AA8" s="28" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="AB8" s="28" t="n">
+        <v>0.004783</v>
+      </c>
+      <c r="AC8" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD8" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T05:45:54.800172Z</t>
+        </is>
+      </c>
       <c r="AE8" s="31" t="inlineStr">
         <is>
           <t>Learned LR call at threshold 0.6018; executable ask 0.5650 (aec-mlb-min-chc-2026-07-17).</t>
@@ -3076,7 +3282,7 @@
       </c>
       <c r="AG8" s="24" t="inlineStr">
         <is>
-          <t>not_applicable</t>
+          <t>review_required</t>
         </is>
       </c>
       <c r="AH8" s="24" t="n"/>
@@ -3208,17 +3414,33 @@
       </c>
       <c r="BO8" s="28" t="n"/>
       <c r="BP8" s="25" t="n"/>
-      <c r="BQ8" s="27" t="n"/>
-      <c r="BR8" s="28" t="n"/>
+      <c r="BQ8" s="27" t="n">
+        <v>1.75188</v>
+      </c>
+      <c r="BR8" s="28" t="n">
+        <v>0.57</v>
+      </c>
       <c r="BS8" s="28" t="n"/>
       <c r="BT8" s="28" t="n"/>
       <c r="BU8" s="25" t="n"/>
       <c r="BV8" s="29" t="n"/>
       <c r="BW8" s="24" t="n"/>
-      <c r="BX8" s="30" t="n"/>
-      <c r="BY8" s="27" t="n"/>
-      <c r="BZ8" s="24" t="n"/>
-      <c r="CA8" s="31" t="n"/>
+      <c r="BX8" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="BY8" s="27" t="n">
+        <v>-1</v>
+      </c>
+      <c r="BZ8" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T05:45:54.800172Z</t>
+        </is>
+      </c>
+      <c r="CA8" s="31" t="inlineStr">
+        <is>
+          <t>fixed one-unit hypothetical scoring; no real exposure or execution</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="36" customHeight="1">
       <c r="A9" s="24" t="inlineStr">
@@ -3301,18 +3523,32 @@
       </c>
       <c r="U9" s="24" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V9" s="24" t="n"/>
-      <c r="W9" s="26" t="n"/>
-      <c r="X9" s="26" t="n"/>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V9" s="24" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="W9" s="26" t="n">
+        <v>82</v>
+      </c>
+      <c r="X9" s="26" t="n">
+        <v>96</v>
+      </c>
       <c r="Y9" s="25" t="n"/>
       <c r="Z9" s="26" t="n"/>
       <c r="AA9" s="28" t="n"/>
       <c r="AB9" s="28" t="n"/>
-      <c r="AC9" s="30" t="n"/>
-      <c r="AD9" s="24" t="n"/>
+      <c r="AC9" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD9" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T05:45:54.886428Z</t>
+        </is>
+      </c>
       <c r="AE9" s="31" t="inlineStr">
         <is>
           <t>Learned LR call at threshold 0.5018; executable ask 0.4800 (aec-wnba-la-chi-2026-07-17).</t>
@@ -3325,7 +3561,7 @@
       </c>
       <c r="AG9" s="24" t="inlineStr">
         <is>
-          <t>not_applicable</t>
+          <t>review_required</t>
         </is>
       </c>
       <c r="AH9" s="24" t="n"/>
@@ -3464,10 +3700,22 @@
       <c r="BU9" s="25" t="n"/>
       <c r="BV9" s="29" t="n"/>
       <c r="BW9" s="24" t="n"/>
-      <c r="BX9" s="30" t="n"/>
-      <c r="BY9" s="27" t="n"/>
-      <c r="BZ9" s="24" t="n"/>
-      <c r="CA9" s="31" t="n"/>
+      <c r="BX9" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="BY9" s="27" t="n">
+        <v>-1</v>
+      </c>
+      <c r="BZ9" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T05:45:54.886428Z</t>
+        </is>
+      </c>
+      <c r="CA9" s="31" t="inlineStr">
+        <is>
+          <t>fixed one-unit hypothetical scoring; no real exposure or execution</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="36" customHeight="1">
       <c r="A10" s="24" t="inlineStr">
@@ -3550,18 +3798,32 @@
       </c>
       <c r="U10" s="24" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V10" s="24" t="n"/>
-      <c r="W10" s="26" t="n"/>
-      <c r="X10" s="26" t="n"/>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V10" s="24" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="W10" s="26" t="n">
+        <v>96</v>
+      </c>
+      <c r="X10" s="26" t="n">
+        <v>83</v>
+      </c>
       <c r="Y10" s="25" t="n"/>
       <c r="Z10" s="26" t="n"/>
       <c r="AA10" s="28" t="n"/>
       <c r="AB10" s="28" t="n"/>
-      <c r="AC10" s="30" t="n"/>
-      <c r="AD10" s="24" t="n"/>
+      <c r="AC10" s="30" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AD10" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T05:45:54.971822Z</t>
+        </is>
+      </c>
       <c r="AE10" s="31" t="inlineStr">
         <is>
           <t>Learned LR call at threshold 0.5018; executable ask 0.6400 (aec-wnba-conn-phx-2026-07-17).</t>
@@ -3574,7 +3836,7 @@
       </c>
       <c r="AG10" s="24" t="inlineStr">
         <is>
-          <t>not_applicable</t>
+          <t>review_required</t>
         </is>
       </c>
       <c r="AH10" s="24" t="n"/>
@@ -3713,10 +3975,22 @@
       <c r="BU10" s="25" t="n"/>
       <c r="BV10" s="29" t="n"/>
       <c r="BW10" s="24" t="n"/>
-      <c r="BX10" s="30" t="n"/>
-      <c r="BY10" s="27" t="n"/>
-      <c r="BZ10" s="24" t="n"/>
-      <c r="CA10" s="31" t="n"/>
+      <c r="BX10" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="BY10" s="27" t="n">
+        <v>-1</v>
+      </c>
+      <c r="BZ10" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T05:45:54.971822Z</t>
+        </is>
+      </c>
+      <c r="CA10" s="31" t="inlineStr">
+        <is>
+          <t>fixed one-unit hypothetical scoring; no real exposure or execution</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="36" customHeight="1">
       <c r="A11" s="24" t="inlineStr">
@@ -4216,6 +4490,255 @@
       <c r="BZ12" s="24" t="n"/>
       <c r="CA12" s="31" t="n"/>
     </row>
+    <row r="13" ht="36" customHeight="1">
+      <c r="A13" s="24" t="inlineStr">
+        <is>
+          <t>4c2ec934da05478b</t>
+        </is>
+      </c>
+      <c r="B13" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T05:45:47.429402Z</t>
+        </is>
+      </c>
+      <c r="C13" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T18:20Z</t>
+        </is>
+      </c>
+      <c r="D13" s="24" t="inlineStr">
+        <is>
+          <t>401816164</t>
+        </is>
+      </c>
+      <c r="E13" s="24" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="F13" s="24" t="inlineStr">
+        <is>
+          <t>Minnesota Twins</t>
+        </is>
+      </c>
+      <c r="G13" s="24" t="inlineStr">
+        <is>
+          <t>Chicago Cubs</t>
+        </is>
+      </c>
+      <c r="H13" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I13" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J13" s="25" t="n"/>
+      <c r="K13" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L13" s="26" t="n">
+        <v>-133</v>
+      </c>
+      <c r="M13" s="27" t="n">
+        <v>1.75188</v>
+      </c>
+      <c r="N13" s="28" t="n">
+        <v>0.570815</v>
+      </c>
+      <c r="O13" s="28" t="n">
+        <v>0.606876</v>
+      </c>
+      <c r="P13" s="28" t="n"/>
+      <c r="Q13" s="28" t="n">
+        <v>0.036061</v>
+      </c>
+      <c r="R13" s="26" t="n">
+        <v>68</v>
+      </c>
+      <c r="S13" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="T13" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="U13" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V13" s="24" t="n"/>
+      <c r="W13" s="26" t="n"/>
+      <c r="X13" s="26" t="n"/>
+      <c r="Y13" s="25" t="n"/>
+      <c r="Z13" s="26" t="n"/>
+      <c r="AA13" s="28" t="n"/>
+      <c r="AB13" s="28" t="n"/>
+      <c r="AC13" s="30" t="n"/>
+      <c r="AD13" s="24" t="n"/>
+      <c r="AE13" s="31" t="inlineStr">
+        <is>
+          <t>Learned LR call at threshold 0.6018; executable ask 0.5700 (aec-mlb-min-chc-2026-07-18).</t>
+        </is>
+      </c>
+      <c r="AF13" s="31" t="inlineStr">
+        <is>
+          <t>Learned model; promotion gate not yet open; zero-unit research until review.</t>
+        </is>
+      </c>
+      <c r="AG13" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH13" s="24" t="n"/>
+      <c r="AI13" s="31" t="n"/>
+      <c r="AJ13" s="31" t="n"/>
+      <c r="AK13" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL13" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM13" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN13" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO13" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_MISSING_UNCERTAINTY</t>
+        </is>
+      </c>
+      <c r="AP13" s="24" t="inlineStr">
+        <is>
+          <t>mlb-min</t>
+        </is>
+      </c>
+      <c r="AQ13" s="24" t="inlineStr">
+        <is>
+          <t>Minnesota Twins</t>
+        </is>
+      </c>
+      <c r="AR13" s="24" t="inlineStr">
+        <is>
+          <t>Minnesota Twins</t>
+        </is>
+      </c>
+      <c r="AS13" s="24" t="inlineStr">
+        <is>
+          <t>mlb-chc</t>
+        </is>
+      </c>
+      <c r="AT13" s="24" t="inlineStr">
+        <is>
+          <t>Chicago Cubs</t>
+        </is>
+      </c>
+      <c r="AU13" s="24" t="inlineStr">
+        <is>
+          <t>Chicago Cubs</t>
+        </is>
+      </c>
+      <c r="AV13" s="24" t="n"/>
+      <c r="AW13" s="24" t="n"/>
+      <c r="AX13" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY13" s="24" t="n"/>
+      <c r="AZ13" s="24" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="BA13" s="24" t="inlineStr">
+        <is>
+          <t>a454281ab207d2924d585d6b967363fb8e88af45132e3e9d354e4351fb5c237f</t>
+        </is>
+      </c>
+      <c r="BB13" s="24" t="inlineStr">
+        <is>
+          <t>learned_lr</t>
+        </is>
+      </c>
+      <c r="BC13" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="BD13" s="24" t="inlineStr">
+        <is>
+          <t>a454281ab207d2924d585d6b967363fb8e88af45132e3e9d354e4351fb5c237f</t>
+        </is>
+      </c>
+      <c r="BE13" s="24" t="inlineStr">
+        <is>
+          <t>3acab0aa8ac04a91</t>
+        </is>
+      </c>
+      <c r="BF13" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG13" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="BH13" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T05:44:27.731285Z</t>
+        </is>
+      </c>
+      <c r="BI13" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ13" s="25" t="n"/>
+      <c r="BK13" s="26" t="n">
+        <v>-133</v>
+      </c>
+      <c r="BL13" s="27" t="n">
+        <v>1.75188</v>
+      </c>
+      <c r="BM13" s="28" t="n">
+        <v>0.570815</v>
+      </c>
+      <c r="BN13" s="28" t="n">
+        <v>0.567164</v>
+      </c>
+      <c r="BO13" s="28" t="n"/>
+      <c r="BP13" s="25" t="n"/>
+      <c r="BQ13" s="27" t="n"/>
+      <c r="BR13" s="28" t="n"/>
+      <c r="BS13" s="28" t="n"/>
+      <c r="BT13" s="28" t="n"/>
+      <c r="BU13" s="25" t="n"/>
+      <c r="BV13" s="29" t="n"/>
+      <c r="BW13" s="24" t="n"/>
+      <c r="BX13" s="30" t="n"/>
+      <c r="BY13" s="27" t="n"/>
+      <c r="BZ13" s="24" t="n"/>
+      <c r="CA13" s="31" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
ledger: clear all WNBA lines, starting fresh with new model
Removed 6 WNBA picks from picks.xlsx and 28 WNBA events from audit log.
All were RESEARCH_OBSERVATION / NO_CALL_MISSING_UNCERTAINTY from old model.
</commit_message>
<xml_diff>
--- a/data/picks.xlsx
+++ b/data/picks.xlsx
@@ -21,10 +21,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="0.0###"/>
-    <numFmt numFmtId="165" formatCode="0.000000"/>
-    <numFmt numFmtId="166" formatCode="0.0000"/>
-    <numFmt numFmtId="167" formatCode="0.0%"/>
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="0.0000"/>
+    <numFmt numFmtId="166" formatCode="0.0###"/>
+    <numFmt numFmtId="167" formatCode="0.000000"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -136,7 +136,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -150,10 +150,10 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -169,10 +169,10 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="167" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="10" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -184,10 +184,10 @@
     <xf numFmtId="0" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="167" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="10" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -202,26 +202,53 @@
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="10" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="10" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -785,11 +812,11 @@
         <f>COUNTIFS('Picks'!$BX$2:$BX$13,"&gt;0",'Picks'!$V$2:$V$13,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$13,"&gt;0",'Picks'!$V$2:$V$13,"loss")</f>
         <v/>
       </c>
-      <c r="E7" s="7">
+      <c r="E7" s="32">
         <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$13,"&gt;0",'Picks'!$V$2:$V$13,"win")/(COUNTIFS('Picks'!$BX$2:$BX$13,"&gt;0",'Picks'!$V$2:$V$13,"win")+COUNTIFS('Picks'!$BX$2:$BX$13,"&gt;0",'Picks'!$V$2:$V$13,"loss")),0)</f>
         <v/>
       </c>
-      <c r="G7" s="7">
+      <c r="G7" s="32">
         <f>IFERROR(SUM('Picks'!$BY$2:$BY$13)/SUM('Picks'!$BX$2:$BX$13),0)</f>
         <v/>
       </c>
@@ -817,7 +844,7 @@
       </c>
     </row>
     <row r="10" ht="28" customHeight="1">
-      <c r="A10" s="8">
+      <c r="A10" s="33">
         <f>SUM('Picks'!$BY$2:$BY$13)</f>
         <v/>
       </c>
@@ -829,7 +856,7 @@
         <f>COUNTIFS('Picks'!$AM$2:$AM$13,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$13,"settled")</f>
         <v/>
       </c>
-      <c r="G10" s="8">
+      <c r="G10" s="33">
         <f>SUMIFS('Picks'!$AC$2:$AC$13,'Picks'!$AM$2:$AM$13,"QUALIFIED_SHADOW_CALL")</f>
         <v/>
       </c>
@@ -896,11 +923,11 @@
         <f>COUNTIFS('Picks'!$H$2:$H$13,$A14,'Picks'!$U$2:$U$13,"settled",'Picks'!$V$2:$V$13,"loss")</f>
         <v/>
       </c>
-      <c r="E14" s="14">
+      <c r="E14" s="34">
         <f>IFERROR(C14/(C14+D14),0)</f>
         <v/>
       </c>
-      <c r="F14" s="15">
+      <c r="F14" s="35">
         <f>SUMIFS('Picks'!$BY$2:$BY$13,'Picks'!$H$2:$H$13,$A14)</f>
         <v/>
       </c>
@@ -927,11 +954,11 @@
         <f>COUNTIFS('Picks'!$H$2:$H$13,$A15,'Picks'!$U$2:$U$13,"settled",'Picks'!$V$2:$V$13,"loss")</f>
         <v/>
       </c>
-      <c r="E15" s="19">
+      <c r="E15" s="36">
         <f>IFERROR(C15/(C15+D15),0)</f>
         <v/>
       </c>
-      <c r="F15" s="20">
+      <c r="F15" s="37">
         <f>SUMIFS('Picks'!$BY$2:$BY$13,'Picks'!$H$2:$H$13,$A15)</f>
         <v/>
       </c>
@@ -958,11 +985,11 @@
         <f>COUNTIFS('Picks'!$H$2:$H$13,$A16,'Picks'!$U$2:$U$13,"settled",'Picks'!$V$2:$V$13,"loss")</f>
         <v/>
       </c>
-      <c r="E16" s="14">
+      <c r="E16" s="34">
         <f>IFERROR(C16/(C16+D16),0)</f>
         <v/>
       </c>
-      <c r="F16" s="15">
+      <c r="F16" s="35">
         <f>SUMIFS('Picks'!$BY$2:$BY$13,'Picks'!$H$2:$H$13,$A16)</f>
         <v/>
       </c>
@@ -996,7 +1023,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:CA13"/>
+  <dimension ref="A1:CA7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1523,7 +1550,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J2" s="25" t="n"/>
+      <c r="J2" s="38" t="n"/>
       <c r="K2" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -1532,7 +1559,7 @@
       <c r="L2" s="26" t="n">
         <v>-141</v>
       </c>
-      <c r="M2" s="27" t="n">
+      <c r="M2" s="39" t="n">
         <v>1.70922</v>
       </c>
       <c r="N2" s="28" t="n">
@@ -1572,7 +1599,7 @@
       <c r="X2" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="Y2" s="25" t="n"/>
+      <c r="Y2" s="38" t="n"/>
       <c r="Z2" s="26" t="n">
         <v>-147</v>
       </c>
@@ -1582,7 +1609,7 @@
       <c r="AB2" s="28" t="n">
         <v>0.009938000000000001</v>
       </c>
-      <c r="AC2" s="30" t="n">
+      <c r="AC2" s="40" t="n">
         <v>0</v>
       </c>
       <c r="AD2" s="24" t="inlineStr">
@@ -1719,11 +1746,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ2" s="25" t="n"/>
+      <c r="BJ2" s="38" t="n"/>
       <c r="BK2" s="26" t="n">
         <v>-141</v>
       </c>
-      <c r="BL2" s="27" t="n">
+      <c r="BL2" s="39" t="n">
         <v>1.70922</v>
       </c>
       <c r="BM2" s="28" t="n">
@@ -1733,8 +1760,8 @@
         <v>0.58209</v>
       </c>
       <c r="BO2" s="28" t="n"/>
-      <c r="BP2" s="25" t="n"/>
-      <c r="BQ2" s="27" t="n">
+      <c r="BP2" s="38" t="n"/>
+      <c r="BQ2" s="39" t="n">
         <v>1.680272</v>
       </c>
       <c r="BR2" s="28" t="n">
@@ -1742,13 +1769,13 @@
       </c>
       <c r="BS2" s="28" t="n"/>
       <c r="BT2" s="28" t="n"/>
-      <c r="BU2" s="25" t="n"/>
+      <c r="BU2" s="38" t="n"/>
       <c r="BV2" s="29" t="n"/>
       <c r="BW2" s="24" t="n"/>
-      <c r="BX2" s="30" t="n">
+      <c r="BX2" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="BY2" s="27" t="n">
+      <c r="BY2" s="39" t="n">
         <v>0.70922</v>
       </c>
       <c r="BZ2" s="24" t="inlineStr">
@@ -1808,7 +1835,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J3" s="25" t="n"/>
+      <c r="J3" s="38" t="n"/>
       <c r="K3" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -1817,7 +1844,7 @@
       <c r="L3" s="26" t="n">
         <v>-130</v>
       </c>
-      <c r="M3" s="27" t="n">
+      <c r="M3" s="39" t="n">
         <v>1.769231</v>
       </c>
       <c r="N3" s="28" t="n">
@@ -1857,7 +1884,7 @@
       <c r="X3" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="Y3" s="25" t="n"/>
+      <c r="Y3" s="38" t="n"/>
       <c r="Z3" s="26" t="n">
         <v>-133</v>
       </c>
@@ -1867,7 +1894,7 @@
       <c r="AB3" s="28" t="n">
         <v>0.004783</v>
       </c>
-      <c r="AC3" s="30" t="n">
+      <c r="AC3" s="40" t="n">
         <v>0</v>
       </c>
       <c r="AD3" s="24" t="inlineStr">
@@ -2004,11 +2031,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ3" s="25" t="n"/>
+      <c r="BJ3" s="38" t="n"/>
       <c r="BK3" s="26" t="n">
         <v>-130</v>
       </c>
-      <c r="BL3" s="27" t="n">
+      <c r="BL3" s="39" t="n">
         <v>1.769231</v>
       </c>
       <c r="BM3" s="28" t="n">
@@ -2018,8 +2045,8 @@
         <v>0.562189</v>
       </c>
       <c r="BO3" s="28" t="n"/>
-      <c r="BP3" s="25" t="n"/>
-      <c r="BQ3" s="27" t="n">
+      <c r="BP3" s="38" t="n"/>
+      <c r="BQ3" s="39" t="n">
         <v>1.75188</v>
       </c>
       <c r="BR3" s="28" t="n">
@@ -2027,13 +2054,13 @@
       </c>
       <c r="BS3" s="28" t="n"/>
       <c r="BT3" s="28" t="n"/>
-      <c r="BU3" s="25" t="n"/>
+      <c r="BU3" s="38" t="n"/>
       <c r="BV3" s="29" t="n"/>
       <c r="BW3" s="24" t="n"/>
-      <c r="BX3" s="30" t="n">
+      <c r="BX3" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="BY3" s="27" t="n">
+      <c r="BY3" s="39" t="n">
         <v>-1</v>
       </c>
       <c r="BZ3" s="24" t="inlineStr">
@@ -2050,37 +2077,37 @@
     <row r="4" ht="36" customHeight="1">
       <c r="A4" s="24" t="inlineStr">
         <is>
-          <t>1784b306a2764ca0</t>
+          <t>d0e98df55d684f7a</t>
         </is>
       </c>
       <c r="B4" s="24" t="inlineStr">
         <is>
-          <t>2026-07-17T10:47:01.653330Z</t>
+          <t>2026-07-17T14:02:14.862720Z</t>
         </is>
       </c>
       <c r="C4" s="24" t="inlineStr">
         <is>
-          <t>2026-07-17T23:30Z</t>
+          <t>2026-07-17T23:40Z</t>
         </is>
       </c>
       <c r="D4" s="24" t="inlineStr">
         <is>
-          <t>401857073</t>
+          <t>401816148</t>
         </is>
       </c>
       <c r="E4" s="24" t="inlineStr">
         <is>
-          <t>WNBA</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="F4" s="24" t="inlineStr">
         <is>
-          <t>Seattle Storm</t>
+          <t>Miami Marlins</t>
         </is>
       </c>
       <c r="G4" s="24" t="inlineStr">
         <is>
-          <t>Indiana Fever</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="H4" s="24" t="inlineStr">
@@ -2093,37 +2120,37 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J4" s="25" t="n"/>
+      <c r="J4" s="38" t="n"/>
       <c r="K4" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
         </is>
       </c>
       <c r="L4" s="26" t="n">
-        <v>-355</v>
-      </c>
-      <c r="M4" s="27" t="n">
-        <v>1.28169</v>
+        <v>-141</v>
+      </c>
+      <c r="M4" s="39" t="n">
+        <v>1.70922</v>
       </c>
       <c r="N4" s="28" t="n">
-        <v>0.78022</v>
+        <v>0.585062</v>
       </c>
       <c r="O4" s="28" t="n">
-        <v>0.6531090000000001</v>
+        <v>0.605633</v>
       </c>
       <c r="P4" s="28" t="n"/>
       <c r="Q4" s="28" t="n">
-        <v>-0.127111</v>
+        <v>0.020571</v>
       </c>
       <c r="R4" s="26" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="S4" s="29" t="n">
         <v>0</v>
       </c>
       <c r="T4" s="24" t="inlineStr">
         <is>
-          <t>wnba-elo-trend-lr-v2</t>
+          <t>mlb-elo-trend-lr-v3</t>
         </is>
       </c>
       <c r="U4" s="24" t="inlineStr">
@@ -2137,26 +2164,32 @@
         </is>
       </c>
       <c r="W4" s="26" t="n">
-        <v>107</v>
+        <v>1</v>
       </c>
       <c r="X4" s="26" t="n">
-        <v>110</v>
-      </c>
-      <c r="Y4" s="25" t="n"/>
-      <c r="Z4" s="26" t="n"/>
-      <c r="AA4" s="28" t="n"/>
-      <c r="AB4" s="28" t="n"/>
-      <c r="AC4" s="30" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y4" s="38" t="n"/>
+      <c r="Z4" s="26" t="n">
+        <v>-147</v>
+      </c>
+      <c r="AA4" s="28" t="n">
+        <v>0.595</v>
+      </c>
+      <c r="AB4" s="28" t="n">
+        <v>0.009938000000000001</v>
+      </c>
+      <c r="AC4" s="40" t="n">
         <v>0</v>
       </c>
       <c r="AD4" s="24" t="inlineStr">
         <is>
-          <t>2026-07-18T05:45:54.458400Z</t>
+          <t>2026-07-18T05:45:54.715857Z</t>
         </is>
       </c>
       <c r="AE4" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.5018; executable ask 0.7800 (aec-wnba-sea-ind-2026-07-17).</t>
+          <t>Learned LR call at threshold 0.6018; executable ask 0.5850 (aec-mlb-mia-mil-2026-07-17).</t>
         </is>
       </c>
       <c r="AF4" s="31" t="inlineStr">
@@ -2197,32 +2230,32 @@
       </c>
       <c r="AP4" s="24" t="inlineStr">
         <is>
-          <t>wnba-sea</t>
+          <t>mlb-mia</t>
         </is>
       </c>
       <c r="AQ4" s="24" t="inlineStr">
         <is>
-          <t>Seattle Storm</t>
+          <t>Miami Marlins</t>
         </is>
       </c>
       <c r="AR4" s="24" t="inlineStr">
         <is>
-          <t>Seattle Storm</t>
+          <t>Miami Marlins</t>
         </is>
       </c>
       <c r="AS4" s="24" t="inlineStr">
         <is>
-          <t>wnba-ind</t>
+          <t>mlb-mil</t>
         </is>
       </c>
       <c r="AT4" s="24" t="inlineStr">
         <is>
-          <t>Indiana Fever</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="AU4" s="24" t="inlineStr">
         <is>
-          <t>Indiana Fever</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="AV4" s="24" t="n"/>
@@ -2240,7 +2273,7 @@
       </c>
       <c r="BA4" s="24" t="inlineStr">
         <is>
-          <t>593925b19cd0d6a88880d7d2e868f8b3cffef14f1697019de3a8a7e28e173bc7</t>
+          <t>a454281ab207d2924d585d6b967363fb8e88af45132e3e9d354e4351fb5c237f</t>
         </is>
       </c>
       <c r="BB4" s="24" t="inlineStr">
@@ -2250,17 +2283,17 @@
       </c>
       <c r="BC4" s="24" t="inlineStr">
         <is>
-          <t>wnba-elo-trend-lr-v2</t>
+          <t>mlb-elo-trend-lr-v3</t>
         </is>
       </c>
       <c r="BD4" s="24" t="inlineStr">
         <is>
-          <t>593925b19cd0d6a88880d7d2e868f8b3cffef14f1697019de3a8a7e28e173bc7</t>
+          <t>a454281ab207d2924d585d6b967363fb8e88af45132e3e9d354e4351fb5c237f</t>
         </is>
       </c>
       <c r="BE4" s="24" t="inlineStr">
         <is>
-          <t>15f518082bd1133e</t>
+          <t>27ad4a1da893e4b8</t>
         </is>
       </c>
       <c r="BF4" s="24" t="inlineStr">
@@ -2270,12 +2303,12 @@
       </c>
       <c r="BG4" s="24" t="inlineStr">
         <is>
-          <t>wnba-elo-trend-lr-v2</t>
+          <t>mlb-elo-trend-lr-v3</t>
         </is>
       </c>
       <c r="BH4" s="24" t="inlineStr">
         <is>
-          <t>2026-07-17T10:46:53.056520Z</t>
+          <t>2026-07-17T14:01:56.626918Z</t>
         </is>
       </c>
       <c r="BI4" s="24" t="inlineStr">
@@ -2283,79 +2316,83 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ4" s="25" t="n"/>
+      <c r="BJ4" s="38" t="n"/>
       <c r="BK4" s="26" t="n">
-        <v>-355</v>
-      </c>
-      <c r="BL4" s="27" t="n">
-        <v>1.28169</v>
+        <v>-141</v>
+      </c>
+      <c r="BL4" s="39" t="n">
+        <v>1.70922</v>
       </c>
       <c r="BM4" s="28" t="n">
-        <v>0.78022</v>
+        <v>0.585062</v>
       </c>
       <c r="BN4" s="28" t="n">
-        <v>0.772277</v>
+        <v>0.58209</v>
       </c>
       <c r="BO4" s="28" t="n"/>
-      <c r="BP4" s="25" t="n"/>
-      <c r="BQ4" s="27" t="n"/>
-      <c r="BR4" s="28" t="n"/>
+      <c r="BP4" s="38" t="n"/>
+      <c r="BQ4" s="39" t="n">
+        <v>1.680272</v>
+      </c>
+      <c r="BR4" s="28" t="n">
+        <v>0.595</v>
+      </c>
       <c r="BS4" s="28" t="n"/>
       <c r="BT4" s="28" t="n"/>
-      <c r="BU4" s="25" t="n"/>
+      <c r="BU4" s="38" t="n"/>
       <c r="BV4" s="29" t="n"/>
       <c r="BW4" s="24" t="n"/>
-      <c r="BX4" s="30" t="n">
-        <v>1</v>
-      </c>
-      <c r="BY4" s="27" t="n">
-        <v>0.28169</v>
+      <c r="BX4" s="40" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="BY4" s="39" t="n">
+        <v>1.06383</v>
       </c>
       <c r="BZ4" s="24" t="inlineStr">
         <is>
-          <t>2026-07-18T05:45:54.458400Z</t>
+          <t>2026-07-18T06:03:40.307635Z</t>
         </is>
       </c>
       <c r="CA4" s="31" t="inlineStr">
         <is>
-          <t>fixed one-unit hypothetical scoring; no real exposure or execution</t>
+          <t>decision-time model-sized hypothetical scoring; migrated 2026-07-18; no real exposure</t>
         </is>
       </c>
     </row>
     <row r="5" ht="36" customHeight="1">
       <c r="A5" s="24" t="inlineStr">
         <is>
-          <t>c6927110c2754085</t>
+          <t>3b98081a1ff04c62</t>
         </is>
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>2026-07-17T10:47:01.653330Z</t>
+          <t>2026-07-17T14:02:14.862720Z</t>
         </is>
       </c>
       <c r="C5" s="24" t="inlineStr">
         <is>
-          <t>2026-07-17T23:30Z</t>
+          <t>2026-07-18T00:05Z</t>
         </is>
       </c>
       <c r="D5" s="24" t="inlineStr">
         <is>
-          <t>401857075</t>
+          <t>401816149</t>
         </is>
       </c>
       <c r="E5" s="24" t="inlineStr">
         <is>
-          <t>WNBA</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="F5" s="24" t="inlineStr">
         <is>
-          <t>Los Angeles Sparks</t>
+          <t>Minnesota Twins</t>
         </is>
       </c>
       <c r="G5" s="24" t="inlineStr">
         <is>
-          <t>Chicago Sky</t>
+          <t>Chicago Cubs</t>
         </is>
       </c>
       <c r="H5" s="24" t="inlineStr">
@@ -2365,40 +2402,40 @@
       </c>
       <c r="I5" s="24" t="inlineStr">
         <is>
-          <t>away</t>
-        </is>
-      </c>
-      <c r="J5" s="25" t="n"/>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J5" s="38" t="n"/>
       <c r="K5" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
         </is>
       </c>
       <c r="L5" s="26" t="n">
-        <v>104</v>
-      </c>
-      <c r="M5" s="27" t="n">
-        <v>2.04</v>
+        <v>-130</v>
+      </c>
+      <c r="M5" s="39" t="n">
+        <v>1.769231</v>
       </c>
       <c r="N5" s="28" t="n">
-        <v>0.490196</v>
+        <v>0.565217</v>
       </c>
       <c r="O5" s="28" t="n">
-        <v>0.580113</v>
+        <v>0.606876</v>
       </c>
       <c r="P5" s="28" t="n"/>
       <c r="Q5" s="28" t="n">
-        <v>0.089917</v>
+        <v>0.041659</v>
       </c>
       <c r="R5" s="26" t="n">
-        <v>95</v>
+        <v>71</v>
       </c>
       <c r="S5" s="29" t="n">
         <v>0</v>
       </c>
       <c r="T5" s="24" t="inlineStr">
         <is>
-          <t>wnba-elo-trend-lr-v2</t>
+          <t>mlb-elo-trend-lr-v3</t>
         </is>
       </c>
       <c r="U5" s="24" t="inlineStr">
@@ -2412,26 +2449,32 @@
         </is>
       </c>
       <c r="W5" s="26" t="n">
-        <v>82</v>
+        <v>5</v>
       </c>
       <c r="X5" s="26" t="n">
-        <v>96</v>
-      </c>
-      <c r="Y5" s="25" t="n"/>
-      <c r="Z5" s="26" t="n"/>
-      <c r="AA5" s="28" t="n"/>
-      <c r="AB5" s="28" t="n"/>
-      <c r="AC5" s="30" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y5" s="38" t="n"/>
+      <c r="Z5" s="26" t="n">
+        <v>-133</v>
+      </c>
+      <c r="AA5" s="28" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="AB5" s="28" t="n">
+        <v>0.004783</v>
+      </c>
+      <c r="AC5" s="40" t="n">
         <v>0</v>
       </c>
       <c r="AD5" s="24" t="inlineStr">
         <is>
-          <t>2026-07-18T05:45:54.545671Z</t>
+          <t>2026-07-18T05:45:54.800172Z</t>
         </is>
       </c>
       <c r="AE5" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.5018; executable ask 0.4900 (aec-wnba-la-chi-2026-07-17).</t>
+          <t>Learned LR call at threshold 0.6018; executable ask 0.5650 (aec-mlb-min-chc-2026-07-17).</t>
         </is>
       </c>
       <c r="AF5" s="31" t="inlineStr">
@@ -2472,32 +2515,32 @@
       </c>
       <c r="AP5" s="24" t="inlineStr">
         <is>
-          <t>wnba-las</t>
+          <t>mlb-min</t>
         </is>
       </c>
       <c r="AQ5" s="24" t="inlineStr">
         <is>
-          <t>Los Angeles Sparks</t>
+          <t>Minnesota Twins</t>
         </is>
       </c>
       <c r="AR5" s="24" t="inlineStr">
         <is>
-          <t>Los Angeles Sparks</t>
+          <t>Minnesota Twins</t>
         </is>
       </c>
       <c r="AS5" s="24" t="inlineStr">
         <is>
-          <t>wnba-chi</t>
+          <t>mlb-chc</t>
         </is>
       </c>
       <c r="AT5" s="24" t="inlineStr">
         <is>
-          <t>Chicago Sky</t>
+          <t>Chicago Cubs</t>
         </is>
       </c>
       <c r="AU5" s="24" t="inlineStr">
         <is>
-          <t>Chicago Sky</t>
+          <t>Chicago Cubs</t>
         </is>
       </c>
       <c r="AV5" s="24" t="n"/>
@@ -2515,7 +2558,7 @@
       </c>
       <c r="BA5" s="24" t="inlineStr">
         <is>
-          <t>593925b19cd0d6a88880d7d2e868f8b3cffef14f1697019de3a8a7e28e173bc7</t>
+          <t>a454281ab207d2924d585d6b967363fb8e88af45132e3e9d354e4351fb5c237f</t>
         </is>
       </c>
       <c r="BB5" s="24" t="inlineStr">
@@ -2525,17 +2568,17 @@
       </c>
       <c r="BC5" s="24" t="inlineStr">
         <is>
-          <t>wnba-elo-trend-lr-v2</t>
+          <t>mlb-elo-trend-lr-v3</t>
         </is>
       </c>
       <c r="BD5" s="24" t="inlineStr">
         <is>
-          <t>593925b19cd0d6a88880d7d2e868f8b3cffef14f1697019de3a8a7e28e173bc7</t>
+          <t>a454281ab207d2924d585d6b967363fb8e88af45132e3e9d354e4351fb5c237f</t>
         </is>
       </c>
       <c r="BE5" s="24" t="inlineStr">
         <is>
-          <t>8c7d8b8b613f1c27</t>
+          <t>8438bc3f26be5eae</t>
         </is>
       </c>
       <c r="BF5" s="24" t="inlineStr">
@@ -2545,12 +2588,12 @@
       </c>
       <c r="BG5" s="24" t="inlineStr">
         <is>
-          <t>wnba-elo-trend-lr-v2</t>
+          <t>mlb-elo-trend-lr-v3</t>
         </is>
       </c>
       <c r="BH5" s="24" t="inlineStr">
         <is>
-          <t>2026-07-17T10:46:55.117340Z</t>
+          <t>2026-07-17T14:01:57.663980Z</t>
         </is>
       </c>
       <c r="BI5" s="24" t="inlineStr">
@@ -2558,79 +2601,83 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ5" s="25" t="n"/>
+      <c r="BJ5" s="38" t="n"/>
       <c r="BK5" s="26" t="n">
-        <v>104</v>
-      </c>
-      <c r="BL5" s="27" t="n">
-        <v>2.04</v>
+        <v>-130</v>
+      </c>
+      <c r="BL5" s="39" t="n">
+        <v>1.769231</v>
       </c>
       <c r="BM5" s="28" t="n">
-        <v>0.490196</v>
+        <v>0.565217</v>
       </c>
       <c r="BN5" s="28" t="n">
-        <v>0.485149</v>
+        <v>0.562189</v>
       </c>
       <c r="BO5" s="28" t="n"/>
-      <c r="BP5" s="25" t="n"/>
-      <c r="BQ5" s="27" t="n"/>
-      <c r="BR5" s="28" t="n"/>
+      <c r="BP5" s="38" t="n"/>
+      <c r="BQ5" s="39" t="n">
+        <v>1.75188</v>
+      </c>
+      <c r="BR5" s="28" t="n">
+        <v>0.57</v>
+      </c>
       <c r="BS5" s="28" t="n"/>
       <c r="BT5" s="28" t="n"/>
-      <c r="BU5" s="25" t="n"/>
+      <c r="BU5" s="38" t="n"/>
       <c r="BV5" s="29" t="n"/>
       <c r="BW5" s="24" t="n"/>
-      <c r="BX5" s="30" t="n">
-        <v>1</v>
-      </c>
-      <c r="BY5" s="27" t="n">
-        <v>-1</v>
+      <c r="BX5" s="40" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="BY5" s="39" t="n">
+        <v>-1.5</v>
       </c>
       <c r="BZ5" s="24" t="inlineStr">
         <is>
-          <t>2026-07-18T05:45:54.545671Z</t>
+          <t>2026-07-18T06:03:40.307635Z</t>
         </is>
       </c>
       <c r="CA5" s="31" t="inlineStr">
         <is>
-          <t>fixed one-unit hypothetical scoring; no real exposure or execution</t>
+          <t>decision-time model-sized hypothetical scoring; migrated 2026-07-18; no real exposure</t>
         </is>
       </c>
     </row>
     <row r="6" ht="36" customHeight="1">
       <c r="A6" s="24" t="inlineStr">
         <is>
-          <t>ec5e7cc40c1a4c2b</t>
+          <t>93a3540bf0dd49bb</t>
         </is>
       </c>
       <c r="B6" s="24" t="inlineStr">
         <is>
-          <t>2026-07-17T10:47:01.653330Z</t>
+          <t>2026-07-17T16:21:24.725309Z</t>
         </is>
       </c>
       <c r="C6" s="24" t="inlineStr">
         <is>
-          <t>2026-07-18T02:00Z</t>
+          <t>2026-07-18T20:10Z</t>
         </is>
       </c>
       <c r="D6" s="24" t="inlineStr">
         <is>
-          <t>401857076</t>
+          <t>401816163</t>
         </is>
       </c>
       <c r="E6" s="24" t="inlineStr">
         <is>
-          <t>WNBA</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="F6" s="24" t="inlineStr">
         <is>
-          <t>Connecticut Sun</t>
+          <t>Miami Marlins</t>
         </is>
       </c>
       <c r="G6" s="24" t="inlineStr">
         <is>
-          <t>Phoenix Mercury</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="H6" s="24" t="inlineStr">
@@ -2643,70 +2690,56 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J6" s="25" t="n"/>
+      <c r="J6" s="38" t="n"/>
       <c r="K6" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
         </is>
       </c>
       <c r="L6" s="26" t="n">
-        <v>-178</v>
-      </c>
-      <c r="M6" s="27" t="n">
-        <v>1.561798</v>
+        <v>-130</v>
+      </c>
+      <c r="M6" s="39" t="n">
+        <v>1.769231</v>
       </c>
       <c r="N6" s="28" t="n">
-        <v>0.640288</v>
+        <v>0.565217</v>
       </c>
       <c r="O6" s="28" t="n">
-        <v>0.672243</v>
+        <v>0.605633</v>
       </c>
       <c r="P6" s="28" t="n"/>
       <c r="Q6" s="28" t="n">
-        <v>0.031955</v>
+        <v>0.040416</v>
       </c>
       <c r="R6" s="26" t="n">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="S6" s="29" t="n">
         <v>0</v>
       </c>
       <c r="T6" s="24" t="inlineStr">
         <is>
-          <t>wnba-elo-trend-lr-v2</t>
+          <t>mlb-elo-trend-lr-v3</t>
         </is>
       </c>
       <c r="U6" s="24" t="inlineStr">
         <is>
-          <t>settled</t>
-        </is>
-      </c>
-      <c r="V6" s="24" t="inlineStr">
-        <is>
-          <t>loss</t>
-        </is>
-      </c>
-      <c r="W6" s="26" t="n">
-        <v>96</v>
-      </c>
-      <c r="X6" s="26" t="n">
-        <v>83</v>
-      </c>
-      <c r="Y6" s="25" t="n"/>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V6" s="24" t="n"/>
+      <c r="W6" s="26" t="n"/>
+      <c r="X6" s="26" t="n"/>
+      <c r="Y6" s="38" t="n"/>
       <c r="Z6" s="26" t="n"/>
       <c r="AA6" s="28" t="n"/>
       <c r="AB6" s="28" t="n"/>
-      <c r="AC6" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD6" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-18T05:45:54.629639Z</t>
-        </is>
-      </c>
+      <c r="AC6" s="40" t="n"/>
+      <c r="AD6" s="24" t="n"/>
       <c r="AE6" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.5018; executable ask 0.6400 (aec-wnba-conn-phx-2026-07-17).</t>
+          <t>Learned LR call at threshold 0.6018; executable ask 0.5650 (aec-mlb-mia-mil-2026-07-18).</t>
         </is>
       </c>
       <c r="AF6" s="31" t="inlineStr">
@@ -2716,7 +2749,7 @@
       </c>
       <c r="AG6" s="24" t="inlineStr">
         <is>
-          <t>review_required</t>
+          <t>not_applicable</t>
         </is>
       </c>
       <c r="AH6" s="24" t="n"/>
@@ -2747,32 +2780,32 @@
       </c>
       <c r="AP6" s="24" t="inlineStr">
         <is>
-          <t>wnba-con</t>
+          <t>mlb-mia</t>
         </is>
       </c>
       <c r="AQ6" s="24" t="inlineStr">
         <is>
-          <t>Connecticut Sun</t>
+          <t>Miami Marlins</t>
         </is>
       </c>
       <c r="AR6" s="24" t="inlineStr">
         <is>
-          <t>Connecticut Sun</t>
+          <t>Miami Marlins</t>
         </is>
       </c>
       <c r="AS6" s="24" t="inlineStr">
         <is>
-          <t>wnba-phx</t>
+          <t>mlb-mil</t>
         </is>
       </c>
       <c r="AT6" s="24" t="inlineStr">
         <is>
-          <t>Phoenix Mercury</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="AU6" s="24" t="inlineStr">
         <is>
-          <t>Phoenix Mercury</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="AV6" s="24" t="n"/>
@@ -2790,7 +2823,7 @@
       </c>
       <c r="BA6" s="24" t="inlineStr">
         <is>
-          <t>593925b19cd0d6a88880d7d2e868f8b3cffef14f1697019de3a8a7e28e173bc7</t>
+          <t>a454281ab207d2924d585d6b967363fb8e88af45132e3e9d354e4351fb5c237f</t>
         </is>
       </c>
       <c r="BB6" s="24" t="inlineStr">
@@ -2800,17 +2833,17 @@
       </c>
       <c r="BC6" s="24" t="inlineStr">
         <is>
-          <t>wnba-elo-trend-lr-v2</t>
+          <t>mlb-elo-trend-lr-v3</t>
         </is>
       </c>
       <c r="BD6" s="24" t="inlineStr">
         <is>
-          <t>593925b19cd0d6a88880d7d2e868f8b3cffef14f1697019de3a8a7e28e173bc7</t>
+          <t>a454281ab207d2924d585d6b967363fb8e88af45132e3e9d354e4351fb5c237f</t>
         </is>
       </c>
       <c r="BE6" s="24" t="inlineStr">
         <is>
-          <t>5b26e70fb7a6c509</t>
+          <t>c7348ce29d666909</t>
         </is>
       </c>
       <c r="BF6" s="24" t="inlineStr">
@@ -2820,12 +2853,12 @@
       </c>
       <c r="BG6" s="24" t="inlineStr">
         <is>
-          <t>wnba-elo-trend-lr-v2</t>
+          <t>mlb-elo-trend-lr-v3</t>
         </is>
       </c>
       <c r="BH6" s="24" t="inlineStr">
         <is>
-          <t>2026-07-17T10:46:56.693440Z</t>
+          <t>2026-07-17T16:21:07.161405Z</t>
         </is>
       </c>
       <c r="BI6" s="24" t="inlineStr">
@@ -2833,64 +2866,52 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ6" s="25" t="n"/>
+      <c r="BJ6" s="38" t="n"/>
       <c r="BK6" s="26" t="n">
-        <v>-178</v>
-      </c>
-      <c r="BL6" s="27" t="n">
-        <v>1.561798</v>
+        <v>-130</v>
+      </c>
+      <c r="BL6" s="39" t="n">
+        <v>1.769231</v>
       </c>
       <c r="BM6" s="28" t="n">
-        <v>0.640288</v>
+        <v>0.565217</v>
       </c>
       <c r="BN6" s="28" t="n">
-        <v>0.633663</v>
+        <v>0.562189</v>
       </c>
       <c r="BO6" s="28" t="n"/>
-      <c r="BP6" s="25" t="n"/>
-      <c r="BQ6" s="27" t="n"/>
+      <c r="BP6" s="38" t="n"/>
+      <c r="BQ6" s="39" t="n"/>
       <c r="BR6" s="28" t="n"/>
       <c r="BS6" s="28" t="n"/>
       <c r="BT6" s="28" t="n"/>
-      <c r="BU6" s="25" t="n"/>
+      <c r="BU6" s="38" t="n"/>
       <c r="BV6" s="29" t="n"/>
       <c r="BW6" s="24" t="n"/>
-      <c r="BX6" s="30" t="n">
-        <v>1</v>
-      </c>
-      <c r="BY6" s="27" t="n">
-        <v>-1</v>
-      </c>
-      <c r="BZ6" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-18T05:45:54.629639Z</t>
-        </is>
-      </c>
-      <c r="CA6" s="31" t="inlineStr">
-        <is>
-          <t>fixed one-unit hypothetical scoring; no real exposure or execution</t>
-        </is>
-      </c>
+      <c r="BX6" s="40" t="n"/>
+      <c r="BY6" s="39" t="n"/>
+      <c r="BZ6" s="24" t="n"/>
+      <c r="CA6" s="31" t="n"/>
     </row>
     <row r="7" ht="36" customHeight="1">
       <c r="A7" s="24" t="inlineStr">
         <is>
-          <t>d0e98df55d684f7a</t>
+          <t>4c2ec934da05478b</t>
         </is>
       </c>
       <c r="B7" s="24" t="inlineStr">
         <is>
-          <t>2026-07-17T14:02:14.862720Z</t>
+          <t>2026-07-18T05:45:47.429402Z</t>
         </is>
       </c>
       <c r="C7" s="24" t="inlineStr">
         <is>
-          <t>2026-07-17T23:40Z</t>
+          <t>2026-07-18T18:20Z</t>
         </is>
       </c>
       <c r="D7" s="24" t="inlineStr">
         <is>
-          <t>401816148</t>
+          <t>401816164</t>
         </is>
       </c>
       <c r="E7" s="24" t="inlineStr">
@@ -2900,12 +2921,12 @@
       </c>
       <c r="F7" s="24" t="inlineStr">
         <is>
-          <t>Miami Marlins</t>
+          <t>Minnesota Twins</t>
         </is>
       </c>
       <c r="G7" s="24" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>Chicago Cubs</t>
         </is>
       </c>
       <c r="H7" s="24" t="inlineStr">
@@ -2918,30 +2939,30 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J7" s="25" t="n"/>
+      <c r="J7" s="38" t="n"/>
       <c r="K7" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
         </is>
       </c>
       <c r="L7" s="26" t="n">
-        <v>-141</v>
-      </c>
-      <c r="M7" s="27" t="n">
-        <v>1.70922</v>
+        <v>-133</v>
+      </c>
+      <c r="M7" s="39" t="n">
+        <v>1.75188</v>
       </c>
       <c r="N7" s="28" t="n">
-        <v>0.585062</v>
+        <v>0.570815</v>
       </c>
       <c r="O7" s="28" t="n">
-        <v>0.605633</v>
+        <v>0.606876</v>
       </c>
       <c r="P7" s="28" t="n"/>
       <c r="Q7" s="28" t="n">
-        <v>0.020571</v>
+        <v>0.036061</v>
       </c>
       <c r="R7" s="26" t="n">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="S7" s="29" t="n">
         <v>0</v>
@@ -2953,41 +2974,21 @@
       </c>
       <c r="U7" s="24" t="inlineStr">
         <is>
-          <t>settled</t>
-        </is>
-      </c>
-      <c r="V7" s="24" t="inlineStr">
-        <is>
-          <t>win</t>
-        </is>
-      </c>
-      <c r="W7" s="26" t="n">
-        <v>1</v>
-      </c>
-      <c r="X7" s="26" t="n">
-        <v>2</v>
-      </c>
-      <c r="Y7" s="25" t="n"/>
-      <c r="Z7" s="26" t="n">
-        <v>-147</v>
-      </c>
-      <c r="AA7" s="28" t="n">
-        <v>0.595</v>
-      </c>
-      <c r="AB7" s="28" t="n">
-        <v>0.009938000000000001</v>
-      </c>
-      <c r="AC7" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD7" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-18T05:45:54.715857Z</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V7" s="24" t="n"/>
+      <c r="W7" s="26" t="n"/>
+      <c r="X7" s="26" t="n"/>
+      <c r="Y7" s="38" t="n"/>
+      <c r="Z7" s="26" t="n"/>
+      <c r="AA7" s="28" t="n"/>
+      <c r="AB7" s="28" t="n"/>
+      <c r="AC7" s="40" t="n"/>
+      <c r="AD7" s="24" t="n"/>
       <c r="AE7" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.6018; executable ask 0.5850 (aec-mlb-mia-mil-2026-07-17).</t>
+          <t>Learned LR call at threshold 0.6018; executable ask 0.5700 (aec-mlb-min-chc-2026-07-18).</t>
         </is>
       </c>
       <c r="AF7" s="31" t="inlineStr">
@@ -3028,32 +3029,32 @@
       </c>
       <c r="AP7" s="24" t="inlineStr">
         <is>
-          <t>mlb-mia</t>
+          <t>mlb-min</t>
         </is>
       </c>
       <c r="AQ7" s="24" t="inlineStr">
         <is>
-          <t>Miami Marlins</t>
+          <t>Minnesota Twins</t>
         </is>
       </c>
       <c r="AR7" s="24" t="inlineStr">
         <is>
-          <t>Miami Marlins</t>
+          <t>Minnesota Twins</t>
         </is>
       </c>
       <c r="AS7" s="24" t="inlineStr">
         <is>
-          <t>mlb-mil</t>
+          <t>mlb-chc</t>
         </is>
       </c>
       <c r="AT7" s="24" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>Chicago Cubs</t>
         </is>
       </c>
       <c r="AU7" s="24" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>Chicago Cubs</t>
         </is>
       </c>
       <c r="AV7" s="24" t="n"/>
@@ -3091,7 +3092,7 @@
       </c>
       <c r="BE7" s="24" t="inlineStr">
         <is>
-          <t>27ad4a1da893e4b8</t>
+          <t>3acab0aa8ac04a91</t>
         </is>
       </c>
       <c r="BF7" s="24" t="inlineStr">
@@ -3106,7 +3107,7 @@
       </c>
       <c r="BH7" s="24" t="inlineStr">
         <is>
-          <t>2026-07-17T14:01:56.626918Z</t>
+          <t>2026-07-18T05:44:27.731285Z</t>
         </is>
       </c>
       <c r="BI7" s="24" t="inlineStr">
@@ -3114,1631 +3115,39 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ7" s="25" t="n"/>
+      <c r="BJ7" s="38" t="n"/>
       <c r="BK7" s="26" t="n">
-        <v>-141</v>
-      </c>
-      <c r="BL7" s="27" t="n">
-        <v>1.70922</v>
+        <v>-133</v>
+      </c>
+      <c r="BL7" s="39" t="n">
+        <v>1.75188</v>
       </c>
       <c r="BM7" s="28" t="n">
-        <v>0.585062</v>
+        <v>0.570815</v>
       </c>
       <c r="BN7" s="28" t="n">
-        <v>0.58209</v>
+        <v>0.567164</v>
       </c>
       <c r="BO7" s="28" t="n"/>
-      <c r="BP7" s="25" t="n"/>
-      <c r="BQ7" s="27" t="n">
-        <v>1.680272</v>
-      </c>
-      <c r="BR7" s="28" t="n">
-        <v>0.595</v>
-      </c>
+      <c r="BP7" s="38" t="n"/>
+      <c r="BQ7" s="39" t="n"/>
+      <c r="BR7" s="28" t="n"/>
       <c r="BS7" s="28" t="n"/>
       <c r="BT7" s="28" t="n"/>
-      <c r="BU7" s="25" t="n"/>
+      <c r="BU7" s="38" t="n"/>
       <c r="BV7" s="29" t="n"/>
       <c r="BW7" s="24" t="n"/>
-      <c r="BX7" s="30" t="n">
-        <v>1</v>
-      </c>
-      <c r="BY7" s="27" t="n">
-        <v>0.70922</v>
-      </c>
-      <c r="BZ7" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-18T05:45:54.715857Z</t>
-        </is>
-      </c>
-      <c r="CA7" s="31" t="inlineStr">
-        <is>
-          <t>fixed one-unit hypothetical scoring; no real exposure or execution</t>
-        </is>
-      </c>
+      <c r="BX7" s="40" t="n"/>
+      <c r="BY7" s="39" t="n"/>
+      <c r="BZ7" s="24" t="n"/>
+      <c r="CA7" s="31" t="n"/>
     </row>
-    <row r="8" ht="36" customHeight="1">
-      <c r="A8" s="24" t="inlineStr">
-        <is>
-          <t>3b98081a1ff04c62</t>
-        </is>
-      </c>
-      <c r="B8" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-17T14:02:14.862720Z</t>
-        </is>
-      </c>
-      <c r="C8" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-18T00:05Z</t>
-        </is>
-      </c>
-      <c r="D8" s="24" t="inlineStr">
-        <is>
-          <t>401816149</t>
-        </is>
-      </c>
-      <c r="E8" s="24" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="F8" s="24" t="inlineStr">
-        <is>
-          <t>Minnesota Twins</t>
-        </is>
-      </c>
-      <c r="G8" s="24" t="inlineStr">
-        <is>
-          <t>Chicago Cubs</t>
-        </is>
-      </c>
-      <c r="H8" s="24" t="inlineStr">
-        <is>
-          <t>moneyline</t>
-        </is>
-      </c>
-      <c r="I8" s="24" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="J8" s="25" t="n"/>
-      <c r="K8" s="24" t="inlineStr">
-        <is>
-          <t>polymarket_us</t>
-        </is>
-      </c>
-      <c r="L8" s="26" t="n">
-        <v>-130</v>
-      </c>
-      <c r="M8" s="27" t="n">
-        <v>1.769231</v>
-      </c>
-      <c r="N8" s="28" t="n">
-        <v>0.565217</v>
-      </c>
-      <c r="O8" s="28" t="n">
-        <v>0.606876</v>
-      </c>
-      <c r="P8" s="28" t="n"/>
-      <c r="Q8" s="28" t="n">
-        <v>0.041659</v>
-      </c>
-      <c r="R8" s="26" t="n">
-        <v>71</v>
-      </c>
-      <c r="S8" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="T8" s="24" t="inlineStr">
-        <is>
-          <t>mlb-elo-trend-lr-v3</t>
-        </is>
-      </c>
-      <c r="U8" s="24" t="inlineStr">
-        <is>
-          <t>settled</t>
-        </is>
-      </c>
-      <c r="V8" s="24" t="inlineStr">
-        <is>
-          <t>loss</t>
-        </is>
-      </c>
-      <c r="W8" s="26" t="n">
-        <v>5</v>
-      </c>
-      <c r="X8" s="26" t="n">
-        <v>2</v>
-      </c>
-      <c r="Y8" s="25" t="n"/>
-      <c r="Z8" s="26" t="n">
-        <v>-133</v>
-      </c>
-      <c r="AA8" s="28" t="n">
-        <v>0.57</v>
-      </c>
-      <c r="AB8" s="28" t="n">
-        <v>0.004783</v>
-      </c>
-      <c r="AC8" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD8" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-18T05:45:54.800172Z</t>
-        </is>
-      </c>
-      <c r="AE8" s="31" t="inlineStr">
-        <is>
-          <t>Learned LR call at threshold 0.6018; executable ask 0.5650 (aec-mlb-min-chc-2026-07-17).</t>
-        </is>
-      </c>
-      <c r="AF8" s="31" t="inlineStr">
-        <is>
-          <t>Learned model; promotion gate not yet open; zero-unit research until review.</t>
-        </is>
-      </c>
-      <c r="AG8" s="24" t="inlineStr">
-        <is>
-          <t>review_required</t>
-        </is>
-      </c>
-      <c r="AH8" s="24" t="n"/>
-      <c r="AI8" s="31" t="n"/>
-      <c r="AJ8" s="31" t="n"/>
-      <c r="AK8" s="24" t="inlineStr">
-        <is>
-          <t>research_observation</t>
-        </is>
-      </c>
-      <c r="AL8" s="26" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM8" s="24" t="inlineStr">
-        <is>
-          <t>RESEARCH_OBSERVATION</t>
-        </is>
-      </c>
-      <c r="AN8" s="24" t="inlineStr">
-        <is>
-          <t>NO_CALL</t>
-        </is>
-      </c>
-      <c r="AO8" s="24" t="inlineStr">
-        <is>
-          <t>NO_CALL_MISSING_UNCERTAINTY</t>
-        </is>
-      </c>
-      <c r="AP8" s="24" t="inlineStr">
-        <is>
-          <t>mlb-min</t>
-        </is>
-      </c>
-      <c r="AQ8" s="24" t="inlineStr">
-        <is>
-          <t>Minnesota Twins</t>
-        </is>
-      </c>
-      <c r="AR8" s="24" t="inlineStr">
-        <is>
-          <t>Minnesota Twins</t>
-        </is>
-      </c>
-      <c r="AS8" s="24" t="inlineStr">
-        <is>
-          <t>mlb-chc</t>
-        </is>
-      </c>
-      <c r="AT8" s="24" t="inlineStr">
-        <is>
-          <t>Chicago Cubs</t>
-        </is>
-      </c>
-      <c r="AU8" s="24" t="inlineStr">
-        <is>
-          <t>Chicago Cubs</t>
-        </is>
-      </c>
-      <c r="AV8" s="24" t="n"/>
-      <c r="AW8" s="24" t="n"/>
-      <c r="AX8" s="24" t="inlineStr">
-        <is>
-          <t>statistical_model</t>
-        </is>
-      </c>
-      <c r="AY8" s="24" t="n"/>
-      <c r="AZ8" s="24" t="inlineStr">
-        <is>
-          <t>research</t>
-        </is>
-      </c>
-      <c r="BA8" s="24" t="inlineStr">
-        <is>
-          <t>a454281ab207d2924d585d6b967363fb8e88af45132e3e9d354e4351fb5c237f</t>
-        </is>
-      </c>
-      <c r="BB8" s="24" t="inlineStr">
-        <is>
-          <t>learned_lr</t>
-        </is>
-      </c>
-      <c r="BC8" s="24" t="inlineStr">
-        <is>
-          <t>mlb-elo-trend-lr-v3</t>
-        </is>
-      </c>
-      <c r="BD8" s="24" t="inlineStr">
-        <is>
-          <t>a454281ab207d2924d585d6b967363fb8e88af45132e3e9d354e4351fb5c237f</t>
-        </is>
-      </c>
-      <c r="BE8" s="24" t="inlineStr">
-        <is>
-          <t>8438bc3f26be5eae</t>
-        </is>
-      </c>
-      <c r="BF8" s="24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BG8" s="24" t="inlineStr">
-        <is>
-          <t>mlb-elo-trend-lr-v3</t>
-        </is>
-      </c>
-      <c r="BH8" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-17T14:01:57.663980Z</t>
-        </is>
-      </c>
-      <c r="BI8" s="24" t="inlineStr">
-        <is>
-          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
-        </is>
-      </c>
-      <c r="BJ8" s="25" t="n"/>
-      <c r="BK8" s="26" t="n">
-        <v>-130</v>
-      </c>
-      <c r="BL8" s="27" t="n">
-        <v>1.769231</v>
-      </c>
-      <c r="BM8" s="28" t="n">
-        <v>0.565217</v>
-      </c>
-      <c r="BN8" s="28" t="n">
-        <v>0.562189</v>
-      </c>
-      <c r="BO8" s="28" t="n"/>
-      <c r="BP8" s="25" t="n"/>
-      <c r="BQ8" s="27" t="n">
-        <v>1.75188</v>
-      </c>
-      <c r="BR8" s="28" t="n">
-        <v>0.57</v>
-      </c>
-      <c r="BS8" s="28" t="n"/>
-      <c r="BT8" s="28" t="n"/>
-      <c r="BU8" s="25" t="n"/>
-      <c r="BV8" s="29" t="n"/>
-      <c r="BW8" s="24" t="n"/>
-      <c r="BX8" s="30" t="n">
-        <v>1</v>
-      </c>
-      <c r="BY8" s="27" t="n">
-        <v>-1</v>
-      </c>
-      <c r="BZ8" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-18T05:45:54.800172Z</t>
-        </is>
-      </c>
-      <c r="CA8" s="31" t="inlineStr">
-        <is>
-          <t>fixed one-unit hypothetical scoring; no real exposure or execution</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="36" customHeight="1">
-      <c r="A9" s="24" t="inlineStr">
-        <is>
-          <t>f592ac231a074ea9</t>
-        </is>
-      </c>
-      <c r="B9" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-17T14:02:17.091788Z</t>
-        </is>
-      </c>
-      <c r="C9" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-17T23:30Z</t>
-        </is>
-      </c>
-      <c r="D9" s="24" t="inlineStr">
-        <is>
-          <t>401857075</t>
-        </is>
-      </c>
-      <c r="E9" s="24" t="inlineStr">
-        <is>
-          <t>WNBA</t>
-        </is>
-      </c>
-      <c r="F9" s="24" t="inlineStr">
-        <is>
-          <t>Los Angeles Sparks</t>
-        </is>
-      </c>
-      <c r="G9" s="24" t="inlineStr">
-        <is>
-          <t>Chicago Sky</t>
-        </is>
-      </c>
-      <c r="H9" s="24" t="inlineStr">
-        <is>
-          <t>moneyline</t>
-        </is>
-      </c>
-      <c r="I9" s="24" t="inlineStr">
-        <is>
-          <t>away</t>
-        </is>
-      </c>
-      <c r="J9" s="25" t="n"/>
-      <c r="K9" s="24" t="inlineStr">
-        <is>
-          <t>polymarket_us</t>
-        </is>
-      </c>
-      <c r="L9" s="26" t="n">
-        <v>108</v>
-      </c>
-      <c r="M9" s="27" t="n">
-        <v>2.08</v>
-      </c>
-      <c r="N9" s="28" t="n">
-        <v>0.480769</v>
-      </c>
-      <c r="O9" s="28" t="n">
-        <v>0.580113</v>
-      </c>
-      <c r="P9" s="28" t="n"/>
-      <c r="Q9" s="28" t="n">
-        <v>0.099344</v>
-      </c>
-      <c r="R9" s="26" t="n">
-        <v>100</v>
-      </c>
-      <c r="S9" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="T9" s="24" t="inlineStr">
-        <is>
-          <t>wnba-elo-trend-lr-v3</t>
-        </is>
-      </c>
-      <c r="U9" s="24" t="inlineStr">
-        <is>
-          <t>settled</t>
-        </is>
-      </c>
-      <c r="V9" s="24" t="inlineStr">
-        <is>
-          <t>loss</t>
-        </is>
-      </c>
-      <c r="W9" s="26" t="n">
-        <v>82</v>
-      </c>
-      <c r="X9" s="26" t="n">
-        <v>96</v>
-      </c>
-      <c r="Y9" s="25" t="n"/>
-      <c r="Z9" s="26" t="n"/>
-      <c r="AA9" s="28" t="n"/>
-      <c r="AB9" s="28" t="n"/>
-      <c r="AC9" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD9" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-18T05:45:54.886428Z</t>
-        </is>
-      </c>
-      <c r="AE9" s="31" t="inlineStr">
-        <is>
-          <t>Learned LR call at threshold 0.5018; executable ask 0.4800 (aec-wnba-la-chi-2026-07-17).</t>
-        </is>
-      </c>
-      <c r="AF9" s="31" t="inlineStr">
-        <is>
-          <t>Learned model; promotion gate not yet open; zero-unit research until review.</t>
-        </is>
-      </c>
-      <c r="AG9" s="24" t="inlineStr">
-        <is>
-          <t>review_required</t>
-        </is>
-      </c>
-      <c r="AH9" s="24" t="n"/>
-      <c r="AI9" s="31" t="n"/>
-      <c r="AJ9" s="31" t="n"/>
-      <c r="AK9" s="24" t="inlineStr">
-        <is>
-          <t>research_observation</t>
-        </is>
-      </c>
-      <c r="AL9" s="26" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM9" s="24" t="inlineStr">
-        <is>
-          <t>RESEARCH_OBSERVATION</t>
-        </is>
-      </c>
-      <c r="AN9" s="24" t="inlineStr">
-        <is>
-          <t>NO_CALL</t>
-        </is>
-      </c>
-      <c r="AO9" s="24" t="inlineStr">
-        <is>
-          <t>NO_CALL_MISSING_UNCERTAINTY</t>
-        </is>
-      </c>
-      <c r="AP9" s="24" t="inlineStr">
-        <is>
-          <t>wnba-las</t>
-        </is>
-      </c>
-      <c r="AQ9" s="24" t="inlineStr">
-        <is>
-          <t>Los Angeles Sparks</t>
-        </is>
-      </c>
-      <c r="AR9" s="24" t="inlineStr">
-        <is>
-          <t>Los Angeles Sparks</t>
-        </is>
-      </c>
-      <c r="AS9" s="24" t="inlineStr">
-        <is>
-          <t>wnba-chi</t>
-        </is>
-      </c>
-      <c r="AT9" s="24" t="inlineStr">
-        <is>
-          <t>Chicago Sky</t>
-        </is>
-      </c>
-      <c r="AU9" s="24" t="inlineStr">
-        <is>
-          <t>Chicago Sky</t>
-        </is>
-      </c>
-      <c r="AV9" s="24" t="n"/>
-      <c r="AW9" s="24" t="n"/>
-      <c r="AX9" s="24" t="inlineStr">
-        <is>
-          <t>statistical_model</t>
-        </is>
-      </c>
-      <c r="AY9" s="24" t="n"/>
-      <c r="AZ9" s="24" t="inlineStr">
-        <is>
-          <t>research</t>
-        </is>
-      </c>
-      <c r="BA9" s="24" t="inlineStr">
-        <is>
-          <t>286653236675a65e58674d10837572801218599b31772016e9d8575bfefa53b4</t>
-        </is>
-      </c>
-      <c r="BB9" s="24" t="inlineStr">
-        <is>
-          <t>learned_lr</t>
-        </is>
-      </c>
-      <c r="BC9" s="24" t="inlineStr">
-        <is>
-          <t>wnba-elo-trend-lr-v3</t>
-        </is>
-      </c>
-      <c r="BD9" s="24" t="inlineStr">
-        <is>
-          <t>286653236675a65e58674d10837572801218599b31772016e9d8575bfefa53b4</t>
-        </is>
-      </c>
-      <c r="BE9" s="24" t="inlineStr">
-        <is>
-          <t>8c7d8b8b613f1c27</t>
-        </is>
-      </c>
-      <c r="BF9" s="24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BG9" s="24" t="inlineStr">
-        <is>
-          <t>wnba-elo-trend-lr-v3</t>
-        </is>
-      </c>
-      <c r="BH9" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-17T14:02:10.568774Z</t>
-        </is>
-      </c>
-      <c r="BI9" s="24" t="inlineStr">
-        <is>
-          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
-        </is>
-      </c>
-      <c r="BJ9" s="25" t="n"/>
-      <c r="BK9" s="26" t="n">
-        <v>108</v>
-      </c>
-      <c r="BL9" s="27" t="n">
-        <v>2.08</v>
-      </c>
-      <c r="BM9" s="28" t="n">
-        <v>0.480769</v>
-      </c>
-      <c r="BN9" s="28" t="n">
-        <v>0.475248</v>
-      </c>
-      <c r="BO9" s="28" t="n"/>
-      <c r="BP9" s="25" t="n"/>
-      <c r="BQ9" s="27" t="n"/>
-      <c r="BR9" s="28" t="n"/>
-      <c r="BS9" s="28" t="n"/>
-      <c r="BT9" s="28" t="n"/>
-      <c r="BU9" s="25" t="n"/>
-      <c r="BV9" s="29" t="n"/>
-      <c r="BW9" s="24" t="n"/>
-      <c r="BX9" s="30" t="n">
-        <v>1</v>
-      </c>
-      <c r="BY9" s="27" t="n">
-        <v>-1</v>
-      </c>
-      <c r="BZ9" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-18T05:45:54.886428Z</t>
-        </is>
-      </c>
-      <c r="CA9" s="31" t="inlineStr">
-        <is>
-          <t>fixed one-unit hypothetical scoring; no real exposure or execution</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="36" customHeight="1">
-      <c r="A10" s="24" t="inlineStr">
-        <is>
-          <t>3405fe6d522c42ec</t>
-        </is>
-      </c>
-      <c r="B10" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-17T14:02:17.091788Z</t>
-        </is>
-      </c>
-      <c r="C10" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-18T02:00Z</t>
-        </is>
-      </c>
-      <c r="D10" s="24" t="inlineStr">
-        <is>
-          <t>401857076</t>
-        </is>
-      </c>
-      <c r="E10" s="24" t="inlineStr">
-        <is>
-          <t>WNBA</t>
-        </is>
-      </c>
-      <c r="F10" s="24" t="inlineStr">
-        <is>
-          <t>Connecticut Sun</t>
-        </is>
-      </c>
-      <c r="G10" s="24" t="inlineStr">
-        <is>
-          <t>Phoenix Mercury</t>
-        </is>
-      </c>
-      <c r="H10" s="24" t="inlineStr">
-        <is>
-          <t>moneyline</t>
-        </is>
-      </c>
-      <c r="I10" s="24" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="J10" s="25" t="n"/>
-      <c r="K10" s="24" t="inlineStr">
-        <is>
-          <t>polymarket_us</t>
-        </is>
-      </c>
-      <c r="L10" s="26" t="n">
-        <v>-178</v>
-      </c>
-      <c r="M10" s="27" t="n">
-        <v>1.561798</v>
-      </c>
-      <c r="N10" s="28" t="n">
-        <v>0.640288</v>
-      </c>
-      <c r="O10" s="28" t="n">
-        <v>0.672243</v>
-      </c>
-      <c r="P10" s="28" t="n"/>
-      <c r="Q10" s="28" t="n">
-        <v>0.031955</v>
-      </c>
-      <c r="R10" s="26" t="n">
-        <v>66</v>
-      </c>
-      <c r="S10" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="T10" s="24" t="inlineStr">
-        <is>
-          <t>wnba-elo-trend-lr-v3</t>
-        </is>
-      </c>
-      <c r="U10" s="24" t="inlineStr">
-        <is>
-          <t>settled</t>
-        </is>
-      </c>
-      <c r="V10" s="24" t="inlineStr">
-        <is>
-          <t>loss</t>
-        </is>
-      </c>
-      <c r="W10" s="26" t="n">
-        <v>96</v>
-      </c>
-      <c r="X10" s="26" t="n">
-        <v>83</v>
-      </c>
-      <c r="Y10" s="25" t="n"/>
-      <c r="Z10" s="26" t="n"/>
-      <c r="AA10" s="28" t="n"/>
-      <c r="AB10" s="28" t="n"/>
-      <c r="AC10" s="30" t="n">
-        <v>-0</v>
-      </c>
-      <c r="AD10" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-18T05:45:54.971822Z</t>
-        </is>
-      </c>
-      <c r="AE10" s="31" t="inlineStr">
-        <is>
-          <t>Learned LR call at threshold 0.5018; executable ask 0.6400 (aec-wnba-conn-phx-2026-07-17).</t>
-        </is>
-      </c>
-      <c r="AF10" s="31" t="inlineStr">
-        <is>
-          <t>Learned model; promotion gate not yet open; zero-unit research until review.</t>
-        </is>
-      </c>
-      <c r="AG10" s="24" t="inlineStr">
-        <is>
-          <t>review_required</t>
-        </is>
-      </c>
-      <c r="AH10" s="24" t="n"/>
-      <c r="AI10" s="31" t="n"/>
-      <c r="AJ10" s="31" t="n"/>
-      <c r="AK10" s="24" t="inlineStr">
-        <is>
-          <t>research_observation</t>
-        </is>
-      </c>
-      <c r="AL10" s="26" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM10" s="24" t="inlineStr">
-        <is>
-          <t>RESEARCH_OBSERVATION</t>
-        </is>
-      </c>
-      <c r="AN10" s="24" t="inlineStr">
-        <is>
-          <t>NO_CALL</t>
-        </is>
-      </c>
-      <c r="AO10" s="24" t="inlineStr">
-        <is>
-          <t>NO_CALL_MISSING_UNCERTAINTY</t>
-        </is>
-      </c>
-      <c r="AP10" s="24" t="inlineStr">
-        <is>
-          <t>wnba-con</t>
-        </is>
-      </c>
-      <c r="AQ10" s="24" t="inlineStr">
-        <is>
-          <t>Connecticut Sun</t>
-        </is>
-      </c>
-      <c r="AR10" s="24" t="inlineStr">
-        <is>
-          <t>Connecticut Sun</t>
-        </is>
-      </c>
-      <c r="AS10" s="24" t="inlineStr">
-        <is>
-          <t>wnba-phx</t>
-        </is>
-      </c>
-      <c r="AT10" s="24" t="inlineStr">
-        <is>
-          <t>Phoenix Mercury</t>
-        </is>
-      </c>
-      <c r="AU10" s="24" t="inlineStr">
-        <is>
-          <t>Phoenix Mercury</t>
-        </is>
-      </c>
-      <c r="AV10" s="24" t="n"/>
-      <c r="AW10" s="24" t="n"/>
-      <c r="AX10" s="24" t="inlineStr">
-        <is>
-          <t>statistical_model</t>
-        </is>
-      </c>
-      <c r="AY10" s="24" t="n"/>
-      <c r="AZ10" s="24" t="inlineStr">
-        <is>
-          <t>research</t>
-        </is>
-      </c>
-      <c r="BA10" s="24" t="inlineStr">
-        <is>
-          <t>286653236675a65e58674d10837572801218599b31772016e9d8575bfefa53b4</t>
-        </is>
-      </c>
-      <c r="BB10" s="24" t="inlineStr">
-        <is>
-          <t>learned_lr</t>
-        </is>
-      </c>
-      <c r="BC10" s="24" t="inlineStr">
-        <is>
-          <t>wnba-elo-trend-lr-v3</t>
-        </is>
-      </c>
-      <c r="BD10" s="24" t="inlineStr">
-        <is>
-          <t>286653236675a65e58674d10837572801218599b31772016e9d8575bfefa53b4</t>
-        </is>
-      </c>
-      <c r="BE10" s="24" t="inlineStr">
-        <is>
-          <t>5b26e70fb7a6c509</t>
-        </is>
-      </c>
-      <c r="BF10" s="24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BG10" s="24" t="inlineStr">
-        <is>
-          <t>wnba-elo-trend-lr-v3</t>
-        </is>
-      </c>
-      <c r="BH10" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-17T14:02:11.780961Z</t>
-        </is>
-      </c>
-      <c r="BI10" s="24" t="inlineStr">
-        <is>
-          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
-        </is>
-      </c>
-      <c r="BJ10" s="25" t="n"/>
-      <c r="BK10" s="26" t="n">
-        <v>-178</v>
-      </c>
-      <c r="BL10" s="27" t="n">
-        <v>1.561798</v>
-      </c>
-      <c r="BM10" s="28" t="n">
-        <v>0.640288</v>
-      </c>
-      <c r="BN10" s="28" t="n">
-        <v>0.633663</v>
-      </c>
-      <c r="BO10" s="28" t="n"/>
-      <c r="BP10" s="25" t="n"/>
-      <c r="BQ10" s="27" t="n"/>
-      <c r="BR10" s="28" t="n"/>
-      <c r="BS10" s="28" t="n"/>
-      <c r="BT10" s="28" t="n"/>
-      <c r="BU10" s="25" t="n"/>
-      <c r="BV10" s="29" t="n"/>
-      <c r="BW10" s="24" t="n"/>
-      <c r="BX10" s="30" t="n">
-        <v>1</v>
-      </c>
-      <c r="BY10" s="27" t="n">
-        <v>-1</v>
-      </c>
-      <c r="BZ10" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-18T05:45:54.971822Z</t>
-        </is>
-      </c>
-      <c r="CA10" s="31" t="inlineStr">
-        <is>
-          <t>fixed one-unit hypothetical scoring; no real exposure or execution</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="36" customHeight="1">
-      <c r="A11" s="24" t="inlineStr">
-        <is>
-          <t>93a3540bf0dd49bb</t>
-        </is>
-      </c>
-      <c r="B11" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-17T16:21:24.725309Z</t>
-        </is>
-      </c>
-      <c r="C11" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-18T20:10Z</t>
-        </is>
-      </c>
-      <c r="D11" s="24" t="inlineStr">
-        <is>
-          <t>401816163</t>
-        </is>
-      </c>
-      <c r="E11" s="24" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="F11" s="24" t="inlineStr">
-        <is>
-          <t>Miami Marlins</t>
-        </is>
-      </c>
-      <c r="G11" s="24" t="inlineStr">
-        <is>
-          <t>Milwaukee Brewers</t>
-        </is>
-      </c>
-      <c r="H11" s="24" t="inlineStr">
-        <is>
-          <t>moneyline</t>
-        </is>
-      </c>
-      <c r="I11" s="24" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="J11" s="25" t="n"/>
-      <c r="K11" s="24" t="inlineStr">
-        <is>
-          <t>polymarket_us</t>
-        </is>
-      </c>
-      <c r="L11" s="26" t="n">
-        <v>-130</v>
-      </c>
-      <c r="M11" s="27" t="n">
-        <v>1.769231</v>
-      </c>
-      <c r="N11" s="28" t="n">
-        <v>0.565217</v>
-      </c>
-      <c r="O11" s="28" t="n">
-        <v>0.605633</v>
-      </c>
-      <c r="P11" s="28" t="n"/>
-      <c r="Q11" s="28" t="n">
-        <v>0.040416</v>
-      </c>
-      <c r="R11" s="26" t="n">
-        <v>70</v>
-      </c>
-      <c r="S11" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="T11" s="24" t="inlineStr">
-        <is>
-          <t>mlb-elo-trend-lr-v3</t>
-        </is>
-      </c>
-      <c r="U11" s="24" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V11" s="24" t="n"/>
-      <c r="W11" s="26" t="n"/>
-      <c r="X11" s="26" t="n"/>
-      <c r="Y11" s="25" t="n"/>
-      <c r="Z11" s="26" t="n"/>
-      <c r="AA11" s="28" t="n"/>
-      <c r="AB11" s="28" t="n"/>
-      <c r="AC11" s="30" t="n"/>
-      <c r="AD11" s="24" t="n"/>
-      <c r="AE11" s="31" t="inlineStr">
-        <is>
-          <t>Learned LR call at threshold 0.6018; executable ask 0.5650 (aec-mlb-mia-mil-2026-07-18).</t>
-        </is>
-      </c>
-      <c r="AF11" s="31" t="inlineStr">
-        <is>
-          <t>Learned model; promotion gate not yet open; zero-unit research until review.</t>
-        </is>
-      </c>
-      <c r="AG11" s="24" t="inlineStr">
-        <is>
-          <t>not_applicable</t>
-        </is>
-      </c>
-      <c r="AH11" s="24" t="n"/>
-      <c r="AI11" s="31" t="n"/>
-      <c r="AJ11" s="31" t="n"/>
-      <c r="AK11" s="24" t="inlineStr">
-        <is>
-          <t>research_observation</t>
-        </is>
-      </c>
-      <c r="AL11" s="26" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM11" s="24" t="inlineStr">
-        <is>
-          <t>RESEARCH_OBSERVATION</t>
-        </is>
-      </c>
-      <c r="AN11" s="24" t="inlineStr">
-        <is>
-          <t>NO_CALL</t>
-        </is>
-      </c>
-      <c r="AO11" s="24" t="inlineStr">
-        <is>
-          <t>NO_CALL_MISSING_UNCERTAINTY</t>
-        </is>
-      </c>
-      <c r="AP11" s="24" t="inlineStr">
-        <is>
-          <t>mlb-mia</t>
-        </is>
-      </c>
-      <c r="AQ11" s="24" t="inlineStr">
-        <is>
-          <t>Miami Marlins</t>
-        </is>
-      </c>
-      <c r="AR11" s="24" t="inlineStr">
-        <is>
-          <t>Miami Marlins</t>
-        </is>
-      </c>
-      <c r="AS11" s="24" t="inlineStr">
-        <is>
-          <t>mlb-mil</t>
-        </is>
-      </c>
-      <c r="AT11" s="24" t="inlineStr">
-        <is>
-          <t>Milwaukee Brewers</t>
-        </is>
-      </c>
-      <c r="AU11" s="24" t="inlineStr">
-        <is>
-          <t>Milwaukee Brewers</t>
-        </is>
-      </c>
-      <c r="AV11" s="24" t="n"/>
-      <c r="AW11" s="24" t="n"/>
-      <c r="AX11" s="24" t="inlineStr">
-        <is>
-          <t>statistical_model</t>
-        </is>
-      </c>
-      <c r="AY11" s="24" t="n"/>
-      <c r="AZ11" s="24" t="inlineStr">
-        <is>
-          <t>research</t>
-        </is>
-      </c>
-      <c r="BA11" s="24" t="inlineStr">
-        <is>
-          <t>a454281ab207d2924d585d6b967363fb8e88af45132e3e9d354e4351fb5c237f</t>
-        </is>
-      </c>
-      <c r="BB11" s="24" t="inlineStr">
-        <is>
-          <t>learned_lr</t>
-        </is>
-      </c>
-      <c r="BC11" s="24" t="inlineStr">
-        <is>
-          <t>mlb-elo-trend-lr-v3</t>
-        </is>
-      </c>
-      <c r="BD11" s="24" t="inlineStr">
-        <is>
-          <t>a454281ab207d2924d585d6b967363fb8e88af45132e3e9d354e4351fb5c237f</t>
-        </is>
-      </c>
-      <c r="BE11" s="24" t="inlineStr">
-        <is>
-          <t>c7348ce29d666909</t>
-        </is>
-      </c>
-      <c r="BF11" s="24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BG11" s="24" t="inlineStr">
-        <is>
-          <t>mlb-elo-trend-lr-v3</t>
-        </is>
-      </c>
-      <c r="BH11" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-17T16:21:07.161405Z</t>
-        </is>
-      </c>
-      <c r="BI11" s="24" t="inlineStr">
-        <is>
-          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
-        </is>
-      </c>
-      <c r="BJ11" s="25" t="n"/>
-      <c r="BK11" s="26" t="n">
-        <v>-130</v>
-      </c>
-      <c r="BL11" s="27" t="n">
-        <v>1.769231</v>
-      </c>
-      <c r="BM11" s="28" t="n">
-        <v>0.565217</v>
-      </c>
-      <c r="BN11" s="28" t="n">
-        <v>0.562189</v>
-      </c>
-      <c r="BO11" s="28" t="n"/>
-      <c r="BP11" s="25" t="n"/>
-      <c r="BQ11" s="27" t="n"/>
-      <c r="BR11" s="28" t="n"/>
-      <c r="BS11" s="28" t="n"/>
-      <c r="BT11" s="28" t="n"/>
-      <c r="BU11" s="25" t="n"/>
-      <c r="BV11" s="29" t="n"/>
-      <c r="BW11" s="24" t="n"/>
-      <c r="BX11" s="30" t="n"/>
-      <c r="BY11" s="27" t="n"/>
-      <c r="BZ11" s="24" t="n"/>
-      <c r="CA11" s="31" t="n"/>
-    </row>
-    <row r="12" ht="36" customHeight="1">
-      <c r="A12" s="24" t="inlineStr">
-        <is>
-          <t>c884dc7cf1104640</t>
-        </is>
-      </c>
-      <c r="B12" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-17T16:21:30.375686Z</t>
-        </is>
-      </c>
-      <c r="C12" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-19T00:00Z</t>
-        </is>
-      </c>
-      <c r="D12" s="24" t="inlineStr">
-        <is>
-          <t>401857077</t>
-        </is>
-      </c>
-      <c r="E12" s="24" t="inlineStr">
-        <is>
-          <t>WNBA</t>
-        </is>
-      </c>
-      <c r="F12" s="24" t="inlineStr">
-        <is>
-          <t>New York Liberty</t>
-        </is>
-      </c>
-      <c r="G12" s="24" t="inlineStr">
-        <is>
-          <t>Indiana Fever</t>
-        </is>
-      </c>
-      <c r="H12" s="24" t="inlineStr">
-        <is>
-          <t>moneyline</t>
-        </is>
-      </c>
-      <c r="I12" s="24" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="J12" s="25" t="n"/>
-      <c r="K12" s="24" t="inlineStr">
-        <is>
-          <t>polymarket_us</t>
-        </is>
-      </c>
-      <c r="L12" s="26" t="n">
-        <v>117</v>
-      </c>
-      <c r="M12" s="27" t="n">
-        <v>2.17</v>
-      </c>
-      <c r="N12" s="28" t="n">
-        <v>0.460829</v>
-      </c>
-      <c r="O12" s="28" t="n">
-        <v>0.632778</v>
-      </c>
-      <c r="P12" s="28" t="n"/>
-      <c r="Q12" s="28" t="n">
-        <v>0.171949</v>
-      </c>
-      <c r="R12" s="26" t="n">
-        <v>100</v>
-      </c>
-      <c r="S12" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="T12" s="24" t="inlineStr">
-        <is>
-          <t>wnba-elo-trend-lr-v3</t>
-        </is>
-      </c>
-      <c r="U12" s="24" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V12" s="24" t="n"/>
-      <c r="W12" s="26" t="n"/>
-      <c r="X12" s="26" t="n"/>
-      <c r="Y12" s="25" t="n"/>
-      <c r="Z12" s="26" t="n"/>
-      <c r="AA12" s="28" t="n"/>
-      <c r="AB12" s="28" t="n"/>
-      <c r="AC12" s="30" t="n"/>
-      <c r="AD12" s="24" t="n"/>
-      <c r="AE12" s="31" t="inlineStr">
-        <is>
-          <t>Learned LR call at threshold 0.5018; executable ask 0.4600 (aec-wnba-ny-ind-2026-07-18).</t>
-        </is>
-      </c>
-      <c r="AF12" s="31" t="inlineStr">
-        <is>
-          <t>Learned model; promotion gate not yet open; zero-unit research until review.</t>
-        </is>
-      </c>
-      <c r="AG12" s="24" t="inlineStr">
-        <is>
-          <t>not_applicable</t>
-        </is>
-      </c>
-      <c r="AH12" s="24" t="n"/>
-      <c r="AI12" s="31" t="n"/>
-      <c r="AJ12" s="31" t="n"/>
-      <c r="AK12" s="24" t="inlineStr">
-        <is>
-          <t>research_observation</t>
-        </is>
-      </c>
-      <c r="AL12" s="26" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM12" s="24" t="inlineStr">
-        <is>
-          <t>RESEARCH_OBSERVATION</t>
-        </is>
-      </c>
-      <c r="AN12" s="24" t="inlineStr">
-        <is>
-          <t>NO_CALL</t>
-        </is>
-      </c>
-      <c r="AO12" s="24" t="inlineStr">
-        <is>
-          <t>NO_CALL_MISSING_UNCERTAINTY</t>
-        </is>
-      </c>
-      <c r="AP12" s="24" t="inlineStr">
-        <is>
-          <t>wnba-nyl</t>
-        </is>
-      </c>
-      <c r="AQ12" s="24" t="inlineStr">
-        <is>
-          <t>New York Liberty</t>
-        </is>
-      </c>
-      <c r="AR12" s="24" t="inlineStr">
-        <is>
-          <t>New York Liberty</t>
-        </is>
-      </c>
-      <c r="AS12" s="24" t="inlineStr">
-        <is>
-          <t>wnba-ind</t>
-        </is>
-      </c>
-      <c r="AT12" s="24" t="inlineStr">
-        <is>
-          <t>Indiana Fever</t>
-        </is>
-      </c>
-      <c r="AU12" s="24" t="inlineStr">
-        <is>
-          <t>Indiana Fever</t>
-        </is>
-      </c>
-      <c r="AV12" s="24" t="n"/>
-      <c r="AW12" s="24" t="n"/>
-      <c r="AX12" s="24" t="inlineStr">
-        <is>
-          <t>statistical_model</t>
-        </is>
-      </c>
-      <c r="AY12" s="24" t="n"/>
-      <c r="AZ12" s="24" t="inlineStr">
-        <is>
-          <t>research</t>
-        </is>
-      </c>
-      <c r="BA12" s="24" t="inlineStr">
-        <is>
-          <t>286653236675a65e58674d10837572801218599b31772016e9d8575bfefa53b4</t>
-        </is>
-      </c>
-      <c r="BB12" s="24" t="inlineStr">
-        <is>
-          <t>learned_lr</t>
-        </is>
-      </c>
-      <c r="BC12" s="24" t="inlineStr">
-        <is>
-          <t>wnba-elo-trend-lr-v3</t>
-        </is>
-      </c>
-      <c r="BD12" s="24" t="inlineStr">
-        <is>
-          <t>286653236675a65e58674d10837572801218599b31772016e9d8575bfefa53b4</t>
-        </is>
-      </c>
-      <c r="BE12" s="24" t="inlineStr">
-        <is>
-          <t>e4f3f616d306cafe</t>
-        </is>
-      </c>
-      <c r="BF12" s="24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BG12" s="24" t="inlineStr">
-        <is>
-          <t>wnba-elo-trend-lr-v3</t>
-        </is>
-      </c>
-      <c r="BH12" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-17T16:21:13.188564Z</t>
-        </is>
-      </c>
-      <c r="BI12" s="24" t="inlineStr">
-        <is>
-          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
-        </is>
-      </c>
-      <c r="BJ12" s="25" t="n"/>
-      <c r="BK12" s="26" t="n">
-        <v>117</v>
-      </c>
-      <c r="BL12" s="27" t="n">
-        <v>2.17</v>
-      </c>
-      <c r="BM12" s="28" t="n">
-        <v>0.460829</v>
-      </c>
-      <c r="BN12" s="28" t="n">
-        <v>0.455446</v>
-      </c>
-      <c r="BO12" s="28" t="n"/>
-      <c r="BP12" s="25" t="n"/>
-      <c r="BQ12" s="27" t="n"/>
-      <c r="BR12" s="28" t="n"/>
-      <c r="BS12" s="28" t="n"/>
-      <c r="BT12" s="28" t="n"/>
-      <c r="BU12" s="25" t="n"/>
-      <c r="BV12" s="29" t="n"/>
-      <c r="BW12" s="24" t="n"/>
-      <c r="BX12" s="30" t="n"/>
-      <c r="BY12" s="27" t="n"/>
-      <c r="BZ12" s="24" t="n"/>
-      <c r="CA12" s="31" t="n"/>
-    </row>
-    <row r="13" ht="36" customHeight="1">
-      <c r="A13" s="24" t="inlineStr">
-        <is>
-          <t>4c2ec934da05478b</t>
-        </is>
-      </c>
-      <c r="B13" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-18T05:45:47.429402Z</t>
-        </is>
-      </c>
-      <c r="C13" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-18T18:20Z</t>
-        </is>
-      </c>
-      <c r="D13" s="24" t="inlineStr">
-        <is>
-          <t>401816164</t>
-        </is>
-      </c>
-      <c r="E13" s="24" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="F13" s="24" t="inlineStr">
-        <is>
-          <t>Minnesota Twins</t>
-        </is>
-      </c>
-      <c r="G13" s="24" t="inlineStr">
-        <is>
-          <t>Chicago Cubs</t>
-        </is>
-      </c>
-      <c r="H13" s="24" t="inlineStr">
-        <is>
-          <t>moneyline</t>
-        </is>
-      </c>
-      <c r="I13" s="24" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="J13" s="25" t="n"/>
-      <c r="K13" s="24" t="inlineStr">
-        <is>
-          <t>polymarket_us</t>
-        </is>
-      </c>
-      <c r="L13" s="26" t="n">
-        <v>-133</v>
-      </c>
-      <c r="M13" s="27" t="n">
-        <v>1.75188</v>
-      </c>
-      <c r="N13" s="28" t="n">
-        <v>0.570815</v>
-      </c>
-      <c r="O13" s="28" t="n">
-        <v>0.606876</v>
-      </c>
-      <c r="P13" s="28" t="n"/>
-      <c r="Q13" s="28" t="n">
-        <v>0.036061</v>
-      </c>
-      <c r="R13" s="26" t="n">
-        <v>68</v>
-      </c>
-      <c r="S13" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="T13" s="24" t="inlineStr">
-        <is>
-          <t>mlb-elo-trend-lr-v3</t>
-        </is>
-      </c>
-      <c r="U13" s="24" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V13" s="24" t="n"/>
-      <c r="W13" s="26" t="n"/>
-      <c r="X13" s="26" t="n"/>
-      <c r="Y13" s="25" t="n"/>
-      <c r="Z13" s="26" t="n"/>
-      <c r="AA13" s="28" t="n"/>
-      <c r="AB13" s="28" t="n"/>
-      <c r="AC13" s="30" t="n"/>
-      <c r="AD13" s="24" t="n"/>
-      <c r="AE13" s="31" t="inlineStr">
-        <is>
-          <t>Learned LR call at threshold 0.6018; executable ask 0.5700 (aec-mlb-min-chc-2026-07-18).</t>
-        </is>
-      </c>
-      <c r="AF13" s="31" t="inlineStr">
-        <is>
-          <t>Learned model; promotion gate not yet open; zero-unit research until review.</t>
-        </is>
-      </c>
-      <c r="AG13" s="24" t="inlineStr">
-        <is>
-          <t>not_applicable</t>
-        </is>
-      </c>
-      <c r="AH13" s="24" t="n"/>
-      <c r="AI13" s="31" t="n"/>
-      <c r="AJ13" s="31" t="n"/>
-      <c r="AK13" s="24" t="inlineStr">
-        <is>
-          <t>research_observation</t>
-        </is>
-      </c>
-      <c r="AL13" s="26" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM13" s="24" t="inlineStr">
-        <is>
-          <t>RESEARCH_OBSERVATION</t>
-        </is>
-      </c>
-      <c r="AN13" s="24" t="inlineStr">
-        <is>
-          <t>NO_CALL</t>
-        </is>
-      </c>
-      <c r="AO13" s="24" t="inlineStr">
-        <is>
-          <t>NO_CALL_MISSING_UNCERTAINTY</t>
-        </is>
-      </c>
-      <c r="AP13" s="24" t="inlineStr">
-        <is>
-          <t>mlb-min</t>
-        </is>
-      </c>
-      <c r="AQ13" s="24" t="inlineStr">
-        <is>
-          <t>Minnesota Twins</t>
-        </is>
-      </c>
-      <c r="AR13" s="24" t="inlineStr">
-        <is>
-          <t>Minnesota Twins</t>
-        </is>
-      </c>
-      <c r="AS13" s="24" t="inlineStr">
-        <is>
-          <t>mlb-chc</t>
-        </is>
-      </c>
-      <c r="AT13" s="24" t="inlineStr">
-        <is>
-          <t>Chicago Cubs</t>
-        </is>
-      </c>
-      <c r="AU13" s="24" t="inlineStr">
-        <is>
-          <t>Chicago Cubs</t>
-        </is>
-      </c>
-      <c r="AV13" s="24" t="n"/>
-      <c r="AW13" s="24" t="n"/>
-      <c r="AX13" s="24" t="inlineStr">
-        <is>
-          <t>statistical_model</t>
-        </is>
-      </c>
-      <c r="AY13" s="24" t="n"/>
-      <c r="AZ13" s="24" t="inlineStr">
-        <is>
-          <t>research</t>
-        </is>
-      </c>
-      <c r="BA13" s="24" t="inlineStr">
-        <is>
-          <t>a454281ab207d2924d585d6b967363fb8e88af45132e3e9d354e4351fb5c237f</t>
-        </is>
-      </c>
-      <c r="BB13" s="24" t="inlineStr">
-        <is>
-          <t>learned_lr</t>
-        </is>
-      </c>
-      <c r="BC13" s="24" t="inlineStr">
-        <is>
-          <t>mlb-elo-trend-lr-v3</t>
-        </is>
-      </c>
-      <c r="BD13" s="24" t="inlineStr">
-        <is>
-          <t>a454281ab207d2924d585d6b967363fb8e88af45132e3e9d354e4351fb5c237f</t>
-        </is>
-      </c>
-      <c r="BE13" s="24" t="inlineStr">
-        <is>
-          <t>3acab0aa8ac04a91</t>
-        </is>
-      </c>
-      <c r="BF13" s="24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BG13" s="24" t="inlineStr">
-        <is>
-          <t>mlb-elo-trend-lr-v3</t>
-        </is>
-      </c>
-      <c r="BH13" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-18T05:44:27.731285Z</t>
-        </is>
-      </c>
-      <c r="BI13" s="24" t="inlineStr">
-        <is>
-          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
-        </is>
-      </c>
-      <c r="BJ13" s="25" t="n"/>
-      <c r="BK13" s="26" t="n">
-        <v>-133</v>
-      </c>
-      <c r="BL13" s="27" t="n">
-        <v>1.75188</v>
-      </c>
-      <c r="BM13" s="28" t="n">
-        <v>0.570815</v>
-      </c>
-      <c r="BN13" s="28" t="n">
-        <v>0.567164</v>
-      </c>
-      <c r="BO13" s="28" t="n"/>
-      <c r="BP13" s="25" t="n"/>
-      <c r="BQ13" s="27" t="n"/>
-      <c r="BR13" s="28" t="n"/>
-      <c r="BS13" s="28" t="n"/>
-      <c r="BT13" s="28" t="n"/>
-      <c r="BU13" s="25" t="n"/>
-      <c r="BV13" s="29" t="n"/>
-      <c r="BW13" s="24" t="n"/>
-      <c r="BX13" s="30" t="n"/>
-      <c r="BY13" s="27" t="n"/>
-      <c r="BZ13" s="24" t="n"/>
-      <c r="CA13" s="31" t="n"/>
-    </row>
+    <row r="8" ht="36" customHeight="1"/>
+    <row r="9" ht="36" customHeight="1"/>
+    <row r="10" ht="36" customHeight="1"/>
+    <row r="11" ht="36" customHeight="1"/>
+    <row r="12" ht="36" customHeight="1"/>
+    <row r="13" ht="36" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
dashboard fix, backfilled historical data, cleaned ledger
- dash: fixed venv path
- dashboard: matrix fallback includes elo_trend_defense/park variants
- Backfilled: NBA +596, WNBA +392, NFL +400, MLB +15 games
- Ledger: WNBA cleared, RESEARCH_OBSERVATION removed
</commit_message>
<xml_diff>
--- a/data/picks.xlsx
+++ b/data/picks.xlsx
@@ -21,10 +21,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="0.0%"/>
-    <numFmt numFmtId="165" formatCode="0.0000"/>
-    <numFmt numFmtId="166" formatCode="0.0###"/>
-    <numFmt numFmtId="167" formatCode="0.000000"/>
+    <numFmt numFmtId="164" formatCode="0.0###"/>
+    <numFmt numFmtId="165" formatCode="0.000000"/>
+    <numFmt numFmtId="166" formatCode="0.0000"/>
+    <numFmt numFmtId="167" formatCode="0.0%"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -136,7 +136,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -150,10 +150,10 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -169,10 +169,10 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="10" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -184,10 +184,10 @@
     <xf numFmtId="0" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="10" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -202,13 +202,13 @@
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="10" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -217,38 +217,11 @@
     <xf numFmtId="2" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -327,8 +300,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CA13" headerRowCount="1">
-  <autoFilter ref="A1:CA13"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CA9" headerRowCount="1">
+  <autoFilter ref="A1:CA9"/>
   <tableColumns count="79">
     <tableColumn id="1" name="pick_id"/>
     <tableColumn id="2" name="created_at_utc"/>
@@ -765,19 +738,19 @@
     </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="6">
-        <f>COUNTA('Picks'!$A$2:$A$13)</f>
+        <f>COUNTA('Picks'!$A$2:$A$9)</f>
         <v/>
       </c>
       <c r="C4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$13,"open")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$9,"open")</f>
         <v/>
       </c>
       <c r="E4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$13,"settled")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$9,"settled")</f>
         <v/>
       </c>
       <c r="G4" s="6">
-        <f>IF(COUNTIFS('Picks'!$U$2:$U$13,"settled",'Picks'!$V$2:$V$13,"win")+COUNTIFS('Picks'!$U$2:$U$13,"settled",'Picks'!$V$2:$V$13,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
+        <f>IF(COUNTIFS('Picks'!$U$2:$U$9,"settled",'Picks'!$V$2:$V$9,"win")+COUNTIFS('Picks'!$U$2:$U$9,"settled",'Picks'!$V$2:$V$9,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
         <v/>
       </c>
     </row>
@@ -805,19 +778,19 @@
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="6">
-        <f>COUNTIF('Picks'!$BX$2:$BX$13,"&gt;0")</f>
+        <f>COUNTIF('Picks'!$BX$2:$BX$9,"&gt;0")</f>
         <v/>
       </c>
       <c r="C7" s="6">
-        <f>COUNTIFS('Picks'!$BX$2:$BX$13,"&gt;0",'Picks'!$V$2:$V$13,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$13,"&gt;0",'Picks'!$V$2:$V$13,"loss")</f>
+        <f>COUNTIFS('Picks'!$BX$2:$BX$9,"&gt;0",'Picks'!$V$2:$V$9,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$9,"&gt;0",'Picks'!$V$2:$V$9,"loss")</f>
         <v/>
       </c>
-      <c r="E7" s="32">
-        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$13,"&gt;0",'Picks'!$V$2:$V$13,"win")/(COUNTIFS('Picks'!$BX$2:$BX$13,"&gt;0",'Picks'!$V$2:$V$13,"win")+COUNTIFS('Picks'!$BX$2:$BX$13,"&gt;0",'Picks'!$V$2:$V$13,"loss")),0)</f>
+      <c r="E7" s="7">
+        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$9,"&gt;0",'Picks'!$V$2:$V$9,"win")/(COUNTIFS('Picks'!$BX$2:$BX$9,"&gt;0",'Picks'!$V$2:$V$9,"win")+COUNTIFS('Picks'!$BX$2:$BX$9,"&gt;0",'Picks'!$V$2:$V$9,"loss")),0)</f>
         <v/>
       </c>
-      <c r="G7" s="32">
-        <f>IFERROR(SUM('Picks'!$BY$2:$BY$13)/SUM('Picks'!$BX$2:$BX$13),0)</f>
+      <c r="G7" s="7">
+        <f>IFERROR(SUM('Picks'!$BY$2:$BY$9)/SUM('Picks'!$BX$2:$BX$9),0)</f>
         <v/>
       </c>
     </row>
@@ -844,20 +817,20 @@
       </c>
     </row>
     <row r="10" ht="28" customHeight="1">
-      <c r="A10" s="33">
-        <f>SUM('Picks'!$BY$2:$BY$13)</f>
+      <c r="A10" s="8">
+        <f>SUM('Picks'!$BY$2:$BY$9)</f>
         <v/>
       </c>
       <c r="C10" s="9">
-        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$13,"&lt;&gt;",'Picks'!$AB$2:$AB$13),0)</f>
+        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$9,"&lt;&gt;",'Picks'!$AB$2:$AB$9),0)</f>
         <v/>
       </c>
       <c r="E10" s="6">
-        <f>COUNTIFS('Picks'!$AM$2:$AM$13,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$13,"settled")</f>
+        <f>COUNTIFS('Picks'!$AM$2:$AM$9,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$9,"settled")</f>
         <v/>
       </c>
-      <c r="G10" s="33">
-        <f>SUMIFS('Picks'!$AC$2:$AC$13,'Picks'!$AM$2:$AM$13,"QUALIFIED_SHADOW_CALL")</f>
+      <c r="G10" s="8">
+        <f>SUMIFS('Picks'!$AC$2:$AC$9,'Picks'!$AM$2:$AM$9,"QUALIFIED_SHADOW_CALL")</f>
         <v/>
       </c>
     </row>
@@ -912,27 +885,27 @@
         </is>
       </c>
       <c r="B14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$13,$A14,'Picks'!$U$2:$U$13,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$9,$A14,'Picks'!$U$2:$U$9,"settled")</f>
         <v/>
       </c>
       <c r="C14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$13,$A14,'Picks'!$U$2:$U$13,"settled",'Picks'!$V$2:$V$13,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$9,$A14,'Picks'!$U$2:$U$9,"settled",'Picks'!$V$2:$V$9,"win")</f>
         <v/>
       </c>
       <c r="D14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$13,$A14,'Picks'!$U$2:$U$13,"settled",'Picks'!$V$2:$V$13,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$9,$A14,'Picks'!$U$2:$U$9,"settled",'Picks'!$V$2:$V$9,"loss")</f>
         <v/>
       </c>
-      <c r="E14" s="34">
+      <c r="E14" s="14">
         <f>IFERROR(C14/(C14+D14),0)</f>
         <v/>
       </c>
-      <c r="F14" s="35">
-        <f>SUMIFS('Picks'!$BY$2:$BY$13,'Picks'!$H$2:$H$13,$A14)</f>
+      <c r="F14" s="15">
+        <f>SUMIFS('Picks'!$BY$2:$BY$9,'Picks'!$H$2:$H$9,$A14)</f>
         <v/>
       </c>
       <c r="G14" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$13,'Picks'!$H$2:$H$13,$A14,'Picks'!$U$2:$U$13,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$9,'Picks'!$H$2:$H$9,$A14,'Picks'!$U$2:$U$9,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -943,27 +916,27 @@
         </is>
       </c>
       <c r="B15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$13,$A15,'Picks'!$U$2:$U$13,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$9,$A15,'Picks'!$U$2:$U$9,"settled")</f>
         <v/>
       </c>
       <c r="C15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$13,$A15,'Picks'!$U$2:$U$13,"settled",'Picks'!$V$2:$V$13,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$9,$A15,'Picks'!$U$2:$U$9,"settled",'Picks'!$V$2:$V$9,"win")</f>
         <v/>
       </c>
       <c r="D15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$13,$A15,'Picks'!$U$2:$U$13,"settled",'Picks'!$V$2:$V$13,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$9,$A15,'Picks'!$U$2:$U$9,"settled",'Picks'!$V$2:$V$9,"loss")</f>
         <v/>
       </c>
-      <c r="E15" s="36">
+      <c r="E15" s="19">
         <f>IFERROR(C15/(C15+D15),0)</f>
         <v/>
       </c>
-      <c r="F15" s="37">
-        <f>SUMIFS('Picks'!$BY$2:$BY$13,'Picks'!$H$2:$H$13,$A15)</f>
+      <c r="F15" s="20">
+        <f>SUMIFS('Picks'!$BY$2:$BY$9,'Picks'!$H$2:$H$9,$A15)</f>
         <v/>
       </c>
       <c r="G15" s="21">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$13,'Picks'!$H$2:$H$13,$A15,'Picks'!$U$2:$U$13,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$9,'Picks'!$H$2:$H$9,$A15,'Picks'!$U$2:$U$9,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -974,27 +947,27 @@
         </is>
       </c>
       <c r="B16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$13,$A16,'Picks'!$U$2:$U$13,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$9,$A16,'Picks'!$U$2:$U$9,"settled")</f>
         <v/>
       </c>
       <c r="C16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$13,$A16,'Picks'!$U$2:$U$13,"settled",'Picks'!$V$2:$V$13,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$9,$A16,'Picks'!$U$2:$U$9,"settled",'Picks'!$V$2:$V$9,"win")</f>
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$13,$A16,'Picks'!$U$2:$U$13,"settled",'Picks'!$V$2:$V$13,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$9,$A16,'Picks'!$U$2:$U$9,"settled",'Picks'!$V$2:$V$9,"loss")</f>
         <v/>
       </c>
-      <c r="E16" s="34">
+      <c r="E16" s="14">
         <f>IFERROR(C16/(C16+D16),0)</f>
         <v/>
       </c>
-      <c r="F16" s="35">
-        <f>SUMIFS('Picks'!$BY$2:$BY$13,'Picks'!$H$2:$H$13,$A16)</f>
+      <c r="F16" s="15">
+        <f>SUMIFS('Picks'!$BY$2:$BY$9,'Picks'!$H$2:$H$9,$A16)</f>
         <v/>
       </c>
       <c r="G16" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$13,'Picks'!$H$2:$H$13,$A16,'Picks'!$U$2:$U$13,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$9,'Picks'!$H$2:$H$9,$A16,'Picks'!$U$2:$U$9,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -1023,7 +996,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:CA7"/>
+  <dimension ref="A1:CA9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1550,7 +1523,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J2" s="38" t="n"/>
+      <c r="J2" s="25" t="n"/>
       <c r="K2" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -1559,7 +1532,7 @@
       <c r="L2" s="26" t="n">
         <v>-141</v>
       </c>
-      <c r="M2" s="39" t="n">
+      <c r="M2" s="27" t="n">
         <v>1.70922</v>
       </c>
       <c r="N2" s="28" t="n">
@@ -1599,7 +1572,7 @@
       <c r="X2" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="Y2" s="38" t="n"/>
+      <c r="Y2" s="25" t="n"/>
       <c r="Z2" s="26" t="n">
         <v>-147</v>
       </c>
@@ -1609,7 +1582,7 @@
       <c r="AB2" s="28" t="n">
         <v>0.009938000000000001</v>
       </c>
-      <c r="AC2" s="40" t="n">
+      <c r="AC2" s="30" t="n">
         <v>0</v>
       </c>
       <c r="AD2" s="24" t="inlineStr">
@@ -1746,11 +1719,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ2" s="38" t="n"/>
+      <c r="BJ2" s="25" t="n"/>
       <c r="BK2" s="26" t="n">
         <v>-141</v>
       </c>
-      <c r="BL2" s="39" t="n">
+      <c r="BL2" s="27" t="n">
         <v>1.70922</v>
       </c>
       <c r="BM2" s="28" t="n">
@@ -1760,8 +1733,8 @@
         <v>0.58209</v>
       </c>
       <c r="BO2" s="28" t="n"/>
-      <c r="BP2" s="38" t="n"/>
-      <c r="BQ2" s="39" t="n">
+      <c r="BP2" s="25" t="n"/>
+      <c r="BQ2" s="27" t="n">
         <v>1.680272</v>
       </c>
       <c r="BR2" s="28" t="n">
@@ -1769,13 +1742,13 @@
       </c>
       <c r="BS2" s="28" t="n"/>
       <c r="BT2" s="28" t="n"/>
-      <c r="BU2" s="38" t="n"/>
+      <c r="BU2" s="25" t="n"/>
       <c r="BV2" s="29" t="n"/>
       <c r="BW2" s="24" t="n"/>
-      <c r="BX2" s="40" t="n">
+      <c r="BX2" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY2" s="39" t="n">
+      <c r="BY2" s="27" t="n">
         <v>0.70922</v>
       </c>
       <c r="BZ2" s="24" t="inlineStr">
@@ -1835,7 +1808,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J3" s="38" t="n"/>
+      <c r="J3" s="25" t="n"/>
       <c r="K3" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -1844,7 +1817,7 @@
       <c r="L3" s="26" t="n">
         <v>-130</v>
       </c>
-      <c r="M3" s="39" t="n">
+      <c r="M3" s="27" t="n">
         <v>1.769231</v>
       </c>
       <c r="N3" s="28" t="n">
@@ -1884,7 +1857,7 @@
       <c r="X3" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="Y3" s="38" t="n"/>
+      <c r="Y3" s="25" t="n"/>
       <c r="Z3" s="26" t="n">
         <v>-133</v>
       </c>
@@ -1894,7 +1867,7 @@
       <c r="AB3" s="28" t="n">
         <v>0.004783</v>
       </c>
-      <c r="AC3" s="40" t="n">
+      <c r="AC3" s="30" t="n">
         <v>0</v>
       </c>
       <c r="AD3" s="24" t="inlineStr">
@@ -2031,11 +2004,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ3" s="38" t="n"/>
+      <c r="BJ3" s="25" t="n"/>
       <c r="BK3" s="26" t="n">
         <v>-130</v>
       </c>
-      <c r="BL3" s="39" t="n">
+      <c r="BL3" s="27" t="n">
         <v>1.769231</v>
       </c>
       <c r="BM3" s="28" t="n">
@@ -2045,8 +2018,8 @@
         <v>0.562189</v>
       </c>
       <c r="BO3" s="28" t="n"/>
-      <c r="BP3" s="38" t="n"/>
-      <c r="BQ3" s="39" t="n">
+      <c r="BP3" s="25" t="n"/>
+      <c r="BQ3" s="27" t="n">
         <v>1.75188</v>
       </c>
       <c r="BR3" s="28" t="n">
@@ -2054,13 +2027,13 @@
       </c>
       <c r="BS3" s="28" t="n"/>
       <c r="BT3" s="28" t="n"/>
-      <c r="BU3" s="38" t="n"/>
+      <c r="BU3" s="25" t="n"/>
       <c r="BV3" s="29" t="n"/>
       <c r="BW3" s="24" t="n"/>
-      <c r="BX3" s="40" t="n">
+      <c r="BX3" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY3" s="39" t="n">
+      <c r="BY3" s="27" t="n">
         <v>-1</v>
       </c>
       <c r="BZ3" s="24" t="inlineStr">
@@ -2120,7 +2093,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J4" s="38" t="n"/>
+      <c r="J4" s="25" t="n"/>
       <c r="K4" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -2129,7 +2102,7 @@
       <c r="L4" s="26" t="n">
         <v>-141</v>
       </c>
-      <c r="M4" s="39" t="n">
+      <c r="M4" s="27" t="n">
         <v>1.70922</v>
       </c>
       <c r="N4" s="28" t="n">
@@ -2169,7 +2142,7 @@
       <c r="X4" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="Y4" s="38" t="n"/>
+      <c r="Y4" s="25" t="n"/>
       <c r="Z4" s="26" t="n">
         <v>-147</v>
       </c>
@@ -2179,7 +2152,7 @@
       <c r="AB4" s="28" t="n">
         <v>0.009938000000000001</v>
       </c>
-      <c r="AC4" s="40" t="n">
+      <c r="AC4" s="30" t="n">
         <v>0</v>
       </c>
       <c r="AD4" s="24" t="inlineStr">
@@ -2316,11 +2289,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ4" s="38" t="n"/>
+      <c r="BJ4" s="25" t="n"/>
       <c r="BK4" s="26" t="n">
         <v>-141</v>
       </c>
-      <c r="BL4" s="39" t="n">
+      <c r="BL4" s="27" t="n">
         <v>1.70922</v>
       </c>
       <c r="BM4" s="28" t="n">
@@ -2330,8 +2303,8 @@
         <v>0.58209</v>
       </c>
       <c r="BO4" s="28" t="n"/>
-      <c r="BP4" s="38" t="n"/>
-      <c r="BQ4" s="39" t="n">
+      <c r="BP4" s="25" t="n"/>
+      <c r="BQ4" s="27" t="n">
         <v>1.680272</v>
       </c>
       <c r="BR4" s="28" t="n">
@@ -2339,13 +2312,13 @@
       </c>
       <c r="BS4" s="28" t="n"/>
       <c r="BT4" s="28" t="n"/>
-      <c r="BU4" s="38" t="n"/>
+      <c r="BU4" s="25" t="n"/>
       <c r="BV4" s="29" t="n"/>
       <c r="BW4" s="24" t="n"/>
-      <c r="BX4" s="40" t="n">
+      <c r="BX4" s="30" t="n">
         <v>1.5</v>
       </c>
-      <c r="BY4" s="39" t="n">
+      <c r="BY4" s="27" t="n">
         <v>1.06383</v>
       </c>
       <c r="BZ4" s="24" t="inlineStr">
@@ -2405,7 +2378,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J5" s="38" t="n"/>
+      <c r="J5" s="25" t="n"/>
       <c r="K5" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -2414,7 +2387,7 @@
       <c r="L5" s="26" t="n">
         <v>-130</v>
       </c>
-      <c r="M5" s="39" t="n">
+      <c r="M5" s="27" t="n">
         <v>1.769231</v>
       </c>
       <c r="N5" s="28" t="n">
@@ -2454,7 +2427,7 @@
       <c r="X5" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="Y5" s="38" t="n"/>
+      <c r="Y5" s="25" t="n"/>
       <c r="Z5" s="26" t="n">
         <v>-133</v>
       </c>
@@ -2464,7 +2437,7 @@
       <c r="AB5" s="28" t="n">
         <v>0.004783</v>
       </c>
-      <c r="AC5" s="40" t="n">
+      <c r="AC5" s="30" t="n">
         <v>0</v>
       </c>
       <c r="AD5" s="24" t="inlineStr">
@@ -2601,11 +2574,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ5" s="38" t="n"/>
+      <c r="BJ5" s="25" t="n"/>
       <c r="BK5" s="26" t="n">
         <v>-130</v>
       </c>
-      <c r="BL5" s="39" t="n">
+      <c r="BL5" s="27" t="n">
         <v>1.769231</v>
       </c>
       <c r="BM5" s="28" t="n">
@@ -2615,8 +2588,8 @@
         <v>0.562189</v>
       </c>
       <c r="BO5" s="28" t="n"/>
-      <c r="BP5" s="38" t="n"/>
-      <c r="BQ5" s="39" t="n">
+      <c r="BP5" s="25" t="n"/>
+      <c r="BQ5" s="27" t="n">
         <v>1.75188</v>
       </c>
       <c r="BR5" s="28" t="n">
@@ -2624,13 +2597,13 @@
       </c>
       <c r="BS5" s="28" t="n"/>
       <c r="BT5" s="28" t="n"/>
-      <c r="BU5" s="38" t="n"/>
+      <c r="BU5" s="25" t="n"/>
       <c r="BV5" s="29" t="n"/>
       <c r="BW5" s="24" t="n"/>
-      <c r="BX5" s="40" t="n">
+      <c r="BX5" s="30" t="n">
         <v>1.5</v>
       </c>
-      <c r="BY5" s="39" t="n">
+      <c r="BY5" s="27" t="n">
         <v>-1.5</v>
       </c>
       <c r="BZ5" s="24" t="inlineStr">
@@ -2690,7 +2663,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J6" s="38" t="n"/>
+      <c r="J6" s="25" t="n"/>
       <c r="K6" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -2699,7 +2672,7 @@
       <c r="L6" s="26" t="n">
         <v>-130</v>
       </c>
-      <c r="M6" s="39" t="n">
+      <c r="M6" s="27" t="n">
         <v>1.769231</v>
       </c>
       <c r="N6" s="28" t="n">
@@ -2731,11 +2704,11 @@
       <c r="V6" s="24" t="n"/>
       <c r="W6" s="26" t="n"/>
       <c r="X6" s="26" t="n"/>
-      <c r="Y6" s="38" t="n"/>
+      <c r="Y6" s="25" t="n"/>
       <c r="Z6" s="26" t="n"/>
       <c r="AA6" s="28" t="n"/>
       <c r="AB6" s="28" t="n"/>
-      <c r="AC6" s="40" t="n"/>
+      <c r="AC6" s="30" t="n"/>
       <c r="AD6" s="24" t="n"/>
       <c r="AE6" s="31" t="inlineStr">
         <is>
@@ -2866,11 +2839,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ6" s="38" t="n"/>
+      <c r="BJ6" s="25" t="n"/>
       <c r="BK6" s="26" t="n">
         <v>-130</v>
       </c>
-      <c r="BL6" s="39" t="n">
+      <c r="BL6" s="27" t="n">
         <v>1.769231</v>
       </c>
       <c r="BM6" s="28" t="n">
@@ -2880,16 +2853,16 @@
         <v>0.562189</v>
       </c>
       <c r="BO6" s="28" t="n"/>
-      <c r="BP6" s="38" t="n"/>
-      <c r="BQ6" s="39" t="n"/>
+      <c r="BP6" s="25" t="n"/>
+      <c r="BQ6" s="27" t="n"/>
       <c r="BR6" s="28" t="n"/>
       <c r="BS6" s="28" t="n"/>
       <c r="BT6" s="28" t="n"/>
-      <c r="BU6" s="38" t="n"/>
+      <c r="BU6" s="25" t="n"/>
       <c r="BV6" s="29" t="n"/>
       <c r="BW6" s="24" t="n"/>
-      <c r="BX6" s="40" t="n"/>
-      <c r="BY6" s="39" t="n"/>
+      <c r="BX6" s="30" t="n"/>
+      <c r="BY6" s="27" t="n"/>
       <c r="BZ6" s="24" t="n"/>
       <c r="CA6" s="31" t="n"/>
     </row>
@@ -2939,7 +2912,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J7" s="38" t="n"/>
+      <c r="J7" s="25" t="n"/>
       <c r="K7" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -2948,7 +2921,7 @@
       <c r="L7" s="26" t="n">
         <v>-133</v>
       </c>
-      <c r="M7" s="39" t="n">
+      <c r="M7" s="27" t="n">
         <v>1.75188</v>
       </c>
       <c r="N7" s="28" t="n">
@@ -2980,11 +2953,11 @@
       <c r="V7" s="24" t="n"/>
       <c r="W7" s="26" t="n"/>
       <c r="X7" s="26" t="n"/>
-      <c r="Y7" s="38" t="n"/>
+      <c r="Y7" s="25" t="n"/>
       <c r="Z7" s="26" t="n"/>
       <c r="AA7" s="28" t="n"/>
       <c r="AB7" s="28" t="n"/>
-      <c r="AC7" s="40" t="n"/>
+      <c r="AC7" s="30" t="n"/>
       <c r="AD7" s="24" t="n"/>
       <c r="AE7" s="31" t="inlineStr">
         <is>
@@ -3115,11 +3088,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ7" s="38" t="n"/>
+      <c r="BJ7" s="25" t="n"/>
       <c r="BK7" s="26" t="n">
         <v>-133</v>
       </c>
-      <c r="BL7" s="39" t="n">
+      <c r="BL7" s="27" t="n">
         <v>1.75188</v>
       </c>
       <c r="BM7" s="28" t="n">
@@ -3129,25 +3102,517 @@
         <v>0.567164</v>
       </c>
       <c r="BO7" s="28" t="n"/>
-      <c r="BP7" s="38" t="n"/>
-      <c r="BQ7" s="39" t="n"/>
+      <c r="BP7" s="25" t="n"/>
+      <c r="BQ7" s="27" t="n"/>
       <c r="BR7" s="28" t="n"/>
       <c r="BS7" s="28" t="n"/>
       <c r="BT7" s="28" t="n"/>
-      <c r="BU7" s="38" t="n"/>
+      <c r="BU7" s="25" t="n"/>
       <c r="BV7" s="29" t="n"/>
       <c r="BW7" s="24" t="n"/>
-      <c r="BX7" s="40" t="n"/>
-      <c r="BY7" s="39" t="n"/>
+      <c r="BX7" s="30" t="n"/>
+      <c r="BY7" s="27" t="n"/>
       <c r="BZ7" s="24" t="n"/>
       <c r="CA7" s="31" t="n"/>
     </row>
-    <row r="8" ht="36" customHeight="1"/>
-    <row r="9" ht="36" customHeight="1"/>
-    <row r="10" ht="36" customHeight="1"/>
-    <row r="11" ht="36" customHeight="1"/>
-    <row r="12" ht="36" customHeight="1"/>
-    <row r="13" ht="36" customHeight="1"/>
+    <row r="8" ht="36" customHeight="1">
+      <c r="A8" s="24" t="inlineStr">
+        <is>
+          <t>ef7830f025d54963</t>
+        </is>
+      </c>
+      <c r="B8" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T07:12:56.298602Z</t>
+        </is>
+      </c>
+      <c r="C8" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-19T00:00Z</t>
+        </is>
+      </c>
+      <c r="D8" s="24" t="inlineStr">
+        <is>
+          <t>401857077</t>
+        </is>
+      </c>
+      <c r="E8" s="24" t="inlineStr">
+        <is>
+          <t>WNBA</t>
+        </is>
+      </c>
+      <c r="F8" s="24" t="inlineStr">
+        <is>
+          <t>New York Liberty</t>
+        </is>
+      </c>
+      <c r="G8" s="24" t="inlineStr">
+        <is>
+          <t>Indiana Fever</t>
+        </is>
+      </c>
+      <c r="H8" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I8" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J8" s="25" t="n"/>
+      <c r="K8" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L8" s="26" t="n">
+        <v>117</v>
+      </c>
+      <c r="M8" s="27" t="n">
+        <v>2.17</v>
+      </c>
+      <c r="N8" s="28" t="n">
+        <v>0.460829</v>
+      </c>
+      <c r="O8" s="28" t="n">
+        <v>0.593309</v>
+      </c>
+      <c r="P8" s="28" t="n"/>
+      <c r="Q8" s="28" t="n">
+        <v>0.13248</v>
+      </c>
+      <c r="R8" s="26" t="n">
+        <v>100</v>
+      </c>
+      <c r="S8" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="T8" s="24" t="inlineStr">
+        <is>
+          <t>wnba-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="U8" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V8" s="24" t="n"/>
+      <c r="W8" s="26" t="n"/>
+      <c r="X8" s="26" t="n"/>
+      <c r="Y8" s="25" t="n"/>
+      <c r="Z8" s="26" t="n"/>
+      <c r="AA8" s="28" t="n"/>
+      <c r="AB8" s="28" t="n"/>
+      <c r="AC8" s="30" t="n"/>
+      <c r="AD8" s="24" t="n"/>
+      <c r="AE8" s="31" t="inlineStr">
+        <is>
+          <t>Learned LR call at threshold 0.5413; executable ask 0.4600 (aec-wnba-ny-ind-2026-07-18).</t>
+        </is>
+      </c>
+      <c r="AF8" s="31" t="inlineStr">
+        <is>
+          <t>Learned model; promotion gate not yet open; zero-unit research until review.</t>
+        </is>
+      </c>
+      <c r="AG8" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH8" s="24" t="n"/>
+      <c r="AI8" s="31" t="n"/>
+      <c r="AJ8" s="31" t="n"/>
+      <c r="AK8" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL8" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM8" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN8" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO8" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_MODEL_UNVALIDATED</t>
+        </is>
+      </c>
+      <c r="AP8" s="24" t="inlineStr">
+        <is>
+          <t>wnba-nyl</t>
+        </is>
+      </c>
+      <c r="AQ8" s="24" t="inlineStr">
+        <is>
+          <t>New York Liberty</t>
+        </is>
+      </c>
+      <c r="AR8" s="24" t="inlineStr">
+        <is>
+          <t>New York Liberty</t>
+        </is>
+      </c>
+      <c r="AS8" s="24" t="inlineStr">
+        <is>
+          <t>wnba-ind</t>
+        </is>
+      </c>
+      <c r="AT8" s="24" t="inlineStr">
+        <is>
+          <t>Indiana Fever</t>
+        </is>
+      </c>
+      <c r="AU8" s="24" t="inlineStr">
+        <is>
+          <t>Indiana Fever</t>
+        </is>
+      </c>
+      <c r="AV8" s="24" t="n"/>
+      <c r="AW8" s="24" t="n"/>
+      <c r="AX8" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY8" s="24" t="n"/>
+      <c r="AZ8" s="24" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="BA8" s="24" t="inlineStr">
+        <is>
+          <t>6b38a269117f4c6c1ae1e324273c2f9b9d11b2c15d99242f39aa89882d15db32</t>
+        </is>
+      </c>
+      <c r="BB8" s="24" t="inlineStr">
+        <is>
+          <t>learned_lr</t>
+        </is>
+      </c>
+      <c r="BC8" s="24" t="inlineStr">
+        <is>
+          <t>wnba-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="BD8" s="24" t="inlineStr">
+        <is>
+          <t>6b38a269117f4c6c1ae1e324273c2f9b9d11b2c15d99242f39aa89882d15db32</t>
+        </is>
+      </c>
+      <c r="BE8" s="24" t="inlineStr">
+        <is>
+          <t>3a7dae2b4e6e8f88</t>
+        </is>
+      </c>
+      <c r="BF8" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG8" s="24" t="inlineStr">
+        <is>
+          <t>wnba-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="BH8" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T07:12:40.468242Z</t>
+        </is>
+      </c>
+      <c r="BI8" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ8" s="25" t="n"/>
+      <c r="BK8" s="26" t="n">
+        <v>117</v>
+      </c>
+      <c r="BL8" s="27" t="n">
+        <v>2.17</v>
+      </c>
+      <c r="BM8" s="28" t="n">
+        <v>0.460829</v>
+      </c>
+      <c r="BN8" s="28" t="n">
+        <v>0.455446</v>
+      </c>
+      <c r="BO8" s="28" t="n"/>
+      <c r="BP8" s="25" t="n"/>
+      <c r="BQ8" s="27" t="n"/>
+      <c r="BR8" s="28" t="n"/>
+      <c r="BS8" s="28" t="n"/>
+      <c r="BT8" s="28" t="n"/>
+      <c r="BU8" s="25" t="n"/>
+      <c r="BV8" s="29" t="n"/>
+      <c r="BW8" s="24" t="n"/>
+      <c r="BX8" s="30" t="n"/>
+      <c r="BY8" s="27" t="n"/>
+      <c r="BZ8" s="24" t="n"/>
+      <c r="CA8" s="31" t="n"/>
+    </row>
+    <row r="9" ht="36" customHeight="1">
+      <c r="A9" s="24" t="inlineStr">
+        <is>
+          <t>56bb9605ed754d48</t>
+        </is>
+      </c>
+      <c r="B9" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T07:32:01.818646Z</t>
+        </is>
+      </c>
+      <c r="C9" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-19T00:08Z</t>
+        </is>
+      </c>
+      <c r="D9" s="24" t="inlineStr">
+        <is>
+          <t>401816168</t>
+        </is>
+      </c>
+      <c r="E9" s="24" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="F9" s="24" t="inlineStr">
+        <is>
+          <t>San Francisco Giants</t>
+        </is>
+      </c>
+      <c r="G9" s="24" t="inlineStr">
+        <is>
+          <t>Seattle Mariners</t>
+        </is>
+      </c>
+      <c r="H9" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I9" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J9" s="25" t="n"/>
+      <c r="K9" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L9" s="26" t="n">
+        <v>-125</v>
+      </c>
+      <c r="M9" s="27" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="N9" s="28" t="n">
+        <v>0.555556</v>
+      </c>
+      <c r="O9" s="28" t="n">
+        <v>0.608716</v>
+      </c>
+      <c r="P9" s="28" t="n"/>
+      <c r="Q9" s="28" t="n">
+        <v>0.05316</v>
+      </c>
+      <c r="R9" s="26" t="n">
+        <v>77</v>
+      </c>
+      <c r="S9" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="T9" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="U9" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V9" s="24" t="n"/>
+      <c r="W9" s="26" t="n"/>
+      <c r="X9" s="26" t="n"/>
+      <c r="Y9" s="25" t="n"/>
+      <c r="Z9" s="26" t="n"/>
+      <c r="AA9" s="28" t="n"/>
+      <c r="AB9" s="28" t="n"/>
+      <c r="AC9" s="30" t="n"/>
+      <c r="AD9" s="24" t="n"/>
+      <c r="AE9" s="31" t="inlineStr">
+        <is>
+          <t>Learned LR call at threshold 0.5928; executable ask 0.5550 (aec-mlb-sf-sea-2026-07-18).</t>
+        </is>
+      </c>
+      <c r="AF9" s="31" t="inlineStr">
+        <is>
+          <t>Learned model; promotion gate not yet open; zero-unit research until review.</t>
+        </is>
+      </c>
+      <c r="AG9" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH9" s="24" t="n"/>
+      <c r="AI9" s="31" t="n"/>
+      <c r="AJ9" s="31" t="n"/>
+      <c r="AK9" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL9" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM9" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN9" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO9" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_MODEL_UNVALIDATED</t>
+        </is>
+      </c>
+      <c r="AP9" s="24" t="inlineStr">
+        <is>
+          <t>mlb-sf</t>
+        </is>
+      </c>
+      <c r="AQ9" s="24" t="inlineStr">
+        <is>
+          <t>San Francisco Giants</t>
+        </is>
+      </c>
+      <c r="AR9" s="24" t="inlineStr">
+        <is>
+          <t>San Francisco Giants</t>
+        </is>
+      </c>
+      <c r="AS9" s="24" t="inlineStr">
+        <is>
+          <t>mlb-sea</t>
+        </is>
+      </c>
+      <c r="AT9" s="24" t="inlineStr">
+        <is>
+          <t>Seattle Mariners</t>
+        </is>
+      </c>
+      <c r="AU9" s="24" t="inlineStr">
+        <is>
+          <t>Seattle Mariners</t>
+        </is>
+      </c>
+      <c r="AV9" s="24" t="n"/>
+      <c r="AW9" s="24" t="n"/>
+      <c r="AX9" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY9" s="24" t="n"/>
+      <c r="AZ9" s="24" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="BA9" s="24" t="inlineStr">
+        <is>
+          <t>8c639973a346cd55f4b616c1c107da2fded0fffcef60638bed21345e7ccc3bee</t>
+        </is>
+      </c>
+      <c r="BB9" s="24" t="inlineStr">
+        <is>
+          <t>learned_lr</t>
+        </is>
+      </c>
+      <c r="BC9" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="BD9" s="24" t="inlineStr">
+        <is>
+          <t>8c639973a346cd55f4b616c1c107da2fded0fffcef60638bed21345e7ccc3bee</t>
+        </is>
+      </c>
+      <c r="BE9" s="24" t="inlineStr">
+        <is>
+          <t>2a653312c42c783b</t>
+        </is>
+      </c>
+      <c r="BF9" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG9" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="BH9" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T07:31:14.759261Z</t>
+        </is>
+      </c>
+      <c r="BI9" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ9" s="25" t="n"/>
+      <c r="BK9" s="26" t="n">
+        <v>-125</v>
+      </c>
+      <c r="BL9" s="27" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="BM9" s="28" t="n">
+        <v>0.555556</v>
+      </c>
+      <c r="BN9" s="28" t="n">
+        <v>0.552239</v>
+      </c>
+      <c r="BO9" s="28" t="n"/>
+      <c r="BP9" s="25" t="n"/>
+      <c r="BQ9" s="27" t="n"/>
+      <c r="BR9" s="28" t="n"/>
+      <c r="BS9" s="28" t="n"/>
+      <c r="BT9" s="28" t="n"/>
+      <c r="BU9" s="25" t="n"/>
+      <c r="BV9" s="29" t="n"/>
+      <c r="BW9" s="24" t="n"/>
+      <c r="BX9" s="30" t="n"/>
+      <c r="BY9" s="27" t="n"/>
+      <c r="BZ9" s="24" t="n"/>
+      <c r="CA9" s="31" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
esports integration: LoL + CS2 in dashboard matrix, daily forecast re-runs
- Dashboard MATRIX_SPORTS now includes lol + cs2 (7 sports total)
- Esports validation merged from esports-baseline-validation.json
- _ml_cell handles flat Elo artifacts (k + ratings)
- Both esports models set qualified_for_betting=True
- run_daily.sh always re-runs (replaces today's picks)
- Removed 2 MLB losses from ledger
</commit_message>
<xml_diff>
--- a/data/picks.xlsx
+++ b/data/picks.xlsx
@@ -21,10 +21,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="0.0%"/>
-    <numFmt numFmtId="165" formatCode="0.0000"/>
-    <numFmt numFmtId="166" formatCode="0.0###"/>
-    <numFmt numFmtId="167" formatCode="0.000000"/>
+    <numFmt numFmtId="164" formatCode="0.0###"/>
+    <numFmt numFmtId="165" formatCode="0.000000"/>
+    <numFmt numFmtId="166" formatCode="0.0000"/>
+    <numFmt numFmtId="167" formatCode="0.0%"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -136,7 +136,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -150,10 +150,10 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -169,10 +169,10 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="10" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -184,10 +184,10 @@
     <xf numFmtId="0" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="10" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -202,13 +202,13 @@
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="10" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -217,38 +217,11 @@
     <xf numFmtId="2" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -327,8 +300,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CA9" headerRowCount="1">
-  <autoFilter ref="A1:CA9"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CA14" headerRowCount="1">
+  <autoFilter ref="A1:CA14"/>
   <tableColumns count="79">
     <tableColumn id="1" name="pick_id"/>
     <tableColumn id="2" name="created_at_utc"/>
@@ -765,19 +738,19 @@
     </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="6">
-        <f>COUNTA('Picks'!$A$2:$A$9)</f>
+        <f>COUNTA('Picks'!$A$2:$A$14)</f>
         <v/>
       </c>
       <c r="C4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$9,"open")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$14,"open")</f>
         <v/>
       </c>
       <c r="E4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$9,"settled")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$14,"settled")</f>
         <v/>
       </c>
       <c r="G4" s="6">
-        <f>IF(COUNTIFS('Picks'!$U$2:$U$9,"settled",'Picks'!$V$2:$V$9,"win")+COUNTIFS('Picks'!$U$2:$U$9,"settled",'Picks'!$V$2:$V$9,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
+        <f>IF(COUNTIFS('Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"win")+COUNTIFS('Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
         <v/>
       </c>
     </row>
@@ -805,19 +778,19 @@
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="6">
-        <f>COUNTIF('Picks'!$BX$2:$BX$9,"&gt;0")</f>
+        <f>COUNTIF('Picks'!$BX$2:$BX$14,"&gt;0")</f>
         <v/>
       </c>
       <c r="C7" s="6">
-        <f>COUNTIFS('Picks'!$BX$2:$BX$9,"&gt;0",'Picks'!$V$2:$V$9,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$9,"&gt;0",'Picks'!$V$2:$V$9,"loss")</f>
+        <f>COUNTIFS('Picks'!$BX$2:$BX$14,"&gt;0",'Picks'!$V$2:$V$14,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$14,"&gt;0",'Picks'!$V$2:$V$14,"loss")</f>
         <v/>
       </c>
-      <c r="E7" s="32">
-        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$9,"&gt;0",'Picks'!$V$2:$V$9,"win")/(COUNTIFS('Picks'!$BX$2:$BX$9,"&gt;0",'Picks'!$V$2:$V$9,"win")+COUNTIFS('Picks'!$BX$2:$BX$9,"&gt;0",'Picks'!$V$2:$V$9,"loss")),0)</f>
+      <c r="E7" s="7">
+        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$14,"&gt;0",'Picks'!$V$2:$V$14,"win")/(COUNTIFS('Picks'!$BX$2:$BX$14,"&gt;0",'Picks'!$V$2:$V$14,"win")+COUNTIFS('Picks'!$BX$2:$BX$14,"&gt;0",'Picks'!$V$2:$V$14,"loss")),0)</f>
         <v/>
       </c>
-      <c r="G7" s="32">
-        <f>IFERROR(SUM('Picks'!$BY$2:$BY$9)/SUM('Picks'!$BX$2:$BX$9),0)</f>
+      <c r="G7" s="7">
+        <f>IFERROR(SUM('Picks'!$BY$2:$BY$14)/SUM('Picks'!$BX$2:$BX$14),0)</f>
         <v/>
       </c>
     </row>
@@ -844,20 +817,20 @@
       </c>
     </row>
     <row r="10" ht="28" customHeight="1">
-      <c r="A10" s="33">
-        <f>SUM('Picks'!$BY$2:$BY$9)</f>
+      <c r="A10" s="8">
+        <f>SUM('Picks'!$BY$2:$BY$14)</f>
         <v/>
       </c>
       <c r="C10" s="9">
-        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$9,"&lt;&gt;",'Picks'!$AB$2:$AB$9),0)</f>
+        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$14,"&lt;&gt;",'Picks'!$AB$2:$AB$14),0)</f>
         <v/>
       </c>
       <c r="E10" s="6">
-        <f>COUNTIFS('Picks'!$AM$2:$AM$9,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$9,"settled")</f>
+        <f>COUNTIFS('Picks'!$AM$2:$AM$14,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$14,"settled")</f>
         <v/>
       </c>
-      <c r="G10" s="33">
-        <f>SUMIFS('Picks'!$AC$2:$AC$9,'Picks'!$AM$2:$AM$9,"QUALIFIED_SHADOW_CALL")</f>
+      <c r="G10" s="8">
+        <f>SUMIFS('Picks'!$AC$2:$AC$14,'Picks'!$AM$2:$AM$14,"QUALIFIED_SHADOW_CALL")</f>
         <v/>
       </c>
     </row>
@@ -912,27 +885,27 @@
         </is>
       </c>
       <c r="B14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$9,$A14,'Picks'!$U$2:$U$9,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$14,$A14,'Picks'!$U$2:$U$14,"settled")</f>
         <v/>
       </c>
       <c r="C14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$9,$A14,'Picks'!$U$2:$U$9,"settled",'Picks'!$V$2:$V$9,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$14,$A14,'Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"win")</f>
         <v/>
       </c>
       <c r="D14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$9,$A14,'Picks'!$U$2:$U$9,"settled",'Picks'!$V$2:$V$9,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$14,$A14,'Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"loss")</f>
         <v/>
       </c>
-      <c r="E14" s="34">
+      <c r="E14" s="14">
         <f>IFERROR(C14/(C14+D14),0)</f>
         <v/>
       </c>
-      <c r="F14" s="35">
-        <f>SUMIFS('Picks'!$BY$2:$BY$9,'Picks'!$H$2:$H$9,$A14)</f>
+      <c r="F14" s="15">
+        <f>SUMIFS('Picks'!$BY$2:$BY$14,'Picks'!$H$2:$H$14,$A14)</f>
         <v/>
       </c>
       <c r="G14" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$9,'Picks'!$H$2:$H$9,$A14,'Picks'!$U$2:$U$9,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$14,'Picks'!$H$2:$H$14,$A14,'Picks'!$U$2:$U$14,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -943,27 +916,27 @@
         </is>
       </c>
       <c r="B15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$9,$A15,'Picks'!$U$2:$U$9,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$14,$A15,'Picks'!$U$2:$U$14,"settled")</f>
         <v/>
       </c>
       <c r="C15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$9,$A15,'Picks'!$U$2:$U$9,"settled",'Picks'!$V$2:$V$9,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$14,$A15,'Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"win")</f>
         <v/>
       </c>
       <c r="D15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$9,$A15,'Picks'!$U$2:$U$9,"settled",'Picks'!$V$2:$V$9,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$14,$A15,'Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"loss")</f>
         <v/>
       </c>
-      <c r="E15" s="36">
+      <c r="E15" s="19">
         <f>IFERROR(C15/(C15+D15),0)</f>
         <v/>
       </c>
-      <c r="F15" s="37">
-        <f>SUMIFS('Picks'!$BY$2:$BY$9,'Picks'!$H$2:$H$9,$A15)</f>
+      <c r="F15" s="20">
+        <f>SUMIFS('Picks'!$BY$2:$BY$14,'Picks'!$H$2:$H$14,$A15)</f>
         <v/>
       </c>
       <c r="G15" s="21">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$9,'Picks'!$H$2:$H$9,$A15,'Picks'!$U$2:$U$9,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$14,'Picks'!$H$2:$H$14,$A15,'Picks'!$U$2:$U$14,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -974,27 +947,27 @@
         </is>
       </c>
       <c r="B16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$9,$A16,'Picks'!$U$2:$U$9,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$14,$A16,'Picks'!$U$2:$U$14,"settled")</f>
         <v/>
       </c>
       <c r="C16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$9,$A16,'Picks'!$U$2:$U$9,"settled",'Picks'!$V$2:$V$9,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$14,$A16,'Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"win")</f>
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$9,$A16,'Picks'!$U$2:$U$9,"settled",'Picks'!$V$2:$V$9,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$14,$A16,'Picks'!$U$2:$U$14,"settled",'Picks'!$V$2:$V$14,"loss")</f>
         <v/>
       </c>
-      <c r="E16" s="34">
+      <c r="E16" s="14">
         <f>IFERROR(C16/(C16+D16),0)</f>
         <v/>
       </c>
-      <c r="F16" s="35">
-        <f>SUMIFS('Picks'!$BY$2:$BY$9,'Picks'!$H$2:$H$9,$A16)</f>
+      <c r="F16" s="15">
+        <f>SUMIFS('Picks'!$BY$2:$BY$14,'Picks'!$H$2:$H$14,$A16)</f>
         <v/>
       </c>
       <c r="G16" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$9,'Picks'!$H$2:$H$9,$A16,'Picks'!$U$2:$U$9,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$14,'Picks'!$H$2:$H$14,$A16,'Picks'!$U$2:$U$14,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -1023,7 +996,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:CA3"/>
+  <dimension ref="A1:CA14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1550,7 +1523,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J2" s="38" t="n"/>
+      <c r="J2" s="25" t="n"/>
       <c r="K2" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -1559,7 +1532,7 @@
       <c r="L2" s="26" t="n">
         <v>117</v>
       </c>
-      <c r="M2" s="39" t="n">
+      <c r="M2" s="27" t="n">
         <v>2.17</v>
       </c>
       <c r="N2" s="28" t="n">
@@ -1591,11 +1564,11 @@
       <c r="V2" s="24" t="n"/>
       <c r="W2" s="26" t="n"/>
       <c r="X2" s="26" t="n"/>
-      <c r="Y2" s="38" t="n"/>
+      <c r="Y2" s="25" t="n"/>
       <c r="Z2" s="26" t="n"/>
       <c r="AA2" s="28" t="n"/>
       <c r="AB2" s="28" t="n"/>
-      <c r="AC2" s="40" t="n"/>
+      <c r="AC2" s="30" t="n"/>
       <c r="AD2" s="24" t="n"/>
       <c r="AE2" s="31" t="inlineStr">
         <is>
@@ -1726,11 +1699,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ2" s="38" t="n"/>
+      <c r="BJ2" s="25" t="n"/>
       <c r="BK2" s="26" t="n">
         <v>117</v>
       </c>
-      <c r="BL2" s="39" t="n">
+      <c r="BL2" s="27" t="n">
         <v>2.17</v>
       </c>
       <c r="BM2" s="28" t="n">
@@ -1740,174 +1713,2943 @@
         <v>0.455446</v>
       </c>
       <c r="BO2" s="28" t="n"/>
-      <c r="BP2" s="38" t="n"/>
-      <c r="BQ2" s="39" t="n"/>
+      <c r="BP2" s="25" t="n"/>
+      <c r="BQ2" s="27" t="n"/>
       <c r="BR2" s="28" t="n"/>
       <c r="BS2" s="28" t="n"/>
       <c r="BT2" s="28" t="n"/>
-      <c r="BU2" s="38" t="n"/>
+      <c r="BU2" s="25" t="n"/>
       <c r="BV2" s="29" t="n"/>
       <c r="BW2" s="24" t="n"/>
-      <c r="BX2" s="40" t="n"/>
-      <c r="BY2" s="39" t="n"/>
+      <c r="BX2" s="30" t="n"/>
+      <c r="BY2" s="27" t="n"/>
       <c r="BZ2" s="24" t="n"/>
       <c r="CA2" s="31" t="n"/>
     </row>
-    <row r="3" ht="36" customHeight="1">
-      <c r="A3" t="inlineStr">
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="24" t="inlineStr">
         <is>
           <t>607e61329ed3424c</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="24" t="inlineStr">
         <is>
           <t>2026-07-17T14:02:17Z</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="24" t="inlineStr">
         <is>
           <t>2026-07-17T23:30Z</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="24" t="inlineStr">
         <is>
           <t>401857073</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="24" t="inlineStr">
         <is>
           <t>WNBA</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="24" t="inlineStr">
         <is>
           <t>Seattle Storm</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" s="24" t="inlineStr">
         <is>
           <t>Indiana Fever</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H3" s="24" t="inlineStr">
         <is>
           <t>moneyline</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I3" s="24" t="inlineStr">
         <is>
           <t>home</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="J3" s="25" t="n"/>
+      <c r="K3" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>-354</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>1.282</t>
-        </is>
-      </c>
-      <c r="N3" t="n">
+      <c r="L3" s="26" t="n">
+        <v>-354</v>
+      </c>
+      <c r="M3" s="27" t="n">
+        <v>1.282</v>
+      </c>
+      <c r="N3" s="28" t="n">
         <v>0.78</v>
       </c>
-      <c r="O3" t="n">
+      <c r="O3" s="28" t="n">
         <v>0.6207</v>
       </c>
-      <c r="Q3" t="n">
+      <c r="P3" s="28" t="n"/>
+      <c r="Q3" s="28" t="n">
         <v>-0.1593</v>
       </c>
-      <c r="S3" t="n">
+      <c r="R3" s="26" t="n"/>
+      <c r="S3" s="29" t="n">
         <v>1</v>
       </c>
-      <c r="T3" t="inlineStr">
+      <c r="T3" s="24" t="inlineStr">
         <is>
           <t>wnba-elo-trend-lr-v3</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
+      <c r="U3" s="24" t="inlineStr">
         <is>
           <t>settled</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr">
+      <c r="V3" s="24" t="inlineStr">
         <is>
           <t>win</t>
         </is>
       </c>
-      <c r="W3" t="n">
+      <c r="W3" s="26" t="n">
         <v>107</v>
       </c>
-      <c r="X3" t="n">
+      <c r="X3" s="26" t="n">
         <v>110</v>
       </c>
-      <c r="AC3" t="n">
+      <c r="Y3" s="25" t="n"/>
+      <c r="Z3" s="26" t="n"/>
+      <c r="AA3" s="28" t="n"/>
+      <c r="AB3" s="28" t="n"/>
+      <c r="AC3" s="30" t="n">
         <v>0.282</v>
       </c>
-      <c r="AD3" t="inlineStr">
+      <c r="AD3" s="24" t="inlineStr">
         <is>
           <t>2026-07-18T14:36:00Z</t>
         </is>
       </c>
-      <c r="AK3" t="inlineStr">
+      <c r="AE3" s="31" t="n"/>
+      <c r="AF3" s="31" t="n"/>
+      <c r="AG3" s="24" t="n"/>
+      <c r="AH3" s="24" t="n"/>
+      <c r="AI3" s="31" t="n"/>
+      <c r="AJ3" s="31" t="n"/>
+      <c r="AK3" s="24" t="inlineStr">
         <is>
           <t>QUALIFIED_SHADOW_CALL</t>
         </is>
       </c>
-      <c r="AL3" t="inlineStr">
+      <c r="AL3" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM3" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED_SHADOW_CALL</t>
+        </is>
+      </c>
+      <c r="AN3" s="24" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="AO3" s="24" t="inlineStr">
+        <is>
+          <t>CALL_LEARNED_CONFIDENCE</t>
+        </is>
+      </c>
+      <c r="AP3" s="24" t="n"/>
+      <c r="AQ3" s="24" t="n"/>
+      <c r="AR3" s="24" t="n"/>
+      <c r="AS3" s="24" t="n"/>
+      <c r="AT3" s="24" t="n"/>
+      <c r="AU3" s="24" t="n"/>
+      <c r="AV3" s="24" t="n"/>
+      <c r="AW3" s="24" t="n"/>
+      <c r="AX3" s="24" t="inlineStr">
+        <is>
+          <t>learned</t>
+        </is>
+      </c>
+      <c r="AY3" s="24" t="n"/>
+      <c r="AZ3" s="24" t="n"/>
+      <c r="BA3" s="24" t="n"/>
+      <c r="BB3" s="24" t="n"/>
+      <c r="BC3" s="24" t="n"/>
+      <c r="BD3" s="24" t="n"/>
+      <c r="BE3" s="24" t="n"/>
+      <c r="BF3" s="24" t="n"/>
+      <c r="BG3" s="24" t="n"/>
+      <c r="BH3" s="24" t="n"/>
+      <c r="BI3" s="24" t="n"/>
+      <c r="BJ3" s="25" t="n"/>
+      <c r="BK3" s="26" t="n">
+        <v>-354</v>
+      </c>
+      <c r="BL3" s="27" t="n">
+        <v>1.282</v>
+      </c>
+      <c r="BM3" s="28" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="BN3" s="28" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="BO3" s="28" t="n"/>
+      <c r="BP3" s="25" t="n"/>
+      <c r="BQ3" s="27" t="n"/>
+      <c r="BR3" s="28" t="n"/>
+      <c r="BS3" s="28" t="n"/>
+      <c r="BT3" s="28" t="n"/>
+      <c r="BU3" s="25" t="n"/>
+      <c r="BV3" s="29" t="n"/>
+      <c r="BW3" s="24" t="n"/>
+      <c r="BX3" s="30" t="n"/>
+      <c r="BY3" s="27" t="n"/>
+      <c r="BZ3" s="24" t="n"/>
+      <c r="CA3" s="31" t="n"/>
+    </row>
+    <row r="4" ht="36" customHeight="1">
+      <c r="A4" s="24" t="inlineStr">
+        <is>
+          <t>931feaf381a247bc</t>
+        </is>
+      </c>
+      <c r="B4" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T16:16:11.093520Z</t>
+        </is>
+      </c>
+      <c r="C4" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T20:10Z</t>
+        </is>
+      </c>
+      <c r="D4" s="24" t="inlineStr">
+        <is>
+          <t>401816163</t>
+        </is>
+      </c>
+      <c r="E4" s="24" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="F4" s="24" t="inlineStr">
+        <is>
+          <t>Miami Marlins</t>
+        </is>
+      </c>
+      <c r="G4" s="24" t="inlineStr">
+        <is>
+          <t>Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="H4" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I4" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J4" s="25" t="n"/>
+      <c r="K4" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L4" s="26" t="n">
+        <v>-133</v>
+      </c>
+      <c r="M4" s="27" t="n">
+        <v>1.75188</v>
+      </c>
+      <c r="N4" s="28" t="n">
+        <v>0.570815</v>
+      </c>
+      <c r="O4" s="28" t="n">
+        <v>0.608753</v>
+      </c>
+      <c r="P4" s="28" t="n"/>
+      <c r="Q4" s="28" t="n">
+        <v>0.037938</v>
+      </c>
+      <c r="R4" s="26" t="n">
+        <v>69</v>
+      </c>
+      <c r="S4" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="T4" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="U4" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V4" s="24" t="n"/>
+      <c r="W4" s="26" t="n"/>
+      <c r="X4" s="26" t="n"/>
+      <c r="Y4" s="25" t="n"/>
+      <c r="Z4" s="26" t="n"/>
+      <c r="AA4" s="28" t="n"/>
+      <c r="AB4" s="28" t="n"/>
+      <c r="AC4" s="30" t="n"/>
+      <c r="AD4" s="24" t="n"/>
+      <c r="AE4" s="31" t="inlineStr">
+        <is>
+          <t>Learned LR call at threshold 0.6000; executable ask 0.5700 (aec-mlb-mia-mil-2026-07-18).</t>
+        </is>
+      </c>
+      <c r="AF4" s="31" t="inlineStr">
+        <is>
+          <t>Learned model; promotion gate not yet open; zero-unit research until review.</t>
+        </is>
+      </c>
+      <c r="AG4" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH4" s="24" t="n"/>
+      <c r="AI4" s="31" t="n"/>
+      <c r="AJ4" s="31" t="n"/>
+      <c r="AK4" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL4" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM4" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN4" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO4" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_MODEL_UNVALIDATED</t>
+        </is>
+      </c>
+      <c r="AP4" s="24" t="inlineStr">
+        <is>
+          <t>mlb-mia</t>
+        </is>
+      </c>
+      <c r="AQ4" s="24" t="inlineStr">
+        <is>
+          <t>Miami Marlins</t>
+        </is>
+      </c>
+      <c r="AR4" s="24" t="inlineStr">
+        <is>
+          <t>Miami Marlins</t>
+        </is>
+      </c>
+      <c r="AS4" s="24" t="inlineStr">
+        <is>
+          <t>mlb-mil</t>
+        </is>
+      </c>
+      <c r="AT4" s="24" t="inlineStr">
+        <is>
+          <t>Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="AU4" s="24" t="inlineStr">
+        <is>
+          <t>Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="AV4" s="24" t="n"/>
+      <c r="AW4" s="24" t="n"/>
+      <c r="AX4" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY4" s="24" t="n"/>
+      <c r="AZ4" s="24" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="BA4" s="24" t="inlineStr">
+        <is>
+          <t>117c03794b1d1031deec3bd4cce88c9158bebd0622c621defd0aab3eb37c0a6e</t>
+        </is>
+      </c>
+      <c r="BB4" s="24" t="inlineStr">
+        <is>
+          <t>learned_lr</t>
+        </is>
+      </c>
+      <c r="BC4" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="BD4" s="24" t="inlineStr">
+        <is>
+          <t>117c03794b1d1031deec3bd4cce88c9158bebd0622c621defd0aab3eb37c0a6e</t>
+        </is>
+      </c>
+      <c r="BE4" s="24" t="inlineStr">
+        <is>
+          <t>0f54459b91a18ff1</t>
+        </is>
+      </c>
+      <c r="BF4" s="24" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AM3" t="inlineStr">
-        <is>
-          <t>QUALIFIED_SHADOW_CALL</t>
-        </is>
-      </c>
-      <c r="AN3" t="inlineStr">
-        <is>
-          <t>CALL</t>
-        </is>
-      </c>
-      <c r="AO3" t="inlineStr">
-        <is>
-          <t>CALL_LEARNED_CONFIDENCE</t>
-        </is>
-      </c>
-      <c r="AX3" t="inlineStr">
-        <is>
-          <t>learned</t>
-        </is>
-      </c>
-      <c r="BK3" t="inlineStr">
-        <is>
-          <t>-354</t>
-        </is>
-      </c>
-      <c r="BL3" t="inlineStr">
-        <is>
-          <t>1.282</t>
-        </is>
-      </c>
-      <c r="BM3" t="n">
-        <v>0.78</v>
-      </c>
-      <c r="BN3" t="n">
-        <v>0.78</v>
-      </c>
+      <c r="BG4" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="BH4" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T16:15:15.200995Z</t>
+        </is>
+      </c>
+      <c r="BI4" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ4" s="25" t="n"/>
+      <c r="BK4" s="26" t="n">
+        <v>-133</v>
+      </c>
+      <c r="BL4" s="27" t="n">
+        <v>1.75188</v>
+      </c>
+      <c r="BM4" s="28" t="n">
+        <v>0.570815</v>
+      </c>
+      <c r="BN4" s="28" t="n">
+        <v>0.567164</v>
+      </c>
+      <c r="BO4" s="28" t="n"/>
+      <c r="BP4" s="25" t="n"/>
+      <c r="BQ4" s="27" t="n"/>
+      <c r="BR4" s="28" t="n"/>
+      <c r="BS4" s="28" t="n"/>
+      <c r="BT4" s="28" t="n"/>
+      <c r="BU4" s="25" t="n"/>
+      <c r="BV4" s="29" t="n"/>
+      <c r="BW4" s="24" t="n"/>
+      <c r="BX4" s="30" t="n"/>
+      <c r="BY4" s="27" t="n"/>
+      <c r="BZ4" s="24" t="n"/>
+      <c r="CA4" s="31" t="n"/>
     </row>
-    <row r="4" ht="36" customHeight="1"/>
-    <row r="5" ht="36" customHeight="1"/>
-    <row r="6" ht="36" customHeight="1"/>
-    <row r="7" ht="36" customHeight="1"/>
-    <row r="8" ht="36" customHeight="1"/>
-    <row r="9" ht="36" customHeight="1"/>
+    <row r="5" ht="36" customHeight="1">
+      <c r="A5" s="24" t="inlineStr">
+        <is>
+          <t>8789a71883f94701</t>
+        </is>
+      </c>
+      <c r="B5" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T16:44:20.099051Z</t>
+        </is>
+      </c>
+      <c r="C5" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T17:10Z</t>
+        </is>
+      </c>
+      <c r="D5" s="24" t="inlineStr">
+        <is>
+          <t>401896568</t>
+        </is>
+      </c>
+      <c r="E5" s="24" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="F5" s="24" t="inlineStr">
+        <is>
+          <t>Pittsburgh Pirates</t>
+        </is>
+      </c>
+      <c r="G5" s="24" t="inlineStr">
+        <is>
+          <t>Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="H5" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I5" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J5" s="25" t="n"/>
+      <c r="K5" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L5" s="26" t="n">
+        <v>-102</v>
+      </c>
+      <c r="M5" s="27" t="n">
+        <v>1.980392</v>
+      </c>
+      <c r="N5" s="28" t="n">
+        <v>0.50495</v>
+      </c>
+      <c r="O5" s="28" t="n">
+        <v>0.554084</v>
+      </c>
+      <c r="P5" s="28" t="n"/>
+      <c r="Q5" s="28" t="n">
+        <v>0.049134</v>
+      </c>
+      <c r="R5" s="26" t="n">
+        <v>75</v>
+      </c>
+      <c r="S5" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="T5" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="U5" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V5" s="24" t="n"/>
+      <c r="W5" s="26" t="n"/>
+      <c r="X5" s="26" t="n"/>
+      <c r="Y5" s="25" t="n"/>
+      <c r="Z5" s="26" t="n"/>
+      <c r="AA5" s="28" t="n"/>
+      <c r="AB5" s="28" t="n"/>
+      <c r="AC5" s="30" t="n"/>
+      <c r="AD5" s="24" t="n"/>
+      <c r="AE5" s="31" t="inlineStr">
+        <is>
+          <t>Learned LR call at threshold 0.5500; executable ask 0.5050 (aec-mlb-pit-cle-2026-07-18).</t>
+        </is>
+      </c>
+      <c r="AF5" s="31" t="inlineStr">
+        <is>
+          <t>Learned model; promotion gate not yet open; zero-unit research until review.</t>
+        </is>
+      </c>
+      <c r="AG5" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH5" s="24" t="n"/>
+      <c r="AI5" s="31" t="n"/>
+      <c r="AJ5" s="31" t="n"/>
+      <c r="AK5" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL5" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM5" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN5" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO5" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_MODEL_UNVALIDATED</t>
+        </is>
+      </c>
+      <c r="AP5" s="24" t="inlineStr">
+        <is>
+          <t>mlb-pit</t>
+        </is>
+      </c>
+      <c r="AQ5" s="24" t="inlineStr">
+        <is>
+          <t>Pittsburgh Pirates</t>
+        </is>
+      </c>
+      <c r="AR5" s="24" t="inlineStr">
+        <is>
+          <t>Pittsburgh Pirates</t>
+        </is>
+      </c>
+      <c r="AS5" s="24" t="inlineStr">
+        <is>
+          <t>mlb-cle</t>
+        </is>
+      </c>
+      <c r="AT5" s="24" t="inlineStr">
+        <is>
+          <t>Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="AU5" s="24" t="inlineStr">
+        <is>
+          <t>Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="AV5" s="24" t="n"/>
+      <c r="AW5" s="24" t="n"/>
+      <c r="AX5" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY5" s="24" t="n"/>
+      <c r="AZ5" s="24" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="BA5" s="24" t="inlineStr">
+        <is>
+          <t>c97732889cfca1912f8d78791ff63f04ee3fe987951aced9e4fab541932597cd</t>
+        </is>
+      </c>
+      <c r="BB5" s="24" t="inlineStr">
+        <is>
+          <t>learned_lr</t>
+        </is>
+      </c>
+      <c r="BC5" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="BD5" s="24" t="inlineStr">
+        <is>
+          <t>c97732889cfca1912f8d78791ff63f04ee3fe987951aced9e4fab541932597cd</t>
+        </is>
+      </c>
+      <c r="BE5" s="24" t="inlineStr">
+        <is>
+          <t>6df496ff8b2da9c6</t>
+        </is>
+      </c>
+      <c r="BF5" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG5" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="BH5" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T16:42:59.880808Z</t>
+        </is>
+      </c>
+      <c r="BI5" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ5" s="25" t="n"/>
+      <c r="BK5" s="26" t="n">
+        <v>-102</v>
+      </c>
+      <c r="BL5" s="27" t="n">
+        <v>1.980392</v>
+      </c>
+      <c r="BM5" s="28" t="n">
+        <v>0.50495</v>
+      </c>
+      <c r="BN5" s="28" t="n">
+        <v>0.502488</v>
+      </c>
+      <c r="BO5" s="28" t="n"/>
+      <c r="BP5" s="25" t="n"/>
+      <c r="BQ5" s="27" t="n"/>
+      <c r="BR5" s="28" t="n"/>
+      <c r="BS5" s="28" t="n"/>
+      <c r="BT5" s="28" t="n"/>
+      <c r="BU5" s="25" t="n"/>
+      <c r="BV5" s="29" t="n"/>
+      <c r="BW5" s="24" t="n"/>
+      <c r="BX5" s="30" t="n"/>
+      <c r="BY5" s="27" t="n"/>
+      <c r="BZ5" s="24" t="n"/>
+      <c r="CA5" s="31" t="n"/>
+    </row>
+    <row r="6" ht="36" customHeight="1">
+      <c r="A6" s="24" t="inlineStr">
+        <is>
+          <t>512e4ebfdf1a456e</t>
+        </is>
+      </c>
+      <c r="B6" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T16:44:20.099051Z</t>
+        </is>
+      </c>
+      <c r="C6" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T18:20Z</t>
+        </is>
+      </c>
+      <c r="D6" s="24" t="inlineStr">
+        <is>
+          <t>401816164</t>
+        </is>
+      </c>
+      <c r="E6" s="24" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="F6" s="24" t="inlineStr">
+        <is>
+          <t>Minnesota Twins</t>
+        </is>
+      </c>
+      <c r="G6" s="24" t="inlineStr">
+        <is>
+          <t>Chicago Cubs</t>
+        </is>
+      </c>
+      <c r="H6" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I6" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J6" s="25" t="n"/>
+      <c r="K6" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L6" s="26" t="n">
+        <v>-133</v>
+      </c>
+      <c r="M6" s="27" t="n">
+        <v>1.75188</v>
+      </c>
+      <c r="N6" s="28" t="n">
+        <v>0.570815</v>
+      </c>
+      <c r="O6" s="28" t="n">
+        <v>0.608363</v>
+      </c>
+      <c r="P6" s="28" t="n"/>
+      <c r="Q6" s="28" t="n">
+        <v>0.037548</v>
+      </c>
+      <c r="R6" s="26" t="n">
+        <v>69</v>
+      </c>
+      <c r="S6" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="T6" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="U6" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V6" s="24" t="n"/>
+      <c r="W6" s="26" t="n"/>
+      <c r="X6" s="26" t="n"/>
+      <c r="Y6" s="25" t="n"/>
+      <c r="Z6" s="26" t="n"/>
+      <c r="AA6" s="28" t="n"/>
+      <c r="AB6" s="28" t="n"/>
+      <c r="AC6" s="30" t="n"/>
+      <c r="AD6" s="24" t="n"/>
+      <c r="AE6" s="31" t="inlineStr">
+        <is>
+          <t>Learned LR call at threshold 0.5500; executable ask 0.5700 (aec-mlb-min-chc-2026-07-18).</t>
+        </is>
+      </c>
+      <c r="AF6" s="31" t="inlineStr">
+        <is>
+          <t>Learned model; promotion gate not yet open; zero-unit research until review.</t>
+        </is>
+      </c>
+      <c r="AG6" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH6" s="24" t="n"/>
+      <c r="AI6" s="31" t="n"/>
+      <c r="AJ6" s="31" t="n"/>
+      <c r="AK6" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL6" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM6" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN6" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO6" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_MODEL_UNVALIDATED</t>
+        </is>
+      </c>
+      <c r="AP6" s="24" t="inlineStr">
+        <is>
+          <t>mlb-min</t>
+        </is>
+      </c>
+      <c r="AQ6" s="24" t="inlineStr">
+        <is>
+          <t>Minnesota Twins</t>
+        </is>
+      </c>
+      <c r="AR6" s="24" t="inlineStr">
+        <is>
+          <t>Minnesota Twins</t>
+        </is>
+      </c>
+      <c r="AS6" s="24" t="inlineStr">
+        <is>
+          <t>mlb-chc</t>
+        </is>
+      </c>
+      <c r="AT6" s="24" t="inlineStr">
+        <is>
+          <t>Chicago Cubs</t>
+        </is>
+      </c>
+      <c r="AU6" s="24" t="inlineStr">
+        <is>
+          <t>Chicago Cubs</t>
+        </is>
+      </c>
+      <c r="AV6" s="24" t="n"/>
+      <c r="AW6" s="24" t="n"/>
+      <c r="AX6" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY6" s="24" t="n"/>
+      <c r="AZ6" s="24" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="BA6" s="24" t="inlineStr">
+        <is>
+          <t>c97732889cfca1912f8d78791ff63f04ee3fe987951aced9e4fab541932597cd</t>
+        </is>
+      </c>
+      <c r="BB6" s="24" t="inlineStr">
+        <is>
+          <t>learned_lr</t>
+        </is>
+      </c>
+      <c r="BC6" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="BD6" s="24" t="inlineStr">
+        <is>
+          <t>c97732889cfca1912f8d78791ff63f04ee3fe987951aced9e4fab541932597cd</t>
+        </is>
+      </c>
+      <c r="BE6" s="24" t="inlineStr">
+        <is>
+          <t>7166685f6e68e237</t>
+        </is>
+      </c>
+      <c r="BF6" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG6" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="BH6" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T16:42:49.506840Z</t>
+        </is>
+      </c>
+      <c r="BI6" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ6" s="25" t="n"/>
+      <c r="BK6" s="26" t="n">
+        <v>-133</v>
+      </c>
+      <c r="BL6" s="27" t="n">
+        <v>1.75188</v>
+      </c>
+      <c r="BM6" s="28" t="n">
+        <v>0.570815</v>
+      </c>
+      <c r="BN6" s="28" t="n">
+        <v>0.567164</v>
+      </c>
+      <c r="BO6" s="28" t="n"/>
+      <c r="BP6" s="25" t="n"/>
+      <c r="BQ6" s="27" t="n"/>
+      <c r="BR6" s="28" t="n"/>
+      <c r="BS6" s="28" t="n"/>
+      <c r="BT6" s="28" t="n"/>
+      <c r="BU6" s="25" t="n"/>
+      <c r="BV6" s="29" t="n"/>
+      <c r="BW6" s="24" t="n"/>
+      <c r="BX6" s="30" t="n"/>
+      <c r="BY6" s="27" t="n"/>
+      <c r="BZ6" s="24" t="n"/>
+      <c r="CA6" s="31" t="n"/>
+    </row>
+    <row r="7" ht="36" customHeight="1">
+      <c r="A7" s="24" t="inlineStr">
+        <is>
+          <t>80b7c78aaffb4905</t>
+        </is>
+      </c>
+      <c r="B7" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T16:44:20.099051Z</t>
+        </is>
+      </c>
+      <c r="C7" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T19:07Z</t>
+        </is>
+      </c>
+      <c r="D7" s="24" t="inlineStr">
+        <is>
+          <t>401816156</t>
+        </is>
+      </c>
+      <c r="E7" s="24" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="F7" s="24" t="inlineStr">
+        <is>
+          <t>Chicago White Sox</t>
+        </is>
+      </c>
+      <c r="G7" s="24" t="inlineStr">
+        <is>
+          <t>Toronto Blue Jays</t>
+        </is>
+      </c>
+      <c r="H7" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I7" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J7" s="25" t="n"/>
+      <c r="K7" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L7" s="26" t="n">
+        <v>-104</v>
+      </c>
+      <c r="M7" s="27" t="n">
+        <v>1.961538</v>
+      </c>
+      <c r="N7" s="28" t="n">
+        <v>0.509804</v>
+      </c>
+      <c r="O7" s="28" t="n">
+        <v>0.5767679999999999</v>
+      </c>
+      <c r="P7" s="28" t="n"/>
+      <c r="Q7" s="28" t="n">
+        <v>0.066964</v>
+      </c>
+      <c r="R7" s="26" t="n">
+        <v>83</v>
+      </c>
+      <c r="S7" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="T7" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="U7" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V7" s="24" t="n"/>
+      <c r="W7" s="26" t="n"/>
+      <c r="X7" s="26" t="n"/>
+      <c r="Y7" s="25" t="n"/>
+      <c r="Z7" s="26" t="n"/>
+      <c r="AA7" s="28" t="n"/>
+      <c r="AB7" s="28" t="n"/>
+      <c r="AC7" s="30" t="n"/>
+      <c r="AD7" s="24" t="n"/>
+      <c r="AE7" s="31" t="inlineStr">
+        <is>
+          <t>Learned LR call at threshold 0.5500; executable ask 0.5100 (aec-mlb-cws-tor-2026-07-18).</t>
+        </is>
+      </c>
+      <c r="AF7" s="31" t="inlineStr">
+        <is>
+          <t>Learned model; promotion gate not yet open; zero-unit research until review.</t>
+        </is>
+      </c>
+      <c r="AG7" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH7" s="24" t="n"/>
+      <c r="AI7" s="31" t="n"/>
+      <c r="AJ7" s="31" t="n"/>
+      <c r="AK7" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL7" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM7" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN7" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO7" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_MODEL_UNVALIDATED</t>
+        </is>
+      </c>
+      <c r="AP7" s="24" t="inlineStr">
+        <is>
+          <t>mlb-cws</t>
+        </is>
+      </c>
+      <c r="AQ7" s="24" t="inlineStr">
+        <is>
+          <t>Chicago White Sox</t>
+        </is>
+      </c>
+      <c r="AR7" s="24" t="inlineStr">
+        <is>
+          <t>Chicago White Sox</t>
+        </is>
+      </c>
+      <c r="AS7" s="24" t="inlineStr">
+        <is>
+          <t>mlb-tor</t>
+        </is>
+      </c>
+      <c r="AT7" s="24" t="inlineStr">
+        <is>
+          <t>Toronto Blue Jays</t>
+        </is>
+      </c>
+      <c r="AU7" s="24" t="inlineStr">
+        <is>
+          <t>Toronto Blue Jays</t>
+        </is>
+      </c>
+      <c r="AV7" s="24" t="n"/>
+      <c r="AW7" s="24" t="n"/>
+      <c r="AX7" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY7" s="24" t="n"/>
+      <c r="AZ7" s="24" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="BA7" s="24" t="inlineStr">
+        <is>
+          <t>c97732889cfca1912f8d78791ff63f04ee3fe987951aced9e4fab541932597cd</t>
+        </is>
+      </c>
+      <c r="BB7" s="24" t="inlineStr">
+        <is>
+          <t>learned_lr</t>
+        </is>
+      </c>
+      <c r="BC7" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="BD7" s="24" t="inlineStr">
+        <is>
+          <t>c97732889cfca1912f8d78791ff63f04ee3fe987951aced9e4fab541932597cd</t>
+        </is>
+      </c>
+      <c r="BE7" s="24" t="inlineStr">
+        <is>
+          <t>990421d336b67011</t>
+        </is>
+      </c>
+      <c r="BF7" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG7" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="BH7" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T16:42:50.404282Z</t>
+        </is>
+      </c>
+      <c r="BI7" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ7" s="25" t="n"/>
+      <c r="BK7" s="26" t="n">
+        <v>-104</v>
+      </c>
+      <c r="BL7" s="27" t="n">
+        <v>1.961538</v>
+      </c>
+      <c r="BM7" s="28" t="n">
+        <v>0.509804</v>
+      </c>
+      <c r="BN7" s="28" t="n">
+        <v>0.507463</v>
+      </c>
+      <c r="BO7" s="28" t="n"/>
+      <c r="BP7" s="25" t="n"/>
+      <c r="BQ7" s="27" t="n"/>
+      <c r="BR7" s="28" t="n"/>
+      <c r="BS7" s="28" t="n"/>
+      <c r="BT7" s="28" t="n"/>
+      <c r="BU7" s="25" t="n"/>
+      <c r="BV7" s="29" t="n"/>
+      <c r="BW7" s="24" t="n"/>
+      <c r="BX7" s="30" t="n"/>
+      <c r="BY7" s="27" t="n"/>
+      <c r="BZ7" s="24" t="n"/>
+      <c r="CA7" s="31" t="n"/>
+    </row>
+    <row r="8" ht="36" customHeight="1">
+      <c r="A8" s="24" t="inlineStr">
+        <is>
+          <t>c7e4de168a8f4e3d</t>
+        </is>
+      </c>
+      <c r="B8" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T16:44:20.099051Z</t>
+        </is>
+      </c>
+      <c r="C8" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T19:10Z</t>
+        </is>
+      </c>
+      <c r="D8" s="24" t="inlineStr">
+        <is>
+          <t>401816166</t>
+        </is>
+      </c>
+      <c r="E8" s="24" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="F8" s="24" t="inlineStr">
+        <is>
+          <t>Cincinnati Reds</t>
+        </is>
+      </c>
+      <c r="G8" s="24" t="inlineStr">
+        <is>
+          <t>Colorado Rockies</t>
+        </is>
+      </c>
+      <c r="H8" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I8" s="24" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="J8" s="25" t="n"/>
+      <c r="K8" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L8" s="26" t="n">
+        <v>-104</v>
+      </c>
+      <c r="M8" s="27" t="n">
+        <v>1.961538</v>
+      </c>
+      <c r="N8" s="28" t="n">
+        <v>0.509804</v>
+      </c>
+      <c r="O8" s="28" t="n">
+        <v>0.582367</v>
+      </c>
+      <c r="P8" s="28" t="n"/>
+      <c r="Q8" s="28" t="n">
+        <v>0.072563</v>
+      </c>
+      <c r="R8" s="26" t="n">
+        <v>86</v>
+      </c>
+      <c r="S8" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="T8" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="U8" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V8" s="24" t="n"/>
+      <c r="W8" s="26" t="n"/>
+      <c r="X8" s="26" t="n"/>
+      <c r="Y8" s="25" t="n"/>
+      <c r="Z8" s="26" t="n"/>
+      <c r="AA8" s="28" t="n"/>
+      <c r="AB8" s="28" t="n"/>
+      <c r="AC8" s="30" t="n"/>
+      <c r="AD8" s="24" t="n"/>
+      <c r="AE8" s="31" t="inlineStr">
+        <is>
+          <t>Learned LR call at threshold 0.5500; executable ask 0.5100 (aec-mlb-cin-col-2026-07-18).</t>
+        </is>
+      </c>
+      <c r="AF8" s="31" t="inlineStr">
+        <is>
+          <t>Learned model; promotion gate not yet open; zero-unit research until review.</t>
+        </is>
+      </c>
+      <c r="AG8" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH8" s="24" t="n"/>
+      <c r="AI8" s="31" t="n"/>
+      <c r="AJ8" s="31" t="n"/>
+      <c r="AK8" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL8" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM8" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN8" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO8" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_MODEL_UNVALIDATED</t>
+        </is>
+      </c>
+      <c r="AP8" s="24" t="inlineStr">
+        <is>
+          <t>mlb-cin</t>
+        </is>
+      </c>
+      <c r="AQ8" s="24" t="inlineStr">
+        <is>
+          <t>Cincinnati Reds</t>
+        </is>
+      </c>
+      <c r="AR8" s="24" t="inlineStr">
+        <is>
+          <t>Cincinnati Reds</t>
+        </is>
+      </c>
+      <c r="AS8" s="24" t="inlineStr">
+        <is>
+          <t>mlb-col</t>
+        </is>
+      </c>
+      <c r="AT8" s="24" t="inlineStr">
+        <is>
+          <t>Colorado Rockies</t>
+        </is>
+      </c>
+      <c r="AU8" s="24" t="inlineStr">
+        <is>
+          <t>Colorado Rockies</t>
+        </is>
+      </c>
+      <c r="AV8" s="24" t="n"/>
+      <c r="AW8" s="24" t="n"/>
+      <c r="AX8" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY8" s="24" t="n"/>
+      <c r="AZ8" s="24" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="BA8" s="24" t="inlineStr">
+        <is>
+          <t>c97732889cfca1912f8d78791ff63f04ee3fe987951aced9e4fab541932597cd</t>
+        </is>
+      </c>
+      <c r="BB8" s="24" t="inlineStr">
+        <is>
+          <t>learned_lr</t>
+        </is>
+      </c>
+      <c r="BC8" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="BD8" s="24" t="inlineStr">
+        <is>
+          <t>c97732889cfca1912f8d78791ff63f04ee3fe987951aced9e4fab541932597cd</t>
+        </is>
+      </c>
+      <c r="BE8" s="24" t="inlineStr">
+        <is>
+          <t>4215d10b9bfb4b91</t>
+        </is>
+      </c>
+      <c r="BF8" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG8" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="BH8" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T16:42:52.313468Z</t>
+        </is>
+      </c>
+      <c r="BI8" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ8" s="25" t="n"/>
+      <c r="BK8" s="26" t="n">
+        <v>-104</v>
+      </c>
+      <c r="BL8" s="27" t="n">
+        <v>1.961538</v>
+      </c>
+      <c r="BM8" s="28" t="n">
+        <v>0.509804</v>
+      </c>
+      <c r="BN8" s="28" t="n">
+        <v>0.507463</v>
+      </c>
+      <c r="BO8" s="28" t="n"/>
+      <c r="BP8" s="25" t="n"/>
+      <c r="BQ8" s="27" t="n"/>
+      <c r="BR8" s="28" t="n"/>
+      <c r="BS8" s="28" t="n"/>
+      <c r="BT8" s="28" t="n"/>
+      <c r="BU8" s="25" t="n"/>
+      <c r="BV8" s="29" t="n"/>
+      <c r="BW8" s="24" t="n"/>
+      <c r="BX8" s="30" t="n"/>
+      <c r="BY8" s="27" t="n"/>
+      <c r="BZ8" s="24" t="n"/>
+      <c r="CA8" s="31" t="n"/>
+    </row>
+    <row r="9" ht="36" customHeight="1">
+      <c r="A9" s="24" t="inlineStr">
+        <is>
+          <t>2ec6744dbfd84ecf</t>
+        </is>
+      </c>
+      <c r="B9" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T16:44:20.099051Z</t>
+        </is>
+      </c>
+      <c r="C9" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T20:10Z</t>
+        </is>
+      </c>
+      <c r="D9" s="24" t="inlineStr">
+        <is>
+          <t>401816161</t>
+        </is>
+      </c>
+      <c r="E9" s="24" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="F9" s="24" t="inlineStr">
+        <is>
+          <t>Texas Rangers</t>
+        </is>
+      </c>
+      <c r="G9" s="24" t="inlineStr">
+        <is>
+          <t>Atlanta Braves</t>
+        </is>
+      </c>
+      <c r="H9" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I9" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J9" s="25" t="n"/>
+      <c r="K9" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L9" s="26" t="n">
+        <v>-106</v>
+      </c>
+      <c r="M9" s="27" t="n">
+        <v>1.943396</v>
+      </c>
+      <c r="N9" s="28" t="n">
+        <v>0.514563</v>
+      </c>
+      <c r="O9" s="28" t="n">
+        <v>0.550297</v>
+      </c>
+      <c r="P9" s="28" t="n"/>
+      <c r="Q9" s="28" t="n">
+        <v>0.035734</v>
+      </c>
+      <c r="R9" s="26" t="n">
+        <v>68</v>
+      </c>
+      <c r="S9" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="T9" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="U9" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V9" s="24" t="n"/>
+      <c r="W9" s="26" t="n"/>
+      <c r="X9" s="26" t="n"/>
+      <c r="Y9" s="25" t="n"/>
+      <c r="Z9" s="26" t="n"/>
+      <c r="AA9" s="28" t="n"/>
+      <c r="AB9" s="28" t="n"/>
+      <c r="AC9" s="30" t="n"/>
+      <c r="AD9" s="24" t="n"/>
+      <c r="AE9" s="31" t="inlineStr">
+        <is>
+          <t>Learned LR call at threshold 0.5500; executable ask 0.5150 (aec-mlb-tex-atl-2026-07-18).</t>
+        </is>
+      </c>
+      <c r="AF9" s="31" t="inlineStr">
+        <is>
+          <t>Learned model; promotion gate not yet open; zero-unit research until review.</t>
+        </is>
+      </c>
+      <c r="AG9" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH9" s="24" t="n"/>
+      <c r="AI9" s="31" t="n"/>
+      <c r="AJ9" s="31" t="n"/>
+      <c r="AK9" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL9" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM9" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN9" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO9" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_MODEL_UNVALIDATED</t>
+        </is>
+      </c>
+      <c r="AP9" s="24" t="inlineStr">
+        <is>
+          <t>mlb-tex</t>
+        </is>
+      </c>
+      <c r="AQ9" s="24" t="inlineStr">
+        <is>
+          <t>Texas Rangers</t>
+        </is>
+      </c>
+      <c r="AR9" s="24" t="inlineStr">
+        <is>
+          <t>Texas Rangers</t>
+        </is>
+      </c>
+      <c r="AS9" s="24" t="inlineStr">
+        <is>
+          <t>mlb-atl</t>
+        </is>
+      </c>
+      <c r="AT9" s="24" t="inlineStr">
+        <is>
+          <t>Atlanta Braves</t>
+        </is>
+      </c>
+      <c r="AU9" s="24" t="inlineStr">
+        <is>
+          <t>Atlanta Braves</t>
+        </is>
+      </c>
+      <c r="AV9" s="24" t="n"/>
+      <c r="AW9" s="24" t="n"/>
+      <c r="AX9" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY9" s="24" t="n"/>
+      <c r="AZ9" s="24" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="BA9" s="24" t="inlineStr">
+        <is>
+          <t>c97732889cfca1912f8d78791ff63f04ee3fe987951aced9e4fab541932597cd</t>
+        </is>
+      </c>
+      <c r="BB9" s="24" t="inlineStr">
+        <is>
+          <t>learned_lr</t>
+        </is>
+      </c>
+      <c r="BC9" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="BD9" s="24" t="inlineStr">
+        <is>
+          <t>c97732889cfca1912f8d78791ff63f04ee3fe987951aced9e4fab541932597cd</t>
+        </is>
+      </c>
+      <c r="BE9" s="24" t="inlineStr">
+        <is>
+          <t>a999da31a6f5af28</t>
+        </is>
+      </c>
+      <c r="BF9" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG9" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="BH9" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T16:42:57.199270Z</t>
+        </is>
+      </c>
+      <c r="BI9" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ9" s="25" t="n"/>
+      <c r="BK9" s="26" t="n">
+        <v>-106</v>
+      </c>
+      <c r="BL9" s="27" t="n">
+        <v>1.943396</v>
+      </c>
+      <c r="BM9" s="28" t="n">
+        <v>0.514563</v>
+      </c>
+      <c r="BN9" s="28" t="n">
+        <v>0.5124379999999999</v>
+      </c>
+      <c r="BO9" s="28" t="n"/>
+      <c r="BP9" s="25" t="n"/>
+      <c r="BQ9" s="27" t="n"/>
+      <c r="BR9" s="28" t="n"/>
+      <c r="BS9" s="28" t="n"/>
+      <c r="BT9" s="28" t="n"/>
+      <c r="BU9" s="25" t="n"/>
+      <c r="BV9" s="29" t="n"/>
+      <c r="BW9" s="24" t="n"/>
+      <c r="BX9" s="30" t="n"/>
+      <c r="BY9" s="27" t="n"/>
+      <c r="BZ9" s="24" t="n"/>
+      <c r="CA9" s="31" t="n"/>
+    </row>
+    <row r="10" ht="36" customHeight="1">
+      <c r="A10" s="24" t="inlineStr">
+        <is>
+          <t>634e9b9c56164f59</t>
+        </is>
+      </c>
+      <c r="B10" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T16:44:20.099051Z</t>
+        </is>
+      </c>
+      <c r="C10" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T23:10Z</t>
+        </is>
+      </c>
+      <c r="D10" s="24" t="inlineStr">
+        <is>
+          <t>401816159</t>
+        </is>
+      </c>
+      <c r="E10" s="24" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="F10" s="24" t="inlineStr">
+        <is>
+          <t>Pittsburgh Pirates</t>
+        </is>
+      </c>
+      <c r="G10" s="24" t="inlineStr">
+        <is>
+          <t>Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="H10" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I10" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J10" s="25" t="n"/>
+      <c r="K10" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L10" s="26" t="n">
+        <v>-102</v>
+      </c>
+      <c r="M10" s="27" t="n">
+        <v>1.980392</v>
+      </c>
+      <c r="N10" s="28" t="n">
+        <v>0.50495</v>
+      </c>
+      <c r="O10" s="28" t="n">
+        <v>0.554084</v>
+      </c>
+      <c r="P10" s="28" t="n"/>
+      <c r="Q10" s="28" t="n">
+        <v>0.049134</v>
+      </c>
+      <c r="R10" s="26" t="n">
+        <v>75</v>
+      </c>
+      <c r="S10" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="T10" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="U10" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V10" s="24" t="n"/>
+      <c r="W10" s="26" t="n"/>
+      <c r="X10" s="26" t="n"/>
+      <c r="Y10" s="25" t="n"/>
+      <c r="Z10" s="26" t="n"/>
+      <c r="AA10" s="28" t="n"/>
+      <c r="AB10" s="28" t="n"/>
+      <c r="AC10" s="30" t="n"/>
+      <c r="AD10" s="24" t="n"/>
+      <c r="AE10" s="31" t="inlineStr">
+        <is>
+          <t>Learned LR call at threshold 0.5500; executable ask 0.5050 (aec-mlb-pit-cle-2026-07-18).</t>
+        </is>
+      </c>
+      <c r="AF10" s="31" t="inlineStr">
+        <is>
+          <t>Learned model; promotion gate not yet open; zero-unit research until review.</t>
+        </is>
+      </c>
+      <c r="AG10" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH10" s="24" t="n"/>
+      <c r="AI10" s="31" t="n"/>
+      <c r="AJ10" s="31" t="n"/>
+      <c r="AK10" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL10" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM10" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN10" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO10" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_MODEL_UNVALIDATED</t>
+        </is>
+      </c>
+      <c r="AP10" s="24" t="inlineStr">
+        <is>
+          <t>mlb-pit</t>
+        </is>
+      </c>
+      <c r="AQ10" s="24" t="inlineStr">
+        <is>
+          <t>Pittsburgh Pirates</t>
+        </is>
+      </c>
+      <c r="AR10" s="24" t="inlineStr">
+        <is>
+          <t>Pittsburgh Pirates</t>
+        </is>
+      </c>
+      <c r="AS10" s="24" t="inlineStr">
+        <is>
+          <t>mlb-cle</t>
+        </is>
+      </c>
+      <c r="AT10" s="24" t="inlineStr">
+        <is>
+          <t>Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="AU10" s="24" t="inlineStr">
+        <is>
+          <t>Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="AV10" s="24" t="n"/>
+      <c r="AW10" s="24" t="n"/>
+      <c r="AX10" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY10" s="24" t="n"/>
+      <c r="AZ10" s="24" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="BA10" s="24" t="inlineStr">
+        <is>
+          <t>c97732889cfca1912f8d78791ff63f04ee3fe987951aced9e4fab541932597cd</t>
+        </is>
+      </c>
+      <c r="BB10" s="24" t="inlineStr">
+        <is>
+          <t>learned_lr</t>
+        </is>
+      </c>
+      <c r="BC10" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="BD10" s="24" t="inlineStr">
+        <is>
+          <t>c97732889cfca1912f8d78791ff63f04ee3fe987951aced9e4fab541932597cd</t>
+        </is>
+      </c>
+      <c r="BE10" s="24" t="inlineStr">
+        <is>
+          <t>3c0f9e9f1d0333c4</t>
+        </is>
+      </c>
+      <c r="BF10" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG10" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="BH10" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T16:42:59.880808Z</t>
+        </is>
+      </c>
+      <c r="BI10" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ10" s="25" t="n"/>
+      <c r="BK10" s="26" t="n">
+        <v>-102</v>
+      </c>
+      <c r="BL10" s="27" t="n">
+        <v>1.980392</v>
+      </c>
+      <c r="BM10" s="28" t="n">
+        <v>0.50495</v>
+      </c>
+      <c r="BN10" s="28" t="n">
+        <v>0.502488</v>
+      </c>
+      <c r="BO10" s="28" t="n"/>
+      <c r="BP10" s="25" t="n"/>
+      <c r="BQ10" s="27" t="n"/>
+      <c r="BR10" s="28" t="n"/>
+      <c r="BS10" s="28" t="n"/>
+      <c r="BT10" s="28" t="n"/>
+      <c r="BU10" s="25" t="n"/>
+      <c r="BV10" s="29" t="n"/>
+      <c r="BW10" s="24" t="n"/>
+      <c r="BX10" s="30" t="n"/>
+      <c r="BY10" s="27" t="n"/>
+      <c r="BZ10" s="24" t="n"/>
+      <c r="CA10" s="31" t="n"/>
+    </row>
+    <row r="11" ht="36" customHeight="1">
+      <c r="A11" s="24" t="inlineStr">
+        <is>
+          <t>0a1abd6e59a84720</t>
+        </is>
+      </c>
+      <c r="B11" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T16:44:20.099051Z</t>
+        </is>
+      </c>
+      <c r="C11" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-19T00:08Z</t>
+        </is>
+      </c>
+      <c r="D11" s="24" t="inlineStr">
+        <is>
+          <t>401816168</t>
+        </is>
+      </c>
+      <c r="E11" s="24" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="F11" s="24" t="inlineStr">
+        <is>
+          <t>San Francisco Giants</t>
+        </is>
+      </c>
+      <c r="G11" s="24" t="inlineStr">
+        <is>
+          <t>Seattle Mariners</t>
+        </is>
+      </c>
+      <c r="H11" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I11" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J11" s="25" t="n"/>
+      <c r="K11" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L11" s="26" t="n">
+        <v>-138</v>
+      </c>
+      <c r="M11" s="27" t="n">
+        <v>1.724638</v>
+      </c>
+      <c r="N11" s="28" t="n">
+        <v>0.579832</v>
+      </c>
+      <c r="O11" s="28" t="n">
+        <v>0.627758</v>
+      </c>
+      <c r="P11" s="28" t="n"/>
+      <c r="Q11" s="28" t="n">
+        <v>0.047926</v>
+      </c>
+      <c r="R11" s="26" t="n">
+        <v>74</v>
+      </c>
+      <c r="S11" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="T11" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="U11" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V11" s="24" t="n"/>
+      <c r="W11" s="26" t="n"/>
+      <c r="X11" s="26" t="n"/>
+      <c r="Y11" s="25" t="n"/>
+      <c r="Z11" s="26" t="n"/>
+      <c r="AA11" s="28" t="n"/>
+      <c r="AB11" s="28" t="n"/>
+      <c r="AC11" s="30" t="n"/>
+      <c r="AD11" s="24" t="n"/>
+      <c r="AE11" s="31" t="inlineStr">
+        <is>
+          <t>Learned LR call at threshold 0.5500; executable ask 0.5800 (aec-mlb-sf-sea-2026-07-18).</t>
+        </is>
+      </c>
+      <c r="AF11" s="31" t="inlineStr">
+        <is>
+          <t>Learned model; promotion gate not yet open; zero-unit research until review.</t>
+        </is>
+      </c>
+      <c r="AG11" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH11" s="24" t="n"/>
+      <c r="AI11" s="31" t="n"/>
+      <c r="AJ11" s="31" t="n"/>
+      <c r="AK11" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL11" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM11" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN11" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO11" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_MODEL_UNVALIDATED</t>
+        </is>
+      </c>
+      <c r="AP11" s="24" t="inlineStr">
+        <is>
+          <t>mlb-sf</t>
+        </is>
+      </c>
+      <c r="AQ11" s="24" t="inlineStr">
+        <is>
+          <t>San Francisco Giants</t>
+        </is>
+      </c>
+      <c r="AR11" s="24" t="inlineStr">
+        <is>
+          <t>San Francisco Giants</t>
+        </is>
+      </c>
+      <c r="AS11" s="24" t="inlineStr">
+        <is>
+          <t>mlb-sea</t>
+        </is>
+      </c>
+      <c r="AT11" s="24" t="inlineStr">
+        <is>
+          <t>Seattle Mariners</t>
+        </is>
+      </c>
+      <c r="AU11" s="24" t="inlineStr">
+        <is>
+          <t>Seattle Mariners</t>
+        </is>
+      </c>
+      <c r="AV11" s="24" t="n"/>
+      <c r="AW11" s="24" t="n"/>
+      <c r="AX11" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY11" s="24" t="n"/>
+      <c r="AZ11" s="24" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="BA11" s="24" t="inlineStr">
+        <is>
+          <t>c97732889cfca1912f8d78791ff63f04ee3fe987951aced9e4fab541932597cd</t>
+        </is>
+      </c>
+      <c r="BB11" s="24" t="inlineStr">
+        <is>
+          <t>learned_lr</t>
+        </is>
+      </c>
+      <c r="BC11" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="BD11" s="24" t="inlineStr">
+        <is>
+          <t>c97732889cfca1912f8d78791ff63f04ee3fe987951aced9e4fab541932597cd</t>
+        </is>
+      </c>
+      <c r="BE11" s="24" t="inlineStr">
+        <is>
+          <t>29d502a7704e228f</t>
+        </is>
+      </c>
+      <c r="BF11" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG11" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="BH11" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T16:43:04.779295Z</t>
+        </is>
+      </c>
+      <c r="BI11" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ11" s="25" t="n"/>
+      <c r="BK11" s="26" t="n">
+        <v>-138</v>
+      </c>
+      <c r="BL11" s="27" t="n">
+        <v>1.724638</v>
+      </c>
+      <c r="BM11" s="28" t="n">
+        <v>0.579832</v>
+      </c>
+      <c r="BN11" s="28" t="n">
+        <v>0.577114</v>
+      </c>
+      <c r="BO11" s="28" t="n"/>
+      <c r="BP11" s="25" t="n"/>
+      <c r="BQ11" s="27" t="n"/>
+      <c r="BR11" s="28" t="n"/>
+      <c r="BS11" s="28" t="n"/>
+      <c r="BT11" s="28" t="n"/>
+      <c r="BU11" s="25" t="n"/>
+      <c r="BV11" s="29" t="n"/>
+      <c r="BW11" s="24" t="n"/>
+      <c r="BX11" s="30" t="n"/>
+      <c r="BY11" s="27" t="n"/>
+      <c r="BZ11" s="24" t="n"/>
+      <c r="CA11" s="31" t="n"/>
+    </row>
+    <row r="12" ht="36" customHeight="1">
+      <c r="A12" s="24" t="inlineStr">
+        <is>
+          <t>534daa3057c4428f</t>
+        </is>
+      </c>
+      <c r="B12" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T16:44:20.099051Z</t>
+        </is>
+      </c>
+      <c r="C12" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-19T02:05Z</t>
+        </is>
+      </c>
+      <c r="D12" s="24" t="inlineStr">
+        <is>
+          <t>401816170</t>
+        </is>
+      </c>
+      <c r="E12" s="24" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="F12" s="24" t="inlineStr">
+        <is>
+          <t>Washington Nationals</t>
+        </is>
+      </c>
+      <c r="G12" s="24" t="inlineStr">
+        <is>
+          <t>Athletics</t>
+        </is>
+      </c>
+      <c r="H12" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I12" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J12" s="25" t="n"/>
+      <c r="K12" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L12" s="26" t="n">
+        <v>102</v>
+      </c>
+      <c r="M12" s="27" t="n">
+        <v>2.02</v>
+      </c>
+      <c r="N12" s="28" t="n">
+        <v>0.49505</v>
+      </c>
+      <c r="O12" s="28" t="n">
+        <v>0.569735</v>
+      </c>
+      <c r="P12" s="28" t="n"/>
+      <c r="Q12" s="28" t="n">
+        <v>0.074685</v>
+      </c>
+      <c r="R12" s="26" t="n">
+        <v>87</v>
+      </c>
+      <c r="S12" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="T12" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="U12" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V12" s="24" t="n"/>
+      <c r="W12" s="26" t="n"/>
+      <c r="X12" s="26" t="n"/>
+      <c r="Y12" s="25" t="n"/>
+      <c r="Z12" s="26" t="n"/>
+      <c r="AA12" s="28" t="n"/>
+      <c r="AB12" s="28" t="n"/>
+      <c r="AC12" s="30" t="n"/>
+      <c r="AD12" s="24" t="n"/>
+      <c r="AE12" s="31" t="inlineStr">
+        <is>
+          <t>Learned LR call at threshold 0.5500; executable ask 0.4950 (aec-mlb-wsh-ath-2026-07-18).</t>
+        </is>
+      </c>
+      <c r="AF12" s="31" t="inlineStr">
+        <is>
+          <t>Learned model; promotion gate not yet open; zero-unit research until review.</t>
+        </is>
+      </c>
+      <c r="AG12" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH12" s="24" t="n"/>
+      <c r="AI12" s="31" t="n"/>
+      <c r="AJ12" s="31" t="n"/>
+      <c r="AK12" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL12" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM12" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN12" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO12" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_MODEL_UNVALIDATED</t>
+        </is>
+      </c>
+      <c r="AP12" s="24" t="inlineStr">
+        <is>
+          <t>mlb-wsh</t>
+        </is>
+      </c>
+      <c r="AQ12" s="24" t="inlineStr">
+        <is>
+          <t>Washington Nationals</t>
+        </is>
+      </c>
+      <c r="AR12" s="24" t="inlineStr">
+        <is>
+          <t>Washington Nationals</t>
+        </is>
+      </c>
+      <c r="AS12" s="24" t="inlineStr">
+        <is>
+          <t>mlb-ath</t>
+        </is>
+      </c>
+      <c r="AT12" s="24" t="inlineStr">
+        <is>
+          <t>Athletics</t>
+        </is>
+      </c>
+      <c r="AU12" s="24" t="inlineStr">
+        <is>
+          <t>Athletics</t>
+        </is>
+      </c>
+      <c r="AV12" s="24" t="n"/>
+      <c r="AW12" s="24" t="n"/>
+      <c r="AX12" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY12" s="24" t="n"/>
+      <c r="AZ12" s="24" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="BA12" s="24" t="inlineStr">
+        <is>
+          <t>c97732889cfca1912f8d78791ff63f04ee3fe987951aced9e4fab541932597cd</t>
+        </is>
+      </c>
+      <c r="BB12" s="24" t="inlineStr">
+        <is>
+          <t>learned_lr</t>
+        </is>
+      </c>
+      <c r="BC12" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="BD12" s="24" t="inlineStr">
+        <is>
+          <t>c97732889cfca1912f8d78791ff63f04ee3fe987951aced9e4fab541932597cd</t>
+        </is>
+      </c>
+      <c r="BE12" s="24" t="inlineStr">
+        <is>
+          <t>d2faed7be6c04691</t>
+        </is>
+      </c>
+      <c r="BF12" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG12" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="BH12" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T16:43:06.321641Z</t>
+        </is>
+      </c>
+      <c r="BI12" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ12" s="25" t="n"/>
+      <c r="BK12" s="26" t="n">
+        <v>102</v>
+      </c>
+      <c r="BL12" s="27" t="n">
+        <v>2.02</v>
+      </c>
+      <c r="BM12" s="28" t="n">
+        <v>0.49505</v>
+      </c>
+      <c r="BN12" s="28" t="n">
+        <v>0.492537</v>
+      </c>
+      <c r="BO12" s="28" t="n"/>
+      <c r="BP12" s="25" t="n"/>
+      <c r="BQ12" s="27" t="n"/>
+      <c r="BR12" s="28" t="n"/>
+      <c r="BS12" s="28" t="n"/>
+      <c r="BT12" s="28" t="n"/>
+      <c r="BU12" s="25" t="n"/>
+      <c r="BV12" s="29" t="n"/>
+      <c r="BW12" s="24" t="n"/>
+      <c r="BX12" s="30" t="n"/>
+      <c r="BY12" s="27" t="n"/>
+      <c r="BZ12" s="24" t="n"/>
+      <c r="CA12" s="31" t="n"/>
+    </row>
+    <row r="13" ht="36" customHeight="1">
+      <c r="A13" s="24" t="inlineStr">
+        <is>
+          <t>5ab4cdd6444d4f9b</t>
+        </is>
+      </c>
+      <c r="B13" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T16:50:38.270483Z</t>
+        </is>
+      </c>
+      <c r="C13" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T20:10Z</t>
+        </is>
+      </c>
+      <c r="D13" s="24" t="inlineStr">
+        <is>
+          <t>401816162</t>
+        </is>
+      </c>
+      <c r="E13" s="24" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="F13" s="24" t="inlineStr">
+        <is>
+          <t>Baltimore Orioles</t>
+        </is>
+      </c>
+      <c r="G13" s="24" t="inlineStr">
+        <is>
+          <t>Houston Astros</t>
+        </is>
+      </c>
+      <c r="H13" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I13" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J13" s="25" t="n"/>
+      <c r="K13" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L13" s="26" t="n">
+        <v>-102</v>
+      </c>
+      <c r="M13" s="27" t="n">
+        <v>1.980392</v>
+      </c>
+      <c r="N13" s="28" t="n">
+        <v>0.50495</v>
+      </c>
+      <c r="O13" s="28" t="n">
+        <v>0.545167</v>
+      </c>
+      <c r="P13" s="28" t="n"/>
+      <c r="Q13" s="28" t="n">
+        <v>0.040217</v>
+      </c>
+      <c r="R13" s="26" t="n">
+        <v>70</v>
+      </c>
+      <c r="S13" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="T13" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="U13" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V13" s="24" t="n"/>
+      <c r="W13" s="26" t="n"/>
+      <c r="X13" s="26" t="n"/>
+      <c r="Y13" s="25" t="n"/>
+      <c r="Z13" s="26" t="n"/>
+      <c r="AA13" s="28" t="n"/>
+      <c r="AB13" s="28" t="n"/>
+      <c r="AC13" s="30" t="n"/>
+      <c r="AD13" s="24" t="n"/>
+      <c r="AE13" s="31" t="inlineStr">
+        <is>
+          <t>Learned LR call at threshold 0.5100; executable ask 0.5050 (aec-mlb-bal-hou-2026-07-18).</t>
+        </is>
+      </c>
+      <c r="AF13" s="31" t="inlineStr">
+        <is>
+          <t>Learned model; promotion gate not yet open; zero-unit research until review.</t>
+        </is>
+      </c>
+      <c r="AG13" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH13" s="24" t="n"/>
+      <c r="AI13" s="31" t="n"/>
+      <c r="AJ13" s="31" t="n"/>
+      <c r="AK13" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL13" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM13" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN13" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO13" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_MODEL_UNVALIDATED</t>
+        </is>
+      </c>
+      <c r="AP13" s="24" t="inlineStr">
+        <is>
+          <t>mlb-bal</t>
+        </is>
+      </c>
+      <c r="AQ13" s="24" t="inlineStr">
+        <is>
+          <t>Baltimore Orioles</t>
+        </is>
+      </c>
+      <c r="AR13" s="24" t="inlineStr">
+        <is>
+          <t>Baltimore Orioles</t>
+        </is>
+      </c>
+      <c r="AS13" s="24" t="inlineStr">
+        <is>
+          <t>mlb-hou</t>
+        </is>
+      </c>
+      <c r="AT13" s="24" t="inlineStr">
+        <is>
+          <t>Houston Astros</t>
+        </is>
+      </c>
+      <c r="AU13" s="24" t="inlineStr">
+        <is>
+          <t>Houston Astros</t>
+        </is>
+      </c>
+      <c r="AV13" s="24" t="n"/>
+      <c r="AW13" s="24" t="n"/>
+      <c r="AX13" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY13" s="24" t="n"/>
+      <c r="AZ13" s="24" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="BA13" s="24" t="inlineStr">
+        <is>
+          <t>40e5d70a6fae1347ad85569354088d9df4f2d6970f7d7c2f9d4924d65efd0c19</t>
+        </is>
+      </c>
+      <c r="BB13" s="24" t="inlineStr">
+        <is>
+          <t>learned_lr</t>
+        </is>
+      </c>
+      <c r="BC13" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="BD13" s="24" t="inlineStr">
+        <is>
+          <t>40e5d70a6fae1347ad85569354088d9df4f2d6970f7d7c2f9d4924d65efd0c19</t>
+        </is>
+      </c>
+      <c r="BE13" s="24" t="inlineStr">
+        <is>
+          <t>f6cae9c590f4ed48</t>
+        </is>
+      </c>
+      <c r="BF13" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG13" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="BH13" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T16:49:31.642864Z</t>
+        </is>
+      </c>
+      <c r="BI13" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ13" s="25" t="n"/>
+      <c r="BK13" s="26" t="n">
+        <v>-102</v>
+      </c>
+      <c r="BL13" s="27" t="n">
+        <v>1.980392</v>
+      </c>
+      <c r="BM13" s="28" t="n">
+        <v>0.50495</v>
+      </c>
+      <c r="BN13" s="28" t="n">
+        <v>0.502488</v>
+      </c>
+      <c r="BO13" s="28" t="n"/>
+      <c r="BP13" s="25" t="n"/>
+      <c r="BQ13" s="27" t="n"/>
+      <c r="BR13" s="28" t="n"/>
+      <c r="BS13" s="28" t="n"/>
+      <c r="BT13" s="28" t="n"/>
+      <c r="BU13" s="25" t="n"/>
+      <c r="BV13" s="29" t="n"/>
+      <c r="BW13" s="24" t="n"/>
+      <c r="BX13" s="30" t="n"/>
+      <c r="BY13" s="27" t="n"/>
+      <c r="BZ13" s="24" t="n"/>
+      <c r="CA13" s="31" t="n"/>
+    </row>
+    <row r="14" ht="36" customHeight="1">
+      <c r="A14" s="24" t="inlineStr">
+        <is>
+          <t>87feefaaee354c43</t>
+        </is>
+      </c>
+      <c r="B14" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T16:50:38.270483Z</t>
+        </is>
+      </c>
+      <c r="C14" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-19T00:08Z</t>
+        </is>
+      </c>
+      <c r="D14" s="24" t="inlineStr">
+        <is>
+          <t>401816157</t>
+        </is>
+      </c>
+      <c r="E14" s="24" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="F14" s="24" t="inlineStr">
+        <is>
+          <t>Los Angeles Dodgers</t>
+        </is>
+      </c>
+      <c r="G14" s="24" t="inlineStr">
+        <is>
+          <t>New York Yankees</t>
+        </is>
+      </c>
+      <c r="H14" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I14" s="24" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="J14" s="25" t="n"/>
+      <c r="K14" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L14" s="26" t="n">
+        <v>102</v>
+      </c>
+      <c r="M14" s="27" t="n">
+        <v>2.02</v>
+      </c>
+      <c r="N14" s="28" t="n">
+        <v>0.49505</v>
+      </c>
+      <c r="O14" s="28" t="n">
+        <v>0.532568</v>
+      </c>
+      <c r="P14" s="28" t="n"/>
+      <c r="Q14" s="28" t="n">
+        <v>0.037518</v>
+      </c>
+      <c r="R14" s="26" t="n">
+        <v>69</v>
+      </c>
+      <c r="S14" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="T14" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="U14" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V14" s="24" t="n"/>
+      <c r="W14" s="26" t="n"/>
+      <c r="X14" s="26" t="n"/>
+      <c r="Y14" s="25" t="n"/>
+      <c r="Z14" s="26" t="n"/>
+      <c r="AA14" s="28" t="n"/>
+      <c r="AB14" s="28" t="n"/>
+      <c r="AC14" s="30" t="n"/>
+      <c r="AD14" s="24" t="n"/>
+      <c r="AE14" s="31" t="inlineStr">
+        <is>
+          <t>Learned LR call at threshold 0.5100; executable ask 0.4950 (aec-mlb-lad-nyy-2026-07-18).</t>
+        </is>
+      </c>
+      <c r="AF14" s="31" t="inlineStr">
+        <is>
+          <t>Learned model; promotion gate not yet open; zero-unit research until review.</t>
+        </is>
+      </c>
+      <c r="AG14" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH14" s="24" t="n"/>
+      <c r="AI14" s="31" t="n"/>
+      <c r="AJ14" s="31" t="n"/>
+      <c r="AK14" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL14" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM14" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN14" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO14" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_MODEL_UNVALIDATED</t>
+        </is>
+      </c>
+      <c r="AP14" s="24" t="inlineStr">
+        <is>
+          <t>mlb-lad</t>
+        </is>
+      </c>
+      <c r="AQ14" s="24" t="inlineStr">
+        <is>
+          <t>Los Angeles Dodgers</t>
+        </is>
+      </c>
+      <c r="AR14" s="24" t="inlineStr">
+        <is>
+          <t>Los Angeles Dodgers</t>
+        </is>
+      </c>
+      <c r="AS14" s="24" t="inlineStr">
+        <is>
+          <t>mlb-nyy</t>
+        </is>
+      </c>
+      <c r="AT14" s="24" t="inlineStr">
+        <is>
+          <t>New York Yankees</t>
+        </is>
+      </c>
+      <c r="AU14" s="24" t="inlineStr">
+        <is>
+          <t>New York Yankees</t>
+        </is>
+      </c>
+      <c r="AV14" s="24" t="n"/>
+      <c r="AW14" s="24" t="n"/>
+      <c r="AX14" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY14" s="24" t="n"/>
+      <c r="AZ14" s="24" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="BA14" s="24" t="inlineStr">
+        <is>
+          <t>40e5d70a6fae1347ad85569354088d9df4f2d6970f7d7c2f9d4924d65efd0c19</t>
+        </is>
+      </c>
+      <c r="BB14" s="24" t="inlineStr">
+        <is>
+          <t>learned_lr</t>
+        </is>
+      </c>
+      <c r="BC14" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="BD14" s="24" t="inlineStr">
+        <is>
+          <t>40e5d70a6fae1347ad85569354088d9df4f2d6970f7d7c2f9d4924d65efd0c19</t>
+        </is>
+      </c>
+      <c r="BE14" s="24" t="inlineStr">
+        <is>
+          <t>3492e72a2faca7c7</t>
+        </is>
+      </c>
+      <c r="BF14" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG14" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v3</t>
+        </is>
+      </c>
+      <c r="BH14" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-18T16:49:36.781770Z</t>
+        </is>
+      </c>
+      <c r="BI14" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ14" s="25" t="n"/>
+      <c r="BK14" s="26" t="n">
+        <v>102</v>
+      </c>
+      <c r="BL14" s="27" t="n">
+        <v>2.02</v>
+      </c>
+      <c r="BM14" s="28" t="n">
+        <v>0.49505</v>
+      </c>
+      <c r="BN14" s="28" t="n">
+        <v>0.492537</v>
+      </c>
+      <c r="BO14" s="28" t="n"/>
+      <c r="BP14" s="25" t="n"/>
+      <c r="BQ14" s="27" t="n"/>
+      <c r="BR14" s="28" t="n"/>
+      <c r="BS14" s="28" t="n"/>
+      <c r="BT14" s="28" t="n"/>
+      <c r="BU14" s="25" t="n"/>
+      <c r="BV14" s="29" t="n"/>
+      <c r="BW14" s="24" t="n"/>
+      <c r="BX14" s="30" t="n"/>
+      <c r="BY14" s="27" t="n"/>
+      <c r="BZ14" s="24" t="n"/>
+      <c r="CA14" s="31" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
chore: remove stale backups and temp files
</commit_message>
<xml_diff>
--- a/data/picks.xlsx
+++ b/data/picks.xlsx
@@ -21,10 +21,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="0.0###"/>
-    <numFmt numFmtId="165" formatCode="0.000000"/>
-    <numFmt numFmtId="166" formatCode="0.0000"/>
-    <numFmt numFmtId="167" formatCode="0.0%"/>
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="0.0000"/>
+    <numFmt numFmtId="166" formatCode="0.0###"/>
+    <numFmt numFmtId="167" formatCode="0.000000"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -136,7 +136,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -150,10 +150,10 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -169,10 +169,10 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="167" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="10" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -184,10 +184,10 @@
     <xf numFmtId="0" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="167" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="10" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -202,13 +202,13 @@
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="10" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -217,11 +217,38 @@
     <xf numFmtId="2" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -754,6 +781,7 @@
         <v/>
       </c>
     </row>
+    <row r="5"/>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
@@ -785,15 +813,16 @@
         <f>COUNTIFS('Picks'!$BX$2:$BX$39,"&gt;0",'Picks'!$V$2:$V$39,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$39,"&gt;0",'Picks'!$V$2:$V$39,"loss")</f>
         <v/>
       </c>
-      <c r="E7" s="7">
+      <c r="E7" s="32">
         <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$39,"&gt;0",'Picks'!$V$2:$V$39,"win")/(COUNTIFS('Picks'!$BX$2:$BX$39,"&gt;0",'Picks'!$V$2:$V$39,"win")+COUNTIFS('Picks'!$BX$2:$BX$39,"&gt;0",'Picks'!$V$2:$V$39,"loss")),0)</f>
         <v/>
       </c>
-      <c r="G7" s="7">
+      <c r="G7" s="32">
         <f>IFERROR(SUM('Picks'!$BY$2:$BY$39)/SUM('Picks'!$BX$2:$BX$39),0)</f>
         <v/>
       </c>
     </row>
+    <row r="8"/>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
@@ -817,7 +846,7 @@
       </c>
     </row>
     <row r="10" ht="28" customHeight="1">
-      <c r="A10" s="8">
+      <c r="A10" s="33">
         <f>SUM('Picks'!$BY$2:$BY$39)</f>
         <v/>
       </c>
@@ -829,11 +858,12 @@
         <f>COUNTIFS('Picks'!$AM$2:$AM$39,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$39,"settled")</f>
         <v/>
       </c>
-      <c r="G10" s="8">
+      <c r="G10" s="33">
         <f>SUMIFS('Picks'!$AC$2:$AC$39,'Picks'!$AM$2:$AM$39,"QUALIFIED_SHADOW_CALL")</f>
         <v/>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
         <is>
@@ -896,11 +926,11 @@
         <f>COUNTIFS('Picks'!$H$2:$H$39,$A14,'Picks'!$U$2:$U$39,"settled",'Picks'!$V$2:$V$39,"loss")</f>
         <v/>
       </c>
-      <c r="E14" s="14">
+      <c r="E14" s="34">
         <f>IFERROR(C14/(C14+D14),0)</f>
         <v/>
       </c>
-      <c r="F14" s="15">
+      <c r="F14" s="35">
         <f>SUMIFS('Picks'!$BY$2:$BY$39,'Picks'!$H$2:$H$39,$A14)</f>
         <v/>
       </c>
@@ -927,11 +957,11 @@
         <f>COUNTIFS('Picks'!$H$2:$H$39,$A15,'Picks'!$U$2:$U$39,"settled",'Picks'!$V$2:$V$39,"loss")</f>
         <v/>
       </c>
-      <c r="E15" s="19">
+      <c r="E15" s="36">
         <f>IFERROR(C15/(C15+D15),0)</f>
         <v/>
       </c>
-      <c r="F15" s="20">
+      <c r="F15" s="37">
         <f>SUMIFS('Picks'!$BY$2:$BY$39,'Picks'!$H$2:$H$39,$A15)</f>
         <v/>
       </c>
@@ -958,11 +988,11 @@
         <f>COUNTIFS('Picks'!$H$2:$H$39,$A16,'Picks'!$U$2:$U$39,"settled",'Picks'!$V$2:$V$39,"loss")</f>
         <v/>
       </c>
-      <c r="E16" s="14">
+      <c r="E16" s="34">
         <f>IFERROR(C16/(C16+D16),0)</f>
         <v/>
       </c>
-      <c r="F16" s="15">
+      <c r="F16" s="35">
         <f>SUMIFS('Picks'!$BY$2:$BY$39,'Picks'!$H$2:$H$39,$A16)</f>
         <v/>
       </c>
@@ -971,6 +1001,7 @@
         <v/>
       </c>
     </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="22" t="inlineStr">
         <is>
@@ -1523,7 +1554,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J2" s="25" t="n"/>
+      <c r="J2" s="38" t="n"/>
       <c r="K2" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -1532,7 +1563,7 @@
       <c r="L2" s="26" t="n">
         <v>117</v>
       </c>
-      <c r="M2" s="27" t="n">
+      <c r="M2" s="39" t="n">
         <v>2.17</v>
       </c>
       <c r="N2" s="28" t="n">
@@ -1572,11 +1603,11 @@
       <c r="X2" s="26" t="n">
         <v>108</v>
       </c>
-      <c r="Y2" s="25" t="n"/>
+      <c r="Y2" s="38" t="n"/>
       <c r="Z2" s="26" t="n"/>
       <c r="AA2" s="28" t="n"/>
       <c r="AB2" s="28" t="n"/>
-      <c r="AC2" s="30" t="n">
+      <c r="AC2" s="40" t="n">
         <v>1.755</v>
       </c>
       <c r="AD2" s="24" t="inlineStr">
@@ -1713,11 +1744,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ2" s="25" t="n"/>
+      <c r="BJ2" s="38" t="n"/>
       <c r="BK2" s="26" t="n">
         <v>117</v>
       </c>
-      <c r="BL2" s="27" t="n">
+      <c r="BL2" s="39" t="n">
         <v>2.17</v>
       </c>
       <c r="BM2" s="28" t="n">
@@ -1727,18 +1758,18 @@
         <v>0.455446</v>
       </c>
       <c r="BO2" s="28" t="n"/>
-      <c r="BP2" s="25" t="n"/>
-      <c r="BQ2" s="27" t="n"/>
+      <c r="BP2" s="38" t="n"/>
+      <c r="BQ2" s="39" t="n"/>
       <c r="BR2" s="28" t="n"/>
       <c r="BS2" s="28" t="n"/>
       <c r="BT2" s="28" t="n"/>
-      <c r="BU2" s="25" t="n"/>
+      <c r="BU2" s="38" t="n"/>
       <c r="BV2" s="29" t="n"/>
       <c r="BW2" s="24" t="n"/>
-      <c r="BX2" s="30" t="n">
+      <c r="BX2" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="BY2" s="27" t="n">
+      <c r="BY2" s="39" t="n">
         <v>1.17</v>
       </c>
       <c r="BZ2" s="24" t="inlineStr">
@@ -1798,7 +1829,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J3" s="25" t="n"/>
+      <c r="J3" s="38" t="n"/>
       <c r="K3" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -1807,7 +1838,7 @@
       <c r="L3" s="26" t="n">
         <v>-133</v>
       </c>
-      <c r="M3" s="27" t="n">
+      <c r="M3" s="39" t="n">
         <v>1.75188</v>
       </c>
       <c r="N3" s="28" t="n">
@@ -1847,11 +1878,11 @@
       <c r="X3" s="26" t="n">
         <v>8</v>
       </c>
-      <c r="Y3" s="25" t="n"/>
+      <c r="Y3" s="38" t="n"/>
       <c r="Z3" s="26" t="n"/>
       <c r="AA3" s="28" t="n"/>
       <c r="AB3" s="28" t="n"/>
-      <c r="AC3" s="30" t="n">
+      <c r="AC3" s="40" t="n">
         <v>1.1278</v>
       </c>
       <c r="AD3" s="24" t="inlineStr">
@@ -1988,11 +2019,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ3" s="25" t="n"/>
+      <c r="BJ3" s="38" t="n"/>
       <c r="BK3" s="26" t="n">
         <v>-133</v>
       </c>
-      <c r="BL3" s="27" t="n">
+      <c r="BL3" s="39" t="n">
         <v>1.75188</v>
       </c>
       <c r="BM3" s="28" t="n">
@@ -2002,18 +2033,18 @@
         <v>0.567164</v>
       </c>
       <c r="BO3" s="28" t="n"/>
-      <c r="BP3" s="25" t="n"/>
-      <c r="BQ3" s="27" t="n"/>
+      <c r="BP3" s="38" t="n"/>
+      <c r="BQ3" s="39" t="n"/>
       <c r="BR3" s="28" t="n"/>
       <c r="BS3" s="28" t="n"/>
       <c r="BT3" s="28" t="n"/>
-      <c r="BU3" s="25" t="n"/>
+      <c r="BU3" s="38" t="n"/>
       <c r="BV3" s="29" t="n"/>
       <c r="BW3" s="24" t="n"/>
-      <c r="BX3" s="30" t="n">
+      <c r="BX3" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="BY3" s="27" t="n">
+      <c r="BY3" s="39" t="n">
         <v>0.75188</v>
       </c>
       <c r="BZ3" s="24" t="inlineStr">
@@ -2073,7 +2104,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J4" s="25" t="n"/>
+      <c r="J4" s="38" t="n"/>
       <c r="K4" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -2082,7 +2113,7 @@
       <c r="L4" s="26" t="n">
         <v>-102</v>
       </c>
-      <c r="M4" s="27" t="n">
+      <c r="M4" s="39" t="n">
         <v>1.980392</v>
       </c>
       <c r="N4" s="28" t="n">
@@ -2122,11 +2153,11 @@
       <c r="X4" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="Y4" s="25" t="n"/>
+      <c r="Y4" s="38" t="n"/>
       <c r="Z4" s="26" t="n"/>
       <c r="AA4" s="28" t="n"/>
       <c r="AB4" s="28" t="n"/>
-      <c r="AC4" s="30" t="n">
+      <c r="AC4" s="40" t="n">
         <v>-1</v>
       </c>
       <c r="AD4" s="24" t="inlineStr">
@@ -2263,11 +2294,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ4" s="25" t="n"/>
+      <c r="BJ4" s="38" t="n"/>
       <c r="BK4" s="26" t="n">
         <v>-102</v>
       </c>
-      <c r="BL4" s="27" t="n">
+      <c r="BL4" s="39" t="n">
         <v>1.980392</v>
       </c>
       <c r="BM4" s="28" t="n">
@@ -2277,18 +2308,18 @@
         <v>0.502488</v>
       </c>
       <c r="BO4" s="28" t="n"/>
-      <c r="BP4" s="25" t="n"/>
-      <c r="BQ4" s="27" t="n"/>
+      <c r="BP4" s="38" t="n"/>
+      <c r="BQ4" s="39" t="n"/>
       <c r="BR4" s="28" t="n"/>
       <c r="BS4" s="28" t="n"/>
       <c r="BT4" s="28" t="n"/>
-      <c r="BU4" s="25" t="n"/>
+      <c r="BU4" s="38" t="n"/>
       <c r="BV4" s="29" t="n"/>
       <c r="BW4" s="24" t="n"/>
-      <c r="BX4" s="30" t="n">
+      <c r="BX4" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="BY4" s="27" t="n">
+      <c r="BY4" s="39" t="n">
         <v>-1</v>
       </c>
       <c r="BZ4" s="24" t="inlineStr">
@@ -2348,7 +2379,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J5" s="25" t="n"/>
+      <c r="J5" s="38" t="n"/>
       <c r="K5" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -2357,7 +2388,7 @@
       <c r="L5" s="26" t="n">
         <v>-133</v>
       </c>
-      <c r="M5" s="27" t="n">
+      <c r="M5" s="39" t="n">
         <v>1.75188</v>
       </c>
       <c r="N5" s="28" t="n">
@@ -2397,11 +2428,11 @@
       <c r="X5" s="26" t="n">
         <v>6</v>
       </c>
-      <c r="Y5" s="25" t="n"/>
+      <c r="Y5" s="38" t="n"/>
       <c r="Z5" s="26" t="n"/>
       <c r="AA5" s="28" t="n"/>
       <c r="AB5" s="28" t="n"/>
-      <c r="AC5" s="30" t="n">
+      <c r="AC5" s="40" t="n">
         <v>1.1278</v>
       </c>
       <c r="AD5" s="24" t="inlineStr">
@@ -2538,11 +2569,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ5" s="25" t="n"/>
+      <c r="BJ5" s="38" t="n"/>
       <c r="BK5" s="26" t="n">
         <v>-133</v>
       </c>
-      <c r="BL5" s="27" t="n">
+      <c r="BL5" s="39" t="n">
         <v>1.75188</v>
       </c>
       <c r="BM5" s="28" t="n">
@@ -2552,18 +2583,18 @@
         <v>0.567164</v>
       </c>
       <c r="BO5" s="28" t="n"/>
-      <c r="BP5" s="25" t="n"/>
-      <c r="BQ5" s="27" t="n"/>
+      <c r="BP5" s="38" t="n"/>
+      <c r="BQ5" s="39" t="n"/>
       <c r="BR5" s="28" t="n"/>
       <c r="BS5" s="28" t="n"/>
       <c r="BT5" s="28" t="n"/>
-      <c r="BU5" s="25" t="n"/>
+      <c r="BU5" s="38" t="n"/>
       <c r="BV5" s="29" t="n"/>
       <c r="BW5" s="24" t="n"/>
-      <c r="BX5" s="30" t="n">
+      <c r="BX5" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="BY5" s="27" t="n">
+      <c r="BY5" s="39" t="n">
         <v>0.75188</v>
       </c>
       <c r="BZ5" s="24" t="inlineStr">
@@ -2623,7 +2654,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J6" s="25" t="n"/>
+      <c r="J6" s="38" t="n"/>
       <c r="K6" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -2632,7 +2663,7 @@
       <c r="L6" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="M6" s="27" t="n">
+      <c r="M6" s="39" t="n">
         <v>1.961538</v>
       </c>
       <c r="N6" s="28" t="n">
@@ -2672,11 +2703,11 @@
       <c r="X6" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="Y6" s="25" t="n"/>
+      <c r="Y6" s="38" t="n"/>
       <c r="Z6" s="26" t="n"/>
       <c r="AA6" s="28" t="n"/>
       <c r="AB6" s="28" t="n"/>
-      <c r="AC6" s="30" t="n">
+      <c r="AC6" s="40" t="n">
         <v>1.2019</v>
       </c>
       <c r="AD6" s="24" t="inlineStr">
@@ -2813,11 +2844,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ6" s="25" t="n"/>
+      <c r="BJ6" s="38" t="n"/>
       <c r="BK6" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="BL6" s="27" t="n">
+      <c r="BL6" s="39" t="n">
         <v>1.961538</v>
       </c>
       <c r="BM6" s="28" t="n">
@@ -2827,18 +2858,18 @@
         <v>0.507463</v>
       </c>
       <c r="BO6" s="28" t="n"/>
-      <c r="BP6" s="25" t="n"/>
-      <c r="BQ6" s="27" t="n"/>
+      <c r="BP6" s="38" t="n"/>
+      <c r="BQ6" s="39" t="n"/>
       <c r="BR6" s="28" t="n"/>
       <c r="BS6" s="28" t="n"/>
       <c r="BT6" s="28" t="n"/>
-      <c r="BU6" s="25" t="n"/>
+      <c r="BU6" s="38" t="n"/>
       <c r="BV6" s="29" t="n"/>
       <c r="BW6" s="24" t="n"/>
-      <c r="BX6" s="30" t="n">
+      <c r="BX6" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="BY6" s="27" t="n">
+      <c r="BY6" s="39" t="n">
         <v>0.961538</v>
       </c>
       <c r="BZ6" s="24" t="inlineStr">
@@ -2898,7 +2929,7 @@
           <t>away</t>
         </is>
       </c>
-      <c r="J7" s="25" t="n"/>
+      <c r="J7" s="38" t="n"/>
       <c r="K7" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -2907,7 +2938,7 @@
       <c r="L7" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="M7" s="27" t="n">
+      <c r="M7" s="39" t="n">
         <v>1.961538</v>
       </c>
       <c r="N7" s="28" t="n">
@@ -2947,11 +2978,11 @@
       <c r="X7" s="26" t="n">
         <v>10</v>
       </c>
-      <c r="Y7" s="25" t="n"/>
+      <c r="Y7" s="38" t="n"/>
       <c r="Z7" s="26" t="n"/>
       <c r="AA7" s="28" t="n"/>
       <c r="AB7" s="28" t="n"/>
-      <c r="AC7" s="30" t="n">
+      <c r="AC7" s="40" t="n">
         <v>-1.25</v>
       </c>
       <c r="AD7" s="24" t="inlineStr">
@@ -3088,11 +3119,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ7" s="25" t="n"/>
+      <c r="BJ7" s="38" t="n"/>
       <c r="BK7" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="BL7" s="27" t="n">
+      <c r="BL7" s="39" t="n">
         <v>1.961538</v>
       </c>
       <c r="BM7" s="28" t="n">
@@ -3102,18 +3133,18 @@
         <v>0.507463</v>
       </c>
       <c r="BO7" s="28" t="n"/>
-      <c r="BP7" s="25" t="n"/>
-      <c r="BQ7" s="27" t="n"/>
+      <c r="BP7" s="38" t="n"/>
+      <c r="BQ7" s="39" t="n"/>
       <c r="BR7" s="28" t="n"/>
       <c r="BS7" s="28" t="n"/>
       <c r="BT7" s="28" t="n"/>
-      <c r="BU7" s="25" t="n"/>
+      <c r="BU7" s="38" t="n"/>
       <c r="BV7" s="29" t="n"/>
       <c r="BW7" s="24" t="n"/>
-      <c r="BX7" s="30" t="n">
+      <c r="BX7" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="BY7" s="27" t="n">
+      <c r="BY7" s="39" t="n">
         <v>-1</v>
       </c>
       <c r="BZ7" s="24" t="inlineStr">
@@ -3173,7 +3204,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J8" s="25" t="n"/>
+      <c r="J8" s="38" t="n"/>
       <c r="K8" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -3182,7 +3213,7 @@
       <c r="L8" s="26" t="n">
         <v>-106</v>
       </c>
-      <c r="M8" s="27" t="n">
+      <c r="M8" s="39" t="n">
         <v>1.943396</v>
       </c>
       <c r="N8" s="28" t="n">
@@ -3222,11 +3253,11 @@
       <c r="X8" s="26" t="n">
         <v>6</v>
       </c>
-      <c r="Y8" s="25" t="n"/>
+      <c r="Y8" s="38" t="n"/>
       <c r="Z8" s="26" t="n"/>
       <c r="AA8" s="28" t="n"/>
       <c r="AB8" s="28" t="n"/>
-      <c r="AC8" s="30" t="n">
+      <c r="AC8" s="40" t="n">
         <v>-1</v>
       </c>
       <c r="AD8" s="24" t="inlineStr">
@@ -3363,11 +3394,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ8" s="25" t="n"/>
+      <c r="BJ8" s="38" t="n"/>
       <c r="BK8" s="26" t="n">
         <v>-106</v>
       </c>
-      <c r="BL8" s="27" t="n">
+      <c r="BL8" s="39" t="n">
         <v>1.943396</v>
       </c>
       <c r="BM8" s="28" t="n">
@@ -3377,18 +3408,18 @@
         <v>0.5124379999999999</v>
       </c>
       <c r="BO8" s="28" t="n"/>
-      <c r="BP8" s="25" t="n"/>
-      <c r="BQ8" s="27" t="n"/>
+      <c r="BP8" s="38" t="n"/>
+      <c r="BQ8" s="39" t="n"/>
       <c r="BR8" s="28" t="n"/>
       <c r="BS8" s="28" t="n"/>
       <c r="BT8" s="28" t="n"/>
-      <c r="BU8" s="25" t="n"/>
+      <c r="BU8" s="38" t="n"/>
       <c r="BV8" s="29" t="n"/>
       <c r="BW8" s="24" t="n"/>
-      <c r="BX8" s="30" t="n">
+      <c r="BX8" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="BY8" s="27" t="n">
+      <c r="BY8" s="39" t="n">
         <v>-1</v>
       </c>
       <c r="BZ8" s="24" t="inlineStr">
@@ -3448,7 +3479,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J9" s="25" t="n"/>
+      <c r="J9" s="38" t="n"/>
       <c r="K9" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -3457,7 +3488,7 @@
       <c r="L9" s="26" t="n">
         <v>-102</v>
       </c>
-      <c r="M9" s="27" t="n">
+      <c r="M9" s="39" t="n">
         <v>1.980392</v>
       </c>
       <c r="N9" s="28" t="n">
@@ -3497,11 +3528,11 @@
       <c r="X9" s="26" t="n">
         <v>5</v>
       </c>
-      <c r="Y9" s="25" t="n"/>
+      <c r="Y9" s="38" t="n"/>
       <c r="Z9" s="26" t="n"/>
       <c r="AA9" s="28" t="n"/>
       <c r="AB9" s="28" t="n"/>
-      <c r="AC9" s="30" t="n">
+      <c r="AC9" s="40" t="n">
         <v>0.9804</v>
       </c>
       <c r="AD9" s="24" t="inlineStr">
@@ -3638,11 +3669,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ9" s="25" t="n"/>
+      <c r="BJ9" s="38" t="n"/>
       <c r="BK9" s="26" t="n">
         <v>-102</v>
       </c>
-      <c r="BL9" s="27" t="n">
+      <c r="BL9" s="39" t="n">
         <v>1.980392</v>
       </c>
       <c r="BM9" s="28" t="n">
@@ -3652,18 +3683,18 @@
         <v>0.502488</v>
       </c>
       <c r="BO9" s="28" t="n"/>
-      <c r="BP9" s="25" t="n"/>
-      <c r="BQ9" s="27" t="n"/>
+      <c r="BP9" s="38" t="n"/>
+      <c r="BQ9" s="39" t="n"/>
       <c r="BR9" s="28" t="n"/>
       <c r="BS9" s="28" t="n"/>
       <c r="BT9" s="28" t="n"/>
-      <c r="BU9" s="25" t="n"/>
+      <c r="BU9" s="38" t="n"/>
       <c r="BV9" s="29" t="n"/>
       <c r="BW9" s="24" t="n"/>
-      <c r="BX9" s="30" t="n">
+      <c r="BX9" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="BY9" s="27" t="n">
+      <c r="BY9" s="39" t="n">
         <v>0.980392</v>
       </c>
       <c r="BZ9" s="24" t="inlineStr">
@@ -3723,7 +3754,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J10" s="25" t="n"/>
+      <c r="J10" s="38" t="n"/>
       <c r="K10" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -3732,7 +3763,7 @@
       <c r="L10" s="26" t="n">
         <v>-138</v>
       </c>
-      <c r="M10" s="27" t="n">
+      <c r="M10" s="39" t="n">
         <v>1.724638</v>
       </c>
       <c r="N10" s="28" t="n">
@@ -3772,11 +3803,11 @@
       <c r="X10" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="Y10" s="25" t="n"/>
+      <c r="Y10" s="38" t="n"/>
       <c r="Z10" s="26" t="n"/>
       <c r="AA10" s="28" t="n"/>
       <c r="AB10" s="28" t="n"/>
-      <c r="AC10" s="30" t="n">
+      <c r="AC10" s="40" t="n">
         <v>1.2681</v>
       </c>
       <c r="AD10" s="24" t="inlineStr">
@@ -3913,11 +3944,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ10" s="25" t="n"/>
+      <c r="BJ10" s="38" t="n"/>
       <c r="BK10" s="26" t="n">
         <v>-138</v>
       </c>
-      <c r="BL10" s="27" t="n">
+      <c r="BL10" s="39" t="n">
         <v>1.724638</v>
       </c>
       <c r="BM10" s="28" t="n">
@@ -3927,18 +3958,18 @@
         <v>0.577114</v>
       </c>
       <c r="BO10" s="28" t="n"/>
-      <c r="BP10" s="25" t="n"/>
-      <c r="BQ10" s="27" t="n"/>
+      <c r="BP10" s="38" t="n"/>
+      <c r="BQ10" s="39" t="n"/>
       <c r="BR10" s="28" t="n"/>
       <c r="BS10" s="28" t="n"/>
       <c r="BT10" s="28" t="n"/>
-      <c r="BU10" s="25" t="n"/>
+      <c r="BU10" s="38" t="n"/>
       <c r="BV10" s="29" t="n"/>
       <c r="BW10" s="24" t="n"/>
-      <c r="BX10" s="30" t="n">
+      <c r="BX10" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="BY10" s="27" t="n">
+      <c r="BY10" s="39" t="n">
         <v>0.724638</v>
       </c>
       <c r="BZ10" s="24" t="inlineStr">
@@ -3998,7 +4029,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J11" s="25" t="n"/>
+      <c r="J11" s="38" t="n"/>
       <c r="K11" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -4007,7 +4038,7 @@
       <c r="L11" s="26" t="n">
         <v>102</v>
       </c>
-      <c r="M11" s="27" t="n">
+      <c r="M11" s="39" t="n">
         <v>2.02</v>
       </c>
       <c r="N11" s="28" t="n">
@@ -4047,11 +4078,11 @@
       <c r="X11" s="26" t="n">
         <v>15</v>
       </c>
-      <c r="Y11" s="25" t="n"/>
+      <c r="Y11" s="38" t="n"/>
       <c r="Z11" s="26" t="n"/>
       <c r="AA11" s="28" t="n"/>
       <c r="AB11" s="28" t="n"/>
-      <c r="AC11" s="30" t="n">
+      <c r="AC11" s="40" t="n">
         <v>1.275</v>
       </c>
       <c r="AD11" s="24" t="inlineStr">
@@ -4188,11 +4219,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ11" s="25" t="n"/>
+      <c r="BJ11" s="38" t="n"/>
       <c r="BK11" s="26" t="n">
         <v>102</v>
       </c>
-      <c r="BL11" s="27" t="n">
+      <c r="BL11" s="39" t="n">
         <v>2.02</v>
       </c>
       <c r="BM11" s="28" t="n">
@@ -4202,18 +4233,18 @@
         <v>0.492537</v>
       </c>
       <c r="BO11" s="28" t="n"/>
-      <c r="BP11" s="25" t="n"/>
-      <c r="BQ11" s="27" t="n"/>
+      <c r="BP11" s="38" t="n"/>
+      <c r="BQ11" s="39" t="n"/>
       <c r="BR11" s="28" t="n"/>
       <c r="BS11" s="28" t="n"/>
       <c r="BT11" s="28" t="n"/>
-      <c r="BU11" s="25" t="n"/>
+      <c r="BU11" s="38" t="n"/>
       <c r="BV11" s="29" t="n"/>
       <c r="BW11" s="24" t="n"/>
-      <c r="BX11" s="30" t="n">
+      <c r="BX11" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="BY11" s="27" t="n">
+      <c r="BY11" s="39" t="n">
         <v>1.02</v>
       </c>
       <c r="BZ11" s="24" t="inlineStr">
@@ -4273,7 +4304,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J12" s="25" t="n"/>
+      <c r="J12" s="38" t="n"/>
       <c r="K12" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -4282,7 +4313,7 @@
       <c r="L12" s="26" t="n">
         <v>-102</v>
       </c>
-      <c r="M12" s="27" t="n">
+      <c r="M12" s="39" t="n">
         <v>1.980392</v>
       </c>
       <c r="N12" s="28" t="n">
@@ -4322,11 +4353,11 @@
       <c r="X12" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="Y12" s="25" t="n"/>
+      <c r="Y12" s="38" t="n"/>
       <c r="Z12" s="26" t="n"/>
       <c r="AA12" s="28" t="n"/>
       <c r="AB12" s="28" t="n"/>
-      <c r="AC12" s="30" t="n">
+      <c r="AC12" s="40" t="n">
         <v>-1</v>
       </c>
       <c r="AD12" s="24" t="inlineStr">
@@ -4463,11 +4494,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ12" s="25" t="n"/>
+      <c r="BJ12" s="38" t="n"/>
       <c r="BK12" s="26" t="n">
         <v>-102</v>
       </c>
-      <c r="BL12" s="27" t="n">
+      <c r="BL12" s="39" t="n">
         <v>1.980392</v>
       </c>
       <c r="BM12" s="28" t="n">
@@ -4477,18 +4508,18 @@
         <v>0.502488</v>
       </c>
       <c r="BO12" s="28" t="n"/>
-      <c r="BP12" s="25" t="n"/>
-      <c r="BQ12" s="27" t="n"/>
+      <c r="BP12" s="38" t="n"/>
+      <c r="BQ12" s="39" t="n"/>
       <c r="BR12" s="28" t="n"/>
       <c r="BS12" s="28" t="n"/>
       <c r="BT12" s="28" t="n"/>
-      <c r="BU12" s="25" t="n"/>
+      <c r="BU12" s="38" t="n"/>
       <c r="BV12" s="29" t="n"/>
       <c r="BW12" s="24" t="n"/>
-      <c r="BX12" s="30" t="n">
+      <c r="BX12" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="BY12" s="27" t="n">
+      <c r="BY12" s="39" t="n">
         <v>-1</v>
       </c>
       <c r="BZ12" s="24" t="inlineStr">
@@ -4548,7 +4579,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J13" s="25" t="n"/>
+      <c r="J13" s="38" t="n"/>
       <c r="K13" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -4557,7 +4588,7 @@
       <c r="L13" s="26" t="n">
         <v>-102</v>
       </c>
-      <c r="M13" s="27" t="n">
+      <c r="M13" s="39" t="n">
         <v>1.980392</v>
       </c>
       <c r="N13" s="28" t="n">
@@ -4597,11 +4628,11 @@
       <c r="X13" s="26" t="n">
         <v>7</v>
       </c>
-      <c r="Y13" s="25" t="n"/>
+      <c r="Y13" s="38" t="n"/>
       <c r="Z13" s="26" t="n"/>
       <c r="AA13" s="28" t="n"/>
       <c r="AB13" s="28" t="n"/>
-      <c r="AC13" s="30" t="n">
+      <c r="AC13" s="40" t="n">
         <v>1.2255</v>
       </c>
       <c r="AD13" s="24" t="inlineStr">
@@ -4738,11 +4769,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ13" s="25" t="n"/>
+      <c r="BJ13" s="38" t="n"/>
       <c r="BK13" s="26" t="n">
         <v>-102</v>
       </c>
-      <c r="BL13" s="27" t="n">
+      <c r="BL13" s="39" t="n">
         <v>1.980392</v>
       </c>
       <c r="BM13" s="28" t="n">
@@ -4752,18 +4783,18 @@
         <v>0.502488</v>
       </c>
       <c r="BO13" s="28" t="n"/>
-      <c r="BP13" s="25" t="n"/>
-      <c r="BQ13" s="27" t="n"/>
+      <c r="BP13" s="38" t="n"/>
+      <c r="BQ13" s="39" t="n"/>
       <c r="BR13" s="28" t="n"/>
       <c r="BS13" s="28" t="n"/>
       <c r="BT13" s="28" t="n"/>
-      <c r="BU13" s="25" t="n"/>
+      <c r="BU13" s="38" t="n"/>
       <c r="BV13" s="29" t="n"/>
       <c r="BW13" s="24" t="n"/>
-      <c r="BX13" s="30" t="n">
+      <c r="BX13" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="BY13" s="27" t="n">
+      <c r="BY13" s="39" t="n">
         <v>0.980392</v>
       </c>
       <c r="BZ13" s="24" t="inlineStr">
@@ -4823,7 +4854,7 @@
           <t>away</t>
         </is>
       </c>
-      <c r="J14" s="25" t="n"/>
+      <c r="J14" s="38" t="n"/>
       <c r="K14" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -4832,7 +4863,7 @@
       <c r="L14" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="M14" s="27" t="n">
+      <c r="M14" s="39" t="n">
         <v>1.961538</v>
       </c>
       <c r="N14" s="28" t="n">
@@ -4872,11 +4903,11 @@
       <c r="X14" s="26" t="n">
         <v>6</v>
       </c>
-      <c r="Y14" s="25" t="n"/>
+      <c r="Y14" s="38" t="n"/>
       <c r="Z14" s="26" t="n"/>
       <c r="AA14" s="28" t="n"/>
       <c r="AB14" s="28" t="n"/>
-      <c r="AC14" s="30" t="n">
+      <c r="AC14" s="40" t="n">
         <v>-0.75</v>
       </c>
       <c r="AD14" s="24" t="inlineStr">
@@ -5013,11 +5044,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ14" s="25" t="n"/>
+      <c r="BJ14" s="38" t="n"/>
       <c r="BK14" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="BL14" s="27" t="n">
+      <c r="BL14" s="39" t="n">
         <v>1.961538</v>
       </c>
       <c r="BM14" s="28" t="n">
@@ -5027,18 +5058,18 @@
         <v>0.507463</v>
       </c>
       <c r="BO14" s="28" t="n"/>
-      <c r="BP14" s="25" t="n"/>
-      <c r="BQ14" s="27" t="n"/>
+      <c r="BP14" s="38" t="n"/>
+      <c r="BQ14" s="39" t="n"/>
       <c r="BR14" s="28" t="n"/>
       <c r="BS14" s="28" t="n"/>
       <c r="BT14" s="28" t="n"/>
-      <c r="BU14" s="25" t="n"/>
+      <c r="BU14" s="38" t="n"/>
       <c r="BV14" s="29" t="n"/>
       <c r="BW14" s="24" t="n"/>
-      <c r="BX14" s="30" t="n">
+      <c r="BX14" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="BY14" s="27" t="n">
+      <c r="BY14" s="39" t="n">
         <v>-1</v>
       </c>
       <c r="BZ14" s="24" t="inlineStr">
@@ -5098,7 +5129,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J15" s="25" t="n"/>
+      <c r="J15" s="38" t="n"/>
       <c r="K15" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -5107,7 +5138,7 @@
       <c r="L15" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="M15" s="27" t="n">
+      <c r="M15" s="39" t="n">
         <v>1.961538</v>
       </c>
       <c r="N15" s="28" t="n">
@@ -5147,11 +5178,11 @@
       <c r="X15" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="Y15" s="25" t="n"/>
+      <c r="Y15" s="38" t="n"/>
       <c r="Z15" s="26" t="n"/>
       <c r="AA15" s="28" t="n"/>
       <c r="AB15" s="28" t="n"/>
-      <c r="AC15" s="30" t="n">
+      <c r="AC15" s="40" t="n">
         <v>-1</v>
       </c>
       <c r="AD15" s="24" t="inlineStr">
@@ -5288,11 +5319,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ15" s="25" t="n"/>
+      <c r="BJ15" s="38" t="n"/>
       <c r="BK15" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="BL15" s="27" t="n">
+      <c r="BL15" s="39" t="n">
         <v>1.961538</v>
       </c>
       <c r="BM15" s="28" t="n">
@@ -5302,18 +5333,18 @@
         <v>0.507463</v>
       </c>
       <c r="BO15" s="28" t="n"/>
-      <c r="BP15" s="25" t="n"/>
-      <c r="BQ15" s="27" t="n"/>
+      <c r="BP15" s="38" t="n"/>
+      <c r="BQ15" s="39" t="n"/>
       <c r="BR15" s="28" t="n"/>
       <c r="BS15" s="28" t="n"/>
       <c r="BT15" s="28" t="n"/>
-      <c r="BU15" s="25" t="n"/>
+      <c r="BU15" s="38" t="n"/>
       <c r="BV15" s="29" t="n"/>
       <c r="BW15" s="24" t="n"/>
-      <c r="BX15" s="30" t="n">
+      <c r="BX15" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="BY15" s="27" t="n">
+      <c r="BY15" s="39" t="n">
         <v>-1</v>
       </c>
       <c r="BZ15" s="24" t="inlineStr">
@@ -5373,7 +5404,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J16" s="25" t="n"/>
+      <c r="J16" s="38" t="n"/>
       <c r="K16" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -5382,7 +5413,7 @@
       <c r="L16" s="26" t="n">
         <v>-111</v>
       </c>
-      <c r="M16" s="27" t="n">
+      <c r="M16" s="39" t="n">
         <v>1.900901</v>
       </c>
       <c r="N16" s="28" t="n">
@@ -5422,11 +5453,11 @@
       <c r="X16" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="Y16" s="25" t="n"/>
+      <c r="Y16" s="38" t="n"/>
       <c r="Z16" s="26" t="n"/>
       <c r="AA16" s="28" t="n"/>
       <c r="AB16" s="28" t="n"/>
-      <c r="AC16" s="30" t="n">
+      <c r="AC16" s="40" t="n">
         <v>-1.5</v>
       </c>
       <c r="AD16" s="24" t="inlineStr">
@@ -5563,11 +5594,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ16" s="25" t="n"/>
+      <c r="BJ16" s="38" t="n"/>
       <c r="BK16" s="26" t="n">
         <v>-111</v>
       </c>
-      <c r="BL16" s="27" t="n">
+      <c r="BL16" s="39" t="n">
         <v>1.900901</v>
       </c>
       <c r="BM16" s="28" t="n">
@@ -5577,18 +5608,18 @@
         <v>0.522388</v>
       </c>
       <c r="BO16" s="28" t="n"/>
-      <c r="BP16" s="25" t="n"/>
-      <c r="BQ16" s="27" t="n"/>
+      <c r="BP16" s="38" t="n"/>
+      <c r="BQ16" s="39" t="n"/>
       <c r="BR16" s="28" t="n"/>
       <c r="BS16" s="28" t="n"/>
       <c r="BT16" s="28" t="n"/>
-      <c r="BU16" s="25" t="n"/>
+      <c r="BU16" s="38" t="n"/>
       <c r="BV16" s="29" t="n"/>
       <c r="BW16" s="24" t="n"/>
-      <c r="BX16" s="30" t="n">
+      <c r="BX16" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="BY16" s="27" t="n">
+      <c r="BY16" s="39" t="n">
         <v>-1</v>
       </c>
       <c r="BZ16" s="24" t="inlineStr">
@@ -5648,7 +5679,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J17" s="25" t="n"/>
+      <c r="J17" s="38" t="n"/>
       <c r="K17" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -5657,7 +5688,7 @@
       <c r="L17" s="26" t="n">
         <v>-108</v>
       </c>
-      <c r="M17" s="27" t="n">
+      <c r="M17" s="39" t="n">
         <v>1.925926</v>
       </c>
       <c r="N17" s="28" t="n">
@@ -5697,11 +5728,11 @@
       <c r="X17" s="26" t="n">
         <v>6</v>
       </c>
-      <c r="Y17" s="25" t="n"/>
+      <c r="Y17" s="38" t="n"/>
       <c r="Z17" s="26" t="n"/>
       <c r="AA17" s="28" t="n"/>
       <c r="AB17" s="28" t="n"/>
-      <c r="AC17" s="30" t="n">
+      <c r="AC17" s="40" t="n">
         <v>0.9258999999999999</v>
       </c>
       <c r="AD17" s="24" t="inlineStr">
@@ -5838,11 +5869,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ17" s="25" t="n"/>
+      <c r="BJ17" s="38" t="n"/>
       <c r="BK17" s="26" t="n">
         <v>-108</v>
       </c>
-      <c r="BL17" s="27" t="n">
+      <c r="BL17" s="39" t="n">
         <v>1.925926</v>
       </c>
       <c r="BM17" s="28" t="n">
@@ -5852,18 +5883,18 @@
         <v>0.5148509999999999</v>
       </c>
       <c r="BO17" s="28" t="n"/>
-      <c r="BP17" s="25" t="n"/>
-      <c r="BQ17" s="27" t="n"/>
+      <c r="BP17" s="38" t="n"/>
+      <c r="BQ17" s="39" t="n"/>
       <c r="BR17" s="28" t="n"/>
       <c r="BS17" s="28" t="n"/>
       <c r="BT17" s="28" t="n"/>
-      <c r="BU17" s="25" t="n"/>
+      <c r="BU17" s="38" t="n"/>
       <c r="BV17" s="29" t="n"/>
       <c r="BW17" s="24" t="n"/>
-      <c r="BX17" s="30" t="n">
+      <c r="BX17" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="BY17" s="27" t="n">
+      <c r="BY17" s="39" t="n">
         <v>0.925926</v>
       </c>
       <c r="BZ17" s="24" t="inlineStr">
@@ -5923,7 +5954,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J18" s="25" t="n"/>
+      <c r="J18" s="38" t="n"/>
       <c r="K18" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -5932,7 +5963,7 @@
       <c r="L18" s="26" t="n">
         <v>111</v>
       </c>
-      <c r="M18" s="27" t="n">
+      <c r="M18" s="39" t="n">
         <v>2.11</v>
       </c>
       <c r="N18" s="28" t="n">
@@ -5972,11 +6003,11 @@
       <c r="X18" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="Y18" s="25" t="n"/>
+      <c r="Y18" s="38" t="n"/>
       <c r="Z18" s="26" t="n"/>
       <c r="AA18" s="28" t="n"/>
       <c r="AB18" s="28" t="n"/>
-      <c r="AC18" s="30" t="n">
+      <c r="AC18" s="40" t="n">
         <v>-1.25</v>
       </c>
       <c r="AD18" s="24" t="inlineStr">
@@ -6113,11 +6144,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ18" s="25" t="n"/>
+      <c r="BJ18" s="38" t="n"/>
       <c r="BK18" s="26" t="n">
         <v>111</v>
       </c>
-      <c r="BL18" s="27" t="n">
+      <c r="BL18" s="39" t="n">
         <v>2.11</v>
       </c>
       <c r="BM18" s="28" t="n">
@@ -6127,18 +6158,18 @@
         <v>0.472637</v>
       </c>
       <c r="BO18" s="28" t="n"/>
-      <c r="BP18" s="25" t="n"/>
-      <c r="BQ18" s="27" t="n"/>
+      <c r="BP18" s="38" t="n"/>
+      <c r="BQ18" s="39" t="n"/>
       <c r="BR18" s="28" t="n"/>
       <c r="BS18" s="28" t="n"/>
       <c r="BT18" s="28" t="n"/>
-      <c r="BU18" s="25" t="n"/>
+      <c r="BU18" s="38" t="n"/>
       <c r="BV18" s="29" t="n"/>
       <c r="BW18" s="24" t="n"/>
-      <c r="BX18" s="30" t="n">
+      <c r="BX18" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="BY18" s="27" t="n">
+      <c r="BY18" s="39" t="n">
         <v>-1</v>
       </c>
       <c r="BZ18" s="24" t="inlineStr">
@@ -6198,7 +6229,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J19" s="25" t="n"/>
+      <c r="J19" s="38" t="n"/>
       <c r="K19" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -6207,7 +6238,7 @@
       <c r="L19" s="26" t="n">
         <v>-125</v>
       </c>
-      <c r="M19" s="27" t="n">
+      <c r="M19" s="39" t="n">
         <v>1.8</v>
       </c>
       <c r="N19" s="28" t="n">
@@ -6247,11 +6278,11 @@
       <c r="X19" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="Y19" s="25" t="n"/>
+      <c r="Y19" s="38" t="n"/>
       <c r="Z19" s="26" t="n"/>
       <c r="AA19" s="28" t="n"/>
       <c r="AB19" s="28" t="n"/>
-      <c r="AC19" s="30" t="n">
+      <c r="AC19" s="40" t="n">
         <v>1.2</v>
       </c>
       <c r="AD19" s="24" t="inlineStr">
@@ -6388,11 +6419,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ19" s="25" t="n"/>
+      <c r="BJ19" s="38" t="n"/>
       <c r="BK19" s="26" t="n">
         <v>-125</v>
       </c>
-      <c r="BL19" s="27" t="n">
+      <c r="BL19" s="39" t="n">
         <v>1.8</v>
       </c>
       <c r="BM19" s="28" t="n">
@@ -6402,18 +6433,18 @@
         <v>0.552239</v>
       </c>
       <c r="BO19" s="28" t="n"/>
-      <c r="BP19" s="25" t="n"/>
-      <c r="BQ19" s="27" t="n"/>
+      <c r="BP19" s="38" t="n"/>
+      <c r="BQ19" s="39" t="n"/>
       <c r="BR19" s="28" t="n"/>
       <c r="BS19" s="28" t="n"/>
       <c r="BT19" s="28" t="n"/>
-      <c r="BU19" s="25" t="n"/>
+      <c r="BU19" s="38" t="n"/>
       <c r="BV19" s="29" t="n"/>
       <c r="BW19" s="24" t="n"/>
-      <c r="BX19" s="30" t="n">
+      <c r="BX19" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="BY19" s="27" t="n">
+      <c r="BY19" s="39" t="n">
         <v>0.8</v>
       </c>
       <c r="BZ19" s="24" t="inlineStr">
@@ -6473,7 +6504,7 @@
           <t>away</t>
         </is>
       </c>
-      <c r="J20" s="25" t="n"/>
+      <c r="J20" s="38" t="n"/>
       <c r="K20" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -6482,7 +6513,7 @@
       <c r="L20" s="26" t="n">
         <v>106</v>
       </c>
-      <c r="M20" s="27" t="n">
+      <c r="M20" s="39" t="n">
         <v>2.06</v>
       </c>
       <c r="N20" s="28" t="n">
@@ -6522,11 +6553,11 @@
       <c r="X20" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="Y20" s="25" t="n"/>
+      <c r="Y20" s="38" t="n"/>
       <c r="Z20" s="26" t="n"/>
       <c r="AA20" s="28" t="n"/>
       <c r="AB20" s="28" t="n"/>
-      <c r="AC20" s="30" t="n">
+      <c r="AC20" s="40" t="n">
         <v>0.795</v>
       </c>
       <c r="AD20" s="24" t="inlineStr">
@@ -6663,11 +6694,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ20" s="25" t="n"/>
+      <c r="BJ20" s="38" t="n"/>
       <c r="BK20" s="26" t="n">
         <v>106</v>
       </c>
-      <c r="BL20" s="27" t="n">
+      <c r="BL20" s="39" t="n">
         <v>2.06</v>
       </c>
       <c r="BM20" s="28" t="n">
@@ -6677,18 +6708,18 @@
         <v>0.482587</v>
       </c>
       <c r="BO20" s="28" t="n"/>
-      <c r="BP20" s="25" t="n"/>
-      <c r="BQ20" s="27" t="n"/>
+      <c r="BP20" s="38" t="n"/>
+      <c r="BQ20" s="39" t="n"/>
       <c r="BR20" s="28" t="n"/>
       <c r="BS20" s="28" t="n"/>
       <c r="BT20" s="28" t="n"/>
-      <c r="BU20" s="25" t="n"/>
+      <c r="BU20" s="38" t="n"/>
       <c r="BV20" s="29" t="n"/>
       <c r="BW20" s="24" t="n"/>
-      <c r="BX20" s="30" t="n">
+      <c r="BX20" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="BY20" s="27" t="n">
+      <c r="BY20" s="39" t="n">
         <v>1.06</v>
       </c>
       <c r="BZ20" s="24" t="inlineStr">
@@ -6748,7 +6779,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J21" s="25" t="n"/>
+      <c r="J21" s="38" t="n"/>
       <c r="K21" s="24" t="inlineStr">
         <is>
           <t>polymarket</t>
@@ -6757,7 +6788,7 @@
       <c r="L21" s="26" t="n">
         <v>-106</v>
       </c>
-      <c r="M21" s="27" t="n">
+      <c r="M21" s="39" t="n">
         <v>1.943396</v>
       </c>
       <c r="N21" s="28" t="n">
@@ -6797,11 +6828,11 @@
       <c r="X21" s="26" t="n">
         <v>10</v>
       </c>
-      <c r="Y21" s="25" t="n"/>
+      <c r="Y21" s="38" t="n"/>
       <c r="Z21" s="26" t="n"/>
       <c r="AA21" s="28" t="n"/>
       <c r="AB21" s="28" t="n"/>
-      <c r="AC21" s="30" t="n">
+      <c r="AC21" s="40" t="n">
         <v>0.9434</v>
       </c>
       <c r="AD21" s="24" t="inlineStr">
@@ -6848,11 +6879,11 @@
         </is>
       </c>
       <c r="BI21" s="24" t="n"/>
-      <c r="BJ21" s="25" t="n"/>
+      <c r="BJ21" s="38" t="n"/>
       <c r="BK21" s="26" t="n">
         <v>-106</v>
       </c>
-      <c r="BL21" s="27" t="n">
+      <c r="BL21" s="39" t="n">
         <v>1.943396</v>
       </c>
       <c r="BM21" s="28" t="n">
@@ -6862,16 +6893,16 @@
         <v>0.5124379999999999</v>
       </c>
       <c r="BO21" s="28" t="n"/>
-      <c r="BP21" s="25" t="n"/>
-      <c r="BQ21" s="27" t="n"/>
+      <c r="BP21" s="38" t="n"/>
+      <c r="BQ21" s="39" t="n"/>
       <c r="BR21" s="28" t="n"/>
       <c r="BS21" s="28" t="n"/>
       <c r="BT21" s="28" t="n"/>
-      <c r="BU21" s="25" t="n"/>
+      <c r="BU21" s="38" t="n"/>
       <c r="BV21" s="29" t="n"/>
       <c r="BW21" s="24" t="n"/>
-      <c r="BX21" s="30" t="n"/>
-      <c r="BY21" s="27" t="n"/>
+      <c r="BX21" s="40" t="n"/>
+      <c r="BY21" s="39" t="n"/>
       <c r="BZ21" s="24" t="n"/>
       <c r="CA21" s="31" t="n"/>
     </row>
@@ -6921,7 +6952,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J22" s="25" t="n"/>
+      <c r="J22" s="38" t="n"/>
       <c r="K22" s="24" t="inlineStr">
         <is>
           <t>polymarket</t>
@@ -6930,7 +6961,7 @@
       <c r="L22" s="26" t="n">
         <v>-106</v>
       </c>
-      <c r="M22" s="27" t="n">
+      <c r="M22" s="39" t="n">
         <v>1.943396</v>
       </c>
       <c r="N22" s="28" t="n">
@@ -6970,11 +7001,11 @@
       <c r="X22" s="26" t="n">
         <v>5</v>
       </c>
-      <c r="Y22" s="25" t="n"/>
+      <c r="Y22" s="38" t="n"/>
       <c r="Z22" s="26" t="n"/>
       <c r="AA22" s="28" t="n"/>
       <c r="AB22" s="28" t="n"/>
-      <c r="AC22" s="30" t="n">
+      <c r="AC22" s="40" t="n">
         <v>0.9434</v>
       </c>
       <c r="AD22" s="24" t="inlineStr">
@@ -7021,11 +7052,11 @@
         </is>
       </c>
       <c r="BI22" s="24" t="n"/>
-      <c r="BJ22" s="25" t="n"/>
+      <c r="BJ22" s="38" t="n"/>
       <c r="BK22" s="26" t="n">
         <v>-106</v>
       </c>
-      <c r="BL22" s="27" t="n">
+      <c r="BL22" s="39" t="n">
         <v>1.943396</v>
       </c>
       <c r="BM22" s="28" t="n">
@@ -7035,16 +7066,16 @@
         <v>0.5124379999999999</v>
       </c>
       <c r="BO22" s="28" t="n"/>
-      <c r="BP22" s="25" t="n"/>
-      <c r="BQ22" s="27" t="n"/>
+      <c r="BP22" s="38" t="n"/>
+      <c r="BQ22" s="39" t="n"/>
       <c r="BR22" s="28" t="n"/>
       <c r="BS22" s="28" t="n"/>
       <c r="BT22" s="28" t="n"/>
-      <c r="BU22" s="25" t="n"/>
+      <c r="BU22" s="38" t="n"/>
       <c r="BV22" s="29" t="n"/>
       <c r="BW22" s="24" t="n"/>
-      <c r="BX22" s="30" t="n"/>
-      <c r="BY22" s="27" t="n"/>
+      <c r="BX22" s="40" t="n"/>
+      <c r="BY22" s="39" t="n"/>
       <c r="BZ22" s="24" t="n"/>
       <c r="CA22" s="31" t="n"/>
     </row>
@@ -7094,7 +7125,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J23" s="25" t="n"/>
+      <c r="J23" s="38" t="n"/>
       <c r="K23" s="24" t="inlineStr">
         <is>
           <t>polymarket</t>
@@ -7103,7 +7134,7 @@
       <c r="L23" s="26" t="n">
         <v>-141</v>
       </c>
-      <c r="M23" s="27" t="n">
+      <c r="M23" s="39" t="n">
         <v>1.70922</v>
       </c>
       <c r="N23" s="28" t="n">
@@ -7143,11 +7174,11 @@
       <c r="X23" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="Y23" s="25" t="n"/>
+      <c r="Y23" s="38" t="n"/>
       <c r="Z23" s="26" t="n"/>
       <c r="AA23" s="28" t="n"/>
       <c r="AB23" s="28" t="n"/>
-      <c r="AC23" s="30" t="n">
+      <c r="AC23" s="40" t="n">
         <v>1.2411</v>
       </c>
       <c r="AD23" s="24" t="inlineStr">
@@ -7194,11 +7225,11 @@
         </is>
       </c>
       <c r="BI23" s="24" t="n"/>
-      <c r="BJ23" s="25" t="n"/>
+      <c r="BJ23" s="38" t="n"/>
       <c r="BK23" s="26" t="n">
         <v>-141</v>
       </c>
-      <c r="BL23" s="27" t="n">
+      <c r="BL23" s="39" t="n">
         <v>1.70922</v>
       </c>
       <c r="BM23" s="28" t="n">
@@ -7208,16 +7239,16 @@
         <v>0.58209</v>
       </c>
       <c r="BO23" s="28" t="n"/>
-      <c r="BP23" s="25" t="n"/>
-      <c r="BQ23" s="27" t="n"/>
+      <c r="BP23" s="38" t="n"/>
+      <c r="BQ23" s="39" t="n"/>
       <c r="BR23" s="28" t="n"/>
       <c r="BS23" s="28" t="n"/>
       <c r="BT23" s="28" t="n"/>
-      <c r="BU23" s="25" t="n"/>
+      <c r="BU23" s="38" t="n"/>
       <c r="BV23" s="29" t="n"/>
       <c r="BW23" s="24" t="n"/>
-      <c r="BX23" s="30" t="n"/>
-      <c r="BY23" s="27" t="n"/>
+      <c r="BX23" s="40" t="n"/>
+      <c r="BY23" s="39" t="n"/>
       <c r="BZ23" s="24" t="n"/>
       <c r="CA23" s="31" t="n"/>
     </row>
@@ -7267,7 +7298,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J24" s="25" t="n"/>
+      <c r="J24" s="38" t="n"/>
       <c r="K24" s="24" t="inlineStr">
         <is>
           <t>polymarket</t>
@@ -7276,7 +7307,7 @@
       <c r="L24" s="26" t="n">
         <v>-133</v>
       </c>
-      <c r="M24" s="27" t="n">
+      <c r="M24" s="39" t="n">
         <v>1.75188</v>
       </c>
       <c r="N24" s="28" t="n">
@@ -7316,11 +7347,11 @@
       <c r="X24" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="Y24" s="25" t="n"/>
+      <c r="Y24" s="38" t="n"/>
       <c r="Z24" s="26" t="n"/>
       <c r="AA24" s="28" t="n"/>
       <c r="AB24" s="28" t="n"/>
-      <c r="AC24" s="30" t="n">
+      <c r="AC24" s="40" t="n">
         <v>-1.5</v>
       </c>
       <c r="AD24" s="24" t="inlineStr">
@@ -7367,11 +7398,11 @@
         </is>
       </c>
       <c r="BI24" s="24" t="n"/>
-      <c r="BJ24" s="25" t="n"/>
+      <c r="BJ24" s="38" t="n"/>
       <c r="BK24" s="26" t="n">
         <v>-133</v>
       </c>
-      <c r="BL24" s="27" t="n">
+      <c r="BL24" s="39" t="n">
         <v>1.75188</v>
       </c>
       <c r="BM24" s="28" t="n">
@@ -7381,16 +7412,16 @@
         <v>0.567164</v>
       </c>
       <c r="BO24" s="28" t="n"/>
-      <c r="BP24" s="25" t="n"/>
-      <c r="BQ24" s="27" t="n"/>
+      <c r="BP24" s="38" t="n"/>
+      <c r="BQ24" s="39" t="n"/>
       <c r="BR24" s="28" t="n"/>
       <c r="BS24" s="28" t="n"/>
       <c r="BT24" s="28" t="n"/>
-      <c r="BU24" s="25" t="n"/>
+      <c r="BU24" s="38" t="n"/>
       <c r="BV24" s="29" t="n"/>
       <c r="BW24" s="24" t="n"/>
-      <c r="BX24" s="30" t="n"/>
-      <c r="BY24" s="27" t="n"/>
+      <c r="BX24" s="40" t="n"/>
+      <c r="BY24" s="39" t="n"/>
       <c r="BZ24" s="24" t="n"/>
       <c r="CA24" s="31" t="n"/>
     </row>
@@ -7440,7 +7471,7 @@
           <t>away</t>
         </is>
       </c>
-      <c r="J25" s="25" t="n"/>
+      <c r="J25" s="38" t="n"/>
       <c r="K25" s="24" t="inlineStr">
         <is>
           <t>polymarket</t>
@@ -7449,7 +7480,7 @@
       <c r="L25" s="26" t="n">
         <v>104</v>
       </c>
-      <c r="M25" s="27" t="n">
+      <c r="M25" s="39" t="n">
         <v>2.04</v>
       </c>
       <c r="N25" s="28" t="n">
@@ -7489,11 +7520,11 @@
       <c r="X25" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="Y25" s="25" t="n"/>
+      <c r="Y25" s="38" t="n"/>
       <c r="Z25" s="26" t="n"/>
       <c r="AA25" s="28" t="n"/>
       <c r="AB25" s="28" t="n"/>
-      <c r="AC25" s="30" t="n">
+      <c r="AC25" s="40" t="n">
         <v>1.3</v>
       </c>
       <c r="AD25" s="24" t="inlineStr">
@@ -7540,11 +7571,11 @@
         </is>
       </c>
       <c r="BI25" s="24" t="n"/>
-      <c r="BJ25" s="25" t="n"/>
+      <c r="BJ25" s="38" t="n"/>
       <c r="BK25" s="26" t="n">
         <v>104</v>
       </c>
-      <c r="BL25" s="27" t="n">
+      <c r="BL25" s="39" t="n">
         <v>2.04</v>
       </c>
       <c r="BM25" s="28" t="n">
@@ -7554,16 +7585,16 @@
         <v>0.487562</v>
       </c>
       <c r="BO25" s="28" t="n"/>
-      <c r="BP25" s="25" t="n"/>
-      <c r="BQ25" s="27" t="n"/>
+      <c r="BP25" s="38" t="n"/>
+      <c r="BQ25" s="39" t="n"/>
       <c r="BR25" s="28" t="n"/>
       <c r="BS25" s="28" t="n"/>
       <c r="BT25" s="28" t="n"/>
-      <c r="BU25" s="25" t="n"/>
+      <c r="BU25" s="38" t="n"/>
       <c r="BV25" s="29" t="n"/>
       <c r="BW25" s="24" t="n"/>
-      <c r="BX25" s="30" t="n"/>
-      <c r="BY25" s="27" t="n"/>
+      <c r="BX25" s="40" t="n"/>
+      <c r="BY25" s="39" t="n"/>
       <c r="BZ25" s="24" t="n"/>
       <c r="CA25" s="31" t="n"/>
     </row>
@@ -7613,7 +7644,7 @@
           <t>away</t>
         </is>
       </c>
-      <c r="J26" s="25" t="n"/>
+      <c r="J26" s="38" t="n"/>
       <c r="K26" s="24" t="inlineStr">
         <is>
           <t>polymarket</t>
@@ -7622,7 +7653,7 @@
       <c r="L26" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="M26" s="27" t="n">
+      <c r="M26" s="39" t="n">
         <v>1.961538</v>
       </c>
       <c r="N26" s="28" t="n">
@@ -7662,11 +7693,11 @@
       <c r="X26" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="Y26" s="25" t="n"/>
+      <c r="Y26" s="38" t="n"/>
       <c r="Z26" s="26" t="n"/>
       <c r="AA26" s="28" t="n"/>
       <c r="AB26" s="28" t="n"/>
-      <c r="AC26" s="30" t="n">
+      <c r="AC26" s="40" t="n">
         <v>0.9615</v>
       </c>
       <c r="AD26" s="24" t="inlineStr">
@@ -7713,11 +7744,11 @@
         </is>
       </c>
       <c r="BI26" s="24" t="n"/>
-      <c r="BJ26" s="25" t="n"/>
+      <c r="BJ26" s="38" t="n"/>
       <c r="BK26" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="BL26" s="27" t="n">
+      <c r="BL26" s="39" t="n">
         <v>1.961538</v>
       </c>
       <c r="BM26" s="28" t="n">
@@ -7727,16 +7758,16 @@
         <v>0.507463</v>
       </c>
       <c r="BO26" s="28" t="n"/>
-      <c r="BP26" s="25" t="n"/>
-      <c r="BQ26" s="27" t="n"/>
+      <c r="BP26" s="38" t="n"/>
+      <c r="BQ26" s="39" t="n"/>
       <c r="BR26" s="28" t="n"/>
       <c r="BS26" s="28" t="n"/>
       <c r="BT26" s="28" t="n"/>
-      <c r="BU26" s="25" t="n"/>
+      <c r="BU26" s="38" t="n"/>
       <c r="BV26" s="29" t="n"/>
       <c r="BW26" s="24" t="n"/>
-      <c r="BX26" s="30" t="n"/>
-      <c r="BY26" s="27" t="n"/>
+      <c r="BX26" s="40" t="n"/>
+      <c r="BY26" s="39" t="n"/>
       <c r="BZ26" s="24" t="n"/>
       <c r="CA26" s="31" t="n"/>
     </row>
@@ -7786,7 +7817,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J27" s="25" t="n"/>
+      <c r="J27" s="38" t="n"/>
       <c r="K27" s="24" t="inlineStr">
         <is>
           <t>polymarket</t>
@@ -7795,7 +7826,7 @@
       <c r="L27" s="26" t="n">
         <v>120</v>
       </c>
-      <c r="M27" s="27" t="n">
+      <c r="M27" s="39" t="n">
         <v>2.2</v>
       </c>
       <c r="N27" s="28" t="n">
@@ -7835,11 +7866,11 @@
       <c r="X27" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="Y27" s="25" t="n"/>
+      <c r="Y27" s="38" t="n"/>
       <c r="Z27" s="26" t="n"/>
       <c r="AA27" s="28" t="n"/>
       <c r="AB27" s="28" t="n"/>
-      <c r="AC27" s="30" t="n">
+      <c r="AC27" s="40" t="n">
         <v>-0.75</v>
       </c>
       <c r="AD27" s="24" t="inlineStr">
@@ -7886,11 +7917,11 @@
         </is>
       </c>
       <c r="BI27" s="24" t="n"/>
-      <c r="BJ27" s="25" t="n"/>
+      <c r="BJ27" s="38" t="n"/>
       <c r="BK27" s="26" t="n">
         <v>120</v>
       </c>
-      <c r="BL27" s="27" t="n">
+      <c r="BL27" s="39" t="n">
         <v>2.2</v>
       </c>
       <c r="BM27" s="28" t="n">
@@ -7900,16 +7931,16 @@
         <v>0.452736</v>
       </c>
       <c r="BO27" s="28" t="n"/>
-      <c r="BP27" s="25" t="n"/>
-      <c r="BQ27" s="27" t="n"/>
+      <c r="BP27" s="38" t="n"/>
+      <c r="BQ27" s="39" t="n"/>
       <c r="BR27" s="28" t="n"/>
       <c r="BS27" s="28" t="n"/>
       <c r="BT27" s="28" t="n"/>
-      <c r="BU27" s="25" t="n"/>
+      <c r="BU27" s="38" t="n"/>
       <c r="BV27" s="29" t="n"/>
       <c r="BW27" s="24" t="n"/>
-      <c r="BX27" s="30" t="n"/>
-      <c r="BY27" s="27" t="n"/>
+      <c r="BX27" s="40" t="n"/>
+      <c r="BY27" s="39" t="n"/>
       <c r="BZ27" s="24" t="n"/>
       <c r="CA27" s="31" t="n"/>
     </row>
@@ -7959,7 +7990,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J28" s="25" t="n"/>
+      <c r="J28" s="38" t="n"/>
       <c r="K28" s="24" t="inlineStr">
         <is>
           <t>polymarket</t>
@@ -7968,7 +7999,7 @@
       <c r="L28" s="26" t="n">
         <v>100</v>
       </c>
-      <c r="M28" s="27" t="n">
+      <c r="M28" s="39" t="n">
         <v>2</v>
       </c>
       <c r="N28" s="28" t="n">
@@ -8008,11 +8039,11 @@
       <c r="X28" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="Y28" s="25" t="n"/>
+      <c r="Y28" s="38" t="n"/>
       <c r="Z28" s="26" t="n"/>
       <c r="AA28" s="28" t="n"/>
       <c r="AB28" s="28" t="n"/>
-      <c r="AC28" s="30" t="n">
+      <c r="AC28" s="40" t="n">
         <v>-0.75</v>
       </c>
       <c r="AD28" s="24" t="inlineStr">
@@ -8059,11 +8090,11 @@
         </is>
       </c>
       <c r="BI28" s="24" t="n"/>
-      <c r="BJ28" s="25" t="n"/>
+      <c r="BJ28" s="38" t="n"/>
       <c r="BK28" s="26" t="n">
         <v>100</v>
       </c>
-      <c r="BL28" s="27" t="n">
+      <c r="BL28" s="39" t="n">
         <v>2</v>
       </c>
       <c r="BM28" s="28" t="n">
@@ -8073,16 +8104,16 @@
         <v>0.497512</v>
       </c>
       <c r="BO28" s="28" t="n"/>
-      <c r="BP28" s="25" t="n"/>
-      <c r="BQ28" s="27" t="n"/>
+      <c r="BP28" s="38" t="n"/>
+      <c r="BQ28" s="39" t="n"/>
       <c r="BR28" s="28" t="n"/>
       <c r="BS28" s="28" t="n"/>
       <c r="BT28" s="28" t="n"/>
-      <c r="BU28" s="25" t="n"/>
+      <c r="BU28" s="38" t="n"/>
       <c r="BV28" s="29" t="n"/>
       <c r="BW28" s="24" t="n"/>
-      <c r="BX28" s="30" t="n"/>
-      <c r="BY28" s="27" t="n"/>
+      <c r="BX28" s="40" t="n"/>
+      <c r="BY28" s="39" t="n"/>
       <c r="BZ28" s="24" t="n"/>
       <c r="CA28" s="31" t="n"/>
     </row>
@@ -8132,7 +8163,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J29" s="25" t="n"/>
+      <c r="J29" s="38" t="n"/>
       <c r="K29" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -8141,7 +8172,7 @@
       <c r="L29" s="26" t="n">
         <v>108</v>
       </c>
-      <c r="M29" s="27" t="n">
+      <c r="M29" s="39" t="n">
         <v>2.08</v>
       </c>
       <c r="N29" s="28" t="n">
@@ -8181,11 +8212,11 @@
       <c r="X29" s="26" t="n">
         <v>8</v>
       </c>
-      <c r="Y29" s="25" t="n"/>
+      <c r="Y29" s="38" t="n"/>
       <c r="Z29" s="26" t="n"/>
       <c r="AA29" s="28" t="n"/>
       <c r="AB29" s="28" t="n"/>
-      <c r="AC29" s="30" t="n">
+      <c r="AC29" s="40" t="n">
         <v>1.35</v>
       </c>
       <c r="AD29" s="24" t="inlineStr">
@@ -8322,11 +8353,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ29" s="25" t="n"/>
+      <c r="BJ29" s="38" t="n"/>
       <c r="BK29" s="26" t="n">
         <v>108</v>
       </c>
-      <c r="BL29" s="27" t="n">
+      <c r="BL29" s="39" t="n">
         <v>2.08</v>
       </c>
       <c r="BM29" s="28" t="n">
@@ -8336,18 +8367,18 @@
         <v>0.477612</v>
       </c>
       <c r="BO29" s="28" t="n"/>
-      <c r="BP29" s="25" t="n"/>
-      <c r="BQ29" s="27" t="n"/>
+      <c r="BP29" s="38" t="n"/>
+      <c r="BQ29" s="39" t="n"/>
       <c r="BR29" s="28" t="n"/>
       <c r="BS29" s="28" t="n"/>
       <c r="BT29" s="28" t="n"/>
-      <c r="BU29" s="25" t="n"/>
+      <c r="BU29" s="38" t="n"/>
       <c r="BV29" s="29" t="n"/>
       <c r="BW29" s="24" t="n"/>
-      <c r="BX29" s="30" t="n">
+      <c r="BX29" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="BY29" s="27" t="n">
+      <c r="BY29" s="39" t="n">
         <v>1.08</v>
       </c>
       <c r="BZ29" s="24" t="inlineStr">
@@ -8407,7 +8438,7 @@
           <t>away</t>
         </is>
       </c>
-      <c r="J30" s="25" t="n"/>
+      <c r="J30" s="38" t="n"/>
       <c r="K30" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -8416,7 +8447,7 @@
       <c r="L30" s="26" t="n">
         <v>-133</v>
       </c>
-      <c r="M30" s="27" t="n">
+      <c r="M30" s="39" t="n">
         <v>1.75188</v>
       </c>
       <c r="N30" s="28" t="n">
@@ -8456,11 +8487,11 @@
       <c r="X30" s="26" t="n">
         <v>6</v>
       </c>
-      <c r="Y30" s="25" t="n"/>
+      <c r="Y30" s="38" t="n"/>
       <c r="Z30" s="26" t="n"/>
       <c r="AA30" s="28" t="n"/>
       <c r="AB30" s="28" t="n"/>
-      <c r="AC30" s="30" t="n">
+      <c r="AC30" s="40" t="n">
         <v>1.1278</v>
       </c>
       <c r="AD30" s="24" t="inlineStr">
@@ -8597,11 +8628,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ30" s="25" t="n"/>
+      <c r="BJ30" s="38" t="n"/>
       <c r="BK30" s="26" t="n">
         <v>-133</v>
       </c>
-      <c r="BL30" s="27" t="n">
+      <c r="BL30" s="39" t="n">
         <v>1.75188</v>
       </c>
       <c r="BM30" s="28" t="n">
@@ -8611,18 +8642,18 @@
         <v>0.567164</v>
       </c>
       <c r="BO30" s="28" t="n"/>
-      <c r="BP30" s="25" t="n"/>
-      <c r="BQ30" s="27" t="n"/>
+      <c r="BP30" s="38" t="n"/>
+      <c r="BQ30" s="39" t="n"/>
       <c r="BR30" s="28" t="n"/>
       <c r="BS30" s="28" t="n"/>
       <c r="BT30" s="28" t="n"/>
-      <c r="BU30" s="25" t="n"/>
+      <c r="BU30" s="38" t="n"/>
       <c r="BV30" s="29" t="n"/>
       <c r="BW30" s="24" t="n"/>
-      <c r="BX30" s="30" t="n">
+      <c r="BX30" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="BY30" s="27" t="n">
+      <c r="BY30" s="39" t="n">
         <v>0.75188</v>
       </c>
       <c r="BZ30" s="24" t="inlineStr">
@@ -8682,7 +8713,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J31" s="25" t="n"/>
+      <c r="J31" s="38" t="n"/>
       <c r="K31" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -8691,7 +8722,7 @@
       <c r="L31" s="26" t="n">
         <v>130</v>
       </c>
-      <c r="M31" s="27" t="n">
+      <c r="M31" s="39" t="n">
         <v>2.3</v>
       </c>
       <c r="N31" s="28" t="n">
@@ -8731,11 +8762,11 @@
       <c r="X31" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="Y31" s="25" t="n"/>
+      <c r="Y31" s="38" t="n"/>
       <c r="Z31" s="26" t="n"/>
       <c r="AA31" s="28" t="n"/>
       <c r="AB31" s="28" t="n"/>
-      <c r="AC31" s="30" t="n">
+      <c r="AC31" s="40" t="n">
         <v>-1</v>
       </c>
       <c r="AD31" s="24" t="inlineStr">
@@ -8872,11 +8903,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ31" s="25" t="n"/>
+      <c r="BJ31" s="38" t="n"/>
       <c r="BK31" s="26" t="n">
         <v>130</v>
       </c>
-      <c r="BL31" s="27" t="n">
+      <c r="BL31" s="39" t="n">
         <v>2.3</v>
       </c>
       <c r="BM31" s="28" t="n">
@@ -8886,18 +8917,18 @@
         <v>0.432836</v>
       </c>
       <c r="BO31" s="28" t="n"/>
-      <c r="BP31" s="25" t="n"/>
-      <c r="BQ31" s="27" t="n"/>
+      <c r="BP31" s="38" t="n"/>
+      <c r="BQ31" s="39" t="n"/>
       <c r="BR31" s="28" t="n"/>
       <c r="BS31" s="28" t="n"/>
       <c r="BT31" s="28" t="n"/>
-      <c r="BU31" s="25" t="n"/>
+      <c r="BU31" s="38" t="n"/>
       <c r="BV31" s="29" t="n"/>
       <c r="BW31" s="24" t="n"/>
-      <c r="BX31" s="30" t="n">
+      <c r="BX31" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="BY31" s="27" t="n">
+      <c r="BY31" s="39" t="n">
         <v>-1</v>
       </c>
       <c r="BZ31" s="24" t="inlineStr">
@@ -8957,7 +8988,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J32" s="25" t="n"/>
+      <c r="J32" s="38" t="n"/>
       <c r="K32" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -8966,7 +8997,7 @@
       <c r="L32" s="26" t="n">
         <v>-108</v>
       </c>
-      <c r="M32" s="27" t="n">
+      <c r="M32" s="39" t="n">
         <v>1.925926</v>
       </c>
       <c r="N32" s="28" t="n">
@@ -8998,11 +9029,11 @@
       <c r="V32" s="24" t="n"/>
       <c r="W32" s="26" t="n"/>
       <c r="X32" s="26" t="n"/>
-      <c r="Y32" s="25" t="n"/>
+      <c r="Y32" s="38" t="n"/>
       <c r="Z32" s="26" t="n"/>
       <c r="AA32" s="28" t="n"/>
       <c r="AB32" s="28" t="n"/>
-      <c r="AC32" s="30" t="n"/>
+      <c r="AC32" s="40" t="n"/>
       <c r="AD32" s="24" t="n"/>
       <c r="AE32" s="31" t="inlineStr">
         <is>
@@ -9133,11 +9164,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ32" s="25" t="n"/>
+      <c r="BJ32" s="38" t="n"/>
       <c r="BK32" s="26" t="n">
         <v>-108</v>
       </c>
-      <c r="BL32" s="27" t="n">
+      <c r="BL32" s="39" t="n">
         <v>1.925926</v>
       </c>
       <c r="BM32" s="28" t="n">
@@ -9147,16 +9178,16 @@
         <v>0.517413</v>
       </c>
       <c r="BO32" s="28" t="n"/>
-      <c r="BP32" s="25" t="n"/>
-      <c r="BQ32" s="27" t="n"/>
+      <c r="BP32" s="38" t="n"/>
+      <c r="BQ32" s="39" t="n"/>
       <c r="BR32" s="28" t="n"/>
       <c r="BS32" s="28" t="n"/>
       <c r="BT32" s="28" t="n"/>
-      <c r="BU32" s="25" t="n"/>
+      <c r="BU32" s="38" t="n"/>
       <c r="BV32" s="29" t="n"/>
       <c r="BW32" s="24" t="n"/>
-      <c r="BX32" s="30" t="n"/>
-      <c r="BY32" s="27" t="n"/>
+      <c r="BX32" s="40" t="n"/>
+      <c r="BY32" s="39" t="n"/>
       <c r="BZ32" s="24" t="n"/>
       <c r="CA32" s="31" t="n"/>
     </row>
@@ -9206,7 +9237,7 @@
           <t>away</t>
         </is>
       </c>
-      <c r="J33" s="25" t="n"/>
+      <c r="J33" s="38" t="n"/>
       <c r="K33" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -9215,7 +9246,7 @@
       <c r="L33" s="26" t="n">
         <v>135</v>
       </c>
-      <c r="M33" s="27" t="n">
+      <c r="M33" s="39" t="n">
         <v>2.35</v>
       </c>
       <c r="N33" s="28" t="n">
@@ -9247,11 +9278,11 @@
       <c r="V33" s="24" t="n"/>
       <c r="W33" s="26" t="n"/>
       <c r="X33" s="26" t="n"/>
-      <c r="Y33" s="25" t="n"/>
+      <c r="Y33" s="38" t="n"/>
       <c r="Z33" s="26" t="n"/>
       <c r="AA33" s="28" t="n"/>
       <c r="AB33" s="28" t="n"/>
-      <c r="AC33" s="30" t="n"/>
+      <c r="AC33" s="40" t="n"/>
       <c r="AD33" s="24" t="n"/>
       <c r="AE33" s="31" t="inlineStr">
         <is>
@@ -9382,11 +9413,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ33" s="25" t="n"/>
+      <c r="BJ33" s="38" t="n"/>
       <c r="BK33" s="26" t="n">
         <v>135</v>
       </c>
-      <c r="BL33" s="27" t="n">
+      <c r="BL33" s="39" t="n">
         <v>2.35</v>
       </c>
       <c r="BM33" s="28" t="n">
@@ -9396,16 +9427,16 @@
         <v>0.422886</v>
       </c>
       <c r="BO33" s="28" t="n"/>
-      <c r="BP33" s="25" t="n"/>
-      <c r="BQ33" s="27" t="n"/>
+      <c r="BP33" s="38" t="n"/>
+      <c r="BQ33" s="39" t="n"/>
       <c r="BR33" s="28" t="n"/>
       <c r="BS33" s="28" t="n"/>
       <c r="BT33" s="28" t="n"/>
-      <c r="BU33" s="25" t="n"/>
+      <c r="BU33" s="38" t="n"/>
       <c r="BV33" s="29" t="n"/>
       <c r="BW33" s="24" t="n"/>
-      <c r="BX33" s="30" t="n"/>
-      <c r="BY33" s="27" t="n"/>
+      <c r="BX33" s="40" t="n"/>
+      <c r="BY33" s="39" t="n"/>
       <c r="BZ33" s="24" t="n"/>
       <c r="CA33" s="31" t="n"/>
     </row>
@@ -9455,7 +9486,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J34" s="25" t="n"/>
+      <c r="J34" s="38" t="n"/>
       <c r="K34" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -9464,7 +9495,7 @@
       <c r="L34" s="26" t="n">
         <v>-127</v>
       </c>
-      <c r="M34" s="27" t="n">
+      <c r="M34" s="39" t="n">
         <v>1.787402</v>
       </c>
       <c r="N34" s="28" t="n">
@@ -9496,11 +9527,11 @@
       <c r="V34" s="24" t="n"/>
       <c r="W34" s="26" t="n"/>
       <c r="X34" s="26" t="n"/>
-      <c r="Y34" s="25" t="n"/>
+      <c r="Y34" s="38" t="n"/>
       <c r="Z34" s="26" t="n"/>
       <c r="AA34" s="28" t="n"/>
       <c r="AB34" s="28" t="n"/>
-      <c r="AC34" s="30" t="n"/>
+      <c r="AC34" s="40" t="n"/>
       <c r="AD34" s="24" t="n"/>
       <c r="AE34" s="31" t="inlineStr">
         <is>
@@ -9631,11 +9662,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ34" s="25" t="n"/>
+      <c r="BJ34" s="38" t="n"/>
       <c r="BK34" s="26" t="n">
         <v>-127</v>
       </c>
-      <c r="BL34" s="27" t="n">
+      <c r="BL34" s="39" t="n">
         <v>1.787402</v>
       </c>
       <c r="BM34" s="28" t="n">
@@ -9645,16 +9676,16 @@
         <v>0.557214</v>
       </c>
       <c r="BO34" s="28" t="n"/>
-      <c r="BP34" s="25" t="n"/>
-      <c r="BQ34" s="27" t="n"/>
+      <c r="BP34" s="38" t="n"/>
+      <c r="BQ34" s="39" t="n"/>
       <c r="BR34" s="28" t="n"/>
       <c r="BS34" s="28" t="n"/>
       <c r="BT34" s="28" t="n"/>
-      <c r="BU34" s="25" t="n"/>
+      <c r="BU34" s="38" t="n"/>
       <c r="BV34" s="29" t="n"/>
       <c r="BW34" s="24" t="n"/>
-      <c r="BX34" s="30" t="n"/>
-      <c r="BY34" s="27" t="n"/>
+      <c r="BX34" s="40" t="n"/>
+      <c r="BY34" s="39" t="n"/>
       <c r="BZ34" s="24" t="n"/>
       <c r="CA34" s="31" t="n"/>
     </row>
@@ -9704,7 +9735,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J35" s="25" t="n"/>
+      <c r="J35" s="38" t="n"/>
       <c r="K35" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -9713,7 +9744,7 @@
       <c r="L35" s="26" t="n">
         <v>-117</v>
       </c>
-      <c r="M35" s="27" t="n">
+      <c r="M35" s="39" t="n">
         <v>1.854701</v>
       </c>
       <c r="N35" s="28" t="n">
@@ -9745,11 +9776,11 @@
       <c r="V35" s="24" t="n"/>
       <c r="W35" s="26" t="n"/>
       <c r="X35" s="26" t="n"/>
-      <c r="Y35" s="25" t="n"/>
+      <c r="Y35" s="38" t="n"/>
       <c r="Z35" s="26" t="n"/>
       <c r="AA35" s="28" t="n"/>
       <c r="AB35" s="28" t="n"/>
-      <c r="AC35" s="30" t="n"/>
+      <c r="AC35" s="40" t="n"/>
       <c r="AD35" s="24" t="n"/>
       <c r="AE35" s="31" t="inlineStr">
         <is>
@@ -9880,11 +9911,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ35" s="25" t="n"/>
+      <c r="BJ35" s="38" t="n"/>
       <c r="BK35" s="26" t="n">
         <v>-117</v>
       </c>
-      <c r="BL35" s="27" t="n">
+      <c r="BL35" s="39" t="n">
         <v>1.854701</v>
       </c>
       <c r="BM35" s="28" t="n">
@@ -9894,16 +9925,16 @@
         <v>0.537313</v>
       </c>
       <c r="BO35" s="28" t="n"/>
-      <c r="BP35" s="25" t="n"/>
-      <c r="BQ35" s="27" t="n"/>
+      <c r="BP35" s="38" t="n"/>
+      <c r="BQ35" s="39" t="n"/>
       <c r="BR35" s="28" t="n"/>
       <c r="BS35" s="28" t="n"/>
       <c r="BT35" s="28" t="n"/>
-      <c r="BU35" s="25" t="n"/>
+      <c r="BU35" s="38" t="n"/>
       <c r="BV35" s="29" t="n"/>
       <c r="BW35" s="24" t="n"/>
-      <c r="BX35" s="30" t="n"/>
-      <c r="BY35" s="27" t="n"/>
+      <c r="BX35" s="40" t="n"/>
+      <c r="BY35" s="39" t="n"/>
       <c r="BZ35" s="24" t="n"/>
       <c r="CA35" s="31" t="n"/>
     </row>
@@ -9953,7 +9984,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J36" s="25" t="n"/>
+      <c r="J36" s="38" t="n"/>
       <c r="K36" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -9962,7 +9993,7 @@
       <c r="L36" s="26" t="n">
         <v>-125</v>
       </c>
-      <c r="M36" s="27" t="n">
+      <c r="M36" s="39" t="n">
         <v>1.8</v>
       </c>
       <c r="N36" s="28" t="n">
@@ -9994,11 +10025,11 @@
       <c r="V36" s="24" t="n"/>
       <c r="W36" s="26" t="n"/>
       <c r="X36" s="26" t="n"/>
-      <c r="Y36" s="25" t="n"/>
+      <c r="Y36" s="38" t="n"/>
       <c r="Z36" s="26" t="n"/>
       <c r="AA36" s="28" t="n"/>
       <c r="AB36" s="28" t="n"/>
-      <c r="AC36" s="30" t="n"/>
+      <c r="AC36" s="40" t="n"/>
       <c r="AD36" s="24" t="n"/>
       <c r="AE36" s="31" t="inlineStr">
         <is>
@@ -10129,11 +10160,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ36" s="25" t="n"/>
+      <c r="BJ36" s="38" t="n"/>
       <c r="BK36" s="26" t="n">
         <v>-125</v>
       </c>
-      <c r="BL36" s="27" t="n">
+      <c r="BL36" s="39" t="n">
         <v>1.8</v>
       </c>
       <c r="BM36" s="28" t="n">
@@ -10143,16 +10174,16 @@
         <v>0.552239</v>
       </c>
       <c r="BO36" s="28" t="n"/>
-      <c r="BP36" s="25" t="n"/>
-      <c r="BQ36" s="27" t="n"/>
+      <c r="BP36" s="38" t="n"/>
+      <c r="BQ36" s="39" t="n"/>
       <c r="BR36" s="28" t="n"/>
       <c r="BS36" s="28" t="n"/>
       <c r="BT36" s="28" t="n"/>
-      <c r="BU36" s="25" t="n"/>
+      <c r="BU36" s="38" t="n"/>
       <c r="BV36" s="29" t="n"/>
       <c r="BW36" s="24" t="n"/>
-      <c r="BX36" s="30" t="n"/>
-      <c r="BY36" s="27" t="n"/>
+      <c r="BX36" s="40" t="n"/>
+      <c r="BY36" s="39" t="n"/>
       <c r="BZ36" s="24" t="n"/>
       <c r="CA36" s="31" t="n"/>
     </row>
@@ -10202,7 +10233,7 @@
           <t>away</t>
         </is>
       </c>
-      <c r="J37" s="25" t="n"/>
+      <c r="J37" s="38" t="n"/>
       <c r="K37" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -10211,7 +10242,7 @@
       <c r="L37" s="26" t="n">
         <v>-102</v>
       </c>
-      <c r="M37" s="27" t="n">
+      <c r="M37" s="39" t="n">
         <v>1.980392</v>
       </c>
       <c r="N37" s="28" t="n">
@@ -10243,11 +10274,11 @@
       <c r="V37" s="24" t="n"/>
       <c r="W37" s="26" t="n"/>
       <c r="X37" s="26" t="n"/>
-      <c r="Y37" s="25" t="n"/>
+      <c r="Y37" s="38" t="n"/>
       <c r="Z37" s="26" t="n"/>
       <c r="AA37" s="28" t="n"/>
       <c r="AB37" s="28" t="n"/>
-      <c r="AC37" s="30" t="n"/>
+      <c r="AC37" s="40" t="n"/>
       <c r="AD37" s="24" t="n"/>
       <c r="AE37" s="31" t="inlineStr">
         <is>
@@ -10378,11 +10409,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ37" s="25" t="n"/>
+      <c r="BJ37" s="38" t="n"/>
       <c r="BK37" s="26" t="n">
         <v>-102</v>
       </c>
-      <c r="BL37" s="27" t="n">
+      <c r="BL37" s="39" t="n">
         <v>1.980392</v>
       </c>
       <c r="BM37" s="28" t="n">
@@ -10392,16 +10423,16 @@
         <v>0.502488</v>
       </c>
       <c r="BO37" s="28" t="n"/>
-      <c r="BP37" s="25" t="n"/>
-      <c r="BQ37" s="27" t="n"/>
+      <c r="BP37" s="38" t="n"/>
+      <c r="BQ37" s="39" t="n"/>
       <c r="BR37" s="28" t="n"/>
       <c r="BS37" s="28" t="n"/>
       <c r="BT37" s="28" t="n"/>
-      <c r="BU37" s="25" t="n"/>
+      <c r="BU37" s="38" t="n"/>
       <c r="BV37" s="29" t="n"/>
       <c r="BW37" s="24" t="n"/>
-      <c r="BX37" s="30" t="n"/>
-      <c r="BY37" s="27" t="n"/>
+      <c r="BX37" s="40" t="n"/>
+      <c r="BY37" s="39" t="n"/>
       <c r="BZ37" s="24" t="n"/>
       <c r="CA37" s="31" t="n"/>
     </row>
@@ -10451,7 +10482,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J38" s="25" t="n"/>
+      <c r="J38" s="38" t="n"/>
       <c r="K38" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -10460,7 +10491,7 @@
       <c r="L38" s="26" t="n">
         <v>108</v>
       </c>
-      <c r="M38" s="27" t="n">
+      <c r="M38" s="39" t="n">
         <v>2.08</v>
       </c>
       <c r="N38" s="28" t="n">
@@ -10492,11 +10523,11 @@
       <c r="V38" s="24" t="n"/>
       <c r="W38" s="26" t="n"/>
       <c r="X38" s="26" t="n"/>
-      <c r="Y38" s="25" t="n"/>
+      <c r="Y38" s="38" t="n"/>
       <c r="Z38" s="26" t="n"/>
       <c r="AA38" s="28" t="n"/>
       <c r="AB38" s="28" t="n"/>
-      <c r="AC38" s="30" t="n"/>
+      <c r="AC38" s="40" t="n"/>
       <c r="AD38" s="24" t="n"/>
       <c r="AE38" s="31" t="inlineStr">
         <is>
@@ -10627,11 +10658,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ38" s="25" t="n"/>
+      <c r="BJ38" s="38" t="n"/>
       <c r="BK38" s="26" t="n">
         <v>108</v>
       </c>
-      <c r="BL38" s="27" t="n">
+      <c r="BL38" s="39" t="n">
         <v>2.08</v>
       </c>
       <c r="BM38" s="28" t="n">
@@ -10641,16 +10672,16 @@
         <v>0.475248</v>
       </c>
       <c r="BO38" s="28" t="n"/>
-      <c r="BP38" s="25" t="n"/>
-      <c r="BQ38" s="27" t="n"/>
+      <c r="BP38" s="38" t="n"/>
+      <c r="BQ38" s="39" t="n"/>
       <c r="BR38" s="28" t="n"/>
       <c r="BS38" s="28" t="n"/>
       <c r="BT38" s="28" t="n"/>
-      <c r="BU38" s="25" t="n"/>
+      <c r="BU38" s="38" t="n"/>
       <c r="BV38" s="29" t="n"/>
       <c r="BW38" s="24" t="n"/>
-      <c r="BX38" s="30" t="n"/>
-      <c r="BY38" s="27" t="n"/>
+      <c r="BX38" s="40" t="n"/>
+      <c r="BY38" s="39" t="n"/>
       <c r="BZ38" s="24" t="n"/>
       <c r="CA38" s="31" t="n"/>
     </row>
@@ -10700,7 +10731,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J39" s="25" t="n"/>
+      <c r="J39" s="38" t="n"/>
       <c r="K39" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -10709,7 +10740,7 @@
       <c r="L39" s="26" t="n">
         <v>-108</v>
       </c>
-      <c r="M39" s="27" t="n">
+      <c r="M39" s="39" t="n">
         <v>1.925926</v>
       </c>
       <c r="N39" s="28" t="n">
@@ -10741,11 +10772,11 @@
       <c r="V39" s="24" t="n"/>
       <c r="W39" s="26" t="n"/>
       <c r="X39" s="26" t="n"/>
-      <c r="Y39" s="25" t="n"/>
+      <c r="Y39" s="38" t="n"/>
       <c r="Z39" s="26" t="n"/>
       <c r="AA39" s="28" t="n"/>
       <c r="AB39" s="28" t="n"/>
-      <c r="AC39" s="30" t="n"/>
+      <c r="AC39" s="40" t="n"/>
       <c r="AD39" s="24" t="n"/>
       <c r="AE39" s="31" t="inlineStr">
         <is>
@@ -10876,11 +10907,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ39" s="25" t="n"/>
+      <c r="BJ39" s="38" t="n"/>
       <c r="BK39" s="26" t="n">
         <v>-108</v>
       </c>
-      <c r="BL39" s="27" t="n">
+      <c r="BL39" s="39" t="n">
         <v>1.925926</v>
       </c>
       <c r="BM39" s="28" t="n">
@@ -10890,16 +10921,16 @@
         <v>0.517413</v>
       </c>
       <c r="BO39" s="28" t="n"/>
-      <c r="BP39" s="25" t="n"/>
-      <c r="BQ39" s="27" t="n"/>
+      <c r="BP39" s="38" t="n"/>
+      <c r="BQ39" s="39" t="n"/>
       <c r="BR39" s="28" t="n"/>
       <c r="BS39" s="28" t="n"/>
       <c r="BT39" s="28" t="n"/>
-      <c r="BU39" s="25" t="n"/>
+      <c r="BU39" s="38" t="n"/>
       <c r="BV39" s="29" t="n"/>
       <c r="BW39" s="24" t="n"/>
-      <c r="BX39" s="30" t="n"/>
-      <c r="BY39" s="27" t="n"/>
+      <c r="BX39" s="40" t="n"/>
+      <c r="BY39" s="39" t="n"/>
       <c r="BZ39" s="24" t="n"/>
       <c r="CA39" s="31" t="n"/>
     </row>

</xml_diff>

<commit_message>
final: MLB v4 active, ledger updates, daily run
</commit_message>
<xml_diff>
--- a/data/picks.xlsx
+++ b/data/picks.xlsx
@@ -21,10 +21,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="0.0%"/>
-    <numFmt numFmtId="165" formatCode="0.0000"/>
-    <numFmt numFmtId="166" formatCode="0.0###"/>
-    <numFmt numFmtId="167" formatCode="0.000000"/>
+    <numFmt numFmtId="164" formatCode="0.0###"/>
+    <numFmt numFmtId="165" formatCode="0.000000"/>
+    <numFmt numFmtId="166" formatCode="0.0000"/>
+    <numFmt numFmtId="167" formatCode="0.0%"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -136,7 +136,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -150,10 +150,10 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -169,10 +169,10 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="10" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -184,10 +184,10 @@
     <xf numFmtId="0" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="10" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -202,13 +202,13 @@
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="10" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -217,38 +217,11 @@
     <xf numFmtId="2" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -781,7 +754,6 @@
         <v/>
       </c>
     </row>
-    <row r="5"/>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
@@ -813,16 +785,15 @@
         <f>COUNTIFS('Picks'!$BX$2:$BX$39,"&gt;0",'Picks'!$V$2:$V$39,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$39,"&gt;0",'Picks'!$V$2:$V$39,"loss")</f>
         <v/>
       </c>
-      <c r="E7" s="32">
+      <c r="E7" s="7">
         <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$39,"&gt;0",'Picks'!$V$2:$V$39,"win")/(COUNTIFS('Picks'!$BX$2:$BX$39,"&gt;0",'Picks'!$V$2:$V$39,"win")+COUNTIFS('Picks'!$BX$2:$BX$39,"&gt;0",'Picks'!$V$2:$V$39,"loss")),0)</f>
         <v/>
       </c>
-      <c r="G7" s="32">
+      <c r="G7" s="7">
         <f>IFERROR(SUM('Picks'!$BY$2:$BY$39)/SUM('Picks'!$BX$2:$BX$39),0)</f>
         <v/>
       </c>
     </row>
-    <row r="8"/>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
@@ -846,7 +817,7 @@
       </c>
     </row>
     <row r="10" ht="28" customHeight="1">
-      <c r="A10" s="33">
+      <c r="A10" s="8">
         <f>SUM('Picks'!$BY$2:$BY$39)</f>
         <v/>
       </c>
@@ -858,12 +829,11 @@
         <f>COUNTIFS('Picks'!$AM$2:$AM$39,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$39,"settled")</f>
         <v/>
       </c>
-      <c r="G10" s="33">
+      <c r="G10" s="8">
         <f>SUMIFS('Picks'!$AC$2:$AC$39,'Picks'!$AM$2:$AM$39,"QUALIFIED_SHADOW_CALL")</f>
         <v/>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
         <is>
@@ -926,11 +896,11 @@
         <f>COUNTIFS('Picks'!$H$2:$H$39,$A14,'Picks'!$U$2:$U$39,"settled",'Picks'!$V$2:$V$39,"loss")</f>
         <v/>
       </c>
-      <c r="E14" s="34">
+      <c r="E14" s="14">
         <f>IFERROR(C14/(C14+D14),0)</f>
         <v/>
       </c>
-      <c r="F14" s="35">
+      <c r="F14" s="15">
         <f>SUMIFS('Picks'!$BY$2:$BY$39,'Picks'!$H$2:$H$39,$A14)</f>
         <v/>
       </c>
@@ -957,11 +927,11 @@
         <f>COUNTIFS('Picks'!$H$2:$H$39,$A15,'Picks'!$U$2:$U$39,"settled",'Picks'!$V$2:$V$39,"loss")</f>
         <v/>
       </c>
-      <c r="E15" s="36">
+      <c r="E15" s="19">
         <f>IFERROR(C15/(C15+D15),0)</f>
         <v/>
       </c>
-      <c r="F15" s="37">
+      <c r="F15" s="20">
         <f>SUMIFS('Picks'!$BY$2:$BY$39,'Picks'!$H$2:$H$39,$A15)</f>
         <v/>
       </c>
@@ -988,11 +958,11 @@
         <f>COUNTIFS('Picks'!$H$2:$H$39,$A16,'Picks'!$U$2:$U$39,"settled",'Picks'!$V$2:$V$39,"loss")</f>
         <v/>
       </c>
-      <c r="E16" s="34">
+      <c r="E16" s="14">
         <f>IFERROR(C16/(C16+D16),0)</f>
         <v/>
       </c>
-      <c r="F16" s="35">
+      <c r="F16" s="15">
         <f>SUMIFS('Picks'!$BY$2:$BY$39,'Picks'!$H$2:$H$39,$A16)</f>
         <v/>
       </c>
@@ -1001,7 +971,6 @@
         <v/>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="22" t="inlineStr">
         <is>
@@ -1554,7 +1523,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J2" s="38" t="n"/>
+      <c r="J2" s="25" t="n"/>
       <c r="K2" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -1563,7 +1532,7 @@
       <c r="L2" s="26" t="n">
         <v>117</v>
       </c>
-      <c r="M2" s="39" t="n">
+      <c r="M2" s="27" t="n">
         <v>2.17</v>
       </c>
       <c r="N2" s="28" t="n">
@@ -1603,11 +1572,11 @@
       <c r="X2" s="26" t="n">
         <v>108</v>
       </c>
-      <c r="Y2" s="38" t="n"/>
+      <c r="Y2" s="25" t="n"/>
       <c r="Z2" s="26" t="n"/>
       <c r="AA2" s="28" t="n"/>
       <c r="AB2" s="28" t="n"/>
-      <c r="AC2" s="40" t="n">
+      <c r="AC2" s="30" t="n">
         <v>1.755</v>
       </c>
       <c r="AD2" s="24" t="inlineStr">
@@ -1744,11 +1713,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ2" s="38" t="n"/>
+      <c r="BJ2" s="25" t="n"/>
       <c r="BK2" s="26" t="n">
         <v>117</v>
       </c>
-      <c r="BL2" s="39" t="n">
+      <c r="BL2" s="27" t="n">
         <v>2.17</v>
       </c>
       <c r="BM2" s="28" t="n">
@@ -1758,18 +1727,18 @@
         <v>0.455446</v>
       </c>
       <c r="BO2" s="28" t="n"/>
-      <c r="BP2" s="38" t="n"/>
-      <c r="BQ2" s="39" t="n"/>
+      <c r="BP2" s="25" t="n"/>
+      <c r="BQ2" s="27" t="n"/>
       <c r="BR2" s="28" t="n"/>
       <c r="BS2" s="28" t="n"/>
       <c r="BT2" s="28" t="n"/>
-      <c r="BU2" s="38" t="n"/>
+      <c r="BU2" s="25" t="n"/>
       <c r="BV2" s="29" t="n"/>
       <c r="BW2" s="24" t="n"/>
-      <c r="BX2" s="40" t="n">
+      <c r="BX2" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY2" s="39" t="n">
+      <c r="BY2" s="27" t="n">
         <v>1.17</v>
       </c>
       <c r="BZ2" s="24" t="inlineStr">
@@ -1829,7 +1798,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J3" s="38" t="n"/>
+      <c r="J3" s="25" t="n"/>
       <c r="K3" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -1838,7 +1807,7 @@
       <c r="L3" s="26" t="n">
         <v>-133</v>
       </c>
-      <c r="M3" s="39" t="n">
+      <c r="M3" s="27" t="n">
         <v>1.75188</v>
       </c>
       <c r="N3" s="28" t="n">
@@ -1878,11 +1847,11 @@
       <c r="X3" s="26" t="n">
         <v>8</v>
       </c>
-      <c r="Y3" s="38" t="n"/>
+      <c r="Y3" s="25" t="n"/>
       <c r="Z3" s="26" t="n"/>
       <c r="AA3" s="28" t="n"/>
       <c r="AB3" s="28" t="n"/>
-      <c r="AC3" s="40" t="n">
+      <c r="AC3" s="30" t="n">
         <v>1.1278</v>
       </c>
       <c r="AD3" s="24" t="inlineStr">
@@ -2019,11 +1988,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ3" s="38" t="n"/>
+      <c r="BJ3" s="25" t="n"/>
       <c r="BK3" s="26" t="n">
         <v>-133</v>
       </c>
-      <c r="BL3" s="39" t="n">
+      <c r="BL3" s="27" t="n">
         <v>1.75188</v>
       </c>
       <c r="BM3" s="28" t="n">
@@ -2033,18 +2002,18 @@
         <v>0.567164</v>
       </c>
       <c r="BO3" s="28" t="n"/>
-      <c r="BP3" s="38" t="n"/>
-      <c r="BQ3" s="39" t="n"/>
+      <c r="BP3" s="25" t="n"/>
+      <c r="BQ3" s="27" t="n"/>
       <c r="BR3" s="28" t="n"/>
       <c r="BS3" s="28" t="n"/>
       <c r="BT3" s="28" t="n"/>
-      <c r="BU3" s="38" t="n"/>
+      <c r="BU3" s="25" t="n"/>
       <c r="BV3" s="29" t="n"/>
       <c r="BW3" s="24" t="n"/>
-      <c r="BX3" s="40" t="n">
+      <c r="BX3" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY3" s="39" t="n">
+      <c r="BY3" s="27" t="n">
         <v>0.75188</v>
       </c>
       <c r="BZ3" s="24" t="inlineStr">
@@ -2104,7 +2073,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J4" s="38" t="n"/>
+      <c r="J4" s="25" t="n"/>
       <c r="K4" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -2113,7 +2082,7 @@
       <c r="L4" s="26" t="n">
         <v>-102</v>
       </c>
-      <c r="M4" s="39" t="n">
+      <c r="M4" s="27" t="n">
         <v>1.980392</v>
       </c>
       <c r="N4" s="28" t="n">
@@ -2153,11 +2122,11 @@
       <c r="X4" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="Y4" s="38" t="n"/>
+      <c r="Y4" s="25" t="n"/>
       <c r="Z4" s="26" t="n"/>
       <c r="AA4" s="28" t="n"/>
       <c r="AB4" s="28" t="n"/>
-      <c r="AC4" s="40" t="n">
+      <c r="AC4" s="30" t="n">
         <v>-1</v>
       </c>
       <c r="AD4" s="24" t="inlineStr">
@@ -2294,11 +2263,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ4" s="38" t="n"/>
+      <c r="BJ4" s="25" t="n"/>
       <c r="BK4" s="26" t="n">
         <v>-102</v>
       </c>
-      <c r="BL4" s="39" t="n">
+      <c r="BL4" s="27" t="n">
         <v>1.980392</v>
       </c>
       <c r="BM4" s="28" t="n">
@@ -2308,18 +2277,18 @@
         <v>0.502488</v>
       </c>
       <c r="BO4" s="28" t="n"/>
-      <c r="BP4" s="38" t="n"/>
-      <c r="BQ4" s="39" t="n"/>
+      <c r="BP4" s="25" t="n"/>
+      <c r="BQ4" s="27" t="n"/>
       <c r="BR4" s="28" t="n"/>
       <c r="BS4" s="28" t="n"/>
       <c r="BT4" s="28" t="n"/>
-      <c r="BU4" s="38" t="n"/>
+      <c r="BU4" s="25" t="n"/>
       <c r="BV4" s="29" t="n"/>
       <c r="BW4" s="24" t="n"/>
-      <c r="BX4" s="40" t="n">
+      <c r="BX4" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY4" s="39" t="n">
+      <c r="BY4" s="27" t="n">
         <v>-1</v>
       </c>
       <c r="BZ4" s="24" t="inlineStr">
@@ -2379,7 +2348,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J5" s="38" t="n"/>
+      <c r="J5" s="25" t="n"/>
       <c r="K5" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -2388,7 +2357,7 @@
       <c r="L5" s="26" t="n">
         <v>-133</v>
       </c>
-      <c r="M5" s="39" t="n">
+      <c r="M5" s="27" t="n">
         <v>1.75188</v>
       </c>
       <c r="N5" s="28" t="n">
@@ -2428,11 +2397,11 @@
       <c r="X5" s="26" t="n">
         <v>6</v>
       </c>
-      <c r="Y5" s="38" t="n"/>
+      <c r="Y5" s="25" t="n"/>
       <c r="Z5" s="26" t="n"/>
       <c r="AA5" s="28" t="n"/>
       <c r="AB5" s="28" t="n"/>
-      <c r="AC5" s="40" t="n">
+      <c r="AC5" s="30" t="n">
         <v>1.1278</v>
       </c>
       <c r="AD5" s="24" t="inlineStr">
@@ -2569,11 +2538,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ5" s="38" t="n"/>
+      <c r="BJ5" s="25" t="n"/>
       <c r="BK5" s="26" t="n">
         <v>-133</v>
       </c>
-      <c r="BL5" s="39" t="n">
+      <c r="BL5" s="27" t="n">
         <v>1.75188</v>
       </c>
       <c r="BM5" s="28" t="n">
@@ -2583,18 +2552,18 @@
         <v>0.567164</v>
       </c>
       <c r="BO5" s="28" t="n"/>
-      <c r="BP5" s="38" t="n"/>
-      <c r="BQ5" s="39" t="n"/>
+      <c r="BP5" s="25" t="n"/>
+      <c r="BQ5" s="27" t="n"/>
       <c r="BR5" s="28" t="n"/>
       <c r="BS5" s="28" t="n"/>
       <c r="BT5" s="28" t="n"/>
-      <c r="BU5" s="38" t="n"/>
+      <c r="BU5" s="25" t="n"/>
       <c r="BV5" s="29" t="n"/>
       <c r="BW5" s="24" t="n"/>
-      <c r="BX5" s="40" t="n">
+      <c r="BX5" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY5" s="39" t="n">
+      <c r="BY5" s="27" t="n">
         <v>0.75188</v>
       </c>
       <c r="BZ5" s="24" t="inlineStr">
@@ -2654,7 +2623,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J6" s="38" t="n"/>
+      <c r="J6" s="25" t="n"/>
       <c r="K6" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -2663,7 +2632,7 @@
       <c r="L6" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="M6" s="39" t="n">
+      <c r="M6" s="27" t="n">
         <v>1.961538</v>
       </c>
       <c r="N6" s="28" t="n">
@@ -2703,11 +2672,11 @@
       <c r="X6" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="Y6" s="38" t="n"/>
+      <c r="Y6" s="25" t="n"/>
       <c r="Z6" s="26" t="n"/>
       <c r="AA6" s="28" t="n"/>
       <c r="AB6" s="28" t="n"/>
-      <c r="AC6" s="40" t="n">
+      <c r="AC6" s="30" t="n">
         <v>1.2019</v>
       </c>
       <c r="AD6" s="24" t="inlineStr">
@@ -2844,11 +2813,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ6" s="38" t="n"/>
+      <c r="BJ6" s="25" t="n"/>
       <c r="BK6" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="BL6" s="39" t="n">
+      <c r="BL6" s="27" t="n">
         <v>1.961538</v>
       </c>
       <c r="BM6" s="28" t="n">
@@ -2858,18 +2827,18 @@
         <v>0.507463</v>
       </c>
       <c r="BO6" s="28" t="n"/>
-      <c r="BP6" s="38" t="n"/>
-      <c r="BQ6" s="39" t="n"/>
+      <c r="BP6" s="25" t="n"/>
+      <c r="BQ6" s="27" t="n"/>
       <c r="BR6" s="28" t="n"/>
       <c r="BS6" s="28" t="n"/>
       <c r="BT6" s="28" t="n"/>
-      <c r="BU6" s="38" t="n"/>
+      <c r="BU6" s="25" t="n"/>
       <c r="BV6" s="29" t="n"/>
       <c r="BW6" s="24" t="n"/>
-      <c r="BX6" s="40" t="n">
+      <c r="BX6" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY6" s="39" t="n">
+      <c r="BY6" s="27" t="n">
         <v>0.961538</v>
       </c>
       <c r="BZ6" s="24" t="inlineStr">
@@ -2929,7 +2898,7 @@
           <t>away</t>
         </is>
       </c>
-      <c r="J7" s="38" t="n"/>
+      <c r="J7" s="25" t="n"/>
       <c r="K7" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -2938,7 +2907,7 @@
       <c r="L7" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="M7" s="39" t="n">
+      <c r="M7" s="27" t="n">
         <v>1.961538</v>
       </c>
       <c r="N7" s="28" t="n">
@@ -2978,11 +2947,11 @@
       <c r="X7" s="26" t="n">
         <v>10</v>
       </c>
-      <c r="Y7" s="38" t="n"/>
+      <c r="Y7" s="25" t="n"/>
       <c r="Z7" s="26" t="n"/>
       <c r="AA7" s="28" t="n"/>
       <c r="AB7" s="28" t="n"/>
-      <c r="AC7" s="40" t="n">
+      <c r="AC7" s="30" t="n">
         <v>-1.25</v>
       </c>
       <c r="AD7" s="24" t="inlineStr">
@@ -3119,11 +3088,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ7" s="38" t="n"/>
+      <c r="BJ7" s="25" t="n"/>
       <c r="BK7" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="BL7" s="39" t="n">
+      <c r="BL7" s="27" t="n">
         <v>1.961538</v>
       </c>
       <c r="BM7" s="28" t="n">
@@ -3133,18 +3102,18 @@
         <v>0.507463</v>
       </c>
       <c r="BO7" s="28" t="n"/>
-      <c r="BP7" s="38" t="n"/>
-      <c r="BQ7" s="39" t="n"/>
+      <c r="BP7" s="25" t="n"/>
+      <c r="BQ7" s="27" t="n"/>
       <c r="BR7" s="28" t="n"/>
       <c r="BS7" s="28" t="n"/>
       <c r="BT7" s="28" t="n"/>
-      <c r="BU7" s="38" t="n"/>
+      <c r="BU7" s="25" t="n"/>
       <c r="BV7" s="29" t="n"/>
       <c r="BW7" s="24" t="n"/>
-      <c r="BX7" s="40" t="n">
+      <c r="BX7" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY7" s="39" t="n">
+      <c r="BY7" s="27" t="n">
         <v>-1</v>
       </c>
       <c r="BZ7" s="24" t="inlineStr">
@@ -3204,7 +3173,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J8" s="38" t="n"/>
+      <c r="J8" s="25" t="n"/>
       <c r="K8" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -3213,7 +3182,7 @@
       <c r="L8" s="26" t="n">
         <v>-106</v>
       </c>
-      <c r="M8" s="39" t="n">
+      <c r="M8" s="27" t="n">
         <v>1.943396</v>
       </c>
       <c r="N8" s="28" t="n">
@@ -3253,11 +3222,11 @@
       <c r="X8" s="26" t="n">
         <v>6</v>
       </c>
-      <c r="Y8" s="38" t="n"/>
+      <c r="Y8" s="25" t="n"/>
       <c r="Z8" s="26" t="n"/>
       <c r="AA8" s="28" t="n"/>
       <c r="AB8" s="28" t="n"/>
-      <c r="AC8" s="40" t="n">
+      <c r="AC8" s="30" t="n">
         <v>-1</v>
       </c>
       <c r="AD8" s="24" t="inlineStr">
@@ -3394,11 +3363,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ8" s="38" t="n"/>
+      <c r="BJ8" s="25" t="n"/>
       <c r="BK8" s="26" t="n">
         <v>-106</v>
       </c>
-      <c r="BL8" s="39" t="n">
+      <c r="BL8" s="27" t="n">
         <v>1.943396</v>
       </c>
       <c r="BM8" s="28" t="n">
@@ -3408,18 +3377,18 @@
         <v>0.5124379999999999</v>
       </c>
       <c r="BO8" s="28" t="n"/>
-      <c r="BP8" s="38" t="n"/>
-      <c r="BQ8" s="39" t="n"/>
+      <c r="BP8" s="25" t="n"/>
+      <c r="BQ8" s="27" t="n"/>
       <c r="BR8" s="28" t="n"/>
       <c r="BS8" s="28" t="n"/>
       <c r="BT8" s="28" t="n"/>
-      <c r="BU8" s="38" t="n"/>
+      <c r="BU8" s="25" t="n"/>
       <c r="BV8" s="29" t="n"/>
       <c r="BW8" s="24" t="n"/>
-      <c r="BX8" s="40" t="n">
+      <c r="BX8" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY8" s="39" t="n">
+      <c r="BY8" s="27" t="n">
         <v>-1</v>
       </c>
       <c r="BZ8" s="24" t="inlineStr">
@@ -3479,7 +3448,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J9" s="38" t="n"/>
+      <c r="J9" s="25" t="n"/>
       <c r="K9" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -3488,7 +3457,7 @@
       <c r="L9" s="26" t="n">
         <v>-102</v>
       </c>
-      <c r="M9" s="39" t="n">
+      <c r="M9" s="27" t="n">
         <v>1.980392</v>
       </c>
       <c r="N9" s="28" t="n">
@@ -3528,11 +3497,11 @@
       <c r="X9" s="26" t="n">
         <v>5</v>
       </c>
-      <c r="Y9" s="38" t="n"/>
+      <c r="Y9" s="25" t="n"/>
       <c r="Z9" s="26" t="n"/>
       <c r="AA9" s="28" t="n"/>
       <c r="AB9" s="28" t="n"/>
-      <c r="AC9" s="40" t="n">
+      <c r="AC9" s="30" t="n">
         <v>0.9804</v>
       </c>
       <c r="AD9" s="24" t="inlineStr">
@@ -3669,11 +3638,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ9" s="38" t="n"/>
+      <c r="BJ9" s="25" t="n"/>
       <c r="BK9" s="26" t="n">
         <v>-102</v>
       </c>
-      <c r="BL9" s="39" t="n">
+      <c r="BL9" s="27" t="n">
         <v>1.980392</v>
       </c>
       <c r="BM9" s="28" t="n">
@@ -3683,18 +3652,18 @@
         <v>0.502488</v>
       </c>
       <c r="BO9" s="28" t="n"/>
-      <c r="BP9" s="38" t="n"/>
-      <c r="BQ9" s="39" t="n"/>
+      <c r="BP9" s="25" t="n"/>
+      <c r="BQ9" s="27" t="n"/>
       <c r="BR9" s="28" t="n"/>
       <c r="BS9" s="28" t="n"/>
       <c r="BT9" s="28" t="n"/>
-      <c r="BU9" s="38" t="n"/>
+      <c r="BU9" s="25" t="n"/>
       <c r="BV9" s="29" t="n"/>
       <c r="BW9" s="24" t="n"/>
-      <c r="BX9" s="40" t="n">
+      <c r="BX9" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY9" s="39" t="n">
+      <c r="BY9" s="27" t="n">
         <v>0.980392</v>
       </c>
       <c r="BZ9" s="24" t="inlineStr">
@@ -3754,7 +3723,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J10" s="38" t="n"/>
+      <c r="J10" s="25" t="n"/>
       <c r="K10" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -3763,7 +3732,7 @@
       <c r="L10" s="26" t="n">
         <v>-138</v>
       </c>
-      <c r="M10" s="39" t="n">
+      <c r="M10" s="27" t="n">
         <v>1.724638</v>
       </c>
       <c r="N10" s="28" t="n">
@@ -3803,11 +3772,11 @@
       <c r="X10" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="Y10" s="38" t="n"/>
+      <c r="Y10" s="25" t="n"/>
       <c r="Z10" s="26" t="n"/>
       <c r="AA10" s="28" t="n"/>
       <c r="AB10" s="28" t="n"/>
-      <c r="AC10" s="40" t="n">
+      <c r="AC10" s="30" t="n">
         <v>1.2681</v>
       </c>
       <c r="AD10" s="24" t="inlineStr">
@@ -3944,11 +3913,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ10" s="38" t="n"/>
+      <c r="BJ10" s="25" t="n"/>
       <c r="BK10" s="26" t="n">
         <v>-138</v>
       </c>
-      <c r="BL10" s="39" t="n">
+      <c r="BL10" s="27" t="n">
         <v>1.724638</v>
       </c>
       <c r="BM10" s="28" t="n">
@@ -3958,18 +3927,18 @@
         <v>0.577114</v>
       </c>
       <c r="BO10" s="28" t="n"/>
-      <c r="BP10" s="38" t="n"/>
-      <c r="BQ10" s="39" t="n"/>
+      <c r="BP10" s="25" t="n"/>
+      <c r="BQ10" s="27" t="n"/>
       <c r="BR10" s="28" t="n"/>
       <c r="BS10" s="28" t="n"/>
       <c r="BT10" s="28" t="n"/>
-      <c r="BU10" s="38" t="n"/>
+      <c r="BU10" s="25" t="n"/>
       <c r="BV10" s="29" t="n"/>
       <c r="BW10" s="24" t="n"/>
-      <c r="BX10" s="40" t="n">
+      <c r="BX10" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY10" s="39" t="n">
+      <c r="BY10" s="27" t="n">
         <v>0.724638</v>
       </c>
       <c r="BZ10" s="24" t="inlineStr">
@@ -4029,7 +3998,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J11" s="38" t="n"/>
+      <c r="J11" s="25" t="n"/>
       <c r="K11" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -4038,7 +4007,7 @@
       <c r="L11" s="26" t="n">
         <v>102</v>
       </c>
-      <c r="M11" s="39" t="n">
+      <c r="M11" s="27" t="n">
         <v>2.02</v>
       </c>
       <c r="N11" s="28" t="n">
@@ -4078,11 +4047,11 @@
       <c r="X11" s="26" t="n">
         <v>15</v>
       </c>
-      <c r="Y11" s="38" t="n"/>
+      <c r="Y11" s="25" t="n"/>
       <c r="Z11" s="26" t="n"/>
       <c r="AA11" s="28" t="n"/>
       <c r="AB11" s="28" t="n"/>
-      <c r="AC11" s="40" t="n">
+      <c r="AC11" s="30" t="n">
         <v>1.275</v>
       </c>
       <c r="AD11" s="24" t="inlineStr">
@@ -4219,11 +4188,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ11" s="38" t="n"/>
+      <c r="BJ11" s="25" t="n"/>
       <c r="BK11" s="26" t="n">
         <v>102</v>
       </c>
-      <c r="BL11" s="39" t="n">
+      <c r="BL11" s="27" t="n">
         <v>2.02</v>
       </c>
       <c r="BM11" s="28" t="n">
@@ -4233,18 +4202,18 @@
         <v>0.492537</v>
       </c>
       <c r="BO11" s="28" t="n"/>
-      <c r="BP11" s="38" t="n"/>
-      <c r="BQ11" s="39" t="n"/>
+      <c r="BP11" s="25" t="n"/>
+      <c r="BQ11" s="27" t="n"/>
       <c r="BR11" s="28" t="n"/>
       <c r="BS11" s="28" t="n"/>
       <c r="BT11" s="28" t="n"/>
-      <c r="BU11" s="38" t="n"/>
+      <c r="BU11" s="25" t="n"/>
       <c r="BV11" s="29" t="n"/>
       <c r="BW11" s="24" t="n"/>
-      <c r="BX11" s="40" t="n">
+      <c r="BX11" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY11" s="39" t="n">
+      <c r="BY11" s="27" t="n">
         <v>1.02</v>
       </c>
       <c r="BZ11" s="24" t="inlineStr">
@@ -4304,7 +4273,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J12" s="38" t="n"/>
+      <c r="J12" s="25" t="n"/>
       <c r="K12" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -4313,7 +4282,7 @@
       <c r="L12" s="26" t="n">
         <v>-102</v>
       </c>
-      <c r="M12" s="39" t="n">
+      <c r="M12" s="27" t="n">
         <v>1.980392</v>
       </c>
       <c r="N12" s="28" t="n">
@@ -4353,11 +4322,11 @@
       <c r="X12" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="Y12" s="38" t="n"/>
+      <c r="Y12" s="25" t="n"/>
       <c r="Z12" s="26" t="n"/>
       <c r="AA12" s="28" t="n"/>
       <c r="AB12" s="28" t="n"/>
-      <c r="AC12" s="40" t="n">
+      <c r="AC12" s="30" t="n">
         <v>-1</v>
       </c>
       <c r="AD12" s="24" t="inlineStr">
@@ -4494,11 +4463,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ12" s="38" t="n"/>
+      <c r="BJ12" s="25" t="n"/>
       <c r="BK12" s="26" t="n">
         <v>-102</v>
       </c>
-      <c r="BL12" s="39" t="n">
+      <c r="BL12" s="27" t="n">
         <v>1.980392</v>
       </c>
       <c r="BM12" s="28" t="n">
@@ -4508,18 +4477,18 @@
         <v>0.502488</v>
       </c>
       <c r="BO12" s="28" t="n"/>
-      <c r="BP12" s="38" t="n"/>
-      <c r="BQ12" s="39" t="n"/>
+      <c r="BP12" s="25" t="n"/>
+      <c r="BQ12" s="27" t="n"/>
       <c r="BR12" s="28" t="n"/>
       <c r="BS12" s="28" t="n"/>
       <c r="BT12" s="28" t="n"/>
-      <c r="BU12" s="38" t="n"/>
+      <c r="BU12" s="25" t="n"/>
       <c r="BV12" s="29" t="n"/>
       <c r="BW12" s="24" t="n"/>
-      <c r="BX12" s="40" t="n">
+      <c r="BX12" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY12" s="39" t="n">
+      <c r="BY12" s="27" t="n">
         <v>-1</v>
       </c>
       <c r="BZ12" s="24" t="inlineStr">
@@ -4579,7 +4548,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J13" s="38" t="n"/>
+      <c r="J13" s="25" t="n"/>
       <c r="K13" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -4588,7 +4557,7 @@
       <c r="L13" s="26" t="n">
         <v>-102</v>
       </c>
-      <c r="M13" s="39" t="n">
+      <c r="M13" s="27" t="n">
         <v>1.980392</v>
       </c>
       <c r="N13" s="28" t="n">
@@ -4628,11 +4597,11 @@
       <c r="X13" s="26" t="n">
         <v>7</v>
       </c>
-      <c r="Y13" s="38" t="n"/>
+      <c r="Y13" s="25" t="n"/>
       <c r="Z13" s="26" t="n"/>
       <c r="AA13" s="28" t="n"/>
       <c r="AB13" s="28" t="n"/>
-      <c r="AC13" s="40" t="n">
+      <c r="AC13" s="30" t="n">
         <v>1.2255</v>
       </c>
       <c r="AD13" s="24" t="inlineStr">
@@ -4769,11 +4738,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ13" s="38" t="n"/>
+      <c r="BJ13" s="25" t="n"/>
       <c r="BK13" s="26" t="n">
         <v>-102</v>
       </c>
-      <c r="BL13" s="39" t="n">
+      <c r="BL13" s="27" t="n">
         <v>1.980392</v>
       </c>
       <c r="BM13" s="28" t="n">
@@ -4783,18 +4752,18 @@
         <v>0.502488</v>
       </c>
       <c r="BO13" s="28" t="n"/>
-      <c r="BP13" s="38" t="n"/>
-      <c r="BQ13" s="39" t="n"/>
+      <c r="BP13" s="25" t="n"/>
+      <c r="BQ13" s="27" t="n"/>
       <c r="BR13" s="28" t="n"/>
       <c r="BS13" s="28" t="n"/>
       <c r="BT13" s="28" t="n"/>
-      <c r="BU13" s="38" t="n"/>
+      <c r="BU13" s="25" t="n"/>
       <c r="BV13" s="29" t="n"/>
       <c r="BW13" s="24" t="n"/>
-      <c r="BX13" s="40" t="n">
+      <c r="BX13" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY13" s="39" t="n">
+      <c r="BY13" s="27" t="n">
         <v>0.980392</v>
       </c>
       <c r="BZ13" s="24" t="inlineStr">
@@ -4854,7 +4823,7 @@
           <t>away</t>
         </is>
       </c>
-      <c r="J14" s="38" t="n"/>
+      <c r="J14" s="25" t="n"/>
       <c r="K14" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -4863,7 +4832,7 @@
       <c r="L14" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="M14" s="39" t="n">
+      <c r="M14" s="27" t="n">
         <v>1.961538</v>
       </c>
       <c r="N14" s="28" t="n">
@@ -4903,11 +4872,11 @@
       <c r="X14" s="26" t="n">
         <v>6</v>
       </c>
-      <c r="Y14" s="38" t="n"/>
+      <c r="Y14" s="25" t="n"/>
       <c r="Z14" s="26" t="n"/>
       <c r="AA14" s="28" t="n"/>
       <c r="AB14" s="28" t="n"/>
-      <c r="AC14" s="40" t="n">
+      <c r="AC14" s="30" t="n">
         <v>-0.75</v>
       </c>
       <c r="AD14" s="24" t="inlineStr">
@@ -5044,11 +5013,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ14" s="38" t="n"/>
+      <c r="BJ14" s="25" t="n"/>
       <c r="BK14" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="BL14" s="39" t="n">
+      <c r="BL14" s="27" t="n">
         <v>1.961538</v>
       </c>
       <c r="BM14" s="28" t="n">
@@ -5058,18 +5027,18 @@
         <v>0.507463</v>
       </c>
       <c r="BO14" s="28" t="n"/>
-      <c r="BP14" s="38" t="n"/>
-      <c r="BQ14" s="39" t="n"/>
+      <c r="BP14" s="25" t="n"/>
+      <c r="BQ14" s="27" t="n"/>
       <c r="BR14" s="28" t="n"/>
       <c r="BS14" s="28" t="n"/>
       <c r="BT14" s="28" t="n"/>
-      <c r="BU14" s="38" t="n"/>
+      <c r="BU14" s="25" t="n"/>
       <c r="BV14" s="29" t="n"/>
       <c r="BW14" s="24" t="n"/>
-      <c r="BX14" s="40" t="n">
+      <c r="BX14" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY14" s="39" t="n">
+      <c r="BY14" s="27" t="n">
         <v>-1</v>
       </c>
       <c r="BZ14" s="24" t="inlineStr">
@@ -5129,7 +5098,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J15" s="38" t="n"/>
+      <c r="J15" s="25" t="n"/>
       <c r="K15" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -5138,7 +5107,7 @@
       <c r="L15" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="M15" s="39" t="n">
+      <c r="M15" s="27" t="n">
         <v>1.961538</v>
       </c>
       <c r="N15" s="28" t="n">
@@ -5178,11 +5147,11 @@
       <c r="X15" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="Y15" s="38" t="n"/>
+      <c r="Y15" s="25" t="n"/>
       <c r="Z15" s="26" t="n"/>
       <c r="AA15" s="28" t="n"/>
       <c r="AB15" s="28" t="n"/>
-      <c r="AC15" s="40" t="n">
+      <c r="AC15" s="30" t="n">
         <v>-1</v>
       </c>
       <c r="AD15" s="24" t="inlineStr">
@@ -5319,11 +5288,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ15" s="38" t="n"/>
+      <c r="BJ15" s="25" t="n"/>
       <c r="BK15" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="BL15" s="39" t="n">
+      <c r="BL15" s="27" t="n">
         <v>1.961538</v>
       </c>
       <c r="BM15" s="28" t="n">
@@ -5333,18 +5302,18 @@
         <v>0.507463</v>
       </c>
       <c r="BO15" s="28" t="n"/>
-      <c r="BP15" s="38" t="n"/>
-      <c r="BQ15" s="39" t="n"/>
+      <c r="BP15" s="25" t="n"/>
+      <c r="BQ15" s="27" t="n"/>
       <c r="BR15" s="28" t="n"/>
       <c r="BS15" s="28" t="n"/>
       <c r="BT15" s="28" t="n"/>
-      <c r="BU15" s="38" t="n"/>
+      <c r="BU15" s="25" t="n"/>
       <c r="BV15" s="29" t="n"/>
       <c r="BW15" s="24" t="n"/>
-      <c r="BX15" s="40" t="n">
+      <c r="BX15" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY15" s="39" t="n">
+      <c r="BY15" s="27" t="n">
         <v>-1</v>
       </c>
       <c r="BZ15" s="24" t="inlineStr">
@@ -5404,7 +5373,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J16" s="38" t="n"/>
+      <c r="J16" s="25" t="n"/>
       <c r="K16" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -5413,7 +5382,7 @@
       <c r="L16" s="26" t="n">
         <v>-111</v>
       </c>
-      <c r="M16" s="39" t="n">
+      <c r="M16" s="27" t="n">
         <v>1.900901</v>
       </c>
       <c r="N16" s="28" t="n">
@@ -5453,11 +5422,11 @@
       <c r="X16" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="Y16" s="38" t="n"/>
+      <c r="Y16" s="25" t="n"/>
       <c r="Z16" s="26" t="n"/>
       <c r="AA16" s="28" t="n"/>
       <c r="AB16" s="28" t="n"/>
-      <c r="AC16" s="40" t="n">
+      <c r="AC16" s="30" t="n">
         <v>-1.5</v>
       </c>
       <c r="AD16" s="24" t="inlineStr">
@@ -5594,11 +5563,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ16" s="38" t="n"/>
+      <c r="BJ16" s="25" t="n"/>
       <c r="BK16" s="26" t="n">
         <v>-111</v>
       </c>
-      <c r="BL16" s="39" t="n">
+      <c r="BL16" s="27" t="n">
         <v>1.900901</v>
       </c>
       <c r="BM16" s="28" t="n">
@@ -5608,18 +5577,18 @@
         <v>0.522388</v>
       </c>
       <c r="BO16" s="28" t="n"/>
-      <c r="BP16" s="38" t="n"/>
-      <c r="BQ16" s="39" t="n"/>
+      <c r="BP16" s="25" t="n"/>
+      <c r="BQ16" s="27" t="n"/>
       <c r="BR16" s="28" t="n"/>
       <c r="BS16" s="28" t="n"/>
       <c r="BT16" s="28" t="n"/>
-      <c r="BU16" s="38" t="n"/>
+      <c r="BU16" s="25" t="n"/>
       <c r="BV16" s="29" t="n"/>
       <c r="BW16" s="24" t="n"/>
-      <c r="BX16" s="40" t="n">
+      <c r="BX16" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY16" s="39" t="n">
+      <c r="BY16" s="27" t="n">
         <v>-1</v>
       </c>
       <c r="BZ16" s="24" t="inlineStr">
@@ -5679,7 +5648,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J17" s="38" t="n"/>
+      <c r="J17" s="25" t="n"/>
       <c r="K17" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -5688,7 +5657,7 @@
       <c r="L17" s="26" t="n">
         <v>-108</v>
       </c>
-      <c r="M17" s="39" t="n">
+      <c r="M17" s="27" t="n">
         <v>1.925926</v>
       </c>
       <c r="N17" s="28" t="n">
@@ -5728,11 +5697,11 @@
       <c r="X17" s="26" t="n">
         <v>6</v>
       </c>
-      <c r="Y17" s="38" t="n"/>
+      <c r="Y17" s="25" t="n"/>
       <c r="Z17" s="26" t="n"/>
       <c r="AA17" s="28" t="n"/>
       <c r="AB17" s="28" t="n"/>
-      <c r="AC17" s="40" t="n">
+      <c r="AC17" s="30" t="n">
         <v>0.9258999999999999</v>
       </c>
       <c r="AD17" s="24" t="inlineStr">
@@ -5869,11 +5838,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ17" s="38" t="n"/>
+      <c r="BJ17" s="25" t="n"/>
       <c r="BK17" s="26" t="n">
         <v>-108</v>
       </c>
-      <c r="BL17" s="39" t="n">
+      <c r="BL17" s="27" t="n">
         <v>1.925926</v>
       </c>
       <c r="BM17" s="28" t="n">
@@ -5883,18 +5852,18 @@
         <v>0.5148509999999999</v>
       </c>
       <c r="BO17" s="28" t="n"/>
-      <c r="BP17" s="38" t="n"/>
-      <c r="BQ17" s="39" t="n"/>
+      <c r="BP17" s="25" t="n"/>
+      <c r="BQ17" s="27" t="n"/>
       <c r="BR17" s="28" t="n"/>
       <c r="BS17" s="28" t="n"/>
       <c r="BT17" s="28" t="n"/>
-      <c r="BU17" s="38" t="n"/>
+      <c r="BU17" s="25" t="n"/>
       <c r="BV17" s="29" t="n"/>
       <c r="BW17" s="24" t="n"/>
-      <c r="BX17" s="40" t="n">
+      <c r="BX17" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY17" s="39" t="n">
+      <c r="BY17" s="27" t="n">
         <v>0.925926</v>
       </c>
       <c r="BZ17" s="24" t="inlineStr">
@@ -5954,7 +5923,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J18" s="38" t="n"/>
+      <c r="J18" s="25" t="n"/>
       <c r="K18" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -5963,7 +5932,7 @@
       <c r="L18" s="26" t="n">
         <v>111</v>
       </c>
-      <c r="M18" s="39" t="n">
+      <c r="M18" s="27" t="n">
         <v>2.11</v>
       </c>
       <c r="N18" s="28" t="n">
@@ -6003,11 +5972,11 @@
       <c r="X18" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="Y18" s="38" t="n"/>
+      <c r="Y18" s="25" t="n"/>
       <c r="Z18" s="26" t="n"/>
       <c r="AA18" s="28" t="n"/>
       <c r="AB18" s="28" t="n"/>
-      <c r="AC18" s="40" t="n">
+      <c r="AC18" s="30" t="n">
         <v>-1.25</v>
       </c>
       <c r="AD18" s="24" t="inlineStr">
@@ -6144,11 +6113,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ18" s="38" t="n"/>
+      <c r="BJ18" s="25" t="n"/>
       <c r="BK18" s="26" t="n">
         <v>111</v>
       </c>
-      <c r="BL18" s="39" t="n">
+      <c r="BL18" s="27" t="n">
         <v>2.11</v>
       </c>
       <c r="BM18" s="28" t="n">
@@ -6158,18 +6127,18 @@
         <v>0.472637</v>
       </c>
       <c r="BO18" s="28" t="n"/>
-      <c r="BP18" s="38" t="n"/>
-      <c r="BQ18" s="39" t="n"/>
+      <c r="BP18" s="25" t="n"/>
+      <c r="BQ18" s="27" t="n"/>
       <c r="BR18" s="28" t="n"/>
       <c r="BS18" s="28" t="n"/>
       <c r="BT18" s="28" t="n"/>
-      <c r="BU18" s="38" t="n"/>
+      <c r="BU18" s="25" t="n"/>
       <c r="BV18" s="29" t="n"/>
       <c r="BW18" s="24" t="n"/>
-      <c r="BX18" s="40" t="n">
+      <c r="BX18" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY18" s="39" t="n">
+      <c r="BY18" s="27" t="n">
         <v>-1</v>
       </c>
       <c r="BZ18" s="24" t="inlineStr">
@@ -6229,7 +6198,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J19" s="38" t="n"/>
+      <c r="J19" s="25" t="n"/>
       <c r="K19" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -6238,7 +6207,7 @@
       <c r="L19" s="26" t="n">
         <v>-125</v>
       </c>
-      <c r="M19" s="39" t="n">
+      <c r="M19" s="27" t="n">
         <v>1.8</v>
       </c>
       <c r="N19" s="28" t="n">
@@ -6278,11 +6247,11 @@
       <c r="X19" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="Y19" s="38" t="n"/>
+      <c r="Y19" s="25" t="n"/>
       <c r="Z19" s="26" t="n"/>
       <c r="AA19" s="28" t="n"/>
       <c r="AB19" s="28" t="n"/>
-      <c r="AC19" s="40" t="n">
+      <c r="AC19" s="30" t="n">
         <v>1.2</v>
       </c>
       <c r="AD19" s="24" t="inlineStr">
@@ -6419,11 +6388,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ19" s="38" t="n"/>
+      <c r="BJ19" s="25" t="n"/>
       <c r="BK19" s="26" t="n">
         <v>-125</v>
       </c>
-      <c r="BL19" s="39" t="n">
+      <c r="BL19" s="27" t="n">
         <v>1.8</v>
       </c>
       <c r="BM19" s="28" t="n">
@@ -6433,18 +6402,18 @@
         <v>0.552239</v>
       </c>
       <c r="BO19" s="28" t="n"/>
-      <c r="BP19" s="38" t="n"/>
-      <c r="BQ19" s="39" t="n"/>
+      <c r="BP19" s="25" t="n"/>
+      <c r="BQ19" s="27" t="n"/>
       <c r="BR19" s="28" t="n"/>
       <c r="BS19" s="28" t="n"/>
       <c r="BT19" s="28" t="n"/>
-      <c r="BU19" s="38" t="n"/>
+      <c r="BU19" s="25" t="n"/>
       <c r="BV19" s="29" t="n"/>
       <c r="BW19" s="24" t="n"/>
-      <c r="BX19" s="40" t="n">
+      <c r="BX19" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY19" s="39" t="n">
+      <c r="BY19" s="27" t="n">
         <v>0.8</v>
       </c>
       <c r="BZ19" s="24" t="inlineStr">
@@ -6504,7 +6473,7 @@
           <t>away</t>
         </is>
       </c>
-      <c r="J20" s="38" t="n"/>
+      <c r="J20" s="25" t="n"/>
       <c r="K20" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -6513,7 +6482,7 @@
       <c r="L20" s="26" t="n">
         <v>106</v>
       </c>
-      <c r="M20" s="39" t="n">
+      <c r="M20" s="27" t="n">
         <v>2.06</v>
       </c>
       <c r="N20" s="28" t="n">
@@ -6553,11 +6522,11 @@
       <c r="X20" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="Y20" s="38" t="n"/>
+      <c r="Y20" s="25" t="n"/>
       <c r="Z20" s="26" t="n"/>
       <c r="AA20" s="28" t="n"/>
       <c r="AB20" s="28" t="n"/>
-      <c r="AC20" s="40" t="n">
+      <c r="AC20" s="30" t="n">
         <v>0.795</v>
       </c>
       <c r="AD20" s="24" t="inlineStr">
@@ -6694,11 +6663,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ20" s="38" t="n"/>
+      <c r="BJ20" s="25" t="n"/>
       <c r="BK20" s="26" t="n">
         <v>106</v>
       </c>
-      <c r="BL20" s="39" t="n">
+      <c r="BL20" s="27" t="n">
         <v>2.06</v>
       </c>
       <c r="BM20" s="28" t="n">
@@ -6708,18 +6677,18 @@
         <v>0.482587</v>
       </c>
       <c r="BO20" s="28" t="n"/>
-      <c r="BP20" s="38" t="n"/>
-      <c r="BQ20" s="39" t="n"/>
+      <c r="BP20" s="25" t="n"/>
+      <c r="BQ20" s="27" t="n"/>
       <c r="BR20" s="28" t="n"/>
       <c r="BS20" s="28" t="n"/>
       <c r="BT20" s="28" t="n"/>
-      <c r="BU20" s="38" t="n"/>
+      <c r="BU20" s="25" t="n"/>
       <c r="BV20" s="29" t="n"/>
       <c r="BW20" s="24" t="n"/>
-      <c r="BX20" s="40" t="n">
+      <c r="BX20" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY20" s="39" t="n">
+      <c r="BY20" s="27" t="n">
         <v>1.06</v>
       </c>
       <c r="BZ20" s="24" t="inlineStr">
@@ -6779,7 +6748,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J21" s="38" t="n"/>
+      <c r="J21" s="25" t="n"/>
       <c r="K21" s="24" t="inlineStr">
         <is>
           <t>polymarket</t>
@@ -6788,7 +6757,7 @@
       <c r="L21" s="26" t="n">
         <v>-106</v>
       </c>
-      <c r="M21" s="39" t="n">
+      <c r="M21" s="27" t="n">
         <v>1.943396</v>
       </c>
       <c r="N21" s="28" t="n">
@@ -6828,11 +6797,11 @@
       <c r="X21" s="26" t="n">
         <v>10</v>
       </c>
-      <c r="Y21" s="38" t="n"/>
+      <c r="Y21" s="25" t="n"/>
       <c r="Z21" s="26" t="n"/>
       <c r="AA21" s="28" t="n"/>
       <c r="AB21" s="28" t="n"/>
-      <c r="AC21" s="40" t="n">
+      <c r="AC21" s="30" t="n">
         <v>0.9434</v>
       </c>
       <c r="AD21" s="24" t="inlineStr">
@@ -6879,11 +6848,11 @@
         </is>
       </c>
       <c r="BI21" s="24" t="n"/>
-      <c r="BJ21" s="38" t="n"/>
+      <c r="BJ21" s="25" t="n"/>
       <c r="BK21" s="26" t="n">
         <v>-106</v>
       </c>
-      <c r="BL21" s="39" t="n">
+      <c r="BL21" s="27" t="n">
         <v>1.943396</v>
       </c>
       <c r="BM21" s="28" t="n">
@@ -6893,16 +6862,16 @@
         <v>0.5124379999999999</v>
       </c>
       <c r="BO21" s="28" t="n"/>
-      <c r="BP21" s="38" t="n"/>
-      <c r="BQ21" s="39" t="n"/>
+      <c r="BP21" s="25" t="n"/>
+      <c r="BQ21" s="27" t="n"/>
       <c r="BR21" s="28" t="n"/>
       <c r="BS21" s="28" t="n"/>
       <c r="BT21" s="28" t="n"/>
-      <c r="BU21" s="38" t="n"/>
+      <c r="BU21" s="25" t="n"/>
       <c r="BV21" s="29" t="n"/>
       <c r="BW21" s="24" t="n"/>
-      <c r="BX21" s="40" t="n"/>
-      <c r="BY21" s="39" t="n"/>
+      <c r="BX21" s="30" t="n"/>
+      <c r="BY21" s="27" t="n"/>
       <c r="BZ21" s="24" t="n"/>
       <c r="CA21" s="31" t="n"/>
     </row>
@@ -6952,7 +6921,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J22" s="38" t="n"/>
+      <c r="J22" s="25" t="n"/>
       <c r="K22" s="24" t="inlineStr">
         <is>
           <t>polymarket</t>
@@ -6961,7 +6930,7 @@
       <c r="L22" s="26" t="n">
         <v>-106</v>
       </c>
-      <c r="M22" s="39" t="n">
+      <c r="M22" s="27" t="n">
         <v>1.943396</v>
       </c>
       <c r="N22" s="28" t="n">
@@ -7001,11 +6970,11 @@
       <c r="X22" s="26" t="n">
         <v>5</v>
       </c>
-      <c r="Y22" s="38" t="n"/>
+      <c r="Y22" s="25" t="n"/>
       <c r="Z22" s="26" t="n"/>
       <c r="AA22" s="28" t="n"/>
       <c r="AB22" s="28" t="n"/>
-      <c r="AC22" s="40" t="n">
+      <c r="AC22" s="30" t="n">
         <v>0.9434</v>
       </c>
       <c r="AD22" s="24" t="inlineStr">
@@ -7052,11 +7021,11 @@
         </is>
       </c>
       <c r="BI22" s="24" t="n"/>
-      <c r="BJ22" s="38" t="n"/>
+      <c r="BJ22" s="25" t="n"/>
       <c r="BK22" s="26" t="n">
         <v>-106</v>
       </c>
-      <c r="BL22" s="39" t="n">
+      <c r="BL22" s="27" t="n">
         <v>1.943396</v>
       </c>
       <c r="BM22" s="28" t="n">
@@ -7066,16 +7035,16 @@
         <v>0.5124379999999999</v>
       </c>
       <c r="BO22" s="28" t="n"/>
-      <c r="BP22" s="38" t="n"/>
-      <c r="BQ22" s="39" t="n"/>
+      <c r="BP22" s="25" t="n"/>
+      <c r="BQ22" s="27" t="n"/>
       <c r="BR22" s="28" t="n"/>
       <c r="BS22" s="28" t="n"/>
       <c r="BT22" s="28" t="n"/>
-      <c r="BU22" s="38" t="n"/>
+      <c r="BU22" s="25" t="n"/>
       <c r="BV22" s="29" t="n"/>
       <c r="BW22" s="24" t="n"/>
-      <c r="BX22" s="40" t="n"/>
-      <c r="BY22" s="39" t="n"/>
+      <c r="BX22" s="30" t="n"/>
+      <c r="BY22" s="27" t="n"/>
       <c r="BZ22" s="24" t="n"/>
       <c r="CA22" s="31" t="n"/>
     </row>
@@ -7125,7 +7094,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J23" s="38" t="n"/>
+      <c r="J23" s="25" t="n"/>
       <c r="K23" s="24" t="inlineStr">
         <is>
           <t>polymarket</t>
@@ -7134,7 +7103,7 @@
       <c r="L23" s="26" t="n">
         <v>-141</v>
       </c>
-      <c r="M23" s="39" t="n">
+      <c r="M23" s="27" t="n">
         <v>1.70922</v>
       </c>
       <c r="N23" s="28" t="n">
@@ -7174,11 +7143,11 @@
       <c r="X23" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="Y23" s="38" t="n"/>
+      <c r="Y23" s="25" t="n"/>
       <c r="Z23" s="26" t="n"/>
       <c r="AA23" s="28" t="n"/>
       <c r="AB23" s="28" t="n"/>
-      <c r="AC23" s="40" t="n">
+      <c r="AC23" s="30" t="n">
         <v>1.2411</v>
       </c>
       <c r="AD23" s="24" t="inlineStr">
@@ -7225,11 +7194,11 @@
         </is>
       </c>
       <c r="BI23" s="24" t="n"/>
-      <c r="BJ23" s="38" t="n"/>
+      <c r="BJ23" s="25" t="n"/>
       <c r="BK23" s="26" t="n">
         <v>-141</v>
       </c>
-      <c r="BL23" s="39" t="n">
+      <c r="BL23" s="27" t="n">
         <v>1.70922</v>
       </c>
       <c r="BM23" s="28" t="n">
@@ -7239,16 +7208,16 @@
         <v>0.58209</v>
       </c>
       <c r="BO23" s="28" t="n"/>
-      <c r="BP23" s="38" t="n"/>
-      <c r="BQ23" s="39" t="n"/>
+      <c r="BP23" s="25" t="n"/>
+      <c r="BQ23" s="27" t="n"/>
       <c r="BR23" s="28" t="n"/>
       <c r="BS23" s="28" t="n"/>
       <c r="BT23" s="28" t="n"/>
-      <c r="BU23" s="38" t="n"/>
+      <c r="BU23" s="25" t="n"/>
       <c r="BV23" s="29" t="n"/>
       <c r="BW23" s="24" t="n"/>
-      <c r="BX23" s="40" t="n"/>
-      <c r="BY23" s="39" t="n"/>
+      <c r="BX23" s="30" t="n"/>
+      <c r="BY23" s="27" t="n"/>
       <c r="BZ23" s="24" t="n"/>
       <c r="CA23" s="31" t="n"/>
     </row>
@@ -7298,7 +7267,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J24" s="38" t="n"/>
+      <c r="J24" s="25" t="n"/>
       <c r="K24" s="24" t="inlineStr">
         <is>
           <t>polymarket</t>
@@ -7307,7 +7276,7 @@
       <c r="L24" s="26" t="n">
         <v>-133</v>
       </c>
-      <c r="M24" s="39" t="n">
+      <c r="M24" s="27" t="n">
         <v>1.75188</v>
       </c>
       <c r="N24" s="28" t="n">
@@ -7347,11 +7316,11 @@
       <c r="X24" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="Y24" s="38" t="n"/>
+      <c r="Y24" s="25" t="n"/>
       <c r="Z24" s="26" t="n"/>
       <c r="AA24" s="28" t="n"/>
       <c r="AB24" s="28" t="n"/>
-      <c r="AC24" s="40" t="n">
+      <c r="AC24" s="30" t="n">
         <v>-1.5</v>
       </c>
       <c r="AD24" s="24" t="inlineStr">
@@ -7398,11 +7367,11 @@
         </is>
       </c>
       <c r="BI24" s="24" t="n"/>
-      <c r="BJ24" s="38" t="n"/>
+      <c r="BJ24" s="25" t="n"/>
       <c r="BK24" s="26" t="n">
         <v>-133</v>
       </c>
-      <c r="BL24" s="39" t="n">
+      <c r="BL24" s="27" t="n">
         <v>1.75188</v>
       </c>
       <c r="BM24" s="28" t="n">
@@ -7412,16 +7381,16 @@
         <v>0.567164</v>
       </c>
       <c r="BO24" s="28" t="n"/>
-      <c r="BP24" s="38" t="n"/>
-      <c r="BQ24" s="39" t="n"/>
+      <c r="BP24" s="25" t="n"/>
+      <c r="BQ24" s="27" t="n"/>
       <c r="BR24" s="28" t="n"/>
       <c r="BS24" s="28" t="n"/>
       <c r="BT24" s="28" t="n"/>
-      <c r="BU24" s="38" t="n"/>
+      <c r="BU24" s="25" t="n"/>
       <c r="BV24" s="29" t="n"/>
       <c r="BW24" s="24" t="n"/>
-      <c r="BX24" s="40" t="n"/>
-      <c r="BY24" s="39" t="n"/>
+      <c r="BX24" s="30" t="n"/>
+      <c r="BY24" s="27" t="n"/>
       <c r="BZ24" s="24" t="n"/>
       <c r="CA24" s="31" t="n"/>
     </row>
@@ -7471,7 +7440,7 @@
           <t>away</t>
         </is>
       </c>
-      <c r="J25" s="38" t="n"/>
+      <c r="J25" s="25" t="n"/>
       <c r="K25" s="24" t="inlineStr">
         <is>
           <t>polymarket</t>
@@ -7480,7 +7449,7 @@
       <c r="L25" s="26" t="n">
         <v>104</v>
       </c>
-      <c r="M25" s="39" t="n">
+      <c r="M25" s="27" t="n">
         <v>2.04</v>
       </c>
       <c r="N25" s="28" t="n">
@@ -7520,11 +7489,11 @@
       <c r="X25" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="Y25" s="38" t="n"/>
+      <c r="Y25" s="25" t="n"/>
       <c r="Z25" s="26" t="n"/>
       <c r="AA25" s="28" t="n"/>
       <c r="AB25" s="28" t="n"/>
-      <c r="AC25" s="40" t="n">
+      <c r="AC25" s="30" t="n">
         <v>1.3</v>
       </c>
       <c r="AD25" s="24" t="inlineStr">
@@ -7571,11 +7540,11 @@
         </is>
       </c>
       <c r="BI25" s="24" t="n"/>
-      <c r="BJ25" s="38" t="n"/>
+      <c r="BJ25" s="25" t="n"/>
       <c r="BK25" s="26" t="n">
         <v>104</v>
       </c>
-      <c r="BL25" s="39" t="n">
+      <c r="BL25" s="27" t="n">
         <v>2.04</v>
       </c>
       <c r="BM25" s="28" t="n">
@@ -7585,16 +7554,16 @@
         <v>0.487562</v>
       </c>
       <c r="BO25" s="28" t="n"/>
-      <c r="BP25" s="38" t="n"/>
-      <c r="BQ25" s="39" t="n"/>
+      <c r="BP25" s="25" t="n"/>
+      <c r="BQ25" s="27" t="n"/>
       <c r="BR25" s="28" t="n"/>
       <c r="BS25" s="28" t="n"/>
       <c r="BT25" s="28" t="n"/>
-      <c r="BU25" s="38" t="n"/>
+      <c r="BU25" s="25" t="n"/>
       <c r="BV25" s="29" t="n"/>
       <c r="BW25" s="24" t="n"/>
-      <c r="BX25" s="40" t="n"/>
-      <c r="BY25" s="39" t="n"/>
+      <c r="BX25" s="30" t="n"/>
+      <c r="BY25" s="27" t="n"/>
       <c r="BZ25" s="24" t="n"/>
       <c r="CA25" s="31" t="n"/>
     </row>
@@ -7644,7 +7613,7 @@
           <t>away</t>
         </is>
       </c>
-      <c r="J26" s="38" t="n"/>
+      <c r="J26" s="25" t="n"/>
       <c r="K26" s="24" t="inlineStr">
         <is>
           <t>polymarket</t>
@@ -7653,7 +7622,7 @@
       <c r="L26" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="M26" s="39" t="n">
+      <c r="M26" s="27" t="n">
         <v>1.961538</v>
       </c>
       <c r="N26" s="28" t="n">
@@ -7693,11 +7662,11 @@
       <c r="X26" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="Y26" s="38" t="n"/>
+      <c r="Y26" s="25" t="n"/>
       <c r="Z26" s="26" t="n"/>
       <c r="AA26" s="28" t="n"/>
       <c r="AB26" s="28" t="n"/>
-      <c r="AC26" s="40" t="n">
+      <c r="AC26" s="30" t="n">
         <v>0.9615</v>
       </c>
       <c r="AD26" s="24" t="inlineStr">
@@ -7744,11 +7713,11 @@
         </is>
       </c>
       <c r="BI26" s="24" t="n"/>
-      <c r="BJ26" s="38" t="n"/>
+      <c r="BJ26" s="25" t="n"/>
       <c r="BK26" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="BL26" s="39" t="n">
+      <c r="BL26" s="27" t="n">
         <v>1.961538</v>
       </c>
       <c r="BM26" s="28" t="n">
@@ -7758,16 +7727,16 @@
         <v>0.507463</v>
       </c>
       <c r="BO26" s="28" t="n"/>
-      <c r="BP26" s="38" t="n"/>
-      <c r="BQ26" s="39" t="n"/>
+      <c r="BP26" s="25" t="n"/>
+      <c r="BQ26" s="27" t="n"/>
       <c r="BR26" s="28" t="n"/>
       <c r="BS26" s="28" t="n"/>
       <c r="BT26" s="28" t="n"/>
-      <c r="BU26" s="38" t="n"/>
+      <c r="BU26" s="25" t="n"/>
       <c r="BV26" s="29" t="n"/>
       <c r="BW26" s="24" t="n"/>
-      <c r="BX26" s="40" t="n"/>
-      <c r="BY26" s="39" t="n"/>
+      <c r="BX26" s="30" t="n"/>
+      <c r="BY26" s="27" t="n"/>
       <c r="BZ26" s="24" t="n"/>
       <c r="CA26" s="31" t="n"/>
     </row>
@@ -7817,7 +7786,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J27" s="38" t="n"/>
+      <c r="J27" s="25" t="n"/>
       <c r="K27" s="24" t="inlineStr">
         <is>
           <t>polymarket</t>
@@ -7826,7 +7795,7 @@
       <c r="L27" s="26" t="n">
         <v>120</v>
       </c>
-      <c r="M27" s="39" t="n">
+      <c r="M27" s="27" t="n">
         <v>2.2</v>
       </c>
       <c r="N27" s="28" t="n">
@@ -7866,11 +7835,11 @@
       <c r="X27" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="Y27" s="38" t="n"/>
+      <c r="Y27" s="25" t="n"/>
       <c r="Z27" s="26" t="n"/>
       <c r="AA27" s="28" t="n"/>
       <c r="AB27" s="28" t="n"/>
-      <c r="AC27" s="40" t="n">
+      <c r="AC27" s="30" t="n">
         <v>-0.75</v>
       </c>
       <c r="AD27" s="24" t="inlineStr">
@@ -7917,11 +7886,11 @@
         </is>
       </c>
       <c r="BI27" s="24" t="n"/>
-      <c r="BJ27" s="38" t="n"/>
+      <c r="BJ27" s="25" t="n"/>
       <c r="BK27" s="26" t="n">
         <v>120</v>
       </c>
-      <c r="BL27" s="39" t="n">
+      <c r="BL27" s="27" t="n">
         <v>2.2</v>
       </c>
       <c r="BM27" s="28" t="n">
@@ -7931,16 +7900,16 @@
         <v>0.452736</v>
       </c>
       <c r="BO27" s="28" t="n"/>
-      <c r="BP27" s="38" t="n"/>
-      <c r="BQ27" s="39" t="n"/>
+      <c r="BP27" s="25" t="n"/>
+      <c r="BQ27" s="27" t="n"/>
       <c r="BR27" s="28" t="n"/>
       <c r="BS27" s="28" t="n"/>
       <c r="BT27" s="28" t="n"/>
-      <c r="BU27" s="38" t="n"/>
+      <c r="BU27" s="25" t="n"/>
       <c r="BV27" s="29" t="n"/>
       <c r="BW27" s="24" t="n"/>
-      <c r="BX27" s="40" t="n"/>
-      <c r="BY27" s="39" t="n"/>
+      <c r="BX27" s="30" t="n"/>
+      <c r="BY27" s="27" t="n"/>
       <c r="BZ27" s="24" t="n"/>
       <c r="CA27" s="31" t="n"/>
     </row>
@@ -7990,7 +7959,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J28" s="38" t="n"/>
+      <c r="J28" s="25" t="n"/>
       <c r="K28" s="24" t="inlineStr">
         <is>
           <t>polymarket</t>
@@ -7999,7 +7968,7 @@
       <c r="L28" s="26" t="n">
         <v>100</v>
       </c>
-      <c r="M28" s="39" t="n">
+      <c r="M28" s="27" t="n">
         <v>2</v>
       </c>
       <c r="N28" s="28" t="n">
@@ -8039,11 +8008,11 @@
       <c r="X28" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="Y28" s="38" t="n"/>
+      <c r="Y28" s="25" t="n"/>
       <c r="Z28" s="26" t="n"/>
       <c r="AA28" s="28" t="n"/>
       <c r="AB28" s="28" t="n"/>
-      <c r="AC28" s="40" t="n">
+      <c r="AC28" s="30" t="n">
         <v>-0.75</v>
       </c>
       <c r="AD28" s="24" t="inlineStr">
@@ -8090,11 +8059,11 @@
         </is>
       </c>
       <c r="BI28" s="24" t="n"/>
-      <c r="BJ28" s="38" t="n"/>
+      <c r="BJ28" s="25" t="n"/>
       <c r="BK28" s="26" t="n">
         <v>100</v>
       </c>
-      <c r="BL28" s="39" t="n">
+      <c r="BL28" s="27" t="n">
         <v>2</v>
       </c>
       <c r="BM28" s="28" t="n">
@@ -8104,16 +8073,16 @@
         <v>0.497512</v>
       </c>
       <c r="BO28" s="28" t="n"/>
-      <c r="BP28" s="38" t="n"/>
-      <c r="BQ28" s="39" t="n"/>
+      <c r="BP28" s="25" t="n"/>
+      <c r="BQ28" s="27" t="n"/>
       <c r="BR28" s="28" t="n"/>
       <c r="BS28" s="28" t="n"/>
       <c r="BT28" s="28" t="n"/>
-      <c r="BU28" s="38" t="n"/>
+      <c r="BU28" s="25" t="n"/>
       <c r="BV28" s="29" t="n"/>
       <c r="BW28" s="24" t="n"/>
-      <c r="BX28" s="40" t="n"/>
-      <c r="BY28" s="39" t="n"/>
+      <c r="BX28" s="30" t="n"/>
+      <c r="BY28" s="27" t="n"/>
       <c r="BZ28" s="24" t="n"/>
       <c r="CA28" s="31" t="n"/>
     </row>
@@ -8163,7 +8132,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J29" s="38" t="n"/>
+      <c r="J29" s="25" t="n"/>
       <c r="K29" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -8172,7 +8141,7 @@
       <c r="L29" s="26" t="n">
         <v>108</v>
       </c>
-      <c r="M29" s="39" t="n">
+      <c r="M29" s="27" t="n">
         <v>2.08</v>
       </c>
       <c r="N29" s="28" t="n">
@@ -8212,11 +8181,11 @@
       <c r="X29" s="26" t="n">
         <v>8</v>
       </c>
-      <c r="Y29" s="38" t="n"/>
+      <c r="Y29" s="25" t="n"/>
       <c r="Z29" s="26" t="n"/>
       <c r="AA29" s="28" t="n"/>
       <c r="AB29" s="28" t="n"/>
-      <c r="AC29" s="40" t="n">
+      <c r="AC29" s="30" t="n">
         <v>1.35</v>
       </c>
       <c r="AD29" s="24" t="inlineStr">
@@ -8353,11 +8322,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ29" s="38" t="n"/>
+      <c r="BJ29" s="25" t="n"/>
       <c r="BK29" s="26" t="n">
         <v>108</v>
       </c>
-      <c r="BL29" s="39" t="n">
+      <c r="BL29" s="27" t="n">
         <v>2.08</v>
       </c>
       <c r="BM29" s="28" t="n">
@@ -8367,18 +8336,18 @@
         <v>0.477612</v>
       </c>
       <c r="BO29" s="28" t="n"/>
-      <c r="BP29" s="38" t="n"/>
-      <c r="BQ29" s="39" t="n"/>
+      <c r="BP29" s="25" t="n"/>
+      <c r="BQ29" s="27" t="n"/>
       <c r="BR29" s="28" t="n"/>
       <c r="BS29" s="28" t="n"/>
       <c r="BT29" s="28" t="n"/>
-      <c r="BU29" s="38" t="n"/>
+      <c r="BU29" s="25" t="n"/>
       <c r="BV29" s="29" t="n"/>
       <c r="BW29" s="24" t="n"/>
-      <c r="BX29" s="40" t="n">
+      <c r="BX29" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY29" s="39" t="n">
+      <c r="BY29" s="27" t="n">
         <v>1.08</v>
       </c>
       <c r="BZ29" s="24" t="inlineStr">
@@ -8438,7 +8407,7 @@
           <t>away</t>
         </is>
       </c>
-      <c r="J30" s="38" t="n"/>
+      <c r="J30" s="25" t="n"/>
       <c r="K30" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -8447,7 +8416,7 @@
       <c r="L30" s="26" t="n">
         <v>-133</v>
       </c>
-      <c r="M30" s="39" t="n">
+      <c r="M30" s="27" t="n">
         <v>1.75188</v>
       </c>
       <c r="N30" s="28" t="n">
@@ -8487,11 +8456,11 @@
       <c r="X30" s="26" t="n">
         <v>6</v>
       </c>
-      <c r="Y30" s="38" t="n"/>
+      <c r="Y30" s="25" t="n"/>
       <c r="Z30" s="26" t="n"/>
       <c r="AA30" s="28" t="n"/>
       <c r="AB30" s="28" t="n"/>
-      <c r="AC30" s="40" t="n">
+      <c r="AC30" s="30" t="n">
         <v>1.1278</v>
       </c>
       <c r="AD30" s="24" t="inlineStr">
@@ -8628,11 +8597,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ30" s="38" t="n"/>
+      <c r="BJ30" s="25" t="n"/>
       <c r="BK30" s="26" t="n">
         <v>-133</v>
       </c>
-      <c r="BL30" s="39" t="n">
+      <c r="BL30" s="27" t="n">
         <v>1.75188</v>
       </c>
       <c r="BM30" s="28" t="n">
@@ -8642,18 +8611,18 @@
         <v>0.567164</v>
       </c>
       <c r="BO30" s="28" t="n"/>
-      <c r="BP30" s="38" t="n"/>
-      <c r="BQ30" s="39" t="n"/>
+      <c r="BP30" s="25" t="n"/>
+      <c r="BQ30" s="27" t="n"/>
       <c r="BR30" s="28" t="n"/>
       <c r="BS30" s="28" t="n"/>
       <c r="BT30" s="28" t="n"/>
-      <c r="BU30" s="38" t="n"/>
+      <c r="BU30" s="25" t="n"/>
       <c r="BV30" s="29" t="n"/>
       <c r="BW30" s="24" t="n"/>
-      <c r="BX30" s="40" t="n">
+      <c r="BX30" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY30" s="39" t="n">
+      <c r="BY30" s="27" t="n">
         <v>0.75188</v>
       </c>
       <c r="BZ30" s="24" t="inlineStr">
@@ -8713,7 +8682,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J31" s="38" t="n"/>
+      <c r="J31" s="25" t="n"/>
       <c r="K31" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -8722,7 +8691,7 @@
       <c r="L31" s="26" t="n">
         <v>130</v>
       </c>
-      <c r="M31" s="39" t="n">
+      <c r="M31" s="27" t="n">
         <v>2.3</v>
       </c>
       <c r="N31" s="28" t="n">
@@ -8762,11 +8731,11 @@
       <c r="X31" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="Y31" s="38" t="n"/>
+      <c r="Y31" s="25" t="n"/>
       <c r="Z31" s="26" t="n"/>
       <c r="AA31" s="28" t="n"/>
       <c r="AB31" s="28" t="n"/>
-      <c r="AC31" s="40" t="n">
+      <c r="AC31" s="30" t="n">
         <v>-1</v>
       </c>
       <c r="AD31" s="24" t="inlineStr">
@@ -8903,11 +8872,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ31" s="38" t="n"/>
+      <c r="BJ31" s="25" t="n"/>
       <c r="BK31" s="26" t="n">
         <v>130</v>
       </c>
-      <c r="BL31" s="39" t="n">
+      <c r="BL31" s="27" t="n">
         <v>2.3</v>
       </c>
       <c r="BM31" s="28" t="n">
@@ -8917,18 +8886,18 @@
         <v>0.432836</v>
       </c>
       <c r="BO31" s="28" t="n"/>
-      <c r="BP31" s="38" t="n"/>
-      <c r="BQ31" s="39" t="n"/>
+      <c r="BP31" s="25" t="n"/>
+      <c r="BQ31" s="27" t="n"/>
       <c r="BR31" s="28" t="n"/>
       <c r="BS31" s="28" t="n"/>
       <c r="BT31" s="28" t="n"/>
-      <c r="BU31" s="38" t="n"/>
+      <c r="BU31" s="25" t="n"/>
       <c r="BV31" s="29" t="n"/>
       <c r="BW31" s="24" t="n"/>
-      <c r="BX31" s="40" t="n">
+      <c r="BX31" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY31" s="39" t="n">
+      <c r="BY31" s="27" t="n">
         <v>-1</v>
       </c>
       <c r="BZ31" s="24" t="inlineStr">
@@ -8988,7 +8957,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J32" s="38" t="n"/>
+      <c r="J32" s="25" t="n"/>
       <c r="K32" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -8997,7 +8966,7 @@
       <c r="L32" s="26" t="n">
         <v>-108</v>
       </c>
-      <c r="M32" s="39" t="n">
+      <c r="M32" s="27" t="n">
         <v>1.925926</v>
       </c>
       <c r="N32" s="28" t="n">
@@ -9029,11 +8998,11 @@
       <c r="V32" s="24" t="n"/>
       <c r="W32" s="26" t="n"/>
       <c r="X32" s="26" t="n"/>
-      <c r="Y32" s="38" t="n"/>
+      <c r="Y32" s="25" t="n"/>
       <c r="Z32" s="26" t="n"/>
       <c r="AA32" s="28" t="n"/>
       <c r="AB32" s="28" t="n"/>
-      <c r="AC32" s="40" t="n"/>
+      <c r="AC32" s="30" t="n"/>
       <c r="AD32" s="24" t="n"/>
       <c r="AE32" s="31" t="inlineStr">
         <is>
@@ -9164,11 +9133,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ32" s="38" t="n"/>
+      <c r="BJ32" s="25" t="n"/>
       <c r="BK32" s="26" t="n">
         <v>-108</v>
       </c>
-      <c r="BL32" s="39" t="n">
+      <c r="BL32" s="27" t="n">
         <v>1.925926</v>
       </c>
       <c r="BM32" s="28" t="n">
@@ -9178,16 +9147,16 @@
         <v>0.517413</v>
       </c>
       <c r="BO32" s="28" t="n"/>
-      <c r="BP32" s="38" t="n"/>
-      <c r="BQ32" s="39" t="n"/>
+      <c r="BP32" s="25" t="n"/>
+      <c r="BQ32" s="27" t="n"/>
       <c r="BR32" s="28" t="n"/>
       <c r="BS32" s="28" t="n"/>
       <c r="BT32" s="28" t="n"/>
-      <c r="BU32" s="38" t="n"/>
+      <c r="BU32" s="25" t="n"/>
       <c r="BV32" s="29" t="n"/>
       <c r="BW32" s="24" t="n"/>
-      <c r="BX32" s="40" t="n"/>
-      <c r="BY32" s="39" t="n"/>
+      <c r="BX32" s="30" t="n"/>
+      <c r="BY32" s="27" t="n"/>
       <c r="BZ32" s="24" t="n"/>
       <c r="CA32" s="31" t="n"/>
     </row>
@@ -9237,7 +9206,7 @@
           <t>away</t>
         </is>
       </c>
-      <c r="J33" s="38" t="n"/>
+      <c r="J33" s="25" t="n"/>
       <c r="K33" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -9246,7 +9215,7 @@
       <c r="L33" s="26" t="n">
         <v>135</v>
       </c>
-      <c r="M33" s="39" t="n">
+      <c r="M33" s="27" t="n">
         <v>2.35</v>
       </c>
       <c r="N33" s="28" t="n">
@@ -9278,11 +9247,11 @@
       <c r="V33" s="24" t="n"/>
       <c r="W33" s="26" t="n"/>
       <c r="X33" s="26" t="n"/>
-      <c r="Y33" s="38" t="n"/>
+      <c r="Y33" s="25" t="n"/>
       <c r="Z33" s="26" t="n"/>
       <c r="AA33" s="28" t="n"/>
       <c r="AB33" s="28" t="n"/>
-      <c r="AC33" s="40" t="n"/>
+      <c r="AC33" s="30" t="n"/>
       <c r="AD33" s="24" t="n"/>
       <c r="AE33" s="31" t="inlineStr">
         <is>
@@ -9413,11 +9382,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ33" s="38" t="n"/>
+      <c r="BJ33" s="25" t="n"/>
       <c r="BK33" s="26" t="n">
         <v>135</v>
       </c>
-      <c r="BL33" s="39" t="n">
+      <c r="BL33" s="27" t="n">
         <v>2.35</v>
       </c>
       <c r="BM33" s="28" t="n">
@@ -9427,16 +9396,16 @@
         <v>0.422886</v>
       </c>
       <c r="BO33" s="28" t="n"/>
-      <c r="BP33" s="38" t="n"/>
-      <c r="BQ33" s="39" t="n"/>
+      <c r="BP33" s="25" t="n"/>
+      <c r="BQ33" s="27" t="n"/>
       <c r="BR33" s="28" t="n"/>
       <c r="BS33" s="28" t="n"/>
       <c r="BT33" s="28" t="n"/>
-      <c r="BU33" s="38" t="n"/>
+      <c r="BU33" s="25" t="n"/>
       <c r="BV33" s="29" t="n"/>
       <c r="BW33" s="24" t="n"/>
-      <c r="BX33" s="40" t="n"/>
-      <c r="BY33" s="39" t="n"/>
+      <c r="BX33" s="30" t="n"/>
+      <c r="BY33" s="27" t="n"/>
       <c r="BZ33" s="24" t="n"/>
       <c r="CA33" s="31" t="n"/>
     </row>
@@ -9486,7 +9455,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J34" s="38" t="n"/>
+      <c r="J34" s="25" t="n"/>
       <c r="K34" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -9495,7 +9464,7 @@
       <c r="L34" s="26" t="n">
         <v>-127</v>
       </c>
-      <c r="M34" s="39" t="n">
+      <c r="M34" s="27" t="n">
         <v>1.787402</v>
       </c>
       <c r="N34" s="28" t="n">
@@ -9527,11 +9496,11 @@
       <c r="V34" s="24" t="n"/>
       <c r="W34" s="26" t="n"/>
       <c r="X34" s="26" t="n"/>
-      <c r="Y34" s="38" t="n"/>
+      <c r="Y34" s="25" t="n"/>
       <c r="Z34" s="26" t="n"/>
       <c r="AA34" s="28" t="n"/>
       <c r="AB34" s="28" t="n"/>
-      <c r="AC34" s="40" t="n"/>
+      <c r="AC34" s="30" t="n"/>
       <c r="AD34" s="24" t="n"/>
       <c r="AE34" s="31" t="inlineStr">
         <is>
@@ -9662,11 +9631,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ34" s="38" t="n"/>
+      <c r="BJ34" s="25" t="n"/>
       <c r="BK34" s="26" t="n">
         <v>-127</v>
       </c>
-      <c r="BL34" s="39" t="n">
+      <c r="BL34" s="27" t="n">
         <v>1.787402</v>
       </c>
       <c r="BM34" s="28" t="n">
@@ -9676,16 +9645,16 @@
         <v>0.557214</v>
       </c>
       <c r="BO34" s="28" t="n"/>
-      <c r="BP34" s="38" t="n"/>
-      <c r="BQ34" s="39" t="n"/>
+      <c r="BP34" s="25" t="n"/>
+      <c r="BQ34" s="27" t="n"/>
       <c r="BR34" s="28" t="n"/>
       <c r="BS34" s="28" t="n"/>
       <c r="BT34" s="28" t="n"/>
-      <c r="BU34" s="38" t="n"/>
+      <c r="BU34" s="25" t="n"/>
       <c r="BV34" s="29" t="n"/>
       <c r="BW34" s="24" t="n"/>
-      <c r="BX34" s="40" t="n"/>
-      <c r="BY34" s="39" t="n"/>
+      <c r="BX34" s="30" t="n"/>
+      <c r="BY34" s="27" t="n"/>
       <c r="BZ34" s="24" t="n"/>
       <c r="CA34" s="31" t="n"/>
     </row>
@@ -9735,7 +9704,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J35" s="38" t="n"/>
+      <c r="J35" s="25" t="n"/>
       <c r="K35" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -9744,7 +9713,7 @@
       <c r="L35" s="26" t="n">
         <v>-117</v>
       </c>
-      <c r="M35" s="39" t="n">
+      <c r="M35" s="27" t="n">
         <v>1.854701</v>
       </c>
       <c r="N35" s="28" t="n">
@@ -9776,11 +9745,11 @@
       <c r="V35" s="24" t="n"/>
       <c r="W35" s="26" t="n"/>
       <c r="X35" s="26" t="n"/>
-      <c r="Y35" s="38" t="n"/>
+      <c r="Y35" s="25" t="n"/>
       <c r="Z35" s="26" t="n"/>
       <c r="AA35" s="28" t="n"/>
       <c r="AB35" s="28" t="n"/>
-      <c r="AC35" s="40" t="n"/>
+      <c r="AC35" s="30" t="n"/>
       <c r="AD35" s="24" t="n"/>
       <c r="AE35" s="31" t="inlineStr">
         <is>
@@ -9911,11 +9880,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ35" s="38" t="n"/>
+      <c r="BJ35" s="25" t="n"/>
       <c r="BK35" s="26" t="n">
         <v>-117</v>
       </c>
-      <c r="BL35" s="39" t="n">
+      <c r="BL35" s="27" t="n">
         <v>1.854701</v>
       </c>
       <c r="BM35" s="28" t="n">
@@ -9925,16 +9894,16 @@
         <v>0.537313</v>
       </c>
       <c r="BO35" s="28" t="n"/>
-      <c r="BP35" s="38" t="n"/>
-      <c r="BQ35" s="39" t="n"/>
+      <c r="BP35" s="25" t="n"/>
+      <c r="BQ35" s="27" t="n"/>
       <c r="BR35" s="28" t="n"/>
       <c r="BS35" s="28" t="n"/>
       <c r="BT35" s="28" t="n"/>
-      <c r="BU35" s="38" t="n"/>
+      <c r="BU35" s="25" t="n"/>
       <c r="BV35" s="29" t="n"/>
       <c r="BW35" s="24" t="n"/>
-      <c r="BX35" s="40" t="n"/>
-      <c r="BY35" s="39" t="n"/>
+      <c r="BX35" s="30" t="n"/>
+      <c r="BY35" s="27" t="n"/>
       <c r="BZ35" s="24" t="n"/>
       <c r="CA35" s="31" t="n"/>
     </row>
@@ -9984,7 +9953,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J36" s="38" t="n"/>
+      <c r="J36" s="25" t="n"/>
       <c r="K36" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -9993,7 +9962,7 @@
       <c r="L36" s="26" t="n">
         <v>-125</v>
       </c>
-      <c r="M36" s="39" t="n">
+      <c r="M36" s="27" t="n">
         <v>1.8</v>
       </c>
       <c r="N36" s="28" t="n">
@@ -10025,11 +9994,11 @@
       <c r="V36" s="24" t="n"/>
       <c r="W36" s="26" t="n"/>
       <c r="X36" s="26" t="n"/>
-      <c r="Y36" s="38" t="n"/>
+      <c r="Y36" s="25" t="n"/>
       <c r="Z36" s="26" t="n"/>
       <c r="AA36" s="28" t="n"/>
       <c r="AB36" s="28" t="n"/>
-      <c r="AC36" s="40" t="n"/>
+      <c r="AC36" s="30" t="n"/>
       <c r="AD36" s="24" t="n"/>
       <c r="AE36" s="31" t="inlineStr">
         <is>
@@ -10160,11 +10129,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ36" s="38" t="n"/>
+      <c r="BJ36" s="25" t="n"/>
       <c r="BK36" s="26" t="n">
         <v>-125</v>
       </c>
-      <c r="BL36" s="39" t="n">
+      <c r="BL36" s="27" t="n">
         <v>1.8</v>
       </c>
       <c r="BM36" s="28" t="n">
@@ -10174,16 +10143,16 @@
         <v>0.552239</v>
       </c>
       <c r="BO36" s="28" t="n"/>
-      <c r="BP36" s="38" t="n"/>
-      <c r="BQ36" s="39" t="n"/>
+      <c r="BP36" s="25" t="n"/>
+      <c r="BQ36" s="27" t="n"/>
       <c r="BR36" s="28" t="n"/>
       <c r="BS36" s="28" t="n"/>
       <c r="BT36" s="28" t="n"/>
-      <c r="BU36" s="38" t="n"/>
+      <c r="BU36" s="25" t="n"/>
       <c r="BV36" s="29" t="n"/>
       <c r="BW36" s="24" t="n"/>
-      <c r="BX36" s="40" t="n"/>
-      <c r="BY36" s="39" t="n"/>
+      <c r="BX36" s="30" t="n"/>
+      <c r="BY36" s="27" t="n"/>
       <c r="BZ36" s="24" t="n"/>
       <c r="CA36" s="31" t="n"/>
     </row>
@@ -10233,7 +10202,7 @@
           <t>away</t>
         </is>
       </c>
-      <c r="J37" s="38" t="n"/>
+      <c r="J37" s="25" t="n"/>
       <c r="K37" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -10242,7 +10211,7 @@
       <c r="L37" s="26" t="n">
         <v>-102</v>
       </c>
-      <c r="M37" s="39" t="n">
+      <c r="M37" s="27" t="n">
         <v>1.980392</v>
       </c>
       <c r="N37" s="28" t="n">
@@ -10274,11 +10243,11 @@
       <c r="V37" s="24" t="n"/>
       <c r="W37" s="26" t="n"/>
       <c r="X37" s="26" t="n"/>
-      <c r="Y37" s="38" t="n"/>
+      <c r="Y37" s="25" t="n"/>
       <c r="Z37" s="26" t="n"/>
       <c r="AA37" s="28" t="n"/>
       <c r="AB37" s="28" t="n"/>
-      <c r="AC37" s="40" t="n"/>
+      <c r="AC37" s="30" t="n"/>
       <c r="AD37" s="24" t="n"/>
       <c r="AE37" s="31" t="inlineStr">
         <is>
@@ -10409,11 +10378,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ37" s="38" t="n"/>
+      <c r="BJ37" s="25" t="n"/>
       <c r="BK37" s="26" t="n">
         <v>-102</v>
       </c>
-      <c r="BL37" s="39" t="n">
+      <c r="BL37" s="27" t="n">
         <v>1.980392</v>
       </c>
       <c r="BM37" s="28" t="n">
@@ -10423,16 +10392,16 @@
         <v>0.502488</v>
       </c>
       <c r="BO37" s="28" t="n"/>
-      <c r="BP37" s="38" t="n"/>
-      <c r="BQ37" s="39" t="n"/>
+      <c r="BP37" s="25" t="n"/>
+      <c r="BQ37" s="27" t="n"/>
       <c r="BR37" s="28" t="n"/>
       <c r="BS37" s="28" t="n"/>
       <c r="BT37" s="28" t="n"/>
-      <c r="BU37" s="38" t="n"/>
+      <c r="BU37" s="25" t="n"/>
       <c r="BV37" s="29" t="n"/>
       <c r="BW37" s="24" t="n"/>
-      <c r="BX37" s="40" t="n"/>
-      <c r="BY37" s="39" t="n"/>
+      <c r="BX37" s="30" t="n"/>
+      <c r="BY37" s="27" t="n"/>
       <c r="BZ37" s="24" t="n"/>
       <c r="CA37" s="31" t="n"/>
     </row>
@@ -10482,7 +10451,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J38" s="38" t="n"/>
+      <c r="J38" s="25" t="n"/>
       <c r="K38" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -10491,7 +10460,7 @@
       <c r="L38" s="26" t="n">
         <v>108</v>
       </c>
-      <c r="M38" s="39" t="n">
+      <c r="M38" s="27" t="n">
         <v>2.08</v>
       </c>
       <c r="N38" s="28" t="n">
@@ -10523,11 +10492,11 @@
       <c r="V38" s="24" t="n"/>
       <c r="W38" s="26" t="n"/>
       <c r="X38" s="26" t="n"/>
-      <c r="Y38" s="38" t="n"/>
+      <c r="Y38" s="25" t="n"/>
       <c r="Z38" s="26" t="n"/>
       <c r="AA38" s="28" t="n"/>
       <c r="AB38" s="28" t="n"/>
-      <c r="AC38" s="40" t="n"/>
+      <c r="AC38" s="30" t="n"/>
       <c r="AD38" s="24" t="n"/>
       <c r="AE38" s="31" t="inlineStr">
         <is>
@@ -10658,11 +10627,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ38" s="38" t="n"/>
+      <c r="BJ38" s="25" t="n"/>
       <c r="BK38" s="26" t="n">
         <v>108</v>
       </c>
-      <c r="BL38" s="39" t="n">
+      <c r="BL38" s="27" t="n">
         <v>2.08</v>
       </c>
       <c r="BM38" s="28" t="n">
@@ -10672,16 +10641,16 @@
         <v>0.475248</v>
       </c>
       <c r="BO38" s="28" t="n"/>
-      <c r="BP38" s="38" t="n"/>
-      <c r="BQ38" s="39" t="n"/>
+      <c r="BP38" s="25" t="n"/>
+      <c r="BQ38" s="27" t="n"/>
       <c r="BR38" s="28" t="n"/>
       <c r="BS38" s="28" t="n"/>
       <c r="BT38" s="28" t="n"/>
-      <c r="BU38" s="38" t="n"/>
+      <c r="BU38" s="25" t="n"/>
       <c r="BV38" s="29" t="n"/>
       <c r="BW38" s="24" t="n"/>
-      <c r="BX38" s="40" t="n"/>
-      <c r="BY38" s="39" t="n"/>
+      <c r="BX38" s="30" t="n"/>
+      <c r="BY38" s="27" t="n"/>
       <c r="BZ38" s="24" t="n"/>
       <c r="CA38" s="31" t="n"/>
     </row>
@@ -10731,7 +10700,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J39" s="38" t="n"/>
+      <c r="J39" s="25" t="n"/>
       <c r="K39" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -10740,7 +10709,7 @@
       <c r="L39" s="26" t="n">
         <v>-108</v>
       </c>
-      <c r="M39" s="39" t="n">
+      <c r="M39" s="27" t="n">
         <v>1.925926</v>
       </c>
       <c r="N39" s="28" t="n">
@@ -10772,11 +10741,11 @@
       <c r="V39" s="24" t="n"/>
       <c r="W39" s="26" t="n"/>
       <c r="X39" s="26" t="n"/>
-      <c r="Y39" s="38" t="n"/>
+      <c r="Y39" s="25" t="n"/>
       <c r="Z39" s="26" t="n"/>
       <c r="AA39" s="28" t="n"/>
       <c r="AB39" s="28" t="n"/>
-      <c r="AC39" s="40" t="n"/>
+      <c r="AC39" s="30" t="n"/>
       <c r="AD39" s="24" t="n"/>
       <c r="AE39" s="31" t="inlineStr">
         <is>
@@ -10907,11 +10876,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ39" s="38" t="n"/>
+      <c r="BJ39" s="25" t="n"/>
       <c r="BK39" s="26" t="n">
         <v>-108</v>
       </c>
-      <c r="BL39" s="39" t="n">
+      <c r="BL39" s="27" t="n">
         <v>1.925926</v>
       </c>
       <c r="BM39" s="28" t="n">
@@ -10921,16 +10890,16 @@
         <v>0.517413</v>
       </c>
       <c r="BO39" s="28" t="n"/>
-      <c r="BP39" s="38" t="n"/>
-      <c r="BQ39" s="39" t="n"/>
+      <c r="BP39" s="25" t="n"/>
+      <c r="BQ39" s="27" t="n"/>
       <c r="BR39" s="28" t="n"/>
       <c r="BS39" s="28" t="n"/>
       <c r="BT39" s="28" t="n"/>
-      <c r="BU39" s="38" t="n"/>
+      <c r="BU39" s="25" t="n"/>
       <c r="BV39" s="29" t="n"/>
       <c r="BW39" s="24" t="n"/>
-      <c r="BX39" s="40" t="n"/>
-      <c r="BY39" s="39" t="n"/>
+      <c r="BX39" s="30" t="n"/>
+      <c r="BY39" s="27" t="n"/>
       <c r="BZ39" s="24" t="n"/>
       <c r="CA39" s="31" t="n"/>
     </row>

</xml_diff>

<commit_message>
feat: esports ledger integration + daily forecast fix
- cli.py: _log_esports_forecast() converts esports slate results to
  PickLedger rows (one per contract, best model side). Edge-gated for
  main ledger, all predictions for flat.
- cli.py: daily forecast now logs esports to both main (edge-gated)
  and flat (all) ledgers via _log_esports_forecast
- cli.py: SPORTS reverted to Polymarket keys only; ESPORTS_TITLES
  constant for CLI argument choices; removed duplicate local imports
- learned_market.py: qualified property now checks top-level qualified
  key (MLB v4 artifact format) in addition to nested qualification block
- All 266 tests pass, daily forecast runs clean
</commit_message>
<xml_diff>
--- a/data/picks.xlsx
+++ b/data/picks.xlsx
@@ -21,10 +21,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="0.0%"/>
-    <numFmt numFmtId="165" formatCode="0.0000"/>
-    <numFmt numFmtId="166" formatCode="0.0###"/>
-    <numFmt numFmtId="167" formatCode="0.000000"/>
+    <numFmt numFmtId="164" formatCode="0.0###"/>
+    <numFmt numFmtId="165" formatCode="0.000000"/>
+    <numFmt numFmtId="166" formatCode="0.0000"/>
+    <numFmt numFmtId="167" formatCode="0.0%"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -136,7 +136,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -150,10 +150,10 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -169,10 +169,10 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="10" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -184,10 +184,10 @@
     <xf numFmtId="0" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="10" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -202,13 +202,13 @@
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="10" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -217,38 +217,11 @@
     <xf numFmtId="2" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -327,8 +300,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CA35" headerRowCount="1">
-  <autoFilter ref="A1:CA35"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CA43" headerRowCount="1">
+  <autoFilter ref="A1:CA43"/>
   <tableColumns count="79">
     <tableColumn id="1" name="pick_id"/>
     <tableColumn id="2" name="created_at_utc"/>
@@ -765,23 +738,22 @@
     </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="6">
-        <f>COUNTA('Picks'!$A$2:$A$35)</f>
+        <f>COUNTA('Picks'!$A$2:$A$43)</f>
         <v/>
       </c>
       <c r="C4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$35,"open")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$43,"open")</f>
         <v/>
       </c>
       <c r="E4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$35,"settled")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$43,"settled")</f>
         <v/>
       </c>
       <c r="G4" s="6">
-        <f>IF(COUNTIFS('Picks'!$U$2:$U$35,"settled",'Picks'!$V$2:$V$35,"win")+COUNTIFS('Picks'!$U$2:$U$35,"settled",'Picks'!$V$2:$V$35,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
+        <f>IF(COUNTIFS('Picks'!$U$2:$U$43,"settled",'Picks'!$V$2:$V$43,"win")+COUNTIFS('Picks'!$U$2:$U$43,"settled",'Picks'!$V$2:$V$43,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
         <v/>
       </c>
     </row>
-    <row r="5"/>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
@@ -806,23 +778,22 @@
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="6">
-        <f>COUNTIF('Picks'!$BX$2:$BX$35,"&gt;0")</f>
+        <f>COUNTIF('Picks'!$BX$2:$BX$43,"&gt;0")</f>
         <v/>
       </c>
       <c r="C7" s="6">
-        <f>COUNTIFS('Picks'!$BX$2:$BX$35,"&gt;0",'Picks'!$V$2:$V$35,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$35,"&gt;0",'Picks'!$V$2:$V$35,"loss")</f>
+        <f>COUNTIFS('Picks'!$BX$2:$BX$43,"&gt;0",'Picks'!$V$2:$V$43,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$43,"&gt;0",'Picks'!$V$2:$V$43,"loss")</f>
         <v/>
       </c>
-      <c r="E7" s="32">
-        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$35,"&gt;0",'Picks'!$V$2:$V$35,"win")/(COUNTIFS('Picks'!$BX$2:$BX$35,"&gt;0",'Picks'!$V$2:$V$35,"win")+COUNTIFS('Picks'!$BX$2:$BX$35,"&gt;0",'Picks'!$V$2:$V$35,"loss")),0)</f>
+      <c r="E7" s="7">
+        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$43,"&gt;0",'Picks'!$V$2:$V$43,"win")/(COUNTIFS('Picks'!$BX$2:$BX$43,"&gt;0",'Picks'!$V$2:$V$43,"win")+COUNTIFS('Picks'!$BX$2:$BX$43,"&gt;0",'Picks'!$V$2:$V$43,"loss")),0)</f>
         <v/>
       </c>
-      <c r="G7" s="32">
-        <f>IFERROR(SUM('Picks'!$BY$2:$BY$35)/SUM('Picks'!$BX$2:$BX$35),0)</f>
+      <c r="G7" s="7">
+        <f>IFERROR(SUM('Picks'!$BY$2:$BY$43)/SUM('Picks'!$BX$2:$BX$43),0)</f>
         <v/>
       </c>
     </row>
-    <row r="8"/>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
@@ -846,24 +817,23 @@
       </c>
     </row>
     <row r="10" ht="28" customHeight="1">
-      <c r="A10" s="33">
-        <f>SUM('Picks'!$BY$2:$BY$35)</f>
+      <c r="A10" s="8">
+        <f>SUM('Picks'!$BY$2:$BY$43)</f>
         <v/>
       </c>
       <c r="C10" s="9">
-        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$35,"&lt;&gt;",'Picks'!$AB$2:$AB$35),0)</f>
+        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$43,"&lt;&gt;",'Picks'!$AB$2:$AB$43),0)</f>
         <v/>
       </c>
       <c r="E10" s="6">
-        <f>COUNTIFS('Picks'!$AM$2:$AM$35,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$35,"settled")</f>
+        <f>COUNTIFS('Picks'!$AM$2:$AM$43,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$43,"settled")</f>
         <v/>
       </c>
-      <c r="G10" s="33">
-        <f>SUMIFS('Picks'!$AC$2:$AC$35,'Picks'!$AM$2:$AM$35,"QUALIFIED_SHADOW_CALL")</f>
+      <c r="G10" s="8">
+        <f>SUMIFS('Picks'!$AC$2:$AC$43,'Picks'!$AM$2:$AM$43,"QUALIFIED_SHADOW_CALL")</f>
         <v/>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
         <is>
@@ -915,27 +885,27 @@
         </is>
       </c>
       <c r="B14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$35,$A14,'Picks'!$U$2:$U$35,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$43,$A14,'Picks'!$U$2:$U$43,"settled")</f>
         <v/>
       </c>
       <c r="C14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$35,$A14,'Picks'!$U$2:$U$35,"settled",'Picks'!$V$2:$V$35,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$43,$A14,'Picks'!$U$2:$U$43,"settled",'Picks'!$V$2:$V$43,"win")</f>
         <v/>
       </c>
       <c r="D14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$35,$A14,'Picks'!$U$2:$U$35,"settled",'Picks'!$V$2:$V$35,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$43,$A14,'Picks'!$U$2:$U$43,"settled",'Picks'!$V$2:$V$43,"loss")</f>
         <v/>
       </c>
-      <c r="E14" s="34">
+      <c r="E14" s="14">
         <f>IFERROR(C14/(C14+D14),0)</f>
         <v/>
       </c>
-      <c r="F14" s="35">
-        <f>SUMIFS('Picks'!$BY$2:$BY$35,'Picks'!$H$2:$H$35,$A14)</f>
+      <c r="F14" s="15">
+        <f>SUMIFS('Picks'!$BY$2:$BY$43,'Picks'!$H$2:$H$43,$A14)</f>
         <v/>
       </c>
       <c r="G14" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$35,'Picks'!$H$2:$H$35,$A14,'Picks'!$U$2:$U$35,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$43,'Picks'!$H$2:$H$43,$A14,'Picks'!$U$2:$U$43,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -946,27 +916,27 @@
         </is>
       </c>
       <c r="B15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$35,$A15,'Picks'!$U$2:$U$35,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$43,$A15,'Picks'!$U$2:$U$43,"settled")</f>
         <v/>
       </c>
       <c r="C15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$35,$A15,'Picks'!$U$2:$U$35,"settled",'Picks'!$V$2:$V$35,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$43,$A15,'Picks'!$U$2:$U$43,"settled",'Picks'!$V$2:$V$43,"win")</f>
         <v/>
       </c>
       <c r="D15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$35,$A15,'Picks'!$U$2:$U$35,"settled",'Picks'!$V$2:$V$35,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$43,$A15,'Picks'!$U$2:$U$43,"settled",'Picks'!$V$2:$V$43,"loss")</f>
         <v/>
       </c>
-      <c r="E15" s="36">
+      <c r="E15" s="19">
         <f>IFERROR(C15/(C15+D15),0)</f>
         <v/>
       </c>
-      <c r="F15" s="37">
-        <f>SUMIFS('Picks'!$BY$2:$BY$35,'Picks'!$H$2:$H$35,$A15)</f>
+      <c r="F15" s="20">
+        <f>SUMIFS('Picks'!$BY$2:$BY$43,'Picks'!$H$2:$H$43,$A15)</f>
         <v/>
       </c>
       <c r="G15" s="21">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$35,'Picks'!$H$2:$H$35,$A15,'Picks'!$U$2:$U$35,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$43,'Picks'!$H$2:$H$43,$A15,'Picks'!$U$2:$U$43,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -977,31 +947,30 @@
         </is>
       </c>
       <c r="B16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$35,$A16,'Picks'!$U$2:$U$35,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$43,$A16,'Picks'!$U$2:$U$43,"settled")</f>
         <v/>
       </c>
       <c r="C16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$35,$A16,'Picks'!$U$2:$U$35,"settled",'Picks'!$V$2:$V$35,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$43,$A16,'Picks'!$U$2:$U$43,"settled",'Picks'!$V$2:$V$43,"win")</f>
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$35,$A16,'Picks'!$U$2:$U$35,"settled",'Picks'!$V$2:$V$35,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$43,$A16,'Picks'!$U$2:$U$43,"settled",'Picks'!$V$2:$V$43,"loss")</f>
         <v/>
       </c>
-      <c r="E16" s="34">
+      <c r="E16" s="14">
         <f>IFERROR(C16/(C16+D16),0)</f>
         <v/>
       </c>
-      <c r="F16" s="35">
-        <f>SUMIFS('Picks'!$BY$2:$BY$35,'Picks'!$H$2:$H$35,$A16)</f>
+      <c r="F16" s="15">
+        <f>SUMIFS('Picks'!$BY$2:$BY$43,'Picks'!$H$2:$H$43,$A16)</f>
         <v/>
       </c>
       <c r="G16" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$35,'Picks'!$H$2:$H$35,$A16,'Picks'!$U$2:$U$35,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$43,'Picks'!$H$2:$H$43,$A16,'Picks'!$U$2:$U$43,"settled"),0)</f>
         <v/>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="22" t="inlineStr">
         <is>
@@ -1027,7 +996,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:CA35"/>
+  <dimension ref="A1:CA43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1554,7 +1523,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J2" s="38" t="n"/>
+      <c r="J2" s="25" t="n"/>
       <c r="K2" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -1563,7 +1532,7 @@
       <c r="L2" s="26" t="n">
         <v>117</v>
       </c>
-      <c r="M2" s="39" t="n">
+      <c r="M2" s="27" t="n">
         <v>2.17</v>
       </c>
       <c r="N2" s="28" t="n">
@@ -1603,11 +1572,11 @@
       <c r="X2" s="26" t="n">
         <v>108</v>
       </c>
-      <c r="Y2" s="38" t="n"/>
+      <c r="Y2" s="25" t="n"/>
       <c r="Z2" s="26" t="n"/>
       <c r="AA2" s="28" t="n"/>
       <c r="AB2" s="28" t="n"/>
-      <c r="AC2" s="40" t="n">
+      <c r="AC2" s="30" t="n">
         <v>1.755</v>
       </c>
       <c r="AD2" s="24" t="inlineStr">
@@ -1744,11 +1713,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ2" s="38" t="n"/>
+      <c r="BJ2" s="25" t="n"/>
       <c r="BK2" s="26" t="n">
         <v>117</v>
       </c>
-      <c r="BL2" s="39" t="n">
+      <c r="BL2" s="27" t="n">
         <v>2.17</v>
       </c>
       <c r="BM2" s="28" t="n">
@@ -1758,18 +1727,18 @@
         <v>0.455446</v>
       </c>
       <c r="BO2" s="28" t="n"/>
-      <c r="BP2" s="38" t="n"/>
-      <c r="BQ2" s="39" t="n"/>
+      <c r="BP2" s="25" t="n"/>
+      <c r="BQ2" s="27" t="n"/>
       <c r="BR2" s="28" t="n"/>
       <c r="BS2" s="28" t="n"/>
       <c r="BT2" s="28" t="n"/>
-      <c r="BU2" s="38" t="n"/>
+      <c r="BU2" s="25" t="n"/>
       <c r="BV2" s="29" t="n"/>
       <c r="BW2" s="24" t="n"/>
-      <c r="BX2" s="40" t="n">
+      <c r="BX2" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY2" s="39" t="n">
+      <c r="BY2" s="27" t="n">
         <v>1.17</v>
       </c>
       <c r="BZ2" s="24" t="inlineStr">
@@ -1829,7 +1798,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J3" s="38" t="n"/>
+      <c r="J3" s="25" t="n"/>
       <c r="K3" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -1838,7 +1807,7 @@
       <c r="L3" s="26" t="n">
         <v>-133</v>
       </c>
-      <c r="M3" s="39" t="n">
+      <c r="M3" s="27" t="n">
         <v>1.75188</v>
       </c>
       <c r="N3" s="28" t="n">
@@ -1878,11 +1847,11 @@
       <c r="X3" s="26" t="n">
         <v>8</v>
       </c>
-      <c r="Y3" s="38" t="n"/>
+      <c r="Y3" s="25" t="n"/>
       <c r="Z3" s="26" t="n"/>
       <c r="AA3" s="28" t="n"/>
       <c r="AB3" s="28" t="n"/>
-      <c r="AC3" s="40" t="n">
+      <c r="AC3" s="30" t="n">
         <v>1.1278</v>
       </c>
       <c r="AD3" s="24" t="inlineStr">
@@ -2019,11 +1988,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ3" s="38" t="n"/>
+      <c r="BJ3" s="25" t="n"/>
       <c r="BK3" s="26" t="n">
         <v>-133</v>
       </c>
-      <c r="BL3" s="39" t="n">
+      <c r="BL3" s="27" t="n">
         <v>1.75188</v>
       </c>
       <c r="BM3" s="28" t="n">
@@ -2033,18 +2002,18 @@
         <v>0.567164</v>
       </c>
       <c r="BO3" s="28" t="n"/>
-      <c r="BP3" s="38" t="n"/>
-      <c r="BQ3" s="39" t="n"/>
+      <c r="BP3" s="25" t="n"/>
+      <c r="BQ3" s="27" t="n"/>
       <c r="BR3" s="28" t="n"/>
       <c r="BS3" s="28" t="n"/>
       <c r="BT3" s="28" t="n"/>
-      <c r="BU3" s="38" t="n"/>
+      <c r="BU3" s="25" t="n"/>
       <c r="BV3" s="29" t="n"/>
       <c r="BW3" s="24" t="n"/>
-      <c r="BX3" s="40" t="n">
+      <c r="BX3" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY3" s="39" t="n">
+      <c r="BY3" s="27" t="n">
         <v>0.75188</v>
       </c>
       <c r="BZ3" s="24" t="inlineStr">
@@ -2104,7 +2073,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J4" s="38" t="n"/>
+      <c r="J4" s="25" t="n"/>
       <c r="K4" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -2113,7 +2082,7 @@
       <c r="L4" s="26" t="n">
         <v>-102</v>
       </c>
-      <c r="M4" s="39" t="n">
+      <c r="M4" s="27" t="n">
         <v>1.980392</v>
       </c>
       <c r="N4" s="28" t="n">
@@ -2153,11 +2122,11 @@
       <c r="X4" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="Y4" s="38" t="n"/>
+      <c r="Y4" s="25" t="n"/>
       <c r="Z4" s="26" t="n"/>
       <c r="AA4" s="28" t="n"/>
       <c r="AB4" s="28" t="n"/>
-      <c r="AC4" s="40" t="n">
+      <c r="AC4" s="30" t="n">
         <v>-1</v>
       </c>
       <c r="AD4" s="24" t="inlineStr">
@@ -2294,11 +2263,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ4" s="38" t="n"/>
+      <c r="BJ4" s="25" t="n"/>
       <c r="BK4" s="26" t="n">
         <v>-102</v>
       </c>
-      <c r="BL4" s="39" t="n">
+      <c r="BL4" s="27" t="n">
         <v>1.980392</v>
       </c>
       <c r="BM4" s="28" t="n">
@@ -2308,18 +2277,18 @@
         <v>0.502488</v>
       </c>
       <c r="BO4" s="28" t="n"/>
-      <c r="BP4" s="38" t="n"/>
-      <c r="BQ4" s="39" t="n"/>
+      <c r="BP4" s="25" t="n"/>
+      <c r="BQ4" s="27" t="n"/>
       <c r="BR4" s="28" t="n"/>
       <c r="BS4" s="28" t="n"/>
       <c r="BT4" s="28" t="n"/>
-      <c r="BU4" s="38" t="n"/>
+      <c r="BU4" s="25" t="n"/>
       <c r="BV4" s="29" t="n"/>
       <c r="BW4" s="24" t="n"/>
-      <c r="BX4" s="40" t="n">
+      <c r="BX4" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY4" s="39" t="n">
+      <c r="BY4" s="27" t="n">
         <v>-1</v>
       </c>
       <c r="BZ4" s="24" t="inlineStr">
@@ -2379,7 +2348,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J5" s="38" t="n"/>
+      <c r="J5" s="25" t="n"/>
       <c r="K5" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -2388,7 +2357,7 @@
       <c r="L5" s="26" t="n">
         <v>-133</v>
       </c>
-      <c r="M5" s="39" t="n">
+      <c r="M5" s="27" t="n">
         <v>1.75188</v>
       </c>
       <c r="N5" s="28" t="n">
@@ -2428,11 +2397,11 @@
       <c r="X5" s="26" t="n">
         <v>6</v>
       </c>
-      <c r="Y5" s="38" t="n"/>
+      <c r="Y5" s="25" t="n"/>
       <c r="Z5" s="26" t="n"/>
       <c r="AA5" s="28" t="n"/>
       <c r="AB5" s="28" t="n"/>
-      <c r="AC5" s="40" t="n">
+      <c r="AC5" s="30" t="n">
         <v>1.1278</v>
       </c>
       <c r="AD5" s="24" t="inlineStr">
@@ -2569,11 +2538,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ5" s="38" t="n"/>
+      <c r="BJ5" s="25" t="n"/>
       <c r="BK5" s="26" t="n">
         <v>-133</v>
       </c>
-      <c r="BL5" s="39" t="n">
+      <c r="BL5" s="27" t="n">
         <v>1.75188</v>
       </c>
       <c r="BM5" s="28" t="n">
@@ -2583,18 +2552,18 @@
         <v>0.567164</v>
       </c>
       <c r="BO5" s="28" t="n"/>
-      <c r="BP5" s="38" t="n"/>
-      <c r="BQ5" s="39" t="n"/>
+      <c r="BP5" s="25" t="n"/>
+      <c r="BQ5" s="27" t="n"/>
       <c r="BR5" s="28" t="n"/>
       <c r="BS5" s="28" t="n"/>
       <c r="BT5" s="28" t="n"/>
-      <c r="BU5" s="38" t="n"/>
+      <c r="BU5" s="25" t="n"/>
       <c r="BV5" s="29" t="n"/>
       <c r="BW5" s="24" t="n"/>
-      <c r="BX5" s="40" t="n">
+      <c r="BX5" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY5" s="39" t="n">
+      <c r="BY5" s="27" t="n">
         <v>0.75188</v>
       </c>
       <c r="BZ5" s="24" t="inlineStr">
@@ -2654,7 +2623,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J6" s="38" t="n"/>
+      <c r="J6" s="25" t="n"/>
       <c r="K6" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -2663,7 +2632,7 @@
       <c r="L6" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="M6" s="39" t="n">
+      <c r="M6" s="27" t="n">
         <v>1.961538</v>
       </c>
       <c r="N6" s="28" t="n">
@@ -2703,11 +2672,11 @@
       <c r="X6" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="Y6" s="38" t="n"/>
+      <c r="Y6" s="25" t="n"/>
       <c r="Z6" s="26" t="n"/>
       <c r="AA6" s="28" t="n"/>
       <c r="AB6" s="28" t="n"/>
-      <c r="AC6" s="40" t="n">
+      <c r="AC6" s="30" t="n">
         <v>1.2019</v>
       </c>
       <c r="AD6" s="24" t="inlineStr">
@@ -2844,11 +2813,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ6" s="38" t="n"/>
+      <c r="BJ6" s="25" t="n"/>
       <c r="BK6" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="BL6" s="39" t="n">
+      <c r="BL6" s="27" t="n">
         <v>1.961538</v>
       </c>
       <c r="BM6" s="28" t="n">
@@ -2858,18 +2827,18 @@
         <v>0.507463</v>
       </c>
       <c r="BO6" s="28" t="n"/>
-      <c r="BP6" s="38" t="n"/>
-      <c r="BQ6" s="39" t="n"/>
+      <c r="BP6" s="25" t="n"/>
+      <c r="BQ6" s="27" t="n"/>
       <c r="BR6" s="28" t="n"/>
       <c r="BS6" s="28" t="n"/>
       <c r="BT6" s="28" t="n"/>
-      <c r="BU6" s="38" t="n"/>
+      <c r="BU6" s="25" t="n"/>
       <c r="BV6" s="29" t="n"/>
       <c r="BW6" s="24" t="n"/>
-      <c r="BX6" s="40" t="n">
+      <c r="BX6" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY6" s="39" t="n">
+      <c r="BY6" s="27" t="n">
         <v>0.961538</v>
       </c>
       <c r="BZ6" s="24" t="inlineStr">
@@ -2929,7 +2898,7 @@
           <t>away</t>
         </is>
       </c>
-      <c r="J7" s="38" t="n"/>
+      <c r="J7" s="25" t="n"/>
       <c r="K7" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -2938,7 +2907,7 @@
       <c r="L7" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="M7" s="39" t="n">
+      <c r="M7" s="27" t="n">
         <v>1.961538</v>
       </c>
       <c r="N7" s="28" t="n">
@@ -2978,11 +2947,11 @@
       <c r="X7" s="26" t="n">
         <v>10</v>
       </c>
-      <c r="Y7" s="38" t="n"/>
+      <c r="Y7" s="25" t="n"/>
       <c r="Z7" s="26" t="n"/>
       <c r="AA7" s="28" t="n"/>
       <c r="AB7" s="28" t="n"/>
-      <c r="AC7" s="40" t="n">
+      <c r="AC7" s="30" t="n">
         <v>-1.25</v>
       </c>
       <c r="AD7" s="24" t="inlineStr">
@@ -3119,11 +3088,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ7" s="38" t="n"/>
+      <c r="BJ7" s="25" t="n"/>
       <c r="BK7" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="BL7" s="39" t="n">
+      <c r="BL7" s="27" t="n">
         <v>1.961538</v>
       </c>
       <c r="BM7" s="28" t="n">
@@ -3133,18 +3102,18 @@
         <v>0.507463</v>
       </c>
       <c r="BO7" s="28" t="n"/>
-      <c r="BP7" s="38" t="n"/>
-      <c r="BQ7" s="39" t="n"/>
+      <c r="BP7" s="25" t="n"/>
+      <c r="BQ7" s="27" t="n"/>
       <c r="BR7" s="28" t="n"/>
       <c r="BS7" s="28" t="n"/>
       <c r="BT7" s="28" t="n"/>
-      <c r="BU7" s="38" t="n"/>
+      <c r="BU7" s="25" t="n"/>
       <c r="BV7" s="29" t="n"/>
       <c r="BW7" s="24" t="n"/>
-      <c r="BX7" s="40" t="n">
+      <c r="BX7" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY7" s="39" t="n">
+      <c r="BY7" s="27" t="n">
         <v>-1</v>
       </c>
       <c r="BZ7" s="24" t="inlineStr">
@@ -3204,7 +3173,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J8" s="38" t="n"/>
+      <c r="J8" s="25" t="n"/>
       <c r="K8" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -3213,7 +3182,7 @@
       <c r="L8" s="26" t="n">
         <v>-106</v>
       </c>
-      <c r="M8" s="39" t="n">
+      <c r="M8" s="27" t="n">
         <v>1.943396</v>
       </c>
       <c r="N8" s="28" t="n">
@@ -3253,11 +3222,11 @@
       <c r="X8" s="26" t="n">
         <v>6</v>
       </c>
-      <c r="Y8" s="38" t="n"/>
+      <c r="Y8" s="25" t="n"/>
       <c r="Z8" s="26" t="n"/>
       <c r="AA8" s="28" t="n"/>
       <c r="AB8" s="28" t="n"/>
-      <c r="AC8" s="40" t="n">
+      <c r="AC8" s="30" t="n">
         <v>-1</v>
       </c>
       <c r="AD8" s="24" t="inlineStr">
@@ -3394,11 +3363,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ8" s="38" t="n"/>
+      <c r="BJ8" s="25" t="n"/>
       <c r="BK8" s="26" t="n">
         <v>-106</v>
       </c>
-      <c r="BL8" s="39" t="n">
+      <c r="BL8" s="27" t="n">
         <v>1.943396</v>
       </c>
       <c r="BM8" s="28" t="n">
@@ -3408,18 +3377,18 @@
         <v>0.5124379999999999</v>
       </c>
       <c r="BO8" s="28" t="n"/>
-      <c r="BP8" s="38" t="n"/>
-      <c r="BQ8" s="39" t="n"/>
+      <c r="BP8" s="25" t="n"/>
+      <c r="BQ8" s="27" t="n"/>
       <c r="BR8" s="28" t="n"/>
       <c r="BS8" s="28" t="n"/>
       <c r="BT8" s="28" t="n"/>
-      <c r="BU8" s="38" t="n"/>
+      <c r="BU8" s="25" t="n"/>
       <c r="BV8" s="29" t="n"/>
       <c r="BW8" s="24" t="n"/>
-      <c r="BX8" s="40" t="n">
+      <c r="BX8" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY8" s="39" t="n">
+      <c r="BY8" s="27" t="n">
         <v>-1</v>
       </c>
       <c r="BZ8" s="24" t="inlineStr">
@@ -3479,7 +3448,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J9" s="38" t="n"/>
+      <c r="J9" s="25" t="n"/>
       <c r="K9" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -3488,7 +3457,7 @@
       <c r="L9" s="26" t="n">
         <v>-102</v>
       </c>
-      <c r="M9" s="39" t="n">
+      <c r="M9" s="27" t="n">
         <v>1.980392</v>
       </c>
       <c r="N9" s="28" t="n">
@@ -3528,11 +3497,11 @@
       <c r="X9" s="26" t="n">
         <v>5</v>
       </c>
-      <c r="Y9" s="38" t="n"/>
+      <c r="Y9" s="25" t="n"/>
       <c r="Z9" s="26" t="n"/>
       <c r="AA9" s="28" t="n"/>
       <c r="AB9" s="28" t="n"/>
-      <c r="AC9" s="40" t="n">
+      <c r="AC9" s="30" t="n">
         <v>0.9804</v>
       </c>
       <c r="AD9" s="24" t="inlineStr">
@@ -3669,11 +3638,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ9" s="38" t="n"/>
+      <c r="BJ9" s="25" t="n"/>
       <c r="BK9" s="26" t="n">
         <v>-102</v>
       </c>
-      <c r="BL9" s="39" t="n">
+      <c r="BL9" s="27" t="n">
         <v>1.980392</v>
       </c>
       <c r="BM9" s="28" t="n">
@@ -3683,18 +3652,18 @@
         <v>0.502488</v>
       </c>
       <c r="BO9" s="28" t="n"/>
-      <c r="BP9" s="38" t="n"/>
-      <c r="BQ9" s="39" t="n"/>
+      <c r="BP9" s="25" t="n"/>
+      <c r="BQ9" s="27" t="n"/>
       <c r="BR9" s="28" t="n"/>
       <c r="BS9" s="28" t="n"/>
       <c r="BT9" s="28" t="n"/>
-      <c r="BU9" s="38" t="n"/>
+      <c r="BU9" s="25" t="n"/>
       <c r="BV9" s="29" t="n"/>
       <c r="BW9" s="24" t="n"/>
-      <c r="BX9" s="40" t="n">
+      <c r="BX9" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY9" s="39" t="n">
+      <c r="BY9" s="27" t="n">
         <v>0.980392</v>
       </c>
       <c r="BZ9" s="24" t="inlineStr">
@@ -3754,7 +3723,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J10" s="38" t="n"/>
+      <c r="J10" s="25" t="n"/>
       <c r="K10" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -3763,7 +3732,7 @@
       <c r="L10" s="26" t="n">
         <v>-138</v>
       </c>
-      <c r="M10" s="39" t="n">
+      <c r="M10" s="27" t="n">
         <v>1.724638</v>
       </c>
       <c r="N10" s="28" t="n">
@@ -3803,11 +3772,11 @@
       <c r="X10" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="Y10" s="38" t="n"/>
+      <c r="Y10" s="25" t="n"/>
       <c r="Z10" s="26" t="n"/>
       <c r="AA10" s="28" t="n"/>
       <c r="AB10" s="28" t="n"/>
-      <c r="AC10" s="40" t="n">
+      <c r="AC10" s="30" t="n">
         <v>1.2681</v>
       </c>
       <c r="AD10" s="24" t="inlineStr">
@@ -3944,11 +3913,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ10" s="38" t="n"/>
+      <c r="BJ10" s="25" t="n"/>
       <c r="BK10" s="26" t="n">
         <v>-138</v>
       </c>
-      <c r="BL10" s="39" t="n">
+      <c r="BL10" s="27" t="n">
         <v>1.724638</v>
       </c>
       <c r="BM10" s="28" t="n">
@@ -3958,18 +3927,18 @@
         <v>0.577114</v>
       </c>
       <c r="BO10" s="28" t="n"/>
-      <c r="BP10" s="38" t="n"/>
-      <c r="BQ10" s="39" t="n"/>
+      <c r="BP10" s="25" t="n"/>
+      <c r="BQ10" s="27" t="n"/>
       <c r="BR10" s="28" t="n"/>
       <c r="BS10" s="28" t="n"/>
       <c r="BT10" s="28" t="n"/>
-      <c r="BU10" s="38" t="n"/>
+      <c r="BU10" s="25" t="n"/>
       <c r="BV10" s="29" t="n"/>
       <c r="BW10" s="24" t="n"/>
-      <c r="BX10" s="40" t="n">
+      <c r="BX10" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY10" s="39" t="n">
+      <c r="BY10" s="27" t="n">
         <v>0.724638</v>
       </c>
       <c r="BZ10" s="24" t="inlineStr">
@@ -4029,7 +3998,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J11" s="38" t="n"/>
+      <c r="J11" s="25" t="n"/>
       <c r="K11" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -4038,7 +4007,7 @@
       <c r="L11" s="26" t="n">
         <v>102</v>
       </c>
-      <c r="M11" s="39" t="n">
+      <c r="M11" s="27" t="n">
         <v>2.02</v>
       </c>
       <c r="N11" s="28" t="n">
@@ -4078,11 +4047,11 @@
       <c r="X11" s="26" t="n">
         <v>15</v>
       </c>
-      <c r="Y11" s="38" t="n"/>
+      <c r="Y11" s="25" t="n"/>
       <c r="Z11" s="26" t="n"/>
       <c r="AA11" s="28" t="n"/>
       <c r="AB11" s="28" t="n"/>
-      <c r="AC11" s="40" t="n">
+      <c r="AC11" s="30" t="n">
         <v>1.275</v>
       </c>
       <c r="AD11" s="24" t="inlineStr">
@@ -4219,11 +4188,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ11" s="38" t="n"/>
+      <c r="BJ11" s="25" t="n"/>
       <c r="BK11" s="26" t="n">
         <v>102</v>
       </c>
-      <c r="BL11" s="39" t="n">
+      <c r="BL11" s="27" t="n">
         <v>2.02</v>
       </c>
       <c r="BM11" s="28" t="n">
@@ -4233,18 +4202,18 @@
         <v>0.492537</v>
       </c>
       <c r="BO11" s="28" t="n"/>
-      <c r="BP11" s="38" t="n"/>
-      <c r="BQ11" s="39" t="n"/>
+      <c r="BP11" s="25" t="n"/>
+      <c r="BQ11" s="27" t="n"/>
       <c r="BR11" s="28" t="n"/>
       <c r="BS11" s="28" t="n"/>
       <c r="BT11" s="28" t="n"/>
-      <c r="BU11" s="38" t="n"/>
+      <c r="BU11" s="25" t="n"/>
       <c r="BV11" s="29" t="n"/>
       <c r="BW11" s="24" t="n"/>
-      <c r="BX11" s="40" t="n">
+      <c r="BX11" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY11" s="39" t="n">
+      <c r="BY11" s="27" t="n">
         <v>1.02</v>
       </c>
       <c r="BZ11" s="24" t="inlineStr">
@@ -4304,7 +4273,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J12" s="38" t="n"/>
+      <c r="J12" s="25" t="n"/>
       <c r="K12" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -4313,7 +4282,7 @@
       <c r="L12" s="26" t="n">
         <v>-102</v>
       </c>
-      <c r="M12" s="39" t="n">
+      <c r="M12" s="27" t="n">
         <v>1.980392</v>
       </c>
       <c r="N12" s="28" t="n">
@@ -4353,11 +4322,11 @@
       <c r="X12" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="Y12" s="38" t="n"/>
+      <c r="Y12" s="25" t="n"/>
       <c r="Z12" s="26" t="n"/>
       <c r="AA12" s="28" t="n"/>
       <c r="AB12" s="28" t="n"/>
-      <c r="AC12" s="40" t="n">
+      <c r="AC12" s="30" t="n">
         <v>-1</v>
       </c>
       <c r="AD12" s="24" t="inlineStr">
@@ -4494,11 +4463,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ12" s="38" t="n"/>
+      <c r="BJ12" s="25" t="n"/>
       <c r="BK12" s="26" t="n">
         <v>-102</v>
       </c>
-      <c r="BL12" s="39" t="n">
+      <c r="BL12" s="27" t="n">
         <v>1.980392</v>
       </c>
       <c r="BM12" s="28" t="n">
@@ -4508,18 +4477,18 @@
         <v>0.502488</v>
       </c>
       <c r="BO12" s="28" t="n"/>
-      <c r="BP12" s="38" t="n"/>
-      <c r="BQ12" s="39" t="n"/>
+      <c r="BP12" s="25" t="n"/>
+      <c r="BQ12" s="27" t="n"/>
       <c r="BR12" s="28" t="n"/>
       <c r="BS12" s="28" t="n"/>
       <c r="BT12" s="28" t="n"/>
-      <c r="BU12" s="38" t="n"/>
+      <c r="BU12" s="25" t="n"/>
       <c r="BV12" s="29" t="n"/>
       <c r="BW12" s="24" t="n"/>
-      <c r="BX12" s="40" t="n">
+      <c r="BX12" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY12" s="39" t="n">
+      <c r="BY12" s="27" t="n">
         <v>-1</v>
       </c>
       <c r="BZ12" s="24" t="inlineStr">
@@ -4579,7 +4548,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J13" s="38" t="n"/>
+      <c r="J13" s="25" t="n"/>
       <c r="K13" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -4588,7 +4557,7 @@
       <c r="L13" s="26" t="n">
         <v>-102</v>
       </c>
-      <c r="M13" s="39" t="n">
+      <c r="M13" s="27" t="n">
         <v>1.980392</v>
       </c>
       <c r="N13" s="28" t="n">
@@ -4628,11 +4597,11 @@
       <c r="X13" s="26" t="n">
         <v>7</v>
       </c>
-      <c r="Y13" s="38" t="n"/>
+      <c r="Y13" s="25" t="n"/>
       <c r="Z13" s="26" t="n"/>
       <c r="AA13" s="28" t="n"/>
       <c r="AB13" s="28" t="n"/>
-      <c r="AC13" s="40" t="n">
+      <c r="AC13" s="30" t="n">
         <v>1.2255</v>
       </c>
       <c r="AD13" s="24" t="inlineStr">
@@ -4769,11 +4738,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ13" s="38" t="n"/>
+      <c r="BJ13" s="25" t="n"/>
       <c r="BK13" s="26" t="n">
         <v>-102</v>
       </c>
-      <c r="BL13" s="39" t="n">
+      <c r="BL13" s="27" t="n">
         <v>1.980392</v>
       </c>
       <c r="BM13" s="28" t="n">
@@ -4783,18 +4752,18 @@
         <v>0.502488</v>
       </c>
       <c r="BO13" s="28" t="n"/>
-      <c r="BP13" s="38" t="n"/>
-      <c r="BQ13" s="39" t="n"/>
+      <c r="BP13" s="25" t="n"/>
+      <c r="BQ13" s="27" t="n"/>
       <c r="BR13" s="28" t="n"/>
       <c r="BS13" s="28" t="n"/>
       <c r="BT13" s="28" t="n"/>
-      <c r="BU13" s="38" t="n"/>
+      <c r="BU13" s="25" t="n"/>
       <c r="BV13" s="29" t="n"/>
       <c r="BW13" s="24" t="n"/>
-      <c r="BX13" s="40" t="n">
+      <c r="BX13" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY13" s="39" t="n">
+      <c r="BY13" s="27" t="n">
         <v>0.980392</v>
       </c>
       <c r="BZ13" s="24" t="inlineStr">
@@ -4854,7 +4823,7 @@
           <t>away</t>
         </is>
       </c>
-      <c r="J14" s="38" t="n"/>
+      <c r="J14" s="25" t="n"/>
       <c r="K14" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -4863,7 +4832,7 @@
       <c r="L14" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="M14" s="39" t="n">
+      <c r="M14" s="27" t="n">
         <v>1.961538</v>
       </c>
       <c r="N14" s="28" t="n">
@@ -4903,11 +4872,11 @@
       <c r="X14" s="26" t="n">
         <v>6</v>
       </c>
-      <c r="Y14" s="38" t="n"/>
+      <c r="Y14" s="25" t="n"/>
       <c r="Z14" s="26" t="n"/>
       <c r="AA14" s="28" t="n"/>
       <c r="AB14" s="28" t="n"/>
-      <c r="AC14" s="40" t="n">
+      <c r="AC14" s="30" t="n">
         <v>-0.75</v>
       </c>
       <c r="AD14" s="24" t="inlineStr">
@@ -5044,11 +5013,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ14" s="38" t="n"/>
+      <c r="BJ14" s="25" t="n"/>
       <c r="BK14" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="BL14" s="39" t="n">
+      <c r="BL14" s="27" t="n">
         <v>1.961538</v>
       </c>
       <c r="BM14" s="28" t="n">
@@ -5058,18 +5027,18 @@
         <v>0.507463</v>
       </c>
       <c r="BO14" s="28" t="n"/>
-      <c r="BP14" s="38" t="n"/>
-      <c r="BQ14" s="39" t="n"/>
+      <c r="BP14" s="25" t="n"/>
+      <c r="BQ14" s="27" t="n"/>
       <c r="BR14" s="28" t="n"/>
       <c r="BS14" s="28" t="n"/>
       <c r="BT14" s="28" t="n"/>
-      <c r="BU14" s="38" t="n"/>
+      <c r="BU14" s="25" t="n"/>
       <c r="BV14" s="29" t="n"/>
       <c r="BW14" s="24" t="n"/>
-      <c r="BX14" s="40" t="n">
+      <c r="BX14" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY14" s="39" t="n">
+      <c r="BY14" s="27" t="n">
         <v>-1</v>
       </c>
       <c r="BZ14" s="24" t="inlineStr">
@@ -5129,7 +5098,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J15" s="38" t="n"/>
+      <c r="J15" s="25" t="n"/>
       <c r="K15" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -5138,7 +5107,7 @@
       <c r="L15" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="M15" s="39" t="n">
+      <c r="M15" s="27" t="n">
         <v>1.961538</v>
       </c>
       <c r="N15" s="28" t="n">
@@ -5178,11 +5147,11 @@
       <c r="X15" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="Y15" s="38" t="n"/>
+      <c r="Y15" s="25" t="n"/>
       <c r="Z15" s="26" t="n"/>
       <c r="AA15" s="28" t="n"/>
       <c r="AB15" s="28" t="n"/>
-      <c r="AC15" s="40" t="n">
+      <c r="AC15" s="30" t="n">
         <v>-1</v>
       </c>
       <c r="AD15" s="24" t="inlineStr">
@@ -5319,11 +5288,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ15" s="38" t="n"/>
+      <c r="BJ15" s="25" t="n"/>
       <c r="BK15" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="BL15" s="39" t="n">
+      <c r="BL15" s="27" t="n">
         <v>1.961538</v>
       </c>
       <c r="BM15" s="28" t="n">
@@ -5333,18 +5302,18 @@
         <v>0.507463</v>
       </c>
       <c r="BO15" s="28" t="n"/>
-      <c r="BP15" s="38" t="n"/>
-      <c r="BQ15" s="39" t="n"/>
+      <c r="BP15" s="25" t="n"/>
+      <c r="BQ15" s="27" t="n"/>
       <c r="BR15" s="28" t="n"/>
       <c r="BS15" s="28" t="n"/>
       <c r="BT15" s="28" t="n"/>
-      <c r="BU15" s="38" t="n"/>
+      <c r="BU15" s="25" t="n"/>
       <c r="BV15" s="29" t="n"/>
       <c r="BW15" s="24" t="n"/>
-      <c r="BX15" s="40" t="n">
+      <c r="BX15" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY15" s="39" t="n">
+      <c r="BY15" s="27" t="n">
         <v>-1</v>
       </c>
       <c r="BZ15" s="24" t="inlineStr">
@@ -5404,7 +5373,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J16" s="38" t="n"/>
+      <c r="J16" s="25" t="n"/>
       <c r="K16" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -5413,7 +5382,7 @@
       <c r="L16" s="26" t="n">
         <v>-111</v>
       </c>
-      <c r="M16" s="39" t="n">
+      <c r="M16" s="27" t="n">
         <v>1.900901</v>
       </c>
       <c r="N16" s="28" t="n">
@@ -5453,11 +5422,11 @@
       <c r="X16" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="Y16" s="38" t="n"/>
+      <c r="Y16" s="25" t="n"/>
       <c r="Z16" s="26" t="n"/>
       <c r="AA16" s="28" t="n"/>
       <c r="AB16" s="28" t="n"/>
-      <c r="AC16" s="40" t="n">
+      <c r="AC16" s="30" t="n">
         <v>-1.5</v>
       </c>
       <c r="AD16" s="24" t="inlineStr">
@@ -5594,11 +5563,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ16" s="38" t="n"/>
+      <c r="BJ16" s="25" t="n"/>
       <c r="BK16" s="26" t="n">
         <v>-111</v>
       </c>
-      <c r="BL16" s="39" t="n">
+      <c r="BL16" s="27" t="n">
         <v>1.900901</v>
       </c>
       <c r="BM16" s="28" t="n">
@@ -5608,18 +5577,18 @@
         <v>0.522388</v>
       </c>
       <c r="BO16" s="28" t="n"/>
-      <c r="BP16" s="38" t="n"/>
-      <c r="BQ16" s="39" t="n"/>
+      <c r="BP16" s="25" t="n"/>
+      <c r="BQ16" s="27" t="n"/>
       <c r="BR16" s="28" t="n"/>
       <c r="BS16" s="28" t="n"/>
       <c r="BT16" s="28" t="n"/>
-      <c r="BU16" s="38" t="n"/>
+      <c r="BU16" s="25" t="n"/>
       <c r="BV16" s="29" t="n"/>
       <c r="BW16" s="24" t="n"/>
-      <c r="BX16" s="40" t="n">
+      <c r="BX16" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY16" s="39" t="n">
+      <c r="BY16" s="27" t="n">
         <v>-1</v>
       </c>
       <c r="BZ16" s="24" t="inlineStr">
@@ -5679,7 +5648,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J17" s="38" t="n"/>
+      <c r="J17" s="25" t="n"/>
       <c r="K17" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -5688,7 +5657,7 @@
       <c r="L17" s="26" t="n">
         <v>-108</v>
       </c>
-      <c r="M17" s="39" t="n">
+      <c r="M17" s="27" t="n">
         <v>1.925926</v>
       </c>
       <c r="N17" s="28" t="n">
@@ -5728,11 +5697,11 @@
       <c r="X17" s="26" t="n">
         <v>6</v>
       </c>
-      <c r="Y17" s="38" t="n"/>
+      <c r="Y17" s="25" t="n"/>
       <c r="Z17" s="26" t="n"/>
       <c r="AA17" s="28" t="n"/>
       <c r="AB17" s="28" t="n"/>
-      <c r="AC17" s="40" t="n">
+      <c r="AC17" s="30" t="n">
         <v>0.9258999999999999</v>
       </c>
       <c r="AD17" s="24" t="inlineStr">
@@ -5869,11 +5838,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ17" s="38" t="n"/>
+      <c r="BJ17" s="25" t="n"/>
       <c r="BK17" s="26" t="n">
         <v>-108</v>
       </c>
-      <c r="BL17" s="39" t="n">
+      <c r="BL17" s="27" t="n">
         <v>1.925926</v>
       </c>
       <c r="BM17" s="28" t="n">
@@ -5883,18 +5852,18 @@
         <v>0.5148509999999999</v>
       </c>
       <c r="BO17" s="28" t="n"/>
-      <c r="BP17" s="38" t="n"/>
-      <c r="BQ17" s="39" t="n"/>
+      <c r="BP17" s="25" t="n"/>
+      <c r="BQ17" s="27" t="n"/>
       <c r="BR17" s="28" t="n"/>
       <c r="BS17" s="28" t="n"/>
       <c r="BT17" s="28" t="n"/>
-      <c r="BU17" s="38" t="n"/>
+      <c r="BU17" s="25" t="n"/>
       <c r="BV17" s="29" t="n"/>
       <c r="BW17" s="24" t="n"/>
-      <c r="BX17" s="40" t="n">
+      <c r="BX17" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY17" s="39" t="n">
+      <c r="BY17" s="27" t="n">
         <v>0.925926</v>
       </c>
       <c r="BZ17" s="24" t="inlineStr">
@@ -5954,7 +5923,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J18" s="38" t="n"/>
+      <c r="J18" s="25" t="n"/>
       <c r="K18" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -5963,7 +5932,7 @@
       <c r="L18" s="26" t="n">
         <v>111</v>
       </c>
-      <c r="M18" s="39" t="n">
+      <c r="M18" s="27" t="n">
         <v>2.11</v>
       </c>
       <c r="N18" s="28" t="n">
@@ -6003,11 +5972,11 @@
       <c r="X18" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="Y18" s="38" t="n"/>
+      <c r="Y18" s="25" t="n"/>
       <c r="Z18" s="26" t="n"/>
       <c r="AA18" s="28" t="n"/>
       <c r="AB18" s="28" t="n"/>
-      <c r="AC18" s="40" t="n">
+      <c r="AC18" s="30" t="n">
         <v>-1.25</v>
       </c>
       <c r="AD18" s="24" t="inlineStr">
@@ -6144,11 +6113,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ18" s="38" t="n"/>
+      <c r="BJ18" s="25" t="n"/>
       <c r="BK18" s="26" t="n">
         <v>111</v>
       </c>
-      <c r="BL18" s="39" t="n">
+      <c r="BL18" s="27" t="n">
         <v>2.11</v>
       </c>
       <c r="BM18" s="28" t="n">
@@ -6158,18 +6127,18 @@
         <v>0.472637</v>
       </c>
       <c r="BO18" s="28" t="n"/>
-      <c r="BP18" s="38" t="n"/>
-      <c r="BQ18" s="39" t="n"/>
+      <c r="BP18" s="25" t="n"/>
+      <c r="BQ18" s="27" t="n"/>
       <c r="BR18" s="28" t="n"/>
       <c r="BS18" s="28" t="n"/>
       <c r="BT18" s="28" t="n"/>
-      <c r="BU18" s="38" t="n"/>
+      <c r="BU18" s="25" t="n"/>
       <c r="BV18" s="29" t="n"/>
       <c r="BW18" s="24" t="n"/>
-      <c r="BX18" s="40" t="n">
+      <c r="BX18" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY18" s="39" t="n">
+      <c r="BY18" s="27" t="n">
         <v>-1</v>
       </c>
       <c r="BZ18" s="24" t="inlineStr">
@@ -6229,7 +6198,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J19" s="38" t="n"/>
+      <c r="J19" s="25" t="n"/>
       <c r="K19" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -6238,7 +6207,7 @@
       <c r="L19" s="26" t="n">
         <v>-125</v>
       </c>
-      <c r="M19" s="39" t="n">
+      <c r="M19" s="27" t="n">
         <v>1.8</v>
       </c>
       <c r="N19" s="28" t="n">
@@ -6278,11 +6247,11 @@
       <c r="X19" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="Y19" s="38" t="n"/>
+      <c r="Y19" s="25" t="n"/>
       <c r="Z19" s="26" t="n"/>
       <c r="AA19" s="28" t="n"/>
       <c r="AB19" s="28" t="n"/>
-      <c r="AC19" s="40" t="n">
+      <c r="AC19" s="30" t="n">
         <v>1.2</v>
       </c>
       <c r="AD19" s="24" t="inlineStr">
@@ -6419,11 +6388,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ19" s="38" t="n"/>
+      <c r="BJ19" s="25" t="n"/>
       <c r="BK19" s="26" t="n">
         <v>-125</v>
       </c>
-      <c r="BL19" s="39" t="n">
+      <c r="BL19" s="27" t="n">
         <v>1.8</v>
       </c>
       <c r="BM19" s="28" t="n">
@@ -6433,18 +6402,18 @@
         <v>0.552239</v>
       </c>
       <c r="BO19" s="28" t="n"/>
-      <c r="BP19" s="38" t="n"/>
-      <c r="BQ19" s="39" t="n"/>
+      <c r="BP19" s="25" t="n"/>
+      <c r="BQ19" s="27" t="n"/>
       <c r="BR19" s="28" t="n"/>
       <c r="BS19" s="28" t="n"/>
       <c r="BT19" s="28" t="n"/>
-      <c r="BU19" s="38" t="n"/>
+      <c r="BU19" s="25" t="n"/>
       <c r="BV19" s="29" t="n"/>
       <c r="BW19" s="24" t="n"/>
-      <c r="BX19" s="40" t="n">
+      <c r="BX19" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY19" s="39" t="n">
+      <c r="BY19" s="27" t="n">
         <v>0.8</v>
       </c>
       <c r="BZ19" s="24" t="inlineStr">
@@ -6504,7 +6473,7 @@
           <t>away</t>
         </is>
       </c>
-      <c r="J20" s="38" t="n"/>
+      <c r="J20" s="25" t="n"/>
       <c r="K20" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -6513,7 +6482,7 @@
       <c r="L20" s="26" t="n">
         <v>106</v>
       </c>
-      <c r="M20" s="39" t="n">
+      <c r="M20" s="27" t="n">
         <v>2.06</v>
       </c>
       <c r="N20" s="28" t="n">
@@ -6553,11 +6522,11 @@
       <c r="X20" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="Y20" s="38" t="n"/>
+      <c r="Y20" s="25" t="n"/>
       <c r="Z20" s="26" t="n"/>
       <c r="AA20" s="28" t="n"/>
       <c r="AB20" s="28" t="n"/>
-      <c r="AC20" s="40" t="n">
+      <c r="AC20" s="30" t="n">
         <v>0.795</v>
       </c>
       <c r="AD20" s="24" t="inlineStr">
@@ -6694,11 +6663,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ20" s="38" t="n"/>
+      <c r="BJ20" s="25" t="n"/>
       <c r="BK20" s="26" t="n">
         <v>106</v>
       </c>
-      <c r="BL20" s="39" t="n">
+      <c r="BL20" s="27" t="n">
         <v>2.06</v>
       </c>
       <c r="BM20" s="28" t="n">
@@ -6708,18 +6677,18 @@
         <v>0.482587</v>
       </c>
       <c r="BO20" s="28" t="n"/>
-      <c r="BP20" s="38" t="n"/>
-      <c r="BQ20" s="39" t="n"/>
+      <c r="BP20" s="25" t="n"/>
+      <c r="BQ20" s="27" t="n"/>
       <c r="BR20" s="28" t="n"/>
       <c r="BS20" s="28" t="n"/>
       <c r="BT20" s="28" t="n"/>
-      <c r="BU20" s="38" t="n"/>
+      <c r="BU20" s="25" t="n"/>
       <c r="BV20" s="29" t="n"/>
       <c r="BW20" s="24" t="n"/>
-      <c r="BX20" s="40" t="n">
+      <c r="BX20" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY20" s="39" t="n">
+      <c r="BY20" s="27" t="n">
         <v>1.06</v>
       </c>
       <c r="BZ20" s="24" t="inlineStr">
@@ -6779,7 +6748,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J21" s="38" t="n"/>
+      <c r="J21" s="25" t="n"/>
       <c r="K21" s="24" t="inlineStr">
         <is>
           <t>polymarket</t>
@@ -6788,7 +6757,7 @@
       <c r="L21" s="26" t="n">
         <v>-106</v>
       </c>
-      <c r="M21" s="39" t="n">
+      <c r="M21" s="27" t="n">
         <v>1.943396</v>
       </c>
       <c r="N21" s="28" t="n">
@@ -6830,11 +6799,11 @@
       <c r="X21" s="26" t="n">
         <v>10</v>
       </c>
-      <c r="Y21" s="38" t="n"/>
+      <c r="Y21" s="25" t="n"/>
       <c r="Z21" s="26" t="n"/>
       <c r="AA21" s="28" t="n"/>
       <c r="AB21" s="28" t="n"/>
-      <c r="AC21" s="40" t="n">
+      <c r="AC21" s="30" t="n">
         <v>0.9434</v>
       </c>
       <c r="AD21" s="24" t="inlineStr">
@@ -6893,11 +6862,11 @@
         </is>
       </c>
       <c r="BI21" s="24" t="n"/>
-      <c r="BJ21" s="38" t="n"/>
+      <c r="BJ21" s="25" t="n"/>
       <c r="BK21" s="26" t="n">
         <v>-106</v>
       </c>
-      <c r="BL21" s="39" t="n">
+      <c r="BL21" s="27" t="n">
         <v>1.943396</v>
       </c>
       <c r="BM21" s="28" t="n">
@@ -6907,16 +6876,16 @@
         <v>0.5124379999999999</v>
       </c>
       <c r="BO21" s="28" t="n"/>
-      <c r="BP21" s="38" t="n"/>
-      <c r="BQ21" s="39" t="n"/>
+      <c r="BP21" s="25" t="n"/>
+      <c r="BQ21" s="27" t="n"/>
       <c r="BR21" s="28" t="n"/>
       <c r="BS21" s="28" t="n"/>
       <c r="BT21" s="28" t="n"/>
-      <c r="BU21" s="38" t="n"/>
+      <c r="BU21" s="25" t="n"/>
       <c r="BV21" s="29" t="n"/>
       <c r="BW21" s="24" t="n"/>
-      <c r="BX21" s="40" t="n"/>
-      <c r="BY21" s="39" t="n"/>
+      <c r="BX21" s="30" t="n"/>
+      <c r="BY21" s="27" t="n"/>
       <c r="BZ21" s="24" t="n"/>
       <c r="CA21" s="31" t="n"/>
     </row>
@@ -6966,7 +6935,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J22" s="38" t="n"/>
+      <c r="J22" s="25" t="n"/>
       <c r="K22" s="24" t="inlineStr">
         <is>
           <t>polymarket</t>
@@ -6975,7 +6944,7 @@
       <c r="L22" s="26" t="n">
         <v>-106</v>
       </c>
-      <c r="M22" s="39" t="n">
+      <c r="M22" s="27" t="n">
         <v>1.943396</v>
       </c>
       <c r="N22" s="28" t="n">
@@ -7017,11 +6986,11 @@
       <c r="X22" s="26" t="n">
         <v>5</v>
       </c>
-      <c r="Y22" s="38" t="n"/>
+      <c r="Y22" s="25" t="n"/>
       <c r="Z22" s="26" t="n"/>
       <c r="AA22" s="28" t="n"/>
       <c r="AB22" s="28" t="n"/>
-      <c r="AC22" s="40" t="n">
+      <c r="AC22" s="30" t="n">
         <v>0.9434</v>
       </c>
       <c r="AD22" s="24" t="inlineStr">
@@ -7080,11 +7049,11 @@
         </is>
       </c>
       <c r="BI22" s="24" t="n"/>
-      <c r="BJ22" s="38" t="n"/>
+      <c r="BJ22" s="25" t="n"/>
       <c r="BK22" s="26" t="n">
         <v>-106</v>
       </c>
-      <c r="BL22" s="39" t="n">
+      <c r="BL22" s="27" t="n">
         <v>1.943396</v>
       </c>
       <c r="BM22" s="28" t="n">
@@ -7094,16 +7063,16 @@
         <v>0.5124379999999999</v>
       </c>
       <c r="BO22" s="28" t="n"/>
-      <c r="BP22" s="38" t="n"/>
-      <c r="BQ22" s="39" t="n"/>
+      <c r="BP22" s="25" t="n"/>
+      <c r="BQ22" s="27" t="n"/>
       <c r="BR22" s="28" t="n"/>
       <c r="BS22" s="28" t="n"/>
       <c r="BT22" s="28" t="n"/>
-      <c r="BU22" s="38" t="n"/>
+      <c r="BU22" s="25" t="n"/>
       <c r="BV22" s="29" t="n"/>
       <c r="BW22" s="24" t="n"/>
-      <c r="BX22" s="40" t="n"/>
-      <c r="BY22" s="39" t="n"/>
+      <c r="BX22" s="30" t="n"/>
+      <c r="BY22" s="27" t="n"/>
       <c r="BZ22" s="24" t="n"/>
       <c r="CA22" s="31" t="n"/>
     </row>
@@ -7153,7 +7122,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J23" s="38" t="n"/>
+      <c r="J23" s="25" t="n"/>
       <c r="K23" s="24" t="inlineStr">
         <is>
           <t>polymarket</t>
@@ -7162,7 +7131,7 @@
       <c r="L23" s="26" t="n">
         <v>-141</v>
       </c>
-      <c r="M23" s="39" t="n">
+      <c r="M23" s="27" t="n">
         <v>1.70922</v>
       </c>
       <c r="N23" s="28" t="n">
@@ -7204,11 +7173,11 @@
       <c r="X23" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="Y23" s="38" t="n"/>
+      <c r="Y23" s="25" t="n"/>
       <c r="Z23" s="26" t="n"/>
       <c r="AA23" s="28" t="n"/>
       <c r="AB23" s="28" t="n"/>
-      <c r="AC23" s="40" t="n">
+      <c r="AC23" s="30" t="n">
         <v>1.2411</v>
       </c>
       <c r="AD23" s="24" t="inlineStr">
@@ -7267,11 +7236,11 @@
         </is>
       </c>
       <c r="BI23" s="24" t="n"/>
-      <c r="BJ23" s="38" t="n"/>
+      <c r="BJ23" s="25" t="n"/>
       <c r="BK23" s="26" t="n">
         <v>-141</v>
       </c>
-      <c r="BL23" s="39" t="n">
+      <c r="BL23" s="27" t="n">
         <v>1.70922</v>
       </c>
       <c r="BM23" s="28" t="n">
@@ -7281,16 +7250,16 @@
         <v>0.58209</v>
       </c>
       <c r="BO23" s="28" t="n"/>
-      <c r="BP23" s="38" t="n"/>
-      <c r="BQ23" s="39" t="n"/>
+      <c r="BP23" s="25" t="n"/>
+      <c r="BQ23" s="27" t="n"/>
       <c r="BR23" s="28" t="n"/>
       <c r="BS23" s="28" t="n"/>
       <c r="BT23" s="28" t="n"/>
-      <c r="BU23" s="38" t="n"/>
+      <c r="BU23" s="25" t="n"/>
       <c r="BV23" s="29" t="n"/>
       <c r="BW23" s="24" t="n"/>
-      <c r="BX23" s="40" t="n"/>
-      <c r="BY23" s="39" t="n"/>
+      <c r="BX23" s="30" t="n"/>
+      <c r="BY23" s="27" t="n"/>
       <c r="BZ23" s="24" t="n"/>
       <c r="CA23" s="31" t="n"/>
     </row>
@@ -7340,7 +7309,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J24" s="38" t="n"/>
+      <c r="J24" s="25" t="n"/>
       <c r="K24" s="24" t="inlineStr">
         <is>
           <t>polymarket</t>
@@ -7349,7 +7318,7 @@
       <c r="L24" s="26" t="n">
         <v>-133</v>
       </c>
-      <c r="M24" s="39" t="n">
+      <c r="M24" s="27" t="n">
         <v>1.75188</v>
       </c>
       <c r="N24" s="28" t="n">
@@ -7391,11 +7360,11 @@
       <c r="X24" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="Y24" s="38" t="n"/>
+      <c r="Y24" s="25" t="n"/>
       <c r="Z24" s="26" t="n"/>
       <c r="AA24" s="28" t="n"/>
       <c r="AB24" s="28" t="n"/>
-      <c r="AC24" s="40" t="n">
+      <c r="AC24" s="30" t="n">
         <v>-1.5</v>
       </c>
       <c r="AD24" s="24" t="inlineStr">
@@ -7454,11 +7423,11 @@
         </is>
       </c>
       <c r="BI24" s="24" t="n"/>
-      <c r="BJ24" s="38" t="n"/>
+      <c r="BJ24" s="25" t="n"/>
       <c r="BK24" s="26" t="n">
         <v>-133</v>
       </c>
-      <c r="BL24" s="39" t="n">
+      <c r="BL24" s="27" t="n">
         <v>1.75188</v>
       </c>
       <c r="BM24" s="28" t="n">
@@ -7468,16 +7437,16 @@
         <v>0.567164</v>
       </c>
       <c r="BO24" s="28" t="n"/>
-      <c r="BP24" s="38" t="n"/>
-      <c r="BQ24" s="39" t="n"/>
+      <c r="BP24" s="25" t="n"/>
+      <c r="BQ24" s="27" t="n"/>
       <c r="BR24" s="28" t="n"/>
       <c r="BS24" s="28" t="n"/>
       <c r="BT24" s="28" t="n"/>
-      <c r="BU24" s="38" t="n"/>
+      <c r="BU24" s="25" t="n"/>
       <c r="BV24" s="29" t="n"/>
       <c r="BW24" s="24" t="n"/>
-      <c r="BX24" s="40" t="n"/>
-      <c r="BY24" s="39" t="n"/>
+      <c r="BX24" s="30" t="n"/>
+      <c r="BY24" s="27" t="n"/>
       <c r="BZ24" s="24" t="n"/>
       <c r="CA24" s="31" t="n"/>
     </row>
@@ -7527,7 +7496,7 @@
           <t>away</t>
         </is>
       </c>
-      <c r="J25" s="38" t="n"/>
+      <c r="J25" s="25" t="n"/>
       <c r="K25" s="24" t="inlineStr">
         <is>
           <t>polymarket</t>
@@ -7536,7 +7505,7 @@
       <c r="L25" s="26" t="n">
         <v>104</v>
       </c>
-      <c r="M25" s="39" t="n">
+      <c r="M25" s="27" t="n">
         <v>2.04</v>
       </c>
       <c r="N25" s="28" t="n">
@@ -7578,11 +7547,11 @@
       <c r="X25" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="Y25" s="38" t="n"/>
+      <c r="Y25" s="25" t="n"/>
       <c r="Z25" s="26" t="n"/>
       <c r="AA25" s="28" t="n"/>
       <c r="AB25" s="28" t="n"/>
-      <c r="AC25" s="40" t="n">
+      <c r="AC25" s="30" t="n">
         <v>1.3</v>
       </c>
       <c r="AD25" s="24" t="inlineStr">
@@ -7641,11 +7610,11 @@
         </is>
       </c>
       <c r="BI25" s="24" t="n"/>
-      <c r="BJ25" s="38" t="n"/>
+      <c r="BJ25" s="25" t="n"/>
       <c r="BK25" s="26" t="n">
         <v>104</v>
       </c>
-      <c r="BL25" s="39" t="n">
+      <c r="BL25" s="27" t="n">
         <v>2.04</v>
       </c>
       <c r="BM25" s="28" t="n">
@@ -7655,16 +7624,16 @@
         <v>0.487562</v>
       </c>
       <c r="BO25" s="28" t="n"/>
-      <c r="BP25" s="38" t="n"/>
-      <c r="BQ25" s="39" t="n"/>
+      <c r="BP25" s="25" t="n"/>
+      <c r="BQ25" s="27" t="n"/>
       <c r="BR25" s="28" t="n"/>
       <c r="BS25" s="28" t="n"/>
       <c r="BT25" s="28" t="n"/>
-      <c r="BU25" s="38" t="n"/>
+      <c r="BU25" s="25" t="n"/>
       <c r="BV25" s="29" t="n"/>
       <c r="BW25" s="24" t="n"/>
-      <c r="BX25" s="40" t="n"/>
-      <c r="BY25" s="39" t="n"/>
+      <c r="BX25" s="30" t="n"/>
+      <c r="BY25" s="27" t="n"/>
       <c r="BZ25" s="24" t="n"/>
       <c r="CA25" s="31" t="n"/>
     </row>
@@ -7714,7 +7683,7 @@
           <t>away</t>
         </is>
       </c>
-      <c r="J26" s="38" t="n"/>
+      <c r="J26" s="25" t="n"/>
       <c r="K26" s="24" t="inlineStr">
         <is>
           <t>polymarket</t>
@@ -7723,7 +7692,7 @@
       <c r="L26" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="M26" s="39" t="n">
+      <c r="M26" s="27" t="n">
         <v>1.961538</v>
       </c>
       <c r="N26" s="28" t="n">
@@ -7765,11 +7734,11 @@
       <c r="X26" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="Y26" s="38" t="n"/>
+      <c r="Y26" s="25" t="n"/>
       <c r="Z26" s="26" t="n"/>
       <c r="AA26" s="28" t="n"/>
       <c r="AB26" s="28" t="n"/>
-      <c r="AC26" s="40" t="n">
+      <c r="AC26" s="30" t="n">
         <v>0.9615</v>
       </c>
       <c r="AD26" s="24" t="inlineStr">
@@ -7828,11 +7797,11 @@
         </is>
       </c>
       <c r="BI26" s="24" t="n"/>
-      <c r="BJ26" s="38" t="n"/>
+      <c r="BJ26" s="25" t="n"/>
       <c r="BK26" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="BL26" s="39" t="n">
+      <c r="BL26" s="27" t="n">
         <v>1.961538</v>
       </c>
       <c r="BM26" s="28" t="n">
@@ -7842,16 +7811,16 @@
         <v>0.507463</v>
       </c>
       <c r="BO26" s="28" t="n"/>
-      <c r="BP26" s="38" t="n"/>
-      <c r="BQ26" s="39" t="n"/>
+      <c r="BP26" s="25" t="n"/>
+      <c r="BQ26" s="27" t="n"/>
       <c r="BR26" s="28" t="n"/>
       <c r="BS26" s="28" t="n"/>
       <c r="BT26" s="28" t="n"/>
-      <c r="BU26" s="38" t="n"/>
+      <c r="BU26" s="25" t="n"/>
       <c r="BV26" s="29" t="n"/>
       <c r="BW26" s="24" t="n"/>
-      <c r="BX26" s="40" t="n"/>
-      <c r="BY26" s="39" t="n"/>
+      <c r="BX26" s="30" t="n"/>
+      <c r="BY26" s="27" t="n"/>
       <c r="BZ26" s="24" t="n"/>
       <c r="CA26" s="31" t="n"/>
     </row>
@@ -7901,7 +7870,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J27" s="38" t="n"/>
+      <c r="J27" s="25" t="n"/>
       <c r="K27" s="24" t="inlineStr">
         <is>
           <t>polymarket</t>
@@ -7910,7 +7879,7 @@
       <c r="L27" s="26" t="n">
         <v>120</v>
       </c>
-      <c r="M27" s="39" t="n">
+      <c r="M27" s="27" t="n">
         <v>2.2</v>
       </c>
       <c r="N27" s="28" t="n">
@@ -7952,11 +7921,11 @@
       <c r="X27" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="Y27" s="38" t="n"/>
+      <c r="Y27" s="25" t="n"/>
       <c r="Z27" s="26" t="n"/>
       <c r="AA27" s="28" t="n"/>
       <c r="AB27" s="28" t="n"/>
-      <c r="AC27" s="40" t="n">
+      <c r="AC27" s="30" t="n">
         <v>-0.75</v>
       </c>
       <c r="AD27" s="24" t="inlineStr">
@@ -8015,11 +7984,11 @@
         </is>
       </c>
       <c r="BI27" s="24" t="n"/>
-      <c r="BJ27" s="38" t="n"/>
+      <c r="BJ27" s="25" t="n"/>
       <c r="BK27" s="26" t="n">
         <v>120</v>
       </c>
-      <c r="BL27" s="39" t="n">
+      <c r="BL27" s="27" t="n">
         <v>2.2</v>
       </c>
       <c r="BM27" s="28" t="n">
@@ -8029,16 +7998,16 @@
         <v>0.452736</v>
       </c>
       <c r="BO27" s="28" t="n"/>
-      <c r="BP27" s="38" t="n"/>
-      <c r="BQ27" s="39" t="n"/>
+      <c r="BP27" s="25" t="n"/>
+      <c r="BQ27" s="27" t="n"/>
       <c r="BR27" s="28" t="n"/>
       <c r="BS27" s="28" t="n"/>
       <c r="BT27" s="28" t="n"/>
-      <c r="BU27" s="38" t="n"/>
+      <c r="BU27" s="25" t="n"/>
       <c r="BV27" s="29" t="n"/>
       <c r="BW27" s="24" t="n"/>
-      <c r="BX27" s="40" t="n"/>
-      <c r="BY27" s="39" t="n"/>
+      <c r="BX27" s="30" t="n"/>
+      <c r="BY27" s="27" t="n"/>
       <c r="BZ27" s="24" t="n"/>
       <c r="CA27" s="31" t="n"/>
     </row>
@@ -8088,7 +8057,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J28" s="38" t="n"/>
+      <c r="J28" s="25" t="n"/>
       <c r="K28" s="24" t="inlineStr">
         <is>
           <t>polymarket</t>
@@ -8097,7 +8066,7 @@
       <c r="L28" s="26" t="n">
         <v>100</v>
       </c>
-      <c r="M28" s="39" t="n">
+      <c r="M28" s="27" t="n">
         <v>2</v>
       </c>
       <c r="N28" s="28" t="n">
@@ -8139,11 +8108,11 @@
       <c r="X28" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="Y28" s="38" t="n"/>
+      <c r="Y28" s="25" t="n"/>
       <c r="Z28" s="26" t="n"/>
       <c r="AA28" s="28" t="n"/>
       <c r="AB28" s="28" t="n"/>
-      <c r="AC28" s="40" t="n">
+      <c r="AC28" s="30" t="n">
         <v>-0.75</v>
       </c>
       <c r="AD28" s="24" t="inlineStr">
@@ -8202,11 +8171,11 @@
         </is>
       </c>
       <c r="BI28" s="24" t="n"/>
-      <c r="BJ28" s="38" t="n"/>
+      <c r="BJ28" s="25" t="n"/>
       <c r="BK28" s="26" t="n">
         <v>100</v>
       </c>
-      <c r="BL28" s="39" t="n">
+      <c r="BL28" s="27" t="n">
         <v>2</v>
       </c>
       <c r="BM28" s="28" t="n">
@@ -8216,16 +8185,16 @@
         <v>0.497512</v>
       </c>
       <c r="BO28" s="28" t="n"/>
-      <c r="BP28" s="38" t="n"/>
-      <c r="BQ28" s="39" t="n"/>
+      <c r="BP28" s="25" t="n"/>
+      <c r="BQ28" s="27" t="n"/>
       <c r="BR28" s="28" t="n"/>
       <c r="BS28" s="28" t="n"/>
       <c r="BT28" s="28" t="n"/>
-      <c r="BU28" s="38" t="n"/>
+      <c r="BU28" s="25" t="n"/>
       <c r="BV28" s="29" t="n"/>
       <c r="BW28" s="24" t="n"/>
-      <c r="BX28" s="40" t="n"/>
-      <c r="BY28" s="39" t="n"/>
+      <c r="BX28" s="30" t="n"/>
+      <c r="BY28" s="27" t="n"/>
       <c r="BZ28" s="24" t="n"/>
       <c r="CA28" s="31" t="n"/>
     </row>
@@ -8275,7 +8244,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J29" s="38" t="n"/>
+      <c r="J29" s="25" t="n"/>
       <c r="K29" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -8284,7 +8253,7 @@
       <c r="L29" s="26" t="n">
         <v>108</v>
       </c>
-      <c r="M29" s="39" t="n">
+      <c r="M29" s="27" t="n">
         <v>2.08</v>
       </c>
       <c r="N29" s="28" t="n">
@@ -8324,11 +8293,11 @@
       <c r="X29" s="26" t="n">
         <v>8</v>
       </c>
-      <c r="Y29" s="38" t="n"/>
+      <c r="Y29" s="25" t="n"/>
       <c r="Z29" s="26" t="n"/>
       <c r="AA29" s="28" t="n"/>
       <c r="AB29" s="28" t="n"/>
-      <c r="AC29" s="40" t="n">
+      <c r="AC29" s="30" t="n">
         <v>1.35</v>
       </c>
       <c r="AD29" s="24" t="inlineStr">
@@ -8465,11 +8434,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ29" s="38" t="n"/>
+      <c r="BJ29" s="25" t="n"/>
       <c r="BK29" s="26" t="n">
         <v>108</v>
       </c>
-      <c r="BL29" s="39" t="n">
+      <c r="BL29" s="27" t="n">
         <v>2.08</v>
       </c>
       <c r="BM29" s="28" t="n">
@@ -8479,18 +8448,18 @@
         <v>0.477612</v>
       </c>
       <c r="BO29" s="28" t="n"/>
-      <c r="BP29" s="38" t="n"/>
-      <c r="BQ29" s="39" t="n"/>
+      <c r="BP29" s="25" t="n"/>
+      <c r="BQ29" s="27" t="n"/>
       <c r="BR29" s="28" t="n"/>
       <c r="BS29" s="28" t="n"/>
       <c r="BT29" s="28" t="n"/>
-      <c r="BU29" s="38" t="n"/>
+      <c r="BU29" s="25" t="n"/>
       <c r="BV29" s="29" t="n"/>
       <c r="BW29" s="24" t="n"/>
-      <c r="BX29" s="40" t="n">
+      <c r="BX29" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY29" s="39" t="n">
+      <c r="BY29" s="27" t="n">
         <v>1.08</v>
       </c>
       <c r="BZ29" s="24" t="inlineStr">
@@ -8550,7 +8519,7 @@
           <t>away</t>
         </is>
       </c>
-      <c r="J30" s="38" t="n"/>
+      <c r="J30" s="25" t="n"/>
       <c r="K30" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -8559,7 +8528,7 @@
       <c r="L30" s="26" t="n">
         <v>-133</v>
       </c>
-      <c r="M30" s="39" t="n">
+      <c r="M30" s="27" t="n">
         <v>1.75188</v>
       </c>
       <c r="N30" s="28" t="n">
@@ -8599,11 +8568,11 @@
       <c r="X30" s="26" t="n">
         <v>6</v>
       </c>
-      <c r="Y30" s="38" t="n"/>
+      <c r="Y30" s="25" t="n"/>
       <c r="Z30" s="26" t="n"/>
       <c r="AA30" s="28" t="n"/>
       <c r="AB30" s="28" t="n"/>
-      <c r="AC30" s="40" t="n">
+      <c r="AC30" s="30" t="n">
         <v>1.1278</v>
       </c>
       <c r="AD30" s="24" t="inlineStr">
@@ -8740,11 +8709,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ30" s="38" t="n"/>
+      <c r="BJ30" s="25" t="n"/>
       <c r="BK30" s="26" t="n">
         <v>-133</v>
       </c>
-      <c r="BL30" s="39" t="n">
+      <c r="BL30" s="27" t="n">
         <v>1.75188</v>
       </c>
       <c r="BM30" s="28" t="n">
@@ -8754,18 +8723,18 @@
         <v>0.567164</v>
       </c>
       <c r="BO30" s="28" t="n"/>
-      <c r="BP30" s="38" t="n"/>
-      <c r="BQ30" s="39" t="n"/>
+      <c r="BP30" s="25" t="n"/>
+      <c r="BQ30" s="27" t="n"/>
       <c r="BR30" s="28" t="n"/>
       <c r="BS30" s="28" t="n"/>
       <c r="BT30" s="28" t="n"/>
-      <c r="BU30" s="38" t="n"/>
+      <c r="BU30" s="25" t="n"/>
       <c r="BV30" s="29" t="n"/>
       <c r="BW30" s="24" t="n"/>
-      <c r="BX30" s="40" t="n">
+      <c r="BX30" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY30" s="39" t="n">
+      <c r="BY30" s="27" t="n">
         <v>0.75188</v>
       </c>
       <c r="BZ30" s="24" t="inlineStr">
@@ -8825,7 +8794,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J31" s="38" t="n"/>
+      <c r="J31" s="25" t="n"/>
       <c r="K31" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -8834,7 +8803,7 @@
       <c r="L31" s="26" t="n">
         <v>130</v>
       </c>
-      <c r="M31" s="39" t="n">
+      <c r="M31" s="27" t="n">
         <v>2.3</v>
       </c>
       <c r="N31" s="28" t="n">
@@ -8874,11 +8843,11 @@
       <c r="X31" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="Y31" s="38" t="n"/>
+      <c r="Y31" s="25" t="n"/>
       <c r="Z31" s="26" t="n"/>
       <c r="AA31" s="28" t="n"/>
       <c r="AB31" s="28" t="n"/>
-      <c r="AC31" s="40" t="n">
+      <c r="AC31" s="30" t="n">
         <v>-1</v>
       </c>
       <c r="AD31" s="24" t="inlineStr">
@@ -9015,11 +8984,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ31" s="38" t="n"/>
+      <c r="BJ31" s="25" t="n"/>
       <c r="BK31" s="26" t="n">
         <v>130</v>
       </c>
-      <c r="BL31" s="39" t="n">
+      <c r="BL31" s="27" t="n">
         <v>2.3</v>
       </c>
       <c r="BM31" s="28" t="n">
@@ -9029,18 +8998,18 @@
         <v>0.432836</v>
       </c>
       <c r="BO31" s="28" t="n"/>
-      <c r="BP31" s="38" t="n"/>
-      <c r="BQ31" s="39" t="n"/>
+      <c r="BP31" s="25" t="n"/>
+      <c r="BQ31" s="27" t="n"/>
       <c r="BR31" s="28" t="n"/>
       <c r="BS31" s="28" t="n"/>
       <c r="BT31" s="28" t="n"/>
-      <c r="BU31" s="38" t="n"/>
+      <c r="BU31" s="25" t="n"/>
       <c r="BV31" s="29" t="n"/>
       <c r="BW31" s="24" t="n"/>
-      <c r="BX31" s="40" t="n">
+      <c r="BX31" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY31" s="39" t="n">
+      <c r="BY31" s="27" t="n">
         <v>-1</v>
       </c>
       <c r="BZ31" s="24" t="inlineStr">
@@ -9057,12 +9026,12 @@
     <row r="32" ht="36" customHeight="1">
       <c r="A32" s="24" t="inlineStr">
         <is>
-          <t>3b298c42597d4a62</t>
+          <t>ad621924660a4d49</t>
         </is>
       </c>
       <c r="B32" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T15:22:23.198190Z</t>
+          <t>2026-07-20T15:44:08.951770Z</t>
         </is>
       </c>
       <c r="C32" s="24" t="inlineStr">
@@ -9100,30 +9069,30 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J32" s="38" t="n"/>
+      <c r="J32" s="25" t="n"/>
       <c r="K32" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
         </is>
       </c>
       <c r="L32" s="26" t="n">
-        <v>111</v>
-      </c>
-      <c r="M32" s="39" t="n">
-        <v>2.11</v>
+        <v>113</v>
+      </c>
+      <c r="M32" s="27" t="n">
+        <v>2.13</v>
       </c>
       <c r="N32" s="28" t="n">
-        <v>0.473934</v>
+        <v>0.469484</v>
       </c>
       <c r="O32" s="28" t="n">
         <v>0.5726869999999999</v>
       </c>
       <c r="P32" s="28" t="n"/>
       <c r="Q32" s="28" t="n">
-        <v>0.09875299999999999</v>
+        <v>0.103203</v>
       </c>
       <c r="R32" s="26" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="S32" s="29" t="n">
         <v>1.25</v>
@@ -9141,15 +9110,15 @@
       <c r="V32" s="24" t="n"/>
       <c r="W32" s="26" t="n"/>
       <c r="X32" s="26" t="n"/>
-      <c r="Y32" s="38" t="n"/>
+      <c r="Y32" s="25" t="n"/>
       <c r="Z32" s="26" t="n"/>
       <c r="AA32" s="28" t="n"/>
       <c r="AB32" s="28" t="n"/>
-      <c r="AC32" s="40" t="n"/>
+      <c r="AC32" s="30" t="n"/>
       <c r="AD32" s="24" t="n"/>
       <c r="AE32" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.5500; executable ask 0.4750 (aec-mlb-min-cle-2026-07-20).</t>
+          <t>Learned LR call at threshold 0.5500; executable ask 0.4700 (aec-mlb-min-cle-2026-07-20).</t>
         </is>
       </c>
       <c r="AF32" s="31" t="inlineStr">
@@ -9268,7 +9237,7 @@
       </c>
       <c r="BH32" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T14:57:32.219947Z</t>
+          <t>2026-07-20T15:40:37.473344Z</t>
         </is>
       </c>
       <c r="BI32" s="24" t="inlineStr">
@@ -9276,42 +9245,42 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ32" s="38" t="n"/>
+      <c r="BJ32" s="25" t="n"/>
       <c r="BK32" s="26" t="n">
-        <v>111</v>
-      </c>
-      <c r="BL32" s="39" t="n">
-        <v>2.11</v>
+        <v>113</v>
+      </c>
+      <c r="BL32" s="27" t="n">
+        <v>2.13</v>
       </c>
       <c r="BM32" s="28" t="n">
-        <v>0.473934</v>
+        <v>0.469484</v>
       </c>
       <c r="BN32" s="28" t="n">
-        <v>0.472637</v>
+        <v>0.467662</v>
       </c>
       <c r="BO32" s="28" t="n"/>
-      <c r="BP32" s="38" t="n"/>
-      <c r="BQ32" s="39" t="n"/>
+      <c r="BP32" s="25" t="n"/>
+      <c r="BQ32" s="27" t="n"/>
       <c r="BR32" s="28" t="n"/>
       <c r="BS32" s="28" t="n"/>
       <c r="BT32" s="28" t="n"/>
-      <c r="BU32" s="38" t="n"/>
+      <c r="BU32" s="25" t="n"/>
       <c r="BV32" s="29" t="n"/>
       <c r="BW32" s="24" t="n"/>
-      <c r="BX32" s="40" t="n"/>
-      <c r="BY32" s="39" t="n"/>
+      <c r="BX32" s="30" t="n"/>
+      <c r="BY32" s="27" t="n"/>
       <c r="BZ32" s="24" t="n"/>
       <c r="CA32" s="31" t="n"/>
     </row>
     <row r="33" ht="36" customHeight="1">
       <c r="A33" s="24" t="inlineStr">
         <is>
-          <t>81ad16e9351d4806</t>
+          <t>a72d0dab60924d62</t>
         </is>
       </c>
       <c r="B33" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T15:22:23.198190Z</t>
+          <t>2026-07-20T15:44:08.951770Z</t>
         </is>
       </c>
       <c r="C33" s="24" t="inlineStr">
@@ -9349,7 +9318,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J33" s="38" t="n"/>
+      <c r="J33" s="25" t="n"/>
       <c r="K33" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -9358,7 +9327,7 @@
       <c r="L33" s="26" t="n">
         <v>-108</v>
       </c>
-      <c r="M33" s="39" t="n">
+      <c r="M33" s="27" t="n">
         <v>1.925926</v>
       </c>
       <c r="N33" s="28" t="n">
@@ -9390,11 +9359,11 @@
       <c r="V33" s="24" t="n"/>
       <c r="W33" s="26" t="n"/>
       <c r="X33" s="26" t="n"/>
-      <c r="Y33" s="38" t="n"/>
+      <c r="Y33" s="25" t="n"/>
       <c r="Z33" s="26" t="n"/>
       <c r="AA33" s="28" t="n"/>
       <c r="AB33" s="28" t="n"/>
-      <c r="AC33" s="40" t="n"/>
+      <c r="AC33" s="30" t="n"/>
       <c r="AD33" s="24" t="n"/>
       <c r="AE33" s="31" t="inlineStr">
         <is>
@@ -9517,7 +9486,7 @@
       </c>
       <c r="BH33" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T14:57:35.056972Z</t>
+          <t>2026-07-20T15:40:38.983839Z</t>
         </is>
       </c>
       <c r="BI33" s="24" t="inlineStr">
@@ -9525,11 +9494,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ33" s="38" t="n"/>
+      <c r="BJ33" s="25" t="n"/>
       <c r="BK33" s="26" t="n">
         <v>-108</v>
       </c>
-      <c r="BL33" s="39" t="n">
+      <c r="BL33" s="27" t="n">
         <v>1.925926</v>
       </c>
       <c r="BM33" s="28" t="n">
@@ -9539,28 +9508,28 @@
         <v>0.517413</v>
       </c>
       <c r="BO33" s="28" t="n"/>
-      <c r="BP33" s="38" t="n"/>
-      <c r="BQ33" s="39" t="n"/>
+      <c r="BP33" s="25" t="n"/>
+      <c r="BQ33" s="27" t="n"/>
       <c r="BR33" s="28" t="n"/>
       <c r="BS33" s="28" t="n"/>
       <c r="BT33" s="28" t="n"/>
-      <c r="BU33" s="38" t="n"/>
+      <c r="BU33" s="25" t="n"/>
       <c r="BV33" s="29" t="n"/>
       <c r="BW33" s="24" t="n"/>
-      <c r="BX33" s="40" t="n"/>
-      <c r="BY33" s="39" t="n"/>
+      <c r="BX33" s="30" t="n"/>
+      <c r="BY33" s="27" t="n"/>
       <c r="BZ33" s="24" t="n"/>
       <c r="CA33" s="31" t="n"/>
     </row>
     <row r="34" ht="36" customHeight="1">
       <c r="A34" s="24" t="inlineStr">
         <is>
-          <t>d928b5795af74522</t>
+          <t>f96e5bd1ebcc4c62</t>
         </is>
       </c>
       <c r="B34" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T15:22:23.198190Z</t>
+          <t>2026-07-20T15:44:08.951770Z</t>
         </is>
       </c>
       <c r="C34" s="24" t="inlineStr">
@@ -9598,7 +9567,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J34" s="38" t="n"/>
+      <c r="J34" s="25" t="n"/>
       <c r="K34" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -9607,7 +9576,7 @@
       <c r="L34" s="26" t="n">
         <v>-108</v>
       </c>
-      <c r="M34" s="39" t="n">
+      <c r="M34" s="27" t="n">
         <v>1.925926</v>
       </c>
       <c r="N34" s="28" t="n">
@@ -9639,11 +9608,11 @@
       <c r="V34" s="24" t="n"/>
       <c r="W34" s="26" t="n"/>
       <c r="X34" s="26" t="n"/>
-      <c r="Y34" s="38" t="n"/>
+      <c r="Y34" s="25" t="n"/>
       <c r="Z34" s="26" t="n"/>
       <c r="AA34" s="28" t="n"/>
       <c r="AB34" s="28" t="n"/>
-      <c r="AC34" s="40" t="n"/>
+      <c r="AC34" s="30" t="n"/>
       <c r="AD34" s="24" t="n"/>
       <c r="AE34" s="31" t="inlineStr">
         <is>
@@ -9766,7 +9735,7 @@
       </c>
       <c r="BH34" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T14:57:46.871986Z</t>
+          <t>2026-07-20T15:40:51.564498Z</t>
         </is>
       </c>
       <c r="BI34" s="24" t="inlineStr">
@@ -9774,42 +9743,42 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ34" s="38" t="n"/>
+      <c r="BJ34" s="25" t="n"/>
       <c r="BK34" s="26" t="n">
         <v>-108</v>
       </c>
-      <c r="BL34" s="39" t="n">
+      <c r="BL34" s="27" t="n">
         <v>1.925926</v>
       </c>
       <c r="BM34" s="28" t="n">
         <v>0.519231</v>
       </c>
       <c r="BN34" s="28" t="n">
-        <v>0.517413</v>
+        <v>0.5148509999999999</v>
       </c>
       <c r="BO34" s="28" t="n"/>
-      <c r="BP34" s="38" t="n"/>
-      <c r="BQ34" s="39" t="n"/>
+      <c r="BP34" s="25" t="n"/>
+      <c r="BQ34" s="27" t="n"/>
       <c r="BR34" s="28" t="n"/>
       <c r="BS34" s="28" t="n"/>
       <c r="BT34" s="28" t="n"/>
-      <c r="BU34" s="38" t="n"/>
+      <c r="BU34" s="25" t="n"/>
       <c r="BV34" s="29" t="n"/>
       <c r="BW34" s="24" t="n"/>
-      <c r="BX34" s="40" t="n"/>
-      <c r="BY34" s="39" t="n"/>
+      <c r="BX34" s="30" t="n"/>
+      <c r="BY34" s="27" t="n"/>
       <c r="BZ34" s="24" t="n"/>
       <c r="CA34" s="31" t="n"/>
     </row>
     <row r="35" ht="36" customHeight="1">
       <c r="A35" s="24" t="inlineStr">
         <is>
-          <t>1b170fab0ebb46ee</t>
+          <t>147749d13cbd4451</t>
         </is>
       </c>
       <c r="B35" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T15:28:43.848060Z</t>
+          <t>2026-07-20T15:44:12.511288Z</t>
         </is>
       </c>
       <c r="C35" s="24" t="inlineStr">
@@ -9847,27 +9816,27 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J35" s="38" t="n"/>
+      <c r="J35" s="25" t="n"/>
       <c r="K35" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
         </is>
       </c>
       <c r="L35" s="26" t="n">
-        <v>156</v>
-      </c>
-      <c r="M35" s="39" t="n">
-        <v>2.56</v>
+        <v>150</v>
+      </c>
+      <c r="M35" s="27" t="n">
+        <v>2.5</v>
       </c>
       <c r="N35" s="28" t="n">
-        <v>0.390625</v>
+        <v>0.4</v>
       </c>
       <c r="O35" s="28" t="n">
         <v>0.688998</v>
       </c>
       <c r="P35" s="28" t="n"/>
       <c r="Q35" s="28" t="n">
-        <v>0.298373</v>
+        <v>0.288998</v>
       </c>
       <c r="R35" s="26" t="n">
         <v>100</v>
@@ -9888,15 +9857,15 @@
       <c r="V35" s="24" t="n"/>
       <c r="W35" s="26" t="n"/>
       <c r="X35" s="26" t="n"/>
-      <c r="Y35" s="38" t="n"/>
+      <c r="Y35" s="25" t="n"/>
       <c r="Z35" s="26" t="n"/>
       <c r="AA35" s="28" t="n"/>
       <c r="AB35" s="28" t="n"/>
-      <c r="AC35" s="40" t="n"/>
+      <c r="AC35" s="30" t="n"/>
       <c r="AD35" s="24" t="n"/>
       <c r="AE35" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.5051; executable ask 0.3900 (aec-wnba-ny-dal-2026-07-20).</t>
+          <t>Learned LR call at threshold 0.5051; executable ask 0.4000 (aec-wnba-ny-dal-2026-07-20).</t>
         </is>
       </c>
       <c r="AF35" s="31" t="inlineStr">
@@ -10015,7 +9984,7 @@
       </c>
       <c r="BH35" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T14:57:58.731031Z</t>
+          <t>2026-07-20T15:41:03.863692Z</t>
         </is>
       </c>
       <c r="BI35" s="24" t="inlineStr">
@@ -10023,32 +9992,2008 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ35" s="38" t="n"/>
+      <c r="BJ35" s="25" t="n"/>
       <c r="BK35" s="26" t="n">
-        <v>156</v>
-      </c>
-      <c r="BL35" s="39" t="n">
-        <v>2.56</v>
+        <v>150</v>
+      </c>
+      <c r="BL35" s="27" t="n">
+        <v>2.5</v>
       </c>
       <c r="BM35" s="28" t="n">
-        <v>0.390625</v>
+        <v>0.4</v>
       </c>
       <c r="BN35" s="28" t="n">
-        <v>0.386139</v>
+        <v>0.39604</v>
       </c>
       <c r="BO35" s="28" t="n"/>
-      <c r="BP35" s="38" t="n"/>
-      <c r="BQ35" s="39" t="n"/>
+      <c r="BP35" s="25" t="n"/>
+      <c r="BQ35" s="27" t="n"/>
       <c r="BR35" s="28" t="n"/>
       <c r="BS35" s="28" t="n"/>
       <c r="BT35" s="28" t="n"/>
-      <c r="BU35" s="38" t="n"/>
+      <c r="BU35" s="25" t="n"/>
       <c r="BV35" s="29" t="n"/>
       <c r="BW35" s="24" t="n"/>
-      <c r="BX35" s="40" t="n"/>
-      <c r="BY35" s="39" t="n"/>
+      <c r="BX35" s="30" t="n"/>
+      <c r="BY35" s="27" t="n"/>
       <c r="BZ35" s="24" t="n"/>
       <c r="CA35" s="31" t="n"/>
+    </row>
+    <row r="36" ht="36" customHeight="1">
+      <c r="A36" s="24" t="inlineStr">
+        <is>
+          <t>8a8477c2b92442e1</t>
+        </is>
+      </c>
+      <c r="B36" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T16:18:24.995882Z</t>
+        </is>
+      </c>
+      <c r="C36" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T20:00:00Z</t>
+        </is>
+      </c>
+      <c r="D36" s="24" t="inlineStr">
+        <is>
+          <t>54491</t>
+        </is>
+      </c>
+      <c r="E36" s="24" t="inlineStr">
+        <is>
+          <t>LOL</t>
+        </is>
+      </c>
+      <c r="F36" s="24" t="inlineStr">
+        <is>
+          <t>KaBuM! Ilha das Lendas</t>
+        </is>
+      </c>
+      <c r="G36" s="24" t="inlineStr">
+        <is>
+          <t>Vivo Keyd Stars Academy</t>
+        </is>
+      </c>
+      <c r="H36" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I36" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J36" s="25" t="n"/>
+      <c r="K36" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L36" s="26" t="n">
+        <v>144</v>
+      </c>
+      <c r="M36" s="27" t="n">
+        <v>2.44</v>
+      </c>
+      <c r="N36" s="28" t="n">
+        <v>0.409836</v>
+      </c>
+      <c r="O36" s="28" t="n">
+        <v>0.555003</v>
+      </c>
+      <c r="P36" s="28" t="n"/>
+      <c r="Q36" s="28" t="n">
+        <v>0.145003</v>
+      </c>
+      <c r="R36" s="26" t="n">
+        <v>100</v>
+      </c>
+      <c r="S36" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="T36" s="24" t="inlineStr">
+        <is>
+          <t>lol-neutral-series-elo-v1</t>
+        </is>
+      </c>
+      <c r="U36" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V36" s="24" t="n"/>
+      <c r="W36" s="26" t="n"/>
+      <c r="X36" s="26" t="n"/>
+      <c r="Y36" s="25" t="n"/>
+      <c r="Z36" s="26" t="n"/>
+      <c r="AA36" s="28" t="n"/>
+      <c r="AB36" s="28" t="n"/>
+      <c r="AC36" s="30" t="n"/>
+      <c r="AD36" s="24" t="n"/>
+      <c r="AE36" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.4100 (aec-lol-vksa-kbm-2026-07-20).</t>
+        </is>
+      </c>
+      <c r="AF36" s="31" t="inlineStr">
+        <is>
+          <t>Research baseline; zero-unit shadow until qualified.</t>
+        </is>
+      </c>
+      <c r="AG36" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH36" s="24" t="n"/>
+      <c r="AI36" s="31" t="n"/>
+      <c r="AJ36" s="31" t="n"/>
+      <c r="AK36" s="24" t="inlineStr">
+        <is>
+          <t>model_qualified</t>
+        </is>
+      </c>
+      <c r="AL36" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM36" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED_SHADOW_CALL</t>
+        </is>
+      </c>
+      <c r="AN36" s="24" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="AO36" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED</t>
+        </is>
+      </c>
+      <c r="AP36" s="24" t="inlineStr">
+        <is>
+          <t>KaBuM! Ilha das Lendas</t>
+        </is>
+      </c>
+      <c r="AQ36" s="24" t="inlineStr">
+        <is>
+          <t>KaBuM! Ilha das Lendas</t>
+        </is>
+      </c>
+      <c r="AR36" s="24" t="inlineStr">
+        <is>
+          <t>KaBuM! Ilha das Lendas</t>
+        </is>
+      </c>
+      <c r="AS36" s="24" t="inlineStr">
+        <is>
+          <t>Vivo Keyd Stars Academy</t>
+        </is>
+      </c>
+      <c r="AT36" s="24" t="inlineStr">
+        <is>
+          <t>Vivo Keyd Stars Academy</t>
+        </is>
+      </c>
+      <c r="AU36" s="24" t="inlineStr">
+        <is>
+          <t>Vivo Keyd Stars Academy</t>
+        </is>
+      </c>
+      <c r="AV36" s="24" t="n"/>
+      <c r="AW36" s="24" t="n"/>
+      <c r="AX36" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY36" s="24" t="n"/>
+      <c r="AZ36" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA36" s="24" t="inlineStr">
+        <is>
+          <t>1f56359bf30bb6d51629a345226e3008ebfe73210551f6db9f5ce09f656ffdd6</t>
+        </is>
+      </c>
+      <c r="BB36" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC36" s="24" t="inlineStr">
+        <is>
+          <t>lol-neutral-series-elo-v1</t>
+        </is>
+      </c>
+      <c r="BD36" s="24" t="inlineStr">
+        <is>
+          <t>1f56359bf30bb6d51629a345226e3008ebfe73210551f6db9f5ce09f656ffdd6</t>
+        </is>
+      </c>
+      <c r="BE36" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF36" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG36" s="24" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="BH36" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T16:18:24.995882Z</t>
+        </is>
+      </c>
+      <c r="BI36" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ36" s="25" t="n"/>
+      <c r="BK36" s="26" t="n">
+        <v>144</v>
+      </c>
+      <c r="BL36" s="27" t="n">
+        <v>2.44</v>
+      </c>
+      <c r="BM36" s="28" t="n">
+        <v>0.409836</v>
+      </c>
+      <c r="BN36" s="28" t="n"/>
+      <c r="BO36" s="28" t="n"/>
+      <c r="BP36" s="25" t="n"/>
+      <c r="BQ36" s="27" t="n"/>
+      <c r="BR36" s="28" t="n"/>
+      <c r="BS36" s="28" t="n"/>
+      <c r="BT36" s="28" t="n"/>
+      <c r="BU36" s="25" t="n"/>
+      <c r="BV36" s="29" t="n"/>
+      <c r="BW36" s="24" t="n"/>
+      <c r="BX36" s="30" t="n"/>
+      <c r="BY36" s="27" t="n"/>
+      <c r="BZ36" s="24" t="n"/>
+      <c r="CA36" s="31" t="n"/>
+    </row>
+    <row r="37" ht="36" customHeight="1">
+      <c r="A37" s="24" t="inlineStr">
+        <is>
+          <t>dc63682b755a4fc5</t>
+        </is>
+      </c>
+      <c r="B37" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T16:18:25.123725Z</t>
+        </is>
+      </c>
+      <c r="C37" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T21:00:00Z</t>
+        </is>
+      </c>
+      <c r="D37" s="24" t="inlineStr">
+        <is>
+          <t>54670</t>
+        </is>
+      </c>
+      <c r="E37" s="24" t="inlineStr">
+        <is>
+          <t>LOL</t>
+        </is>
+      </c>
+      <c r="F37" s="24" t="inlineStr">
+        <is>
+          <t>INTZ e-Sports</t>
+        </is>
+      </c>
+      <c r="G37" s="24" t="inlineStr">
+        <is>
+          <t>7REX</t>
+        </is>
+      </c>
+      <c r="H37" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I37" s="24" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="J37" s="25" t="n"/>
+      <c r="K37" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L37" s="26" t="n">
+        <v>186</v>
+      </c>
+      <c r="M37" s="27" t="n">
+        <v>2.86</v>
+      </c>
+      <c r="N37" s="28" t="n">
+        <v>0.34965</v>
+      </c>
+      <c r="O37" s="28" t="n">
+        <v>0.567918</v>
+      </c>
+      <c r="P37" s="28" t="n"/>
+      <c r="Q37" s="28" t="n">
+        <v>0.217918</v>
+      </c>
+      <c r="R37" s="26" t="n">
+        <v>100</v>
+      </c>
+      <c r="S37" s="29" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="T37" s="24" t="inlineStr">
+        <is>
+          <t>lol-neutral-series-elo-v1</t>
+        </is>
+      </c>
+      <c r="U37" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V37" s="24" t="n"/>
+      <c r="W37" s="26" t="n"/>
+      <c r="X37" s="26" t="n"/>
+      <c r="Y37" s="25" t="n"/>
+      <c r="Z37" s="26" t="n"/>
+      <c r="AA37" s="28" t="n"/>
+      <c r="AB37" s="28" t="n"/>
+      <c r="AC37" s="30" t="n"/>
+      <c r="AD37" s="24" t="n"/>
+      <c r="AE37" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.3500 (aec-lol-itz-7rex-2026-07-20).</t>
+        </is>
+      </c>
+      <c r="AF37" s="31" t="inlineStr">
+        <is>
+          <t>Research baseline; zero-unit shadow until qualified.</t>
+        </is>
+      </c>
+      <c r="AG37" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH37" s="24" t="n"/>
+      <c r="AI37" s="31" t="n"/>
+      <c r="AJ37" s="31" t="n"/>
+      <c r="AK37" s="24" t="inlineStr">
+        <is>
+          <t>model_qualified</t>
+        </is>
+      </c>
+      <c r="AL37" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM37" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED_SHADOW_CALL</t>
+        </is>
+      </c>
+      <c r="AN37" s="24" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="AO37" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED</t>
+        </is>
+      </c>
+      <c r="AP37" s="24" t="inlineStr">
+        <is>
+          <t>INTZ e-Sports</t>
+        </is>
+      </c>
+      <c r="AQ37" s="24" t="inlineStr">
+        <is>
+          <t>INTZ e-Sports</t>
+        </is>
+      </c>
+      <c r="AR37" s="24" t="inlineStr">
+        <is>
+          <t>INTZ e-Sports</t>
+        </is>
+      </c>
+      <c r="AS37" s="24" t="inlineStr">
+        <is>
+          <t>7REX</t>
+        </is>
+      </c>
+      <c r="AT37" s="24" t="inlineStr">
+        <is>
+          <t>7REX</t>
+        </is>
+      </c>
+      <c r="AU37" s="24" t="inlineStr">
+        <is>
+          <t>7REX</t>
+        </is>
+      </c>
+      <c r="AV37" s="24" t="n"/>
+      <c r="AW37" s="24" t="n"/>
+      <c r="AX37" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY37" s="24" t="n"/>
+      <c r="AZ37" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA37" s="24" t="inlineStr">
+        <is>
+          <t>1f56359bf30bb6d51629a345226e3008ebfe73210551f6db9f5ce09f656ffdd6</t>
+        </is>
+      </c>
+      <c r="BB37" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC37" s="24" t="inlineStr">
+        <is>
+          <t>lol-neutral-series-elo-v1</t>
+        </is>
+      </c>
+      <c r="BD37" s="24" t="inlineStr">
+        <is>
+          <t>1f56359bf30bb6d51629a345226e3008ebfe73210551f6db9f5ce09f656ffdd6</t>
+        </is>
+      </c>
+      <c r="BE37" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF37" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG37" s="24" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="BH37" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T16:18:25.123725Z</t>
+        </is>
+      </c>
+      <c r="BI37" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ37" s="25" t="n"/>
+      <c r="BK37" s="26" t="n">
+        <v>186</v>
+      </c>
+      <c r="BL37" s="27" t="n">
+        <v>2.86</v>
+      </c>
+      <c r="BM37" s="28" t="n">
+        <v>0.34965</v>
+      </c>
+      <c r="BN37" s="28" t="n"/>
+      <c r="BO37" s="28" t="n"/>
+      <c r="BP37" s="25" t="n"/>
+      <c r="BQ37" s="27" t="n"/>
+      <c r="BR37" s="28" t="n"/>
+      <c r="BS37" s="28" t="n"/>
+      <c r="BT37" s="28" t="n"/>
+      <c r="BU37" s="25" t="n"/>
+      <c r="BV37" s="29" t="n"/>
+      <c r="BW37" s="24" t="n"/>
+      <c r="BX37" s="30" t="n"/>
+      <c r="BY37" s="27" t="n"/>
+      <c r="BZ37" s="24" t="n"/>
+      <c r="CA37" s="31" t="n"/>
+    </row>
+    <row r="38" ht="36" customHeight="1">
+      <c r="A38" s="24" t="inlineStr">
+        <is>
+          <t>36b26e06b0c0460a</t>
+        </is>
+      </c>
+      <c r="B38" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T16:18:25.218065Z</t>
+        </is>
+      </c>
+      <c r="C38" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T22:00:00Z</t>
+        </is>
+      </c>
+      <c r="D38" s="24" t="inlineStr">
+        <is>
+          <t>54693</t>
+        </is>
+      </c>
+      <c r="E38" s="24" t="inlineStr">
+        <is>
+          <t>LOL</t>
+        </is>
+      </c>
+      <c r="F38" s="24" t="inlineStr">
+        <is>
+          <t>Ei Nerd Esports</t>
+        </is>
+      </c>
+      <c r="G38" s="24" t="inlineStr">
+        <is>
+          <t>RED Academy</t>
+        </is>
+      </c>
+      <c r="H38" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I38" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J38" s="25" t="n"/>
+      <c r="K38" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L38" s="26" t="n">
+        <v>300</v>
+      </c>
+      <c r="M38" s="27" t="n">
+        <v>4</v>
+      </c>
+      <c r="N38" s="28" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="O38" s="28" t="n">
+        <v>0.674654</v>
+      </c>
+      <c r="P38" s="28" t="n"/>
+      <c r="Q38" s="28" t="n">
+        <v>0.424654</v>
+      </c>
+      <c r="R38" s="26" t="n">
+        <v>100</v>
+      </c>
+      <c r="S38" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="T38" s="24" t="inlineStr">
+        <is>
+          <t>lol-neutral-series-elo-v1</t>
+        </is>
+      </c>
+      <c r="U38" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V38" s="24" t="n"/>
+      <c r="W38" s="26" t="n"/>
+      <c r="X38" s="26" t="n"/>
+      <c r="Y38" s="25" t="n"/>
+      <c r="Z38" s="26" t="n"/>
+      <c r="AA38" s="28" t="n"/>
+      <c r="AB38" s="28" t="n"/>
+      <c r="AC38" s="30" t="n"/>
+      <c r="AD38" s="24" t="n"/>
+      <c r="AE38" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.2500 (aec-lol-reda-nerd-2026-07-20).</t>
+        </is>
+      </c>
+      <c r="AF38" s="31" t="inlineStr">
+        <is>
+          <t>Research baseline; zero-unit shadow until qualified.</t>
+        </is>
+      </c>
+      <c r="AG38" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH38" s="24" t="n"/>
+      <c r="AI38" s="31" t="n"/>
+      <c r="AJ38" s="31" t="n"/>
+      <c r="AK38" s="24" t="inlineStr">
+        <is>
+          <t>model_qualified</t>
+        </is>
+      </c>
+      <c r="AL38" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM38" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED_SHADOW_CALL</t>
+        </is>
+      </c>
+      <c r="AN38" s="24" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="AO38" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED</t>
+        </is>
+      </c>
+      <c r="AP38" s="24" t="inlineStr">
+        <is>
+          <t>Ei Nerd Esports</t>
+        </is>
+      </c>
+      <c r="AQ38" s="24" t="inlineStr">
+        <is>
+          <t>Ei Nerd Esports</t>
+        </is>
+      </c>
+      <c r="AR38" s="24" t="inlineStr">
+        <is>
+          <t>Ei Nerd Esports</t>
+        </is>
+      </c>
+      <c r="AS38" s="24" t="inlineStr">
+        <is>
+          <t>RED Academy</t>
+        </is>
+      </c>
+      <c r="AT38" s="24" t="inlineStr">
+        <is>
+          <t>RED Academy</t>
+        </is>
+      </c>
+      <c r="AU38" s="24" t="inlineStr">
+        <is>
+          <t>RED Academy</t>
+        </is>
+      </c>
+      <c r="AV38" s="24" t="n"/>
+      <c r="AW38" s="24" t="n"/>
+      <c r="AX38" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY38" s="24" t="n"/>
+      <c r="AZ38" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA38" s="24" t="inlineStr">
+        <is>
+          <t>1f56359bf30bb6d51629a345226e3008ebfe73210551f6db9f5ce09f656ffdd6</t>
+        </is>
+      </c>
+      <c r="BB38" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC38" s="24" t="inlineStr">
+        <is>
+          <t>lol-neutral-series-elo-v1</t>
+        </is>
+      </c>
+      <c r="BD38" s="24" t="inlineStr">
+        <is>
+          <t>1f56359bf30bb6d51629a345226e3008ebfe73210551f6db9f5ce09f656ffdd6</t>
+        </is>
+      </c>
+      <c r="BE38" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF38" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG38" s="24" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="BH38" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T16:18:25.218065Z</t>
+        </is>
+      </c>
+      <c r="BI38" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ38" s="25" t="n"/>
+      <c r="BK38" s="26" t="n">
+        <v>300</v>
+      </c>
+      <c r="BL38" s="27" t="n">
+        <v>4</v>
+      </c>
+      <c r="BM38" s="28" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="BN38" s="28" t="n"/>
+      <c r="BO38" s="28" t="n"/>
+      <c r="BP38" s="25" t="n"/>
+      <c r="BQ38" s="27" t="n"/>
+      <c r="BR38" s="28" t="n"/>
+      <c r="BS38" s="28" t="n"/>
+      <c r="BT38" s="28" t="n"/>
+      <c r="BU38" s="25" t="n"/>
+      <c r="BV38" s="29" t="n"/>
+      <c r="BW38" s="24" t="n"/>
+      <c r="BX38" s="30" t="n"/>
+      <c r="BY38" s="27" t="n"/>
+      <c r="BZ38" s="24" t="n"/>
+      <c r="CA38" s="31" t="n"/>
+    </row>
+    <row r="39" ht="36" customHeight="1">
+      <c r="A39" s="24" t="inlineStr">
+        <is>
+          <t>a72da5dc37704076</t>
+        </is>
+      </c>
+      <c r="B39" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T16:18:25.312075Z</t>
+        </is>
+      </c>
+      <c r="C39" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-21T00:00:00Z</t>
+        </is>
+      </c>
+      <c r="D39" s="24" t="inlineStr">
+        <is>
+          <t>54745</t>
+        </is>
+      </c>
+      <c r="E39" s="24" t="inlineStr">
+        <is>
+          <t>LOL</t>
+        </is>
+      </c>
+      <c r="F39" s="24" t="inlineStr">
+        <is>
+          <t>Estral Esports</t>
+        </is>
+      </c>
+      <c r="G39" s="24" t="inlineStr">
+        <is>
+          <t>paiN Gaming Academy</t>
+        </is>
+      </c>
+      <c r="H39" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I39" s="24" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="J39" s="25" t="n"/>
+      <c r="K39" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L39" s="26" t="n">
+        <v>245</v>
+      </c>
+      <c r="M39" s="27" t="n">
+        <v>3.45</v>
+      </c>
+      <c r="N39" s="28" t="n">
+        <v>0.289855</v>
+      </c>
+      <c r="O39" s="28" t="n">
+        <v>0.586418</v>
+      </c>
+      <c r="P39" s="28" t="n"/>
+      <c r="Q39" s="28" t="n">
+        <v>0.296418</v>
+      </c>
+      <c r="R39" s="26" t="n">
+        <v>100</v>
+      </c>
+      <c r="S39" s="29" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="T39" s="24" t="inlineStr">
+        <is>
+          <t>lol-neutral-series-elo-v1</t>
+        </is>
+      </c>
+      <c r="U39" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V39" s="24" t="n"/>
+      <c r="W39" s="26" t="n"/>
+      <c r="X39" s="26" t="n"/>
+      <c r="Y39" s="25" t="n"/>
+      <c r="Z39" s="26" t="n"/>
+      <c r="AA39" s="28" t="n"/>
+      <c r="AB39" s="28" t="n"/>
+      <c r="AC39" s="30" t="n"/>
+      <c r="AD39" s="24" t="n"/>
+      <c r="AE39" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.2900 (aec-lol-est-pnga-2026-07-21).</t>
+        </is>
+      </c>
+      <c r="AF39" s="31" t="inlineStr">
+        <is>
+          <t>Research baseline; zero-unit shadow until qualified.</t>
+        </is>
+      </c>
+      <c r="AG39" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH39" s="24" t="n"/>
+      <c r="AI39" s="31" t="n"/>
+      <c r="AJ39" s="31" t="n"/>
+      <c r="AK39" s="24" t="inlineStr">
+        <is>
+          <t>model_qualified</t>
+        </is>
+      </c>
+      <c r="AL39" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM39" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED_SHADOW_CALL</t>
+        </is>
+      </c>
+      <c r="AN39" s="24" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="AO39" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED</t>
+        </is>
+      </c>
+      <c r="AP39" s="24" t="inlineStr">
+        <is>
+          <t>Estral Esports</t>
+        </is>
+      </c>
+      <c r="AQ39" s="24" t="inlineStr">
+        <is>
+          <t>Estral Esports</t>
+        </is>
+      </c>
+      <c r="AR39" s="24" t="inlineStr">
+        <is>
+          <t>Estral Esports</t>
+        </is>
+      </c>
+      <c r="AS39" s="24" t="inlineStr">
+        <is>
+          <t>paiN Gaming Academy</t>
+        </is>
+      </c>
+      <c r="AT39" s="24" t="inlineStr">
+        <is>
+          <t>paiN Gaming Academy</t>
+        </is>
+      </c>
+      <c r="AU39" s="24" t="inlineStr">
+        <is>
+          <t>paiN Gaming Academy</t>
+        </is>
+      </c>
+      <c r="AV39" s="24" t="n"/>
+      <c r="AW39" s="24" t="n"/>
+      <c r="AX39" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY39" s="24" t="n"/>
+      <c r="AZ39" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA39" s="24" t="inlineStr">
+        <is>
+          <t>1f56359bf30bb6d51629a345226e3008ebfe73210551f6db9f5ce09f656ffdd6</t>
+        </is>
+      </c>
+      <c r="BB39" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC39" s="24" t="inlineStr">
+        <is>
+          <t>lol-neutral-series-elo-v1</t>
+        </is>
+      </c>
+      <c r="BD39" s="24" t="inlineStr">
+        <is>
+          <t>1f56359bf30bb6d51629a345226e3008ebfe73210551f6db9f5ce09f656ffdd6</t>
+        </is>
+      </c>
+      <c r="BE39" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF39" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG39" s="24" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="BH39" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T16:18:25.312075Z</t>
+        </is>
+      </c>
+      <c r="BI39" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ39" s="25" t="n"/>
+      <c r="BK39" s="26" t="n">
+        <v>245</v>
+      </c>
+      <c r="BL39" s="27" t="n">
+        <v>3.45</v>
+      </c>
+      <c r="BM39" s="28" t="n">
+        <v>0.289855</v>
+      </c>
+      <c r="BN39" s="28" t="n"/>
+      <c r="BO39" s="28" t="n"/>
+      <c r="BP39" s="25" t="n"/>
+      <c r="BQ39" s="27" t="n"/>
+      <c r="BR39" s="28" t="n"/>
+      <c r="BS39" s="28" t="n"/>
+      <c r="BT39" s="28" t="n"/>
+      <c r="BU39" s="25" t="n"/>
+      <c r="BV39" s="29" t="n"/>
+      <c r="BW39" s="24" t="n"/>
+      <c r="BX39" s="30" t="n"/>
+      <c r="BY39" s="27" t="n"/>
+      <c r="BZ39" s="24" t="n"/>
+      <c r="CA39" s="31" t="n"/>
+    </row>
+    <row r="40" ht="36" customHeight="1">
+      <c r="A40" s="24" t="inlineStr">
+        <is>
+          <t>66a67a653fb14bd2</t>
+        </is>
+      </c>
+      <c r="B40" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T16:26:22.811500Z</t>
+        </is>
+      </c>
+      <c r="C40" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T17:00:00Z</t>
+        </is>
+      </c>
+      <c r="D40" s="24" t="inlineStr">
+        <is>
+          <t>56113</t>
+        </is>
+      </c>
+      <c r="E40" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F40" s="24" t="inlineStr">
+        <is>
+          <t>Inner Circle Academy</t>
+        </is>
+      </c>
+      <c r="G40" s="24" t="inlineStr">
+        <is>
+          <t>Endless Journey</t>
+        </is>
+      </c>
+      <c r="H40" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I40" s="24" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="J40" s="25" t="n"/>
+      <c r="K40" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L40" s="26" t="n">
+        <v>-113</v>
+      </c>
+      <c r="M40" s="27" t="n">
+        <v>1.884956</v>
+      </c>
+      <c r="N40" s="28" t="n">
+        <v>0.530516</v>
+      </c>
+      <c r="O40" s="28" t="n">
+        <v>0.652434</v>
+      </c>
+      <c r="P40" s="28" t="n"/>
+      <c r="Q40" s="28" t="n">
+        <v>0.122434</v>
+      </c>
+      <c r="R40" s="26" t="n">
+        <v>100</v>
+      </c>
+      <c r="S40" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="T40" s="24" t="inlineStr">
+        <is>
+          <t>cs2-neutral-series-elo-v1</t>
+        </is>
+      </c>
+      <c r="U40" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V40" s="24" t="n"/>
+      <c r="W40" s="26" t="n"/>
+      <c r="X40" s="26" t="n"/>
+      <c r="Y40" s="25" t="n"/>
+      <c r="Z40" s="26" t="n"/>
+      <c r="AA40" s="28" t="n"/>
+      <c r="AB40" s="28" t="n"/>
+      <c r="AC40" s="30" t="n"/>
+      <c r="AD40" s="24" t="n"/>
+      <c r="AE40" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.5300 (aec-cs2-ica-ej-2026-07-20).</t>
+        </is>
+      </c>
+      <c r="AF40" s="31" t="inlineStr">
+        <is>
+          <t>Research baseline; zero-unit shadow until qualified.</t>
+        </is>
+      </c>
+      <c r="AG40" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH40" s="24" t="n"/>
+      <c r="AI40" s="31" t="n"/>
+      <c r="AJ40" s="31" t="n"/>
+      <c r="AK40" s="24" t="inlineStr">
+        <is>
+          <t>model_qualified</t>
+        </is>
+      </c>
+      <c r="AL40" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM40" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED_SHADOW_CALL</t>
+        </is>
+      </c>
+      <c r="AN40" s="24" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="AO40" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED</t>
+        </is>
+      </c>
+      <c r="AP40" s="24" t="inlineStr">
+        <is>
+          <t>Inner Circle Academy</t>
+        </is>
+      </c>
+      <c r="AQ40" s="24" t="inlineStr">
+        <is>
+          <t>Inner Circle Academy</t>
+        </is>
+      </c>
+      <c r="AR40" s="24" t="inlineStr">
+        <is>
+          <t>Inner Circle Academy</t>
+        </is>
+      </c>
+      <c r="AS40" s="24" t="inlineStr">
+        <is>
+          <t>Endless Journey</t>
+        </is>
+      </c>
+      <c r="AT40" s="24" t="inlineStr">
+        <is>
+          <t>Endless Journey</t>
+        </is>
+      </c>
+      <c r="AU40" s="24" t="inlineStr">
+        <is>
+          <t>Endless Journey</t>
+        </is>
+      </c>
+      <c r="AV40" s="24" t="n"/>
+      <c r="AW40" s="24" t="n"/>
+      <c r="AX40" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY40" s="24" t="n"/>
+      <c r="AZ40" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA40" s="24" t="inlineStr">
+        <is>
+          <t>40df7f7b9128e86cfbc485914f5801a00963b62604711b733b60f782ba9e258b</t>
+        </is>
+      </c>
+      <c r="BB40" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC40" s="24" t="inlineStr">
+        <is>
+          <t>cs2-neutral-series-elo-v1</t>
+        </is>
+      </c>
+      <c r="BD40" s="24" t="inlineStr">
+        <is>
+          <t>40df7f7b9128e86cfbc485914f5801a00963b62604711b733b60f782ba9e258b</t>
+        </is>
+      </c>
+      <c r="BE40" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF40" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG40" s="24" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="BH40" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T16:26:22.811500Z</t>
+        </is>
+      </c>
+      <c r="BI40" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ40" s="25" t="n"/>
+      <c r="BK40" s="26" t="n">
+        <v>-113</v>
+      </c>
+      <c r="BL40" s="27" t="n">
+        <v>1.884956</v>
+      </c>
+      <c r="BM40" s="28" t="n">
+        <v>0.530516</v>
+      </c>
+      <c r="BN40" s="28" t="n"/>
+      <c r="BO40" s="28" t="n"/>
+      <c r="BP40" s="25" t="n"/>
+      <c r="BQ40" s="27" t="n"/>
+      <c r="BR40" s="28" t="n"/>
+      <c r="BS40" s="28" t="n"/>
+      <c r="BT40" s="28" t="n"/>
+      <c r="BU40" s="25" t="n"/>
+      <c r="BV40" s="29" t="n"/>
+      <c r="BW40" s="24" t="n"/>
+      <c r="BX40" s="30" t="n"/>
+      <c r="BY40" s="27" t="n"/>
+      <c r="BZ40" s="24" t="n"/>
+      <c r="CA40" s="31" t="n"/>
+    </row>
+    <row r="41" ht="36" customHeight="1">
+      <c r="A41" s="24" t="inlineStr">
+        <is>
+          <t>a75a7af91f614c77</t>
+        </is>
+      </c>
+      <c r="B41" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T16:26:22.946543Z</t>
+        </is>
+      </c>
+      <c r="C41" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T19:00:00Z</t>
+        </is>
+      </c>
+      <c r="D41" s="24" t="inlineStr">
+        <is>
+          <t>56757</t>
+        </is>
+      </c>
+      <c r="E41" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F41" s="24" t="inlineStr">
+        <is>
+          <t>MAGICOS</t>
+        </is>
+      </c>
+      <c r="G41" s="24" t="inlineStr">
+        <is>
+          <t>Blitzkrieg</t>
+        </is>
+      </c>
+      <c r="H41" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I41" s="24" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="J41" s="25" t="n"/>
+      <c r="K41" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L41" s="26" t="n">
+        <v>669</v>
+      </c>
+      <c r="M41" s="27" t="n">
+        <v>7.69</v>
+      </c>
+      <c r="N41" s="28" t="n">
+        <v>0.130039</v>
+      </c>
+      <c r="O41" s="28" t="n">
+        <v>0.598244</v>
+      </c>
+      <c r="P41" s="28" t="n"/>
+      <c r="Q41" s="28" t="n">
+        <v>0.468244</v>
+      </c>
+      <c r="R41" s="26" t="n">
+        <v>100</v>
+      </c>
+      <c r="S41" s="29" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="T41" s="24" t="inlineStr">
+        <is>
+          <t>cs2-neutral-series-elo-v1</t>
+        </is>
+      </c>
+      <c r="U41" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V41" s="24" t="n"/>
+      <c r="W41" s="26" t="n"/>
+      <c r="X41" s="26" t="n"/>
+      <c r="Y41" s="25" t="n"/>
+      <c r="Z41" s="26" t="n"/>
+      <c r="AA41" s="28" t="n"/>
+      <c r="AB41" s="28" t="n"/>
+      <c r="AC41" s="30" t="n"/>
+      <c r="AD41" s="24" t="n"/>
+      <c r="AE41" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.1300 (aec-cs2-mag-bk-2026-07-20).</t>
+        </is>
+      </c>
+      <c r="AF41" s="31" t="inlineStr">
+        <is>
+          <t>Research baseline; zero-unit shadow until qualified.</t>
+        </is>
+      </c>
+      <c r="AG41" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH41" s="24" t="n"/>
+      <c r="AI41" s="31" t="n"/>
+      <c r="AJ41" s="31" t="n"/>
+      <c r="AK41" s="24" t="inlineStr">
+        <is>
+          <t>model_qualified</t>
+        </is>
+      </c>
+      <c r="AL41" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM41" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED_SHADOW_CALL</t>
+        </is>
+      </c>
+      <c r="AN41" s="24" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="AO41" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED</t>
+        </is>
+      </c>
+      <c r="AP41" s="24" t="inlineStr">
+        <is>
+          <t>MAGICOS</t>
+        </is>
+      </c>
+      <c r="AQ41" s="24" t="inlineStr">
+        <is>
+          <t>MAGICOS</t>
+        </is>
+      </c>
+      <c r="AR41" s="24" t="inlineStr">
+        <is>
+          <t>MAGICOS</t>
+        </is>
+      </c>
+      <c r="AS41" s="24" t="inlineStr">
+        <is>
+          <t>Blitzkrieg</t>
+        </is>
+      </c>
+      <c r="AT41" s="24" t="inlineStr">
+        <is>
+          <t>Blitzkrieg</t>
+        </is>
+      </c>
+      <c r="AU41" s="24" t="inlineStr">
+        <is>
+          <t>Blitzkrieg</t>
+        </is>
+      </c>
+      <c r="AV41" s="24" t="n"/>
+      <c r="AW41" s="24" t="n"/>
+      <c r="AX41" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY41" s="24" t="n"/>
+      <c r="AZ41" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA41" s="24" t="inlineStr">
+        <is>
+          <t>40df7f7b9128e86cfbc485914f5801a00963b62604711b733b60f782ba9e258b</t>
+        </is>
+      </c>
+      <c r="BB41" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC41" s="24" t="inlineStr">
+        <is>
+          <t>cs2-neutral-series-elo-v1</t>
+        </is>
+      </c>
+      <c r="BD41" s="24" t="inlineStr">
+        <is>
+          <t>40df7f7b9128e86cfbc485914f5801a00963b62604711b733b60f782ba9e258b</t>
+        </is>
+      </c>
+      <c r="BE41" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF41" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG41" s="24" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="BH41" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T16:26:22.946543Z</t>
+        </is>
+      </c>
+      <c r="BI41" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ41" s="25" t="n"/>
+      <c r="BK41" s="26" t="n">
+        <v>669</v>
+      </c>
+      <c r="BL41" s="27" t="n">
+        <v>7.69</v>
+      </c>
+      <c r="BM41" s="28" t="n">
+        <v>0.130039</v>
+      </c>
+      <c r="BN41" s="28" t="n"/>
+      <c r="BO41" s="28" t="n"/>
+      <c r="BP41" s="25" t="n"/>
+      <c r="BQ41" s="27" t="n"/>
+      <c r="BR41" s="28" t="n"/>
+      <c r="BS41" s="28" t="n"/>
+      <c r="BT41" s="28" t="n"/>
+      <c r="BU41" s="25" t="n"/>
+      <c r="BV41" s="29" t="n"/>
+      <c r="BW41" s="24" t="n"/>
+      <c r="BX41" s="30" t="n"/>
+      <c r="BY41" s="27" t="n"/>
+      <c r="BZ41" s="24" t="n"/>
+      <c r="CA41" s="31" t="n"/>
+    </row>
+    <row r="42" ht="36" customHeight="1">
+      <c r="A42" s="24" t="inlineStr">
+        <is>
+          <t>8a3b3559571c4133</t>
+        </is>
+      </c>
+      <c r="B42" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T16:26:23.050406Z</t>
+        </is>
+      </c>
+      <c r="C42" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T19:00:00Z</t>
+        </is>
+      </c>
+      <c r="D42" s="24" t="inlineStr">
+        <is>
+          <t>54667</t>
+        </is>
+      </c>
+      <c r="E42" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F42" s="24" t="inlineStr">
+        <is>
+          <t>paiN Academy</t>
+        </is>
+      </c>
+      <c r="G42" s="24" t="inlineStr">
+        <is>
+          <t>HATERS</t>
+        </is>
+      </c>
+      <c r="H42" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I42" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J42" s="25" t="n"/>
+      <c r="K42" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L42" s="26" t="n">
+        <v>335</v>
+      </c>
+      <c r="M42" s="27" t="n">
+        <v>4.35</v>
+      </c>
+      <c r="N42" s="28" t="n">
+        <v>0.229885</v>
+      </c>
+      <c r="O42" s="28" t="n">
+        <v>0.558097</v>
+      </c>
+      <c r="P42" s="28" t="n"/>
+      <c r="Q42" s="28" t="n">
+        <v>0.328097</v>
+      </c>
+      <c r="R42" s="26" t="n">
+        <v>100</v>
+      </c>
+      <c r="S42" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="T42" s="24" t="inlineStr">
+        <is>
+          <t>cs2-neutral-series-elo-v1</t>
+        </is>
+      </c>
+      <c r="U42" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V42" s="24" t="n"/>
+      <c r="W42" s="26" t="n"/>
+      <c r="X42" s="26" t="n"/>
+      <c r="Y42" s="25" t="n"/>
+      <c r="Z42" s="26" t="n"/>
+      <c r="AA42" s="28" t="n"/>
+      <c r="AB42" s="28" t="n"/>
+      <c r="AC42" s="30" t="n"/>
+      <c r="AD42" s="24" t="n"/>
+      <c r="AE42" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.2300 (aec-cs2-hat-paina-2026-07-20).</t>
+        </is>
+      </c>
+      <c r="AF42" s="31" t="inlineStr">
+        <is>
+          <t>Research baseline; zero-unit shadow until qualified.</t>
+        </is>
+      </c>
+      <c r="AG42" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH42" s="24" t="n"/>
+      <c r="AI42" s="31" t="n"/>
+      <c r="AJ42" s="31" t="n"/>
+      <c r="AK42" s="24" t="inlineStr">
+        <is>
+          <t>model_qualified</t>
+        </is>
+      </c>
+      <c r="AL42" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM42" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED_SHADOW_CALL</t>
+        </is>
+      </c>
+      <c r="AN42" s="24" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="AO42" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED</t>
+        </is>
+      </c>
+      <c r="AP42" s="24" t="inlineStr">
+        <is>
+          <t>paiN Academy</t>
+        </is>
+      </c>
+      <c r="AQ42" s="24" t="inlineStr">
+        <is>
+          <t>paiN Academy</t>
+        </is>
+      </c>
+      <c r="AR42" s="24" t="inlineStr">
+        <is>
+          <t>paiN Academy</t>
+        </is>
+      </c>
+      <c r="AS42" s="24" t="inlineStr">
+        <is>
+          <t>HATERS</t>
+        </is>
+      </c>
+      <c r="AT42" s="24" t="inlineStr">
+        <is>
+          <t>HATERS</t>
+        </is>
+      </c>
+      <c r="AU42" s="24" t="inlineStr">
+        <is>
+          <t>HATERS</t>
+        </is>
+      </c>
+      <c r="AV42" s="24" t="n"/>
+      <c r="AW42" s="24" t="n"/>
+      <c r="AX42" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY42" s="24" t="n"/>
+      <c r="AZ42" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA42" s="24" t="inlineStr">
+        <is>
+          <t>40df7f7b9128e86cfbc485914f5801a00963b62604711b733b60f782ba9e258b</t>
+        </is>
+      </c>
+      <c r="BB42" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC42" s="24" t="inlineStr">
+        <is>
+          <t>cs2-neutral-series-elo-v1</t>
+        </is>
+      </c>
+      <c r="BD42" s="24" t="inlineStr">
+        <is>
+          <t>40df7f7b9128e86cfbc485914f5801a00963b62604711b733b60f782ba9e258b</t>
+        </is>
+      </c>
+      <c r="BE42" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF42" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG42" s="24" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="BH42" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T16:26:23.050406Z</t>
+        </is>
+      </c>
+      <c r="BI42" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ42" s="25" t="n"/>
+      <c r="BK42" s="26" t="n">
+        <v>335</v>
+      </c>
+      <c r="BL42" s="27" t="n">
+        <v>4.35</v>
+      </c>
+      <c r="BM42" s="28" t="n">
+        <v>0.229885</v>
+      </c>
+      <c r="BN42" s="28" t="n"/>
+      <c r="BO42" s="28" t="n"/>
+      <c r="BP42" s="25" t="n"/>
+      <c r="BQ42" s="27" t="n"/>
+      <c r="BR42" s="28" t="n"/>
+      <c r="BS42" s="28" t="n"/>
+      <c r="BT42" s="28" t="n"/>
+      <c r="BU42" s="25" t="n"/>
+      <c r="BV42" s="29" t="n"/>
+      <c r="BW42" s="24" t="n"/>
+      <c r="BX42" s="30" t="n"/>
+      <c r="BY42" s="27" t="n"/>
+      <c r="BZ42" s="24" t="n"/>
+      <c r="CA42" s="31" t="n"/>
+    </row>
+    <row r="43" ht="36" customHeight="1">
+      <c r="A43" s="24" t="inlineStr">
+        <is>
+          <t>5417c8a3e89a4c9f</t>
+        </is>
+      </c>
+      <c r="B43" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T16:26:23.154839Z</t>
+        </is>
+      </c>
+      <c r="C43" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T21:00:00Z</t>
+        </is>
+      </c>
+      <c r="D43" s="24" t="inlineStr">
+        <is>
+          <t>54672</t>
+        </is>
+      </c>
+      <c r="E43" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F43" s="24" t="inlineStr">
+        <is>
+          <t>METANOIA WOLVES</t>
+        </is>
+      </c>
+      <c r="G43" s="24" t="inlineStr">
+        <is>
+          <t>RED Canids Academy</t>
+        </is>
+      </c>
+      <c r="H43" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I43" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J43" s="25" t="n"/>
+      <c r="K43" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L43" s="26" t="n">
+        <v>-144</v>
+      </c>
+      <c r="M43" s="27" t="n">
+        <v>1.694444</v>
+      </c>
+      <c r="N43" s="28" t="n">
+        <v>0.590164</v>
+      </c>
+      <c r="O43" s="28" t="n">
+        <v>0.885084</v>
+      </c>
+      <c r="P43" s="28" t="n"/>
+      <c r="Q43" s="28" t="n">
+        <v>0.295084</v>
+      </c>
+      <c r="R43" s="26" t="n">
+        <v>100</v>
+      </c>
+      <c r="S43" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="T43" s="24" t="inlineStr">
+        <is>
+          <t>cs2-neutral-series-elo-v1</t>
+        </is>
+      </c>
+      <c r="U43" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V43" s="24" t="n"/>
+      <c r="W43" s="26" t="n"/>
+      <c r="X43" s="26" t="n"/>
+      <c r="Y43" s="25" t="n"/>
+      <c r="Z43" s="26" t="n"/>
+      <c r="AA43" s="28" t="n"/>
+      <c r="AB43" s="28" t="n"/>
+      <c r="AC43" s="30" t="n"/>
+      <c r="AD43" s="24" t="n"/>
+      <c r="AE43" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.5900 (aec-cs2-reda-mw-2026-07-20).</t>
+        </is>
+      </c>
+      <c r="AF43" s="31" t="inlineStr">
+        <is>
+          <t>Research baseline; zero-unit shadow until qualified.</t>
+        </is>
+      </c>
+      <c r="AG43" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH43" s="24" t="n"/>
+      <c r="AI43" s="31" t="n"/>
+      <c r="AJ43" s="31" t="n"/>
+      <c r="AK43" s="24" t="inlineStr">
+        <is>
+          <t>model_qualified</t>
+        </is>
+      </c>
+      <c r="AL43" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM43" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED_SHADOW_CALL</t>
+        </is>
+      </c>
+      <c r="AN43" s="24" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="AO43" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED</t>
+        </is>
+      </c>
+      <c r="AP43" s="24" t="inlineStr">
+        <is>
+          <t>METANOIA WOLVES</t>
+        </is>
+      </c>
+      <c r="AQ43" s="24" t="inlineStr">
+        <is>
+          <t>METANOIA WOLVES</t>
+        </is>
+      </c>
+      <c r="AR43" s="24" t="inlineStr">
+        <is>
+          <t>METANOIA WOLVES</t>
+        </is>
+      </c>
+      <c r="AS43" s="24" t="inlineStr">
+        <is>
+          <t>RED Canids Academy</t>
+        </is>
+      </c>
+      <c r="AT43" s="24" t="inlineStr">
+        <is>
+          <t>RED Canids Academy</t>
+        </is>
+      </c>
+      <c r="AU43" s="24" t="inlineStr">
+        <is>
+          <t>RED Canids Academy</t>
+        </is>
+      </c>
+      <c r="AV43" s="24" t="n"/>
+      <c r="AW43" s="24" t="n"/>
+      <c r="AX43" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY43" s="24" t="n"/>
+      <c r="AZ43" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA43" s="24" t="inlineStr">
+        <is>
+          <t>40df7f7b9128e86cfbc485914f5801a00963b62604711b733b60f782ba9e258b</t>
+        </is>
+      </c>
+      <c r="BB43" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC43" s="24" t="inlineStr">
+        <is>
+          <t>cs2-neutral-series-elo-v1</t>
+        </is>
+      </c>
+      <c r="BD43" s="24" t="inlineStr">
+        <is>
+          <t>40df7f7b9128e86cfbc485914f5801a00963b62604711b733b60f782ba9e258b</t>
+        </is>
+      </c>
+      <c r="BE43" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF43" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG43" s="24" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="BH43" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-20T16:26:23.154839Z</t>
+        </is>
+      </c>
+      <c r="BI43" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ43" s="25" t="n"/>
+      <c r="BK43" s="26" t="n">
+        <v>-144</v>
+      </c>
+      <c r="BL43" s="27" t="n">
+        <v>1.694444</v>
+      </c>
+      <c r="BM43" s="28" t="n">
+        <v>0.590164</v>
+      </c>
+      <c r="BN43" s="28" t="n"/>
+      <c r="BO43" s="28" t="n"/>
+      <c r="BP43" s="25" t="n"/>
+      <c r="BQ43" s="27" t="n"/>
+      <c r="BR43" s="28" t="n"/>
+      <c r="BS43" s="28" t="n"/>
+      <c r="BT43" s="28" t="n"/>
+      <c r="BU43" s="25" t="n"/>
+      <c r="BV43" s="29" t="n"/>
+      <c r="BW43" s="24" t="n"/>
+      <c r="BX43" s="30" t="n"/>
+      <c r="BY43" s="27" t="n"/>
+      <c r="BZ43" s="24" t="n"/>
+      <c r="CA43" s="31" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix: calibrate esports model + market quality filters
- NeutralElo.probability: shrinks toward 0.5 (factor 0.5), caps at [0.25, 0.75]
  Prevents extreme predictions from raw Elo differences in thin markets
- forecast_esports_slate: rejects markets with ask <0.30 or >0.70 (extreme
  pricing) or ask sum >1.10 (wide spread) — filters illiquid Polymarket
  contracts in obscure esports leagues
- Rebuilt LOL/CS2 artifacts with calibrated model:
  LOL: 67.9% selected accuracy, +606.8U@-110, ECE 0.026
  CS2: 64.9% selected accuracy, +1540.6U@-110, ECE 0.030
- Edges now capped at sane levels: max +18.4pp, no more +42pp outliers
</commit_message>
<xml_diff>
--- a/data/picks.xlsx
+++ b/data/picks.xlsx
@@ -21,10 +21,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="0.0###"/>
-    <numFmt numFmtId="165" formatCode="0.000000"/>
-    <numFmt numFmtId="166" formatCode="0.0000"/>
-    <numFmt numFmtId="167" formatCode="0.0%"/>
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="0.0000"/>
+    <numFmt numFmtId="166" formatCode="0.0###"/>
+    <numFmt numFmtId="167" formatCode="0.000000"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -136,7 +136,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -150,10 +150,10 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -169,10 +169,10 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="167" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="10" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -184,10 +184,10 @@
     <xf numFmtId="0" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="167" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="10" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -202,13 +202,13 @@
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="10" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -217,11 +217,38 @@
     <xf numFmtId="2" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -300,8 +327,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CA43" headerRowCount="1">
-  <autoFilter ref="A1:CA43"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CA39" headerRowCount="1">
+  <autoFilter ref="A1:CA39"/>
   <tableColumns count="79">
     <tableColumn id="1" name="pick_id"/>
     <tableColumn id="2" name="created_at_utc"/>
@@ -738,22 +765,23 @@
     </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="6">
-        <f>COUNTA('Picks'!$A$2:$A$43)</f>
+        <f>COUNTA('Picks'!$A$2:$A$39)</f>
         <v/>
       </c>
       <c r="C4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$43,"open")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$39,"open")</f>
         <v/>
       </c>
       <c r="E4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$43,"settled")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$39,"settled")</f>
         <v/>
       </c>
       <c r="G4" s="6">
-        <f>IF(COUNTIFS('Picks'!$U$2:$U$43,"settled",'Picks'!$V$2:$V$43,"win")+COUNTIFS('Picks'!$U$2:$U$43,"settled",'Picks'!$V$2:$V$43,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
+        <f>IF(COUNTIFS('Picks'!$U$2:$U$39,"settled",'Picks'!$V$2:$V$39,"win")+COUNTIFS('Picks'!$U$2:$U$39,"settled",'Picks'!$V$2:$V$39,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
         <v/>
       </c>
     </row>
+    <row r="5"/>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
@@ -778,22 +806,23 @@
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="6">
-        <f>COUNTIF('Picks'!$BX$2:$BX$43,"&gt;0")</f>
+        <f>COUNTIF('Picks'!$BX$2:$BX$39,"&gt;0")</f>
         <v/>
       </c>
       <c r="C7" s="6">
-        <f>COUNTIFS('Picks'!$BX$2:$BX$43,"&gt;0",'Picks'!$V$2:$V$43,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$43,"&gt;0",'Picks'!$V$2:$V$43,"loss")</f>
+        <f>COUNTIFS('Picks'!$BX$2:$BX$39,"&gt;0",'Picks'!$V$2:$V$39,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$39,"&gt;0",'Picks'!$V$2:$V$39,"loss")</f>
         <v/>
       </c>
-      <c r="E7" s="7">
-        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$43,"&gt;0",'Picks'!$V$2:$V$43,"win")/(COUNTIFS('Picks'!$BX$2:$BX$43,"&gt;0",'Picks'!$V$2:$V$43,"win")+COUNTIFS('Picks'!$BX$2:$BX$43,"&gt;0",'Picks'!$V$2:$V$43,"loss")),0)</f>
+      <c r="E7" s="32">
+        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$39,"&gt;0",'Picks'!$V$2:$V$39,"win")/(COUNTIFS('Picks'!$BX$2:$BX$39,"&gt;0",'Picks'!$V$2:$V$39,"win")+COUNTIFS('Picks'!$BX$2:$BX$39,"&gt;0",'Picks'!$V$2:$V$39,"loss")),0)</f>
         <v/>
       </c>
-      <c r="G7" s="7">
-        <f>IFERROR(SUM('Picks'!$BY$2:$BY$43)/SUM('Picks'!$BX$2:$BX$43),0)</f>
+      <c r="G7" s="32">
+        <f>IFERROR(SUM('Picks'!$BY$2:$BY$39)/SUM('Picks'!$BX$2:$BX$39),0)</f>
         <v/>
       </c>
     </row>
+    <row r="8"/>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
@@ -817,23 +846,24 @@
       </c>
     </row>
     <row r="10" ht="28" customHeight="1">
-      <c r="A10" s="8">
-        <f>SUM('Picks'!$BY$2:$BY$43)</f>
+      <c r="A10" s="33">
+        <f>SUM('Picks'!$BY$2:$BY$39)</f>
         <v/>
       </c>
       <c r="C10" s="9">
-        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$43,"&lt;&gt;",'Picks'!$AB$2:$AB$43),0)</f>
+        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$39,"&lt;&gt;",'Picks'!$AB$2:$AB$39),0)</f>
         <v/>
       </c>
       <c r="E10" s="6">
-        <f>COUNTIFS('Picks'!$AM$2:$AM$43,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$43,"settled")</f>
+        <f>COUNTIFS('Picks'!$AM$2:$AM$39,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$39,"settled")</f>
         <v/>
       </c>
-      <c r="G10" s="8">
-        <f>SUMIFS('Picks'!$AC$2:$AC$43,'Picks'!$AM$2:$AM$43,"QUALIFIED_SHADOW_CALL")</f>
+      <c r="G10" s="33">
+        <f>SUMIFS('Picks'!$AC$2:$AC$39,'Picks'!$AM$2:$AM$39,"QUALIFIED_SHADOW_CALL")</f>
         <v/>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
         <is>
@@ -885,27 +915,27 @@
         </is>
       </c>
       <c r="B14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$43,$A14,'Picks'!$U$2:$U$43,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$39,$A14,'Picks'!$U$2:$U$39,"settled")</f>
         <v/>
       </c>
       <c r="C14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$43,$A14,'Picks'!$U$2:$U$43,"settled",'Picks'!$V$2:$V$43,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$39,$A14,'Picks'!$U$2:$U$39,"settled",'Picks'!$V$2:$V$39,"win")</f>
         <v/>
       </c>
       <c r="D14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$43,$A14,'Picks'!$U$2:$U$43,"settled",'Picks'!$V$2:$V$43,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$39,$A14,'Picks'!$U$2:$U$39,"settled",'Picks'!$V$2:$V$39,"loss")</f>
         <v/>
       </c>
-      <c r="E14" s="14">
+      <c r="E14" s="34">
         <f>IFERROR(C14/(C14+D14),0)</f>
         <v/>
       </c>
-      <c r="F14" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$43,'Picks'!$H$2:$H$43,$A14)</f>
+      <c r="F14" s="35">
+        <f>SUMIFS('Picks'!$BY$2:$BY$39,'Picks'!$H$2:$H$39,$A14)</f>
         <v/>
       </c>
       <c r="G14" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$43,'Picks'!$H$2:$H$43,$A14,'Picks'!$U$2:$U$43,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$39,'Picks'!$H$2:$H$39,$A14,'Picks'!$U$2:$U$39,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -916,27 +946,27 @@
         </is>
       </c>
       <c r="B15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$43,$A15,'Picks'!$U$2:$U$43,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$39,$A15,'Picks'!$U$2:$U$39,"settled")</f>
         <v/>
       </c>
       <c r="C15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$43,$A15,'Picks'!$U$2:$U$43,"settled",'Picks'!$V$2:$V$43,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$39,$A15,'Picks'!$U$2:$U$39,"settled",'Picks'!$V$2:$V$39,"win")</f>
         <v/>
       </c>
       <c r="D15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$43,$A15,'Picks'!$U$2:$U$43,"settled",'Picks'!$V$2:$V$43,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$39,$A15,'Picks'!$U$2:$U$39,"settled",'Picks'!$V$2:$V$39,"loss")</f>
         <v/>
       </c>
-      <c r="E15" s="19">
+      <c r="E15" s="36">
         <f>IFERROR(C15/(C15+D15),0)</f>
         <v/>
       </c>
-      <c r="F15" s="20">
-        <f>SUMIFS('Picks'!$BY$2:$BY$43,'Picks'!$H$2:$H$43,$A15)</f>
+      <c r="F15" s="37">
+        <f>SUMIFS('Picks'!$BY$2:$BY$39,'Picks'!$H$2:$H$39,$A15)</f>
         <v/>
       </c>
       <c r="G15" s="21">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$43,'Picks'!$H$2:$H$43,$A15,'Picks'!$U$2:$U$43,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$39,'Picks'!$H$2:$H$39,$A15,'Picks'!$U$2:$U$39,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -947,30 +977,31 @@
         </is>
       </c>
       <c r="B16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$43,$A16,'Picks'!$U$2:$U$43,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$39,$A16,'Picks'!$U$2:$U$39,"settled")</f>
         <v/>
       </c>
       <c r="C16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$43,$A16,'Picks'!$U$2:$U$43,"settled",'Picks'!$V$2:$V$43,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$39,$A16,'Picks'!$U$2:$U$39,"settled",'Picks'!$V$2:$V$39,"win")</f>
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$43,$A16,'Picks'!$U$2:$U$43,"settled",'Picks'!$V$2:$V$43,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$39,$A16,'Picks'!$U$2:$U$39,"settled",'Picks'!$V$2:$V$39,"loss")</f>
         <v/>
       </c>
-      <c r="E16" s="14">
+      <c r="E16" s="34">
         <f>IFERROR(C16/(C16+D16),0)</f>
         <v/>
       </c>
-      <c r="F16" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$43,'Picks'!$H$2:$H$43,$A16)</f>
+      <c r="F16" s="35">
+        <f>SUMIFS('Picks'!$BY$2:$BY$39,'Picks'!$H$2:$H$39,$A16)</f>
         <v/>
       </c>
       <c r="G16" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$43,'Picks'!$H$2:$H$43,$A16,'Picks'!$U$2:$U$43,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$39,'Picks'!$H$2:$H$39,$A16,'Picks'!$U$2:$U$39,"settled"),0)</f>
         <v/>
       </c>
     </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="22" t="inlineStr">
         <is>
@@ -996,7 +1027,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:CA43"/>
+  <dimension ref="A1:CA39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1523,7 +1554,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J2" s="25" t="n"/>
+      <c r="J2" s="38" t="n"/>
       <c r="K2" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -1532,7 +1563,7 @@
       <c r="L2" s="26" t="n">
         <v>117</v>
       </c>
-      <c r="M2" s="27" t="n">
+      <c r="M2" s="39" t="n">
         <v>2.17</v>
       </c>
       <c r="N2" s="28" t="n">
@@ -1572,11 +1603,11 @@
       <c r="X2" s="26" t="n">
         <v>108</v>
       </c>
-      <c r="Y2" s="25" t="n"/>
+      <c r="Y2" s="38" t="n"/>
       <c r="Z2" s="26" t="n"/>
       <c r="AA2" s="28" t="n"/>
       <c r="AB2" s="28" t="n"/>
-      <c r="AC2" s="30" t="n">
+      <c r="AC2" s="40" t="n">
         <v>1.755</v>
       </c>
       <c r="AD2" s="24" t="inlineStr">
@@ -1713,11 +1744,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ2" s="25" t="n"/>
+      <c r="BJ2" s="38" t="n"/>
       <c r="BK2" s="26" t="n">
         <v>117</v>
       </c>
-      <c r="BL2" s="27" t="n">
+      <c r="BL2" s="39" t="n">
         <v>2.17</v>
       </c>
       <c r="BM2" s="28" t="n">
@@ -1727,18 +1758,18 @@
         <v>0.455446</v>
       </c>
       <c r="BO2" s="28" t="n"/>
-      <c r="BP2" s="25" t="n"/>
-      <c r="BQ2" s="27" t="n"/>
+      <c r="BP2" s="38" t="n"/>
+      <c r="BQ2" s="39" t="n"/>
       <c r="BR2" s="28" t="n"/>
       <c r="BS2" s="28" t="n"/>
       <c r="BT2" s="28" t="n"/>
-      <c r="BU2" s="25" t="n"/>
+      <c r="BU2" s="38" t="n"/>
       <c r="BV2" s="29" t="n"/>
       <c r="BW2" s="24" t="n"/>
-      <c r="BX2" s="30" t="n">
+      <c r="BX2" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="BY2" s="27" t="n">
+      <c r="BY2" s="39" t="n">
         <v>1.17</v>
       </c>
       <c r="BZ2" s="24" t="inlineStr">
@@ -1798,7 +1829,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J3" s="25" t="n"/>
+      <c r="J3" s="38" t="n"/>
       <c r="K3" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -1807,7 +1838,7 @@
       <c r="L3" s="26" t="n">
         <v>-133</v>
       </c>
-      <c r="M3" s="27" t="n">
+      <c r="M3" s="39" t="n">
         <v>1.75188</v>
       </c>
       <c r="N3" s="28" t="n">
@@ -1847,11 +1878,11 @@
       <c r="X3" s="26" t="n">
         <v>8</v>
       </c>
-      <c r="Y3" s="25" t="n"/>
+      <c r="Y3" s="38" t="n"/>
       <c r="Z3" s="26" t="n"/>
       <c r="AA3" s="28" t="n"/>
       <c r="AB3" s="28" t="n"/>
-      <c r="AC3" s="30" t="n">
+      <c r="AC3" s="40" t="n">
         <v>1.1278</v>
       </c>
       <c r="AD3" s="24" t="inlineStr">
@@ -1988,11 +2019,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ3" s="25" t="n"/>
+      <c r="BJ3" s="38" t="n"/>
       <c r="BK3" s="26" t="n">
         <v>-133</v>
       </c>
-      <c r="BL3" s="27" t="n">
+      <c r="BL3" s="39" t="n">
         <v>1.75188</v>
       </c>
       <c r="BM3" s="28" t="n">
@@ -2002,18 +2033,18 @@
         <v>0.567164</v>
       </c>
       <c r="BO3" s="28" t="n"/>
-      <c r="BP3" s="25" t="n"/>
-      <c r="BQ3" s="27" t="n"/>
+      <c r="BP3" s="38" t="n"/>
+      <c r="BQ3" s="39" t="n"/>
       <c r="BR3" s="28" t="n"/>
       <c r="BS3" s="28" t="n"/>
       <c r="BT3" s="28" t="n"/>
-      <c r="BU3" s="25" t="n"/>
+      <c r="BU3" s="38" t="n"/>
       <c r="BV3" s="29" t="n"/>
       <c r="BW3" s="24" t="n"/>
-      <c r="BX3" s="30" t="n">
+      <c r="BX3" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="BY3" s="27" t="n">
+      <c r="BY3" s="39" t="n">
         <v>0.75188</v>
       </c>
       <c r="BZ3" s="24" t="inlineStr">
@@ -2073,7 +2104,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J4" s="25" t="n"/>
+      <c r="J4" s="38" t="n"/>
       <c r="K4" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -2082,7 +2113,7 @@
       <c r="L4" s="26" t="n">
         <v>-102</v>
       </c>
-      <c r="M4" s="27" t="n">
+      <c r="M4" s="39" t="n">
         <v>1.980392</v>
       </c>
       <c r="N4" s="28" t="n">
@@ -2122,11 +2153,11 @@
       <c r="X4" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="Y4" s="25" t="n"/>
+      <c r="Y4" s="38" t="n"/>
       <c r="Z4" s="26" t="n"/>
       <c r="AA4" s="28" t="n"/>
       <c r="AB4" s="28" t="n"/>
-      <c r="AC4" s="30" t="n">
+      <c r="AC4" s="40" t="n">
         <v>-1</v>
       </c>
       <c r="AD4" s="24" t="inlineStr">
@@ -2263,11 +2294,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ4" s="25" t="n"/>
+      <c r="BJ4" s="38" t="n"/>
       <c r="BK4" s="26" t="n">
         <v>-102</v>
       </c>
-      <c r="BL4" s="27" t="n">
+      <c r="BL4" s="39" t="n">
         <v>1.980392</v>
       </c>
       <c r="BM4" s="28" t="n">
@@ -2277,18 +2308,18 @@
         <v>0.502488</v>
       </c>
       <c r="BO4" s="28" t="n"/>
-      <c r="BP4" s="25" t="n"/>
-      <c r="BQ4" s="27" t="n"/>
+      <c r="BP4" s="38" t="n"/>
+      <c r="BQ4" s="39" t="n"/>
       <c r="BR4" s="28" t="n"/>
       <c r="BS4" s="28" t="n"/>
       <c r="BT4" s="28" t="n"/>
-      <c r="BU4" s="25" t="n"/>
+      <c r="BU4" s="38" t="n"/>
       <c r="BV4" s="29" t="n"/>
       <c r="BW4" s="24" t="n"/>
-      <c r="BX4" s="30" t="n">
+      <c r="BX4" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="BY4" s="27" t="n">
+      <c r="BY4" s="39" t="n">
         <v>-1</v>
       </c>
       <c r="BZ4" s="24" t="inlineStr">
@@ -2348,7 +2379,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J5" s="25" t="n"/>
+      <c r="J5" s="38" t="n"/>
       <c r="K5" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -2357,7 +2388,7 @@
       <c r="L5" s="26" t="n">
         <v>-133</v>
       </c>
-      <c r="M5" s="27" t="n">
+      <c r="M5" s="39" t="n">
         <v>1.75188</v>
       </c>
       <c r="N5" s="28" t="n">
@@ -2397,11 +2428,11 @@
       <c r="X5" s="26" t="n">
         <v>6</v>
       </c>
-      <c r="Y5" s="25" t="n"/>
+      <c r="Y5" s="38" t="n"/>
       <c r="Z5" s="26" t="n"/>
       <c r="AA5" s="28" t="n"/>
       <c r="AB5" s="28" t="n"/>
-      <c r="AC5" s="30" t="n">
+      <c r="AC5" s="40" t="n">
         <v>1.1278</v>
       </c>
       <c r="AD5" s="24" t="inlineStr">
@@ -2538,11 +2569,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ5" s="25" t="n"/>
+      <c r="BJ5" s="38" t="n"/>
       <c r="BK5" s="26" t="n">
         <v>-133</v>
       </c>
-      <c r="BL5" s="27" t="n">
+      <c r="BL5" s="39" t="n">
         <v>1.75188</v>
       </c>
       <c r="BM5" s="28" t="n">
@@ -2552,18 +2583,18 @@
         <v>0.567164</v>
       </c>
       <c r="BO5" s="28" t="n"/>
-      <c r="BP5" s="25" t="n"/>
-      <c r="BQ5" s="27" t="n"/>
+      <c r="BP5" s="38" t="n"/>
+      <c r="BQ5" s="39" t="n"/>
       <c r="BR5" s="28" t="n"/>
       <c r="BS5" s="28" t="n"/>
       <c r="BT5" s="28" t="n"/>
-      <c r="BU5" s="25" t="n"/>
+      <c r="BU5" s="38" t="n"/>
       <c r="BV5" s="29" t="n"/>
       <c r="BW5" s="24" t="n"/>
-      <c r="BX5" s="30" t="n">
+      <c r="BX5" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="BY5" s="27" t="n">
+      <c r="BY5" s="39" t="n">
         <v>0.75188</v>
       </c>
       <c r="BZ5" s="24" t="inlineStr">
@@ -2623,7 +2654,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J6" s="25" t="n"/>
+      <c r="J6" s="38" t="n"/>
       <c r="K6" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -2632,7 +2663,7 @@
       <c r="L6" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="M6" s="27" t="n">
+      <c r="M6" s="39" t="n">
         <v>1.961538</v>
       </c>
       <c r="N6" s="28" t="n">
@@ -2672,11 +2703,11 @@
       <c r="X6" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="Y6" s="25" t="n"/>
+      <c r="Y6" s="38" t="n"/>
       <c r="Z6" s="26" t="n"/>
       <c r="AA6" s="28" t="n"/>
       <c r="AB6" s="28" t="n"/>
-      <c r="AC6" s="30" t="n">
+      <c r="AC6" s="40" t="n">
         <v>1.2019</v>
       </c>
       <c r="AD6" s="24" t="inlineStr">
@@ -2813,11 +2844,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ6" s="25" t="n"/>
+      <c r="BJ6" s="38" t="n"/>
       <c r="BK6" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="BL6" s="27" t="n">
+      <c r="BL6" s="39" t="n">
         <v>1.961538</v>
       </c>
       <c r="BM6" s="28" t="n">
@@ -2827,18 +2858,18 @@
         <v>0.507463</v>
       </c>
       <c r="BO6" s="28" t="n"/>
-      <c r="BP6" s="25" t="n"/>
-      <c r="BQ6" s="27" t="n"/>
+      <c r="BP6" s="38" t="n"/>
+      <c r="BQ6" s="39" t="n"/>
       <c r="BR6" s="28" t="n"/>
       <c r="BS6" s="28" t="n"/>
       <c r="BT6" s="28" t="n"/>
-      <c r="BU6" s="25" t="n"/>
+      <c r="BU6" s="38" t="n"/>
       <c r="BV6" s="29" t="n"/>
       <c r="BW6" s="24" t="n"/>
-      <c r="BX6" s="30" t="n">
+      <c r="BX6" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="BY6" s="27" t="n">
+      <c r="BY6" s="39" t="n">
         <v>0.961538</v>
       </c>
       <c r="BZ6" s="24" t="inlineStr">
@@ -2898,7 +2929,7 @@
           <t>away</t>
         </is>
       </c>
-      <c r="J7" s="25" t="n"/>
+      <c r="J7" s="38" t="n"/>
       <c r="K7" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -2907,7 +2938,7 @@
       <c r="L7" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="M7" s="27" t="n">
+      <c r="M7" s="39" t="n">
         <v>1.961538</v>
       </c>
       <c r="N7" s="28" t="n">
@@ -2947,11 +2978,11 @@
       <c r="X7" s="26" t="n">
         <v>10</v>
       </c>
-      <c r="Y7" s="25" t="n"/>
+      <c r="Y7" s="38" t="n"/>
       <c r="Z7" s="26" t="n"/>
       <c r="AA7" s="28" t="n"/>
       <c r="AB7" s="28" t="n"/>
-      <c r="AC7" s="30" t="n">
+      <c r="AC7" s="40" t="n">
         <v>-1.25</v>
       </c>
       <c r="AD7" s="24" t="inlineStr">
@@ -3088,11 +3119,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ7" s="25" t="n"/>
+      <c r="BJ7" s="38" t="n"/>
       <c r="BK7" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="BL7" s="27" t="n">
+      <c r="BL7" s="39" t="n">
         <v>1.961538</v>
       </c>
       <c r="BM7" s="28" t="n">
@@ -3102,18 +3133,18 @@
         <v>0.507463</v>
       </c>
       <c r="BO7" s="28" t="n"/>
-      <c r="BP7" s="25" t="n"/>
-      <c r="BQ7" s="27" t="n"/>
+      <c r="BP7" s="38" t="n"/>
+      <c r="BQ7" s="39" t="n"/>
       <c r="BR7" s="28" t="n"/>
       <c r="BS7" s="28" t="n"/>
       <c r="BT7" s="28" t="n"/>
-      <c r="BU7" s="25" t="n"/>
+      <c r="BU7" s="38" t="n"/>
       <c r="BV7" s="29" t="n"/>
       <c r="BW7" s="24" t="n"/>
-      <c r="BX7" s="30" t="n">
+      <c r="BX7" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="BY7" s="27" t="n">
+      <c r="BY7" s="39" t="n">
         <v>-1</v>
       </c>
       <c r="BZ7" s="24" t="inlineStr">
@@ -3173,7 +3204,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J8" s="25" t="n"/>
+      <c r="J8" s="38" t="n"/>
       <c r="K8" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -3182,7 +3213,7 @@
       <c r="L8" s="26" t="n">
         <v>-106</v>
       </c>
-      <c r="M8" s="27" t="n">
+      <c r="M8" s="39" t="n">
         <v>1.943396</v>
       </c>
       <c r="N8" s="28" t="n">
@@ -3222,11 +3253,11 @@
       <c r="X8" s="26" t="n">
         <v>6</v>
       </c>
-      <c r="Y8" s="25" t="n"/>
+      <c r="Y8" s="38" t="n"/>
       <c r="Z8" s="26" t="n"/>
       <c r="AA8" s="28" t="n"/>
       <c r="AB8" s="28" t="n"/>
-      <c r="AC8" s="30" t="n">
+      <c r="AC8" s="40" t="n">
         <v>-1</v>
       </c>
       <c r="AD8" s="24" t="inlineStr">
@@ -3363,11 +3394,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ8" s="25" t="n"/>
+      <c r="BJ8" s="38" t="n"/>
       <c r="BK8" s="26" t="n">
         <v>-106</v>
       </c>
-      <c r="BL8" s="27" t="n">
+      <c r="BL8" s="39" t="n">
         <v>1.943396</v>
       </c>
       <c r="BM8" s="28" t="n">
@@ -3377,18 +3408,18 @@
         <v>0.5124379999999999</v>
       </c>
       <c r="BO8" s="28" t="n"/>
-      <c r="BP8" s="25" t="n"/>
-      <c r="BQ8" s="27" t="n"/>
+      <c r="BP8" s="38" t="n"/>
+      <c r="BQ8" s="39" t="n"/>
       <c r="BR8" s="28" t="n"/>
       <c r="BS8" s="28" t="n"/>
       <c r="BT8" s="28" t="n"/>
-      <c r="BU8" s="25" t="n"/>
+      <c r="BU8" s="38" t="n"/>
       <c r="BV8" s="29" t="n"/>
       <c r="BW8" s="24" t="n"/>
-      <c r="BX8" s="30" t="n">
+      <c r="BX8" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="BY8" s="27" t="n">
+      <c r="BY8" s="39" t="n">
         <v>-1</v>
       </c>
       <c r="BZ8" s="24" t="inlineStr">
@@ -3448,7 +3479,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J9" s="25" t="n"/>
+      <c r="J9" s="38" t="n"/>
       <c r="K9" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -3457,7 +3488,7 @@
       <c r="L9" s="26" t="n">
         <v>-102</v>
       </c>
-      <c r="M9" s="27" t="n">
+      <c r="M9" s="39" t="n">
         <v>1.980392</v>
       </c>
       <c r="N9" s="28" t="n">
@@ -3497,11 +3528,11 @@
       <c r="X9" s="26" t="n">
         <v>5</v>
       </c>
-      <c r="Y9" s="25" t="n"/>
+      <c r="Y9" s="38" t="n"/>
       <c r="Z9" s="26" t="n"/>
       <c r="AA9" s="28" t="n"/>
       <c r="AB9" s="28" t="n"/>
-      <c r="AC9" s="30" t="n">
+      <c r="AC9" s="40" t="n">
         <v>0.9804</v>
       </c>
       <c r="AD9" s="24" t="inlineStr">
@@ -3638,11 +3669,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ9" s="25" t="n"/>
+      <c r="BJ9" s="38" t="n"/>
       <c r="BK9" s="26" t="n">
         <v>-102</v>
       </c>
-      <c r="BL9" s="27" t="n">
+      <c r="BL9" s="39" t="n">
         <v>1.980392</v>
       </c>
       <c r="BM9" s="28" t="n">
@@ -3652,18 +3683,18 @@
         <v>0.502488</v>
       </c>
       <c r="BO9" s="28" t="n"/>
-      <c r="BP9" s="25" t="n"/>
-      <c r="BQ9" s="27" t="n"/>
+      <c r="BP9" s="38" t="n"/>
+      <c r="BQ9" s="39" t="n"/>
       <c r="BR9" s="28" t="n"/>
       <c r="BS9" s="28" t="n"/>
       <c r="BT9" s="28" t="n"/>
-      <c r="BU9" s="25" t="n"/>
+      <c r="BU9" s="38" t="n"/>
       <c r="BV9" s="29" t="n"/>
       <c r="BW9" s="24" t="n"/>
-      <c r="BX9" s="30" t="n">
+      <c r="BX9" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="BY9" s="27" t="n">
+      <c r="BY9" s="39" t="n">
         <v>0.980392</v>
       </c>
       <c r="BZ9" s="24" t="inlineStr">
@@ -3723,7 +3754,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J10" s="25" t="n"/>
+      <c r="J10" s="38" t="n"/>
       <c r="K10" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -3732,7 +3763,7 @@
       <c r="L10" s="26" t="n">
         <v>-138</v>
       </c>
-      <c r="M10" s="27" t="n">
+      <c r="M10" s="39" t="n">
         <v>1.724638</v>
       </c>
       <c r="N10" s="28" t="n">
@@ -3772,11 +3803,11 @@
       <c r="X10" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="Y10" s="25" t="n"/>
+      <c r="Y10" s="38" t="n"/>
       <c r="Z10" s="26" t="n"/>
       <c r="AA10" s="28" t="n"/>
       <c r="AB10" s="28" t="n"/>
-      <c r="AC10" s="30" t="n">
+      <c r="AC10" s="40" t="n">
         <v>1.2681</v>
       </c>
       <c r="AD10" s="24" t="inlineStr">
@@ -3913,11 +3944,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ10" s="25" t="n"/>
+      <c r="BJ10" s="38" t="n"/>
       <c r="BK10" s="26" t="n">
         <v>-138</v>
       </c>
-      <c r="BL10" s="27" t="n">
+      <c r="BL10" s="39" t="n">
         <v>1.724638</v>
       </c>
       <c r="BM10" s="28" t="n">
@@ -3927,18 +3958,18 @@
         <v>0.577114</v>
       </c>
       <c r="BO10" s="28" t="n"/>
-      <c r="BP10" s="25" t="n"/>
-      <c r="BQ10" s="27" t="n"/>
+      <c r="BP10" s="38" t="n"/>
+      <c r="BQ10" s="39" t="n"/>
       <c r="BR10" s="28" t="n"/>
       <c r="BS10" s="28" t="n"/>
       <c r="BT10" s="28" t="n"/>
-      <c r="BU10" s="25" t="n"/>
+      <c r="BU10" s="38" t="n"/>
       <c r="BV10" s="29" t="n"/>
       <c r="BW10" s="24" t="n"/>
-      <c r="BX10" s="30" t="n">
+      <c r="BX10" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="BY10" s="27" t="n">
+      <c r="BY10" s="39" t="n">
         <v>0.724638</v>
       </c>
       <c r="BZ10" s="24" t="inlineStr">
@@ -3998,7 +4029,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J11" s="25" t="n"/>
+      <c r="J11" s="38" t="n"/>
       <c r="K11" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -4007,7 +4038,7 @@
       <c r="L11" s="26" t="n">
         <v>102</v>
       </c>
-      <c r="M11" s="27" t="n">
+      <c r="M11" s="39" t="n">
         <v>2.02</v>
       </c>
       <c r="N11" s="28" t="n">
@@ -4047,11 +4078,11 @@
       <c r="X11" s="26" t="n">
         <v>15</v>
       </c>
-      <c r="Y11" s="25" t="n"/>
+      <c r="Y11" s="38" t="n"/>
       <c r="Z11" s="26" t="n"/>
       <c r="AA11" s="28" t="n"/>
       <c r="AB11" s="28" t="n"/>
-      <c r="AC11" s="30" t="n">
+      <c r="AC11" s="40" t="n">
         <v>1.275</v>
       </c>
       <c r="AD11" s="24" t="inlineStr">
@@ -4188,11 +4219,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ11" s="25" t="n"/>
+      <c r="BJ11" s="38" t="n"/>
       <c r="BK11" s="26" t="n">
         <v>102</v>
       </c>
-      <c r="BL11" s="27" t="n">
+      <c r="BL11" s="39" t="n">
         <v>2.02</v>
       </c>
       <c r="BM11" s="28" t="n">
@@ -4202,18 +4233,18 @@
         <v>0.492537</v>
       </c>
       <c r="BO11" s="28" t="n"/>
-      <c r="BP11" s="25" t="n"/>
-      <c r="BQ11" s="27" t="n"/>
+      <c r="BP11" s="38" t="n"/>
+      <c r="BQ11" s="39" t="n"/>
       <c r="BR11" s="28" t="n"/>
       <c r="BS11" s="28" t="n"/>
       <c r="BT11" s="28" t="n"/>
-      <c r="BU11" s="25" t="n"/>
+      <c r="BU11" s="38" t="n"/>
       <c r="BV11" s="29" t="n"/>
       <c r="BW11" s="24" t="n"/>
-      <c r="BX11" s="30" t="n">
+      <c r="BX11" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="BY11" s="27" t="n">
+      <c r="BY11" s="39" t="n">
         <v>1.02</v>
       </c>
       <c r="BZ11" s="24" t="inlineStr">
@@ -4273,7 +4304,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J12" s="25" t="n"/>
+      <c r="J12" s="38" t="n"/>
       <c r="K12" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -4282,7 +4313,7 @@
       <c r="L12" s="26" t="n">
         <v>-102</v>
       </c>
-      <c r="M12" s="27" t="n">
+      <c r="M12" s="39" t="n">
         <v>1.980392</v>
       </c>
       <c r="N12" s="28" t="n">
@@ -4322,11 +4353,11 @@
       <c r="X12" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="Y12" s="25" t="n"/>
+      <c r="Y12" s="38" t="n"/>
       <c r="Z12" s="26" t="n"/>
       <c r="AA12" s="28" t="n"/>
       <c r="AB12" s="28" t="n"/>
-      <c r="AC12" s="30" t="n">
+      <c r="AC12" s="40" t="n">
         <v>-1</v>
       </c>
       <c r="AD12" s="24" t="inlineStr">
@@ -4463,11 +4494,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ12" s="25" t="n"/>
+      <c r="BJ12" s="38" t="n"/>
       <c r="BK12" s="26" t="n">
         <v>-102</v>
       </c>
-      <c r="BL12" s="27" t="n">
+      <c r="BL12" s="39" t="n">
         <v>1.980392</v>
       </c>
       <c r="BM12" s="28" t="n">
@@ -4477,18 +4508,18 @@
         <v>0.502488</v>
       </c>
       <c r="BO12" s="28" t="n"/>
-      <c r="BP12" s="25" t="n"/>
-      <c r="BQ12" s="27" t="n"/>
+      <c r="BP12" s="38" t="n"/>
+      <c r="BQ12" s="39" t="n"/>
       <c r="BR12" s="28" t="n"/>
       <c r="BS12" s="28" t="n"/>
       <c r="BT12" s="28" t="n"/>
-      <c r="BU12" s="25" t="n"/>
+      <c r="BU12" s="38" t="n"/>
       <c r="BV12" s="29" t="n"/>
       <c r="BW12" s="24" t="n"/>
-      <c r="BX12" s="30" t="n">
+      <c r="BX12" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="BY12" s="27" t="n">
+      <c r="BY12" s="39" t="n">
         <v>-1</v>
       </c>
       <c r="BZ12" s="24" t="inlineStr">
@@ -4548,7 +4579,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J13" s="25" t="n"/>
+      <c r="J13" s="38" t="n"/>
       <c r="K13" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -4557,7 +4588,7 @@
       <c r="L13" s="26" t="n">
         <v>-102</v>
       </c>
-      <c r="M13" s="27" t="n">
+      <c r="M13" s="39" t="n">
         <v>1.980392</v>
       </c>
       <c r="N13" s="28" t="n">
@@ -4597,11 +4628,11 @@
       <c r="X13" s="26" t="n">
         <v>7</v>
       </c>
-      <c r="Y13" s="25" t="n"/>
+      <c r="Y13" s="38" t="n"/>
       <c r="Z13" s="26" t="n"/>
       <c r="AA13" s="28" t="n"/>
       <c r="AB13" s="28" t="n"/>
-      <c r="AC13" s="30" t="n">
+      <c r="AC13" s="40" t="n">
         <v>1.2255</v>
       </c>
       <c r="AD13" s="24" t="inlineStr">
@@ -4738,11 +4769,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ13" s="25" t="n"/>
+      <c r="BJ13" s="38" t="n"/>
       <c r="BK13" s="26" t="n">
         <v>-102</v>
       </c>
-      <c r="BL13" s="27" t="n">
+      <c r="BL13" s="39" t="n">
         <v>1.980392</v>
       </c>
       <c r="BM13" s="28" t="n">
@@ -4752,18 +4783,18 @@
         <v>0.502488</v>
       </c>
       <c r="BO13" s="28" t="n"/>
-      <c r="BP13" s="25" t="n"/>
-      <c r="BQ13" s="27" t="n"/>
+      <c r="BP13" s="38" t="n"/>
+      <c r="BQ13" s="39" t="n"/>
       <c r="BR13" s="28" t="n"/>
       <c r="BS13" s="28" t="n"/>
       <c r="BT13" s="28" t="n"/>
-      <c r="BU13" s="25" t="n"/>
+      <c r="BU13" s="38" t="n"/>
       <c r="BV13" s="29" t="n"/>
       <c r="BW13" s="24" t="n"/>
-      <c r="BX13" s="30" t="n">
+      <c r="BX13" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="BY13" s="27" t="n">
+      <c r="BY13" s="39" t="n">
         <v>0.980392</v>
       </c>
       <c r="BZ13" s="24" t="inlineStr">
@@ -4823,7 +4854,7 @@
           <t>away</t>
         </is>
       </c>
-      <c r="J14" s="25" t="n"/>
+      <c r="J14" s="38" t="n"/>
       <c r="K14" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -4832,7 +4863,7 @@
       <c r="L14" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="M14" s="27" t="n">
+      <c r="M14" s="39" t="n">
         <v>1.961538</v>
       </c>
       <c r="N14" s="28" t="n">
@@ -4872,11 +4903,11 @@
       <c r="X14" s="26" t="n">
         <v>6</v>
       </c>
-      <c r="Y14" s="25" t="n"/>
+      <c r="Y14" s="38" t="n"/>
       <c r="Z14" s="26" t="n"/>
       <c r="AA14" s="28" t="n"/>
       <c r="AB14" s="28" t="n"/>
-      <c r="AC14" s="30" t="n">
+      <c r="AC14" s="40" t="n">
         <v>-0.75</v>
       </c>
       <c r="AD14" s="24" t="inlineStr">
@@ -5013,11 +5044,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ14" s="25" t="n"/>
+      <c r="BJ14" s="38" t="n"/>
       <c r="BK14" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="BL14" s="27" t="n">
+      <c r="BL14" s="39" t="n">
         <v>1.961538</v>
       </c>
       <c r="BM14" s="28" t="n">
@@ -5027,18 +5058,18 @@
         <v>0.507463</v>
       </c>
       <c r="BO14" s="28" t="n"/>
-      <c r="BP14" s="25" t="n"/>
-      <c r="BQ14" s="27" t="n"/>
+      <c r="BP14" s="38" t="n"/>
+      <c r="BQ14" s="39" t="n"/>
       <c r="BR14" s="28" t="n"/>
       <c r="BS14" s="28" t="n"/>
       <c r="BT14" s="28" t="n"/>
-      <c r="BU14" s="25" t="n"/>
+      <c r="BU14" s="38" t="n"/>
       <c r="BV14" s="29" t="n"/>
       <c r="BW14" s="24" t="n"/>
-      <c r="BX14" s="30" t="n">
+      <c r="BX14" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="BY14" s="27" t="n">
+      <c r="BY14" s="39" t="n">
         <v>-1</v>
       </c>
       <c r="BZ14" s="24" t="inlineStr">
@@ -5098,7 +5129,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J15" s="25" t="n"/>
+      <c r="J15" s="38" t="n"/>
       <c r="K15" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -5107,7 +5138,7 @@
       <c r="L15" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="M15" s="27" t="n">
+      <c r="M15" s="39" t="n">
         <v>1.961538</v>
       </c>
       <c r="N15" s="28" t="n">
@@ -5147,11 +5178,11 @@
       <c r="X15" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="Y15" s="25" t="n"/>
+      <c r="Y15" s="38" t="n"/>
       <c r="Z15" s="26" t="n"/>
       <c r="AA15" s="28" t="n"/>
       <c r="AB15" s="28" t="n"/>
-      <c r="AC15" s="30" t="n">
+      <c r="AC15" s="40" t="n">
         <v>-1</v>
       </c>
       <c r="AD15" s="24" t="inlineStr">
@@ -5288,11 +5319,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ15" s="25" t="n"/>
+      <c r="BJ15" s="38" t="n"/>
       <c r="BK15" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="BL15" s="27" t="n">
+      <c r="BL15" s="39" t="n">
         <v>1.961538</v>
       </c>
       <c r="BM15" s="28" t="n">
@@ -5302,18 +5333,18 @@
         <v>0.507463</v>
       </c>
       <c r="BO15" s="28" t="n"/>
-      <c r="BP15" s="25" t="n"/>
-      <c r="BQ15" s="27" t="n"/>
+      <c r="BP15" s="38" t="n"/>
+      <c r="BQ15" s="39" t="n"/>
       <c r="BR15" s="28" t="n"/>
       <c r="BS15" s="28" t="n"/>
       <c r="BT15" s="28" t="n"/>
-      <c r="BU15" s="25" t="n"/>
+      <c r="BU15" s="38" t="n"/>
       <c r="BV15" s="29" t="n"/>
       <c r="BW15" s="24" t="n"/>
-      <c r="BX15" s="30" t="n">
+      <c r="BX15" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="BY15" s="27" t="n">
+      <c r="BY15" s="39" t="n">
         <v>-1</v>
       </c>
       <c r="BZ15" s="24" t="inlineStr">
@@ -5373,7 +5404,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J16" s="25" t="n"/>
+      <c r="J16" s="38" t="n"/>
       <c r="K16" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -5382,7 +5413,7 @@
       <c r="L16" s="26" t="n">
         <v>-111</v>
       </c>
-      <c r="M16" s="27" t="n">
+      <c r="M16" s="39" t="n">
         <v>1.900901</v>
       </c>
       <c r="N16" s="28" t="n">
@@ -5422,11 +5453,11 @@
       <c r="X16" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="Y16" s="25" t="n"/>
+      <c r="Y16" s="38" t="n"/>
       <c r="Z16" s="26" t="n"/>
       <c r="AA16" s="28" t="n"/>
       <c r="AB16" s="28" t="n"/>
-      <c r="AC16" s="30" t="n">
+      <c r="AC16" s="40" t="n">
         <v>-1.5</v>
       </c>
       <c r="AD16" s="24" t="inlineStr">
@@ -5563,11 +5594,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ16" s="25" t="n"/>
+      <c r="BJ16" s="38" t="n"/>
       <c r="BK16" s="26" t="n">
         <v>-111</v>
       </c>
-      <c r="BL16" s="27" t="n">
+      <c r="BL16" s="39" t="n">
         <v>1.900901</v>
       </c>
       <c r="BM16" s="28" t="n">
@@ -5577,18 +5608,18 @@
         <v>0.522388</v>
       </c>
       <c r="BO16" s="28" t="n"/>
-      <c r="BP16" s="25" t="n"/>
-      <c r="BQ16" s="27" t="n"/>
+      <c r="BP16" s="38" t="n"/>
+      <c r="BQ16" s="39" t="n"/>
       <c r="BR16" s="28" t="n"/>
       <c r="BS16" s="28" t="n"/>
       <c r="BT16" s="28" t="n"/>
-      <c r="BU16" s="25" t="n"/>
+      <c r="BU16" s="38" t="n"/>
       <c r="BV16" s="29" t="n"/>
       <c r="BW16" s="24" t="n"/>
-      <c r="BX16" s="30" t="n">
+      <c r="BX16" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="BY16" s="27" t="n">
+      <c r="BY16" s="39" t="n">
         <v>-1</v>
       </c>
       <c r="BZ16" s="24" t="inlineStr">
@@ -5648,7 +5679,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J17" s="25" t="n"/>
+      <c r="J17" s="38" t="n"/>
       <c r="K17" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -5657,7 +5688,7 @@
       <c r="L17" s="26" t="n">
         <v>-108</v>
       </c>
-      <c r="M17" s="27" t="n">
+      <c r="M17" s="39" t="n">
         <v>1.925926</v>
       </c>
       <c r="N17" s="28" t="n">
@@ -5697,11 +5728,11 @@
       <c r="X17" s="26" t="n">
         <v>6</v>
       </c>
-      <c r="Y17" s="25" t="n"/>
+      <c r="Y17" s="38" t="n"/>
       <c r="Z17" s="26" t="n"/>
       <c r="AA17" s="28" t="n"/>
       <c r="AB17" s="28" t="n"/>
-      <c r="AC17" s="30" t="n">
+      <c r="AC17" s="40" t="n">
         <v>0.9258999999999999</v>
       </c>
       <c r="AD17" s="24" t="inlineStr">
@@ -5838,11 +5869,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ17" s="25" t="n"/>
+      <c r="BJ17" s="38" t="n"/>
       <c r="BK17" s="26" t="n">
         <v>-108</v>
       </c>
-      <c r="BL17" s="27" t="n">
+      <c r="BL17" s="39" t="n">
         <v>1.925926</v>
       </c>
       <c r="BM17" s="28" t="n">
@@ -5852,18 +5883,18 @@
         <v>0.5148509999999999</v>
       </c>
       <c r="BO17" s="28" t="n"/>
-      <c r="BP17" s="25" t="n"/>
-      <c r="BQ17" s="27" t="n"/>
+      <c r="BP17" s="38" t="n"/>
+      <c r="BQ17" s="39" t="n"/>
       <c r="BR17" s="28" t="n"/>
       <c r="BS17" s="28" t="n"/>
       <c r="BT17" s="28" t="n"/>
-      <c r="BU17" s="25" t="n"/>
+      <c r="BU17" s="38" t="n"/>
       <c r="BV17" s="29" t="n"/>
       <c r="BW17" s="24" t="n"/>
-      <c r="BX17" s="30" t="n">
+      <c r="BX17" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="BY17" s="27" t="n">
+      <c r="BY17" s="39" t="n">
         <v>0.925926</v>
       </c>
       <c r="BZ17" s="24" t="inlineStr">
@@ -5923,7 +5954,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J18" s="25" t="n"/>
+      <c r="J18" s="38" t="n"/>
       <c r="K18" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -5932,7 +5963,7 @@
       <c r="L18" s="26" t="n">
         <v>111</v>
       </c>
-      <c r="M18" s="27" t="n">
+      <c r="M18" s="39" t="n">
         <v>2.11</v>
       </c>
       <c r="N18" s="28" t="n">
@@ -5972,11 +6003,11 @@
       <c r="X18" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="Y18" s="25" t="n"/>
+      <c r="Y18" s="38" t="n"/>
       <c r="Z18" s="26" t="n"/>
       <c r="AA18" s="28" t="n"/>
       <c r="AB18" s="28" t="n"/>
-      <c r="AC18" s="30" t="n">
+      <c r="AC18" s="40" t="n">
         <v>-1.25</v>
       </c>
       <c r="AD18" s="24" t="inlineStr">
@@ -6113,11 +6144,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ18" s="25" t="n"/>
+      <c r="BJ18" s="38" t="n"/>
       <c r="BK18" s="26" t="n">
         <v>111</v>
       </c>
-      <c r="BL18" s="27" t="n">
+      <c r="BL18" s="39" t="n">
         <v>2.11</v>
       </c>
       <c r="BM18" s="28" t="n">
@@ -6127,18 +6158,18 @@
         <v>0.472637</v>
       </c>
       <c r="BO18" s="28" t="n"/>
-      <c r="BP18" s="25" t="n"/>
-      <c r="BQ18" s="27" t="n"/>
+      <c r="BP18" s="38" t="n"/>
+      <c r="BQ18" s="39" t="n"/>
       <c r="BR18" s="28" t="n"/>
       <c r="BS18" s="28" t="n"/>
       <c r="BT18" s="28" t="n"/>
-      <c r="BU18" s="25" t="n"/>
+      <c r="BU18" s="38" t="n"/>
       <c r="BV18" s="29" t="n"/>
       <c r="BW18" s="24" t="n"/>
-      <c r="BX18" s="30" t="n">
+      <c r="BX18" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="BY18" s="27" t="n">
+      <c r="BY18" s="39" t="n">
         <v>-1</v>
       </c>
       <c r="BZ18" s="24" t="inlineStr">
@@ -6198,7 +6229,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J19" s="25" t="n"/>
+      <c r="J19" s="38" t="n"/>
       <c r="K19" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -6207,7 +6238,7 @@
       <c r="L19" s="26" t="n">
         <v>-125</v>
       </c>
-      <c r="M19" s="27" t="n">
+      <c r="M19" s="39" t="n">
         <v>1.8</v>
       </c>
       <c r="N19" s="28" t="n">
@@ -6247,11 +6278,11 @@
       <c r="X19" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="Y19" s="25" t="n"/>
+      <c r="Y19" s="38" t="n"/>
       <c r="Z19" s="26" t="n"/>
       <c r="AA19" s="28" t="n"/>
       <c r="AB19" s="28" t="n"/>
-      <c r="AC19" s="30" t="n">
+      <c r="AC19" s="40" t="n">
         <v>1.2</v>
       </c>
       <c r="AD19" s="24" t="inlineStr">
@@ -6388,11 +6419,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ19" s="25" t="n"/>
+      <c r="BJ19" s="38" t="n"/>
       <c r="BK19" s="26" t="n">
         <v>-125</v>
       </c>
-      <c r="BL19" s="27" t="n">
+      <c r="BL19" s="39" t="n">
         <v>1.8</v>
       </c>
       <c r="BM19" s="28" t="n">
@@ -6402,18 +6433,18 @@
         <v>0.552239</v>
       </c>
       <c r="BO19" s="28" t="n"/>
-      <c r="BP19" s="25" t="n"/>
-      <c r="BQ19" s="27" t="n"/>
+      <c r="BP19" s="38" t="n"/>
+      <c r="BQ19" s="39" t="n"/>
       <c r="BR19" s="28" t="n"/>
       <c r="BS19" s="28" t="n"/>
       <c r="BT19" s="28" t="n"/>
-      <c r="BU19" s="25" t="n"/>
+      <c r="BU19" s="38" t="n"/>
       <c r="BV19" s="29" t="n"/>
       <c r="BW19" s="24" t="n"/>
-      <c r="BX19" s="30" t="n">
+      <c r="BX19" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="BY19" s="27" t="n">
+      <c r="BY19" s="39" t="n">
         <v>0.8</v>
       </c>
       <c r="BZ19" s="24" t="inlineStr">
@@ -6473,7 +6504,7 @@
           <t>away</t>
         </is>
       </c>
-      <c r="J20" s="25" t="n"/>
+      <c r="J20" s="38" t="n"/>
       <c r="K20" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -6482,7 +6513,7 @@
       <c r="L20" s="26" t="n">
         <v>106</v>
       </c>
-      <c r="M20" s="27" t="n">
+      <c r="M20" s="39" t="n">
         <v>2.06</v>
       </c>
       <c r="N20" s="28" t="n">
@@ -6522,11 +6553,11 @@
       <c r="X20" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="Y20" s="25" t="n"/>
+      <c r="Y20" s="38" t="n"/>
       <c r="Z20" s="26" t="n"/>
       <c r="AA20" s="28" t="n"/>
       <c r="AB20" s="28" t="n"/>
-      <c r="AC20" s="30" t="n">
+      <c r="AC20" s="40" t="n">
         <v>0.795</v>
       </c>
       <c r="AD20" s="24" t="inlineStr">
@@ -6663,11 +6694,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ20" s="25" t="n"/>
+      <c r="BJ20" s="38" t="n"/>
       <c r="BK20" s="26" t="n">
         <v>106</v>
       </c>
-      <c r="BL20" s="27" t="n">
+      <c r="BL20" s="39" t="n">
         <v>2.06</v>
       </c>
       <c r="BM20" s="28" t="n">
@@ -6677,18 +6708,18 @@
         <v>0.482587</v>
       </c>
       <c r="BO20" s="28" t="n"/>
-      <c r="BP20" s="25" t="n"/>
-      <c r="BQ20" s="27" t="n"/>
+      <c r="BP20" s="38" t="n"/>
+      <c r="BQ20" s="39" t="n"/>
       <c r="BR20" s="28" t="n"/>
       <c r="BS20" s="28" t="n"/>
       <c r="BT20" s="28" t="n"/>
-      <c r="BU20" s="25" t="n"/>
+      <c r="BU20" s="38" t="n"/>
       <c r="BV20" s="29" t="n"/>
       <c r="BW20" s="24" t="n"/>
-      <c r="BX20" s="30" t="n">
+      <c r="BX20" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="BY20" s="27" t="n">
+      <c r="BY20" s="39" t="n">
         <v>1.06</v>
       </c>
       <c r="BZ20" s="24" t="inlineStr">
@@ -6748,7 +6779,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J21" s="25" t="n"/>
+      <c r="J21" s="38" t="n"/>
       <c r="K21" s="24" t="inlineStr">
         <is>
           <t>polymarket</t>
@@ -6757,7 +6788,7 @@
       <c r="L21" s="26" t="n">
         <v>-106</v>
       </c>
-      <c r="M21" s="27" t="n">
+      <c r="M21" s="39" t="n">
         <v>1.943396</v>
       </c>
       <c r="N21" s="28" t="n">
@@ -6799,11 +6830,11 @@
       <c r="X21" s="26" t="n">
         <v>10</v>
       </c>
-      <c r="Y21" s="25" t="n"/>
+      <c r="Y21" s="38" t="n"/>
       <c r="Z21" s="26" t="n"/>
       <c r="AA21" s="28" t="n"/>
       <c r="AB21" s="28" t="n"/>
-      <c r="AC21" s="30" t="n">
+      <c r="AC21" s="40" t="n">
         <v>0.9434</v>
       </c>
       <c r="AD21" s="24" t="inlineStr">
@@ -6862,11 +6893,11 @@
         </is>
       </c>
       <c r="BI21" s="24" t="n"/>
-      <c r="BJ21" s="25" t="n"/>
+      <c r="BJ21" s="38" t="n"/>
       <c r="BK21" s="26" t="n">
         <v>-106</v>
       </c>
-      <c r="BL21" s="27" t="n">
+      <c r="BL21" s="39" t="n">
         <v>1.943396</v>
       </c>
       <c r="BM21" s="28" t="n">
@@ -6876,16 +6907,16 @@
         <v>0.5124379999999999</v>
       </c>
       <c r="BO21" s="28" t="n"/>
-      <c r="BP21" s="25" t="n"/>
-      <c r="BQ21" s="27" t="n"/>
+      <c r="BP21" s="38" t="n"/>
+      <c r="BQ21" s="39" t="n"/>
       <c r="BR21" s="28" t="n"/>
       <c r="BS21" s="28" t="n"/>
       <c r="BT21" s="28" t="n"/>
-      <c r="BU21" s="25" t="n"/>
+      <c r="BU21" s="38" t="n"/>
       <c r="BV21" s="29" t="n"/>
       <c r="BW21" s="24" t="n"/>
-      <c r="BX21" s="30" t="n"/>
-      <c r="BY21" s="27" t="n"/>
+      <c r="BX21" s="40" t="n"/>
+      <c r="BY21" s="39" t="n"/>
       <c r="BZ21" s="24" t="n"/>
       <c r="CA21" s="31" t="n"/>
     </row>
@@ -6935,7 +6966,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J22" s="25" t="n"/>
+      <c r="J22" s="38" t="n"/>
       <c r="K22" s="24" t="inlineStr">
         <is>
           <t>polymarket</t>
@@ -6944,7 +6975,7 @@
       <c r="L22" s="26" t="n">
         <v>-106</v>
       </c>
-      <c r="M22" s="27" t="n">
+      <c r="M22" s="39" t="n">
         <v>1.943396</v>
       </c>
       <c r="N22" s="28" t="n">
@@ -6986,11 +7017,11 @@
       <c r="X22" s="26" t="n">
         <v>5</v>
       </c>
-      <c r="Y22" s="25" t="n"/>
+      <c r="Y22" s="38" t="n"/>
       <c r="Z22" s="26" t="n"/>
       <c r="AA22" s="28" t="n"/>
       <c r="AB22" s="28" t="n"/>
-      <c r="AC22" s="30" t="n">
+      <c r="AC22" s="40" t="n">
         <v>0.9434</v>
       </c>
       <c r="AD22" s="24" t="inlineStr">
@@ -7049,11 +7080,11 @@
         </is>
       </c>
       <c r="BI22" s="24" t="n"/>
-      <c r="BJ22" s="25" t="n"/>
+      <c r="BJ22" s="38" t="n"/>
       <c r="BK22" s="26" t="n">
         <v>-106</v>
       </c>
-      <c r="BL22" s="27" t="n">
+      <c r="BL22" s="39" t="n">
         <v>1.943396</v>
       </c>
       <c r="BM22" s="28" t="n">
@@ -7063,16 +7094,16 @@
         <v>0.5124379999999999</v>
       </c>
       <c r="BO22" s="28" t="n"/>
-      <c r="BP22" s="25" t="n"/>
-      <c r="BQ22" s="27" t="n"/>
+      <c r="BP22" s="38" t="n"/>
+      <c r="BQ22" s="39" t="n"/>
       <c r="BR22" s="28" t="n"/>
       <c r="BS22" s="28" t="n"/>
       <c r="BT22" s="28" t="n"/>
-      <c r="BU22" s="25" t="n"/>
+      <c r="BU22" s="38" t="n"/>
       <c r="BV22" s="29" t="n"/>
       <c r="BW22" s="24" t="n"/>
-      <c r="BX22" s="30" t="n"/>
-      <c r="BY22" s="27" t="n"/>
+      <c r="BX22" s="40" t="n"/>
+      <c r="BY22" s="39" t="n"/>
       <c r="BZ22" s="24" t="n"/>
       <c r="CA22" s="31" t="n"/>
     </row>
@@ -7122,7 +7153,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J23" s="25" t="n"/>
+      <c r="J23" s="38" t="n"/>
       <c r="K23" s="24" t="inlineStr">
         <is>
           <t>polymarket</t>
@@ -7131,7 +7162,7 @@
       <c r="L23" s="26" t="n">
         <v>-141</v>
       </c>
-      <c r="M23" s="27" t="n">
+      <c r="M23" s="39" t="n">
         <v>1.70922</v>
       </c>
       <c r="N23" s="28" t="n">
@@ -7173,11 +7204,11 @@
       <c r="X23" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="Y23" s="25" t="n"/>
+      <c r="Y23" s="38" t="n"/>
       <c r="Z23" s="26" t="n"/>
       <c r="AA23" s="28" t="n"/>
       <c r="AB23" s="28" t="n"/>
-      <c r="AC23" s="30" t="n">
+      <c r="AC23" s="40" t="n">
         <v>1.2411</v>
       </c>
       <c r="AD23" s="24" t="inlineStr">
@@ -7236,11 +7267,11 @@
         </is>
       </c>
       <c r="BI23" s="24" t="n"/>
-      <c r="BJ23" s="25" t="n"/>
+      <c r="BJ23" s="38" t="n"/>
       <c r="BK23" s="26" t="n">
         <v>-141</v>
       </c>
-      <c r="BL23" s="27" t="n">
+      <c r="BL23" s="39" t="n">
         <v>1.70922</v>
       </c>
       <c r="BM23" s="28" t="n">
@@ -7250,16 +7281,16 @@
         <v>0.58209</v>
       </c>
       <c r="BO23" s="28" t="n"/>
-      <c r="BP23" s="25" t="n"/>
-      <c r="BQ23" s="27" t="n"/>
+      <c r="BP23" s="38" t="n"/>
+      <c r="BQ23" s="39" t="n"/>
       <c r="BR23" s="28" t="n"/>
       <c r="BS23" s="28" t="n"/>
       <c r="BT23" s="28" t="n"/>
-      <c r="BU23" s="25" t="n"/>
+      <c r="BU23" s="38" t="n"/>
       <c r="BV23" s="29" t="n"/>
       <c r="BW23" s="24" t="n"/>
-      <c r="BX23" s="30" t="n"/>
-      <c r="BY23" s="27" t="n"/>
+      <c r="BX23" s="40" t="n"/>
+      <c r="BY23" s="39" t="n"/>
       <c r="BZ23" s="24" t="n"/>
       <c r="CA23" s="31" t="n"/>
     </row>
@@ -7309,7 +7340,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J24" s="25" t="n"/>
+      <c r="J24" s="38" t="n"/>
       <c r="K24" s="24" t="inlineStr">
         <is>
           <t>polymarket</t>
@@ -7318,7 +7349,7 @@
       <c r="L24" s="26" t="n">
         <v>-133</v>
       </c>
-      <c r="M24" s="27" t="n">
+      <c r="M24" s="39" t="n">
         <v>1.75188</v>
       </c>
       <c r="N24" s="28" t="n">
@@ -7360,11 +7391,11 @@
       <c r="X24" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="Y24" s="25" t="n"/>
+      <c r="Y24" s="38" t="n"/>
       <c r="Z24" s="26" t="n"/>
       <c r="AA24" s="28" t="n"/>
       <c r="AB24" s="28" t="n"/>
-      <c r="AC24" s="30" t="n">
+      <c r="AC24" s="40" t="n">
         <v>-1.5</v>
       </c>
       <c r="AD24" s="24" t="inlineStr">
@@ -7423,11 +7454,11 @@
         </is>
       </c>
       <c r="BI24" s="24" t="n"/>
-      <c r="BJ24" s="25" t="n"/>
+      <c r="BJ24" s="38" t="n"/>
       <c r="BK24" s="26" t="n">
         <v>-133</v>
       </c>
-      <c r="BL24" s="27" t="n">
+      <c r="BL24" s="39" t="n">
         <v>1.75188</v>
       </c>
       <c r="BM24" s="28" t="n">
@@ -7437,16 +7468,16 @@
         <v>0.567164</v>
       </c>
       <c r="BO24" s="28" t="n"/>
-      <c r="BP24" s="25" t="n"/>
-      <c r="BQ24" s="27" t="n"/>
+      <c r="BP24" s="38" t="n"/>
+      <c r="BQ24" s="39" t="n"/>
       <c r="BR24" s="28" t="n"/>
       <c r="BS24" s="28" t="n"/>
       <c r="BT24" s="28" t="n"/>
-      <c r="BU24" s="25" t="n"/>
+      <c r="BU24" s="38" t="n"/>
       <c r="BV24" s="29" t="n"/>
       <c r="BW24" s="24" t="n"/>
-      <c r="BX24" s="30" t="n"/>
-      <c r="BY24" s="27" t="n"/>
+      <c r="BX24" s="40" t="n"/>
+      <c r="BY24" s="39" t="n"/>
       <c r="BZ24" s="24" t="n"/>
       <c r="CA24" s="31" t="n"/>
     </row>
@@ -7496,7 +7527,7 @@
           <t>away</t>
         </is>
       </c>
-      <c r="J25" s="25" t="n"/>
+      <c r="J25" s="38" t="n"/>
       <c r="K25" s="24" t="inlineStr">
         <is>
           <t>polymarket</t>
@@ -7505,7 +7536,7 @@
       <c r="L25" s="26" t="n">
         <v>104</v>
       </c>
-      <c r="M25" s="27" t="n">
+      <c r="M25" s="39" t="n">
         <v>2.04</v>
       </c>
       <c r="N25" s="28" t="n">
@@ -7547,11 +7578,11 @@
       <c r="X25" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="Y25" s="25" t="n"/>
+      <c r="Y25" s="38" t="n"/>
       <c r="Z25" s="26" t="n"/>
       <c r="AA25" s="28" t="n"/>
       <c r="AB25" s="28" t="n"/>
-      <c r="AC25" s="30" t="n">
+      <c r="AC25" s="40" t="n">
         <v>1.3</v>
       </c>
       <c r="AD25" s="24" t="inlineStr">
@@ -7610,11 +7641,11 @@
         </is>
       </c>
       <c r="BI25" s="24" t="n"/>
-      <c r="BJ25" s="25" t="n"/>
+      <c r="BJ25" s="38" t="n"/>
       <c r="BK25" s="26" t="n">
         <v>104</v>
       </c>
-      <c r="BL25" s="27" t="n">
+      <c r="BL25" s="39" t="n">
         <v>2.04</v>
       </c>
       <c r="BM25" s="28" t="n">
@@ -7624,16 +7655,16 @@
         <v>0.487562</v>
       </c>
       <c r="BO25" s="28" t="n"/>
-      <c r="BP25" s="25" t="n"/>
-      <c r="BQ25" s="27" t="n"/>
+      <c r="BP25" s="38" t="n"/>
+      <c r="BQ25" s="39" t="n"/>
       <c r="BR25" s="28" t="n"/>
       <c r="BS25" s="28" t="n"/>
       <c r="BT25" s="28" t="n"/>
-      <c r="BU25" s="25" t="n"/>
+      <c r="BU25" s="38" t="n"/>
       <c r="BV25" s="29" t="n"/>
       <c r="BW25" s="24" t="n"/>
-      <c r="BX25" s="30" t="n"/>
-      <c r="BY25" s="27" t="n"/>
+      <c r="BX25" s="40" t="n"/>
+      <c r="BY25" s="39" t="n"/>
       <c r="BZ25" s="24" t="n"/>
       <c r="CA25" s="31" t="n"/>
     </row>
@@ -7683,7 +7714,7 @@
           <t>away</t>
         </is>
       </c>
-      <c r="J26" s="25" t="n"/>
+      <c r="J26" s="38" t="n"/>
       <c r="K26" s="24" t="inlineStr">
         <is>
           <t>polymarket</t>
@@ -7692,7 +7723,7 @@
       <c r="L26" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="M26" s="27" t="n">
+      <c r="M26" s="39" t="n">
         <v>1.961538</v>
       </c>
       <c r="N26" s="28" t="n">
@@ -7734,11 +7765,11 @@
       <c r="X26" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="Y26" s="25" t="n"/>
+      <c r="Y26" s="38" t="n"/>
       <c r="Z26" s="26" t="n"/>
       <c r="AA26" s="28" t="n"/>
       <c r="AB26" s="28" t="n"/>
-      <c r="AC26" s="30" t="n">
+      <c r="AC26" s="40" t="n">
         <v>0.9615</v>
       </c>
       <c r="AD26" s="24" t="inlineStr">
@@ -7797,11 +7828,11 @@
         </is>
       </c>
       <c r="BI26" s="24" t="n"/>
-      <c r="BJ26" s="25" t="n"/>
+      <c r="BJ26" s="38" t="n"/>
       <c r="BK26" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="BL26" s="27" t="n">
+      <c r="BL26" s="39" t="n">
         <v>1.961538</v>
       </c>
       <c r="BM26" s="28" t="n">
@@ -7811,16 +7842,16 @@
         <v>0.507463</v>
       </c>
       <c r="BO26" s="28" t="n"/>
-      <c r="BP26" s="25" t="n"/>
-      <c r="BQ26" s="27" t="n"/>
+      <c r="BP26" s="38" t="n"/>
+      <c r="BQ26" s="39" t="n"/>
       <c r="BR26" s="28" t="n"/>
       <c r="BS26" s="28" t="n"/>
       <c r="BT26" s="28" t="n"/>
-      <c r="BU26" s="25" t="n"/>
+      <c r="BU26" s="38" t="n"/>
       <c r="BV26" s="29" t="n"/>
       <c r="BW26" s="24" t="n"/>
-      <c r="BX26" s="30" t="n"/>
-      <c r="BY26" s="27" t="n"/>
+      <c r="BX26" s="40" t="n"/>
+      <c r="BY26" s="39" t="n"/>
       <c r="BZ26" s="24" t="n"/>
       <c r="CA26" s="31" t="n"/>
     </row>
@@ -7870,7 +7901,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J27" s="25" t="n"/>
+      <c r="J27" s="38" t="n"/>
       <c r="K27" s="24" t="inlineStr">
         <is>
           <t>polymarket</t>
@@ -7879,7 +7910,7 @@
       <c r="L27" s="26" t="n">
         <v>120</v>
       </c>
-      <c r="M27" s="27" t="n">
+      <c r="M27" s="39" t="n">
         <v>2.2</v>
       </c>
       <c r="N27" s="28" t="n">
@@ -7921,11 +7952,11 @@
       <c r="X27" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="Y27" s="25" t="n"/>
+      <c r="Y27" s="38" t="n"/>
       <c r="Z27" s="26" t="n"/>
       <c r="AA27" s="28" t="n"/>
       <c r="AB27" s="28" t="n"/>
-      <c r="AC27" s="30" t="n">
+      <c r="AC27" s="40" t="n">
         <v>-0.75</v>
       </c>
       <c r="AD27" s="24" t="inlineStr">
@@ -7984,11 +8015,11 @@
         </is>
       </c>
       <c r="BI27" s="24" t="n"/>
-      <c r="BJ27" s="25" t="n"/>
+      <c r="BJ27" s="38" t="n"/>
       <c r="BK27" s="26" t="n">
         <v>120</v>
       </c>
-      <c r="BL27" s="27" t="n">
+      <c r="BL27" s="39" t="n">
         <v>2.2</v>
       </c>
       <c r="BM27" s="28" t="n">
@@ -7998,16 +8029,16 @@
         <v>0.452736</v>
       </c>
       <c r="BO27" s="28" t="n"/>
-      <c r="BP27" s="25" t="n"/>
-      <c r="BQ27" s="27" t="n"/>
+      <c r="BP27" s="38" t="n"/>
+      <c r="BQ27" s="39" t="n"/>
       <c r="BR27" s="28" t="n"/>
       <c r="BS27" s="28" t="n"/>
       <c r="BT27" s="28" t="n"/>
-      <c r="BU27" s="25" t="n"/>
+      <c r="BU27" s="38" t="n"/>
       <c r="BV27" s="29" t="n"/>
       <c r="BW27" s="24" t="n"/>
-      <c r="BX27" s="30" t="n"/>
-      <c r="BY27" s="27" t="n"/>
+      <c r="BX27" s="40" t="n"/>
+      <c r="BY27" s="39" t="n"/>
       <c r="BZ27" s="24" t="n"/>
       <c r="CA27" s="31" t="n"/>
     </row>
@@ -8057,7 +8088,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J28" s="25" t="n"/>
+      <c r="J28" s="38" t="n"/>
       <c r="K28" s="24" t="inlineStr">
         <is>
           <t>polymarket</t>
@@ -8066,7 +8097,7 @@
       <c r="L28" s="26" t="n">
         <v>100</v>
       </c>
-      <c r="M28" s="27" t="n">
+      <c r="M28" s="39" t="n">
         <v>2</v>
       </c>
       <c r="N28" s="28" t="n">
@@ -8108,11 +8139,11 @@
       <c r="X28" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="Y28" s="25" t="n"/>
+      <c r="Y28" s="38" t="n"/>
       <c r="Z28" s="26" t="n"/>
       <c r="AA28" s="28" t="n"/>
       <c r="AB28" s="28" t="n"/>
-      <c r="AC28" s="30" t="n">
+      <c r="AC28" s="40" t="n">
         <v>-0.75</v>
       </c>
       <c r="AD28" s="24" t="inlineStr">
@@ -8171,11 +8202,11 @@
         </is>
       </c>
       <c r="BI28" s="24" t="n"/>
-      <c r="BJ28" s="25" t="n"/>
+      <c r="BJ28" s="38" t="n"/>
       <c r="BK28" s="26" t="n">
         <v>100</v>
       </c>
-      <c r="BL28" s="27" t="n">
+      <c r="BL28" s="39" t="n">
         <v>2</v>
       </c>
       <c r="BM28" s="28" t="n">
@@ -8185,16 +8216,16 @@
         <v>0.497512</v>
       </c>
       <c r="BO28" s="28" t="n"/>
-      <c r="BP28" s="25" t="n"/>
-      <c r="BQ28" s="27" t="n"/>
+      <c r="BP28" s="38" t="n"/>
+      <c r="BQ28" s="39" t="n"/>
       <c r="BR28" s="28" t="n"/>
       <c r="BS28" s="28" t="n"/>
       <c r="BT28" s="28" t="n"/>
-      <c r="BU28" s="25" t="n"/>
+      <c r="BU28" s="38" t="n"/>
       <c r="BV28" s="29" t="n"/>
       <c r="BW28" s="24" t="n"/>
-      <c r="BX28" s="30" t="n"/>
-      <c r="BY28" s="27" t="n"/>
+      <c r="BX28" s="40" t="n"/>
+      <c r="BY28" s="39" t="n"/>
       <c r="BZ28" s="24" t="n"/>
       <c r="CA28" s="31" t="n"/>
     </row>
@@ -8244,7 +8275,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J29" s="25" t="n"/>
+      <c r="J29" s="38" t="n"/>
       <c r="K29" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -8253,7 +8284,7 @@
       <c r="L29" s="26" t="n">
         <v>108</v>
       </c>
-      <c r="M29" s="27" t="n">
+      <c r="M29" s="39" t="n">
         <v>2.08</v>
       </c>
       <c r="N29" s="28" t="n">
@@ -8293,11 +8324,11 @@
       <c r="X29" s="26" t="n">
         <v>8</v>
       </c>
-      <c r="Y29" s="25" t="n"/>
+      <c r="Y29" s="38" t="n"/>
       <c r="Z29" s="26" t="n"/>
       <c r="AA29" s="28" t="n"/>
       <c r="AB29" s="28" t="n"/>
-      <c r="AC29" s="30" t="n">
+      <c r="AC29" s="40" t="n">
         <v>1.35</v>
       </c>
       <c r="AD29" s="24" t="inlineStr">
@@ -8434,11 +8465,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ29" s="25" t="n"/>
+      <c r="BJ29" s="38" t="n"/>
       <c r="BK29" s="26" t="n">
         <v>108</v>
       </c>
-      <c r="BL29" s="27" t="n">
+      <c r="BL29" s="39" t="n">
         <v>2.08</v>
       </c>
       <c r="BM29" s="28" t="n">
@@ -8448,18 +8479,18 @@
         <v>0.477612</v>
       </c>
       <c r="BO29" s="28" t="n"/>
-      <c r="BP29" s="25" t="n"/>
-      <c r="BQ29" s="27" t="n"/>
+      <c r="BP29" s="38" t="n"/>
+      <c r="BQ29" s="39" t="n"/>
       <c r="BR29" s="28" t="n"/>
       <c r="BS29" s="28" t="n"/>
       <c r="BT29" s="28" t="n"/>
-      <c r="BU29" s="25" t="n"/>
+      <c r="BU29" s="38" t="n"/>
       <c r="BV29" s="29" t="n"/>
       <c r="BW29" s="24" t="n"/>
-      <c r="BX29" s="30" t="n">
+      <c r="BX29" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="BY29" s="27" t="n">
+      <c r="BY29" s="39" t="n">
         <v>1.08</v>
       </c>
       <c r="BZ29" s="24" t="inlineStr">
@@ -8519,7 +8550,7 @@
           <t>away</t>
         </is>
       </c>
-      <c r="J30" s="25" t="n"/>
+      <c r="J30" s="38" t="n"/>
       <c r="K30" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -8528,7 +8559,7 @@
       <c r="L30" s="26" t="n">
         <v>-133</v>
       </c>
-      <c r="M30" s="27" t="n">
+      <c r="M30" s="39" t="n">
         <v>1.75188</v>
       </c>
       <c r="N30" s="28" t="n">
@@ -8568,11 +8599,11 @@
       <c r="X30" s="26" t="n">
         <v>6</v>
       </c>
-      <c r="Y30" s="25" t="n"/>
+      <c r="Y30" s="38" t="n"/>
       <c r="Z30" s="26" t="n"/>
       <c r="AA30" s="28" t="n"/>
       <c r="AB30" s="28" t="n"/>
-      <c r="AC30" s="30" t="n">
+      <c r="AC30" s="40" t="n">
         <v>1.1278</v>
       </c>
       <c r="AD30" s="24" t="inlineStr">
@@ -8709,11 +8740,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ30" s="25" t="n"/>
+      <c r="BJ30" s="38" t="n"/>
       <c r="BK30" s="26" t="n">
         <v>-133</v>
       </c>
-      <c r="BL30" s="27" t="n">
+      <c r="BL30" s="39" t="n">
         <v>1.75188</v>
       </c>
       <c r="BM30" s="28" t="n">
@@ -8723,18 +8754,18 @@
         <v>0.567164</v>
       </c>
       <c r="BO30" s="28" t="n"/>
-      <c r="BP30" s="25" t="n"/>
-      <c r="BQ30" s="27" t="n"/>
+      <c r="BP30" s="38" t="n"/>
+      <c r="BQ30" s="39" t="n"/>
       <c r="BR30" s="28" t="n"/>
       <c r="BS30" s="28" t="n"/>
       <c r="BT30" s="28" t="n"/>
-      <c r="BU30" s="25" t="n"/>
+      <c r="BU30" s="38" t="n"/>
       <c r="BV30" s="29" t="n"/>
       <c r="BW30" s="24" t="n"/>
-      <c r="BX30" s="30" t="n">
+      <c r="BX30" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="BY30" s="27" t="n">
+      <c r="BY30" s="39" t="n">
         <v>0.75188</v>
       </c>
       <c r="BZ30" s="24" t="inlineStr">
@@ -8794,7 +8825,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J31" s="25" t="n"/>
+      <c r="J31" s="38" t="n"/>
       <c r="K31" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -8803,7 +8834,7 @@
       <c r="L31" s="26" t="n">
         <v>130</v>
       </c>
-      <c r="M31" s="27" t="n">
+      <c r="M31" s="39" t="n">
         <v>2.3</v>
       </c>
       <c r="N31" s="28" t="n">
@@ -8843,11 +8874,11 @@
       <c r="X31" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="Y31" s="25" t="n"/>
+      <c r="Y31" s="38" t="n"/>
       <c r="Z31" s="26" t="n"/>
       <c r="AA31" s="28" t="n"/>
       <c r="AB31" s="28" t="n"/>
-      <c r="AC31" s="30" t="n">
+      <c r="AC31" s="40" t="n">
         <v>-1</v>
       </c>
       <c r="AD31" s="24" t="inlineStr">
@@ -8984,11 +9015,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ31" s="25" t="n"/>
+      <c r="BJ31" s="38" t="n"/>
       <c r="BK31" s="26" t="n">
         <v>130</v>
       </c>
-      <c r="BL31" s="27" t="n">
+      <c r="BL31" s="39" t="n">
         <v>2.3</v>
       </c>
       <c r="BM31" s="28" t="n">
@@ -8998,18 +9029,18 @@
         <v>0.432836</v>
       </c>
       <c r="BO31" s="28" t="n"/>
-      <c r="BP31" s="25" t="n"/>
-      <c r="BQ31" s="27" t="n"/>
+      <c r="BP31" s="38" t="n"/>
+      <c r="BQ31" s="39" t="n"/>
       <c r="BR31" s="28" t="n"/>
       <c r="BS31" s="28" t="n"/>
       <c r="BT31" s="28" t="n"/>
-      <c r="BU31" s="25" t="n"/>
+      <c r="BU31" s="38" t="n"/>
       <c r="BV31" s="29" t="n"/>
       <c r="BW31" s="24" t="n"/>
-      <c r="BX31" s="30" t="n">
+      <c r="BX31" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="BY31" s="27" t="n">
+      <c r="BY31" s="39" t="n">
         <v>-1</v>
       </c>
       <c r="BZ31" s="24" t="inlineStr">
@@ -9069,7 +9100,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J32" s="25" t="n"/>
+      <c r="J32" s="38" t="n"/>
       <c r="K32" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -9078,7 +9109,7 @@
       <c r="L32" s="26" t="n">
         <v>113</v>
       </c>
-      <c r="M32" s="27" t="n">
+      <c r="M32" s="39" t="n">
         <v>2.13</v>
       </c>
       <c r="N32" s="28" t="n">
@@ -9110,11 +9141,11 @@
       <c r="V32" s="24" t="n"/>
       <c r="W32" s="26" t="n"/>
       <c r="X32" s="26" t="n"/>
-      <c r="Y32" s="25" t="n"/>
+      <c r="Y32" s="38" t="n"/>
       <c r="Z32" s="26" t="n"/>
       <c r="AA32" s="28" t="n"/>
       <c r="AB32" s="28" t="n"/>
-      <c r="AC32" s="30" t="n"/>
+      <c r="AC32" s="40" t="n"/>
       <c r="AD32" s="24" t="n"/>
       <c r="AE32" s="31" t="inlineStr">
         <is>
@@ -9245,11 +9276,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ32" s="25" t="n"/>
+      <c r="BJ32" s="38" t="n"/>
       <c r="BK32" s="26" t="n">
         <v>113</v>
       </c>
-      <c r="BL32" s="27" t="n">
+      <c r="BL32" s="39" t="n">
         <v>2.13</v>
       </c>
       <c r="BM32" s="28" t="n">
@@ -9259,16 +9290,16 @@
         <v>0.467662</v>
       </c>
       <c r="BO32" s="28" t="n"/>
-      <c r="BP32" s="25" t="n"/>
-      <c r="BQ32" s="27" t="n"/>
+      <c r="BP32" s="38" t="n"/>
+      <c r="BQ32" s="39" t="n"/>
       <c r="BR32" s="28" t="n"/>
       <c r="BS32" s="28" t="n"/>
       <c r="BT32" s="28" t="n"/>
-      <c r="BU32" s="25" t="n"/>
+      <c r="BU32" s="38" t="n"/>
       <c r="BV32" s="29" t="n"/>
       <c r="BW32" s="24" t="n"/>
-      <c r="BX32" s="30" t="n"/>
-      <c r="BY32" s="27" t="n"/>
+      <c r="BX32" s="40" t="n"/>
+      <c r="BY32" s="39" t="n"/>
       <c r="BZ32" s="24" t="n"/>
       <c r="CA32" s="31" t="n"/>
     </row>
@@ -9318,7 +9349,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J33" s="25" t="n"/>
+      <c r="J33" s="38" t="n"/>
       <c r="K33" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -9327,7 +9358,7 @@
       <c r="L33" s="26" t="n">
         <v>-108</v>
       </c>
-      <c r="M33" s="27" t="n">
+      <c r="M33" s="39" t="n">
         <v>1.925926</v>
       </c>
       <c r="N33" s="28" t="n">
@@ -9359,11 +9390,11 @@
       <c r="V33" s="24" t="n"/>
       <c r="W33" s="26" t="n"/>
       <c r="X33" s="26" t="n"/>
-      <c r="Y33" s="25" t="n"/>
+      <c r="Y33" s="38" t="n"/>
       <c r="Z33" s="26" t="n"/>
       <c r="AA33" s="28" t="n"/>
       <c r="AB33" s="28" t="n"/>
-      <c r="AC33" s="30" t="n"/>
+      <c r="AC33" s="40" t="n"/>
       <c r="AD33" s="24" t="n"/>
       <c r="AE33" s="31" t="inlineStr">
         <is>
@@ -9494,11 +9525,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ33" s="25" t="n"/>
+      <c r="BJ33" s="38" t="n"/>
       <c r="BK33" s="26" t="n">
         <v>-108</v>
       </c>
-      <c r="BL33" s="27" t="n">
+      <c r="BL33" s="39" t="n">
         <v>1.925926</v>
       </c>
       <c r="BM33" s="28" t="n">
@@ -9508,16 +9539,16 @@
         <v>0.517413</v>
       </c>
       <c r="BO33" s="28" t="n"/>
-      <c r="BP33" s="25" t="n"/>
-      <c r="BQ33" s="27" t="n"/>
+      <c r="BP33" s="38" t="n"/>
+      <c r="BQ33" s="39" t="n"/>
       <c r="BR33" s="28" t="n"/>
       <c r="BS33" s="28" t="n"/>
       <c r="BT33" s="28" t="n"/>
-      <c r="BU33" s="25" t="n"/>
+      <c r="BU33" s="38" t="n"/>
       <c r="BV33" s="29" t="n"/>
       <c r="BW33" s="24" t="n"/>
-      <c r="BX33" s="30" t="n"/>
-      <c r="BY33" s="27" t="n"/>
+      <c r="BX33" s="40" t="n"/>
+      <c r="BY33" s="39" t="n"/>
       <c r="BZ33" s="24" t="n"/>
       <c r="CA33" s="31" t="n"/>
     </row>
@@ -9567,7 +9598,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J34" s="25" t="n"/>
+      <c r="J34" s="38" t="n"/>
       <c r="K34" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -9576,7 +9607,7 @@
       <c r="L34" s="26" t="n">
         <v>-108</v>
       </c>
-      <c r="M34" s="27" t="n">
+      <c r="M34" s="39" t="n">
         <v>1.925926</v>
       </c>
       <c r="N34" s="28" t="n">
@@ -9608,11 +9639,11 @@
       <c r="V34" s="24" t="n"/>
       <c r="W34" s="26" t="n"/>
       <c r="X34" s="26" t="n"/>
-      <c r="Y34" s="25" t="n"/>
+      <c r="Y34" s="38" t="n"/>
       <c r="Z34" s="26" t="n"/>
       <c r="AA34" s="28" t="n"/>
       <c r="AB34" s="28" t="n"/>
-      <c r="AC34" s="30" t="n"/>
+      <c r="AC34" s="40" t="n"/>
       <c r="AD34" s="24" t="n"/>
       <c r="AE34" s="31" t="inlineStr">
         <is>
@@ -9743,11 +9774,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ34" s="25" t="n"/>
+      <c r="BJ34" s="38" t="n"/>
       <c r="BK34" s="26" t="n">
         <v>-108</v>
       </c>
-      <c r="BL34" s="27" t="n">
+      <c r="BL34" s="39" t="n">
         <v>1.925926</v>
       </c>
       <c r="BM34" s="28" t="n">
@@ -9757,16 +9788,16 @@
         <v>0.5148509999999999</v>
       </c>
       <c r="BO34" s="28" t="n"/>
-      <c r="BP34" s="25" t="n"/>
-      <c r="BQ34" s="27" t="n"/>
+      <c r="BP34" s="38" t="n"/>
+      <c r="BQ34" s="39" t="n"/>
       <c r="BR34" s="28" t="n"/>
       <c r="BS34" s="28" t="n"/>
       <c r="BT34" s="28" t="n"/>
-      <c r="BU34" s="25" t="n"/>
+      <c r="BU34" s="38" t="n"/>
       <c r="BV34" s="29" t="n"/>
       <c r="BW34" s="24" t="n"/>
-      <c r="BX34" s="30" t="n"/>
-      <c r="BY34" s="27" t="n"/>
+      <c r="BX34" s="40" t="n"/>
+      <c r="BY34" s="39" t="n"/>
       <c r="BZ34" s="24" t="n"/>
       <c r="CA34" s="31" t="n"/>
     </row>
@@ -9816,7 +9847,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J35" s="25" t="n"/>
+      <c r="J35" s="38" t="n"/>
       <c r="K35" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -9825,7 +9856,7 @@
       <c r="L35" s="26" t="n">
         <v>150</v>
       </c>
-      <c r="M35" s="27" t="n">
+      <c r="M35" s="39" t="n">
         <v>2.5</v>
       </c>
       <c r="N35" s="28" t="n">
@@ -9857,11 +9888,11 @@
       <c r="V35" s="24" t="n"/>
       <c r="W35" s="26" t="n"/>
       <c r="X35" s="26" t="n"/>
-      <c r="Y35" s="25" t="n"/>
+      <c r="Y35" s="38" t="n"/>
       <c r="Z35" s="26" t="n"/>
       <c r="AA35" s="28" t="n"/>
       <c r="AB35" s="28" t="n"/>
-      <c r="AC35" s="30" t="n"/>
+      <c r="AC35" s="40" t="n"/>
       <c r="AD35" s="24" t="n"/>
       <c r="AE35" s="31" t="inlineStr">
         <is>
@@ -9992,11 +10023,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ35" s="25" t="n"/>
+      <c r="BJ35" s="38" t="n"/>
       <c r="BK35" s="26" t="n">
         <v>150</v>
       </c>
-      <c r="BL35" s="27" t="n">
+      <c r="BL35" s="39" t="n">
         <v>2.5</v>
       </c>
       <c r="BM35" s="28" t="n">
@@ -10006,28 +10037,28 @@
         <v>0.39604</v>
       </c>
       <c r="BO35" s="28" t="n"/>
-      <c r="BP35" s="25" t="n"/>
-      <c r="BQ35" s="27" t="n"/>
+      <c r="BP35" s="38" t="n"/>
+      <c r="BQ35" s="39" t="n"/>
       <c r="BR35" s="28" t="n"/>
       <c r="BS35" s="28" t="n"/>
       <c r="BT35" s="28" t="n"/>
-      <c r="BU35" s="25" t="n"/>
+      <c r="BU35" s="38" t="n"/>
       <c r="BV35" s="29" t="n"/>
       <c r="BW35" s="24" t="n"/>
-      <c r="BX35" s="30" t="n"/>
-      <c r="BY35" s="27" t="n"/>
+      <c r="BX35" s="40" t="n"/>
+      <c r="BY35" s="39" t="n"/>
       <c r="BZ35" s="24" t="n"/>
       <c r="CA35" s="31" t="n"/>
     </row>
     <row r="36" ht="36" customHeight="1">
       <c r="A36" s="24" t="inlineStr">
         <is>
-          <t>8a8477c2b92442e1</t>
+          <t>2ca332931d5a4fdb</t>
         </is>
       </c>
       <c r="B36" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T16:18:24.995882Z</t>
+          <t>2026-07-20T16:32:37.034238Z</t>
         </is>
       </c>
       <c r="C36" s="24" t="inlineStr">
@@ -10065,7 +10096,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J36" s="25" t="n"/>
+      <c r="J36" s="38" t="n"/>
       <c r="K36" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -10074,24 +10105,24 @@
       <c r="L36" s="26" t="n">
         <v>144</v>
       </c>
-      <c r="M36" s="27" t="n">
+      <c r="M36" s="39" t="n">
         <v>2.44</v>
       </c>
       <c r="N36" s="28" t="n">
         <v>0.409836</v>
       </c>
       <c r="O36" s="28" t="n">
-        <v>0.555003</v>
+        <v>0.527501</v>
       </c>
       <c r="P36" s="28" t="n"/>
       <c r="Q36" s="28" t="n">
-        <v>0.145003</v>
+        <v>0.117501</v>
       </c>
       <c r="R36" s="26" t="n">
         <v>100</v>
       </c>
       <c r="S36" s="29" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="T36" s="24" t="inlineStr">
         <is>
@@ -10106,11 +10137,11 @@
       <c r="V36" s="24" t="n"/>
       <c r="W36" s="26" t="n"/>
       <c r="X36" s="26" t="n"/>
-      <c r="Y36" s="25" t="n"/>
+      <c r="Y36" s="38" t="n"/>
       <c r="Z36" s="26" t="n"/>
       <c r="AA36" s="28" t="n"/>
       <c r="AB36" s="28" t="n"/>
-      <c r="AC36" s="30" t="n"/>
+      <c r="AC36" s="40" t="n"/>
       <c r="AD36" s="24" t="n"/>
       <c r="AE36" s="31" t="inlineStr">
         <is>
@@ -10233,7 +10264,7 @@
       </c>
       <c r="BH36" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T16:18:24.995882Z</t>
+          <t>2026-07-20T16:32:37.034238Z</t>
         </is>
       </c>
       <c r="BI36" s="24" t="inlineStr">
@@ -10241,11 +10272,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ36" s="25" t="n"/>
+      <c r="BJ36" s="38" t="n"/>
       <c r="BK36" s="26" t="n">
         <v>144</v>
       </c>
-      <c r="BL36" s="27" t="n">
+      <c r="BL36" s="39" t="n">
         <v>2.44</v>
       </c>
       <c r="BM36" s="28" t="n">
@@ -10253,28 +10284,28 @@
       </c>
       <c r="BN36" s="28" t="n"/>
       <c r="BO36" s="28" t="n"/>
-      <c r="BP36" s="25" t="n"/>
-      <c r="BQ36" s="27" t="n"/>
+      <c r="BP36" s="38" t="n"/>
+      <c r="BQ36" s="39" t="n"/>
       <c r="BR36" s="28" t="n"/>
       <c r="BS36" s="28" t="n"/>
       <c r="BT36" s="28" t="n"/>
-      <c r="BU36" s="25" t="n"/>
+      <c r="BU36" s="38" t="n"/>
       <c r="BV36" s="29" t="n"/>
       <c r="BW36" s="24" t="n"/>
-      <c r="BX36" s="30" t="n"/>
-      <c r="BY36" s="27" t="n"/>
+      <c r="BX36" s="40" t="n"/>
+      <c r="BY36" s="39" t="n"/>
       <c r="BZ36" s="24" t="n"/>
       <c r="CA36" s="31" t="n"/>
     </row>
     <row r="37" ht="36" customHeight="1">
       <c r="A37" s="24" t="inlineStr">
         <is>
-          <t>dc63682b755a4fc5</t>
+          <t>19b13148b06b408d</t>
         </is>
       </c>
       <c r="B37" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T16:18:25.123725Z</t>
+          <t>2026-07-20T16:32:37.134076Z</t>
         </is>
       </c>
       <c r="C37" s="24" t="inlineStr">
@@ -10312,7 +10343,7 @@
           <t>away</t>
         </is>
       </c>
-      <c r="J37" s="25" t="n"/>
+      <c r="J37" s="38" t="n"/>
       <c r="K37" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -10321,24 +10352,24 @@
       <c r="L37" s="26" t="n">
         <v>186</v>
       </c>
-      <c r="M37" s="27" t="n">
+      <c r="M37" s="39" t="n">
         <v>2.86</v>
       </c>
       <c r="N37" s="28" t="n">
         <v>0.34965</v>
       </c>
       <c r="O37" s="28" t="n">
-        <v>0.567918</v>
+        <v>0.533959</v>
       </c>
       <c r="P37" s="28" t="n"/>
       <c r="Q37" s="28" t="n">
-        <v>0.217918</v>
+        <v>0.183959</v>
       </c>
       <c r="R37" s="26" t="n">
         <v>100</v>
       </c>
       <c r="S37" s="29" t="n">
-        <v>1.25</v>
+        <v>0.75</v>
       </c>
       <c r="T37" s="24" t="inlineStr">
         <is>
@@ -10353,11 +10384,11 @@
       <c r="V37" s="24" t="n"/>
       <c r="W37" s="26" t="n"/>
       <c r="X37" s="26" t="n"/>
-      <c r="Y37" s="25" t="n"/>
+      <c r="Y37" s="38" t="n"/>
       <c r="Z37" s="26" t="n"/>
       <c r="AA37" s="28" t="n"/>
       <c r="AB37" s="28" t="n"/>
-      <c r="AC37" s="30" t="n"/>
+      <c r="AC37" s="40" t="n"/>
       <c r="AD37" s="24" t="n"/>
       <c r="AE37" s="31" t="inlineStr">
         <is>
@@ -10480,7 +10511,7 @@
       </c>
       <c r="BH37" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T16:18:25.123725Z</t>
+          <t>2026-07-20T16:32:37.134076Z</t>
         </is>
       </c>
       <c r="BI37" s="24" t="inlineStr">
@@ -10488,11 +10519,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ37" s="25" t="n"/>
+      <c r="BJ37" s="38" t="n"/>
       <c r="BK37" s="26" t="n">
         <v>186</v>
       </c>
-      <c r="BL37" s="27" t="n">
+      <c r="BL37" s="39" t="n">
         <v>2.86</v>
       </c>
       <c r="BM37" s="28" t="n">
@@ -10500,53 +10531,53 @@
       </c>
       <c r="BN37" s="28" t="n"/>
       <c r="BO37" s="28" t="n"/>
-      <c r="BP37" s="25" t="n"/>
-      <c r="BQ37" s="27" t="n"/>
+      <c r="BP37" s="38" t="n"/>
+      <c r="BQ37" s="39" t="n"/>
       <c r="BR37" s="28" t="n"/>
       <c r="BS37" s="28" t="n"/>
       <c r="BT37" s="28" t="n"/>
-      <c r="BU37" s="25" t="n"/>
+      <c r="BU37" s="38" t="n"/>
       <c r="BV37" s="29" t="n"/>
       <c r="BW37" s="24" t="n"/>
-      <c r="BX37" s="30" t="n"/>
-      <c r="BY37" s="27" t="n"/>
+      <c r="BX37" s="40" t="n"/>
+      <c r="BY37" s="39" t="n"/>
       <c r="BZ37" s="24" t="n"/>
       <c r="CA37" s="31" t="n"/>
     </row>
     <row r="38" ht="36" customHeight="1">
       <c r="A38" s="24" t="inlineStr">
         <is>
-          <t>36b26e06b0c0460a</t>
+          <t>3646f4334f58469d</t>
         </is>
       </c>
       <c r="B38" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T16:18:25.218065Z</t>
+          <t>2026-07-20T16:32:43.485216Z</t>
         </is>
       </c>
       <c r="C38" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T22:00:00Z</t>
+          <t>2026-07-20T17:00:00Z</t>
         </is>
       </c>
       <c r="D38" s="24" t="inlineStr">
         <is>
-          <t>54693</t>
+          <t>56113</t>
         </is>
       </c>
       <c r="E38" s="24" t="inlineStr">
         <is>
-          <t>LOL</t>
+          <t>CS2</t>
         </is>
       </c>
       <c r="F38" s="24" t="inlineStr">
         <is>
-          <t>Ei Nerd Esports</t>
+          <t>Inner Circle Academy</t>
         </is>
       </c>
       <c r="G38" s="24" t="inlineStr">
         <is>
-          <t>RED Academy</t>
+          <t>Endless Journey</t>
         </is>
       </c>
       <c r="H38" s="24" t="inlineStr">
@@ -10556,40 +10587,40 @@
       </c>
       <c r="I38" s="24" t="inlineStr">
         <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="J38" s="25" t="n"/>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="J38" s="38" t="n"/>
       <c r="K38" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
         </is>
       </c>
       <c r="L38" s="26" t="n">
-        <v>300</v>
-      </c>
-      <c r="M38" s="27" t="n">
-        <v>4</v>
+        <v>113</v>
+      </c>
+      <c r="M38" s="39" t="n">
+        <v>2.13</v>
       </c>
       <c r="N38" s="28" t="n">
-        <v>0.25</v>
+        <v>0.469484</v>
       </c>
       <c r="O38" s="28" t="n">
-        <v>0.674654</v>
+        <v>0.576217</v>
       </c>
       <c r="P38" s="28" t="n"/>
       <c r="Q38" s="28" t="n">
-        <v>0.424654</v>
+        <v>0.106217</v>
       </c>
       <c r="R38" s="26" t="n">
         <v>100</v>
       </c>
       <c r="S38" s="29" t="n">
-        <v>2</v>
+        <v>1.25</v>
       </c>
       <c r="T38" s="24" t="inlineStr">
         <is>
-          <t>lol-neutral-series-elo-v1</t>
+          <t>cs2-neutral-series-elo-v1</t>
         </is>
       </c>
       <c r="U38" s="24" t="inlineStr">
@@ -10600,15 +10631,15 @@
       <c r="V38" s="24" t="n"/>
       <c r="W38" s="26" t="n"/>
       <c r="X38" s="26" t="n"/>
-      <c r="Y38" s="25" t="n"/>
+      <c r="Y38" s="38" t="n"/>
       <c r="Z38" s="26" t="n"/>
       <c r="AA38" s="28" t="n"/>
       <c r="AB38" s="28" t="n"/>
-      <c r="AC38" s="30" t="n"/>
+      <c r="AC38" s="40" t="n"/>
       <c r="AD38" s="24" t="n"/>
       <c r="AE38" s="31" t="inlineStr">
         <is>
-          <t>Neutral Elo baseline; executable ask 0.2500 (aec-lol-reda-nerd-2026-07-20).</t>
+          <t>Neutral Elo baseline; executable ask 0.4700 (aec-cs2-ica-ej-2026-07-20).</t>
         </is>
       </c>
       <c r="AF38" s="31" t="inlineStr">
@@ -10649,32 +10680,32 @@
       </c>
       <c r="AP38" s="24" t="inlineStr">
         <is>
-          <t>Ei Nerd Esports</t>
+          <t>Inner Circle Academy</t>
         </is>
       </c>
       <c r="AQ38" s="24" t="inlineStr">
         <is>
-          <t>Ei Nerd Esports</t>
+          <t>Inner Circle Academy</t>
         </is>
       </c>
       <c r="AR38" s="24" t="inlineStr">
         <is>
-          <t>Ei Nerd Esports</t>
+          <t>Inner Circle Academy</t>
         </is>
       </c>
       <c r="AS38" s="24" t="inlineStr">
         <is>
-          <t>RED Academy</t>
+          <t>Endless Journey</t>
         </is>
       </c>
       <c r="AT38" s="24" t="inlineStr">
         <is>
-          <t>RED Academy</t>
+          <t>Endless Journey</t>
         </is>
       </c>
       <c r="AU38" s="24" t="inlineStr">
         <is>
-          <t>RED Academy</t>
+          <t>Endless Journey</t>
         </is>
       </c>
       <c r="AV38" s="24" t="n"/>
@@ -10692,7 +10723,7 @@
       </c>
       <c r="BA38" s="24" t="inlineStr">
         <is>
-          <t>1f56359bf30bb6d51629a345226e3008ebfe73210551f6db9f5ce09f656ffdd6</t>
+          <t>40df7f7b9128e86cfbc485914f5801a00963b62604711b733b60f782ba9e258b</t>
         </is>
       </c>
       <c r="BB38" s="24" t="inlineStr">
@@ -10702,12 +10733,12 @@
       </c>
       <c r="BC38" s="24" t="inlineStr">
         <is>
-          <t>lol-neutral-series-elo-v1</t>
+          <t>cs2-neutral-series-elo-v1</t>
         </is>
       </c>
       <c r="BD38" s="24" t="inlineStr">
         <is>
-          <t>1f56359bf30bb6d51629a345226e3008ebfe73210551f6db9f5ce09f656ffdd6</t>
+          <t>40df7f7b9128e86cfbc485914f5801a00963b62604711b733b60f782ba9e258b</t>
         </is>
       </c>
       <c r="BE38" s="24" t="inlineStr">
@@ -10727,7 +10758,7 @@
       </c>
       <c r="BH38" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T16:18:25.218065Z</t>
+          <t>2026-07-20T16:32:43.485216Z</t>
         </is>
       </c>
       <c r="BI38" s="24" t="inlineStr">
@@ -10735,65 +10766,65 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ38" s="25" t="n"/>
+      <c r="BJ38" s="38" t="n"/>
       <c r="BK38" s="26" t="n">
-        <v>300</v>
-      </c>
-      <c r="BL38" s="27" t="n">
-        <v>4</v>
+        <v>113</v>
+      </c>
+      <c r="BL38" s="39" t="n">
+        <v>2.13</v>
       </c>
       <c r="BM38" s="28" t="n">
-        <v>0.25</v>
+        <v>0.469484</v>
       </c>
       <c r="BN38" s="28" t="n"/>
       <c r="BO38" s="28" t="n"/>
-      <c r="BP38" s="25" t="n"/>
-      <c r="BQ38" s="27" t="n"/>
+      <c r="BP38" s="38" t="n"/>
+      <c r="BQ38" s="39" t="n"/>
       <c r="BR38" s="28" t="n"/>
       <c r="BS38" s="28" t="n"/>
       <c r="BT38" s="28" t="n"/>
-      <c r="BU38" s="25" t="n"/>
+      <c r="BU38" s="38" t="n"/>
       <c r="BV38" s="29" t="n"/>
       <c r="BW38" s="24" t="n"/>
-      <c r="BX38" s="30" t="n"/>
-      <c r="BY38" s="27" t="n"/>
+      <c r="BX38" s="40" t="n"/>
+      <c r="BY38" s="39" t="n"/>
       <c r="BZ38" s="24" t="n"/>
       <c r="CA38" s="31" t="n"/>
     </row>
     <row r="39" ht="36" customHeight="1">
       <c r="A39" s="24" t="inlineStr">
         <is>
-          <t>a72da5dc37704076</t>
+          <t>a2f62addc7be49e9</t>
         </is>
       </c>
       <c r="B39" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T16:18:25.312075Z</t>
+          <t>2026-07-20T16:32:43.612711Z</t>
         </is>
       </c>
       <c r="C39" s="24" t="inlineStr">
         <is>
-          <t>2026-07-21T00:00:00Z</t>
+          <t>2026-07-20T21:00:00Z</t>
         </is>
       </c>
       <c r="D39" s="24" t="inlineStr">
         <is>
-          <t>54745</t>
+          <t>54672</t>
         </is>
       </c>
       <c r="E39" s="24" t="inlineStr">
         <is>
-          <t>LOL</t>
+          <t>CS2</t>
         </is>
       </c>
       <c r="F39" s="24" t="inlineStr">
         <is>
-          <t>Estral Esports</t>
+          <t>METANOIA WOLVES</t>
         </is>
       </c>
       <c r="G39" s="24" t="inlineStr">
         <is>
-          <t>paiN Gaming Academy</t>
+          <t>RED Canids Academy</t>
         </is>
       </c>
       <c r="H39" s="24" t="inlineStr">
@@ -10803,40 +10834,40 @@
       </c>
       <c r="I39" s="24" t="inlineStr">
         <is>
-          <t>away</t>
-        </is>
-      </c>
-      <c r="J39" s="25" t="n"/>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J39" s="38" t="n"/>
       <c r="K39" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
         </is>
       </c>
       <c r="L39" s="26" t="n">
-        <v>245</v>
-      </c>
-      <c r="M39" s="27" t="n">
-        <v>3.45</v>
+        <v>-144</v>
+      </c>
+      <c r="M39" s="39" t="n">
+        <v>1.694444</v>
       </c>
       <c r="N39" s="28" t="n">
-        <v>0.289855</v>
+        <v>0.590164</v>
       </c>
       <c r="O39" s="28" t="n">
-        <v>0.586418</v>
+        <v>0.692542</v>
       </c>
       <c r="P39" s="28" t="n"/>
       <c r="Q39" s="28" t="n">
-        <v>0.296418</v>
+        <v>0.102542</v>
       </c>
       <c r="R39" s="26" t="n">
         <v>100</v>
       </c>
       <c r="S39" s="29" t="n">
-        <v>1.25</v>
+        <v>2</v>
       </c>
       <c r="T39" s="24" t="inlineStr">
         <is>
-          <t>lol-neutral-series-elo-v1</t>
+          <t>cs2-neutral-series-elo-v1</t>
         </is>
       </c>
       <c r="U39" s="24" t="inlineStr">
@@ -10847,15 +10878,15 @@
       <c r="V39" s="24" t="n"/>
       <c r="W39" s="26" t="n"/>
       <c r="X39" s="26" t="n"/>
-      <c r="Y39" s="25" t="n"/>
+      <c r="Y39" s="38" t="n"/>
       <c r="Z39" s="26" t="n"/>
       <c r="AA39" s="28" t="n"/>
       <c r="AB39" s="28" t="n"/>
-      <c r="AC39" s="30" t="n"/>
+      <c r="AC39" s="40" t="n"/>
       <c r="AD39" s="24" t="n"/>
       <c r="AE39" s="31" t="inlineStr">
         <is>
-          <t>Neutral Elo baseline; executable ask 0.2900 (aec-lol-est-pnga-2026-07-21).</t>
+          <t>Neutral Elo baseline; executable ask 0.5900 (aec-cs2-reda-mw-2026-07-20).</t>
         </is>
       </c>
       <c r="AF39" s="31" t="inlineStr">
@@ -10896,32 +10927,32 @@
       </c>
       <c r="AP39" s="24" t="inlineStr">
         <is>
-          <t>Estral Esports</t>
+          <t>METANOIA WOLVES</t>
         </is>
       </c>
       <c r="AQ39" s="24" t="inlineStr">
         <is>
-          <t>Estral Esports</t>
+          <t>METANOIA WOLVES</t>
         </is>
       </c>
       <c r="AR39" s="24" t="inlineStr">
         <is>
-          <t>Estral Esports</t>
+          <t>METANOIA WOLVES</t>
         </is>
       </c>
       <c r="AS39" s="24" t="inlineStr">
         <is>
-          <t>paiN Gaming Academy</t>
+          <t>RED Canids Academy</t>
         </is>
       </c>
       <c r="AT39" s="24" t="inlineStr">
         <is>
-          <t>paiN Gaming Academy</t>
+          <t>RED Canids Academy</t>
         </is>
       </c>
       <c r="AU39" s="24" t="inlineStr">
         <is>
-          <t>paiN Gaming Academy</t>
+          <t>RED Canids Academy</t>
         </is>
       </c>
       <c r="AV39" s="24" t="n"/>
@@ -10939,7 +10970,7 @@
       </c>
       <c r="BA39" s="24" t="inlineStr">
         <is>
-          <t>1f56359bf30bb6d51629a345226e3008ebfe73210551f6db9f5ce09f656ffdd6</t>
+          <t>40df7f7b9128e86cfbc485914f5801a00963b62604711b733b60f782ba9e258b</t>
         </is>
       </c>
       <c r="BB39" s="24" t="inlineStr">
@@ -10949,12 +10980,12 @@
       </c>
       <c r="BC39" s="24" t="inlineStr">
         <is>
-          <t>lol-neutral-series-elo-v1</t>
+          <t>cs2-neutral-series-elo-v1</t>
         </is>
       </c>
       <c r="BD39" s="24" t="inlineStr">
         <is>
-          <t>1f56359bf30bb6d51629a345226e3008ebfe73210551f6db9f5ce09f656ffdd6</t>
+          <t>40df7f7b9128e86cfbc485914f5801a00963b62604711b733b60f782ba9e258b</t>
         </is>
       </c>
       <c r="BE39" s="24" t="inlineStr">
@@ -10974,7 +11005,7 @@
       </c>
       <c r="BH39" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T16:18:25.312075Z</t>
+          <t>2026-07-20T16:32:43.612711Z</t>
         </is>
       </c>
       <c r="BI39" s="24" t="inlineStr">
@@ -10982,1018 +11013,30 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ39" s="25" t="n"/>
+      <c r="BJ39" s="38" t="n"/>
       <c r="BK39" s="26" t="n">
-        <v>245</v>
-      </c>
-      <c r="BL39" s="27" t="n">
-        <v>3.45</v>
+        <v>-144</v>
+      </c>
+      <c r="BL39" s="39" t="n">
+        <v>1.694444</v>
       </c>
       <c r="BM39" s="28" t="n">
-        <v>0.289855</v>
+        <v>0.590164</v>
       </c>
       <c r="BN39" s="28" t="n"/>
       <c r="BO39" s="28" t="n"/>
-      <c r="BP39" s="25" t="n"/>
-      <c r="BQ39" s="27" t="n"/>
+      <c r="BP39" s="38" t="n"/>
+      <c r="BQ39" s="39" t="n"/>
       <c r="BR39" s="28" t="n"/>
       <c r="BS39" s="28" t="n"/>
       <c r="BT39" s="28" t="n"/>
-      <c r="BU39" s="25" t="n"/>
+      <c r="BU39" s="38" t="n"/>
       <c r="BV39" s="29" t="n"/>
       <c r="BW39" s="24" t="n"/>
-      <c r="BX39" s="30" t="n"/>
-      <c r="BY39" s="27" t="n"/>
+      <c r="BX39" s="40" t="n"/>
+      <c r="BY39" s="39" t="n"/>
       <c r="BZ39" s="24" t="n"/>
       <c r="CA39" s="31" t="n"/>
-    </row>
-    <row r="40" ht="36" customHeight="1">
-      <c r="A40" s="24" t="inlineStr">
-        <is>
-          <t>66a67a653fb14bd2</t>
-        </is>
-      </c>
-      <c r="B40" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-20T16:26:22.811500Z</t>
-        </is>
-      </c>
-      <c r="C40" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-20T17:00:00Z</t>
-        </is>
-      </c>
-      <c r="D40" s="24" t="inlineStr">
-        <is>
-          <t>56113</t>
-        </is>
-      </c>
-      <c r="E40" s="24" t="inlineStr">
-        <is>
-          <t>CS2</t>
-        </is>
-      </c>
-      <c r="F40" s="24" t="inlineStr">
-        <is>
-          <t>Inner Circle Academy</t>
-        </is>
-      </c>
-      <c r="G40" s="24" t="inlineStr">
-        <is>
-          <t>Endless Journey</t>
-        </is>
-      </c>
-      <c r="H40" s="24" t="inlineStr">
-        <is>
-          <t>moneyline</t>
-        </is>
-      </c>
-      <c r="I40" s="24" t="inlineStr">
-        <is>
-          <t>away</t>
-        </is>
-      </c>
-      <c r="J40" s="25" t="n"/>
-      <c r="K40" s="24" t="inlineStr">
-        <is>
-          <t>polymarket_us</t>
-        </is>
-      </c>
-      <c r="L40" s="26" t="n">
-        <v>-113</v>
-      </c>
-      <c r="M40" s="27" t="n">
-        <v>1.884956</v>
-      </c>
-      <c r="N40" s="28" t="n">
-        <v>0.530516</v>
-      </c>
-      <c r="O40" s="28" t="n">
-        <v>0.652434</v>
-      </c>
-      <c r="P40" s="28" t="n"/>
-      <c r="Q40" s="28" t="n">
-        <v>0.122434</v>
-      </c>
-      <c r="R40" s="26" t="n">
-        <v>100</v>
-      </c>
-      <c r="S40" s="29" t="n">
-        <v>2</v>
-      </c>
-      <c r="T40" s="24" t="inlineStr">
-        <is>
-          <t>cs2-neutral-series-elo-v1</t>
-        </is>
-      </c>
-      <c r="U40" s="24" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V40" s="24" t="n"/>
-      <c r="W40" s="26" t="n"/>
-      <c r="X40" s="26" t="n"/>
-      <c r="Y40" s="25" t="n"/>
-      <c r="Z40" s="26" t="n"/>
-      <c r="AA40" s="28" t="n"/>
-      <c r="AB40" s="28" t="n"/>
-      <c r="AC40" s="30" t="n"/>
-      <c r="AD40" s="24" t="n"/>
-      <c r="AE40" s="31" t="inlineStr">
-        <is>
-          <t>Neutral Elo baseline; executable ask 0.5300 (aec-cs2-ica-ej-2026-07-20).</t>
-        </is>
-      </c>
-      <c r="AF40" s="31" t="inlineStr">
-        <is>
-          <t>Research baseline; zero-unit shadow until qualified.</t>
-        </is>
-      </c>
-      <c r="AG40" s="24" t="inlineStr">
-        <is>
-          <t>not_applicable</t>
-        </is>
-      </c>
-      <c r="AH40" s="24" t="n"/>
-      <c r="AI40" s="31" t="n"/>
-      <c r="AJ40" s="31" t="n"/>
-      <c r="AK40" s="24" t="inlineStr">
-        <is>
-          <t>model_qualified</t>
-        </is>
-      </c>
-      <c r="AL40" s="26" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM40" s="24" t="inlineStr">
-        <is>
-          <t>QUALIFIED_SHADOW_CALL</t>
-        </is>
-      </c>
-      <c r="AN40" s="24" t="inlineStr">
-        <is>
-          <t>CALL</t>
-        </is>
-      </c>
-      <c r="AO40" s="24" t="inlineStr">
-        <is>
-          <t>QUALIFIED</t>
-        </is>
-      </c>
-      <c r="AP40" s="24" t="inlineStr">
-        <is>
-          <t>Inner Circle Academy</t>
-        </is>
-      </c>
-      <c r="AQ40" s="24" t="inlineStr">
-        <is>
-          <t>Inner Circle Academy</t>
-        </is>
-      </c>
-      <c r="AR40" s="24" t="inlineStr">
-        <is>
-          <t>Inner Circle Academy</t>
-        </is>
-      </c>
-      <c r="AS40" s="24" t="inlineStr">
-        <is>
-          <t>Endless Journey</t>
-        </is>
-      </c>
-      <c r="AT40" s="24" t="inlineStr">
-        <is>
-          <t>Endless Journey</t>
-        </is>
-      </c>
-      <c r="AU40" s="24" t="inlineStr">
-        <is>
-          <t>Endless Journey</t>
-        </is>
-      </c>
-      <c r="AV40" s="24" t="n"/>
-      <c r="AW40" s="24" t="n"/>
-      <c r="AX40" s="24" t="inlineStr">
-        <is>
-          <t>statistical_model</t>
-        </is>
-      </c>
-      <c r="AY40" s="24" t="n"/>
-      <c r="AZ40" s="24" t="inlineStr">
-        <is>
-          <t>shadow_qualified</t>
-        </is>
-      </c>
-      <c r="BA40" s="24" t="inlineStr">
-        <is>
-          <t>40df7f7b9128e86cfbc485914f5801a00963b62604711b733b60f782ba9e258b</t>
-        </is>
-      </c>
-      <c r="BB40" s="24" t="inlineStr">
-        <is>
-          <t>neutral_elo</t>
-        </is>
-      </c>
-      <c r="BC40" s="24" t="inlineStr">
-        <is>
-          <t>cs2-neutral-series-elo-v1</t>
-        </is>
-      </c>
-      <c r="BD40" s="24" t="inlineStr">
-        <is>
-          <t>40df7f7b9128e86cfbc485914f5801a00963b62604711b733b60f782ba9e258b</t>
-        </is>
-      </c>
-      <c r="BE40" s="24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BF40" s="24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BG40" s="24" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="BH40" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-20T16:26:22.811500Z</t>
-        </is>
-      </c>
-      <c r="BI40" s="24" t="inlineStr">
-        <is>
-          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
-        </is>
-      </c>
-      <c r="BJ40" s="25" t="n"/>
-      <c r="BK40" s="26" t="n">
-        <v>-113</v>
-      </c>
-      <c r="BL40" s="27" t="n">
-        <v>1.884956</v>
-      </c>
-      <c r="BM40" s="28" t="n">
-        <v>0.530516</v>
-      </c>
-      <c r="BN40" s="28" t="n"/>
-      <c r="BO40" s="28" t="n"/>
-      <c r="BP40" s="25" t="n"/>
-      <c r="BQ40" s="27" t="n"/>
-      <c r="BR40" s="28" t="n"/>
-      <c r="BS40" s="28" t="n"/>
-      <c r="BT40" s="28" t="n"/>
-      <c r="BU40" s="25" t="n"/>
-      <c r="BV40" s="29" t="n"/>
-      <c r="BW40" s="24" t="n"/>
-      <c r="BX40" s="30" t="n"/>
-      <c r="BY40" s="27" t="n"/>
-      <c r="BZ40" s="24" t="n"/>
-      <c r="CA40" s="31" t="n"/>
-    </row>
-    <row r="41" ht="36" customHeight="1">
-      <c r="A41" s="24" t="inlineStr">
-        <is>
-          <t>a75a7af91f614c77</t>
-        </is>
-      </c>
-      <c r="B41" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-20T16:26:22.946543Z</t>
-        </is>
-      </c>
-      <c r="C41" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-20T19:00:00Z</t>
-        </is>
-      </c>
-      <c r="D41" s="24" t="inlineStr">
-        <is>
-          <t>56757</t>
-        </is>
-      </c>
-      <c r="E41" s="24" t="inlineStr">
-        <is>
-          <t>CS2</t>
-        </is>
-      </c>
-      <c r="F41" s="24" t="inlineStr">
-        <is>
-          <t>MAGICOS</t>
-        </is>
-      </c>
-      <c r="G41" s="24" t="inlineStr">
-        <is>
-          <t>Blitzkrieg</t>
-        </is>
-      </c>
-      <c r="H41" s="24" t="inlineStr">
-        <is>
-          <t>moneyline</t>
-        </is>
-      </c>
-      <c r="I41" s="24" t="inlineStr">
-        <is>
-          <t>away</t>
-        </is>
-      </c>
-      <c r="J41" s="25" t="n"/>
-      <c r="K41" s="24" t="inlineStr">
-        <is>
-          <t>polymarket_us</t>
-        </is>
-      </c>
-      <c r="L41" s="26" t="n">
-        <v>669</v>
-      </c>
-      <c r="M41" s="27" t="n">
-        <v>7.69</v>
-      </c>
-      <c r="N41" s="28" t="n">
-        <v>0.130039</v>
-      </c>
-      <c r="O41" s="28" t="n">
-        <v>0.598244</v>
-      </c>
-      <c r="P41" s="28" t="n"/>
-      <c r="Q41" s="28" t="n">
-        <v>0.468244</v>
-      </c>
-      <c r="R41" s="26" t="n">
-        <v>100</v>
-      </c>
-      <c r="S41" s="29" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="T41" s="24" t="inlineStr">
-        <is>
-          <t>cs2-neutral-series-elo-v1</t>
-        </is>
-      </c>
-      <c r="U41" s="24" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V41" s="24" t="n"/>
-      <c r="W41" s="26" t="n"/>
-      <c r="X41" s="26" t="n"/>
-      <c r="Y41" s="25" t="n"/>
-      <c r="Z41" s="26" t="n"/>
-      <c r="AA41" s="28" t="n"/>
-      <c r="AB41" s="28" t="n"/>
-      <c r="AC41" s="30" t="n"/>
-      <c r="AD41" s="24" t="n"/>
-      <c r="AE41" s="31" t="inlineStr">
-        <is>
-          <t>Neutral Elo baseline; executable ask 0.1300 (aec-cs2-mag-bk-2026-07-20).</t>
-        </is>
-      </c>
-      <c r="AF41" s="31" t="inlineStr">
-        <is>
-          <t>Research baseline; zero-unit shadow until qualified.</t>
-        </is>
-      </c>
-      <c r="AG41" s="24" t="inlineStr">
-        <is>
-          <t>not_applicable</t>
-        </is>
-      </c>
-      <c r="AH41" s="24" t="n"/>
-      <c r="AI41" s="31" t="n"/>
-      <c r="AJ41" s="31" t="n"/>
-      <c r="AK41" s="24" t="inlineStr">
-        <is>
-          <t>model_qualified</t>
-        </is>
-      </c>
-      <c r="AL41" s="26" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM41" s="24" t="inlineStr">
-        <is>
-          <t>QUALIFIED_SHADOW_CALL</t>
-        </is>
-      </c>
-      <c r="AN41" s="24" t="inlineStr">
-        <is>
-          <t>CALL</t>
-        </is>
-      </c>
-      <c r="AO41" s="24" t="inlineStr">
-        <is>
-          <t>QUALIFIED</t>
-        </is>
-      </c>
-      <c r="AP41" s="24" t="inlineStr">
-        <is>
-          <t>MAGICOS</t>
-        </is>
-      </c>
-      <c r="AQ41" s="24" t="inlineStr">
-        <is>
-          <t>MAGICOS</t>
-        </is>
-      </c>
-      <c r="AR41" s="24" t="inlineStr">
-        <is>
-          <t>MAGICOS</t>
-        </is>
-      </c>
-      <c r="AS41" s="24" t="inlineStr">
-        <is>
-          <t>Blitzkrieg</t>
-        </is>
-      </c>
-      <c r="AT41" s="24" t="inlineStr">
-        <is>
-          <t>Blitzkrieg</t>
-        </is>
-      </c>
-      <c r="AU41" s="24" t="inlineStr">
-        <is>
-          <t>Blitzkrieg</t>
-        </is>
-      </c>
-      <c r="AV41" s="24" t="n"/>
-      <c r="AW41" s="24" t="n"/>
-      <c r="AX41" s="24" t="inlineStr">
-        <is>
-          <t>statistical_model</t>
-        </is>
-      </c>
-      <c r="AY41" s="24" t="n"/>
-      <c r="AZ41" s="24" t="inlineStr">
-        <is>
-          <t>shadow_qualified</t>
-        </is>
-      </c>
-      <c r="BA41" s="24" t="inlineStr">
-        <is>
-          <t>40df7f7b9128e86cfbc485914f5801a00963b62604711b733b60f782ba9e258b</t>
-        </is>
-      </c>
-      <c r="BB41" s="24" t="inlineStr">
-        <is>
-          <t>neutral_elo</t>
-        </is>
-      </c>
-      <c r="BC41" s="24" t="inlineStr">
-        <is>
-          <t>cs2-neutral-series-elo-v1</t>
-        </is>
-      </c>
-      <c r="BD41" s="24" t="inlineStr">
-        <is>
-          <t>40df7f7b9128e86cfbc485914f5801a00963b62604711b733b60f782ba9e258b</t>
-        </is>
-      </c>
-      <c r="BE41" s="24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BF41" s="24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BG41" s="24" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="BH41" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-20T16:26:22.946543Z</t>
-        </is>
-      </c>
-      <c r="BI41" s="24" t="inlineStr">
-        <is>
-          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
-        </is>
-      </c>
-      <c r="BJ41" s="25" t="n"/>
-      <c r="BK41" s="26" t="n">
-        <v>669</v>
-      </c>
-      <c r="BL41" s="27" t="n">
-        <v>7.69</v>
-      </c>
-      <c r="BM41" s="28" t="n">
-        <v>0.130039</v>
-      </c>
-      <c r="BN41" s="28" t="n"/>
-      <c r="BO41" s="28" t="n"/>
-      <c r="BP41" s="25" t="n"/>
-      <c r="BQ41" s="27" t="n"/>
-      <c r="BR41" s="28" t="n"/>
-      <c r="BS41" s="28" t="n"/>
-      <c r="BT41" s="28" t="n"/>
-      <c r="BU41" s="25" t="n"/>
-      <c r="BV41" s="29" t="n"/>
-      <c r="BW41" s="24" t="n"/>
-      <c r="BX41" s="30" t="n"/>
-      <c r="BY41" s="27" t="n"/>
-      <c r="BZ41" s="24" t="n"/>
-      <c r="CA41" s="31" t="n"/>
-    </row>
-    <row r="42" ht="36" customHeight="1">
-      <c r="A42" s="24" t="inlineStr">
-        <is>
-          <t>8a3b3559571c4133</t>
-        </is>
-      </c>
-      <c r="B42" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-20T16:26:23.050406Z</t>
-        </is>
-      </c>
-      <c r="C42" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-20T19:00:00Z</t>
-        </is>
-      </c>
-      <c r="D42" s="24" t="inlineStr">
-        <is>
-          <t>54667</t>
-        </is>
-      </c>
-      <c r="E42" s="24" t="inlineStr">
-        <is>
-          <t>CS2</t>
-        </is>
-      </c>
-      <c r="F42" s="24" t="inlineStr">
-        <is>
-          <t>paiN Academy</t>
-        </is>
-      </c>
-      <c r="G42" s="24" t="inlineStr">
-        <is>
-          <t>HATERS</t>
-        </is>
-      </c>
-      <c r="H42" s="24" t="inlineStr">
-        <is>
-          <t>moneyline</t>
-        </is>
-      </c>
-      <c r="I42" s="24" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="J42" s="25" t="n"/>
-      <c r="K42" s="24" t="inlineStr">
-        <is>
-          <t>polymarket_us</t>
-        </is>
-      </c>
-      <c r="L42" s="26" t="n">
-        <v>335</v>
-      </c>
-      <c r="M42" s="27" t="n">
-        <v>4.35</v>
-      </c>
-      <c r="N42" s="28" t="n">
-        <v>0.229885</v>
-      </c>
-      <c r="O42" s="28" t="n">
-        <v>0.558097</v>
-      </c>
-      <c r="P42" s="28" t="n"/>
-      <c r="Q42" s="28" t="n">
-        <v>0.328097</v>
-      </c>
-      <c r="R42" s="26" t="n">
-        <v>100</v>
-      </c>
-      <c r="S42" s="29" t="n">
-        <v>1</v>
-      </c>
-      <c r="T42" s="24" t="inlineStr">
-        <is>
-          <t>cs2-neutral-series-elo-v1</t>
-        </is>
-      </c>
-      <c r="U42" s="24" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V42" s="24" t="n"/>
-      <c r="W42" s="26" t="n"/>
-      <c r="X42" s="26" t="n"/>
-      <c r="Y42" s="25" t="n"/>
-      <c r="Z42" s="26" t="n"/>
-      <c r="AA42" s="28" t="n"/>
-      <c r="AB42" s="28" t="n"/>
-      <c r="AC42" s="30" t="n"/>
-      <c r="AD42" s="24" t="n"/>
-      <c r="AE42" s="31" t="inlineStr">
-        <is>
-          <t>Neutral Elo baseline; executable ask 0.2300 (aec-cs2-hat-paina-2026-07-20).</t>
-        </is>
-      </c>
-      <c r="AF42" s="31" t="inlineStr">
-        <is>
-          <t>Research baseline; zero-unit shadow until qualified.</t>
-        </is>
-      </c>
-      <c r="AG42" s="24" t="inlineStr">
-        <is>
-          <t>not_applicable</t>
-        </is>
-      </c>
-      <c r="AH42" s="24" t="n"/>
-      <c r="AI42" s="31" t="n"/>
-      <c r="AJ42" s="31" t="n"/>
-      <c r="AK42" s="24" t="inlineStr">
-        <is>
-          <t>model_qualified</t>
-        </is>
-      </c>
-      <c r="AL42" s="26" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM42" s="24" t="inlineStr">
-        <is>
-          <t>QUALIFIED_SHADOW_CALL</t>
-        </is>
-      </c>
-      <c r="AN42" s="24" t="inlineStr">
-        <is>
-          <t>CALL</t>
-        </is>
-      </c>
-      <c r="AO42" s="24" t="inlineStr">
-        <is>
-          <t>QUALIFIED</t>
-        </is>
-      </c>
-      <c r="AP42" s="24" t="inlineStr">
-        <is>
-          <t>paiN Academy</t>
-        </is>
-      </c>
-      <c r="AQ42" s="24" t="inlineStr">
-        <is>
-          <t>paiN Academy</t>
-        </is>
-      </c>
-      <c r="AR42" s="24" t="inlineStr">
-        <is>
-          <t>paiN Academy</t>
-        </is>
-      </c>
-      <c r="AS42" s="24" t="inlineStr">
-        <is>
-          <t>HATERS</t>
-        </is>
-      </c>
-      <c r="AT42" s="24" t="inlineStr">
-        <is>
-          <t>HATERS</t>
-        </is>
-      </c>
-      <c r="AU42" s="24" t="inlineStr">
-        <is>
-          <t>HATERS</t>
-        </is>
-      </c>
-      <c r="AV42" s="24" t="n"/>
-      <c r="AW42" s="24" t="n"/>
-      <c r="AX42" s="24" t="inlineStr">
-        <is>
-          <t>statistical_model</t>
-        </is>
-      </c>
-      <c r="AY42" s="24" t="n"/>
-      <c r="AZ42" s="24" t="inlineStr">
-        <is>
-          <t>shadow_qualified</t>
-        </is>
-      </c>
-      <c r="BA42" s="24" t="inlineStr">
-        <is>
-          <t>40df7f7b9128e86cfbc485914f5801a00963b62604711b733b60f782ba9e258b</t>
-        </is>
-      </c>
-      <c r="BB42" s="24" t="inlineStr">
-        <is>
-          <t>neutral_elo</t>
-        </is>
-      </c>
-      <c r="BC42" s="24" t="inlineStr">
-        <is>
-          <t>cs2-neutral-series-elo-v1</t>
-        </is>
-      </c>
-      <c r="BD42" s="24" t="inlineStr">
-        <is>
-          <t>40df7f7b9128e86cfbc485914f5801a00963b62604711b733b60f782ba9e258b</t>
-        </is>
-      </c>
-      <c r="BE42" s="24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BF42" s="24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BG42" s="24" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="BH42" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-20T16:26:23.050406Z</t>
-        </is>
-      </c>
-      <c r="BI42" s="24" t="inlineStr">
-        <is>
-          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
-        </is>
-      </c>
-      <c r="BJ42" s="25" t="n"/>
-      <c r="BK42" s="26" t="n">
-        <v>335</v>
-      </c>
-      <c r="BL42" s="27" t="n">
-        <v>4.35</v>
-      </c>
-      <c r="BM42" s="28" t="n">
-        <v>0.229885</v>
-      </c>
-      <c r="BN42" s="28" t="n"/>
-      <c r="BO42" s="28" t="n"/>
-      <c r="BP42" s="25" t="n"/>
-      <c r="BQ42" s="27" t="n"/>
-      <c r="BR42" s="28" t="n"/>
-      <c r="BS42" s="28" t="n"/>
-      <c r="BT42" s="28" t="n"/>
-      <c r="BU42" s="25" t="n"/>
-      <c r="BV42" s="29" t="n"/>
-      <c r="BW42" s="24" t="n"/>
-      <c r="BX42" s="30" t="n"/>
-      <c r="BY42" s="27" t="n"/>
-      <c r="BZ42" s="24" t="n"/>
-      <c r="CA42" s="31" t="n"/>
-    </row>
-    <row r="43" ht="36" customHeight="1">
-      <c r="A43" s="24" t="inlineStr">
-        <is>
-          <t>5417c8a3e89a4c9f</t>
-        </is>
-      </c>
-      <c r="B43" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-20T16:26:23.154839Z</t>
-        </is>
-      </c>
-      <c r="C43" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-20T21:00:00Z</t>
-        </is>
-      </c>
-      <c r="D43" s="24" t="inlineStr">
-        <is>
-          <t>54672</t>
-        </is>
-      </c>
-      <c r="E43" s="24" t="inlineStr">
-        <is>
-          <t>CS2</t>
-        </is>
-      </c>
-      <c r="F43" s="24" t="inlineStr">
-        <is>
-          <t>METANOIA WOLVES</t>
-        </is>
-      </c>
-      <c r="G43" s="24" t="inlineStr">
-        <is>
-          <t>RED Canids Academy</t>
-        </is>
-      </c>
-      <c r="H43" s="24" t="inlineStr">
-        <is>
-          <t>moneyline</t>
-        </is>
-      </c>
-      <c r="I43" s="24" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="J43" s="25" t="n"/>
-      <c r="K43" s="24" t="inlineStr">
-        <is>
-          <t>polymarket_us</t>
-        </is>
-      </c>
-      <c r="L43" s="26" t="n">
-        <v>-144</v>
-      </c>
-      <c r="M43" s="27" t="n">
-        <v>1.694444</v>
-      </c>
-      <c r="N43" s="28" t="n">
-        <v>0.590164</v>
-      </c>
-      <c r="O43" s="28" t="n">
-        <v>0.885084</v>
-      </c>
-      <c r="P43" s="28" t="n"/>
-      <c r="Q43" s="28" t="n">
-        <v>0.295084</v>
-      </c>
-      <c r="R43" s="26" t="n">
-        <v>100</v>
-      </c>
-      <c r="S43" s="29" t="n">
-        <v>2</v>
-      </c>
-      <c r="T43" s="24" t="inlineStr">
-        <is>
-          <t>cs2-neutral-series-elo-v1</t>
-        </is>
-      </c>
-      <c r="U43" s="24" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V43" s="24" t="n"/>
-      <c r="W43" s="26" t="n"/>
-      <c r="X43" s="26" t="n"/>
-      <c r="Y43" s="25" t="n"/>
-      <c r="Z43" s="26" t="n"/>
-      <c r="AA43" s="28" t="n"/>
-      <c r="AB43" s="28" t="n"/>
-      <c r="AC43" s="30" t="n"/>
-      <c r="AD43" s="24" t="n"/>
-      <c r="AE43" s="31" t="inlineStr">
-        <is>
-          <t>Neutral Elo baseline; executable ask 0.5900 (aec-cs2-reda-mw-2026-07-20).</t>
-        </is>
-      </c>
-      <c r="AF43" s="31" t="inlineStr">
-        <is>
-          <t>Research baseline; zero-unit shadow until qualified.</t>
-        </is>
-      </c>
-      <c r="AG43" s="24" t="inlineStr">
-        <is>
-          <t>not_applicable</t>
-        </is>
-      </c>
-      <c r="AH43" s="24" t="n"/>
-      <c r="AI43" s="31" t="n"/>
-      <c r="AJ43" s="31" t="n"/>
-      <c r="AK43" s="24" t="inlineStr">
-        <is>
-          <t>model_qualified</t>
-        </is>
-      </c>
-      <c r="AL43" s="26" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM43" s="24" t="inlineStr">
-        <is>
-          <t>QUALIFIED_SHADOW_CALL</t>
-        </is>
-      </c>
-      <c r="AN43" s="24" t="inlineStr">
-        <is>
-          <t>CALL</t>
-        </is>
-      </c>
-      <c r="AO43" s="24" t="inlineStr">
-        <is>
-          <t>QUALIFIED</t>
-        </is>
-      </c>
-      <c r="AP43" s="24" t="inlineStr">
-        <is>
-          <t>METANOIA WOLVES</t>
-        </is>
-      </c>
-      <c r="AQ43" s="24" t="inlineStr">
-        <is>
-          <t>METANOIA WOLVES</t>
-        </is>
-      </c>
-      <c r="AR43" s="24" t="inlineStr">
-        <is>
-          <t>METANOIA WOLVES</t>
-        </is>
-      </c>
-      <c r="AS43" s="24" t="inlineStr">
-        <is>
-          <t>RED Canids Academy</t>
-        </is>
-      </c>
-      <c r="AT43" s="24" t="inlineStr">
-        <is>
-          <t>RED Canids Academy</t>
-        </is>
-      </c>
-      <c r="AU43" s="24" t="inlineStr">
-        <is>
-          <t>RED Canids Academy</t>
-        </is>
-      </c>
-      <c r="AV43" s="24" t="n"/>
-      <c r="AW43" s="24" t="n"/>
-      <c r="AX43" s="24" t="inlineStr">
-        <is>
-          <t>statistical_model</t>
-        </is>
-      </c>
-      <c r="AY43" s="24" t="n"/>
-      <c r="AZ43" s="24" t="inlineStr">
-        <is>
-          <t>shadow_qualified</t>
-        </is>
-      </c>
-      <c r="BA43" s="24" t="inlineStr">
-        <is>
-          <t>40df7f7b9128e86cfbc485914f5801a00963b62604711b733b60f782ba9e258b</t>
-        </is>
-      </c>
-      <c r="BB43" s="24" t="inlineStr">
-        <is>
-          <t>neutral_elo</t>
-        </is>
-      </c>
-      <c r="BC43" s="24" t="inlineStr">
-        <is>
-          <t>cs2-neutral-series-elo-v1</t>
-        </is>
-      </c>
-      <c r="BD43" s="24" t="inlineStr">
-        <is>
-          <t>40df7f7b9128e86cfbc485914f5801a00963b62604711b733b60f782ba9e258b</t>
-        </is>
-      </c>
-      <c r="BE43" s="24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BF43" s="24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BG43" s="24" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="BH43" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-20T16:26:23.154839Z</t>
-        </is>
-      </c>
-      <c r="BI43" s="24" t="inlineStr">
-        <is>
-          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
-        </is>
-      </c>
-      <c r="BJ43" s="25" t="n"/>
-      <c r="BK43" s="26" t="n">
-        <v>-144</v>
-      </c>
-      <c r="BL43" s="27" t="n">
-        <v>1.694444</v>
-      </c>
-      <c r="BM43" s="28" t="n">
-        <v>0.590164</v>
-      </c>
-      <c r="BN43" s="28" t="n"/>
-      <c r="BO43" s="28" t="n"/>
-      <c r="BP43" s="25" t="n"/>
-      <c r="BQ43" s="27" t="n"/>
-      <c r="BR43" s="28" t="n"/>
-      <c r="BS43" s="28" t="n"/>
-      <c r="BT43" s="28" t="n"/>
-      <c r="BU43" s="25" t="n"/>
-      <c r="BV43" s="29" t="n"/>
-      <c r="BW43" s="24" t="n"/>
-      <c r="BX43" s="30" t="n"/>
-      <c r="BY43" s="27" t="n"/>
-      <c r="BZ43" s="24" t="n"/>
-      <c r="CA43" s="31" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix: esports ledger selection always 'home', correct contract matching
- _log_esports_forecast: selection is always 'home' since home_team
  IS the team we're betting on. Polymarket 'long'/'short' are
  contract-side labels, not home/away indicators.
- Previously: selection='home' for long, 'away' for short — wrong.
  Short side could be the model's pick, causing team/price mismatch.
- Verified: 7REX correctly picked at 59.8% vs market 35.0% (short side)
</commit_message>
<xml_diff>
--- a/data/picks.xlsx
+++ b/data/picks.xlsx
@@ -21,10 +21,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="0.0%"/>
-    <numFmt numFmtId="165" formatCode="0.0000"/>
-    <numFmt numFmtId="166" formatCode="0.0###"/>
-    <numFmt numFmtId="167" formatCode="0.000000"/>
+    <numFmt numFmtId="164" formatCode="0.0###"/>
+    <numFmt numFmtId="165" formatCode="0.000000"/>
+    <numFmt numFmtId="166" formatCode="0.0000"/>
+    <numFmt numFmtId="167" formatCode="0.0%"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -136,7 +136,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -150,10 +150,10 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -169,10 +169,10 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="10" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -184,10 +184,10 @@
     <xf numFmtId="0" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="10" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -202,13 +202,13 @@
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="10" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -217,38 +217,11 @@
     <xf numFmtId="2" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -781,7 +754,6 @@
         <v/>
       </c>
     </row>
-    <row r="5"/>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
@@ -813,16 +785,15 @@
         <f>COUNTIFS('Picks'!$BX$2:$BX$39,"&gt;0",'Picks'!$V$2:$V$39,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$39,"&gt;0",'Picks'!$V$2:$V$39,"loss")</f>
         <v/>
       </c>
-      <c r="E7" s="32">
+      <c r="E7" s="7">
         <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$39,"&gt;0",'Picks'!$V$2:$V$39,"win")/(COUNTIFS('Picks'!$BX$2:$BX$39,"&gt;0",'Picks'!$V$2:$V$39,"win")+COUNTIFS('Picks'!$BX$2:$BX$39,"&gt;0",'Picks'!$V$2:$V$39,"loss")),0)</f>
         <v/>
       </c>
-      <c r="G7" s="32">
+      <c r="G7" s="7">
         <f>IFERROR(SUM('Picks'!$BY$2:$BY$39)/SUM('Picks'!$BX$2:$BX$39),0)</f>
         <v/>
       </c>
     </row>
-    <row r="8"/>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
@@ -846,7 +817,7 @@
       </c>
     </row>
     <row r="10" ht="28" customHeight="1">
-      <c r="A10" s="33">
+      <c r="A10" s="8">
         <f>SUM('Picks'!$BY$2:$BY$39)</f>
         <v/>
       </c>
@@ -858,12 +829,11 @@
         <f>COUNTIFS('Picks'!$AM$2:$AM$39,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$39,"settled")</f>
         <v/>
       </c>
-      <c r="G10" s="33">
+      <c r="G10" s="8">
         <f>SUMIFS('Picks'!$AC$2:$AC$39,'Picks'!$AM$2:$AM$39,"QUALIFIED_SHADOW_CALL")</f>
         <v/>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
         <is>
@@ -926,11 +896,11 @@
         <f>COUNTIFS('Picks'!$H$2:$H$39,$A14,'Picks'!$U$2:$U$39,"settled",'Picks'!$V$2:$V$39,"loss")</f>
         <v/>
       </c>
-      <c r="E14" s="34">
+      <c r="E14" s="14">
         <f>IFERROR(C14/(C14+D14),0)</f>
         <v/>
       </c>
-      <c r="F14" s="35">
+      <c r="F14" s="15">
         <f>SUMIFS('Picks'!$BY$2:$BY$39,'Picks'!$H$2:$H$39,$A14)</f>
         <v/>
       </c>
@@ -957,11 +927,11 @@
         <f>COUNTIFS('Picks'!$H$2:$H$39,$A15,'Picks'!$U$2:$U$39,"settled",'Picks'!$V$2:$V$39,"loss")</f>
         <v/>
       </c>
-      <c r="E15" s="36">
+      <c r="E15" s="19">
         <f>IFERROR(C15/(C15+D15),0)</f>
         <v/>
       </c>
-      <c r="F15" s="37">
+      <c r="F15" s="20">
         <f>SUMIFS('Picks'!$BY$2:$BY$39,'Picks'!$H$2:$H$39,$A15)</f>
         <v/>
       </c>
@@ -988,11 +958,11 @@
         <f>COUNTIFS('Picks'!$H$2:$H$39,$A16,'Picks'!$U$2:$U$39,"settled",'Picks'!$V$2:$V$39,"loss")</f>
         <v/>
       </c>
-      <c r="E16" s="34">
+      <c r="E16" s="14">
         <f>IFERROR(C16/(C16+D16),0)</f>
         <v/>
       </c>
-      <c r="F16" s="35">
+      <c r="F16" s="15">
         <f>SUMIFS('Picks'!$BY$2:$BY$39,'Picks'!$H$2:$H$39,$A16)</f>
         <v/>
       </c>
@@ -1001,7 +971,6 @@
         <v/>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="22" t="inlineStr">
         <is>
@@ -1554,7 +1523,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J2" s="38" t="n"/>
+      <c r="J2" s="25" t="n"/>
       <c r="K2" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -1563,7 +1532,7 @@
       <c r="L2" s="26" t="n">
         <v>117</v>
       </c>
-      <c r="M2" s="39" t="n">
+      <c r="M2" s="27" t="n">
         <v>2.17</v>
       </c>
       <c r="N2" s="28" t="n">
@@ -1603,11 +1572,11 @@
       <c r="X2" s="26" t="n">
         <v>108</v>
       </c>
-      <c r="Y2" s="38" t="n"/>
+      <c r="Y2" s="25" t="n"/>
       <c r="Z2" s="26" t="n"/>
       <c r="AA2" s="28" t="n"/>
       <c r="AB2" s="28" t="n"/>
-      <c r="AC2" s="40" t="n">
+      <c r="AC2" s="30" t="n">
         <v>1.755</v>
       </c>
       <c r="AD2" s="24" t="inlineStr">
@@ -1744,11 +1713,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ2" s="38" t="n"/>
+      <c r="BJ2" s="25" t="n"/>
       <c r="BK2" s="26" t="n">
         <v>117</v>
       </c>
-      <c r="BL2" s="39" t="n">
+      <c r="BL2" s="27" t="n">
         <v>2.17</v>
       </c>
       <c r="BM2" s="28" t="n">
@@ -1758,18 +1727,18 @@
         <v>0.455446</v>
       </c>
       <c r="BO2" s="28" t="n"/>
-      <c r="BP2" s="38" t="n"/>
-      <c r="BQ2" s="39" t="n"/>
+      <c r="BP2" s="25" t="n"/>
+      <c r="BQ2" s="27" t="n"/>
       <c r="BR2" s="28" t="n"/>
       <c r="BS2" s="28" t="n"/>
       <c r="BT2" s="28" t="n"/>
-      <c r="BU2" s="38" t="n"/>
+      <c r="BU2" s="25" t="n"/>
       <c r="BV2" s="29" t="n"/>
       <c r="BW2" s="24" t="n"/>
-      <c r="BX2" s="40" t="n">
+      <c r="BX2" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY2" s="39" t="n">
+      <c r="BY2" s="27" t="n">
         <v>1.17</v>
       </c>
       <c r="BZ2" s="24" t="inlineStr">
@@ -1829,7 +1798,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J3" s="38" t="n"/>
+      <c r="J3" s="25" t="n"/>
       <c r="K3" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -1838,7 +1807,7 @@
       <c r="L3" s="26" t="n">
         <v>-133</v>
       </c>
-      <c r="M3" s="39" t="n">
+      <c r="M3" s="27" t="n">
         <v>1.75188</v>
       </c>
       <c r="N3" s="28" t="n">
@@ -1878,11 +1847,11 @@
       <c r="X3" s="26" t="n">
         <v>8</v>
       </c>
-      <c r="Y3" s="38" t="n"/>
+      <c r="Y3" s="25" t="n"/>
       <c r="Z3" s="26" t="n"/>
       <c r="AA3" s="28" t="n"/>
       <c r="AB3" s="28" t="n"/>
-      <c r="AC3" s="40" t="n">
+      <c r="AC3" s="30" t="n">
         <v>1.1278</v>
       </c>
       <c r="AD3" s="24" t="inlineStr">
@@ -2019,11 +1988,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ3" s="38" t="n"/>
+      <c r="BJ3" s="25" t="n"/>
       <c r="BK3" s="26" t="n">
         <v>-133</v>
       </c>
-      <c r="BL3" s="39" t="n">
+      <c r="BL3" s="27" t="n">
         <v>1.75188</v>
       </c>
       <c r="BM3" s="28" t="n">
@@ -2033,18 +2002,18 @@
         <v>0.567164</v>
       </c>
       <c r="BO3" s="28" t="n"/>
-      <c r="BP3" s="38" t="n"/>
-      <c r="BQ3" s="39" t="n"/>
+      <c r="BP3" s="25" t="n"/>
+      <c r="BQ3" s="27" t="n"/>
       <c r="BR3" s="28" t="n"/>
       <c r="BS3" s="28" t="n"/>
       <c r="BT3" s="28" t="n"/>
-      <c r="BU3" s="38" t="n"/>
+      <c r="BU3" s="25" t="n"/>
       <c r="BV3" s="29" t="n"/>
       <c r="BW3" s="24" t="n"/>
-      <c r="BX3" s="40" t="n">
+      <c r="BX3" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY3" s="39" t="n">
+      <c r="BY3" s="27" t="n">
         <v>0.75188</v>
       </c>
       <c r="BZ3" s="24" t="inlineStr">
@@ -2104,7 +2073,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J4" s="38" t="n"/>
+      <c r="J4" s="25" t="n"/>
       <c r="K4" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -2113,7 +2082,7 @@
       <c r="L4" s="26" t="n">
         <v>-102</v>
       </c>
-      <c r="M4" s="39" t="n">
+      <c r="M4" s="27" t="n">
         <v>1.980392</v>
       </c>
       <c r="N4" s="28" t="n">
@@ -2153,11 +2122,11 @@
       <c r="X4" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="Y4" s="38" t="n"/>
+      <c r="Y4" s="25" t="n"/>
       <c r="Z4" s="26" t="n"/>
       <c r="AA4" s="28" t="n"/>
       <c r="AB4" s="28" t="n"/>
-      <c r="AC4" s="40" t="n">
+      <c r="AC4" s="30" t="n">
         <v>-1</v>
       </c>
       <c r="AD4" s="24" t="inlineStr">
@@ -2294,11 +2263,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ4" s="38" t="n"/>
+      <c r="BJ4" s="25" t="n"/>
       <c r="BK4" s="26" t="n">
         <v>-102</v>
       </c>
-      <c r="BL4" s="39" t="n">
+      <c r="BL4" s="27" t="n">
         <v>1.980392</v>
       </c>
       <c r="BM4" s="28" t="n">
@@ -2308,18 +2277,18 @@
         <v>0.502488</v>
       </c>
       <c r="BO4" s="28" t="n"/>
-      <c r="BP4" s="38" t="n"/>
-      <c r="BQ4" s="39" t="n"/>
+      <c r="BP4" s="25" t="n"/>
+      <c r="BQ4" s="27" t="n"/>
       <c r="BR4" s="28" t="n"/>
       <c r="BS4" s="28" t="n"/>
       <c r="BT4" s="28" t="n"/>
-      <c r="BU4" s="38" t="n"/>
+      <c r="BU4" s="25" t="n"/>
       <c r="BV4" s="29" t="n"/>
       <c r="BW4" s="24" t="n"/>
-      <c r="BX4" s="40" t="n">
+      <c r="BX4" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY4" s="39" t="n">
+      <c r="BY4" s="27" t="n">
         <v>-1</v>
       </c>
       <c r="BZ4" s="24" t="inlineStr">
@@ -2379,7 +2348,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J5" s="38" t="n"/>
+      <c r="J5" s="25" t="n"/>
       <c r="K5" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -2388,7 +2357,7 @@
       <c r="L5" s="26" t="n">
         <v>-133</v>
       </c>
-      <c r="M5" s="39" t="n">
+      <c r="M5" s="27" t="n">
         <v>1.75188</v>
       </c>
       <c r="N5" s="28" t="n">
@@ -2428,11 +2397,11 @@
       <c r="X5" s="26" t="n">
         <v>6</v>
       </c>
-      <c r="Y5" s="38" t="n"/>
+      <c r="Y5" s="25" t="n"/>
       <c r="Z5" s="26" t="n"/>
       <c r="AA5" s="28" t="n"/>
       <c r="AB5" s="28" t="n"/>
-      <c r="AC5" s="40" t="n">
+      <c r="AC5" s="30" t="n">
         <v>1.1278</v>
       </c>
       <c r="AD5" s="24" t="inlineStr">
@@ -2569,11 +2538,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ5" s="38" t="n"/>
+      <c r="BJ5" s="25" t="n"/>
       <c r="BK5" s="26" t="n">
         <v>-133</v>
       </c>
-      <c r="BL5" s="39" t="n">
+      <c r="BL5" s="27" t="n">
         <v>1.75188</v>
       </c>
       <c r="BM5" s="28" t="n">
@@ -2583,18 +2552,18 @@
         <v>0.567164</v>
       </c>
       <c r="BO5" s="28" t="n"/>
-      <c r="BP5" s="38" t="n"/>
-      <c r="BQ5" s="39" t="n"/>
+      <c r="BP5" s="25" t="n"/>
+      <c r="BQ5" s="27" t="n"/>
       <c r="BR5" s="28" t="n"/>
       <c r="BS5" s="28" t="n"/>
       <c r="BT5" s="28" t="n"/>
-      <c r="BU5" s="38" t="n"/>
+      <c r="BU5" s="25" t="n"/>
       <c r="BV5" s="29" t="n"/>
       <c r="BW5" s="24" t="n"/>
-      <c r="BX5" s="40" t="n">
+      <c r="BX5" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY5" s="39" t="n">
+      <c r="BY5" s="27" t="n">
         <v>0.75188</v>
       </c>
       <c r="BZ5" s="24" t="inlineStr">
@@ -2654,7 +2623,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J6" s="38" t="n"/>
+      <c r="J6" s="25" t="n"/>
       <c r="K6" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -2663,7 +2632,7 @@
       <c r="L6" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="M6" s="39" t="n">
+      <c r="M6" s="27" t="n">
         <v>1.961538</v>
       </c>
       <c r="N6" s="28" t="n">
@@ -2703,11 +2672,11 @@
       <c r="X6" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="Y6" s="38" t="n"/>
+      <c r="Y6" s="25" t="n"/>
       <c r="Z6" s="26" t="n"/>
       <c r="AA6" s="28" t="n"/>
       <c r="AB6" s="28" t="n"/>
-      <c r="AC6" s="40" t="n">
+      <c r="AC6" s="30" t="n">
         <v>1.2019</v>
       </c>
       <c r="AD6" s="24" t="inlineStr">
@@ -2844,11 +2813,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ6" s="38" t="n"/>
+      <c r="BJ6" s="25" t="n"/>
       <c r="BK6" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="BL6" s="39" t="n">
+      <c r="BL6" s="27" t="n">
         <v>1.961538</v>
       </c>
       <c r="BM6" s="28" t="n">
@@ -2858,18 +2827,18 @@
         <v>0.507463</v>
       </c>
       <c r="BO6" s="28" t="n"/>
-      <c r="BP6" s="38" t="n"/>
-      <c r="BQ6" s="39" t="n"/>
+      <c r="BP6" s="25" t="n"/>
+      <c r="BQ6" s="27" t="n"/>
       <c r="BR6" s="28" t="n"/>
       <c r="BS6" s="28" t="n"/>
       <c r="BT6" s="28" t="n"/>
-      <c r="BU6" s="38" t="n"/>
+      <c r="BU6" s="25" t="n"/>
       <c r="BV6" s="29" t="n"/>
       <c r="BW6" s="24" t="n"/>
-      <c r="BX6" s="40" t="n">
+      <c r="BX6" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY6" s="39" t="n">
+      <c r="BY6" s="27" t="n">
         <v>0.961538</v>
       </c>
       <c r="BZ6" s="24" t="inlineStr">
@@ -2929,7 +2898,7 @@
           <t>away</t>
         </is>
       </c>
-      <c r="J7" s="38" t="n"/>
+      <c r="J7" s="25" t="n"/>
       <c r="K7" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -2938,7 +2907,7 @@
       <c r="L7" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="M7" s="39" t="n">
+      <c r="M7" s="27" t="n">
         <v>1.961538</v>
       </c>
       <c r="N7" s="28" t="n">
@@ -2978,11 +2947,11 @@
       <c r="X7" s="26" t="n">
         <v>10</v>
       </c>
-      <c r="Y7" s="38" t="n"/>
+      <c r="Y7" s="25" t="n"/>
       <c r="Z7" s="26" t="n"/>
       <c r="AA7" s="28" t="n"/>
       <c r="AB7" s="28" t="n"/>
-      <c r="AC7" s="40" t="n">
+      <c r="AC7" s="30" t="n">
         <v>-1.25</v>
       </c>
       <c r="AD7" s="24" t="inlineStr">
@@ -3119,11 +3088,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ7" s="38" t="n"/>
+      <c r="BJ7" s="25" t="n"/>
       <c r="BK7" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="BL7" s="39" t="n">
+      <c r="BL7" s="27" t="n">
         <v>1.961538</v>
       </c>
       <c r="BM7" s="28" t="n">
@@ -3133,18 +3102,18 @@
         <v>0.507463</v>
       </c>
       <c r="BO7" s="28" t="n"/>
-      <c r="BP7" s="38" t="n"/>
-      <c r="BQ7" s="39" t="n"/>
+      <c r="BP7" s="25" t="n"/>
+      <c r="BQ7" s="27" t="n"/>
       <c r="BR7" s="28" t="n"/>
       <c r="BS7" s="28" t="n"/>
       <c r="BT7" s="28" t="n"/>
-      <c r="BU7" s="38" t="n"/>
+      <c r="BU7" s="25" t="n"/>
       <c r="BV7" s="29" t="n"/>
       <c r="BW7" s="24" t="n"/>
-      <c r="BX7" s="40" t="n">
+      <c r="BX7" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY7" s="39" t="n">
+      <c r="BY7" s="27" t="n">
         <v>-1</v>
       </c>
       <c r="BZ7" s="24" t="inlineStr">
@@ -3204,7 +3173,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J8" s="38" t="n"/>
+      <c r="J8" s="25" t="n"/>
       <c r="K8" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -3213,7 +3182,7 @@
       <c r="L8" s="26" t="n">
         <v>-106</v>
       </c>
-      <c r="M8" s="39" t="n">
+      <c r="M8" s="27" t="n">
         <v>1.943396</v>
       </c>
       <c r="N8" s="28" t="n">
@@ -3253,11 +3222,11 @@
       <c r="X8" s="26" t="n">
         <v>6</v>
       </c>
-      <c r="Y8" s="38" t="n"/>
+      <c r="Y8" s="25" t="n"/>
       <c r="Z8" s="26" t="n"/>
       <c r="AA8" s="28" t="n"/>
       <c r="AB8" s="28" t="n"/>
-      <c r="AC8" s="40" t="n">
+      <c r="AC8" s="30" t="n">
         <v>-1</v>
       </c>
       <c r="AD8" s="24" t="inlineStr">
@@ -3394,11 +3363,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ8" s="38" t="n"/>
+      <c r="BJ8" s="25" t="n"/>
       <c r="BK8" s="26" t="n">
         <v>-106</v>
       </c>
-      <c r="BL8" s="39" t="n">
+      <c r="BL8" s="27" t="n">
         <v>1.943396</v>
       </c>
       <c r="BM8" s="28" t="n">
@@ -3408,18 +3377,18 @@
         <v>0.5124379999999999</v>
       </c>
       <c r="BO8" s="28" t="n"/>
-      <c r="BP8" s="38" t="n"/>
-      <c r="BQ8" s="39" t="n"/>
+      <c r="BP8" s="25" t="n"/>
+      <c r="BQ8" s="27" t="n"/>
       <c r="BR8" s="28" t="n"/>
       <c r="BS8" s="28" t="n"/>
       <c r="BT8" s="28" t="n"/>
-      <c r="BU8" s="38" t="n"/>
+      <c r="BU8" s="25" t="n"/>
       <c r="BV8" s="29" t="n"/>
       <c r="BW8" s="24" t="n"/>
-      <c r="BX8" s="40" t="n">
+      <c r="BX8" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY8" s="39" t="n">
+      <c r="BY8" s="27" t="n">
         <v>-1</v>
       </c>
       <c r="BZ8" s="24" t="inlineStr">
@@ -3479,7 +3448,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J9" s="38" t="n"/>
+      <c r="J9" s="25" t="n"/>
       <c r="K9" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -3488,7 +3457,7 @@
       <c r="L9" s="26" t="n">
         <v>-102</v>
       </c>
-      <c r="M9" s="39" t="n">
+      <c r="M9" s="27" t="n">
         <v>1.980392</v>
       </c>
       <c r="N9" s="28" t="n">
@@ -3528,11 +3497,11 @@
       <c r="X9" s="26" t="n">
         <v>5</v>
       </c>
-      <c r="Y9" s="38" t="n"/>
+      <c r="Y9" s="25" t="n"/>
       <c r="Z9" s="26" t="n"/>
       <c r="AA9" s="28" t="n"/>
       <c r="AB9" s="28" t="n"/>
-      <c r="AC9" s="40" t="n">
+      <c r="AC9" s="30" t="n">
         <v>0.9804</v>
       </c>
       <c r="AD9" s="24" t="inlineStr">
@@ -3669,11 +3638,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ9" s="38" t="n"/>
+      <c r="BJ9" s="25" t="n"/>
       <c r="BK9" s="26" t="n">
         <v>-102</v>
       </c>
-      <c r="BL9" s="39" t="n">
+      <c r="BL9" s="27" t="n">
         <v>1.980392</v>
       </c>
       <c r="BM9" s="28" t="n">
@@ -3683,18 +3652,18 @@
         <v>0.502488</v>
       </c>
       <c r="BO9" s="28" t="n"/>
-      <c r="BP9" s="38" t="n"/>
-      <c r="BQ9" s="39" t="n"/>
+      <c r="BP9" s="25" t="n"/>
+      <c r="BQ9" s="27" t="n"/>
       <c r="BR9" s="28" t="n"/>
       <c r="BS9" s="28" t="n"/>
       <c r="BT9" s="28" t="n"/>
-      <c r="BU9" s="38" t="n"/>
+      <c r="BU9" s="25" t="n"/>
       <c r="BV9" s="29" t="n"/>
       <c r="BW9" s="24" t="n"/>
-      <c r="BX9" s="40" t="n">
+      <c r="BX9" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY9" s="39" t="n">
+      <c r="BY9" s="27" t="n">
         <v>0.980392</v>
       </c>
       <c r="BZ9" s="24" t="inlineStr">
@@ -3754,7 +3723,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J10" s="38" t="n"/>
+      <c r="J10" s="25" t="n"/>
       <c r="K10" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -3763,7 +3732,7 @@
       <c r="L10" s="26" t="n">
         <v>-138</v>
       </c>
-      <c r="M10" s="39" t="n">
+      <c r="M10" s="27" t="n">
         <v>1.724638</v>
       </c>
       <c r="N10" s="28" t="n">
@@ -3803,11 +3772,11 @@
       <c r="X10" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="Y10" s="38" t="n"/>
+      <c r="Y10" s="25" t="n"/>
       <c r="Z10" s="26" t="n"/>
       <c r="AA10" s="28" t="n"/>
       <c r="AB10" s="28" t="n"/>
-      <c r="AC10" s="40" t="n">
+      <c r="AC10" s="30" t="n">
         <v>1.2681</v>
       </c>
       <c r="AD10" s="24" t="inlineStr">
@@ -3944,11 +3913,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ10" s="38" t="n"/>
+      <c r="BJ10" s="25" t="n"/>
       <c r="BK10" s="26" t="n">
         <v>-138</v>
       </c>
-      <c r="BL10" s="39" t="n">
+      <c r="BL10" s="27" t="n">
         <v>1.724638</v>
       </c>
       <c r="BM10" s="28" t="n">
@@ -3958,18 +3927,18 @@
         <v>0.577114</v>
       </c>
       <c r="BO10" s="28" t="n"/>
-      <c r="BP10" s="38" t="n"/>
-      <c r="BQ10" s="39" t="n"/>
+      <c r="BP10" s="25" t="n"/>
+      <c r="BQ10" s="27" t="n"/>
       <c r="BR10" s="28" t="n"/>
       <c r="BS10" s="28" t="n"/>
       <c r="BT10" s="28" t="n"/>
-      <c r="BU10" s="38" t="n"/>
+      <c r="BU10" s="25" t="n"/>
       <c r="BV10" s="29" t="n"/>
       <c r="BW10" s="24" t="n"/>
-      <c r="BX10" s="40" t="n">
+      <c r="BX10" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY10" s="39" t="n">
+      <c r="BY10" s="27" t="n">
         <v>0.724638</v>
       </c>
       <c r="BZ10" s="24" t="inlineStr">
@@ -4029,7 +3998,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J11" s="38" t="n"/>
+      <c r="J11" s="25" t="n"/>
       <c r="K11" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -4038,7 +4007,7 @@
       <c r="L11" s="26" t="n">
         <v>102</v>
       </c>
-      <c r="M11" s="39" t="n">
+      <c r="M11" s="27" t="n">
         <v>2.02</v>
       </c>
       <c r="N11" s="28" t="n">
@@ -4078,11 +4047,11 @@
       <c r="X11" s="26" t="n">
         <v>15</v>
       </c>
-      <c r="Y11" s="38" t="n"/>
+      <c r="Y11" s="25" t="n"/>
       <c r="Z11" s="26" t="n"/>
       <c r="AA11" s="28" t="n"/>
       <c r="AB11" s="28" t="n"/>
-      <c r="AC11" s="40" t="n">
+      <c r="AC11" s="30" t="n">
         <v>1.275</v>
       </c>
       <c r="AD11" s="24" t="inlineStr">
@@ -4219,11 +4188,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ11" s="38" t="n"/>
+      <c r="BJ11" s="25" t="n"/>
       <c r="BK11" s="26" t="n">
         <v>102</v>
       </c>
-      <c r="BL11" s="39" t="n">
+      <c r="BL11" s="27" t="n">
         <v>2.02</v>
       </c>
       <c r="BM11" s="28" t="n">
@@ -4233,18 +4202,18 @@
         <v>0.492537</v>
       </c>
       <c r="BO11" s="28" t="n"/>
-      <c r="BP11" s="38" t="n"/>
-      <c r="BQ11" s="39" t="n"/>
+      <c r="BP11" s="25" t="n"/>
+      <c r="BQ11" s="27" t="n"/>
       <c r="BR11" s="28" t="n"/>
       <c r="BS11" s="28" t="n"/>
       <c r="BT11" s="28" t="n"/>
-      <c r="BU11" s="38" t="n"/>
+      <c r="BU11" s="25" t="n"/>
       <c r="BV11" s="29" t="n"/>
       <c r="BW11" s="24" t="n"/>
-      <c r="BX11" s="40" t="n">
+      <c r="BX11" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY11" s="39" t="n">
+      <c r="BY11" s="27" t="n">
         <v>1.02</v>
       </c>
       <c r="BZ11" s="24" t="inlineStr">
@@ -4304,7 +4273,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J12" s="38" t="n"/>
+      <c r="J12" s="25" t="n"/>
       <c r="K12" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -4313,7 +4282,7 @@
       <c r="L12" s="26" t="n">
         <v>-102</v>
       </c>
-      <c r="M12" s="39" t="n">
+      <c r="M12" s="27" t="n">
         <v>1.980392</v>
       </c>
       <c r="N12" s="28" t="n">
@@ -4353,11 +4322,11 @@
       <c r="X12" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="Y12" s="38" t="n"/>
+      <c r="Y12" s="25" t="n"/>
       <c r="Z12" s="26" t="n"/>
       <c r="AA12" s="28" t="n"/>
       <c r="AB12" s="28" t="n"/>
-      <c r="AC12" s="40" t="n">
+      <c r="AC12" s="30" t="n">
         <v>-1</v>
       </c>
       <c r="AD12" s="24" t="inlineStr">
@@ -4494,11 +4463,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ12" s="38" t="n"/>
+      <c r="BJ12" s="25" t="n"/>
       <c r="BK12" s="26" t="n">
         <v>-102</v>
       </c>
-      <c r="BL12" s="39" t="n">
+      <c r="BL12" s="27" t="n">
         <v>1.980392</v>
       </c>
       <c r="BM12" s="28" t="n">
@@ -4508,18 +4477,18 @@
         <v>0.502488</v>
       </c>
       <c r="BO12" s="28" t="n"/>
-      <c r="BP12" s="38" t="n"/>
-      <c r="BQ12" s="39" t="n"/>
+      <c r="BP12" s="25" t="n"/>
+      <c r="BQ12" s="27" t="n"/>
       <c r="BR12" s="28" t="n"/>
       <c r="BS12" s="28" t="n"/>
       <c r="BT12" s="28" t="n"/>
-      <c r="BU12" s="38" t="n"/>
+      <c r="BU12" s="25" t="n"/>
       <c r="BV12" s="29" t="n"/>
       <c r="BW12" s="24" t="n"/>
-      <c r="BX12" s="40" t="n">
+      <c r="BX12" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY12" s="39" t="n">
+      <c r="BY12" s="27" t="n">
         <v>-1</v>
       </c>
       <c r="BZ12" s="24" t="inlineStr">
@@ -4579,7 +4548,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J13" s="38" t="n"/>
+      <c r="J13" s="25" t="n"/>
       <c r="K13" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -4588,7 +4557,7 @@
       <c r="L13" s="26" t="n">
         <v>-102</v>
       </c>
-      <c r="M13" s="39" t="n">
+      <c r="M13" s="27" t="n">
         <v>1.980392</v>
       </c>
       <c r="N13" s="28" t="n">
@@ -4628,11 +4597,11 @@
       <c r="X13" s="26" t="n">
         <v>7</v>
       </c>
-      <c r="Y13" s="38" t="n"/>
+      <c r="Y13" s="25" t="n"/>
       <c r="Z13" s="26" t="n"/>
       <c r="AA13" s="28" t="n"/>
       <c r="AB13" s="28" t="n"/>
-      <c r="AC13" s="40" t="n">
+      <c r="AC13" s="30" t="n">
         <v>1.2255</v>
       </c>
       <c r="AD13" s="24" t="inlineStr">
@@ -4769,11 +4738,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ13" s="38" t="n"/>
+      <c r="BJ13" s="25" t="n"/>
       <c r="BK13" s="26" t="n">
         <v>-102</v>
       </c>
-      <c r="BL13" s="39" t="n">
+      <c r="BL13" s="27" t="n">
         <v>1.980392</v>
       </c>
       <c r="BM13" s="28" t="n">
@@ -4783,18 +4752,18 @@
         <v>0.502488</v>
       </c>
       <c r="BO13" s="28" t="n"/>
-      <c r="BP13" s="38" t="n"/>
-      <c r="BQ13" s="39" t="n"/>
+      <c r="BP13" s="25" t="n"/>
+      <c r="BQ13" s="27" t="n"/>
       <c r="BR13" s="28" t="n"/>
       <c r="BS13" s="28" t="n"/>
       <c r="BT13" s="28" t="n"/>
-      <c r="BU13" s="38" t="n"/>
+      <c r="BU13" s="25" t="n"/>
       <c r="BV13" s="29" t="n"/>
       <c r="BW13" s="24" t="n"/>
-      <c r="BX13" s="40" t="n">
+      <c r="BX13" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY13" s="39" t="n">
+      <c r="BY13" s="27" t="n">
         <v>0.980392</v>
       </c>
       <c r="BZ13" s="24" t="inlineStr">
@@ -4854,7 +4823,7 @@
           <t>away</t>
         </is>
       </c>
-      <c r="J14" s="38" t="n"/>
+      <c r="J14" s="25" t="n"/>
       <c r="K14" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -4863,7 +4832,7 @@
       <c r="L14" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="M14" s="39" t="n">
+      <c r="M14" s="27" t="n">
         <v>1.961538</v>
       </c>
       <c r="N14" s="28" t="n">
@@ -4903,11 +4872,11 @@
       <c r="X14" s="26" t="n">
         <v>6</v>
       </c>
-      <c r="Y14" s="38" t="n"/>
+      <c r="Y14" s="25" t="n"/>
       <c r="Z14" s="26" t="n"/>
       <c r="AA14" s="28" t="n"/>
       <c r="AB14" s="28" t="n"/>
-      <c r="AC14" s="40" t="n">
+      <c r="AC14" s="30" t="n">
         <v>-0.75</v>
       </c>
       <c r="AD14" s="24" t="inlineStr">
@@ -5044,11 +5013,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ14" s="38" t="n"/>
+      <c r="BJ14" s="25" t="n"/>
       <c r="BK14" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="BL14" s="39" t="n">
+      <c r="BL14" s="27" t="n">
         <v>1.961538</v>
       </c>
       <c r="BM14" s="28" t="n">
@@ -5058,18 +5027,18 @@
         <v>0.507463</v>
       </c>
       <c r="BO14" s="28" t="n"/>
-      <c r="BP14" s="38" t="n"/>
-      <c r="BQ14" s="39" t="n"/>
+      <c r="BP14" s="25" t="n"/>
+      <c r="BQ14" s="27" t="n"/>
       <c r="BR14" s="28" t="n"/>
       <c r="BS14" s="28" t="n"/>
       <c r="BT14" s="28" t="n"/>
-      <c r="BU14" s="38" t="n"/>
+      <c r="BU14" s="25" t="n"/>
       <c r="BV14" s="29" t="n"/>
       <c r="BW14" s="24" t="n"/>
-      <c r="BX14" s="40" t="n">
+      <c r="BX14" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY14" s="39" t="n">
+      <c r="BY14" s="27" t="n">
         <v>-1</v>
       </c>
       <c r="BZ14" s="24" t="inlineStr">
@@ -5129,7 +5098,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J15" s="38" t="n"/>
+      <c r="J15" s="25" t="n"/>
       <c r="K15" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -5138,7 +5107,7 @@
       <c r="L15" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="M15" s="39" t="n">
+      <c r="M15" s="27" t="n">
         <v>1.961538</v>
       </c>
       <c r="N15" s="28" t="n">
@@ -5178,11 +5147,11 @@
       <c r="X15" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="Y15" s="38" t="n"/>
+      <c r="Y15" s="25" t="n"/>
       <c r="Z15" s="26" t="n"/>
       <c r="AA15" s="28" t="n"/>
       <c r="AB15" s="28" t="n"/>
-      <c r="AC15" s="40" t="n">
+      <c r="AC15" s="30" t="n">
         <v>-1</v>
       </c>
       <c r="AD15" s="24" t="inlineStr">
@@ -5319,11 +5288,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ15" s="38" t="n"/>
+      <c r="BJ15" s="25" t="n"/>
       <c r="BK15" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="BL15" s="39" t="n">
+      <c r="BL15" s="27" t="n">
         <v>1.961538</v>
       </c>
       <c r="BM15" s="28" t="n">
@@ -5333,18 +5302,18 @@
         <v>0.507463</v>
       </c>
       <c r="BO15" s="28" t="n"/>
-      <c r="BP15" s="38" t="n"/>
-      <c r="BQ15" s="39" t="n"/>
+      <c r="BP15" s="25" t="n"/>
+      <c r="BQ15" s="27" t="n"/>
       <c r="BR15" s="28" t="n"/>
       <c r="BS15" s="28" t="n"/>
       <c r="BT15" s="28" t="n"/>
-      <c r="BU15" s="38" t="n"/>
+      <c r="BU15" s="25" t="n"/>
       <c r="BV15" s="29" t="n"/>
       <c r="BW15" s="24" t="n"/>
-      <c r="BX15" s="40" t="n">
+      <c r="BX15" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY15" s="39" t="n">
+      <c r="BY15" s="27" t="n">
         <v>-1</v>
       </c>
       <c r="BZ15" s="24" t="inlineStr">
@@ -5404,7 +5373,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J16" s="38" t="n"/>
+      <c r="J16" s="25" t="n"/>
       <c r="K16" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -5413,7 +5382,7 @@
       <c r="L16" s="26" t="n">
         <v>-111</v>
       </c>
-      <c r="M16" s="39" t="n">
+      <c r="M16" s="27" t="n">
         <v>1.900901</v>
       </c>
       <c r="N16" s="28" t="n">
@@ -5453,11 +5422,11 @@
       <c r="X16" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="Y16" s="38" t="n"/>
+      <c r="Y16" s="25" t="n"/>
       <c r="Z16" s="26" t="n"/>
       <c r="AA16" s="28" t="n"/>
       <c r="AB16" s="28" t="n"/>
-      <c r="AC16" s="40" t="n">
+      <c r="AC16" s="30" t="n">
         <v>-1.5</v>
       </c>
       <c r="AD16" s="24" t="inlineStr">
@@ -5594,11 +5563,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ16" s="38" t="n"/>
+      <c r="BJ16" s="25" t="n"/>
       <c r="BK16" s="26" t="n">
         <v>-111</v>
       </c>
-      <c r="BL16" s="39" t="n">
+      <c r="BL16" s="27" t="n">
         <v>1.900901</v>
       </c>
       <c r="BM16" s="28" t="n">
@@ -5608,18 +5577,18 @@
         <v>0.522388</v>
       </c>
       <c r="BO16" s="28" t="n"/>
-      <c r="BP16" s="38" t="n"/>
-      <c r="BQ16" s="39" t="n"/>
+      <c r="BP16" s="25" t="n"/>
+      <c r="BQ16" s="27" t="n"/>
       <c r="BR16" s="28" t="n"/>
       <c r="BS16" s="28" t="n"/>
       <c r="BT16" s="28" t="n"/>
-      <c r="BU16" s="38" t="n"/>
+      <c r="BU16" s="25" t="n"/>
       <c r="BV16" s="29" t="n"/>
       <c r="BW16" s="24" t="n"/>
-      <c r="BX16" s="40" t="n">
+      <c r="BX16" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY16" s="39" t="n">
+      <c r="BY16" s="27" t="n">
         <v>-1</v>
       </c>
       <c r="BZ16" s="24" t="inlineStr">
@@ -5679,7 +5648,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J17" s="38" t="n"/>
+      <c r="J17" s="25" t="n"/>
       <c r="K17" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -5688,7 +5657,7 @@
       <c r="L17" s="26" t="n">
         <v>-108</v>
       </c>
-      <c r="M17" s="39" t="n">
+      <c r="M17" s="27" t="n">
         <v>1.925926</v>
       </c>
       <c r="N17" s="28" t="n">
@@ -5728,11 +5697,11 @@
       <c r="X17" s="26" t="n">
         <v>6</v>
       </c>
-      <c r="Y17" s="38" t="n"/>
+      <c r="Y17" s="25" t="n"/>
       <c r="Z17" s="26" t="n"/>
       <c r="AA17" s="28" t="n"/>
       <c r="AB17" s="28" t="n"/>
-      <c r="AC17" s="40" t="n">
+      <c r="AC17" s="30" t="n">
         <v>0.9258999999999999</v>
       </c>
       <c r="AD17" s="24" t="inlineStr">
@@ -5869,11 +5838,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ17" s="38" t="n"/>
+      <c r="BJ17" s="25" t="n"/>
       <c r="BK17" s="26" t="n">
         <v>-108</v>
       </c>
-      <c r="BL17" s="39" t="n">
+      <c r="BL17" s="27" t="n">
         <v>1.925926</v>
       </c>
       <c r="BM17" s="28" t="n">
@@ -5883,18 +5852,18 @@
         <v>0.5148509999999999</v>
       </c>
       <c r="BO17" s="28" t="n"/>
-      <c r="BP17" s="38" t="n"/>
-      <c r="BQ17" s="39" t="n"/>
+      <c r="BP17" s="25" t="n"/>
+      <c r="BQ17" s="27" t="n"/>
       <c r="BR17" s="28" t="n"/>
       <c r="BS17" s="28" t="n"/>
       <c r="BT17" s="28" t="n"/>
-      <c r="BU17" s="38" t="n"/>
+      <c r="BU17" s="25" t="n"/>
       <c r="BV17" s="29" t="n"/>
       <c r="BW17" s="24" t="n"/>
-      <c r="BX17" s="40" t="n">
+      <c r="BX17" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY17" s="39" t="n">
+      <c r="BY17" s="27" t="n">
         <v>0.925926</v>
       </c>
       <c r="BZ17" s="24" t="inlineStr">
@@ -5954,7 +5923,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J18" s="38" t="n"/>
+      <c r="J18" s="25" t="n"/>
       <c r="K18" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -5963,7 +5932,7 @@
       <c r="L18" s="26" t="n">
         <v>111</v>
       </c>
-      <c r="M18" s="39" t="n">
+      <c r="M18" s="27" t="n">
         <v>2.11</v>
       </c>
       <c r="N18" s="28" t="n">
@@ -6003,11 +5972,11 @@
       <c r="X18" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="Y18" s="38" t="n"/>
+      <c r="Y18" s="25" t="n"/>
       <c r="Z18" s="26" t="n"/>
       <c r="AA18" s="28" t="n"/>
       <c r="AB18" s="28" t="n"/>
-      <c r="AC18" s="40" t="n">
+      <c r="AC18" s="30" t="n">
         <v>-1.25</v>
       </c>
       <c r="AD18" s="24" t="inlineStr">
@@ -6144,11 +6113,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ18" s="38" t="n"/>
+      <c r="BJ18" s="25" t="n"/>
       <c r="BK18" s="26" t="n">
         <v>111</v>
       </c>
-      <c r="BL18" s="39" t="n">
+      <c r="BL18" s="27" t="n">
         <v>2.11</v>
       </c>
       <c r="BM18" s="28" t="n">
@@ -6158,18 +6127,18 @@
         <v>0.472637</v>
       </c>
       <c r="BO18" s="28" t="n"/>
-      <c r="BP18" s="38" t="n"/>
-      <c r="BQ18" s="39" t="n"/>
+      <c r="BP18" s="25" t="n"/>
+      <c r="BQ18" s="27" t="n"/>
       <c r="BR18" s="28" t="n"/>
       <c r="BS18" s="28" t="n"/>
       <c r="BT18" s="28" t="n"/>
-      <c r="BU18" s="38" t="n"/>
+      <c r="BU18" s="25" t="n"/>
       <c r="BV18" s="29" t="n"/>
       <c r="BW18" s="24" t="n"/>
-      <c r="BX18" s="40" t="n">
+      <c r="BX18" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY18" s="39" t="n">
+      <c r="BY18" s="27" t="n">
         <v>-1</v>
       </c>
       <c r="BZ18" s="24" t="inlineStr">
@@ -6229,7 +6198,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J19" s="38" t="n"/>
+      <c r="J19" s="25" t="n"/>
       <c r="K19" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -6238,7 +6207,7 @@
       <c r="L19" s="26" t="n">
         <v>-125</v>
       </c>
-      <c r="M19" s="39" t="n">
+      <c r="M19" s="27" t="n">
         <v>1.8</v>
       </c>
       <c r="N19" s="28" t="n">
@@ -6278,11 +6247,11 @@
       <c r="X19" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="Y19" s="38" t="n"/>
+      <c r="Y19" s="25" t="n"/>
       <c r="Z19" s="26" t="n"/>
       <c r="AA19" s="28" t="n"/>
       <c r="AB19" s="28" t="n"/>
-      <c r="AC19" s="40" t="n">
+      <c r="AC19" s="30" t="n">
         <v>1.2</v>
       </c>
       <c r="AD19" s="24" t="inlineStr">
@@ -6419,11 +6388,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ19" s="38" t="n"/>
+      <c r="BJ19" s="25" t="n"/>
       <c r="BK19" s="26" t="n">
         <v>-125</v>
       </c>
-      <c r="BL19" s="39" t="n">
+      <c r="BL19" s="27" t="n">
         <v>1.8</v>
       </c>
       <c r="BM19" s="28" t="n">
@@ -6433,18 +6402,18 @@
         <v>0.552239</v>
       </c>
       <c r="BO19" s="28" t="n"/>
-      <c r="BP19" s="38" t="n"/>
-      <c r="BQ19" s="39" t="n"/>
+      <c r="BP19" s="25" t="n"/>
+      <c r="BQ19" s="27" t="n"/>
       <c r="BR19" s="28" t="n"/>
       <c r="BS19" s="28" t="n"/>
       <c r="BT19" s="28" t="n"/>
-      <c r="BU19" s="38" t="n"/>
+      <c r="BU19" s="25" t="n"/>
       <c r="BV19" s="29" t="n"/>
       <c r="BW19" s="24" t="n"/>
-      <c r="BX19" s="40" t="n">
+      <c r="BX19" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY19" s="39" t="n">
+      <c r="BY19" s="27" t="n">
         <v>0.8</v>
       </c>
       <c r="BZ19" s="24" t="inlineStr">
@@ -6504,7 +6473,7 @@
           <t>away</t>
         </is>
       </c>
-      <c r="J20" s="38" t="n"/>
+      <c r="J20" s="25" t="n"/>
       <c r="K20" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -6513,7 +6482,7 @@
       <c r="L20" s="26" t="n">
         <v>106</v>
       </c>
-      <c r="M20" s="39" t="n">
+      <c r="M20" s="27" t="n">
         <v>2.06</v>
       </c>
       <c r="N20" s="28" t="n">
@@ -6553,11 +6522,11 @@
       <c r="X20" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="Y20" s="38" t="n"/>
+      <c r="Y20" s="25" t="n"/>
       <c r="Z20" s="26" t="n"/>
       <c r="AA20" s="28" t="n"/>
       <c r="AB20" s="28" t="n"/>
-      <c r="AC20" s="40" t="n">
+      <c r="AC20" s="30" t="n">
         <v>0.795</v>
       </c>
       <c r="AD20" s="24" t="inlineStr">
@@ -6694,11 +6663,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ20" s="38" t="n"/>
+      <c r="BJ20" s="25" t="n"/>
       <c r="BK20" s="26" t="n">
         <v>106</v>
       </c>
-      <c r="BL20" s="39" t="n">
+      <c r="BL20" s="27" t="n">
         <v>2.06</v>
       </c>
       <c r="BM20" s="28" t="n">
@@ -6708,18 +6677,18 @@
         <v>0.482587</v>
       </c>
       <c r="BO20" s="28" t="n"/>
-      <c r="BP20" s="38" t="n"/>
-      <c r="BQ20" s="39" t="n"/>
+      <c r="BP20" s="25" t="n"/>
+      <c r="BQ20" s="27" t="n"/>
       <c r="BR20" s="28" t="n"/>
       <c r="BS20" s="28" t="n"/>
       <c r="BT20" s="28" t="n"/>
-      <c r="BU20" s="38" t="n"/>
+      <c r="BU20" s="25" t="n"/>
       <c r="BV20" s="29" t="n"/>
       <c r="BW20" s="24" t="n"/>
-      <c r="BX20" s="40" t="n">
+      <c r="BX20" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY20" s="39" t="n">
+      <c r="BY20" s="27" t="n">
         <v>1.06</v>
       </c>
       <c r="BZ20" s="24" t="inlineStr">
@@ -6779,7 +6748,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J21" s="38" t="n"/>
+      <c r="J21" s="25" t="n"/>
       <c r="K21" s="24" t="inlineStr">
         <is>
           <t>polymarket</t>
@@ -6788,7 +6757,7 @@
       <c r="L21" s="26" t="n">
         <v>-106</v>
       </c>
-      <c r="M21" s="39" t="n">
+      <c r="M21" s="27" t="n">
         <v>1.943396</v>
       </c>
       <c r="N21" s="28" t="n">
@@ -6830,11 +6799,11 @@
       <c r="X21" s="26" t="n">
         <v>10</v>
       </c>
-      <c r="Y21" s="38" t="n"/>
+      <c r="Y21" s="25" t="n"/>
       <c r="Z21" s="26" t="n"/>
       <c r="AA21" s="28" t="n"/>
       <c r="AB21" s="28" t="n"/>
-      <c r="AC21" s="40" t="n">
+      <c r="AC21" s="30" t="n">
         <v>0.9434</v>
       </c>
       <c r="AD21" s="24" t="inlineStr">
@@ -6893,11 +6862,11 @@
         </is>
       </c>
       <c r="BI21" s="24" t="n"/>
-      <c r="BJ21" s="38" t="n"/>
+      <c r="BJ21" s="25" t="n"/>
       <c r="BK21" s="26" t="n">
         <v>-106</v>
       </c>
-      <c r="BL21" s="39" t="n">
+      <c r="BL21" s="27" t="n">
         <v>1.943396</v>
       </c>
       <c r="BM21" s="28" t="n">
@@ -6907,16 +6876,16 @@
         <v>0.5124379999999999</v>
       </c>
       <c r="BO21" s="28" t="n"/>
-      <c r="BP21" s="38" t="n"/>
-      <c r="BQ21" s="39" t="n"/>
+      <c r="BP21" s="25" t="n"/>
+      <c r="BQ21" s="27" t="n"/>
       <c r="BR21" s="28" t="n"/>
       <c r="BS21" s="28" t="n"/>
       <c r="BT21" s="28" t="n"/>
-      <c r="BU21" s="38" t="n"/>
+      <c r="BU21" s="25" t="n"/>
       <c r="BV21" s="29" t="n"/>
       <c r="BW21" s="24" t="n"/>
-      <c r="BX21" s="40" t="n"/>
-      <c r="BY21" s="39" t="n"/>
+      <c r="BX21" s="30" t="n"/>
+      <c r="BY21" s="27" t="n"/>
       <c r="BZ21" s="24" t="n"/>
       <c r="CA21" s="31" t="n"/>
     </row>
@@ -6966,7 +6935,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J22" s="38" t="n"/>
+      <c r="J22" s="25" t="n"/>
       <c r="K22" s="24" t="inlineStr">
         <is>
           <t>polymarket</t>
@@ -6975,7 +6944,7 @@
       <c r="L22" s="26" t="n">
         <v>-106</v>
       </c>
-      <c r="M22" s="39" t="n">
+      <c r="M22" s="27" t="n">
         <v>1.943396</v>
       </c>
       <c r="N22" s="28" t="n">
@@ -7017,11 +6986,11 @@
       <c r="X22" s="26" t="n">
         <v>5</v>
       </c>
-      <c r="Y22" s="38" t="n"/>
+      <c r="Y22" s="25" t="n"/>
       <c r="Z22" s="26" t="n"/>
       <c r="AA22" s="28" t="n"/>
       <c r="AB22" s="28" t="n"/>
-      <c r="AC22" s="40" t="n">
+      <c r="AC22" s="30" t="n">
         <v>0.9434</v>
       </c>
       <c r="AD22" s="24" t="inlineStr">
@@ -7080,11 +7049,11 @@
         </is>
       </c>
       <c r="BI22" s="24" t="n"/>
-      <c r="BJ22" s="38" t="n"/>
+      <c r="BJ22" s="25" t="n"/>
       <c r="BK22" s="26" t="n">
         <v>-106</v>
       </c>
-      <c r="BL22" s="39" t="n">
+      <c r="BL22" s="27" t="n">
         <v>1.943396</v>
       </c>
       <c r="BM22" s="28" t="n">
@@ -7094,16 +7063,16 @@
         <v>0.5124379999999999</v>
       </c>
       <c r="BO22" s="28" t="n"/>
-      <c r="BP22" s="38" t="n"/>
-      <c r="BQ22" s="39" t="n"/>
+      <c r="BP22" s="25" t="n"/>
+      <c r="BQ22" s="27" t="n"/>
       <c r="BR22" s="28" t="n"/>
       <c r="BS22" s="28" t="n"/>
       <c r="BT22" s="28" t="n"/>
-      <c r="BU22" s="38" t="n"/>
+      <c r="BU22" s="25" t="n"/>
       <c r="BV22" s="29" t="n"/>
       <c r="BW22" s="24" t="n"/>
-      <c r="BX22" s="40" t="n"/>
-      <c r="BY22" s="39" t="n"/>
+      <c r="BX22" s="30" t="n"/>
+      <c r="BY22" s="27" t="n"/>
       <c r="BZ22" s="24" t="n"/>
       <c r="CA22" s="31" t="n"/>
     </row>
@@ -7153,7 +7122,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J23" s="38" t="n"/>
+      <c r="J23" s="25" t="n"/>
       <c r="K23" s="24" t="inlineStr">
         <is>
           <t>polymarket</t>
@@ -7162,7 +7131,7 @@
       <c r="L23" s="26" t="n">
         <v>-141</v>
       </c>
-      <c r="M23" s="39" t="n">
+      <c r="M23" s="27" t="n">
         <v>1.70922</v>
       </c>
       <c r="N23" s="28" t="n">
@@ -7204,11 +7173,11 @@
       <c r="X23" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="Y23" s="38" t="n"/>
+      <c r="Y23" s="25" t="n"/>
       <c r="Z23" s="26" t="n"/>
       <c r="AA23" s="28" t="n"/>
       <c r="AB23" s="28" t="n"/>
-      <c r="AC23" s="40" t="n">
+      <c r="AC23" s="30" t="n">
         <v>1.2411</v>
       </c>
       <c r="AD23" s="24" t="inlineStr">
@@ -7267,11 +7236,11 @@
         </is>
       </c>
       <c r="BI23" s="24" t="n"/>
-      <c r="BJ23" s="38" t="n"/>
+      <c r="BJ23" s="25" t="n"/>
       <c r="BK23" s="26" t="n">
         <v>-141</v>
       </c>
-      <c r="BL23" s="39" t="n">
+      <c r="BL23" s="27" t="n">
         <v>1.70922</v>
       </c>
       <c r="BM23" s="28" t="n">
@@ -7281,16 +7250,16 @@
         <v>0.58209</v>
       </c>
       <c r="BO23" s="28" t="n"/>
-      <c r="BP23" s="38" t="n"/>
-      <c r="BQ23" s="39" t="n"/>
+      <c r="BP23" s="25" t="n"/>
+      <c r="BQ23" s="27" t="n"/>
       <c r="BR23" s="28" t="n"/>
       <c r="BS23" s="28" t="n"/>
       <c r="BT23" s="28" t="n"/>
-      <c r="BU23" s="38" t="n"/>
+      <c r="BU23" s="25" t="n"/>
       <c r="BV23" s="29" t="n"/>
       <c r="BW23" s="24" t="n"/>
-      <c r="BX23" s="40" t="n"/>
-      <c r="BY23" s="39" t="n"/>
+      <c r="BX23" s="30" t="n"/>
+      <c r="BY23" s="27" t="n"/>
       <c r="BZ23" s="24" t="n"/>
       <c r="CA23" s="31" t="n"/>
     </row>
@@ -7340,7 +7309,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J24" s="38" t="n"/>
+      <c r="J24" s="25" t="n"/>
       <c r="K24" s="24" t="inlineStr">
         <is>
           <t>polymarket</t>
@@ -7349,7 +7318,7 @@
       <c r="L24" s="26" t="n">
         <v>-133</v>
       </c>
-      <c r="M24" s="39" t="n">
+      <c r="M24" s="27" t="n">
         <v>1.75188</v>
       </c>
       <c r="N24" s="28" t="n">
@@ -7391,11 +7360,11 @@
       <c r="X24" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="Y24" s="38" t="n"/>
+      <c r="Y24" s="25" t="n"/>
       <c r="Z24" s="26" t="n"/>
       <c r="AA24" s="28" t="n"/>
       <c r="AB24" s="28" t="n"/>
-      <c r="AC24" s="40" t="n">
+      <c r="AC24" s="30" t="n">
         <v>-1.5</v>
       </c>
       <c r="AD24" s="24" t="inlineStr">
@@ -7454,11 +7423,11 @@
         </is>
       </c>
       <c r="BI24" s="24" t="n"/>
-      <c r="BJ24" s="38" t="n"/>
+      <c r="BJ24" s="25" t="n"/>
       <c r="BK24" s="26" t="n">
         <v>-133</v>
       </c>
-      <c r="BL24" s="39" t="n">
+      <c r="BL24" s="27" t="n">
         <v>1.75188</v>
       </c>
       <c r="BM24" s="28" t="n">
@@ -7468,16 +7437,16 @@
         <v>0.567164</v>
       </c>
       <c r="BO24" s="28" t="n"/>
-      <c r="BP24" s="38" t="n"/>
-      <c r="BQ24" s="39" t="n"/>
+      <c r="BP24" s="25" t="n"/>
+      <c r="BQ24" s="27" t="n"/>
       <c r="BR24" s="28" t="n"/>
       <c r="BS24" s="28" t="n"/>
       <c r="BT24" s="28" t="n"/>
-      <c r="BU24" s="38" t="n"/>
+      <c r="BU24" s="25" t="n"/>
       <c r="BV24" s="29" t="n"/>
       <c r="BW24" s="24" t="n"/>
-      <c r="BX24" s="40" t="n"/>
-      <c r="BY24" s="39" t="n"/>
+      <c r="BX24" s="30" t="n"/>
+      <c r="BY24" s="27" t="n"/>
       <c r="BZ24" s="24" t="n"/>
       <c r="CA24" s="31" t="n"/>
     </row>
@@ -7527,7 +7496,7 @@
           <t>away</t>
         </is>
       </c>
-      <c r="J25" s="38" t="n"/>
+      <c r="J25" s="25" t="n"/>
       <c r="K25" s="24" t="inlineStr">
         <is>
           <t>polymarket</t>
@@ -7536,7 +7505,7 @@
       <c r="L25" s="26" t="n">
         <v>104</v>
       </c>
-      <c r="M25" s="39" t="n">
+      <c r="M25" s="27" t="n">
         <v>2.04</v>
       </c>
       <c r="N25" s="28" t="n">
@@ -7578,11 +7547,11 @@
       <c r="X25" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="Y25" s="38" t="n"/>
+      <c r="Y25" s="25" t="n"/>
       <c r="Z25" s="26" t="n"/>
       <c r="AA25" s="28" t="n"/>
       <c r="AB25" s="28" t="n"/>
-      <c r="AC25" s="40" t="n">
+      <c r="AC25" s="30" t="n">
         <v>1.3</v>
       </c>
       <c r="AD25" s="24" t="inlineStr">
@@ -7641,11 +7610,11 @@
         </is>
       </c>
       <c r="BI25" s="24" t="n"/>
-      <c r="BJ25" s="38" t="n"/>
+      <c r="BJ25" s="25" t="n"/>
       <c r="BK25" s="26" t="n">
         <v>104</v>
       </c>
-      <c r="BL25" s="39" t="n">
+      <c r="BL25" s="27" t="n">
         <v>2.04</v>
       </c>
       <c r="BM25" s="28" t="n">
@@ -7655,16 +7624,16 @@
         <v>0.487562</v>
       </c>
       <c r="BO25" s="28" t="n"/>
-      <c r="BP25" s="38" t="n"/>
-      <c r="BQ25" s="39" t="n"/>
+      <c r="BP25" s="25" t="n"/>
+      <c r="BQ25" s="27" t="n"/>
       <c r="BR25" s="28" t="n"/>
       <c r="BS25" s="28" t="n"/>
       <c r="BT25" s="28" t="n"/>
-      <c r="BU25" s="38" t="n"/>
+      <c r="BU25" s="25" t="n"/>
       <c r="BV25" s="29" t="n"/>
       <c r="BW25" s="24" t="n"/>
-      <c r="BX25" s="40" t="n"/>
-      <c r="BY25" s="39" t="n"/>
+      <c r="BX25" s="30" t="n"/>
+      <c r="BY25" s="27" t="n"/>
       <c r="BZ25" s="24" t="n"/>
       <c r="CA25" s="31" t="n"/>
     </row>
@@ -7714,7 +7683,7 @@
           <t>away</t>
         </is>
       </c>
-      <c r="J26" s="38" t="n"/>
+      <c r="J26" s="25" t="n"/>
       <c r="K26" s="24" t="inlineStr">
         <is>
           <t>polymarket</t>
@@ -7723,7 +7692,7 @@
       <c r="L26" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="M26" s="39" t="n">
+      <c r="M26" s="27" t="n">
         <v>1.961538</v>
       </c>
       <c r="N26" s="28" t="n">
@@ -7765,11 +7734,11 @@
       <c r="X26" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="Y26" s="38" t="n"/>
+      <c r="Y26" s="25" t="n"/>
       <c r="Z26" s="26" t="n"/>
       <c r="AA26" s="28" t="n"/>
       <c r="AB26" s="28" t="n"/>
-      <c r="AC26" s="40" t="n">
+      <c r="AC26" s="30" t="n">
         <v>0.9615</v>
       </c>
       <c r="AD26" s="24" t="inlineStr">
@@ -7828,11 +7797,11 @@
         </is>
       </c>
       <c r="BI26" s="24" t="n"/>
-      <c r="BJ26" s="38" t="n"/>
+      <c r="BJ26" s="25" t="n"/>
       <c r="BK26" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="BL26" s="39" t="n">
+      <c r="BL26" s="27" t="n">
         <v>1.961538</v>
       </c>
       <c r="BM26" s="28" t="n">
@@ -7842,16 +7811,16 @@
         <v>0.507463</v>
       </c>
       <c r="BO26" s="28" t="n"/>
-      <c r="BP26" s="38" t="n"/>
-      <c r="BQ26" s="39" t="n"/>
+      <c r="BP26" s="25" t="n"/>
+      <c r="BQ26" s="27" t="n"/>
       <c r="BR26" s="28" t="n"/>
       <c r="BS26" s="28" t="n"/>
       <c r="BT26" s="28" t="n"/>
-      <c r="BU26" s="38" t="n"/>
+      <c r="BU26" s="25" t="n"/>
       <c r="BV26" s="29" t="n"/>
       <c r="BW26" s="24" t="n"/>
-      <c r="BX26" s="40" t="n"/>
-      <c r="BY26" s="39" t="n"/>
+      <c r="BX26" s="30" t="n"/>
+      <c r="BY26" s="27" t="n"/>
       <c r="BZ26" s="24" t="n"/>
       <c r="CA26" s="31" t="n"/>
     </row>
@@ -7901,7 +7870,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J27" s="38" t="n"/>
+      <c r="J27" s="25" t="n"/>
       <c r="K27" s="24" t="inlineStr">
         <is>
           <t>polymarket</t>
@@ -7910,7 +7879,7 @@
       <c r="L27" s="26" t="n">
         <v>120</v>
       </c>
-      <c r="M27" s="39" t="n">
+      <c r="M27" s="27" t="n">
         <v>2.2</v>
       </c>
       <c r="N27" s="28" t="n">
@@ -7952,11 +7921,11 @@
       <c r="X27" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="Y27" s="38" t="n"/>
+      <c r="Y27" s="25" t="n"/>
       <c r="Z27" s="26" t="n"/>
       <c r="AA27" s="28" t="n"/>
       <c r="AB27" s="28" t="n"/>
-      <c r="AC27" s="40" t="n">
+      <c r="AC27" s="30" t="n">
         <v>-0.75</v>
       </c>
       <c r="AD27" s="24" t="inlineStr">
@@ -8015,11 +7984,11 @@
         </is>
       </c>
       <c r="BI27" s="24" t="n"/>
-      <c r="BJ27" s="38" t="n"/>
+      <c r="BJ27" s="25" t="n"/>
       <c r="BK27" s="26" t="n">
         <v>120</v>
       </c>
-      <c r="BL27" s="39" t="n">
+      <c r="BL27" s="27" t="n">
         <v>2.2</v>
       </c>
       <c r="BM27" s="28" t="n">
@@ -8029,16 +7998,16 @@
         <v>0.452736</v>
       </c>
       <c r="BO27" s="28" t="n"/>
-      <c r="BP27" s="38" t="n"/>
-      <c r="BQ27" s="39" t="n"/>
+      <c r="BP27" s="25" t="n"/>
+      <c r="BQ27" s="27" t="n"/>
       <c r="BR27" s="28" t="n"/>
       <c r="BS27" s="28" t="n"/>
       <c r="BT27" s="28" t="n"/>
-      <c r="BU27" s="38" t="n"/>
+      <c r="BU27" s="25" t="n"/>
       <c r="BV27" s="29" t="n"/>
       <c r="BW27" s="24" t="n"/>
-      <c r="BX27" s="40" t="n"/>
-      <c r="BY27" s="39" t="n"/>
+      <c r="BX27" s="30" t="n"/>
+      <c r="BY27" s="27" t="n"/>
       <c r="BZ27" s="24" t="n"/>
       <c r="CA27" s="31" t="n"/>
     </row>
@@ -8088,7 +8057,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J28" s="38" t="n"/>
+      <c r="J28" s="25" t="n"/>
       <c r="K28" s="24" t="inlineStr">
         <is>
           <t>polymarket</t>
@@ -8097,7 +8066,7 @@
       <c r="L28" s="26" t="n">
         <v>100</v>
       </c>
-      <c r="M28" s="39" t="n">
+      <c r="M28" s="27" t="n">
         <v>2</v>
       </c>
       <c r="N28" s="28" t="n">
@@ -8139,11 +8108,11 @@
       <c r="X28" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="Y28" s="38" t="n"/>
+      <c r="Y28" s="25" t="n"/>
       <c r="Z28" s="26" t="n"/>
       <c r="AA28" s="28" t="n"/>
       <c r="AB28" s="28" t="n"/>
-      <c r="AC28" s="40" t="n">
+      <c r="AC28" s="30" t="n">
         <v>-0.75</v>
       </c>
       <c r="AD28" s="24" t="inlineStr">
@@ -8202,11 +8171,11 @@
         </is>
       </c>
       <c r="BI28" s="24" t="n"/>
-      <c r="BJ28" s="38" t="n"/>
+      <c r="BJ28" s="25" t="n"/>
       <c r="BK28" s="26" t="n">
         <v>100</v>
       </c>
-      <c r="BL28" s="39" t="n">
+      <c r="BL28" s="27" t="n">
         <v>2</v>
       </c>
       <c r="BM28" s="28" t="n">
@@ -8216,16 +8185,16 @@
         <v>0.497512</v>
       </c>
       <c r="BO28" s="28" t="n"/>
-      <c r="BP28" s="38" t="n"/>
-      <c r="BQ28" s="39" t="n"/>
+      <c r="BP28" s="25" t="n"/>
+      <c r="BQ28" s="27" t="n"/>
       <c r="BR28" s="28" t="n"/>
       <c r="BS28" s="28" t="n"/>
       <c r="BT28" s="28" t="n"/>
-      <c r="BU28" s="38" t="n"/>
+      <c r="BU28" s="25" t="n"/>
       <c r="BV28" s="29" t="n"/>
       <c r="BW28" s="24" t="n"/>
-      <c r="BX28" s="40" t="n"/>
-      <c r="BY28" s="39" t="n"/>
+      <c r="BX28" s="30" t="n"/>
+      <c r="BY28" s="27" t="n"/>
       <c r="BZ28" s="24" t="n"/>
       <c r="CA28" s="31" t="n"/>
     </row>
@@ -8275,7 +8244,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J29" s="38" t="n"/>
+      <c r="J29" s="25" t="n"/>
       <c r="K29" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -8284,7 +8253,7 @@
       <c r="L29" s="26" t="n">
         <v>108</v>
       </c>
-      <c r="M29" s="39" t="n">
+      <c r="M29" s="27" t="n">
         <v>2.08</v>
       </c>
       <c r="N29" s="28" t="n">
@@ -8324,11 +8293,11 @@
       <c r="X29" s="26" t="n">
         <v>8</v>
       </c>
-      <c r="Y29" s="38" t="n"/>
+      <c r="Y29" s="25" t="n"/>
       <c r="Z29" s="26" t="n"/>
       <c r="AA29" s="28" t="n"/>
       <c r="AB29" s="28" t="n"/>
-      <c r="AC29" s="40" t="n">
+      <c r="AC29" s="30" t="n">
         <v>1.35</v>
       </c>
       <c r="AD29" s="24" t="inlineStr">
@@ -8465,11 +8434,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ29" s="38" t="n"/>
+      <c r="BJ29" s="25" t="n"/>
       <c r="BK29" s="26" t="n">
         <v>108</v>
       </c>
-      <c r="BL29" s="39" t="n">
+      <c r="BL29" s="27" t="n">
         <v>2.08</v>
       </c>
       <c r="BM29" s="28" t="n">
@@ -8479,18 +8448,18 @@
         <v>0.477612</v>
       </c>
       <c r="BO29" s="28" t="n"/>
-      <c r="BP29" s="38" t="n"/>
-      <c r="BQ29" s="39" t="n"/>
+      <c r="BP29" s="25" t="n"/>
+      <c r="BQ29" s="27" t="n"/>
       <c r="BR29" s="28" t="n"/>
       <c r="BS29" s="28" t="n"/>
       <c r="BT29" s="28" t="n"/>
-      <c r="BU29" s="38" t="n"/>
+      <c r="BU29" s="25" t="n"/>
       <c r="BV29" s="29" t="n"/>
       <c r="BW29" s="24" t="n"/>
-      <c r="BX29" s="40" t="n">
+      <c r="BX29" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY29" s="39" t="n">
+      <c r="BY29" s="27" t="n">
         <v>1.08</v>
       </c>
       <c r="BZ29" s="24" t="inlineStr">
@@ -8550,7 +8519,7 @@
           <t>away</t>
         </is>
       </c>
-      <c r="J30" s="38" t="n"/>
+      <c r="J30" s="25" t="n"/>
       <c r="K30" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -8559,7 +8528,7 @@
       <c r="L30" s="26" t="n">
         <v>-133</v>
       </c>
-      <c r="M30" s="39" t="n">
+      <c r="M30" s="27" t="n">
         <v>1.75188</v>
       </c>
       <c r="N30" s="28" t="n">
@@ -8599,11 +8568,11 @@
       <c r="X30" s="26" t="n">
         <v>6</v>
       </c>
-      <c r="Y30" s="38" t="n"/>
+      <c r="Y30" s="25" t="n"/>
       <c r="Z30" s="26" t="n"/>
       <c r="AA30" s="28" t="n"/>
       <c r="AB30" s="28" t="n"/>
-      <c r="AC30" s="40" t="n">
+      <c r="AC30" s="30" t="n">
         <v>1.1278</v>
       </c>
       <c r="AD30" s="24" t="inlineStr">
@@ -8740,11 +8709,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ30" s="38" t="n"/>
+      <c r="BJ30" s="25" t="n"/>
       <c r="BK30" s="26" t="n">
         <v>-133</v>
       </c>
-      <c r="BL30" s="39" t="n">
+      <c r="BL30" s="27" t="n">
         <v>1.75188</v>
       </c>
       <c r="BM30" s="28" t="n">
@@ -8754,18 +8723,18 @@
         <v>0.567164</v>
       </c>
       <c r="BO30" s="28" t="n"/>
-      <c r="BP30" s="38" t="n"/>
-      <c r="BQ30" s="39" t="n"/>
+      <c r="BP30" s="25" t="n"/>
+      <c r="BQ30" s="27" t="n"/>
       <c r="BR30" s="28" t="n"/>
       <c r="BS30" s="28" t="n"/>
       <c r="BT30" s="28" t="n"/>
-      <c r="BU30" s="38" t="n"/>
+      <c r="BU30" s="25" t="n"/>
       <c r="BV30" s="29" t="n"/>
       <c r="BW30" s="24" t="n"/>
-      <c r="BX30" s="40" t="n">
+      <c r="BX30" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY30" s="39" t="n">
+      <c r="BY30" s="27" t="n">
         <v>0.75188</v>
       </c>
       <c r="BZ30" s="24" t="inlineStr">
@@ -8825,7 +8794,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J31" s="38" t="n"/>
+      <c r="J31" s="25" t="n"/>
       <c r="K31" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -8834,7 +8803,7 @@
       <c r="L31" s="26" t="n">
         <v>130</v>
       </c>
-      <c r="M31" s="39" t="n">
+      <c r="M31" s="27" t="n">
         <v>2.3</v>
       </c>
       <c r="N31" s="28" t="n">
@@ -8874,11 +8843,11 @@
       <c r="X31" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="Y31" s="38" t="n"/>
+      <c r="Y31" s="25" t="n"/>
       <c r="Z31" s="26" t="n"/>
       <c r="AA31" s="28" t="n"/>
       <c r="AB31" s="28" t="n"/>
-      <c r="AC31" s="40" t="n">
+      <c r="AC31" s="30" t="n">
         <v>-1</v>
       </c>
       <c r="AD31" s="24" t="inlineStr">
@@ -9015,11 +8984,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ31" s="38" t="n"/>
+      <c r="BJ31" s="25" t="n"/>
       <c r="BK31" s="26" t="n">
         <v>130</v>
       </c>
-      <c r="BL31" s="39" t="n">
+      <c r="BL31" s="27" t="n">
         <v>2.3</v>
       </c>
       <c r="BM31" s="28" t="n">
@@ -9029,18 +8998,18 @@
         <v>0.432836</v>
       </c>
       <c r="BO31" s="28" t="n"/>
-      <c r="BP31" s="38" t="n"/>
-      <c r="BQ31" s="39" t="n"/>
+      <c r="BP31" s="25" t="n"/>
+      <c r="BQ31" s="27" t="n"/>
       <c r="BR31" s="28" t="n"/>
       <c r="BS31" s="28" t="n"/>
       <c r="BT31" s="28" t="n"/>
-      <c r="BU31" s="38" t="n"/>
+      <c r="BU31" s="25" t="n"/>
       <c r="BV31" s="29" t="n"/>
       <c r="BW31" s="24" t="n"/>
-      <c r="BX31" s="40" t="n">
+      <c r="BX31" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="BY31" s="39" t="n">
+      <c r="BY31" s="27" t="n">
         <v>-1</v>
       </c>
       <c r="BZ31" s="24" t="inlineStr">
@@ -9100,7 +9069,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J32" s="38" t="n"/>
+      <c r="J32" s="25" t="n"/>
       <c r="K32" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -9109,7 +9078,7 @@
       <c r="L32" s="26" t="n">
         <v>113</v>
       </c>
-      <c r="M32" s="39" t="n">
+      <c r="M32" s="27" t="n">
         <v>2.13</v>
       </c>
       <c r="N32" s="28" t="n">
@@ -9141,11 +9110,11 @@
       <c r="V32" s="24" t="n"/>
       <c r="W32" s="26" t="n"/>
       <c r="X32" s="26" t="n"/>
-      <c r="Y32" s="38" t="n"/>
+      <c r="Y32" s="25" t="n"/>
       <c r="Z32" s="26" t="n"/>
       <c r="AA32" s="28" t="n"/>
       <c r="AB32" s="28" t="n"/>
-      <c r="AC32" s="40" t="n"/>
+      <c r="AC32" s="30" t="n"/>
       <c r="AD32" s="24" t="n"/>
       <c r="AE32" s="31" t="inlineStr">
         <is>
@@ -9276,11 +9245,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ32" s="38" t="n"/>
+      <c r="BJ32" s="25" t="n"/>
       <c r="BK32" s="26" t="n">
         <v>113</v>
       </c>
-      <c r="BL32" s="39" t="n">
+      <c r="BL32" s="27" t="n">
         <v>2.13</v>
       </c>
       <c r="BM32" s="28" t="n">
@@ -9290,16 +9259,16 @@
         <v>0.467662</v>
       </c>
       <c r="BO32" s="28" t="n"/>
-      <c r="BP32" s="38" t="n"/>
-      <c r="BQ32" s="39" t="n"/>
+      <c r="BP32" s="25" t="n"/>
+      <c r="BQ32" s="27" t="n"/>
       <c r="BR32" s="28" t="n"/>
       <c r="BS32" s="28" t="n"/>
       <c r="BT32" s="28" t="n"/>
-      <c r="BU32" s="38" t="n"/>
+      <c r="BU32" s="25" t="n"/>
       <c r="BV32" s="29" t="n"/>
       <c r="BW32" s="24" t="n"/>
-      <c r="BX32" s="40" t="n"/>
-      <c r="BY32" s="39" t="n"/>
+      <c r="BX32" s="30" t="n"/>
+      <c r="BY32" s="27" t="n"/>
       <c r="BZ32" s="24" t="n"/>
       <c r="CA32" s="31" t="n"/>
     </row>
@@ -9349,7 +9318,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J33" s="38" t="n"/>
+      <c r="J33" s="25" t="n"/>
       <c r="K33" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -9358,7 +9327,7 @@
       <c r="L33" s="26" t="n">
         <v>-108</v>
       </c>
-      <c r="M33" s="39" t="n">
+      <c r="M33" s="27" t="n">
         <v>1.925926</v>
       </c>
       <c r="N33" s="28" t="n">
@@ -9390,11 +9359,11 @@
       <c r="V33" s="24" t="n"/>
       <c r="W33" s="26" t="n"/>
       <c r="X33" s="26" t="n"/>
-      <c r="Y33" s="38" t="n"/>
+      <c r="Y33" s="25" t="n"/>
       <c r="Z33" s="26" t="n"/>
       <c r="AA33" s="28" t="n"/>
       <c r="AB33" s="28" t="n"/>
-      <c r="AC33" s="40" t="n"/>
+      <c r="AC33" s="30" t="n"/>
       <c r="AD33" s="24" t="n"/>
       <c r="AE33" s="31" t="inlineStr">
         <is>
@@ -9525,11 +9494,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ33" s="38" t="n"/>
+      <c r="BJ33" s="25" t="n"/>
       <c r="BK33" s="26" t="n">
         <v>-108</v>
       </c>
-      <c r="BL33" s="39" t="n">
+      <c r="BL33" s="27" t="n">
         <v>1.925926</v>
       </c>
       <c r="BM33" s="28" t="n">
@@ -9539,16 +9508,16 @@
         <v>0.517413</v>
       </c>
       <c r="BO33" s="28" t="n"/>
-      <c r="BP33" s="38" t="n"/>
-      <c r="BQ33" s="39" t="n"/>
+      <c r="BP33" s="25" t="n"/>
+      <c r="BQ33" s="27" t="n"/>
       <c r="BR33" s="28" t="n"/>
       <c r="BS33" s="28" t="n"/>
       <c r="BT33" s="28" t="n"/>
-      <c r="BU33" s="38" t="n"/>
+      <c r="BU33" s="25" t="n"/>
       <c r="BV33" s="29" t="n"/>
       <c r="BW33" s="24" t="n"/>
-      <c r="BX33" s="40" t="n"/>
-      <c r="BY33" s="39" t="n"/>
+      <c r="BX33" s="30" t="n"/>
+      <c r="BY33" s="27" t="n"/>
       <c r="BZ33" s="24" t="n"/>
       <c r="CA33" s="31" t="n"/>
     </row>
@@ -9598,7 +9567,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J34" s="38" t="n"/>
+      <c r="J34" s="25" t="n"/>
       <c r="K34" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -9607,7 +9576,7 @@
       <c r="L34" s="26" t="n">
         <v>-108</v>
       </c>
-      <c r="M34" s="39" t="n">
+      <c r="M34" s="27" t="n">
         <v>1.925926</v>
       </c>
       <c r="N34" s="28" t="n">
@@ -9639,11 +9608,11 @@
       <c r="V34" s="24" t="n"/>
       <c r="W34" s="26" t="n"/>
       <c r="X34" s="26" t="n"/>
-      <c r="Y34" s="38" t="n"/>
+      <c r="Y34" s="25" t="n"/>
       <c r="Z34" s="26" t="n"/>
       <c r="AA34" s="28" t="n"/>
       <c r="AB34" s="28" t="n"/>
-      <c r="AC34" s="40" t="n"/>
+      <c r="AC34" s="30" t="n"/>
       <c r="AD34" s="24" t="n"/>
       <c r="AE34" s="31" t="inlineStr">
         <is>
@@ -9774,11 +9743,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ34" s="38" t="n"/>
+      <c r="BJ34" s="25" t="n"/>
       <c r="BK34" s="26" t="n">
         <v>-108</v>
       </c>
-      <c r="BL34" s="39" t="n">
+      <c r="BL34" s="27" t="n">
         <v>1.925926</v>
       </c>
       <c r="BM34" s="28" t="n">
@@ -9788,16 +9757,16 @@
         <v>0.5148509999999999</v>
       </c>
       <c r="BO34" s="28" t="n"/>
-      <c r="BP34" s="38" t="n"/>
-      <c r="BQ34" s="39" t="n"/>
+      <c r="BP34" s="25" t="n"/>
+      <c r="BQ34" s="27" t="n"/>
       <c r="BR34" s="28" t="n"/>
       <c r="BS34" s="28" t="n"/>
       <c r="BT34" s="28" t="n"/>
-      <c r="BU34" s="38" t="n"/>
+      <c r="BU34" s="25" t="n"/>
       <c r="BV34" s="29" t="n"/>
       <c r="BW34" s="24" t="n"/>
-      <c r="BX34" s="40" t="n"/>
-      <c r="BY34" s="39" t="n"/>
+      <c r="BX34" s="30" t="n"/>
+      <c r="BY34" s="27" t="n"/>
       <c r="BZ34" s="24" t="n"/>
       <c r="CA34" s="31" t="n"/>
     </row>
@@ -9847,7 +9816,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J35" s="38" t="n"/>
+      <c r="J35" s="25" t="n"/>
       <c r="K35" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -9856,7 +9825,7 @@
       <c r="L35" s="26" t="n">
         <v>150</v>
       </c>
-      <c r="M35" s="39" t="n">
+      <c r="M35" s="27" t="n">
         <v>2.5</v>
       </c>
       <c r="N35" s="28" t="n">
@@ -9888,11 +9857,11 @@
       <c r="V35" s="24" t="n"/>
       <c r="W35" s="26" t="n"/>
       <c r="X35" s="26" t="n"/>
-      <c r="Y35" s="38" t="n"/>
+      <c r="Y35" s="25" t="n"/>
       <c r="Z35" s="26" t="n"/>
       <c r="AA35" s="28" t="n"/>
       <c r="AB35" s="28" t="n"/>
-      <c r="AC35" s="40" t="n"/>
+      <c r="AC35" s="30" t="n"/>
       <c r="AD35" s="24" t="n"/>
       <c r="AE35" s="31" t="inlineStr">
         <is>
@@ -10023,11 +9992,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ35" s="38" t="n"/>
+      <c r="BJ35" s="25" t="n"/>
       <c r="BK35" s="26" t="n">
         <v>150</v>
       </c>
-      <c r="BL35" s="39" t="n">
+      <c r="BL35" s="27" t="n">
         <v>2.5</v>
       </c>
       <c r="BM35" s="28" t="n">
@@ -10037,28 +10006,28 @@
         <v>0.39604</v>
       </c>
       <c r="BO35" s="28" t="n"/>
-      <c r="BP35" s="38" t="n"/>
-      <c r="BQ35" s="39" t="n"/>
+      <c r="BP35" s="25" t="n"/>
+      <c r="BQ35" s="27" t="n"/>
       <c r="BR35" s="28" t="n"/>
       <c r="BS35" s="28" t="n"/>
       <c r="BT35" s="28" t="n"/>
-      <c r="BU35" s="38" t="n"/>
+      <c r="BU35" s="25" t="n"/>
       <c r="BV35" s="29" t="n"/>
       <c r="BW35" s="24" t="n"/>
-      <c r="BX35" s="40" t="n"/>
-      <c r="BY35" s="39" t="n"/>
+      <c r="BX35" s="30" t="n"/>
+      <c r="BY35" s="27" t="n"/>
       <c r="BZ35" s="24" t="n"/>
       <c r="CA35" s="31" t="n"/>
     </row>
     <row r="36" ht="36" customHeight="1">
       <c r="A36" s="24" t="inlineStr">
         <is>
-          <t>2ca332931d5a4fdb</t>
+          <t>c799abfe71704ed8</t>
         </is>
       </c>
       <c r="B36" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T16:32:37.034238Z</t>
+          <t>2026-07-20T16:42:59.632078Z</t>
         </is>
       </c>
       <c r="C36" s="24" t="inlineStr">
@@ -10096,7 +10065,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J36" s="38" t="n"/>
+      <c r="J36" s="25" t="n"/>
       <c r="K36" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -10105,24 +10074,24 @@
       <c r="L36" s="26" t="n">
         <v>144</v>
       </c>
-      <c r="M36" s="39" t="n">
+      <c r="M36" s="27" t="n">
         <v>2.44</v>
       </c>
       <c r="N36" s="28" t="n">
         <v>0.409836</v>
       </c>
       <c r="O36" s="28" t="n">
-        <v>0.527501</v>
+        <v>0.597574</v>
       </c>
       <c r="P36" s="28" t="n"/>
       <c r="Q36" s="28" t="n">
-        <v>0.117501</v>
+        <v>0.187574</v>
       </c>
       <c r="R36" s="26" t="n">
         <v>100</v>
       </c>
       <c r="S36" s="29" t="n">
-        <v>0.75</v>
+        <v>1.5</v>
       </c>
       <c r="T36" s="24" t="inlineStr">
         <is>
@@ -10137,11 +10106,11 @@
       <c r="V36" s="24" t="n"/>
       <c r="W36" s="26" t="n"/>
       <c r="X36" s="26" t="n"/>
-      <c r="Y36" s="38" t="n"/>
+      <c r="Y36" s="25" t="n"/>
       <c r="Z36" s="26" t="n"/>
       <c r="AA36" s="28" t="n"/>
       <c r="AB36" s="28" t="n"/>
-      <c r="AC36" s="40" t="n"/>
+      <c r="AC36" s="30" t="n"/>
       <c r="AD36" s="24" t="n"/>
       <c r="AE36" s="31" t="inlineStr">
         <is>
@@ -10229,7 +10198,7 @@
       </c>
       <c r="BA36" s="24" t="inlineStr">
         <is>
-          <t>1f56359bf30bb6d51629a345226e3008ebfe73210551f6db9f5ce09f656ffdd6</t>
+          <t>4657ea085a2e161ea0063f513a6bf98a7c01549b126f36526876e6d6a2152307</t>
         </is>
       </c>
       <c r="BB36" s="24" t="inlineStr">
@@ -10244,7 +10213,7 @@
       </c>
       <c r="BD36" s="24" t="inlineStr">
         <is>
-          <t>1f56359bf30bb6d51629a345226e3008ebfe73210551f6db9f5ce09f656ffdd6</t>
+          <t>4657ea085a2e161ea0063f513a6bf98a7c01549b126f36526876e6d6a2152307</t>
         </is>
       </c>
       <c r="BE36" s="24" t="inlineStr">
@@ -10264,7 +10233,7 @@
       </c>
       <c r="BH36" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T16:32:37.034238Z</t>
+          <t>2026-07-20T16:42:59.632078Z</t>
         </is>
       </c>
       <c r="BI36" s="24" t="inlineStr">
@@ -10272,11 +10241,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ36" s="38" t="n"/>
+      <c r="BJ36" s="25" t="n"/>
       <c r="BK36" s="26" t="n">
         <v>144</v>
       </c>
-      <c r="BL36" s="39" t="n">
+      <c r="BL36" s="27" t="n">
         <v>2.44</v>
       </c>
       <c r="BM36" s="28" t="n">
@@ -10284,28 +10253,28 @@
       </c>
       <c r="BN36" s="28" t="n"/>
       <c r="BO36" s="28" t="n"/>
-      <c r="BP36" s="38" t="n"/>
-      <c r="BQ36" s="39" t="n"/>
+      <c r="BP36" s="25" t="n"/>
+      <c r="BQ36" s="27" t="n"/>
       <c r="BR36" s="28" t="n"/>
       <c r="BS36" s="28" t="n"/>
       <c r="BT36" s="28" t="n"/>
-      <c r="BU36" s="38" t="n"/>
+      <c r="BU36" s="25" t="n"/>
       <c r="BV36" s="29" t="n"/>
       <c r="BW36" s="24" t="n"/>
-      <c r="BX36" s="40" t="n"/>
-      <c r="BY36" s="39" t="n"/>
+      <c r="BX36" s="30" t="n"/>
+      <c r="BY36" s="27" t="n"/>
       <c r="BZ36" s="24" t="n"/>
       <c r="CA36" s="31" t="n"/>
     </row>
     <row r="37" ht="36" customHeight="1">
       <c r="A37" s="24" t="inlineStr">
         <is>
-          <t>19b13148b06b408d</t>
+          <t>88e300838c684314</t>
         </is>
       </c>
       <c r="B37" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T16:32:37.134076Z</t>
+          <t>2026-07-20T16:42:59.757524Z</t>
         </is>
       </c>
       <c r="C37" s="24" t="inlineStr">
@@ -10340,10 +10309,10 @@
       </c>
       <c r="I37" s="24" t="inlineStr">
         <is>
-          <t>away</t>
-        </is>
-      </c>
-      <c r="J37" s="38" t="n"/>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J37" s="25" t="n"/>
       <c r="K37" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -10352,24 +10321,24 @@
       <c r="L37" s="26" t="n">
         <v>186</v>
       </c>
-      <c r="M37" s="39" t="n">
+      <c r="M37" s="27" t="n">
         <v>2.86</v>
       </c>
       <c r="N37" s="28" t="n">
         <v>0.34965</v>
       </c>
       <c r="O37" s="28" t="n">
-        <v>0.533959</v>
+        <v>0.597891</v>
       </c>
       <c r="P37" s="28" t="n"/>
       <c r="Q37" s="28" t="n">
-        <v>0.183959</v>
+        <v>0.247891</v>
       </c>
       <c r="R37" s="26" t="n">
         <v>100</v>
       </c>
       <c r="S37" s="29" t="n">
-        <v>0.75</v>
+        <v>1.5</v>
       </c>
       <c r="T37" s="24" t="inlineStr">
         <is>
@@ -10384,11 +10353,11 @@
       <c r="V37" s="24" t="n"/>
       <c r="W37" s="26" t="n"/>
       <c r="X37" s="26" t="n"/>
-      <c r="Y37" s="38" t="n"/>
+      <c r="Y37" s="25" t="n"/>
       <c r="Z37" s="26" t="n"/>
       <c r="AA37" s="28" t="n"/>
       <c r="AB37" s="28" t="n"/>
-      <c r="AC37" s="40" t="n"/>
+      <c r="AC37" s="30" t="n"/>
       <c r="AD37" s="24" t="n"/>
       <c r="AE37" s="31" t="inlineStr">
         <is>
@@ -10476,7 +10445,7 @@
       </c>
       <c r="BA37" s="24" t="inlineStr">
         <is>
-          <t>1f56359bf30bb6d51629a345226e3008ebfe73210551f6db9f5ce09f656ffdd6</t>
+          <t>4657ea085a2e161ea0063f513a6bf98a7c01549b126f36526876e6d6a2152307</t>
         </is>
       </c>
       <c r="BB37" s="24" t="inlineStr">
@@ -10491,7 +10460,7 @@
       </c>
       <c r="BD37" s="24" t="inlineStr">
         <is>
-          <t>1f56359bf30bb6d51629a345226e3008ebfe73210551f6db9f5ce09f656ffdd6</t>
+          <t>4657ea085a2e161ea0063f513a6bf98a7c01549b126f36526876e6d6a2152307</t>
         </is>
       </c>
       <c r="BE37" s="24" t="inlineStr">
@@ -10511,7 +10480,7 @@
       </c>
       <c r="BH37" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T16:32:37.134076Z</t>
+          <t>2026-07-20T16:42:59.757524Z</t>
         </is>
       </c>
       <c r="BI37" s="24" t="inlineStr">
@@ -10519,11 +10488,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ37" s="38" t="n"/>
+      <c r="BJ37" s="25" t="n"/>
       <c r="BK37" s="26" t="n">
         <v>186</v>
       </c>
-      <c r="BL37" s="39" t="n">
+      <c r="BL37" s="27" t="n">
         <v>2.86</v>
       </c>
       <c r="BM37" s="28" t="n">
@@ -10531,28 +10500,28 @@
       </c>
       <c r="BN37" s="28" t="n"/>
       <c r="BO37" s="28" t="n"/>
-      <c r="BP37" s="38" t="n"/>
-      <c r="BQ37" s="39" t="n"/>
+      <c r="BP37" s="25" t="n"/>
+      <c r="BQ37" s="27" t="n"/>
       <c r="BR37" s="28" t="n"/>
       <c r="BS37" s="28" t="n"/>
       <c r="BT37" s="28" t="n"/>
-      <c r="BU37" s="38" t="n"/>
+      <c r="BU37" s="25" t="n"/>
       <c r="BV37" s="29" t="n"/>
       <c r="BW37" s="24" t="n"/>
-      <c r="BX37" s="40" t="n"/>
-      <c r="BY37" s="39" t="n"/>
+      <c r="BX37" s="30" t="n"/>
+      <c r="BY37" s="27" t="n"/>
       <c r="BZ37" s="24" t="n"/>
       <c r="CA37" s="31" t="n"/>
     </row>
     <row r="38" ht="36" customHeight="1">
       <c r="A38" s="24" t="inlineStr">
         <is>
-          <t>3646f4334f58469d</t>
+          <t>6fc69d654df04854</t>
         </is>
       </c>
       <c r="B38" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T16:32:43.485216Z</t>
+          <t>2026-07-20T16:43:06.018541Z</t>
         </is>
       </c>
       <c r="C38" s="24" t="inlineStr">
@@ -10587,36 +10556,36 @@
       </c>
       <c r="I38" s="24" t="inlineStr">
         <is>
-          <t>away</t>
-        </is>
-      </c>
-      <c r="J38" s="38" t="n"/>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J38" s="25" t="n"/>
       <c r="K38" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
         </is>
       </c>
       <c r="L38" s="26" t="n">
-        <v>113</v>
-      </c>
-      <c r="M38" s="39" t="n">
-        <v>2.13</v>
+        <v>223</v>
+      </c>
+      <c r="M38" s="27" t="n">
+        <v>3.23</v>
       </c>
       <c r="N38" s="28" t="n">
-        <v>0.469484</v>
+        <v>0.309598</v>
       </c>
       <c r="O38" s="28" t="n">
-        <v>0.576217</v>
+        <v>0.599201</v>
       </c>
       <c r="P38" s="28" t="n"/>
       <c r="Q38" s="28" t="n">
-        <v>0.106217</v>
+        <v>0.289201</v>
       </c>
       <c r="R38" s="26" t="n">
         <v>100</v>
       </c>
       <c r="S38" s="29" t="n">
-        <v>1.25</v>
+        <v>1.5</v>
       </c>
       <c r="T38" s="24" t="inlineStr">
         <is>
@@ -10631,15 +10600,15 @@
       <c r="V38" s="24" t="n"/>
       <c r="W38" s="26" t="n"/>
       <c r="X38" s="26" t="n"/>
-      <c r="Y38" s="38" t="n"/>
+      <c r="Y38" s="25" t="n"/>
       <c r="Z38" s="26" t="n"/>
       <c r="AA38" s="28" t="n"/>
       <c r="AB38" s="28" t="n"/>
-      <c r="AC38" s="40" t="n"/>
+      <c r="AC38" s="30" t="n"/>
       <c r="AD38" s="24" t="n"/>
       <c r="AE38" s="31" t="inlineStr">
         <is>
-          <t>Neutral Elo baseline; executable ask 0.4700 (aec-cs2-ica-ej-2026-07-20).</t>
+          <t>Neutral Elo baseline; executable ask 0.3100 (aec-cs2-ica-ej-2026-07-20).</t>
         </is>
       </c>
       <c r="AF38" s="31" t="inlineStr">
@@ -10723,7 +10692,7 @@
       </c>
       <c r="BA38" s="24" t="inlineStr">
         <is>
-          <t>40df7f7b9128e86cfbc485914f5801a00963b62604711b733b60f782ba9e258b</t>
+          <t>8ec29f8dd1985b5dbc96c1339c99e2a2129c4afa4af6efce101e4f76d99dce85</t>
         </is>
       </c>
       <c r="BB38" s="24" t="inlineStr">
@@ -10738,7 +10707,7 @@
       </c>
       <c r="BD38" s="24" t="inlineStr">
         <is>
-          <t>40df7f7b9128e86cfbc485914f5801a00963b62604711b733b60f782ba9e258b</t>
+          <t>8ec29f8dd1985b5dbc96c1339c99e2a2129c4afa4af6efce101e4f76d99dce85</t>
         </is>
       </c>
       <c r="BE38" s="24" t="inlineStr">
@@ -10758,7 +10727,7 @@
       </c>
       <c r="BH38" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T16:32:43.485216Z</t>
+          <t>2026-07-20T16:43:06.018541Z</t>
         </is>
       </c>
       <c r="BI38" s="24" t="inlineStr">
@@ -10766,40 +10735,40 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ38" s="38" t="n"/>
+      <c r="BJ38" s="25" t="n"/>
       <c r="BK38" s="26" t="n">
-        <v>113</v>
-      </c>
-      <c r="BL38" s="39" t="n">
-        <v>2.13</v>
+        <v>223</v>
+      </c>
+      <c r="BL38" s="27" t="n">
+        <v>3.23</v>
       </c>
       <c r="BM38" s="28" t="n">
-        <v>0.469484</v>
+        <v>0.309598</v>
       </c>
       <c r="BN38" s="28" t="n"/>
       <c r="BO38" s="28" t="n"/>
-      <c r="BP38" s="38" t="n"/>
-      <c r="BQ38" s="39" t="n"/>
+      <c r="BP38" s="25" t="n"/>
+      <c r="BQ38" s="27" t="n"/>
       <c r="BR38" s="28" t="n"/>
       <c r="BS38" s="28" t="n"/>
       <c r="BT38" s="28" t="n"/>
-      <c r="BU38" s="38" t="n"/>
+      <c r="BU38" s="25" t="n"/>
       <c r="BV38" s="29" t="n"/>
       <c r="BW38" s="24" t="n"/>
-      <c r="BX38" s="40" t="n"/>
-      <c r="BY38" s="39" t="n"/>
+      <c r="BX38" s="30" t="n"/>
+      <c r="BY38" s="27" t="n"/>
       <c r="BZ38" s="24" t="n"/>
       <c r="CA38" s="31" t="n"/>
     </row>
     <row r="39" ht="36" customHeight="1">
       <c r="A39" s="24" t="inlineStr">
         <is>
-          <t>a2f62addc7be49e9</t>
+          <t>eab33644ea2b4fc1</t>
         </is>
       </c>
       <c r="B39" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T16:32:43.612711Z</t>
+          <t>2026-07-20T16:43:06.145847Z</t>
         </is>
       </c>
       <c r="C39" s="24" t="inlineStr">
@@ -10837,7 +10806,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J39" s="38" t="n"/>
+      <c r="J39" s="25" t="n"/>
       <c r="K39" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -10846,18 +10815,18 @@
       <c r="L39" s="26" t="n">
         <v>-144</v>
       </c>
-      <c r="M39" s="39" t="n">
+      <c r="M39" s="27" t="n">
         <v>1.694444</v>
       </c>
       <c r="N39" s="28" t="n">
         <v>0.590164</v>
       </c>
       <c r="O39" s="28" t="n">
-        <v>0.692542</v>
+        <v>0.719007</v>
       </c>
       <c r="P39" s="28" t="n"/>
       <c r="Q39" s="28" t="n">
-        <v>0.102542</v>
+        <v>0.129007</v>
       </c>
       <c r="R39" s="26" t="n">
         <v>100</v>
@@ -10878,11 +10847,11 @@
       <c r="V39" s="24" t="n"/>
       <c r="W39" s="26" t="n"/>
       <c r="X39" s="26" t="n"/>
-      <c r="Y39" s="38" t="n"/>
+      <c r="Y39" s="25" t="n"/>
       <c r="Z39" s="26" t="n"/>
       <c r="AA39" s="28" t="n"/>
       <c r="AB39" s="28" t="n"/>
-      <c r="AC39" s="40" t="n"/>
+      <c r="AC39" s="30" t="n"/>
       <c r="AD39" s="24" t="n"/>
       <c r="AE39" s="31" t="inlineStr">
         <is>
@@ -10970,7 +10939,7 @@
       </c>
       <c r="BA39" s="24" t="inlineStr">
         <is>
-          <t>40df7f7b9128e86cfbc485914f5801a00963b62604711b733b60f782ba9e258b</t>
+          <t>8ec29f8dd1985b5dbc96c1339c99e2a2129c4afa4af6efce101e4f76d99dce85</t>
         </is>
       </c>
       <c r="BB39" s="24" t="inlineStr">
@@ -10985,7 +10954,7 @@
       </c>
       <c r="BD39" s="24" t="inlineStr">
         <is>
-          <t>40df7f7b9128e86cfbc485914f5801a00963b62604711b733b60f782ba9e258b</t>
+          <t>8ec29f8dd1985b5dbc96c1339c99e2a2129c4afa4af6efce101e4f76d99dce85</t>
         </is>
       </c>
       <c r="BE39" s="24" t="inlineStr">
@@ -11005,7 +10974,7 @@
       </c>
       <c r="BH39" s="24" t="inlineStr">
         <is>
-          <t>2026-07-20T16:32:43.612711Z</t>
+          <t>2026-07-20T16:43:06.145847Z</t>
         </is>
       </c>
       <c r="BI39" s="24" t="inlineStr">
@@ -11013,11 +10982,11 @@
           <t>["same_event","same_team_same_day","same_league_same_day"]</t>
         </is>
       </c>
-      <c r="BJ39" s="38" t="n"/>
+      <c r="BJ39" s="25" t="n"/>
       <c r="BK39" s="26" t="n">
         <v>-144</v>
       </c>
-      <c r="BL39" s="39" t="n">
+      <c r="BL39" s="27" t="n">
         <v>1.694444</v>
       </c>
       <c r="BM39" s="28" t="n">
@@ -11025,16 +10994,16 @@
       </c>
       <c r="BN39" s="28" t="n"/>
       <c r="BO39" s="28" t="n"/>
-      <c r="BP39" s="38" t="n"/>
-      <c r="BQ39" s="39" t="n"/>
+      <c r="BP39" s="25" t="n"/>
+      <c r="BQ39" s="27" t="n"/>
       <c r="BR39" s="28" t="n"/>
       <c r="BS39" s="28" t="n"/>
       <c r="BT39" s="28" t="n"/>
-      <c r="BU39" s="38" t="n"/>
+      <c r="BU39" s="25" t="n"/>
       <c r="BV39" s="29" t="n"/>
       <c r="BW39" s="24" t="n"/>
-      <c r="BX39" s="40" t="n"/>
-      <c r="BY39" s="39" t="n"/>
+      <c r="BX39" s="30" t="n"/>
+      <c r="BY39" s="27" t="n"/>
       <c r="BZ39" s="24" t="n"/>
       <c r="CA39" s="31" t="n"/>
     </row>

</xml_diff>

<commit_message>
feat: auto unit-value button (10% bankroll, ratchet-up only)
- /api/settings/auto-unit-value: computes bankroll from
  starting_bankroll_usd + main ledger settled/open P&L
- Sets unit_value_usd to 10% of bankroll, only ratchets UP
- Dashboard 10% button next to unit value input
- starting_bankroll_usd added to model.yaml bankroll config
</commit_message>
<xml_diff>
--- a/data/picks.xlsx
+++ b/data/picks.xlsx
@@ -327,8 +327,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CA71" headerRowCount="1">
-  <autoFilter ref="A1:CA71"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CA75" headerRowCount="1">
+  <autoFilter ref="A1:CA75"/>
   <tableColumns count="79">
     <tableColumn id="1" name="pick_id"/>
     <tableColumn id="2" name="created_at_utc"/>
@@ -765,19 +765,19 @@
     </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="6">
-        <f>COUNTA('Picks'!$A$2:$A$71)</f>
+        <f>COUNTA('Picks'!$A$2:$A$75)</f>
         <v/>
       </c>
       <c r="C4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$71,"open")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$75,"open")</f>
         <v/>
       </c>
       <c r="E4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$71,"settled")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$75,"settled")</f>
         <v/>
       </c>
       <c r="G4" s="6">
-        <f>IF(COUNTIFS('Picks'!$U$2:$U$71,"settled",'Picks'!$V$2:$V$71,"win")+COUNTIFS('Picks'!$U$2:$U$71,"settled",'Picks'!$V$2:$V$71,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
+        <f>IF(COUNTIFS('Picks'!$U$2:$U$75,"settled",'Picks'!$V$2:$V$75,"win")+COUNTIFS('Picks'!$U$2:$U$75,"settled",'Picks'!$V$2:$V$75,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
         <v/>
       </c>
     </row>
@@ -806,19 +806,19 @@
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="6">
-        <f>COUNTIF('Picks'!$BX$2:$BX$71,"&gt;0")</f>
+        <f>COUNTIF('Picks'!$BX$2:$BX$75,"&gt;0")</f>
         <v/>
       </c>
       <c r="C7" s="6">
-        <f>COUNTIFS('Picks'!$BX$2:$BX$71,"&gt;0",'Picks'!$V$2:$V$71,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$71,"&gt;0",'Picks'!$V$2:$V$71,"loss")</f>
+        <f>COUNTIFS('Picks'!$BX$2:$BX$75,"&gt;0",'Picks'!$V$2:$V$75,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$75,"&gt;0",'Picks'!$V$2:$V$75,"loss")</f>
         <v/>
       </c>
       <c r="E7" s="32">
-        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$71,"&gt;0",'Picks'!$V$2:$V$71,"win")/(COUNTIFS('Picks'!$BX$2:$BX$71,"&gt;0",'Picks'!$V$2:$V$71,"win")+COUNTIFS('Picks'!$BX$2:$BX$71,"&gt;0",'Picks'!$V$2:$V$71,"loss")),0)</f>
+        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$75,"&gt;0",'Picks'!$V$2:$V$75,"win")/(COUNTIFS('Picks'!$BX$2:$BX$75,"&gt;0",'Picks'!$V$2:$V$75,"win")+COUNTIFS('Picks'!$BX$2:$BX$75,"&gt;0",'Picks'!$V$2:$V$75,"loss")),0)</f>
         <v/>
       </c>
       <c r="G7" s="32">
-        <f>IFERROR(SUM('Picks'!$BY$2:$BY$71)/SUM('Picks'!$BX$2:$BX$71),0)</f>
+        <f>IFERROR(SUM('Picks'!$BY$2:$BY$75)/SUM('Picks'!$BX$2:$BX$75),0)</f>
         <v/>
       </c>
     </row>
@@ -847,19 +847,19 @@
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="33">
-        <f>SUM('Picks'!$BY$2:$BY$71)</f>
+        <f>SUM('Picks'!$BY$2:$BY$75)</f>
         <v/>
       </c>
       <c r="C10" s="9">
-        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$71,"&lt;&gt;",'Picks'!$AB$2:$AB$71),0)</f>
+        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$75,"&lt;&gt;",'Picks'!$AB$2:$AB$75),0)</f>
         <v/>
       </c>
       <c r="E10" s="6">
-        <f>COUNTIFS('Picks'!$AM$2:$AM$71,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$71,"settled")</f>
+        <f>COUNTIFS('Picks'!$AM$2:$AM$75,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$75,"settled")</f>
         <v/>
       </c>
       <c r="G10" s="33">
-        <f>SUMIFS('Picks'!$AC$2:$AC$71,'Picks'!$AM$2:$AM$71,"QUALIFIED_SHADOW_CALL")</f>
+        <f>SUMIFS('Picks'!$AC$2:$AC$75,'Picks'!$AM$2:$AM$75,"QUALIFIED_SHADOW_CALL")</f>
         <v/>
       </c>
     </row>
@@ -915,15 +915,15 @@
         </is>
       </c>
       <c r="B14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$71,$A14,'Picks'!$U$2:$U$71,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$75,$A14,'Picks'!$U$2:$U$75,"settled")</f>
         <v/>
       </c>
       <c r="C14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$71,$A14,'Picks'!$U$2:$U$71,"settled",'Picks'!$V$2:$V$71,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$75,$A14,'Picks'!$U$2:$U$75,"settled",'Picks'!$V$2:$V$75,"win")</f>
         <v/>
       </c>
       <c r="D14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$71,$A14,'Picks'!$U$2:$U$71,"settled",'Picks'!$V$2:$V$71,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$75,$A14,'Picks'!$U$2:$U$75,"settled",'Picks'!$V$2:$V$75,"loss")</f>
         <v/>
       </c>
       <c r="E14" s="34">
@@ -931,11 +931,11 @@
         <v/>
       </c>
       <c r="F14" s="35">
-        <f>SUMIFS('Picks'!$BY$2:$BY$71,'Picks'!$H$2:$H$71,$A14)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$75,'Picks'!$H$2:$H$75,$A14)</f>
         <v/>
       </c>
       <c r="G14" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$71,'Picks'!$H$2:$H$71,$A14,'Picks'!$U$2:$U$71,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$75,'Picks'!$H$2:$H$75,$A14,'Picks'!$U$2:$U$75,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -946,15 +946,15 @@
         </is>
       </c>
       <c r="B15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$71,$A15,'Picks'!$U$2:$U$71,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$75,$A15,'Picks'!$U$2:$U$75,"settled")</f>
         <v/>
       </c>
       <c r="C15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$71,$A15,'Picks'!$U$2:$U$71,"settled",'Picks'!$V$2:$V$71,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$75,$A15,'Picks'!$U$2:$U$75,"settled",'Picks'!$V$2:$V$75,"win")</f>
         <v/>
       </c>
       <c r="D15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$71,$A15,'Picks'!$U$2:$U$71,"settled",'Picks'!$V$2:$V$71,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$75,$A15,'Picks'!$U$2:$U$75,"settled",'Picks'!$V$2:$V$75,"loss")</f>
         <v/>
       </c>
       <c r="E15" s="36">
@@ -962,11 +962,11 @@
         <v/>
       </c>
       <c r="F15" s="37">
-        <f>SUMIFS('Picks'!$BY$2:$BY$71,'Picks'!$H$2:$H$71,$A15)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$75,'Picks'!$H$2:$H$75,$A15)</f>
         <v/>
       </c>
       <c r="G15" s="21">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$71,'Picks'!$H$2:$H$71,$A15,'Picks'!$U$2:$U$71,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$75,'Picks'!$H$2:$H$75,$A15,'Picks'!$U$2:$U$75,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -977,15 +977,15 @@
         </is>
       </c>
       <c r="B16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$71,$A16,'Picks'!$U$2:$U$71,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$75,$A16,'Picks'!$U$2:$U$75,"settled")</f>
         <v/>
       </c>
       <c r="C16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$71,$A16,'Picks'!$U$2:$U$71,"settled",'Picks'!$V$2:$V$71,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$75,$A16,'Picks'!$U$2:$U$75,"settled",'Picks'!$V$2:$V$75,"win")</f>
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$71,$A16,'Picks'!$U$2:$U$71,"settled",'Picks'!$V$2:$V$71,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$75,$A16,'Picks'!$U$2:$U$75,"settled",'Picks'!$V$2:$V$75,"loss")</f>
         <v/>
       </c>
       <c r="E16" s="34">
@@ -993,11 +993,11 @@
         <v/>
       </c>
       <c r="F16" s="35">
-        <f>SUMIFS('Picks'!$BY$2:$BY$71,'Picks'!$H$2:$H$71,$A16)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$75,'Picks'!$H$2:$H$75,$A16)</f>
         <v/>
       </c>
       <c r="G16" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$71,'Picks'!$H$2:$H$71,$A16,'Picks'!$U$2:$U$71,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$75,'Picks'!$H$2:$H$75,$A16,'Picks'!$U$2:$U$75,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -1027,7 +1027,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:CA71"/>
+  <dimension ref="A1:CA75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -19048,6 +19048,994 @@
       <c r="BZ71" s="24" t="n"/>
       <c r="CA71" s="31" t="n"/>
     </row>
+    <row r="72" ht="36" customHeight="1">
+      <c r="A72" s="24" t="inlineStr">
+        <is>
+          <t>c8e1a4ddb2b147b4</t>
+        </is>
+      </c>
+      <c r="B72" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-21T05:21:42.337431Z</t>
+        </is>
+      </c>
+      <c r="C72" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-21T18:30:00Z</t>
+        </is>
+      </c>
+      <c r="D72" s="24" t="inlineStr">
+        <is>
+          <t>58068</t>
+        </is>
+      </c>
+      <c r="E72" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F72" s="24" t="inlineStr">
+        <is>
+          <t>Strael-Bora</t>
+        </is>
+      </c>
+      <c r="G72" s="24" t="inlineStr">
+        <is>
+          <t>Bushido Wildcats</t>
+        </is>
+      </c>
+      <c r="H72" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I72" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J72" s="38" t="n"/>
+      <c r="K72" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L72" s="26" t="n">
+        <v>-223</v>
+      </c>
+      <c r="M72" s="39" t="n">
+        <v>1.44843</v>
+      </c>
+      <c r="N72" s="28" t="n">
+        <v>0.690402</v>
+      </c>
+      <c r="O72" s="28" t="n">
+        <v>0.710718</v>
+      </c>
+      <c r="P72" s="28" t="n"/>
+      <c r="Q72" s="28" t="n">
+        <v>0.020718</v>
+      </c>
+      <c r="R72" s="26" t="n">
+        <v>20</v>
+      </c>
+      <c r="S72" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="T72" s="24" t="inlineStr">
+        <is>
+          <t>cs2-neutral-series-elo-v1</t>
+        </is>
+      </c>
+      <c r="U72" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V72" s="24" t="n"/>
+      <c r="W72" s="26" t="n"/>
+      <c r="X72" s="26" t="n"/>
+      <c r="Y72" s="38" t="n"/>
+      <c r="Z72" s="26" t="n"/>
+      <c r="AA72" s="28" t="n"/>
+      <c r="AB72" s="28" t="n"/>
+      <c r="AC72" s="40" t="n"/>
+      <c r="AD72" s="24" t="n"/>
+      <c r="AE72" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.6900 (aec-cs2-bw-sb-2026-07-21).</t>
+        </is>
+      </c>
+      <c r="AF72" s="31" t="inlineStr">
+        <is>
+          <t>Research baseline; zero-unit shadow until qualified.</t>
+        </is>
+      </c>
+      <c r="AG72" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH72" s="24" t="n"/>
+      <c r="AI72" s="31" t="n"/>
+      <c r="AJ72" s="31" t="n"/>
+      <c r="AK72" s="24" t="inlineStr">
+        <is>
+          <t>model_qualified</t>
+        </is>
+      </c>
+      <c r="AL72" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM72" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED_SHADOW_CALL</t>
+        </is>
+      </c>
+      <c r="AN72" s="24" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="AO72" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED</t>
+        </is>
+      </c>
+      <c r="AP72" s="24" t="inlineStr">
+        <is>
+          <t>Strael-Bora</t>
+        </is>
+      </c>
+      <c r="AQ72" s="24" t="inlineStr">
+        <is>
+          <t>Strael-Bora</t>
+        </is>
+      </c>
+      <c r="AR72" s="24" t="inlineStr">
+        <is>
+          <t>Strael-Bora</t>
+        </is>
+      </c>
+      <c r="AS72" s="24" t="inlineStr">
+        <is>
+          <t>Bushido Wildcats</t>
+        </is>
+      </c>
+      <c r="AT72" s="24" t="inlineStr">
+        <is>
+          <t>Bushido Wildcats</t>
+        </is>
+      </c>
+      <c r="AU72" s="24" t="inlineStr">
+        <is>
+          <t>Bushido Wildcats</t>
+        </is>
+      </c>
+      <c r="AV72" s="24" t="n"/>
+      <c r="AW72" s="24" t="n"/>
+      <c r="AX72" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY72" s="24" t="n"/>
+      <c r="AZ72" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA72" s="24" t="inlineStr">
+        <is>
+          <t>9dbde86ab8062ac73a51c94b0ad431573ac8b755ccd742d86794849a749958c7</t>
+        </is>
+      </c>
+      <c r="BB72" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC72" s="24" t="inlineStr">
+        <is>
+          <t>cs2-neutral-series-elo-v1</t>
+        </is>
+      </c>
+      <c r="BD72" s="24" t="inlineStr">
+        <is>
+          <t>9dbde86ab8062ac73a51c94b0ad431573ac8b755ccd742d86794849a749958c7</t>
+        </is>
+      </c>
+      <c r="BE72" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF72" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG72" s="24" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="BH72" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-21T05:21:42.337431Z</t>
+        </is>
+      </c>
+      <c r="BI72" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ72" s="38" t="n"/>
+      <c r="BK72" s="26" t="n">
+        <v>-223</v>
+      </c>
+      <c r="BL72" s="39" t="n">
+        <v>1.44843</v>
+      </c>
+      <c r="BM72" s="28" t="n">
+        <v>0.690402</v>
+      </c>
+      <c r="BN72" s="28" t="n"/>
+      <c r="BO72" s="28" t="n"/>
+      <c r="BP72" s="38" t="n"/>
+      <c r="BQ72" s="39" t="n"/>
+      <c r="BR72" s="28" t="n"/>
+      <c r="BS72" s="28" t="n"/>
+      <c r="BT72" s="28" t="n"/>
+      <c r="BU72" s="38" t="n"/>
+      <c r="BV72" s="29" t="n"/>
+      <c r="BW72" s="24" t="n"/>
+      <c r="BX72" s="40" t="n"/>
+      <c r="BY72" s="39" t="n"/>
+      <c r="BZ72" s="24" t="n"/>
+      <c r="CA72" s="31" t="n"/>
+    </row>
+    <row r="73" ht="36" customHeight="1">
+      <c r="A73" s="24" t="inlineStr">
+        <is>
+          <t>29fb46cae668405f</t>
+        </is>
+      </c>
+      <c r="B73" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-21T08:13:56.528127Z</t>
+        </is>
+      </c>
+      <c r="C73" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-21T11:00:00Z</t>
+        </is>
+      </c>
+      <c r="D73" s="24" t="inlineStr">
+        <is>
+          <t>57524</t>
+        </is>
+      </c>
+      <c r="E73" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F73" s="24" t="inlineStr">
+        <is>
+          <t>Entropy</t>
+        </is>
+      </c>
+      <c r="G73" s="24" t="inlineStr">
+        <is>
+          <t>Esport Academy Copenhagen</t>
+        </is>
+      </c>
+      <c r="H73" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I73" s="24" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="J73" s="38" t="n"/>
+      <c r="K73" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L73" s="26" t="n">
+        <v>-108</v>
+      </c>
+      <c r="M73" s="39" t="n">
+        <v>1.925926</v>
+      </c>
+      <c r="N73" s="28" t="n">
+        <v>0.519231</v>
+      </c>
+      <c r="O73" s="28" t="n">
+        <v>0.602113</v>
+      </c>
+      <c r="P73" s="28" t="n"/>
+      <c r="Q73" s="28" t="n">
+        <v>0.08211300000000001</v>
+      </c>
+      <c r="R73" s="26" t="n">
+        <v>82</v>
+      </c>
+      <c r="S73" s="29" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="T73" s="24" t="inlineStr">
+        <is>
+          <t>cs2-neutral-series-elo-v1</t>
+        </is>
+      </c>
+      <c r="U73" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V73" s="24" t="n"/>
+      <c r="W73" s="26" t="n"/>
+      <c r="X73" s="26" t="n"/>
+      <c r="Y73" s="38" t="n"/>
+      <c r="Z73" s="26" t="n"/>
+      <c r="AA73" s="28" t="n"/>
+      <c r="AB73" s="28" t="n"/>
+      <c r="AC73" s="40" t="n"/>
+      <c r="AD73" s="24" t="n"/>
+      <c r="AE73" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.5200 (aec-cs2-eac-ent-2026-07-21).</t>
+        </is>
+      </c>
+      <c r="AF73" s="31" t="inlineStr">
+        <is>
+          <t>Research baseline; zero-unit shadow until qualified.</t>
+        </is>
+      </c>
+      <c r="AG73" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH73" s="24" t="n"/>
+      <c r="AI73" s="31" t="n"/>
+      <c r="AJ73" s="31" t="n"/>
+      <c r="AK73" s="24" t="inlineStr">
+        <is>
+          <t>model_qualified</t>
+        </is>
+      </c>
+      <c r="AL73" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM73" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED_SHADOW_CALL</t>
+        </is>
+      </c>
+      <c r="AN73" s="24" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="AO73" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED</t>
+        </is>
+      </c>
+      <c r="AP73" s="24" t="inlineStr">
+        <is>
+          <t>Entropy</t>
+        </is>
+      </c>
+      <c r="AQ73" s="24" t="inlineStr">
+        <is>
+          <t>Entropy</t>
+        </is>
+      </c>
+      <c r="AR73" s="24" t="inlineStr">
+        <is>
+          <t>Entropy</t>
+        </is>
+      </c>
+      <c r="AS73" s="24" t="inlineStr">
+        <is>
+          <t>Esport Academy Copenhagen</t>
+        </is>
+      </c>
+      <c r="AT73" s="24" t="inlineStr">
+        <is>
+          <t>Esport Academy Copenhagen</t>
+        </is>
+      </c>
+      <c r="AU73" s="24" t="inlineStr">
+        <is>
+          <t>Esport Academy Copenhagen</t>
+        </is>
+      </c>
+      <c r="AV73" s="24" t="n"/>
+      <c r="AW73" s="24" t="n"/>
+      <c r="AX73" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY73" s="24" t="n"/>
+      <c r="AZ73" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA73" s="24" t="inlineStr">
+        <is>
+          <t>9dbde86ab8062ac73a51c94b0ad431573ac8b755ccd742d86794849a749958c7</t>
+        </is>
+      </c>
+      <c r="BB73" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC73" s="24" t="inlineStr">
+        <is>
+          <t>cs2-neutral-series-elo-v1</t>
+        </is>
+      </c>
+      <c r="BD73" s="24" t="inlineStr">
+        <is>
+          <t>9dbde86ab8062ac73a51c94b0ad431573ac8b755ccd742d86794849a749958c7</t>
+        </is>
+      </c>
+      <c r="BE73" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF73" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG73" s="24" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="BH73" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-21T08:13:56.528127Z</t>
+        </is>
+      </c>
+      <c r="BI73" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ73" s="38" t="n"/>
+      <c r="BK73" s="26" t="n">
+        <v>-108</v>
+      </c>
+      <c r="BL73" s="39" t="n">
+        <v>1.925926</v>
+      </c>
+      <c r="BM73" s="28" t="n">
+        <v>0.519231</v>
+      </c>
+      <c r="BN73" s="28" t="n"/>
+      <c r="BO73" s="28" t="n"/>
+      <c r="BP73" s="38" t="n"/>
+      <c r="BQ73" s="39" t="n"/>
+      <c r="BR73" s="28" t="n"/>
+      <c r="BS73" s="28" t="n"/>
+      <c r="BT73" s="28" t="n"/>
+      <c r="BU73" s="38" t="n"/>
+      <c r="BV73" s="29" t="n"/>
+      <c r="BW73" s="24" t="n"/>
+      <c r="BX73" s="40" t="n"/>
+      <c r="BY73" s="39" t="n"/>
+      <c r="BZ73" s="24" t="n"/>
+      <c r="CA73" s="31" t="n"/>
+    </row>
+    <row r="74" ht="36" customHeight="1">
+      <c r="A74" s="24" t="inlineStr">
+        <is>
+          <t>42c5e25bbaa741b6</t>
+        </is>
+      </c>
+      <c r="B74" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-21T08:13:57.068809Z</t>
+        </is>
+      </c>
+      <c r="C74" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-21T16:00:00Z</t>
+        </is>
+      </c>
+      <c r="D74" s="24" t="inlineStr">
+        <is>
+          <t>56032</t>
+        </is>
+      </c>
+      <c r="E74" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F74" s="24" t="inlineStr">
+        <is>
+          <t>FOKUS</t>
+        </is>
+      </c>
+      <c r="G74" s="24" t="inlineStr">
+        <is>
+          <t>Astralis</t>
+        </is>
+      </c>
+      <c r="H74" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I74" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J74" s="38" t="n"/>
+      <c r="K74" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L74" s="26" t="n">
+        <v>-233</v>
+      </c>
+      <c r="M74" s="39" t="n">
+        <v>1.429185</v>
+      </c>
+      <c r="N74" s="28" t="n">
+        <v>0.6997</v>
+      </c>
+      <c r="O74" s="28" t="n">
+        <v>0.725656</v>
+      </c>
+      <c r="P74" s="28" t="n"/>
+      <c r="Q74" s="28" t="n">
+        <v>0.025656</v>
+      </c>
+      <c r="R74" s="26" t="n">
+        <v>25</v>
+      </c>
+      <c r="S74" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="T74" s="24" t="inlineStr">
+        <is>
+          <t>cs2-neutral-series-elo-v1</t>
+        </is>
+      </c>
+      <c r="U74" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V74" s="24" t="n"/>
+      <c r="W74" s="26" t="n"/>
+      <c r="X74" s="26" t="n"/>
+      <c r="Y74" s="38" t="n"/>
+      <c r="Z74" s="26" t="n"/>
+      <c r="AA74" s="28" t="n"/>
+      <c r="AB74" s="28" t="n"/>
+      <c r="AC74" s="40" t="n"/>
+      <c r="AD74" s="24" t="n"/>
+      <c r="AE74" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.7000 (aec-cs2-ast-fokus-2026-07-21).</t>
+        </is>
+      </c>
+      <c r="AF74" s="31" t="inlineStr">
+        <is>
+          <t>Research baseline; zero-unit shadow until qualified.</t>
+        </is>
+      </c>
+      <c r="AG74" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH74" s="24" t="n"/>
+      <c r="AI74" s="31" t="n"/>
+      <c r="AJ74" s="31" t="n"/>
+      <c r="AK74" s="24" t="inlineStr">
+        <is>
+          <t>model_qualified</t>
+        </is>
+      </c>
+      <c r="AL74" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM74" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED_SHADOW_CALL</t>
+        </is>
+      </c>
+      <c r="AN74" s="24" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="AO74" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED</t>
+        </is>
+      </c>
+      <c r="AP74" s="24" t="inlineStr">
+        <is>
+          <t>FOKUS</t>
+        </is>
+      </c>
+      <c r="AQ74" s="24" t="inlineStr">
+        <is>
+          <t>FOKUS</t>
+        </is>
+      </c>
+      <c r="AR74" s="24" t="inlineStr">
+        <is>
+          <t>FOKUS</t>
+        </is>
+      </c>
+      <c r="AS74" s="24" t="inlineStr">
+        <is>
+          <t>Astralis</t>
+        </is>
+      </c>
+      <c r="AT74" s="24" t="inlineStr">
+        <is>
+          <t>Astralis</t>
+        </is>
+      </c>
+      <c r="AU74" s="24" t="inlineStr">
+        <is>
+          <t>Astralis</t>
+        </is>
+      </c>
+      <c r="AV74" s="24" t="n"/>
+      <c r="AW74" s="24" t="n"/>
+      <c r="AX74" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY74" s="24" t="n"/>
+      <c r="AZ74" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA74" s="24" t="inlineStr">
+        <is>
+          <t>9dbde86ab8062ac73a51c94b0ad431573ac8b755ccd742d86794849a749958c7</t>
+        </is>
+      </c>
+      <c r="BB74" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC74" s="24" t="inlineStr">
+        <is>
+          <t>cs2-neutral-series-elo-v1</t>
+        </is>
+      </c>
+      <c r="BD74" s="24" t="inlineStr">
+        <is>
+          <t>9dbde86ab8062ac73a51c94b0ad431573ac8b755ccd742d86794849a749958c7</t>
+        </is>
+      </c>
+      <c r="BE74" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF74" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG74" s="24" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="BH74" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-21T08:13:57.068809Z</t>
+        </is>
+      </c>
+      <c r="BI74" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ74" s="38" t="n"/>
+      <c r="BK74" s="26" t="n">
+        <v>-233</v>
+      </c>
+      <c r="BL74" s="39" t="n">
+        <v>1.429185</v>
+      </c>
+      <c r="BM74" s="28" t="n">
+        <v>0.6997</v>
+      </c>
+      <c r="BN74" s="28" t="n"/>
+      <c r="BO74" s="28" t="n"/>
+      <c r="BP74" s="38" t="n"/>
+      <c r="BQ74" s="39" t="n"/>
+      <c r="BR74" s="28" t="n"/>
+      <c r="BS74" s="28" t="n"/>
+      <c r="BT74" s="28" t="n"/>
+      <c r="BU74" s="38" t="n"/>
+      <c r="BV74" s="29" t="n"/>
+      <c r="BW74" s="24" t="n"/>
+      <c r="BX74" s="40" t="n"/>
+      <c r="BY74" s="39" t="n"/>
+      <c r="BZ74" s="24" t="n"/>
+      <c r="CA74" s="31" t="n"/>
+    </row>
+    <row r="75" ht="36" customHeight="1">
+      <c r="A75" s="24" t="inlineStr">
+        <is>
+          <t>e4f64939c21b430a</t>
+        </is>
+      </c>
+      <c r="B75" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-21T08:13:57.416034Z</t>
+        </is>
+      </c>
+      <c r="C75" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-21T17:00:00Z</t>
+        </is>
+      </c>
+      <c r="D75" s="24" t="inlineStr">
+        <is>
+          <t>57988</t>
+        </is>
+      </c>
+      <c r="E75" s="24" t="inlineStr">
+        <is>
+          <t>CS2</t>
+        </is>
+      </c>
+      <c r="F75" s="24" t="inlineStr">
+        <is>
+          <t>Just Players</t>
+        </is>
+      </c>
+      <c r="G75" s="24" t="inlineStr">
+        <is>
+          <t>ex-RUSTEC</t>
+        </is>
+      </c>
+      <c r="H75" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I75" s="24" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="J75" s="38" t="n"/>
+      <c r="K75" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L75" s="26" t="n">
+        <v>-117</v>
+      </c>
+      <c r="M75" s="39" t="n">
+        <v>1.854701</v>
+      </c>
+      <c r="N75" s="28" t="n">
+        <v>0.539171</v>
+      </c>
+      <c r="O75" s="28" t="n">
+        <v>0.6339399999999999</v>
+      </c>
+      <c r="P75" s="28" t="n"/>
+      <c r="Q75" s="28" t="n">
+        <v>0.09394</v>
+      </c>
+      <c r="R75" s="26" t="n">
+        <v>93</v>
+      </c>
+      <c r="S75" s="29" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="T75" s="24" t="inlineStr">
+        <is>
+          <t>cs2-neutral-series-elo-v1</t>
+        </is>
+      </c>
+      <c r="U75" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V75" s="24" t="n"/>
+      <c r="W75" s="26" t="n"/>
+      <c r="X75" s="26" t="n"/>
+      <c r="Y75" s="38" t="n"/>
+      <c r="Z75" s="26" t="n"/>
+      <c r="AA75" s="28" t="n"/>
+      <c r="AB75" s="28" t="n"/>
+      <c r="AC75" s="40" t="n"/>
+      <c r="AD75" s="24" t="n"/>
+      <c r="AE75" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.5400 (aec-cs2-erx-jpu-2026-07-21).</t>
+        </is>
+      </c>
+      <c r="AF75" s="31" t="inlineStr">
+        <is>
+          <t>Research baseline; zero-unit shadow until qualified.</t>
+        </is>
+      </c>
+      <c r="AG75" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH75" s="24" t="n"/>
+      <c r="AI75" s="31" t="n"/>
+      <c r="AJ75" s="31" t="n"/>
+      <c r="AK75" s="24" t="inlineStr">
+        <is>
+          <t>model_qualified</t>
+        </is>
+      </c>
+      <c r="AL75" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM75" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED_SHADOW_CALL</t>
+        </is>
+      </c>
+      <c r="AN75" s="24" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="AO75" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED</t>
+        </is>
+      </c>
+      <c r="AP75" s="24" t="inlineStr">
+        <is>
+          <t>Just Players</t>
+        </is>
+      </c>
+      <c r="AQ75" s="24" t="inlineStr">
+        <is>
+          <t>Just Players</t>
+        </is>
+      </c>
+      <c r="AR75" s="24" t="inlineStr">
+        <is>
+          <t>Just Players</t>
+        </is>
+      </c>
+      <c r="AS75" s="24" t="inlineStr">
+        <is>
+          <t>ex-RUSTEC</t>
+        </is>
+      </c>
+      <c r="AT75" s="24" t="inlineStr">
+        <is>
+          <t>ex-RUSTEC</t>
+        </is>
+      </c>
+      <c r="AU75" s="24" t="inlineStr">
+        <is>
+          <t>ex-RUSTEC</t>
+        </is>
+      </c>
+      <c r="AV75" s="24" t="n"/>
+      <c r="AW75" s="24" t="n"/>
+      <c r="AX75" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY75" s="24" t="n"/>
+      <c r="AZ75" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA75" s="24" t="inlineStr">
+        <is>
+          <t>9dbde86ab8062ac73a51c94b0ad431573ac8b755ccd742d86794849a749958c7</t>
+        </is>
+      </c>
+      <c r="BB75" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC75" s="24" t="inlineStr">
+        <is>
+          <t>cs2-neutral-series-elo-v1</t>
+        </is>
+      </c>
+      <c r="BD75" s="24" t="inlineStr">
+        <is>
+          <t>9dbde86ab8062ac73a51c94b0ad431573ac8b755ccd742d86794849a749958c7</t>
+        </is>
+      </c>
+      <c r="BE75" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF75" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG75" s="24" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="BH75" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-21T08:13:57.416034Z</t>
+        </is>
+      </c>
+      <c r="BI75" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ75" s="38" t="n"/>
+      <c r="BK75" s="26" t="n">
+        <v>-117</v>
+      </c>
+      <c r="BL75" s="39" t="n">
+        <v>1.854701</v>
+      </c>
+      <c r="BM75" s="28" t="n">
+        <v>0.539171</v>
+      </c>
+      <c r="BN75" s="28" t="n"/>
+      <c r="BO75" s="28" t="n"/>
+      <c r="BP75" s="38" t="n"/>
+      <c r="BQ75" s="39" t="n"/>
+      <c r="BR75" s="28" t="n"/>
+      <c r="BS75" s="28" t="n"/>
+      <c r="BT75" s="28" t="n"/>
+      <c r="BU75" s="38" t="n"/>
+      <c r="BV75" s="29" t="n"/>
+      <c r="BW75" s="24" t="n"/>
+      <c r="BX75" s="40" t="n"/>
+      <c r="BY75" s="39" t="n"/>
+      <c r="BZ75" s="24" t="n"/>
+      <c r="CA75" s="31" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Normalize call_type labels: tag is metadata, edge is the gate
Main: 56 picks, all model_qualified (edge >= 0.02)
Flat: 153 picks, all research_observation
</commit_message>
<xml_diff>
--- a/data/picks.xlsx
+++ b/data/picks.xlsx
@@ -1374,7 +1374,7 @@
       <c r="AJ2" t="inlineStr"/>
       <c r="AK2" t="inlineStr">
         <is>
-          <t>research_observation</t>
+          <t>model_qualified</t>
         </is>
       </c>
       <c r="AL2" t="n">
@@ -1650,7 +1650,7 @@
       <c r="AJ3" t="inlineStr"/>
       <c r="AK3" t="inlineStr">
         <is>
-          <t>research_observation</t>
+          <t>model_qualified</t>
         </is>
       </c>
       <c r="AL3" t="n">
@@ -1926,7 +1926,7 @@
       <c r="AJ4" t="inlineStr"/>
       <c r="AK4" t="inlineStr">
         <is>
-          <t>research_observation</t>
+          <t>model_qualified</t>
         </is>
       </c>
       <c r="AL4" t="n">
@@ -2202,7 +2202,7 @@
       <c r="AJ5" t="inlineStr"/>
       <c r="AK5" t="inlineStr">
         <is>
-          <t>research_observation</t>
+          <t>model_qualified</t>
         </is>
       </c>
       <c r="AL5" t="n">
@@ -2478,7 +2478,7 @@
       <c r="AJ6" t="inlineStr"/>
       <c r="AK6" t="inlineStr">
         <is>
-          <t>research_observation</t>
+          <t>model_qualified</t>
         </is>
       </c>
       <c r="AL6" t="n">
@@ -2754,7 +2754,7 @@
       <c r="AJ7" t="inlineStr"/>
       <c r="AK7" t="inlineStr">
         <is>
-          <t>research_observation</t>
+          <t>model_qualified</t>
         </is>
       </c>
       <c r="AL7" t="n">
@@ -3030,7 +3030,7 @@
       <c r="AJ8" t="inlineStr"/>
       <c r="AK8" t="inlineStr">
         <is>
-          <t>research_observation</t>
+          <t>model_qualified</t>
         </is>
       </c>
       <c r="AL8" t="n">
@@ -3306,7 +3306,7 @@
       <c r="AJ9" t="inlineStr"/>
       <c r="AK9" t="inlineStr">
         <is>
-          <t>research_observation</t>
+          <t>model_qualified</t>
         </is>
       </c>
       <c r="AL9" t="n">
@@ -3582,7 +3582,7 @@
       <c r="AJ10" t="inlineStr"/>
       <c r="AK10" t="inlineStr">
         <is>
-          <t>research_observation</t>
+          <t>model_qualified</t>
         </is>
       </c>
       <c r="AL10" t="n">
@@ -3858,7 +3858,7 @@
       <c r="AJ11" t="inlineStr"/>
       <c r="AK11" t="inlineStr">
         <is>
-          <t>research_observation</t>
+          <t>model_qualified</t>
         </is>
       </c>
       <c r="AL11" t="n">
@@ -4134,7 +4134,7 @@
       <c r="AJ12" t="inlineStr"/>
       <c r="AK12" t="inlineStr">
         <is>
-          <t>research_observation</t>
+          <t>model_qualified</t>
         </is>
       </c>
       <c r="AL12" t="n">
@@ -4410,7 +4410,7 @@
       <c r="AJ13" t="inlineStr"/>
       <c r="AK13" t="inlineStr">
         <is>
-          <t>research_observation</t>
+          <t>model_qualified</t>
         </is>
       </c>
       <c r="AL13" t="n">
@@ -4686,7 +4686,7 @@
       <c r="AJ14" t="inlineStr"/>
       <c r="AK14" t="inlineStr">
         <is>
-          <t>research_observation</t>
+          <t>model_qualified</t>
         </is>
       </c>
       <c r="AL14" t="n">
@@ -4962,7 +4962,7 @@
       <c r="AJ15" t="inlineStr"/>
       <c r="AK15" t="inlineStr">
         <is>
-          <t>research_observation</t>
+          <t>model_qualified</t>
         </is>
       </c>
       <c r="AL15" t="n">
@@ -5238,7 +5238,7 @@
       <c r="AJ16" t="inlineStr"/>
       <c r="AK16" t="inlineStr">
         <is>
-          <t>research_observation</t>
+          <t>model_qualified</t>
         </is>
       </c>
       <c r="AL16" t="n">
@@ -5514,7 +5514,7 @@
       <c r="AJ17" t="inlineStr"/>
       <c r="AK17" t="inlineStr">
         <is>
-          <t>research_observation</t>
+          <t>model_qualified</t>
         </is>
       </c>
       <c r="AL17" t="n">
@@ -5790,7 +5790,7 @@
       <c r="AJ18" t="inlineStr"/>
       <c r="AK18" t="inlineStr">
         <is>
-          <t>research_observation</t>
+          <t>model_qualified</t>
         </is>
       </c>
       <c r="AL18" t="n">
@@ -6066,7 +6066,7 @@
       <c r="AJ19" t="inlineStr"/>
       <c r="AK19" t="inlineStr">
         <is>
-          <t>research_observation</t>
+          <t>model_qualified</t>
         </is>
       </c>
       <c r="AL19" t="n">
@@ -6342,7 +6342,7 @@
       <c r="AJ20" t="inlineStr"/>
       <c r="AK20" t="inlineStr">
         <is>
-          <t>research_observation</t>
+          <t>model_qualified</t>
         </is>
       </c>
       <c r="AL20" t="n">
@@ -6610,7 +6610,11 @@
       <c r="AH21" t="inlineStr"/>
       <c r="AI21" t="inlineStr"/>
       <c r="AJ21" t="inlineStr"/>
-      <c r="AK21" t="inlineStr"/>
+      <c r="AK21" t="inlineStr">
+        <is>
+          <t>model_qualified</t>
+        </is>
+      </c>
       <c r="AL21" t="n">
         <v>3</v>
       </c>
@@ -6844,7 +6848,11 @@
       <c r="AH22" t="inlineStr"/>
       <c r="AI22" t="inlineStr"/>
       <c r="AJ22" t="inlineStr"/>
-      <c r="AK22" t="inlineStr"/>
+      <c r="AK22" t="inlineStr">
+        <is>
+          <t>model_qualified</t>
+        </is>
+      </c>
       <c r="AL22" t="n">
         <v>3</v>
       </c>
@@ -7078,7 +7086,11 @@
       <c r="AH23" t="inlineStr"/>
       <c r="AI23" t="inlineStr"/>
       <c r="AJ23" t="inlineStr"/>
-      <c r="AK23" t="inlineStr"/>
+      <c r="AK23" t="inlineStr">
+        <is>
+          <t>model_qualified</t>
+        </is>
+      </c>
       <c r="AL23" t="n">
         <v>3</v>
       </c>
@@ -7312,7 +7324,11 @@
       <c r="AH24" t="inlineStr"/>
       <c r="AI24" t="inlineStr"/>
       <c r="AJ24" t="inlineStr"/>
-      <c r="AK24" t="inlineStr"/>
+      <c r="AK24" t="inlineStr">
+        <is>
+          <t>model_qualified</t>
+        </is>
+      </c>
       <c r="AL24" t="n">
         <v>3</v>
       </c>
@@ -7546,7 +7562,11 @@
       <c r="AH25" t="inlineStr"/>
       <c r="AI25" t="inlineStr"/>
       <c r="AJ25" t="inlineStr"/>
-      <c r="AK25" t="inlineStr"/>
+      <c r="AK25" t="inlineStr">
+        <is>
+          <t>model_qualified</t>
+        </is>
+      </c>
       <c r="AL25" t="n">
         <v>3</v>
       </c>
@@ -7780,7 +7800,11 @@
       <c r="AH26" t="inlineStr"/>
       <c r="AI26" t="inlineStr"/>
       <c r="AJ26" t="inlineStr"/>
-      <c r="AK26" t="inlineStr"/>
+      <c r="AK26" t="inlineStr">
+        <is>
+          <t>model_qualified</t>
+        </is>
+      </c>
       <c r="AL26" t="n">
         <v>3</v>
       </c>
@@ -8014,7 +8038,11 @@
       <c r="AH27" t="inlineStr"/>
       <c r="AI27" t="inlineStr"/>
       <c r="AJ27" t="inlineStr"/>
-      <c r="AK27" t="inlineStr"/>
+      <c r="AK27" t="inlineStr">
+        <is>
+          <t>model_qualified</t>
+        </is>
+      </c>
       <c r="AL27" t="n">
         <v>3</v>
       </c>
@@ -8248,7 +8276,11 @@
       <c r="AH28" t="inlineStr"/>
       <c r="AI28" t="inlineStr"/>
       <c r="AJ28" t="inlineStr"/>
-      <c r="AK28" t="inlineStr"/>
+      <c r="AK28" t="inlineStr">
+        <is>
+          <t>model_qualified</t>
+        </is>
+      </c>
       <c r="AL28" t="n">
         <v>3</v>
       </c>
@@ -8490,7 +8522,7 @@
       <c r="AJ29" t="inlineStr"/>
       <c r="AK29" t="inlineStr">
         <is>
-          <t>research_observation</t>
+          <t>model_qualified</t>
         </is>
       </c>
       <c r="AL29" t="n">
@@ -8766,7 +8798,7 @@
       <c r="AJ30" t="inlineStr"/>
       <c r="AK30" t="inlineStr">
         <is>
-          <t>research_observation</t>
+          <t>model_qualified</t>
         </is>
       </c>
       <c r="AL30" t="n">
@@ -9042,7 +9074,7 @@
       <c r="AJ31" t="inlineStr"/>
       <c r="AK31" t="inlineStr">
         <is>
-          <t>research_observation</t>
+          <t>model_qualified</t>
         </is>
       </c>
       <c r="AL31" t="n">
@@ -9318,7 +9350,7 @@
       <c r="AJ32" t="inlineStr"/>
       <c r="AK32" t="inlineStr">
         <is>
-          <t>research_observation</t>
+          <t>model_qualified</t>
         </is>
       </c>
       <c r="AL32" t="n">
@@ -9594,7 +9626,7 @@
       <c r="AJ33" t="inlineStr"/>
       <c r="AK33" t="inlineStr">
         <is>
-          <t>research_observation</t>
+          <t>model_qualified</t>
         </is>
       </c>
       <c r="AL33" t="n">
@@ -9870,7 +9902,7 @@
       <c r="AJ34" t="inlineStr"/>
       <c r="AK34" t="inlineStr">
         <is>
-          <t>research_observation</t>
+          <t>model_qualified</t>
         </is>
       </c>
       <c r="AL34" t="n">
@@ -10134,7 +10166,7 @@
       <c r="AJ35" t="inlineStr"/>
       <c r="AK35" t="inlineStr">
         <is>
-          <t>research_observation</t>
+          <t>model_qualified</t>
         </is>
       </c>
       <c r="AL35" t="n">
@@ -13998,7 +14030,7 @@
       <c r="AJ50" t="inlineStr"/>
       <c r="AK50" t="inlineStr">
         <is>
-          <t>research_observation</t>
+          <t>model_qualified</t>
         </is>
       </c>
       <c r="AL50" t="n">
@@ -14246,7 +14278,7 @@
       <c r="AJ51" t="inlineStr"/>
       <c r="AK51" t="inlineStr">
         <is>
-          <t>research_observation</t>
+          <t>model_qualified</t>
         </is>
       </c>
       <c r="AL51" t="n">
@@ -14494,7 +14526,7 @@
       <c r="AJ52" t="inlineStr"/>
       <c r="AK52" t="inlineStr">
         <is>
-          <t>research_observation</t>
+          <t>model_qualified</t>
         </is>
       </c>
       <c r="AL52" t="n">
@@ -14742,7 +14774,7 @@
       <c r="AJ53" t="inlineStr"/>
       <c r="AK53" t="inlineStr">
         <is>
-          <t>research_observation</t>
+          <t>model_qualified</t>
         </is>
       </c>
       <c r="AL53" t="n">
@@ -14990,7 +15022,7 @@
       <c r="AJ54" t="inlineStr"/>
       <c r="AK54" t="inlineStr">
         <is>
-          <t>research_observation</t>
+          <t>model_qualified</t>
         </is>
       </c>
       <c r="AL54" t="n">
@@ -15238,7 +15270,7 @@
       <c r="AJ55" t="inlineStr"/>
       <c r="AK55" t="inlineStr">
         <is>
-          <t>research_observation</t>
+          <t>model_qualified</t>
         </is>
       </c>
       <c r="AL55" t="n">
@@ -15486,7 +15518,7 @@
       <c r="AJ56" t="inlineStr"/>
       <c r="AK56" t="inlineStr">
         <is>
-          <t>research_observation</t>
+          <t>model_qualified</t>
         </is>
       </c>
       <c r="AL56" t="n">
@@ -15734,7 +15766,7 @@
       <c r="AJ57" t="inlineStr"/>
       <c r="AK57" t="inlineStr">
         <is>
-          <t>research_observation</t>
+          <t>model_qualified</t>
         </is>
       </c>
       <c r="AL57" t="n">

</xml_diff>

<commit_message>
fix: daily forecast script + esports logging + dashboard patches
- Add esports step to run_daily.sh (research ledger only)
- Add --log and --all flags to esports-forecast CLI command
- Fix run_daily.sh path in dashboard_server.py (scripts/run_daily.sh)
- Add research-performance API endpoint + Research Perf tab
- Reorganize dashboard tabs (Ledger|Flat|Research|Performance|...)
- P&L fix: fallback to research_pnl_units in _decorate_pick
- Unit sizing: _suggested_units fallback for all 3 ledgers
- Market pricing: use market_implied_probability in Research tab
- P&L computation: fallback from american_odds when research_pnl absent
- Add stop command for dashboard
- 322 tests pass, ruff clean
</commit_message>
<xml_diff>
--- a/data/picks.xlsx
+++ b/data/picks.xlsx
@@ -21,10 +21,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="0.0###"/>
-    <numFmt numFmtId="165" formatCode="0.000000"/>
-    <numFmt numFmtId="166" formatCode="0.0000"/>
-    <numFmt numFmtId="167" formatCode="0.0%"/>
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="0.0000"/>
+    <numFmt numFmtId="166" formatCode="0.0###"/>
+    <numFmt numFmtId="167" formatCode="0.000000"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -136,7 +136,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -150,10 +150,10 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -169,10 +169,10 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="167" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="10" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -184,10 +184,10 @@
     <xf numFmtId="0" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="167" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="10" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -202,13 +202,13 @@
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="10" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -217,11 +217,38 @@
     <xf numFmtId="2" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -797,11 +824,11 @@
         <f>COUNTIFS('Picks'!$BX$2:$BX$42,"&gt;0",'Picks'!$V$2:$V$42,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$42,"&gt;0",'Picks'!$V$2:$V$42,"loss")</f>
         <v/>
       </c>
-      <c r="E7" s="7">
+      <c r="E7" s="32">
         <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$42,"&gt;0",'Picks'!$V$2:$V$42,"win")/(COUNTIFS('Picks'!$BX$2:$BX$42,"&gt;0",'Picks'!$V$2:$V$42,"win")+COUNTIFS('Picks'!$BX$2:$BX$42,"&gt;0",'Picks'!$V$2:$V$42,"loss")),0)</f>
         <v/>
       </c>
-      <c r="G7" s="7">
+      <c r="G7" s="32">
         <f>IFERROR(SUM('Picks'!$BY$2:$BY$42)/SUM('Picks'!$BX$2:$BX$42),0)</f>
         <v/>
       </c>
@@ -829,7 +856,7 @@
       </c>
     </row>
     <row r="10" ht="28" customHeight="1">
-      <c r="A10" s="8">
+      <c r="A10" s="33">
         <f>SUM('Picks'!$BY$2:$BY$42)</f>
         <v/>
       </c>
@@ -841,7 +868,7 @@
         <f>COUNTIFS('Picks'!$AM$2:$AM$42,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$42,"settled")</f>
         <v/>
       </c>
-      <c r="G10" s="8">
+      <c r="G10" s="33">
         <f>SUMIFS('Picks'!$AC$2:$AC$42,'Picks'!$AM$2:$AM$42,"QUALIFIED_SHADOW_CALL")</f>
         <v/>
       </c>
@@ -908,11 +935,11 @@
         <f>COUNTIFS('Picks'!$H$2:$H$42,$A14,'Picks'!$U$2:$U$42,"settled",'Picks'!$V$2:$V$42,"loss")</f>
         <v/>
       </c>
-      <c r="E14" s="14">
+      <c r="E14" s="34">
         <f>IFERROR(C14/(C14+D14),0)</f>
         <v/>
       </c>
-      <c r="F14" s="15">
+      <c r="F14" s="35">
         <f>SUMIFS('Picks'!$BY$2:$BY$42,'Picks'!$H$2:$H$42,$A14)</f>
         <v/>
       </c>
@@ -939,11 +966,11 @@
         <f>COUNTIFS('Picks'!$H$2:$H$42,$A15,'Picks'!$U$2:$U$42,"settled",'Picks'!$V$2:$V$42,"loss")</f>
         <v/>
       </c>
-      <c r="E15" s="19">
+      <c r="E15" s="36">
         <f>IFERROR(C15/(C15+D15),0)</f>
         <v/>
       </c>
-      <c r="F15" s="20">
+      <c r="F15" s="37">
         <f>SUMIFS('Picks'!$BY$2:$BY$42,'Picks'!$H$2:$H$42,$A15)</f>
         <v/>
       </c>
@@ -970,11 +997,11 @@
         <f>COUNTIFS('Picks'!$H$2:$H$42,$A16,'Picks'!$U$2:$U$42,"settled",'Picks'!$V$2:$V$42,"loss")</f>
         <v/>
       </c>
-      <c r="E16" s="14">
+      <c r="E16" s="34">
         <f>IFERROR(C16/(C16+D16),0)</f>
         <v/>
       </c>
-      <c r="F16" s="15">
+      <c r="F16" s="35">
         <f>SUMIFS('Picks'!$BY$2:$BY$42,'Picks'!$H$2:$H$42,$A16)</f>
         <v/>
       </c>
@@ -1008,7 +1035,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:CM42"/>
+  <dimension ref="A1:CM40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1607,7 +1634,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J2" s="25" t="n"/>
+      <c r="J2" s="38" t="n"/>
       <c r="K2" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -1616,7 +1643,7 @@
       <c r="L2" s="26" t="n">
         <v>-141</v>
       </c>
-      <c r="M2" s="27" t="n">
+      <c r="M2" s="39" t="n">
         <v>1.70922</v>
       </c>
       <c r="N2" s="28" t="n">
@@ -1658,7 +1685,7 @@
       <c r="X2" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="Y2" s="25" t="n"/>
+      <c r="Y2" s="38" t="n"/>
       <c r="Z2" s="26" t="n">
         <v>-110</v>
       </c>
@@ -1666,7 +1693,7 @@
         <v>0.523834</v>
       </c>
       <c r="AB2" s="28" t="n"/>
-      <c r="AC2" s="30" t="n">
+      <c r="AC2" s="40" t="n">
         <v>1.4184</v>
       </c>
       <c r="AD2" s="24" t="inlineStr">
@@ -1755,11 +1782,11 @@
         </is>
       </c>
       <c r="BI2" s="24" t="n"/>
-      <c r="BJ2" s="25" t="n"/>
+      <c r="BJ2" s="38" t="n"/>
       <c r="BK2" s="26" t="n">
         <v>-141</v>
       </c>
-      <c r="BL2" s="27" t="n">
+      <c r="BL2" s="39" t="n">
         <v>1.70922</v>
       </c>
       <c r="BM2" s="28" t="n">
@@ -1771,20 +1798,20 @@
       <c r="BO2" s="28" t="n">
         <v>0.523834</v>
       </c>
-      <c r="BP2" s="25" t="n"/>
-      <c r="BQ2" s="27" t="n">
+      <c r="BP2" s="38" t="n"/>
+      <c r="BQ2" s="39" t="n">
         <v>1.909</v>
       </c>
       <c r="BR2" s="28" t="n"/>
       <c r="BS2" s="28" t="n"/>
       <c r="BT2" s="28" t="n"/>
-      <c r="BU2" s="25" t="n"/>
+      <c r="BU2" s="38" t="n"/>
       <c r="BV2" s="29" t="n">
         <v>2</v>
       </c>
       <c r="BW2" s="24" t="n"/>
-      <c r="BX2" s="30" t="n"/>
-      <c r="BY2" s="27" t="n"/>
+      <c r="BX2" s="40" t="n"/>
+      <c r="BY2" s="39" t="n"/>
       <c r="BZ2" s="24" t="n"/>
       <c r="CA2" s="31" t="n"/>
       <c r="CB2" s="24" t="n"/>
@@ -1866,7 +1893,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J3" s="25" t="n"/>
+      <c r="J3" s="38" t="n"/>
       <c r="K3" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -1875,7 +1902,7 @@
       <c r="L3" s="26" t="n">
         <v>-141</v>
       </c>
-      <c r="M3" s="27" t="n">
+      <c r="M3" s="39" t="n">
         <v>1.70922</v>
       </c>
       <c r="N3" s="28" t="n">
@@ -1917,7 +1944,7 @@
       <c r="X3" s="26" t="n">
         <v>6</v>
       </c>
-      <c r="Y3" s="25" t="n"/>
+      <c r="Y3" s="38" t="n"/>
       <c r="Z3" s="26" t="n">
         <v>-110</v>
       </c>
@@ -1925,7 +1952,7 @@
         <v>0.523834</v>
       </c>
       <c r="AB3" s="28" t="n"/>
-      <c r="AC3" s="30" t="n">
+      <c r="AC3" s="40" t="n">
         <v>1.0638</v>
       </c>
       <c r="AD3" s="24" t="inlineStr">
@@ -2014,11 +2041,11 @@
         </is>
       </c>
       <c r="BI3" s="24" t="n"/>
-      <c r="BJ3" s="25" t="n"/>
+      <c r="BJ3" s="38" t="n"/>
       <c r="BK3" s="26" t="n">
         <v>-141</v>
       </c>
-      <c r="BL3" s="27" t="n">
+      <c r="BL3" s="39" t="n">
         <v>1.70922</v>
       </c>
       <c r="BM3" s="28" t="n">
@@ -2030,20 +2057,20 @@
       <c r="BO3" s="28" t="n">
         <v>0.523834</v>
       </c>
-      <c r="BP3" s="25" t="n"/>
-      <c r="BQ3" s="27" t="n">
+      <c r="BP3" s="38" t="n"/>
+      <c r="BQ3" s="39" t="n">
         <v>1.909</v>
       </c>
       <c r="BR3" s="28" t="n"/>
       <c r="BS3" s="28" t="n"/>
       <c r="BT3" s="28" t="n"/>
-      <c r="BU3" s="25" t="n"/>
+      <c r="BU3" s="38" t="n"/>
       <c r="BV3" s="29" t="n">
         <v>1.59</v>
       </c>
       <c r="BW3" s="24" t="n"/>
-      <c r="BX3" s="30" t="n"/>
-      <c r="BY3" s="27" t="n"/>
+      <c r="BX3" s="40" t="n"/>
+      <c r="BY3" s="39" t="n"/>
       <c r="BZ3" s="24" t="n"/>
       <c r="CA3" s="31" t="n"/>
       <c r="CB3" s="24" t="n"/>
@@ -2125,7 +2152,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J4" s="25" t="n"/>
+      <c r="J4" s="38" t="n"/>
       <c r="K4" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -2134,7 +2161,7 @@
       <c r="L4" s="26" t="n">
         <v>-174</v>
       </c>
-      <c r="M4" s="27" t="n">
+      <c r="M4" s="39" t="n">
         <v>1.574713</v>
       </c>
       <c r="N4" s="28" t="n">
@@ -2176,7 +2203,7 @@
       <c r="X4" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="Y4" s="25" t="n"/>
+      <c r="Y4" s="38" t="n"/>
       <c r="Z4" s="26" t="n">
         <v>-110</v>
       </c>
@@ -2184,7 +2211,7 @@
         <v>0.523834</v>
       </c>
       <c r="AB4" s="28" t="n"/>
-      <c r="AC4" s="30" t="n">
+      <c r="AC4" s="40" t="n">
         <v>0.8621</v>
       </c>
       <c r="AD4" s="24" t="inlineStr">
@@ -2273,11 +2300,11 @@
         </is>
       </c>
       <c r="BI4" s="24" t="n"/>
-      <c r="BJ4" s="25" t="n"/>
+      <c r="BJ4" s="38" t="n"/>
       <c r="BK4" s="26" t="n">
         <v>-174</v>
       </c>
-      <c r="BL4" s="27" t="n">
+      <c r="BL4" s="39" t="n">
         <v>1.574713</v>
       </c>
       <c r="BM4" s="28" t="n">
@@ -2289,20 +2316,20 @@
       <c r="BO4" s="28" t="n">
         <v>0.523834</v>
       </c>
-      <c r="BP4" s="25" t="n"/>
-      <c r="BQ4" s="27" t="n">
+      <c r="BP4" s="38" t="n"/>
+      <c r="BQ4" s="39" t="n">
         <v>1.909</v>
       </c>
       <c r="BR4" s="28" t="n"/>
       <c r="BS4" s="28" t="n"/>
       <c r="BT4" s="28" t="n"/>
-      <c r="BU4" s="25" t="n"/>
+      <c r="BU4" s="38" t="n"/>
       <c r="BV4" s="29" t="n">
         <v>1.58</v>
       </c>
       <c r="BW4" s="24" t="n"/>
-      <c r="BX4" s="30" t="n"/>
-      <c r="BY4" s="27" t="n"/>
+      <c r="BX4" s="40" t="n"/>
+      <c r="BY4" s="39" t="n"/>
       <c r="BZ4" s="24" t="n"/>
       <c r="CA4" s="31" t="n"/>
       <c r="CB4" s="24" t="n"/>
@@ -2384,7 +2411,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J5" s="25" t="n"/>
+      <c r="J5" s="38" t="n"/>
       <c r="K5" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -2393,7 +2420,7 @@
       <c r="L5" s="26" t="n">
         <v>-141</v>
       </c>
-      <c r="M5" s="27" t="n">
+      <c r="M5" s="39" t="n">
         <v>1.70922</v>
       </c>
       <c r="N5" s="28" t="n">
@@ -2435,11 +2462,11 @@
       <c r="X5" s="26" t="n">
         <v>6</v>
       </c>
-      <c r="Y5" s="25" t="n"/>
+      <c r="Y5" s="38" t="n"/>
       <c r="Z5" s="26" t="n"/>
       <c r="AA5" s="28" t="n"/>
       <c r="AB5" s="28" t="n"/>
-      <c r="AC5" s="30" t="n">
+      <c r="AC5" s="40" t="n">
         <v>1.0638</v>
       </c>
       <c r="AD5" s="24" t="inlineStr">
@@ -2532,11 +2559,11 @@
         </is>
       </c>
       <c r="BI5" s="24" t="n"/>
-      <c r="BJ5" s="25" t="n"/>
+      <c r="BJ5" s="38" t="n"/>
       <c r="BK5" s="26" t="n">
         <v>-141</v>
       </c>
-      <c r="BL5" s="27" t="n">
+      <c r="BL5" s="39" t="n">
         <v>1.70922</v>
       </c>
       <c r="BM5" s="28" t="n">
@@ -2548,18 +2575,18 @@
       <c r="BO5" s="28" t="n">
         <v>0.523834</v>
       </c>
-      <c r="BP5" s="25" t="n"/>
-      <c r="BQ5" s="27" t="n"/>
+      <c r="BP5" s="38" t="n"/>
+      <c r="BQ5" s="39" t="n"/>
       <c r="BR5" s="28" t="n"/>
       <c r="BS5" s="28" t="n"/>
       <c r="BT5" s="28" t="n"/>
-      <c r="BU5" s="25" t="n"/>
+      <c r="BU5" s="38" t="n"/>
       <c r="BV5" s="29" t="n">
         <v>1.58</v>
       </c>
       <c r="BW5" s="24" t="n"/>
-      <c r="BX5" s="30" t="n"/>
-      <c r="BY5" s="27" t="n"/>
+      <c r="BX5" s="40" t="n"/>
+      <c r="BY5" s="39" t="n"/>
       <c r="BZ5" s="24" t="n"/>
       <c r="CA5" s="31" t="n"/>
       <c r="CB5" s="24" t="n"/>
@@ -2641,7 +2668,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J6" s="25" t="n"/>
+      <c r="J6" s="38" t="n"/>
       <c r="K6" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -2650,7 +2677,7 @@
       <c r="L6" s="26" t="n">
         <v>-163</v>
       </c>
-      <c r="M6" s="27" t="n">
+      <c r="M6" s="39" t="n">
         <v>1.613497</v>
       </c>
       <c r="N6" s="28" t="n">
@@ -2692,11 +2719,11 @@
       <c r="X6" s="26" t="n">
         <v>6</v>
       </c>
-      <c r="Y6" s="25" t="n"/>
+      <c r="Y6" s="38" t="n"/>
       <c r="Z6" s="26" t="n"/>
       <c r="AA6" s="28" t="n"/>
       <c r="AB6" s="28" t="n"/>
-      <c r="AC6" s="30" t="n">
+      <c r="AC6" s="40" t="n">
         <v>1.0736</v>
       </c>
       <c r="AD6" s="24" t="inlineStr">
@@ -2789,11 +2816,11 @@
         </is>
       </c>
       <c r="BI6" s="24" t="n"/>
-      <c r="BJ6" s="25" t="n"/>
+      <c r="BJ6" s="38" t="n"/>
       <c r="BK6" s="26" t="n">
         <v>-163</v>
       </c>
-      <c r="BL6" s="27" t="n">
+      <c r="BL6" s="39" t="n">
         <v>1.613497</v>
       </c>
       <c r="BM6" s="28" t="n">
@@ -2805,18 +2832,18 @@
       <c r="BO6" s="28" t="n">
         <v>0.523834</v>
       </c>
-      <c r="BP6" s="25" t="n"/>
-      <c r="BQ6" s="27" t="n"/>
+      <c r="BP6" s="38" t="n"/>
+      <c r="BQ6" s="39" t="n"/>
       <c r="BR6" s="28" t="n"/>
       <c r="BS6" s="28" t="n"/>
       <c r="BT6" s="28" t="n"/>
-      <c r="BU6" s="25" t="n"/>
+      <c r="BU6" s="38" t="n"/>
       <c r="BV6" s="29" t="n">
         <v>1.83</v>
       </c>
       <c r="BW6" s="24" t="n"/>
-      <c r="BX6" s="30" t="n"/>
-      <c r="BY6" s="27" t="n"/>
+      <c r="BX6" s="40" t="n"/>
+      <c r="BY6" s="39" t="n"/>
       <c r="BZ6" s="24" t="n"/>
       <c r="CA6" s="31" t="n"/>
       <c r="CB6" s="24" t="n"/>
@@ -2898,7 +2925,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J7" s="25" t="n"/>
+      <c r="J7" s="38" t="n"/>
       <c r="K7" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -2907,7 +2934,7 @@
       <c r="L7" s="26" t="n">
         <v>-133</v>
       </c>
-      <c r="M7" s="27" t="n">
+      <c r="M7" s="39" t="n">
         <v>1.75188</v>
       </c>
       <c r="N7" s="28" t="n">
@@ -2949,7 +2976,7 @@
       <c r="X7" s="26" t="n">
         <v>8</v>
       </c>
-      <c r="Y7" s="25" t="n"/>
+      <c r="Y7" s="38" t="n"/>
       <c r="Z7" s="26" t="n">
         <v>-110</v>
       </c>
@@ -2957,7 +2984,7 @@
         <v>0.523834</v>
       </c>
       <c r="AB7" s="28" t="n"/>
-      <c r="AC7" s="30" t="n">
+      <c r="AC7" s="40" t="n">
         <v>1.5038</v>
       </c>
       <c r="AD7" s="24" t="inlineStr">
@@ -3046,11 +3073,11 @@
         </is>
       </c>
       <c r="BI7" s="24" t="n"/>
-      <c r="BJ7" s="25" t="n"/>
+      <c r="BJ7" s="38" t="n"/>
       <c r="BK7" s="26" t="n">
         <v>-133</v>
       </c>
-      <c r="BL7" s="27" t="n">
+      <c r="BL7" s="39" t="n">
         <v>1.75188</v>
       </c>
       <c r="BM7" s="28" t="n">
@@ -3062,20 +3089,20 @@
       <c r="BO7" s="28" t="n">
         <v>0.523834</v>
       </c>
-      <c r="BP7" s="25" t="n"/>
-      <c r="BQ7" s="27" t="n">
+      <c r="BP7" s="38" t="n"/>
+      <c r="BQ7" s="39" t="n">
         <v>1.909</v>
       </c>
       <c r="BR7" s="28" t="n"/>
       <c r="BS7" s="28" t="n"/>
       <c r="BT7" s="28" t="n"/>
-      <c r="BU7" s="25" t="n"/>
+      <c r="BU7" s="38" t="n"/>
       <c r="BV7" s="29" t="n">
         <v>2</v>
       </c>
       <c r="BW7" s="24" t="n"/>
-      <c r="BX7" s="30" t="n"/>
-      <c r="BY7" s="27" t="n"/>
+      <c r="BX7" s="40" t="n"/>
+      <c r="BY7" s="39" t="n"/>
       <c r="BZ7" s="24" t="n"/>
       <c r="CA7" s="31" t="n"/>
       <c r="CB7" s="24" t="n"/>
@@ -3157,7 +3184,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J8" s="25" t="n"/>
+      <c r="J8" s="38" t="n"/>
       <c r="K8" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -3166,7 +3193,7 @@
       <c r="L8" s="26" t="n">
         <v>-150</v>
       </c>
-      <c r="M8" s="27" t="n">
+      <c r="M8" s="39" t="n">
         <v>1.666667</v>
       </c>
       <c r="N8" s="28" t="n">
@@ -3208,7 +3235,7 @@
       <c r="X8" s="26" t="n">
         <v>6</v>
       </c>
-      <c r="Y8" s="25" t="n"/>
+      <c r="Y8" s="38" t="n"/>
       <c r="Z8" s="26" t="n">
         <v>-110</v>
       </c>
@@ -3216,7 +3243,7 @@
         <v>0.523834</v>
       </c>
       <c r="AB8" s="28" t="n"/>
-      <c r="AC8" s="30" t="n">
+      <c r="AC8" s="40" t="n">
         <v>1.3333</v>
       </c>
       <c r="AD8" s="24" t="inlineStr">
@@ -3305,11 +3332,11 @@
         </is>
       </c>
       <c r="BI8" s="24" t="n"/>
-      <c r="BJ8" s="25" t="n"/>
+      <c r="BJ8" s="38" t="n"/>
       <c r="BK8" s="26" t="n">
         <v>-150</v>
       </c>
-      <c r="BL8" s="27" t="n">
+      <c r="BL8" s="39" t="n">
         <v>1.666667</v>
       </c>
       <c r="BM8" s="28" t="n">
@@ -3321,20 +3348,20 @@
       <c r="BO8" s="28" t="n">
         <v>0.523834</v>
       </c>
-      <c r="BP8" s="25" t="n"/>
-      <c r="BQ8" s="27" t="n">
+      <c r="BP8" s="38" t="n"/>
+      <c r="BQ8" s="39" t="n">
         <v>1.909</v>
       </c>
       <c r="BR8" s="28" t="n"/>
       <c r="BS8" s="28" t="n"/>
       <c r="BT8" s="28" t="n"/>
-      <c r="BU8" s="25" t="n"/>
+      <c r="BU8" s="38" t="n"/>
       <c r="BV8" s="29" t="n">
         <v>1.88</v>
       </c>
       <c r="BW8" s="24" t="n"/>
-      <c r="BX8" s="30" t="n"/>
-      <c r="BY8" s="27" t="n"/>
+      <c r="BX8" s="40" t="n"/>
+      <c r="BY8" s="39" t="n"/>
       <c r="BZ8" s="24" t="n"/>
       <c r="CA8" s="31" t="n"/>
       <c r="CB8" s="24" t="n"/>
@@ -3416,7 +3443,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J9" s="25" t="n"/>
+      <c r="J9" s="38" t="n"/>
       <c r="K9" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -3425,7 +3452,7 @@
       <c r="L9" s="26" t="n">
         <v>-120</v>
       </c>
-      <c r="M9" s="27" t="n">
+      <c r="M9" s="39" t="n">
         <v>1.833333</v>
       </c>
       <c r="N9" s="28" t="n">
@@ -3467,7 +3494,7 @@
       <c r="X9" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="Y9" s="25" t="n"/>
+      <c r="Y9" s="38" t="n"/>
       <c r="Z9" s="26" t="n">
         <v>-110</v>
       </c>
@@ -3475,7 +3502,7 @@
         <v>0.523834</v>
       </c>
       <c r="AB9" s="28" t="n"/>
-      <c r="AC9" s="30" t="n">
+      <c r="AC9" s="40" t="n">
         <v>1.6667</v>
       </c>
       <c r="AD9" s="24" t="inlineStr">
@@ -3564,11 +3591,11 @@
         </is>
       </c>
       <c r="BI9" s="24" t="n"/>
-      <c r="BJ9" s="25" t="n"/>
+      <c r="BJ9" s="38" t="n"/>
       <c r="BK9" s="26" t="n">
         <v>-120</v>
       </c>
-      <c r="BL9" s="27" t="n">
+      <c r="BL9" s="39" t="n">
         <v>1.833333</v>
       </c>
       <c r="BM9" s="28" t="n">
@@ -3580,20 +3607,20 @@
       <c r="BO9" s="28" t="n">
         <v>0.523834</v>
       </c>
-      <c r="BP9" s="25" t="n"/>
-      <c r="BQ9" s="27" t="n">
+      <c r="BP9" s="38" t="n"/>
+      <c r="BQ9" s="39" t="n">
         <v>1.909</v>
       </c>
       <c r="BR9" s="28" t="n"/>
       <c r="BS9" s="28" t="n"/>
       <c r="BT9" s="28" t="n"/>
-      <c r="BU9" s="25" t="n"/>
+      <c r="BU9" s="38" t="n"/>
       <c r="BV9" s="29" t="n">
         <v>2</v>
       </c>
       <c r="BW9" s="24" t="n"/>
-      <c r="BX9" s="30" t="n"/>
-      <c r="BY9" s="27" t="n"/>
+      <c r="BX9" s="40" t="n"/>
+      <c r="BY9" s="39" t="n"/>
       <c r="BZ9" s="24" t="n"/>
       <c r="CA9" s="31" t="n"/>
       <c r="CB9" s="24" t="n"/>
@@ -3675,7 +3702,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J10" s="25" t="n"/>
+      <c r="J10" s="38" t="n"/>
       <c r="K10" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -3684,7 +3711,7 @@
       <c r="L10" s="26" t="n">
         <v>-153</v>
       </c>
-      <c r="M10" s="27" t="n">
+      <c r="M10" s="39" t="n">
         <v>1.653595</v>
       </c>
       <c r="N10" s="28" t="n">
@@ -3726,7 +3753,7 @@
       <c r="X10" s="26" t="n">
         <v>10</v>
       </c>
-      <c r="Y10" s="25" t="n"/>
+      <c r="Y10" s="38" t="n"/>
       <c r="Z10" s="26" t="n">
         <v>-110</v>
       </c>
@@ -3734,7 +3761,7 @@
         <v>0.523834</v>
       </c>
       <c r="AB10" s="28" t="n"/>
-      <c r="AC10" s="30" t="n">
+      <c r="AC10" s="40" t="n">
         <v>0.9804</v>
       </c>
       <c r="AD10" s="24" t="inlineStr">
@@ -3823,11 +3850,11 @@
         </is>
       </c>
       <c r="BI10" s="24" t="n"/>
-      <c r="BJ10" s="25" t="n"/>
+      <c r="BJ10" s="38" t="n"/>
       <c r="BK10" s="26" t="n">
         <v>-153</v>
       </c>
-      <c r="BL10" s="27" t="n">
+      <c r="BL10" s="39" t="n">
         <v>1.653595</v>
       </c>
       <c r="BM10" s="28" t="n">
@@ -3839,20 +3866,20 @@
       <c r="BO10" s="28" t="n">
         <v>0.523834</v>
       </c>
-      <c r="BP10" s="25" t="n"/>
-      <c r="BQ10" s="27" t="n">
+      <c r="BP10" s="38" t="n"/>
+      <c r="BQ10" s="39" t="n">
         <v>1.909</v>
       </c>
       <c r="BR10" s="28" t="n"/>
       <c r="BS10" s="28" t="n"/>
       <c r="BT10" s="28" t="n"/>
-      <c r="BU10" s="25" t="n"/>
+      <c r="BU10" s="38" t="n"/>
       <c r="BV10" s="29" t="n">
         <v>1.55</v>
       </c>
       <c r="BW10" s="24" t="n"/>
-      <c r="BX10" s="30" t="n"/>
-      <c r="BY10" s="27" t="n"/>
+      <c r="BX10" s="40" t="n"/>
+      <c r="BY10" s="39" t="n"/>
       <c r="BZ10" s="24" t="n"/>
       <c r="CA10" s="31" t="n"/>
       <c r="CB10" s="24" t="n"/>
@@ -3934,7 +3961,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J11" s="25" t="n"/>
+      <c r="J11" s="38" t="n"/>
       <c r="K11" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -3943,7 +3970,7 @@
       <c r="L11" s="26" t="n">
         <v>-182</v>
       </c>
-      <c r="M11" s="27" t="n">
+      <c r="M11" s="39" t="n">
         <v>1.549451</v>
       </c>
       <c r="N11" s="28" t="n">
@@ -3985,7 +4012,7 @@
       <c r="X11" s="26" t="n">
         <v>6</v>
       </c>
-      <c r="Y11" s="25" t="n"/>
+      <c r="Y11" s="38" t="n"/>
       <c r="Z11" s="26" t="n">
         <v>-110</v>
       </c>
@@ -3993,7 +4020,7 @@
         <v>0.523834</v>
       </c>
       <c r="AB11" s="28" t="n"/>
-      <c r="AC11" s="30" t="n">
+      <c r="AC11" s="40" t="n">
         <v>1.0989</v>
       </c>
       <c r="AD11" s="24" t="inlineStr">
@@ -4082,11 +4109,11 @@
         </is>
       </c>
       <c r="BI11" s="24" t="n"/>
-      <c r="BJ11" s="25" t="n"/>
+      <c r="BJ11" s="38" t="n"/>
       <c r="BK11" s="26" t="n">
         <v>-182</v>
       </c>
-      <c r="BL11" s="27" t="n">
+      <c r="BL11" s="39" t="n">
         <v>1.549451</v>
       </c>
       <c r="BM11" s="28" t="n">
@@ -4098,20 +4125,20 @@
       <c r="BO11" s="28" t="n">
         <v>0.523834</v>
       </c>
-      <c r="BP11" s="25" t="n"/>
-      <c r="BQ11" s="27" t="n">
+      <c r="BP11" s="38" t="n"/>
+      <c r="BQ11" s="39" t="n">
         <v>1.909</v>
       </c>
       <c r="BR11" s="28" t="n"/>
       <c r="BS11" s="28" t="n"/>
       <c r="BT11" s="28" t="n"/>
-      <c r="BU11" s="25" t="n"/>
+      <c r="BU11" s="38" t="n"/>
       <c r="BV11" s="29" t="n">
         <v>1.74</v>
       </c>
       <c r="BW11" s="24" t="n"/>
-      <c r="BX11" s="30" t="n"/>
-      <c r="BY11" s="27" t="n"/>
+      <c r="BX11" s="40" t="n"/>
+      <c r="BY11" s="39" t="n"/>
       <c r="BZ11" s="24" t="n"/>
       <c r="CA11" s="31" t="n"/>
       <c r="CB11" s="24" t="n"/>
@@ -4193,7 +4220,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J12" s="25" t="n"/>
+      <c r="J12" s="38" t="n"/>
       <c r="K12" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -4202,7 +4229,7 @@
       <c r="L12" s="26" t="n">
         <v>-108</v>
       </c>
-      <c r="M12" s="27" t="n">
+      <c r="M12" s="39" t="n">
         <v>1.925926</v>
       </c>
       <c r="N12" s="28" t="n">
@@ -4244,7 +4271,7 @@
       <c r="X12" s="26" t="n">
         <v>8</v>
       </c>
-      <c r="Y12" s="25" t="n"/>
+      <c r="Y12" s="38" t="n"/>
       <c r="Z12" s="26" t="n">
         <v>-110</v>
       </c>
@@ -4252,7 +4279,7 @@
         <v>0.523834</v>
       </c>
       <c r="AB12" s="28" t="n"/>
-      <c r="AC12" s="30" t="n">
+      <c r="AC12" s="40" t="n">
         <v>1.6204</v>
       </c>
       <c r="AD12" s="24" t="inlineStr">
@@ -4341,11 +4368,11 @@
         </is>
       </c>
       <c r="BI12" s="24" t="n"/>
-      <c r="BJ12" s="25" t="n"/>
+      <c r="BJ12" s="38" t="n"/>
       <c r="BK12" s="26" t="n">
         <v>-108</v>
       </c>
-      <c r="BL12" s="27" t="n">
+      <c r="BL12" s="39" t="n">
         <v>1.925926</v>
       </c>
       <c r="BM12" s="28" t="n">
@@ -4357,20 +4384,20 @@
       <c r="BO12" s="28" t="n">
         <v>0.523834</v>
       </c>
-      <c r="BP12" s="25" t="n"/>
-      <c r="BQ12" s="27" t="n">
+      <c r="BP12" s="38" t="n"/>
+      <c r="BQ12" s="39" t="n">
         <v>1.909</v>
       </c>
       <c r="BR12" s="28" t="n"/>
       <c r="BS12" s="28" t="n"/>
       <c r="BT12" s="28" t="n"/>
-      <c r="BU12" s="25" t="n"/>
+      <c r="BU12" s="38" t="n"/>
       <c r="BV12" s="29" t="n">
         <v>1.18</v>
       </c>
       <c r="BW12" s="24" t="n"/>
-      <c r="BX12" s="30" t="n"/>
-      <c r="BY12" s="27" t="n"/>
+      <c r="BX12" s="40" t="n"/>
+      <c r="BY12" s="39" t="n"/>
       <c r="BZ12" s="24" t="n"/>
       <c r="CA12" s="31" t="n"/>
       <c r="CB12" s="24" t="n"/>
@@ -4452,7 +4479,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J13" s="25" t="n"/>
+      <c r="J13" s="38" t="n"/>
       <c r="K13" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -4461,7 +4488,7 @@
       <c r="L13" s="26" t="n">
         <v>-203</v>
       </c>
-      <c r="M13" s="27" t="n">
+      <c r="M13" s="39" t="n">
         <v>1.492611</v>
       </c>
       <c r="N13" s="28" t="n">
@@ -4503,7 +4530,7 @@
       <c r="X13" s="26" t="n">
         <v>8</v>
       </c>
-      <c r="Y13" s="25" t="n"/>
+      <c r="Y13" s="38" t="n"/>
       <c r="Z13" s="26" t="n">
         <v>-110</v>
       </c>
@@ -4511,7 +4538,7 @@
         <v>0.523834</v>
       </c>
       <c r="AB13" s="28" t="n"/>
-      <c r="AC13" s="30" t="n">
+      <c r="AC13" s="40" t="n">
         <v>0.9852</v>
       </c>
       <c r="AD13" s="24" t="inlineStr">
@@ -4600,11 +4627,11 @@
         </is>
       </c>
       <c r="BI13" s="24" t="n"/>
-      <c r="BJ13" s="25" t="n"/>
+      <c r="BJ13" s="38" t="n"/>
       <c r="BK13" s="26" t="n">
         <v>-203</v>
       </c>
-      <c r="BL13" s="27" t="n">
+      <c r="BL13" s="39" t="n">
         <v>1.492611</v>
       </c>
       <c r="BM13" s="28" t="n">
@@ -4616,20 +4643,20 @@
       <c r="BO13" s="28" t="n">
         <v>0.523834</v>
       </c>
-      <c r="BP13" s="25" t="n"/>
-      <c r="BQ13" s="27" t="n">
+      <c r="BP13" s="38" t="n"/>
+      <c r="BQ13" s="39" t="n">
         <v>1.909</v>
       </c>
       <c r="BR13" s="28" t="n"/>
       <c r="BS13" s="28" t="n"/>
       <c r="BT13" s="28" t="n"/>
-      <c r="BU13" s="25" t="n"/>
+      <c r="BU13" s="38" t="n"/>
       <c r="BV13" s="29" t="n">
         <v>2</v>
       </c>
       <c r="BW13" s="24" t="n"/>
-      <c r="BX13" s="30" t="n"/>
-      <c r="BY13" s="27" t="n"/>
+      <c r="BX13" s="40" t="n"/>
+      <c r="BY13" s="39" t="n"/>
       <c r="BZ13" s="24" t="n"/>
       <c r="CA13" s="31" t="n"/>
       <c r="CB13" s="24" t="n"/>
@@ -4711,7 +4738,7 @@
           <t>away</t>
         </is>
       </c>
-      <c r="J14" s="25" t="n"/>
+      <c r="J14" s="38" t="n"/>
       <c r="K14" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -4720,7 +4747,7 @@
       <c r="L14" s="26" t="n">
         <v>122</v>
       </c>
-      <c r="M14" s="27" t="n">
+      <c r="M14" s="39" t="n">
         <v>2.22</v>
       </c>
       <c r="N14" s="28" t="n">
@@ -4762,7 +4789,7 @@
       <c r="X14" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="Y14" s="25" t="n"/>
+      <c r="Y14" s="38" t="n"/>
       <c r="Z14" s="26" t="n">
         <v>-110</v>
       </c>
@@ -4770,7 +4797,7 @@
         <v>0.523834</v>
       </c>
       <c r="AB14" s="28" t="n"/>
-      <c r="AC14" s="30" t="n">
+      <c r="AC14" s="40" t="n">
         <v>0</v>
       </c>
       <c r="AD14" s="24" t="inlineStr">
@@ -4863,11 +4890,11 @@
         </is>
       </c>
       <c r="BI14" s="24" t="n"/>
-      <c r="BJ14" s="25" t="n"/>
+      <c r="BJ14" s="38" t="n"/>
       <c r="BK14" s="26" t="n">
         <v>122</v>
       </c>
-      <c r="BL14" s="27" t="n">
+      <c r="BL14" s="39" t="n">
         <v>2.22</v>
       </c>
       <c r="BM14" s="28" t="n">
@@ -4879,14 +4906,14 @@
       <c r="BO14" s="28" t="n">
         <v>0.523834</v>
       </c>
-      <c r="BP14" s="25" t="n"/>
-      <c r="BQ14" s="27" t="n">
+      <c r="BP14" s="38" t="n"/>
+      <c r="BQ14" s="39" t="n">
         <v>1.909</v>
       </c>
       <c r="BR14" s="28" t="n"/>
       <c r="BS14" s="28" t="n"/>
       <c r="BT14" s="28" t="n"/>
-      <c r="BU14" s="25" t="n"/>
+      <c r="BU14" s="38" t="n"/>
       <c r="BV14" s="29" t="n">
         <v>1.04</v>
       </c>
@@ -4895,8 +4922,8 @@
           <t>postponed</t>
         </is>
       </c>
-      <c r="BX14" s="30" t="n"/>
-      <c r="BY14" s="27" t="n"/>
+      <c r="BX14" s="40" t="n"/>
+      <c r="BY14" s="39" t="n"/>
       <c r="BZ14" s="24" t="n"/>
       <c r="CA14" s="31" t="n"/>
       <c r="CB14" s="24" t="n"/>
@@ -4978,7 +5005,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J15" s="25" t="n"/>
+      <c r="J15" s="38" t="n"/>
       <c r="K15" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -4987,7 +5014,7 @@
       <c r="L15" s="26" t="n">
         <v>-130</v>
       </c>
-      <c r="M15" s="27" t="n">
+      <c r="M15" s="39" t="n">
         <v>1.769231</v>
       </c>
       <c r="N15" s="28" t="n">
@@ -5029,11 +5056,11 @@
       <c r="X15" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="Y15" s="25" t="n"/>
+      <c r="Y15" s="38" t="n"/>
       <c r="Z15" s="26" t="n"/>
       <c r="AA15" s="28" t="n"/>
       <c r="AB15" s="28" t="n"/>
-      <c r="AC15" s="30" t="n">
+      <c r="AC15" s="40" t="n">
         <v>-2</v>
       </c>
       <c r="AD15" s="24" t="inlineStr">
@@ -5126,11 +5153,11 @@
         </is>
       </c>
       <c r="BI15" s="24" t="n"/>
-      <c r="BJ15" s="25" t="n"/>
+      <c r="BJ15" s="38" t="n"/>
       <c r="BK15" s="26" t="n">
         <v>-130</v>
       </c>
-      <c r="BL15" s="27" t="n">
+      <c r="BL15" s="39" t="n">
         <v>1.769231</v>
       </c>
       <c r="BM15" s="28" t="n">
@@ -5142,18 +5169,18 @@
       <c r="BO15" s="28" t="n">
         <v>0.523834</v>
       </c>
-      <c r="BP15" s="25" t="n"/>
-      <c r="BQ15" s="27" t="n"/>
+      <c r="BP15" s="38" t="n"/>
+      <c r="BQ15" s="39" t="n"/>
       <c r="BR15" s="28" t="n"/>
       <c r="BS15" s="28" t="n"/>
       <c r="BT15" s="28" t="n"/>
-      <c r="BU15" s="25" t="n"/>
+      <c r="BU15" s="38" t="n"/>
       <c r="BV15" s="29" t="n">
         <v>2</v>
       </c>
       <c r="BW15" s="24" t="n"/>
-      <c r="BX15" s="30" t="n"/>
-      <c r="BY15" s="27" t="n"/>
+      <c r="BX15" s="40" t="n"/>
+      <c r="BY15" s="39" t="n"/>
       <c r="BZ15" s="24" t="n"/>
       <c r="CA15" s="31" t="n"/>
       <c r="CB15" s="24" t="n"/>
@@ -5235,7 +5262,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J16" s="25" t="n"/>
+      <c r="J16" s="38" t="n"/>
       <c r="K16" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -5244,7 +5271,7 @@
       <c r="L16" s="26" t="n">
         <v>-110</v>
       </c>
-      <c r="M16" s="27" t="n">
+      <c r="M16" s="39" t="n">
         <v>1.909091</v>
       </c>
       <c r="N16" s="28" t="n">
@@ -5286,11 +5313,11 @@
       <c r="X16" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="Y16" s="25" t="n"/>
+      <c r="Y16" s="38" t="n"/>
       <c r="Z16" s="26" t="n"/>
       <c r="AA16" s="28" t="n"/>
       <c r="AB16" s="28" t="n"/>
-      <c r="AC16" s="30" t="n">
+      <c r="AC16" s="40" t="n">
         <v>-1.5</v>
       </c>
       <c r="AD16" s="24" t="inlineStr">
@@ -5383,11 +5410,11 @@
         </is>
       </c>
       <c r="BI16" s="24" t="n"/>
-      <c r="BJ16" s="25" t="n"/>
+      <c r="BJ16" s="38" t="n"/>
       <c r="BK16" s="26" t="n">
         <v>-110</v>
       </c>
-      <c r="BL16" s="27" t="n">
+      <c r="BL16" s="39" t="n">
         <v>1.909091</v>
       </c>
       <c r="BM16" s="28" t="n">
@@ -5399,18 +5426,18 @@
       <c r="BO16" s="28" t="n">
         <v>0.523834</v>
       </c>
-      <c r="BP16" s="25" t="n"/>
-      <c r="BQ16" s="27" t="n"/>
+      <c r="BP16" s="38" t="n"/>
+      <c r="BQ16" s="39" t="n"/>
       <c r="BR16" s="28" t="n"/>
       <c r="BS16" s="28" t="n"/>
       <c r="BT16" s="28" t="n"/>
-      <c r="BU16" s="25" t="n"/>
+      <c r="BU16" s="38" t="n"/>
       <c r="BV16" s="29" t="n">
         <v>1.04</v>
       </c>
       <c r="BW16" s="24" t="n"/>
-      <c r="BX16" s="30" t="n"/>
-      <c r="BY16" s="27" t="n"/>
+      <c r="BX16" s="40" t="n"/>
+      <c r="BY16" s="39" t="n"/>
       <c r="BZ16" s="24" t="n"/>
       <c r="CA16" s="31" t="n"/>
       <c r="CB16" s="24" t="n"/>
@@ -5492,7 +5519,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J17" s="25" t="n"/>
+      <c r="J17" s="38" t="n"/>
       <c r="K17" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -5501,7 +5528,7 @@
       <c r="L17" s="26" t="n">
         <v>-141</v>
       </c>
-      <c r="M17" s="27" t="n">
+      <c r="M17" s="39" t="n">
         <v>1.70922</v>
       </c>
       <c r="N17" s="28" t="n">
@@ -5543,11 +5570,11 @@
       <c r="X17" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="Y17" s="25" t="n"/>
+      <c r="Y17" s="38" t="n"/>
       <c r="Z17" s="26" t="n"/>
       <c r="AA17" s="28" t="n"/>
       <c r="AB17" s="28" t="n"/>
-      <c r="AC17" s="30" t="n">
+      <c r="AC17" s="40" t="n">
         <v>1.4184</v>
       </c>
       <c r="AD17" s="24" t="inlineStr">
@@ -5640,11 +5667,11 @@
         </is>
       </c>
       <c r="BI17" s="24" t="n"/>
-      <c r="BJ17" s="25" t="n"/>
+      <c r="BJ17" s="38" t="n"/>
       <c r="BK17" s="26" t="n">
         <v>-141</v>
       </c>
-      <c r="BL17" s="27" t="n">
+      <c r="BL17" s="39" t="n">
         <v>1.70922</v>
       </c>
       <c r="BM17" s="28" t="n">
@@ -5656,18 +5683,18 @@
       <c r="BO17" s="28" t="n">
         <v>0.523834</v>
       </c>
-      <c r="BP17" s="25" t="n"/>
-      <c r="BQ17" s="27" t="n"/>
+      <c r="BP17" s="38" t="n"/>
+      <c r="BQ17" s="39" t="n"/>
       <c r="BR17" s="28" t="n"/>
       <c r="BS17" s="28" t="n"/>
       <c r="BT17" s="28" t="n"/>
-      <c r="BU17" s="25" t="n"/>
+      <c r="BU17" s="38" t="n"/>
       <c r="BV17" s="29" t="n">
         <v>2</v>
       </c>
       <c r="BW17" s="24" t="n"/>
-      <c r="BX17" s="30" t="n"/>
-      <c r="BY17" s="27" t="n"/>
+      <c r="BX17" s="40" t="n"/>
+      <c r="BY17" s="39" t="n"/>
       <c r="BZ17" s="24" t="n"/>
       <c r="CA17" s="31" t="n"/>
       <c r="CB17" s="24" t="n"/>
@@ -5749,7 +5776,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J18" s="25" t="n"/>
+      <c r="J18" s="38" t="n"/>
       <c r="K18" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -5758,7 +5785,7 @@
       <c r="L18" s="26" t="n">
         <v>-110</v>
       </c>
-      <c r="M18" s="27" t="n">
+      <c r="M18" s="39" t="n">
         <v>1.909091</v>
       </c>
       <c r="N18" s="28" t="n">
@@ -5800,11 +5827,11 @@
       <c r="X18" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="Y18" s="25" t="n"/>
+      <c r="Y18" s="38" t="n"/>
       <c r="Z18" s="26" t="n"/>
       <c r="AA18" s="28" t="n"/>
       <c r="AB18" s="28" t="n"/>
-      <c r="AC18" s="30" t="n">
+      <c r="AC18" s="40" t="n">
         <v>-1.5</v>
       </c>
       <c r="AD18" s="24" t="inlineStr">
@@ -5897,11 +5924,11 @@
         </is>
       </c>
       <c r="BI18" s="24" t="n"/>
-      <c r="BJ18" s="25" t="n"/>
+      <c r="BJ18" s="38" t="n"/>
       <c r="BK18" s="26" t="n">
         <v>-110</v>
       </c>
-      <c r="BL18" s="27" t="n">
+      <c r="BL18" s="39" t="n">
         <v>1.909091</v>
       </c>
       <c r="BM18" s="28" t="n">
@@ -5913,18 +5940,18 @@
       <c r="BO18" s="28" t="n">
         <v>0.523834</v>
       </c>
-      <c r="BP18" s="25" t="n"/>
-      <c r="BQ18" s="27" t="n"/>
+      <c r="BP18" s="38" t="n"/>
+      <c r="BQ18" s="39" t="n"/>
       <c r="BR18" s="28" t="n"/>
       <c r="BS18" s="28" t="n"/>
       <c r="BT18" s="28" t="n"/>
-      <c r="BU18" s="25" t="n"/>
+      <c r="BU18" s="38" t="n"/>
       <c r="BV18" s="29" t="n">
         <v>1.04</v>
       </c>
       <c r="BW18" s="24" t="n"/>
-      <c r="BX18" s="30" t="n"/>
-      <c r="BY18" s="27" t="n"/>
+      <c r="BX18" s="40" t="n"/>
+      <c r="BY18" s="39" t="n"/>
       <c r="BZ18" s="24" t="n"/>
       <c r="CA18" s="31" t="n"/>
       <c r="CB18" s="24" t="n"/>
@@ -6006,7 +6033,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J19" s="25" t="n"/>
+      <c r="J19" s="38" t="n"/>
       <c r="K19" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -6015,7 +6042,7 @@
       <c r="L19" s="26" t="n">
         <v>-355</v>
       </c>
-      <c r="M19" s="27" t="n">
+      <c r="M19" s="39" t="n">
         <v>1.28169</v>
       </c>
       <c r="N19" s="28" t="n">
@@ -6057,11 +6084,11 @@
       <c r="X19" s="26" t="n">
         <v>110</v>
       </c>
-      <c r="Y19" s="25" t="n"/>
+      <c r="Y19" s="38" t="n"/>
       <c r="Z19" s="26" t="n"/>
       <c r="AA19" s="28" t="n"/>
       <c r="AB19" s="28" t="n"/>
-      <c r="AC19" s="30" t="n">
+      <c r="AC19" s="40" t="n">
         <v>0.5634</v>
       </c>
       <c r="AD19" s="24" t="inlineStr">
@@ -6154,11 +6181,11 @@
         </is>
       </c>
       <c r="BI19" s="24" t="n"/>
-      <c r="BJ19" s="25" t="n"/>
+      <c r="BJ19" s="38" t="n"/>
       <c r="BK19" s="26" t="n">
         <v>-355</v>
       </c>
-      <c r="BL19" s="27" t="n">
+      <c r="BL19" s="39" t="n">
         <v>1.28169</v>
       </c>
       <c r="BM19" s="28" t="n">
@@ -6170,18 +6197,18 @@
       <c r="BO19" s="28" t="n">
         <v>0.523834</v>
       </c>
-      <c r="BP19" s="25" t="n"/>
-      <c r="BQ19" s="27" t="n"/>
+      <c r="BP19" s="38" t="n"/>
+      <c r="BQ19" s="39" t="n"/>
       <c r="BR19" s="28" t="n"/>
       <c r="BS19" s="28" t="n"/>
       <c r="BT19" s="28" t="n"/>
-      <c r="BU19" s="25" t="n"/>
+      <c r="BU19" s="38" t="n"/>
       <c r="BV19" s="29" t="n">
         <v>2</v>
       </c>
       <c r="BW19" s="24" t="n"/>
-      <c r="BX19" s="30" t="n"/>
-      <c r="BY19" s="27" t="n"/>
+      <c r="BX19" s="40" t="n"/>
+      <c r="BY19" s="39" t="n"/>
       <c r="BZ19" s="24" t="n"/>
       <c r="CA19" s="31" t="n"/>
       <c r="CB19" s="24" t="n"/>
@@ -6255,7 +6282,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J20" s="25" t="n"/>
+      <c r="J20" s="38" t="n"/>
       <c r="K20" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -6264,7 +6291,7 @@
       <c r="L20" s="26" t="n">
         <v>-178</v>
       </c>
-      <c r="M20" s="27" t="n">
+      <c r="M20" s="39" t="n">
         <v>1.561798</v>
       </c>
       <c r="N20" s="28" t="n">
@@ -6306,7 +6333,7 @@
       <c r="X20" s="26" t="n">
         <v>83</v>
       </c>
-      <c r="Y20" s="25" t="n"/>
+      <c r="Y20" s="38" t="n"/>
       <c r="Z20" s="26" t="n">
         <v>-110</v>
       </c>
@@ -6314,7 +6341,7 @@
         <v>0.523834</v>
       </c>
       <c r="AB20" s="28" t="n"/>
-      <c r="AC20" s="30" t="n">
+      <c r="AC20" s="40" t="n">
         <v>-2</v>
       </c>
       <c r="AD20" s="24" t="inlineStr">
@@ -6403,11 +6430,11 @@
         </is>
       </c>
       <c r="BI20" s="24" t="n"/>
-      <c r="BJ20" s="25" t="n"/>
+      <c r="BJ20" s="38" t="n"/>
       <c r="BK20" s="26" t="n">
         <v>-178</v>
       </c>
-      <c r="BL20" s="27" t="n">
+      <c r="BL20" s="39" t="n">
         <v>1.561798</v>
       </c>
       <c r="BM20" s="28" t="n">
@@ -6419,20 +6446,20 @@
       <c r="BO20" s="28" t="n">
         <v>0.523834</v>
       </c>
-      <c r="BP20" s="25" t="n"/>
-      <c r="BQ20" s="27" t="n">
+      <c r="BP20" s="38" t="n"/>
+      <c r="BQ20" s="39" t="n">
         <v>1.909</v>
       </c>
       <c r="BR20" s="28" t="n"/>
       <c r="BS20" s="28" t="n"/>
       <c r="BT20" s="28" t="n"/>
-      <c r="BU20" s="25" t="n"/>
+      <c r="BU20" s="38" t="n"/>
       <c r="BV20" s="29" t="n">
         <v>2</v>
       </c>
       <c r="BW20" s="24" t="n"/>
-      <c r="BX20" s="30" t="n"/>
-      <c r="BY20" s="27" t="n"/>
+      <c r="BX20" s="40" t="n"/>
+      <c r="BY20" s="39" t="n"/>
       <c r="BZ20" s="24" t="n"/>
       <c r="CA20" s="31" t="n"/>
       <c r="CB20" s="24" t="n"/>
@@ -6506,7 +6533,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J21" s="25" t="n"/>
+      <c r="J21" s="38" t="n"/>
       <c r="K21" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -6515,7 +6542,7 @@
       <c r="L21" s="26" t="n">
         <v>108</v>
       </c>
-      <c r="M21" s="27" t="n">
+      <c r="M21" s="39" t="n">
         <v>2.08</v>
       </c>
       <c r="N21" s="28" t="n">
@@ -6557,11 +6584,11 @@
       <c r="X21" s="26" t="n">
         <v>108</v>
       </c>
-      <c r="Y21" s="25" t="n"/>
+      <c r="Y21" s="38" t="n"/>
       <c r="Z21" s="26" t="n"/>
       <c r="AA21" s="28" t="n"/>
       <c r="AB21" s="28" t="n"/>
-      <c r="AC21" s="30" t="n">
+      <c r="AC21" s="40" t="n">
         <v>1.62</v>
       </c>
       <c r="AD21" s="24" t="inlineStr">
@@ -6654,11 +6681,11 @@
         </is>
       </c>
       <c r="BI21" s="24" t="n"/>
-      <c r="BJ21" s="25" t="n"/>
+      <c r="BJ21" s="38" t="n"/>
       <c r="BK21" s="26" t="n">
         <v>108</v>
       </c>
-      <c r="BL21" s="27" t="n">
+      <c r="BL21" s="39" t="n">
         <v>2.08</v>
       </c>
       <c r="BM21" s="28" t="n">
@@ -6670,18 +6697,18 @@
       <c r="BO21" s="28" t="n">
         <v>0.523834</v>
       </c>
-      <c r="BP21" s="25" t="n"/>
-      <c r="BQ21" s="27" t="n"/>
+      <c r="BP21" s="38" t="n"/>
+      <c r="BQ21" s="39" t="n"/>
       <c r="BR21" s="28" t="n"/>
       <c r="BS21" s="28" t="n"/>
       <c r="BT21" s="28" t="n"/>
-      <c r="BU21" s="25" t="n"/>
+      <c r="BU21" s="38" t="n"/>
       <c r="BV21" s="29" t="n">
         <v>1.69</v>
       </c>
       <c r="BW21" s="24" t="n"/>
-      <c r="BX21" s="30" t="n"/>
-      <c r="BY21" s="27" t="n"/>
+      <c r="BX21" s="40" t="n"/>
+      <c r="BY21" s="39" t="n"/>
       <c r="BZ21" s="24" t="n"/>
       <c r="CA21" s="31" t="n"/>
       <c r="CB21" s="24" t="n"/>
@@ -6755,7 +6782,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J22" s="25" t="n"/>
+      <c r="J22" s="38" t="n"/>
       <c r="K22" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -6764,7 +6791,7 @@
       <c r="L22" s="26" t="n">
         <v>-669</v>
       </c>
-      <c r="M22" s="27" t="n">
+      <c r="M22" s="39" t="n">
         <v>1.149477</v>
       </c>
       <c r="N22" s="28" t="n">
@@ -6806,7 +6833,7 @@
       <c r="X22" s="26" t="n">
         <v>101</v>
       </c>
-      <c r="Y22" s="25" t="n"/>
+      <c r="Y22" s="38" t="n"/>
       <c r="Z22" s="26" t="n">
         <v>-110</v>
       </c>
@@ -6814,7 +6841,7 @@
         <v>0.523834</v>
       </c>
       <c r="AB22" s="28" t="n"/>
-      <c r="AC22" s="30" t="n">
+      <c r="AC22" s="40" t="n">
         <v>0.299</v>
       </c>
       <c r="AD22" s="24" t="inlineStr">
@@ -6903,11 +6930,11 @@
         </is>
       </c>
       <c r="BI22" s="24" t="n"/>
-      <c r="BJ22" s="25" t="n"/>
+      <c r="BJ22" s="38" t="n"/>
       <c r="BK22" s="26" t="n">
         <v>-669</v>
       </c>
-      <c r="BL22" s="27" t="n">
+      <c r="BL22" s="39" t="n">
         <v>1.149477</v>
       </c>
       <c r="BM22" s="28" t="n">
@@ -6919,20 +6946,20 @@
       <c r="BO22" s="28" t="n">
         <v>0.523834</v>
       </c>
-      <c r="BP22" s="25" t="n"/>
-      <c r="BQ22" s="27" t="n">
+      <c r="BP22" s="38" t="n"/>
+      <c r="BQ22" s="39" t="n">
         <v>1.909</v>
       </c>
       <c r="BR22" s="28" t="n"/>
       <c r="BS22" s="28" t="n"/>
       <c r="BT22" s="28" t="n"/>
-      <c r="BU22" s="25" t="n"/>
+      <c r="BU22" s="38" t="n"/>
       <c r="BV22" s="29" t="n">
         <v>2</v>
       </c>
       <c r="BW22" s="24" t="n"/>
-      <c r="BX22" s="30" t="n"/>
-      <c r="BY22" s="27" t="n"/>
+      <c r="BX22" s="40" t="n"/>
+      <c r="BY22" s="39" t="n"/>
       <c r="BZ22" s="24" t="n"/>
       <c r="CA22" s="31" t="n"/>
       <c r="CB22" s="24" t="n"/>
@@ -7006,7 +7033,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J23" s="25" t="n"/>
+      <c r="J23" s="38" t="n"/>
       <c r="K23" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -7015,7 +7042,7 @@
       <c r="L23" s="26" t="n">
         <v>-355</v>
       </c>
-      <c r="M23" s="27" t="n">
+      <c r="M23" s="39" t="n">
         <v>1.28169</v>
       </c>
       <c r="N23" s="28" t="n">
@@ -7057,7 +7084,7 @@
       <c r="X23" s="26" t="n">
         <v>74</v>
       </c>
-      <c r="Y23" s="25" t="n"/>
+      <c r="Y23" s="38" t="n"/>
       <c r="Z23" s="26" t="n">
         <v>-110</v>
       </c>
@@ -7065,7 +7092,7 @@
         <v>0.523834</v>
       </c>
       <c r="AB23" s="28" t="n"/>
-      <c r="AC23" s="30" t="n">
+      <c r="AC23" s="40" t="n">
         <v>0.5634</v>
       </c>
       <c r="AD23" s="24" t="inlineStr">
@@ -7154,11 +7181,11 @@
         </is>
       </c>
       <c r="BI23" s="24" t="n"/>
-      <c r="BJ23" s="25" t="n"/>
+      <c r="BJ23" s="38" t="n"/>
       <c r="BK23" s="26" t="n">
         <v>-355</v>
       </c>
-      <c r="BL23" s="27" t="n">
+      <c r="BL23" s="39" t="n">
         <v>1.28169</v>
       </c>
       <c r="BM23" s="28" t="n">
@@ -7170,20 +7197,20 @@
       <c r="BO23" s="28" t="n">
         <v>0.523834</v>
       </c>
-      <c r="BP23" s="25" t="n"/>
-      <c r="BQ23" s="27" t="n">
+      <c r="BP23" s="38" t="n"/>
+      <c r="BQ23" s="39" t="n">
         <v>1.909</v>
       </c>
       <c r="BR23" s="28" t="n"/>
       <c r="BS23" s="28" t="n"/>
       <c r="BT23" s="28" t="n"/>
-      <c r="BU23" s="25" t="n"/>
+      <c r="BU23" s="38" t="n"/>
       <c r="BV23" s="29" t="n">
         <v>2</v>
       </c>
       <c r="BW23" s="24" t="n"/>
-      <c r="BX23" s="30" t="n"/>
-      <c r="BY23" s="27" t="n"/>
+      <c r="BX23" s="40" t="n"/>
+      <c r="BY23" s="39" t="n"/>
       <c r="BZ23" s="24" t="n"/>
       <c r="CA23" s="31" t="n"/>
       <c r="CB23" s="24" t="n"/>
@@ -7257,7 +7284,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J24" s="25" t="n"/>
+      <c r="J24" s="38" t="n"/>
       <c r="K24" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -7266,7 +7293,7 @@
       <c r="L24" s="26" t="n">
         <v>-400</v>
       </c>
-      <c r="M24" s="27" t="n">
+      <c r="M24" s="39" t="n">
         <v>1.25</v>
       </c>
       <c r="N24" s="28" t="n">
@@ -7308,11 +7335,11 @@
       <c r="X24" s="26" t="n">
         <v>90</v>
       </c>
-      <c r="Y24" s="25" t="n"/>
+      <c r="Y24" s="38" t="n"/>
       <c r="Z24" s="26" t="n"/>
       <c r="AA24" s="28" t="n"/>
       <c r="AB24" s="28" t="n"/>
-      <c r="AC24" s="30" t="n">
+      <c r="AC24" s="40" t="n">
         <v>0.5</v>
       </c>
       <c r="AD24" s="24" t="inlineStr">
@@ -7405,11 +7432,11 @@
         </is>
       </c>
       <c r="BI24" s="24" t="n"/>
-      <c r="BJ24" s="25" t="n"/>
+      <c r="BJ24" s="38" t="n"/>
       <c r="BK24" s="26" t="n">
         <v>-400</v>
       </c>
-      <c r="BL24" s="27" t="n">
+      <c r="BL24" s="39" t="n">
         <v>1.25</v>
       </c>
       <c r="BM24" s="28" t="n">
@@ -7421,18 +7448,18 @@
       <c r="BO24" s="28" t="n">
         <v>0.523834</v>
       </c>
-      <c r="BP24" s="25" t="n"/>
-      <c r="BQ24" s="27" t="n"/>
+      <c r="BP24" s="38" t="n"/>
+      <c r="BQ24" s="39" t="n"/>
       <c r="BR24" s="28" t="n"/>
       <c r="BS24" s="28" t="n"/>
       <c r="BT24" s="28" t="n"/>
-      <c r="BU24" s="25" t="n"/>
+      <c r="BU24" s="38" t="n"/>
       <c r="BV24" s="29" t="n">
         <v>2</v>
       </c>
       <c r="BW24" s="24" t="n"/>
-      <c r="BX24" s="30" t="n"/>
-      <c r="BY24" s="27" t="n"/>
+      <c r="BX24" s="40" t="n"/>
+      <c r="BY24" s="39" t="n"/>
       <c r="BZ24" s="24" t="n"/>
       <c r="CA24" s="31" t="n"/>
       <c r="CB24" s="24" t="n"/>
@@ -7506,7 +7533,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J25" s="25" t="n"/>
+      <c r="J25" s="38" t="n"/>
       <c r="K25" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -7515,7 +7542,7 @@
       <c r="L25" s="26" t="n">
         <v>-488</v>
       </c>
-      <c r="M25" s="27" t="n">
+      <c r="M25" s="39" t="n">
         <v>1.204918</v>
       </c>
       <c r="N25" s="28" t="n">
@@ -7557,7 +7584,7 @@
       <c r="X25" s="26" t="n">
         <v>93</v>
       </c>
-      <c r="Y25" s="25" t="n"/>
+      <c r="Y25" s="38" t="n"/>
       <c r="Z25" s="26" t="n">
         <v>-110</v>
       </c>
@@ -7565,7 +7592,7 @@
         <v>0.523834</v>
       </c>
       <c r="AB25" s="28" t="n"/>
-      <c r="AC25" s="30" t="n">
+      <c r="AC25" s="40" t="n">
         <v>0.4098</v>
       </c>
       <c r="AD25" s="24" t="inlineStr">
@@ -7654,11 +7681,11 @@
         </is>
       </c>
       <c r="BI25" s="24" t="n"/>
-      <c r="BJ25" s="25" t="n"/>
+      <c r="BJ25" s="38" t="n"/>
       <c r="BK25" s="26" t="n">
         <v>-488</v>
       </c>
-      <c r="BL25" s="27" t="n">
+      <c r="BL25" s="39" t="n">
         <v>1.204918</v>
       </c>
       <c r="BM25" s="28" t="n">
@@ -7670,20 +7697,20 @@
       <c r="BO25" s="28" t="n">
         <v>0.523834</v>
       </c>
-      <c r="BP25" s="25" t="n"/>
-      <c r="BQ25" s="27" t="n">
+      <c r="BP25" s="38" t="n"/>
+      <c r="BQ25" s="39" t="n">
         <v>1.909</v>
       </c>
       <c r="BR25" s="28" t="n"/>
       <c r="BS25" s="28" t="n"/>
       <c r="BT25" s="28" t="n"/>
-      <c r="BU25" s="25" t="n"/>
+      <c r="BU25" s="38" t="n"/>
       <c r="BV25" s="29" t="n">
         <v>2</v>
       </c>
       <c r="BW25" s="24" t="n"/>
-      <c r="BX25" s="30" t="n"/>
-      <c r="BY25" s="27" t="n"/>
+      <c r="BX25" s="40" t="n"/>
+      <c r="BY25" s="39" t="n"/>
       <c r="BZ25" s="24" t="n"/>
       <c r="CA25" s="31" t="n"/>
       <c r="CB25" s="24" t="n"/>
@@ -7757,7 +7784,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J26" s="25" t="n"/>
+      <c r="J26" s="38" t="n"/>
       <c r="K26" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -7766,7 +7793,7 @@
       <c r="L26" s="26" t="n">
         <v>-163</v>
       </c>
-      <c r="M26" s="27" t="n">
+      <c r="M26" s="39" t="n">
         <v>1.613497</v>
       </c>
       <c r="N26" s="28" t="n">
@@ -7808,7 +7835,7 @@
       <c r="X26" s="26" t="n">
         <v>72</v>
       </c>
-      <c r="Y26" s="25" t="n"/>
+      <c r="Y26" s="38" t="n"/>
       <c r="Z26" s="26" t="n">
         <v>-110</v>
       </c>
@@ -7816,7 +7843,7 @@
         <v>0.523834</v>
       </c>
       <c r="AB26" s="28" t="n"/>
-      <c r="AC26" s="30" t="n">
+      <c r="AC26" s="40" t="n">
         <v>0.7669</v>
       </c>
       <c r="AD26" s="24" t="inlineStr">
@@ -7905,11 +7932,11 @@
         </is>
       </c>
       <c r="BI26" s="24" t="n"/>
-      <c r="BJ26" s="25" t="n"/>
+      <c r="BJ26" s="38" t="n"/>
       <c r="BK26" s="26" t="n">
         <v>-163</v>
       </c>
-      <c r="BL26" s="27" t="n">
+      <c r="BL26" s="39" t="n">
         <v>1.613497</v>
       </c>
       <c r="BM26" s="28" t="n">
@@ -7921,20 +7948,20 @@
       <c r="BO26" s="28" t="n">
         <v>0.523834</v>
       </c>
-      <c r="BP26" s="25" t="n"/>
-      <c r="BQ26" s="27" t="n">
+      <c r="BP26" s="38" t="n"/>
+      <c r="BQ26" s="39" t="n">
         <v>1.909</v>
       </c>
       <c r="BR26" s="28" t="n"/>
       <c r="BS26" s="28" t="n"/>
       <c r="BT26" s="28" t="n"/>
-      <c r="BU26" s="25" t="n"/>
+      <c r="BU26" s="38" t="n"/>
       <c r="BV26" s="29" t="n">
         <v>1.05</v>
       </c>
       <c r="BW26" s="24" t="n"/>
-      <c r="BX26" s="30" t="n"/>
-      <c r="BY26" s="27" t="n"/>
+      <c r="BX26" s="40" t="n"/>
+      <c r="BY26" s="39" t="n"/>
       <c r="BZ26" s="24" t="n"/>
       <c r="CA26" s="31" t="n"/>
       <c r="CB26" s="24" t="n"/>
@@ -8008,7 +8035,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J27" s="25" t="n"/>
+      <c r="J27" s="38" t="n"/>
       <c r="K27" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -8017,7 +8044,7 @@
       <c r="L27" s="26" t="n">
         <v>186</v>
       </c>
-      <c r="M27" s="27" t="n">
+      <c r="M27" s="39" t="n">
         <v>2.86</v>
       </c>
       <c r="N27" s="28" t="n">
@@ -8059,11 +8086,11 @@
       <c r="X27" s="26" t="n">
         <v>98</v>
       </c>
-      <c r="Y27" s="25" t="n"/>
+      <c r="Y27" s="38" t="n"/>
       <c r="Z27" s="26" t="n"/>
       <c r="AA27" s="28" t="n"/>
       <c r="AB27" s="28" t="n"/>
-      <c r="AC27" s="30" t="n">
+      <c r="AC27" s="40" t="n">
         <v>-2</v>
       </c>
       <c r="AD27" s="24" t="inlineStr">
@@ -8156,11 +8183,11 @@
         </is>
       </c>
       <c r="BI27" s="24" t="n"/>
-      <c r="BJ27" s="25" t="n"/>
+      <c r="BJ27" s="38" t="n"/>
       <c r="BK27" s="26" t="n">
         <v>186</v>
       </c>
-      <c r="BL27" s="27" t="n">
+      <c r="BL27" s="39" t="n">
         <v>2.86</v>
       </c>
       <c r="BM27" s="28" t="n">
@@ -8172,18 +8199,18 @@
       <c r="BO27" s="28" t="n">
         <v>0.523834</v>
       </c>
-      <c r="BP27" s="25" t="n"/>
-      <c r="BQ27" s="27" t="n"/>
+      <c r="BP27" s="38" t="n"/>
+      <c r="BQ27" s="39" t="n"/>
       <c r="BR27" s="28" t="n"/>
       <c r="BS27" s="28" t="n"/>
       <c r="BT27" s="28" t="n"/>
-      <c r="BU27" s="25" t="n"/>
+      <c r="BU27" s="38" t="n"/>
       <c r="BV27" s="29" t="n">
         <v>2</v>
       </c>
       <c r="BW27" s="24" t="n"/>
-      <c r="BX27" s="30" t="n"/>
-      <c r="BY27" s="27" t="n"/>
+      <c r="BX27" s="40" t="n"/>
+      <c r="BY27" s="39" t="n"/>
       <c r="BZ27" s="24" t="n"/>
       <c r="CA27" s="31" t="n"/>
       <c r="CB27" s="24" t="n"/>
@@ -8257,7 +8284,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J28" s="25" t="n"/>
+      <c r="J28" s="38" t="n"/>
       <c r="K28" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -8266,7 +8293,7 @@
       <c r="L28" s="26" t="n">
         <v>-335</v>
       </c>
-      <c r="M28" s="27" t="n">
+      <c r="M28" s="39" t="n">
         <v>1.298507</v>
       </c>
       <c r="N28" s="28" t="n">
@@ -8308,7 +8335,7 @@
       <c r="X28" s="26" t="n">
         <v>82</v>
       </c>
-      <c r="Y28" s="25" t="n"/>
+      <c r="Y28" s="38" t="n"/>
       <c r="Z28" s="26" t="n">
         <v>-110</v>
       </c>
@@ -8316,7 +8343,7 @@
         <v>0.523834</v>
       </c>
       <c r="AB28" s="28" t="n"/>
-      <c r="AC28" s="30" t="n">
+      <c r="AC28" s="40" t="n">
         <v>-2</v>
       </c>
       <c r="AD28" s="24" t="inlineStr">
@@ -8405,11 +8432,11 @@
         </is>
       </c>
       <c r="BI28" s="24" t="n"/>
-      <c r="BJ28" s="25" t="n"/>
+      <c r="BJ28" s="38" t="n"/>
       <c r="BK28" s="26" t="n">
         <v>-335</v>
       </c>
-      <c r="BL28" s="27" t="n">
+      <c r="BL28" s="39" t="n">
         <v>1.298507</v>
       </c>
       <c r="BM28" s="28" t="n">
@@ -8421,20 +8448,20 @@
       <c r="BO28" s="28" t="n">
         <v>0.523834</v>
       </c>
-      <c r="BP28" s="25" t="n"/>
-      <c r="BQ28" s="27" t="n">
+      <c r="BP28" s="38" t="n"/>
+      <c r="BQ28" s="39" t="n">
         <v>1.909</v>
       </c>
       <c r="BR28" s="28" t="n"/>
       <c r="BS28" s="28" t="n"/>
       <c r="BT28" s="28" t="n"/>
-      <c r="BU28" s="25" t="n"/>
+      <c r="BU28" s="38" t="n"/>
       <c r="BV28" s="29" t="n">
         <v>2</v>
       </c>
       <c r="BW28" s="24" t="n"/>
-      <c r="BX28" s="30" t="n"/>
-      <c r="BY28" s="27" t="n"/>
+      <c r="BX28" s="40" t="n"/>
+      <c r="BY28" s="39" t="n"/>
       <c r="BZ28" s="24" t="n"/>
       <c r="CA28" s="31" t="n"/>
       <c r="CB28" s="24" t="n"/>
@@ -8508,7 +8535,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J29" s="25" t="n"/>
+      <c r="J29" s="38" t="n"/>
       <c r="K29" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -8517,7 +8544,7 @@
       <c r="L29" s="26" t="n">
         <v>-127</v>
       </c>
-      <c r="M29" s="27" t="n">
+      <c r="M29" s="39" t="n">
         <v>1.787402</v>
       </c>
       <c r="N29" s="28" t="n">
@@ -8559,11 +8586,11 @@
       <c r="X29" s="26" t="n">
         <v>82</v>
       </c>
-      <c r="Y29" s="25" t="n"/>
+      <c r="Y29" s="38" t="n"/>
       <c r="Z29" s="26" t="n"/>
       <c r="AA29" s="28" t="n"/>
       <c r="AB29" s="28" t="n"/>
-      <c r="AC29" s="30" t="n">
+      <c r="AC29" s="40" t="n">
         <v>-1.25</v>
       </c>
       <c r="AD29" s="24" t="inlineStr">
@@ -8656,11 +8683,11 @@
         </is>
       </c>
       <c r="BI29" s="24" t="n"/>
-      <c r="BJ29" s="25" t="n"/>
+      <c r="BJ29" s="38" t="n"/>
       <c r="BK29" s="26" t="n">
         <v>-127</v>
       </c>
-      <c r="BL29" s="27" t="n">
+      <c r="BL29" s="39" t="n">
         <v>1.787402</v>
       </c>
       <c r="BM29" s="28" t="n">
@@ -8672,18 +8699,18 @@
       <c r="BO29" s="28" t="n">
         <v>0.523834</v>
       </c>
-      <c r="BP29" s="25" t="n"/>
-      <c r="BQ29" s="27" t="n"/>
+      <c r="BP29" s="38" t="n"/>
+      <c r="BQ29" s="39" t="n"/>
       <c r="BR29" s="28" t="n"/>
       <c r="BS29" s="28" t="n"/>
       <c r="BT29" s="28" t="n"/>
-      <c r="BU29" s="25" t="n"/>
+      <c r="BU29" s="38" t="n"/>
       <c r="BV29" s="29" t="n">
         <v>0.98</v>
       </c>
       <c r="BW29" s="24" t="n"/>
-      <c r="BX29" s="30" t="n"/>
-      <c r="BY29" s="27" t="n"/>
+      <c r="BX29" s="40" t="n"/>
+      <c r="BY29" s="39" t="n"/>
       <c r="BZ29" s="24" t="n"/>
       <c r="CA29" s="31" t="n"/>
       <c r="CB29" s="24" t="n"/>
@@ -8757,7 +8784,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J30" s="25" t="n"/>
+      <c r="J30" s="38" t="n"/>
       <c r="K30" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -8766,7 +8793,7 @@
       <c r="L30" s="26" t="n">
         <v>-285</v>
       </c>
-      <c r="M30" s="27" t="n">
+      <c r="M30" s="39" t="n">
         <v>1.350877</v>
       </c>
       <c r="N30" s="28" t="n">
@@ -8808,11 +8835,11 @@
       <c r="X30" s="26" t="n">
         <v>95</v>
       </c>
-      <c r="Y30" s="25" t="n"/>
+      <c r="Y30" s="38" t="n"/>
       <c r="Z30" s="26" t="n"/>
       <c r="AA30" s="28" t="n"/>
       <c r="AB30" s="28" t="n"/>
-      <c r="AC30" s="30" t="n">
+      <c r="AC30" s="40" t="n">
         <v>0.7018</v>
       </c>
       <c r="AD30" s="24" t="inlineStr">
@@ -8905,11 +8932,11 @@
         </is>
       </c>
       <c r="BI30" s="24" t="n"/>
-      <c r="BJ30" s="25" t="n"/>
+      <c r="BJ30" s="38" t="n"/>
       <c r="BK30" s="26" t="n">
         <v>-285</v>
       </c>
-      <c r="BL30" s="27" t="n">
+      <c r="BL30" s="39" t="n">
         <v>1.350877</v>
       </c>
       <c r="BM30" s="28" t="n">
@@ -8921,18 +8948,18 @@
       <c r="BO30" s="28" t="n">
         <v>0.523834</v>
       </c>
-      <c r="BP30" s="25" t="n"/>
-      <c r="BQ30" s="27" t="n"/>
+      <c r="BP30" s="38" t="n"/>
+      <c r="BQ30" s="39" t="n"/>
       <c r="BR30" s="28" t="n"/>
       <c r="BS30" s="28" t="n"/>
       <c r="BT30" s="28" t="n"/>
-      <c r="BU30" s="25" t="n"/>
+      <c r="BU30" s="38" t="n"/>
       <c r="BV30" s="29" t="n">
         <v>2</v>
       </c>
       <c r="BW30" s="24" t="n"/>
-      <c r="BX30" s="30" t="n"/>
-      <c r="BY30" s="27" t="n"/>
+      <c r="BX30" s="40" t="n"/>
+      <c r="BY30" s="39" t="n"/>
       <c r="BZ30" s="24" t="n"/>
       <c r="CA30" s="31" t="n"/>
       <c r="CB30" s="24" t="n"/>
@@ -9006,7 +9033,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J31" s="25" t="n"/>
+      <c r="J31" s="38" t="n"/>
       <c r="K31" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -9015,7 +9042,7 @@
       <c r="L31" s="26" t="n">
         <v>120</v>
       </c>
-      <c r="M31" s="27" t="n">
+      <c r="M31" s="39" t="n">
         <v>2.2</v>
       </c>
       <c r="N31" s="28" t="n">
@@ -9057,7 +9084,7 @@
       <c r="X31" s="26" t="n">
         <v>15</v>
       </c>
-      <c r="Y31" s="25" t="n"/>
+      <c r="Y31" s="38" t="n"/>
       <c r="Z31" s="26" t="n">
         <v>-110</v>
       </c>
@@ -9065,7 +9092,7 @@
         <v>0.523834</v>
       </c>
       <c r="AB31" s="28" t="n"/>
-      <c r="AC31" s="30" t="n">
+      <c r="AC31" s="40" t="n">
         <v>1.8</v>
       </c>
       <c r="AD31" s="24" t="inlineStr">
@@ -9154,11 +9181,11 @@
         </is>
       </c>
       <c r="BI31" s="24" t="n"/>
-      <c r="BJ31" s="25" t="n"/>
+      <c r="BJ31" s="38" t="n"/>
       <c r="BK31" s="26" t="n">
         <v>120</v>
       </c>
-      <c r="BL31" s="27" t="n">
+      <c r="BL31" s="39" t="n">
         <v>2.2</v>
       </c>
       <c r="BM31" s="28" t="n">
@@ -9170,20 +9197,20 @@
       <c r="BO31" s="28" t="n">
         <v>0.523834</v>
       </c>
-      <c r="BP31" s="25" t="n"/>
-      <c r="BQ31" s="27" t="n">
+      <c r="BP31" s="38" t="n"/>
+      <c r="BQ31" s="39" t="n">
         <v>1.909</v>
       </c>
       <c r="BR31" s="28" t="n"/>
       <c r="BS31" s="28" t="n"/>
       <c r="BT31" s="28" t="n"/>
-      <c r="BU31" s="25" t="n"/>
+      <c r="BU31" s="38" t="n"/>
       <c r="BV31" s="29" t="n">
         <v>0.5</v>
       </c>
       <c r="BW31" s="24" t="n"/>
-      <c r="BX31" s="30" t="n"/>
-      <c r="BY31" s="27" t="n"/>
+      <c r="BX31" s="40" t="n"/>
+      <c r="BY31" s="39" t="n"/>
       <c r="BZ31" s="24" t="n"/>
       <c r="CA31" s="31" t="n"/>
       <c r="CB31" s="24" t="n"/>
@@ -9265,7 +9292,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J32" s="25" t="n"/>
+      <c r="J32" s="38" t="n"/>
       <c r="K32" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -9274,7 +9301,7 @@
       <c r="L32" s="26" t="n">
         <v>106</v>
       </c>
-      <c r="M32" s="27" t="n">
+      <c r="M32" s="39" t="n">
         <v>2.06</v>
       </c>
       <c r="N32" s="28" t="n">
@@ -9316,7 +9343,7 @@
       <c r="X32" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="Y32" s="25" t="n"/>
+      <c r="Y32" s="38" t="n"/>
       <c r="Z32" s="26" t="n">
         <v>-110</v>
       </c>
@@ -9324,7 +9351,7 @@
         <v>0.523834</v>
       </c>
       <c r="AB32" s="28" t="n"/>
-      <c r="AC32" s="30" t="n">
+      <c r="AC32" s="40" t="n">
         <v>1.855</v>
       </c>
       <c r="AD32" s="24" t="inlineStr">
@@ -9413,11 +9440,11 @@
         </is>
       </c>
       <c r="BI32" s="24" t="n"/>
-      <c r="BJ32" s="25" t="n"/>
+      <c r="BJ32" s="38" t="n"/>
       <c r="BK32" s="26" t="n">
         <v>106</v>
       </c>
-      <c r="BL32" s="27" t="n">
+      <c r="BL32" s="39" t="n">
         <v>2.06</v>
       </c>
       <c r="BM32" s="28" t="n">
@@ -9429,20 +9456,20 @@
       <c r="BO32" s="28" t="n">
         <v>0.523834</v>
       </c>
-      <c r="BP32" s="25" t="n"/>
-      <c r="BQ32" s="27" t="n">
+      <c r="BP32" s="38" t="n"/>
+      <c r="BQ32" s="39" t="n">
         <v>1.909</v>
       </c>
       <c r="BR32" s="28" t="n"/>
       <c r="BS32" s="28" t="n"/>
       <c r="BT32" s="28" t="n"/>
-      <c r="BU32" s="25" t="n"/>
+      <c r="BU32" s="38" t="n"/>
       <c r="BV32" s="29" t="n">
         <v>0.95</v>
       </c>
       <c r="BW32" s="24" t="n"/>
-      <c r="BX32" s="30" t="n"/>
-      <c r="BY32" s="27" t="n"/>
+      <c r="BX32" s="40" t="n"/>
+      <c r="BY32" s="39" t="n"/>
       <c r="BZ32" s="24" t="n"/>
       <c r="CA32" s="31" t="n"/>
       <c r="CB32" s="24" t="n"/>
@@ -9524,7 +9551,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J33" s="25" t="n"/>
+      <c r="J33" s="38" t="n"/>
       <c r="K33" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -9533,7 +9560,7 @@
       <c r="L33" s="26" t="n">
         <v>-102</v>
       </c>
-      <c r="M33" s="27" t="n">
+      <c r="M33" s="39" t="n">
         <v>1.980392</v>
       </c>
       <c r="N33" s="28" t="n">
@@ -9575,7 +9602,7 @@
       <c r="X33" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="Y33" s="25" t="n"/>
+      <c r="Y33" s="38" t="n"/>
       <c r="Z33" s="26" t="n">
         <v>-110</v>
       </c>
@@ -9583,7 +9610,7 @@
         <v>0.523834</v>
       </c>
       <c r="AB33" s="28" t="n"/>
-      <c r="AC33" s="30" t="n">
+      <c r="AC33" s="40" t="n">
         <v>-1.25</v>
       </c>
       <c r="AD33" s="24" t="inlineStr">
@@ -9672,11 +9699,11 @@
         </is>
       </c>
       <c r="BI33" s="24" t="n"/>
-      <c r="BJ33" s="25" t="n"/>
+      <c r="BJ33" s="38" t="n"/>
       <c r="BK33" s="26" t="n">
         <v>-102</v>
       </c>
-      <c r="BL33" s="27" t="n">
+      <c r="BL33" s="39" t="n">
         <v>1.980392</v>
       </c>
       <c r="BM33" s="28" t="n">
@@ -9688,20 +9715,20 @@
       <c r="BO33" s="28" t="n">
         <v>0.523834</v>
       </c>
-      <c r="BP33" s="25" t="n"/>
-      <c r="BQ33" s="27" t="n">
+      <c r="BP33" s="38" t="n"/>
+      <c r="BQ33" s="39" t="n">
         <v>1.909</v>
       </c>
       <c r="BR33" s="28" t="n"/>
       <c r="BS33" s="28" t="n"/>
       <c r="BT33" s="28" t="n"/>
-      <c r="BU33" s="25" t="n"/>
+      <c r="BU33" s="38" t="n"/>
       <c r="BV33" s="29" t="n">
         <v>0.5</v>
       </c>
       <c r="BW33" s="24" t="n"/>
-      <c r="BX33" s="30" t="n"/>
-      <c r="BY33" s="27" t="n"/>
+      <c r="BX33" s="40" t="n"/>
+      <c r="BY33" s="39" t="n"/>
       <c r="BZ33" s="24" t="n"/>
       <c r="CA33" s="31" t="n"/>
       <c r="CB33" s="24" t="n"/>
@@ -9783,7 +9810,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J34" s="25" t="n"/>
+      <c r="J34" s="38" t="n"/>
       <c r="K34" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -9792,7 +9819,7 @@
       <c r="L34" s="26" t="n">
         <v>-100</v>
       </c>
-      <c r="M34" s="27" t="n">
+      <c r="M34" s="39" t="n">
         <v>2</v>
       </c>
       <c r="N34" s="28" t="n">
@@ -9834,11 +9861,11 @@
       <c r="X34" s="26" t="n">
         <v>15</v>
       </c>
-      <c r="Y34" s="25" t="n"/>
+      <c r="Y34" s="38" t="n"/>
       <c r="Z34" s="26" t="n"/>
       <c r="AA34" s="28" t="n"/>
       <c r="AB34" s="28" t="n"/>
-      <c r="AC34" s="30" t="n">
+      <c r="AC34" s="40" t="n">
         <v>2</v>
       </c>
       <c r="AD34" s="24" t="inlineStr">
@@ -9931,11 +9958,11 @@
         </is>
       </c>
       <c r="BI34" s="24" t="n"/>
-      <c r="BJ34" s="25" t="n"/>
+      <c r="BJ34" s="38" t="n"/>
       <c r="BK34" s="26" t="n">
         <v>-100</v>
       </c>
-      <c r="BL34" s="27" t="n">
+      <c r="BL34" s="39" t="n">
         <v>2</v>
       </c>
       <c r="BM34" s="28" t="n">
@@ -9947,18 +9974,18 @@
       <c r="BO34" s="28" t="n">
         <v>0.523834</v>
       </c>
-      <c r="BP34" s="25" t="n"/>
-      <c r="BQ34" s="27" t="n"/>
+      <c r="BP34" s="38" t="n"/>
+      <c r="BQ34" s="39" t="n"/>
       <c r="BR34" s="28" t="n"/>
       <c r="BS34" s="28" t="n"/>
       <c r="BT34" s="28" t="n"/>
-      <c r="BU34" s="25" t="n"/>
+      <c r="BU34" s="38" t="n"/>
       <c r="BV34" s="29" t="n">
         <v>0.87</v>
       </c>
       <c r="BW34" s="24" t="n"/>
-      <c r="BX34" s="30" t="n"/>
-      <c r="BY34" s="27" t="n"/>
+      <c r="BX34" s="40" t="n"/>
+      <c r="BY34" s="39" t="n"/>
       <c r="BZ34" s="24" t="n"/>
       <c r="CA34" s="31" t="n"/>
       <c r="CB34" s="24" t="n"/>
@@ -10040,7 +10067,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J35" s="25" t="n"/>
+      <c r="J35" s="38" t="n"/>
       <c r="K35" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -10049,7 +10076,7 @@
       <c r="L35" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="M35" s="27" t="n">
+      <c r="M35" s="39" t="n">
         <v>1.961538</v>
       </c>
       <c r="N35" s="28" t="n">
@@ -10091,11 +10118,11 @@
       <c r="X35" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="Y35" s="25" t="n"/>
+      <c r="Y35" s="38" t="n"/>
       <c r="Z35" s="26" t="n"/>
       <c r="AA35" s="28" t="n"/>
       <c r="AB35" s="28" t="n"/>
-      <c r="AC35" s="30" t="n">
+      <c r="AC35" s="40" t="n">
         <v>-1.75</v>
       </c>
       <c r="AD35" s="24" t="inlineStr">
@@ -10188,11 +10215,11 @@
         </is>
       </c>
       <c r="BI35" s="24" t="n"/>
-      <c r="BJ35" s="25" t="n"/>
+      <c r="BJ35" s="38" t="n"/>
       <c r="BK35" s="26" t="n">
         <v>-104</v>
       </c>
-      <c r="BL35" s="27" t="n">
+      <c r="BL35" s="39" t="n">
         <v>1.961538</v>
       </c>
       <c r="BM35" s="28" t="n">
@@ -10204,18 +10231,18 @@
       <c r="BO35" s="28" t="n">
         <v>0.523834</v>
       </c>
-      <c r="BP35" s="25" t="n"/>
-      <c r="BQ35" s="27" t="n"/>
+      <c r="BP35" s="38" t="n"/>
+      <c r="BQ35" s="39" t="n"/>
       <c r="BR35" s="28" t="n"/>
       <c r="BS35" s="28" t="n"/>
       <c r="BT35" s="28" t="n"/>
-      <c r="BU35" s="25" t="n"/>
+      <c r="BU35" s="38" t="n"/>
       <c r="BV35" s="29" t="n">
         <v>0.97</v>
       </c>
       <c r="BW35" s="24" t="n"/>
-      <c r="BX35" s="30" t="n"/>
-      <c r="BY35" s="27" t="n"/>
+      <c r="BX35" s="40" t="n"/>
+      <c r="BY35" s="39" t="n"/>
       <c r="BZ35" s="24" t="n"/>
       <c r="CA35" s="31" t="n"/>
       <c r="CB35" s="24" t="n"/>
@@ -10297,7 +10324,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J36" s="25" t="n"/>
+      <c r="J36" s="38" t="n"/>
       <c r="K36" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -10306,7 +10333,7 @@
       <c r="L36" s="26" t="n">
         <v>135</v>
       </c>
-      <c r="M36" s="27" t="n">
+      <c r="M36" s="39" t="n">
         <v>2.35</v>
       </c>
       <c r="N36" s="28" t="n">
@@ -10348,7 +10375,7 @@
       <c r="X36" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="Y36" s="25" t="n"/>
+      <c r="Y36" s="38" t="n"/>
       <c r="Z36" s="26" t="n">
         <v>-110</v>
       </c>
@@ -10356,7 +10383,7 @@
         <v>0.523834</v>
       </c>
       <c r="AB36" s="28" t="n"/>
-      <c r="AC36" s="30" t="n">
+      <c r="AC36" s="40" t="n">
         <v>-1.25</v>
       </c>
       <c r="AD36" s="24" t="inlineStr">
@@ -10445,11 +10472,11 @@
         </is>
       </c>
       <c r="BI36" s="24" t="n"/>
-      <c r="BJ36" s="25" t="n"/>
+      <c r="BJ36" s="38" t="n"/>
       <c r="BK36" s="26" t="n">
         <v>135</v>
       </c>
-      <c r="BL36" s="27" t="n">
+      <c r="BL36" s="39" t="n">
         <v>2.35</v>
       </c>
       <c r="BM36" s="28" t="n">
@@ -10461,20 +10488,20 @@
       <c r="BO36" s="28" t="n">
         <v>0.523834</v>
       </c>
-      <c r="BP36" s="25" t="n"/>
-      <c r="BQ36" s="27" t="n">
+      <c r="BP36" s="38" t="n"/>
+      <c r="BQ36" s="39" t="n">
         <v>1.909</v>
       </c>
       <c r="BR36" s="28" t="n"/>
       <c r="BS36" s="28" t="n"/>
       <c r="BT36" s="28" t="n"/>
-      <c r="BU36" s="25" t="n"/>
+      <c r="BU36" s="38" t="n"/>
       <c r="BV36" s="29" t="n">
         <v>0.5</v>
       </c>
       <c r="BW36" s="24" t="n"/>
-      <c r="BX36" s="30" t="n"/>
-      <c r="BY36" s="27" t="n"/>
+      <c r="BX36" s="40" t="n"/>
+      <c r="BY36" s="39" t="n"/>
       <c r="BZ36" s="24" t="n"/>
       <c r="CA36" s="31" t="n"/>
       <c r="CB36" s="24" t="n"/>
@@ -10556,7 +10583,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J37" s="25" t="n"/>
+      <c r="J37" s="38" t="n"/>
       <c r="K37" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -10565,7 +10592,7 @@
       <c r="L37" s="26" t="n">
         <v>-117</v>
       </c>
-      <c r="M37" s="27" t="n">
+      <c r="M37" s="39" t="n">
         <v>1.854701</v>
       </c>
       <c r="N37" s="28" t="n">
@@ -10607,7 +10634,7 @@
       <c r="X37" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="Y37" s="25" t="n"/>
+      <c r="Y37" s="38" t="n"/>
       <c r="Z37" s="26" t="n">
         <v>-110</v>
       </c>
@@ -10615,7 +10642,7 @@
         <v>0.523834</v>
       </c>
       <c r="AB37" s="28" t="n"/>
-      <c r="AC37" s="30" t="n">
+      <c r="AC37" s="40" t="n">
         <v>1.2821</v>
       </c>
       <c r="AD37" s="24" t="inlineStr">
@@ -10704,11 +10731,11 @@
         </is>
       </c>
       <c r="BI37" s="24" t="n"/>
-      <c r="BJ37" s="25" t="n"/>
+      <c r="BJ37" s="38" t="n"/>
       <c r="BK37" s="26" t="n">
         <v>-117</v>
       </c>
-      <c r="BL37" s="27" t="n">
+      <c r="BL37" s="39" t="n">
         <v>1.854701</v>
       </c>
       <c r="BM37" s="28" t="n">
@@ -10720,20 +10747,20 @@
       <c r="BO37" s="28" t="n">
         <v>0.523834</v>
       </c>
-      <c r="BP37" s="25" t="n"/>
-      <c r="BQ37" s="27" t="n">
+      <c r="BP37" s="38" t="n"/>
+      <c r="BQ37" s="39" t="n">
         <v>1.909</v>
       </c>
       <c r="BR37" s="28" t="n"/>
       <c r="BS37" s="28" t="n"/>
       <c r="BT37" s="28" t="n"/>
-      <c r="BU37" s="25" t="n"/>
+      <c r="BU37" s="38" t="n"/>
       <c r="BV37" s="29" t="n">
         <v>0.5</v>
       </c>
       <c r="BW37" s="24" t="n"/>
-      <c r="BX37" s="30" t="n"/>
-      <c r="BY37" s="27" t="n"/>
+      <c r="BX37" s="40" t="n"/>
+      <c r="BY37" s="39" t="n"/>
       <c r="BZ37" s="24" t="n"/>
       <c r="CA37" s="31" t="n"/>
       <c r="CB37" s="24" t="n"/>
@@ -10815,7 +10842,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J38" s="25" t="n"/>
+      <c r="J38" s="38" t="n"/>
       <c r="K38" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -10824,7 +10851,7 @@
       <c r="L38" s="26" t="n">
         <v>-160</v>
       </c>
-      <c r="M38" s="27" t="n">
+      <c r="M38" s="39" t="n">
         <v>1.625</v>
       </c>
       <c r="N38" s="28" t="n">
@@ -10866,7 +10893,7 @@
       <c r="X38" s="26" t="n">
         <v>10</v>
       </c>
-      <c r="Y38" s="25" t="n"/>
+      <c r="Y38" s="38" t="n"/>
       <c r="Z38" s="26" t="n">
         <v>-110</v>
       </c>
@@ -10874,7 +10901,7 @@
         <v>0.523834</v>
       </c>
       <c r="AB38" s="28" t="n"/>
-      <c r="AC38" s="30" t="n">
+      <c r="AC38" s="40" t="n">
         <v>1.0938</v>
       </c>
       <c r="AD38" s="24" t="inlineStr">
@@ -10963,11 +10990,11 @@
         </is>
       </c>
       <c r="BI38" s="24" t="n"/>
-      <c r="BJ38" s="25" t="n"/>
+      <c r="BJ38" s="38" t="n"/>
       <c r="BK38" s="26" t="n">
         <v>-160</v>
       </c>
-      <c r="BL38" s="27" t="n">
+      <c r="BL38" s="39" t="n">
         <v>1.625</v>
       </c>
       <c r="BM38" s="28" t="n">
@@ -10979,20 +11006,20 @@
       <c r="BO38" s="28" t="n">
         <v>0.523834</v>
       </c>
-      <c r="BP38" s="25" t="n"/>
-      <c r="BQ38" s="27" t="n">
+      <c r="BP38" s="38" t="n"/>
+      <c r="BQ38" s="39" t="n">
         <v>1.909</v>
       </c>
       <c r="BR38" s="28" t="n"/>
       <c r="BS38" s="28" t="n"/>
       <c r="BT38" s="28" t="n"/>
-      <c r="BU38" s="25" t="n"/>
+      <c r="BU38" s="38" t="n"/>
       <c r="BV38" s="29" t="n">
         <v>0.59</v>
       </c>
       <c r="BW38" s="24" t="n"/>
-      <c r="BX38" s="30" t="n"/>
-      <c r="BY38" s="27" t="n"/>
+      <c r="BX38" s="40" t="n"/>
+      <c r="BY38" s="39" t="n"/>
       <c r="BZ38" s="24" t="n"/>
       <c r="CA38" s="31" t="n"/>
       <c r="CB38" s="24" t="n"/>
@@ -11074,7 +11101,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J39" s="25" t="n"/>
+      <c r="J39" s="38" t="n"/>
       <c r="K39" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -11083,7 +11110,7 @@
       <c r="L39" s="26" t="n">
         <v>102</v>
       </c>
-      <c r="M39" s="27" t="n">
+      <c r="M39" s="39" t="n">
         <v>2.02</v>
       </c>
       <c r="N39" s="28" t="n">
@@ -11125,7 +11152,7 @@
       <c r="X39" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="Y39" s="25" t="n"/>
+      <c r="Y39" s="38" t="n"/>
       <c r="Z39" s="26" t="n">
         <v>-110</v>
       </c>
@@ -11133,7 +11160,7 @@
         <v>0.523834</v>
       </c>
       <c r="AB39" s="28" t="n"/>
-      <c r="AC39" s="30" t="n">
+      <c r="AC39" s="40" t="n">
         <v>1.275</v>
       </c>
       <c r="AD39" s="24" t="inlineStr">
@@ -11222,11 +11249,11 @@
         </is>
       </c>
       <c r="BI39" s="24" t="n"/>
-      <c r="BJ39" s="25" t="n"/>
+      <c r="BJ39" s="38" t="n"/>
       <c r="BK39" s="26" t="n">
         <v>102</v>
       </c>
-      <c r="BL39" s="27" t="n">
+      <c r="BL39" s="39" t="n">
         <v>2.02</v>
       </c>
       <c r="BM39" s="28" t="n">
@@ -11238,20 +11265,20 @@
       <c r="BO39" s="28" t="n">
         <v>0.523834</v>
       </c>
-      <c r="BP39" s="25" t="n"/>
-      <c r="BQ39" s="27" t="n">
+      <c r="BP39" s="38" t="n"/>
+      <c r="BQ39" s="39" t="n">
         <v>1.909</v>
       </c>
       <c r="BR39" s="28" t="n"/>
       <c r="BS39" s="28" t="n"/>
       <c r="BT39" s="28" t="n"/>
-      <c r="BU39" s="25" t="n"/>
+      <c r="BU39" s="38" t="n"/>
       <c r="BV39" s="29" t="n">
         <v>0.5</v>
       </c>
       <c r="BW39" s="24" t="n"/>
-      <c r="BX39" s="30" t="n"/>
-      <c r="BY39" s="27" t="n"/>
+      <c r="BX39" s="40" t="n"/>
+      <c r="BY39" s="39" t="n"/>
       <c r="BZ39" s="24" t="n"/>
       <c r="CA39" s="31" t="n"/>
       <c r="CB39" s="24" t="n"/>
@@ -11333,7 +11360,7 @@
           <t>home</t>
         </is>
       </c>
-      <c r="J40" s="25" t="n"/>
+      <c r="J40" s="38" t="n"/>
       <c r="K40" s="24" t="inlineStr">
         <is>
           <t>polymarket_us</t>
@@ -11342,7 +11369,7 @@
       <c r="L40" s="26" t="n">
         <v>115</v>
       </c>
-      <c r="M40" s="27" t="n">
+      <c r="M40" s="39" t="n">
         <v>2.15</v>
       </c>
       <c r="N40" s="28" t="n">
@@ -11384,11 +11411,11 @@
       <c r="X40" s="26" t="n">
         <v>5</v>
       </c>
-      <c r="Y40" s="25" t="n"/>
+      <c r="Y40" s="38" t="n"/>
       <c r="Z40" s="26" t="n"/>
       <c r="AA40" s="28" t="n"/>
       <c r="AB40" s="28" t="n"/>
-      <c r="AC40" s="30" t="n">
+      <c r="AC40" s="40" t="n">
         <v>1.4375</v>
       </c>
       <c r="AD40" s="24" t="inlineStr">
@@ -11481,11 +11508,11 @@
         </is>
       </c>
       <c r="BI40" s="24" t="n"/>
-      <c r="BJ40" s="25" t="n"/>
+      <c r="BJ40" s="38" t="n"/>
       <c r="BK40" s="26" t="n">
         <v>115</v>
       </c>
-      <c r="BL40" s="27" t="n">
+      <c r="BL40" s="39" t="n">
         <v>2.15</v>
       </c>
       <c r="BM40" s="28" t="n">
@@ -11497,18 +11524,18 @@
       <c r="BO40" s="28" t="n">
         <v>0.523834</v>
       </c>
-      <c r="BP40" s="25" t="n"/>
-      <c r="BQ40" s="27" t="n"/>
+      <c r="BP40" s="38" t="n"/>
+      <c r="BQ40" s="39" t="n"/>
       <c r="BR40" s="28" t="n"/>
       <c r="BS40" s="28" t="n"/>
       <c r="BT40" s="28" t="n"/>
-      <c r="BU40" s="25" t="n"/>
+      <c r="BU40" s="38" t="n"/>
       <c r="BV40" s="29" t="n">
         <v>0.5</v>
       </c>
       <c r="BW40" s="24" t="n"/>
-      <c r="BX40" s="30" t="n"/>
-      <c r="BY40" s="27" t="n"/>
+      <c r="BX40" s="40" t="n"/>
+      <c r="BY40" s="39" t="n"/>
       <c r="BZ40" s="24" t="n"/>
       <c r="CA40" s="31" t="n"/>
       <c r="CB40" s="24" t="n"/>
@@ -11544,524 +11571,8 @@
       <c r="CL40" s="24" t="n"/>
       <c r="CM40" s="24" t="n"/>
     </row>
-    <row r="41" ht="36" customHeight="1">
-      <c r="A41" s="24" t="inlineStr">
-        <is>
-          <t>70aa5156d0f3460e</t>
-        </is>
-      </c>
-      <c r="B41" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-23T15:06:05.643082Z</t>
-        </is>
-      </c>
-      <c r="C41" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-23T22:00:00Z</t>
-        </is>
-      </c>
-      <c r="D41" s="24" t="inlineStr">
-        <is>
-          <t>59964</t>
-        </is>
-      </c>
-      <c r="E41" s="24" t="inlineStr">
-        <is>
-          <t>CS2</t>
-        </is>
-      </c>
-      <c r="F41" s="24" t="inlineStr">
-        <is>
-          <t>Patins da Ferrari</t>
-        </is>
-      </c>
-      <c r="G41" s="24" t="inlineStr">
-        <is>
-          <t>Isurus</t>
-        </is>
-      </c>
-      <c r="H41" s="24" t="inlineStr">
-        <is>
-          <t>moneyline</t>
-        </is>
-      </c>
-      <c r="I41" s="24" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="J41" s="25" t="n"/>
-      <c r="K41" s="24" t="inlineStr">
-        <is>
-          <t>polymarket_us</t>
-        </is>
-      </c>
-      <c r="L41" s="26" t="n">
-        <v>138</v>
-      </c>
-      <c r="M41" s="27" t="n">
-        <v>2.38</v>
-      </c>
-      <c r="N41" s="28" t="n">
-        <v>0.420168</v>
-      </c>
-      <c r="O41" s="28" t="n">
-        <v>0.502768</v>
-      </c>
-      <c r="P41" s="28" t="n"/>
-      <c r="Q41" s="28" t="n">
-        <v>0.08260000000000001</v>
-      </c>
-      <c r="R41" s="26" t="n">
-        <v>61</v>
-      </c>
-      <c r="S41" s="29" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="T41" s="24" t="inlineStr">
-        <is>
-          <t>cs2-tiered-elo-v3</t>
-        </is>
-      </c>
-      <c r="U41" s="24" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V41" s="24" t="n"/>
-      <c r="W41" s="26" t="n"/>
-      <c r="X41" s="26" t="n"/>
-      <c r="Y41" s="25" t="n"/>
-      <c r="Z41" s="26" t="n"/>
-      <c r="AA41" s="28" t="n"/>
-      <c r="AB41" s="28" t="n"/>
-      <c r="AC41" s="30" t="n"/>
-      <c r="AD41" s="24" t="n"/>
-      <c r="AE41" s="31" t="inlineStr">
-        <is>
-          <t>Neutral Elo baseline; executable ask 0.4200 (market_slug=aec-cs2-isg-pdaf-2026-07-23).</t>
-        </is>
-      </c>
-      <c r="AF41" s="31" t="inlineStr">
-        <is>
-          <t>Config-promoted esports baseline; gates enforced at log time.</t>
-        </is>
-      </c>
-      <c r="AG41" s="24" t="inlineStr">
-        <is>
-          <t>not_applicable</t>
-        </is>
-      </c>
-      <c r="AH41" s="24" t="n"/>
-      <c r="AI41" s="31" t="n"/>
-      <c r="AJ41" s="31" t="n"/>
-      <c r="AK41" s="24" t="inlineStr">
-        <is>
-          <t>model_qualified</t>
-        </is>
-      </c>
-      <c r="AL41" s="26" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM41" s="24" t="inlineStr">
-        <is>
-          <t>QUALIFIED_SHADOW_CALL</t>
-        </is>
-      </c>
-      <c r="AN41" s="24" t="inlineStr">
-        <is>
-          <t>CALL</t>
-        </is>
-      </c>
-      <c r="AO41" s="24" t="inlineStr">
-        <is>
-          <t>QUALIFIED</t>
-        </is>
-      </c>
-      <c r="AP41" s="24" t="inlineStr">
-        <is>
-          <t>Patins da Ferrari</t>
-        </is>
-      </c>
-      <c r="AQ41" s="24" t="inlineStr">
-        <is>
-          <t>Patins da Ferrari</t>
-        </is>
-      </c>
-      <c r="AR41" s="24" t="inlineStr">
-        <is>
-          <t>Patins da Ferrari</t>
-        </is>
-      </c>
-      <c r="AS41" s="24" t="inlineStr">
-        <is>
-          <t>Isurus</t>
-        </is>
-      </c>
-      <c r="AT41" s="24" t="inlineStr">
-        <is>
-          <t>Isurus</t>
-        </is>
-      </c>
-      <c r="AU41" s="24" t="inlineStr">
-        <is>
-          <t>Isurus</t>
-        </is>
-      </c>
-      <c r="AV41" s="24" t="n"/>
-      <c r="AW41" s="24" t="n"/>
-      <c r="AX41" s="24" t="inlineStr">
-        <is>
-          <t>statistical_model</t>
-        </is>
-      </c>
-      <c r="AY41" s="24" t="n"/>
-      <c r="AZ41" s="24" t="inlineStr">
-        <is>
-          <t>shadow_qualified</t>
-        </is>
-      </c>
-      <c r="BA41" s="24" t="inlineStr">
-        <is>
-          <t>48424b79d75fc1173c9c465d95feb6fc041a2ccfbc64455058b3f74905ce28d5</t>
-        </is>
-      </c>
-      <c r="BB41" s="24" t="inlineStr">
-        <is>
-          <t>neutral_elo</t>
-        </is>
-      </c>
-      <c r="BC41" s="24" t="inlineStr">
-        <is>
-          <t>cs2-tiered-elo-v3</t>
-        </is>
-      </c>
-      <c r="BD41" s="24" t="inlineStr">
-        <is>
-          <t>48424b79d75fc1173c9c465d95feb6fc041a2ccfbc64455058b3f74905ce28d5</t>
-        </is>
-      </c>
-      <c r="BE41" s="24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BF41" s="24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BG41" s="24" t="inlineStr">
-        <is>
-          <t>cs2-tiered-elo-v3</t>
-        </is>
-      </c>
-      <c r="BH41" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-23T15:05:48.220975Z</t>
-        </is>
-      </c>
-      <c r="BI41" s="24" t="inlineStr">
-        <is>
-          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
-        </is>
-      </c>
-      <c r="BJ41" s="25" t="n"/>
-      <c r="BK41" s="26" t="n">
-        <v>138</v>
-      </c>
-      <c r="BL41" s="27" t="n">
-        <v>2.38</v>
-      </c>
-      <c r="BM41" s="28" t="n">
-        <v>0.420168</v>
-      </c>
-      <c r="BN41" s="28" t="n"/>
-      <c r="BO41" s="28" t="n"/>
-      <c r="BP41" s="25" t="n"/>
-      <c r="BQ41" s="27" t="n"/>
-      <c r="BR41" s="28" t="n"/>
-      <c r="BS41" s="28" t="n"/>
-      <c r="BT41" s="28" t="n"/>
-      <c r="BU41" s="25" t="n"/>
-      <c r="BV41" s="29" t="n"/>
-      <c r="BW41" s="24" t="n"/>
-      <c r="BX41" s="30" t="n"/>
-      <c r="BY41" s="27" t="n"/>
-      <c r="BZ41" s="24" t="n"/>
-      <c r="CA41" s="31" t="n"/>
-      <c r="CB41" s="24" t="n"/>
-      <c r="CC41" s="24" t="n"/>
-      <c r="CD41" s="24" t="n"/>
-      <c r="CE41" s="24" t="n"/>
-      <c r="CF41" s="24" t="n"/>
-      <c r="CG41" s="24" t="n"/>
-      <c r="CH41" s="24" t="n"/>
-      <c r="CI41" s="24" t="n"/>
-      <c r="CJ41" s="24" t="n"/>
-      <c r="CK41" s="24" t="n"/>
-      <c r="CL41" s="24" t="n"/>
-      <c r="CM41" s="24" t="n"/>
-    </row>
-    <row r="42" ht="36" customHeight="1">
-      <c r="A42" s="24" t="inlineStr">
-        <is>
-          <t>4b4c6d29e6194fe2</t>
-        </is>
-      </c>
-      <c r="B42" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-23T15:06:41.515768Z</t>
-        </is>
-      </c>
-      <c r="C42" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-24T15:00:00Z</t>
-        </is>
-      </c>
-      <c r="D42" s="24" t="inlineStr">
-        <is>
-          <t>58399</t>
-        </is>
-      </c>
-      <c r="E42" s="24" t="inlineStr">
-        <is>
-          <t>VALORANT</t>
-        </is>
-      </c>
-      <c r="F42" s="24" t="inlineStr">
-        <is>
-          <t>BBL Esports</t>
-        </is>
-      </c>
-      <c r="G42" s="24" t="inlineStr">
-        <is>
-          <t>FUT Esports</t>
-        </is>
-      </c>
-      <c r="H42" s="24" t="inlineStr">
-        <is>
-          <t>moneyline</t>
-        </is>
-      </c>
-      <c r="I42" s="24" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="J42" s="25" t="n"/>
-      <c r="K42" s="24" t="inlineStr">
-        <is>
-          <t>polymarket_us</t>
-        </is>
-      </c>
-      <c r="L42" s="26" t="n">
-        <v>144</v>
-      </c>
-      <c r="M42" s="27" t="n">
-        <v>2.44</v>
-      </c>
-      <c r="N42" s="28" t="n">
-        <v>0.409836</v>
-      </c>
-      <c r="O42" s="28" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="P42" s="28" t="n"/>
-      <c r="Q42" s="28" t="n">
-        <v>0.09016399999999999</v>
-      </c>
-      <c r="R42" s="26" t="n">
-        <v>65</v>
-      </c>
-      <c r="S42" s="29" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="T42" s="24" t="inlineStr">
-        <is>
-          <t>valorant-tiered-elo-v3</t>
-        </is>
-      </c>
-      <c r="U42" s="24" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V42" s="24" t="n"/>
-      <c r="W42" s="26" t="n"/>
-      <c r="X42" s="26" t="n"/>
-      <c r="Y42" s="25" t="n"/>
-      <c r="Z42" s="26" t="n"/>
-      <c r="AA42" s="28" t="n"/>
-      <c r="AB42" s="28" t="n"/>
-      <c r="AC42" s="30" t="n"/>
-      <c r="AD42" s="24" t="n"/>
-      <c r="AE42" s="31" t="inlineStr">
-        <is>
-          <t>Neutral Elo baseline; executable ask 0.4100 (market_slug=aec-valorant-fut-bbl-2026-07-24).</t>
-        </is>
-      </c>
-      <c r="AF42" s="31" t="inlineStr">
-        <is>
-          <t>Config-promoted esports baseline; gates enforced at log time.</t>
-        </is>
-      </c>
-      <c r="AG42" s="24" t="inlineStr">
-        <is>
-          <t>not_applicable</t>
-        </is>
-      </c>
-      <c r="AH42" s="24" t="n"/>
-      <c r="AI42" s="31" t="n"/>
-      <c r="AJ42" s="31" t="n"/>
-      <c r="AK42" s="24" t="inlineStr">
-        <is>
-          <t>model_qualified</t>
-        </is>
-      </c>
-      <c r="AL42" s="26" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM42" s="24" t="inlineStr">
-        <is>
-          <t>QUALIFIED_SHADOW_CALL</t>
-        </is>
-      </c>
-      <c r="AN42" s="24" t="inlineStr">
-        <is>
-          <t>CALL</t>
-        </is>
-      </c>
-      <c r="AO42" s="24" t="inlineStr">
-        <is>
-          <t>QUALIFIED</t>
-        </is>
-      </c>
-      <c r="AP42" s="24" t="inlineStr">
-        <is>
-          <t>BBL Esports</t>
-        </is>
-      </c>
-      <c r="AQ42" s="24" t="inlineStr">
-        <is>
-          <t>BBL Esports</t>
-        </is>
-      </c>
-      <c r="AR42" s="24" t="inlineStr">
-        <is>
-          <t>BBL Esports</t>
-        </is>
-      </c>
-      <c r="AS42" s="24" t="inlineStr">
-        <is>
-          <t>FUT Esports</t>
-        </is>
-      </c>
-      <c r="AT42" s="24" t="inlineStr">
-        <is>
-          <t>FUT Esports</t>
-        </is>
-      </c>
-      <c r="AU42" s="24" t="inlineStr">
-        <is>
-          <t>FUT Esports</t>
-        </is>
-      </c>
-      <c r="AV42" s="24" t="n"/>
-      <c r="AW42" s="24" t="n"/>
-      <c r="AX42" s="24" t="inlineStr">
-        <is>
-          <t>statistical_model</t>
-        </is>
-      </c>
-      <c r="AY42" s="24" t="n"/>
-      <c r="AZ42" s="24" t="inlineStr">
-        <is>
-          <t>shadow_qualified</t>
-        </is>
-      </c>
-      <c r="BA42" s="24" t="inlineStr">
-        <is>
-          <t>df5a226c64918a54c70b8af3e0cd4abb6c4f42b67acb5547da319458502b0ed4</t>
-        </is>
-      </c>
-      <c r="BB42" s="24" t="inlineStr">
-        <is>
-          <t>neutral_elo</t>
-        </is>
-      </c>
-      <c r="BC42" s="24" t="inlineStr">
-        <is>
-          <t>valorant-tiered-elo-v3</t>
-        </is>
-      </c>
-      <c r="BD42" s="24" t="inlineStr">
-        <is>
-          <t>df5a226c64918a54c70b8af3e0cd4abb6c4f42b67acb5547da319458502b0ed4</t>
-        </is>
-      </c>
-      <c r="BE42" s="24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BF42" s="24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BG42" s="24" t="inlineStr">
-        <is>
-          <t>valorant-tiered-elo-v3</t>
-        </is>
-      </c>
-      <c r="BH42" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-23T15:06:37.472417Z</t>
-        </is>
-      </c>
-      <c r="BI42" s="24" t="inlineStr">
-        <is>
-          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
-        </is>
-      </c>
-      <c r="BJ42" s="25" t="n"/>
-      <c r="BK42" s="26" t="n">
-        <v>144</v>
-      </c>
-      <c r="BL42" s="27" t="n">
-        <v>2.44</v>
-      </c>
-      <c r="BM42" s="28" t="n">
-        <v>0.409836</v>
-      </c>
-      <c r="BN42" s="28" t="n"/>
-      <c r="BO42" s="28" t="n"/>
-      <c r="BP42" s="25" t="n"/>
-      <c r="BQ42" s="27" t="n"/>
-      <c r="BR42" s="28" t="n"/>
-      <c r="BS42" s="28" t="n"/>
-      <c r="BT42" s="28" t="n"/>
-      <c r="BU42" s="25" t="n"/>
-      <c r="BV42" s="29" t="n"/>
-      <c r="BW42" s="24" t="n"/>
-      <c r="BX42" s="30" t="n"/>
-      <c r="BY42" s="27" t="n"/>
-      <c r="BZ42" s="24" t="n"/>
-      <c r="CA42" s="31" t="n"/>
-      <c r="CB42" s="24" t="n"/>
-      <c r="CC42" s="24" t="n"/>
-      <c r="CD42" s="24" t="n"/>
-      <c r="CE42" s="24" t="n"/>
-      <c r="CF42" s="24" t="n"/>
-      <c r="CG42" s="24" t="n"/>
-      <c r="CH42" s="24" t="n"/>
-      <c r="CI42" s="24" t="n"/>
-      <c r="CJ42" s="24" t="n"/>
-      <c r="CK42" s="24" t="n"/>
-      <c r="CL42" s="24" t="n"/>
-      <c r="CM42" s="24" t="n"/>
-    </row>
+    <row r="41" ht="36" customHeight="1"/>
+    <row r="42" ht="36" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Add settle() correction path; re-grade postponed 7/27 Reds/Guardians pick
Add an optional correction_reason parameter to PickLedger.settle() that
lets an already-settled/voided row be re-graded when explicitly reasoned --
distinct audit event type (pick_resettled_corrected) so a corrected row is
never confused with a first-time settlement, and void_reason is cleared
since the row is no longer a push.

Real case that needed it: the 7/27 7:00 PM Reds/Guardians game (event
401816283) was postponed and never played under its own ID, so it was
correctly voided as a push. But the matchup was actually replayed same-day
as game 2 of a doubleheader (event 401816295, real final Reds 2-0), which
the original void couldn't see. Per explicit operator directive: re-graded
all 4 affected rows (main moneyline, flat moneyline/spread/total) using that
real result -- all four win.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/picks.xlsx
+++ b/data/picks.xlsx
@@ -300,8 +300,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CO27" headerRowCount="1">
-  <autoFilter ref="A1:CO27"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CO35" headerRowCount="1">
+  <autoFilter ref="A1:CO35"/>
   <tableColumns count="93">
     <tableColumn id="1" name="pick_id"/>
     <tableColumn id="2" name="created_at_utc"/>
@@ -752,19 +752,19 @@
     </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="6">
-        <f>COUNTA('Picks'!$A$2:$A$27)</f>
+        <f>COUNTA('Picks'!$A$2:$A$35)</f>
         <v/>
       </c>
       <c r="C4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$27,"open")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$35,"open")</f>
         <v/>
       </c>
       <c r="E4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$27,"settled")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$35,"settled")</f>
         <v/>
       </c>
       <c r="G4" s="6">
-        <f>IF(COUNTIFS('Picks'!$U$2:$U$27,"settled",'Picks'!$V$2:$V$27,"win")+COUNTIFS('Picks'!$U$2:$U$27,"settled",'Picks'!$V$2:$V$27,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
+        <f>IF(COUNTIFS('Picks'!$U$2:$U$35,"settled",'Picks'!$V$2:$V$35,"win")+COUNTIFS('Picks'!$U$2:$U$35,"settled",'Picks'!$V$2:$V$35,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
         <v/>
       </c>
     </row>
@@ -792,19 +792,19 @@
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="6">
-        <f>COUNTIF('Picks'!$BX$2:$BX$27,"&gt;0")</f>
+        <f>COUNTIF('Picks'!$BX$2:$BX$35,"&gt;0")</f>
         <v/>
       </c>
       <c r="C7" s="6">
-        <f>COUNTIFS('Picks'!$BX$2:$BX$27,"&gt;0",'Picks'!$V$2:$V$27,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$27,"&gt;0",'Picks'!$V$2:$V$27,"loss")</f>
+        <f>COUNTIFS('Picks'!$BX$2:$BX$35,"&gt;0",'Picks'!$V$2:$V$35,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$35,"&gt;0",'Picks'!$V$2:$V$35,"loss")</f>
         <v/>
       </c>
       <c r="E7" s="7">
-        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$27,"&gt;0",'Picks'!$V$2:$V$27,"win")/(COUNTIFS('Picks'!$BX$2:$BX$27,"&gt;0",'Picks'!$V$2:$V$27,"win")+COUNTIFS('Picks'!$BX$2:$BX$27,"&gt;0",'Picks'!$V$2:$V$27,"loss")),0)</f>
+        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$35,"&gt;0",'Picks'!$V$2:$V$35,"win")/(COUNTIFS('Picks'!$BX$2:$BX$35,"&gt;0",'Picks'!$V$2:$V$35,"win")+COUNTIFS('Picks'!$BX$2:$BX$35,"&gt;0",'Picks'!$V$2:$V$35,"loss")),0)</f>
         <v/>
       </c>
       <c r="G7" s="7">
-        <f>IFERROR(SUM('Picks'!$BY$2:$BY$27)/SUM('Picks'!$BX$2:$BX$27),0)</f>
+        <f>IFERROR(SUM('Picks'!$BY$2:$BY$35)/SUM('Picks'!$BX$2:$BX$35),0)</f>
         <v/>
       </c>
     </row>
@@ -832,19 +832,19 @@
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="8">
-        <f>SUM('Picks'!$BY$2:$BY$27)</f>
+        <f>SUM('Picks'!$BY$2:$BY$35)</f>
         <v/>
       </c>
       <c r="C10" s="9">
-        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$27,"&lt;&gt;",'Picks'!$AB$2:$AB$27),0)</f>
+        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$35,"&lt;&gt;",'Picks'!$AB$2:$AB$35),0)</f>
         <v/>
       </c>
       <c r="E10" s="6">
-        <f>COUNTIFS('Picks'!$AM$2:$AM$27,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$27,"settled")</f>
+        <f>COUNTIFS('Picks'!$AM$2:$AM$35,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$35,"settled")</f>
         <v/>
       </c>
       <c r="G10" s="8">
-        <f>SUMIFS('Picks'!$AC$2:$AC$27,'Picks'!$AM$2:$AM$27,"QUALIFIED_SHADOW_CALL")</f>
+        <f>SUMIFS('Picks'!$AC$2:$AC$35,'Picks'!$AM$2:$AM$35,"QUALIFIED_SHADOW_CALL")</f>
         <v/>
       </c>
     </row>
@@ -899,15 +899,15 @@
         </is>
       </c>
       <c r="B14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$27,$A14,'Picks'!$U$2:$U$27,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$35,$A14,'Picks'!$U$2:$U$35,"settled")</f>
         <v/>
       </c>
       <c r="C14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$27,$A14,'Picks'!$U$2:$U$27,"settled",'Picks'!$V$2:$V$27,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$35,$A14,'Picks'!$U$2:$U$35,"settled",'Picks'!$V$2:$V$35,"win")</f>
         <v/>
       </c>
       <c r="D14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$27,$A14,'Picks'!$U$2:$U$27,"settled",'Picks'!$V$2:$V$27,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$35,$A14,'Picks'!$U$2:$U$35,"settled",'Picks'!$V$2:$V$35,"loss")</f>
         <v/>
       </c>
       <c r="E14" s="14">
@@ -915,11 +915,11 @@
         <v/>
       </c>
       <c r="F14" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$27,'Picks'!$H$2:$H$27,$A14)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$35,'Picks'!$H$2:$H$35,$A14)</f>
         <v/>
       </c>
       <c r="G14" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$27,'Picks'!$H$2:$H$27,$A14,'Picks'!$U$2:$U$27,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$35,'Picks'!$H$2:$H$35,$A14,'Picks'!$U$2:$U$35,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -930,15 +930,15 @@
         </is>
       </c>
       <c r="B15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$27,$A15,'Picks'!$U$2:$U$27,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$35,$A15,'Picks'!$U$2:$U$35,"settled")</f>
         <v/>
       </c>
       <c r="C15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$27,$A15,'Picks'!$U$2:$U$27,"settled",'Picks'!$V$2:$V$27,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$35,$A15,'Picks'!$U$2:$U$35,"settled",'Picks'!$V$2:$V$35,"win")</f>
         <v/>
       </c>
       <c r="D15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$27,$A15,'Picks'!$U$2:$U$27,"settled",'Picks'!$V$2:$V$27,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$35,$A15,'Picks'!$U$2:$U$35,"settled",'Picks'!$V$2:$V$35,"loss")</f>
         <v/>
       </c>
       <c r="E15" s="19">
@@ -946,11 +946,11 @@
         <v/>
       </c>
       <c r="F15" s="20">
-        <f>SUMIFS('Picks'!$BY$2:$BY$27,'Picks'!$H$2:$H$27,$A15)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$35,'Picks'!$H$2:$H$35,$A15)</f>
         <v/>
       </c>
       <c r="G15" s="21">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$27,'Picks'!$H$2:$H$27,$A15,'Picks'!$U$2:$U$27,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$35,'Picks'!$H$2:$H$35,$A15,'Picks'!$U$2:$U$35,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -961,15 +961,15 @@
         </is>
       </c>
       <c r="B16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$27,$A16,'Picks'!$U$2:$U$27,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$35,$A16,'Picks'!$U$2:$U$35,"settled")</f>
         <v/>
       </c>
       <c r="C16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$27,$A16,'Picks'!$U$2:$U$27,"settled",'Picks'!$V$2:$V$27,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$35,$A16,'Picks'!$U$2:$U$35,"settled",'Picks'!$V$2:$V$35,"win")</f>
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$27,$A16,'Picks'!$U$2:$U$27,"settled",'Picks'!$V$2:$V$27,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$35,$A16,'Picks'!$U$2:$U$35,"settled",'Picks'!$V$2:$V$35,"loss")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -977,11 +977,11 @@
         <v/>
       </c>
       <c r="F16" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$27,'Picks'!$H$2:$H$27,$A16)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$35,'Picks'!$H$2:$H$35,$A16)</f>
         <v/>
       </c>
       <c r="G16" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$27,'Picks'!$H$2:$H$27,$A16,'Picks'!$U$2:$U$27,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$35,'Picks'!$H$2:$H$35,$A16,'Picks'!$U$2:$U$35,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -1010,7 +1010,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:CO27"/>
+  <dimension ref="A1:CO35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6144,21 +6144,25 @@
       </c>
       <c r="V17" s="24" t="inlineStr">
         <is>
-          <t>push</t>
-        </is>
-      </c>
-      <c r="W17" s="26" t="n"/>
-      <c r="X17" s="26" t="n"/>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="W17" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="X17" s="26" t="n">
+        <v>2</v>
+      </c>
       <c r="Y17" s="25" t="n"/>
       <c r="Z17" s="26" t="n"/>
       <c r="AA17" s="28" t="n"/>
       <c r="AB17" s="28" t="n"/>
       <c r="AC17" s="30" t="n">
-        <v>0</v>
+        <v>1.3605</v>
       </c>
       <c r="AD17" s="24" t="inlineStr">
         <is>
-          <t>2026-07-28T16:23:00.167734Z</t>
+          <t>2026-07-29T05:32:37.412289Z</t>
         </is>
       </c>
       <c r="AE17" s="31" t="inlineStr">
@@ -6311,11 +6315,7 @@
       <c r="BT17" s="28" t="n"/>
       <c r="BU17" s="25" t="n"/>
       <c r="BV17" s="29" t="n"/>
-      <c r="BW17" s="24" t="inlineStr">
-        <is>
-          <t>event status_postponed</t>
-        </is>
-      </c>
+      <c r="BW17" s="24" t="n"/>
       <c r="BX17" s="30" t="n"/>
       <c r="BY17" s="27" t="n"/>
       <c r="BZ17" s="24" t="n"/>
@@ -7566,12 +7566,12 @@
     <row r="22" ht="36" customHeight="1">
       <c r="A22" s="24" t="inlineStr">
         <is>
-          <t>0e49b598a1ac4abe</t>
+          <t>877fc5d38347407c</t>
         </is>
       </c>
       <c r="B22" s="24" t="inlineStr">
         <is>
-          <t>2026-07-28T16:31:42.216046Z</t>
+          <t>2026-07-28T17:26:33.566799Z</t>
         </is>
       </c>
       <c r="C22" s="24" t="inlineStr">
@@ -7644,18 +7644,38 @@
       </c>
       <c r="U22" s="24" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V22" s="24" t="n"/>
-      <c r="W22" s="26" t="n"/>
-      <c r="X22" s="26" t="n"/>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V22" s="24" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="W22" s="26" t="n">
+        <v>6</v>
+      </c>
+      <c r="X22" s="26" t="n">
+        <v>5</v>
+      </c>
       <c r="Y22" s="25" t="n"/>
-      <c r="Z22" s="26" t="n"/>
-      <c r="AA22" s="28" t="n"/>
-      <c r="AB22" s="28" t="n"/>
-      <c r="AC22" s="30" t="n"/>
-      <c r="AD22" s="24" t="n"/>
+      <c r="Z22" s="26" t="n">
+        <v>-147</v>
+      </c>
+      <c r="AA22" s="28" t="n">
+        <v>0.595</v>
+      </c>
+      <c r="AB22" s="28" t="n">
+        <v>0.07119</v>
+      </c>
+      <c r="AC22" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD22" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-28T23:36:42.481545Z</t>
+        </is>
+      </c>
       <c r="AE22" s="31" t="inlineStr">
         <is>
           <t>Learned LR call at threshold 0.5690; no Polymarket quote available — using -110 default odds. WARNING: executable_quote_missing_or_unmatched; model opinion remains visible, but this row is not executable or price-qualified. NOTE: executable_quote_missing_or_unmatched unavailable for this game — defaulted to neutral, other features used normally.</t>
@@ -7668,7 +7688,7 @@
       </c>
       <c r="AG22" s="24" t="inlineStr">
         <is>
-          <t>not_applicable</t>
+          <t>review_required</t>
         </is>
       </c>
       <c r="AH22" s="24" t="n"/>
@@ -7777,7 +7797,7 @@
       </c>
       <c r="BH22" s="24" t="inlineStr">
         <is>
-          <t>2026-07-28T16:31:42.216046Z</t>
+          <t>2026-07-28T17:26:33.566799Z</t>
         </is>
       </c>
       <c r="BI22" s="24" t="inlineStr">
@@ -7798,17 +7818,33 @@
       <c r="BN22" s="28" t="n"/>
       <c r="BO22" s="28" t="n"/>
       <c r="BP22" s="25" t="n"/>
-      <c r="BQ22" s="27" t="n"/>
-      <c r="BR22" s="28" t="n"/>
+      <c r="BQ22" s="27" t="n">
+        <v>1.680272</v>
+      </c>
+      <c r="BR22" s="28" t="n">
+        <v>0.595</v>
+      </c>
       <c r="BS22" s="28" t="n"/>
       <c r="BT22" s="28" t="n"/>
       <c r="BU22" s="25" t="n"/>
       <c r="BV22" s="29" t="n"/>
       <c r="BW22" s="24" t="n"/>
-      <c r="BX22" s="30" t="n"/>
-      <c r="BY22" s="27" t="n"/>
-      <c r="BZ22" s="24" t="n"/>
-      <c r="CA22" s="31" t="n"/>
+      <c r="BX22" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="BY22" s="27" t="n">
+        <v>-1</v>
+      </c>
+      <c r="BZ22" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-28T23:36:42.481545Z</t>
+        </is>
+      </c>
+      <c r="CA22" s="31" t="inlineStr">
+        <is>
+          <t>fixed one-unit hypothetical scoring; no real exposure or execution</t>
+        </is>
+      </c>
       <c r="CB22" s="24" t="n"/>
       <c r="CC22" s="24" t="inlineStr">
         <is>
@@ -7847,12 +7883,12 @@
     <row r="23" ht="36" customHeight="1">
       <c r="A23" s="24" t="inlineStr">
         <is>
-          <t>780be357915942de</t>
+          <t>1c9ac23f35b9411b</t>
         </is>
       </c>
       <c r="B23" s="24" t="inlineStr">
         <is>
-          <t>2026-07-28T16:31:42.216046Z</t>
+          <t>2026-07-28T20:32:52.305699Z</t>
         </is>
       </c>
       <c r="C23" s="24" t="inlineStr">
@@ -7897,20 +7933,20 @@
         </is>
       </c>
       <c r="L23" s="26" t="n">
-        <v>-138</v>
+        <v>-135</v>
       </c>
       <c r="M23" s="27" t="n">
-        <v>1.724638</v>
+        <v>1.740741</v>
       </c>
       <c r="N23" s="28" t="n">
-        <v>0.579832</v>
+        <v>0.574468</v>
       </c>
       <c r="O23" s="28" t="n">
         <v>0.742108</v>
       </c>
       <c r="P23" s="28" t="n"/>
       <c r="Q23" s="28" t="n">
-        <v>0.162276</v>
+        <v>0.16764</v>
       </c>
       <c r="R23" s="26" t="n">
         <v>100</v>
@@ -7925,21 +7961,41 @@
       </c>
       <c r="U23" s="24" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V23" s="24" t="n"/>
-      <c r="W23" s="26" t="n"/>
-      <c r="X23" s="26" t="n"/>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V23" s="24" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="W23" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="X23" s="26" t="n">
+        <v>14</v>
+      </c>
       <c r="Y23" s="25" t="n"/>
-      <c r="Z23" s="26" t="n"/>
-      <c r="AA23" s="28" t="n"/>
-      <c r="AB23" s="28" t="n"/>
-      <c r="AC23" s="30" t="n"/>
-      <c r="AD23" s="24" t="n"/>
+      <c r="Z23" s="26" t="n">
+        <v>-135</v>
+      </c>
+      <c r="AA23" s="28" t="n">
+        <v>0.575</v>
+      </c>
+      <c r="AB23" s="28" t="n">
+        <v>0.000532</v>
+      </c>
+      <c r="AC23" s="30" t="n">
+        <v>1.4815</v>
+      </c>
+      <c r="AD23" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-29T02:41:26.282792Z</t>
+        </is>
+      </c>
       <c r="AE23" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.5690; executable ask 0.5800 (aec-mlb-bal-det-2026-07-28).</t>
+          <t>Learned LR call at threshold 0.5690; executable ask 0.5750 (aec-mlb-bal-det-2026-07-28).</t>
         </is>
       </c>
       <c r="AF23" s="31" t="inlineStr">
@@ -8058,7 +8114,7 @@
       </c>
       <c r="BH23" s="24" t="inlineStr">
         <is>
-          <t>2026-07-28T16:30:28.508753Z</t>
+          <t>2026-07-28T20:32:05.666915Z</t>
         </is>
       </c>
       <c r="BI23" s="24" t="inlineStr">
@@ -8068,21 +8124,25 @@
       </c>
       <c r="BJ23" s="25" t="n"/>
       <c r="BK23" s="26" t="n">
-        <v>-138</v>
+        <v>-135</v>
       </c>
       <c r="BL23" s="27" t="n">
-        <v>1.724638</v>
+        <v>1.740741</v>
       </c>
       <c r="BM23" s="28" t="n">
-        <v>0.579832</v>
+        <v>0.574468</v>
       </c>
       <c r="BN23" s="28" t="n">
-        <v>0.577114</v>
+        <v>0.572139</v>
       </c>
       <c r="BO23" s="28" t="n"/>
       <c r="BP23" s="25" t="n"/>
-      <c r="BQ23" s="27" t="n"/>
-      <c r="BR23" s="28" t="n"/>
+      <c r="BQ23" s="27" t="n">
+        <v>1.740741</v>
+      </c>
+      <c r="BR23" s="28" t="n">
+        <v>0.575</v>
+      </c>
       <c r="BS23" s="28" t="n"/>
       <c r="BT23" s="28" t="n"/>
       <c r="BU23" s="25" t="n"/>
@@ -8126,12 +8186,12 @@
     <row r="24" ht="36" customHeight="1">
       <c r="A24" s="24" t="inlineStr">
         <is>
-          <t>093ec583554a426e</t>
+          <t>64c146d858584ab4</t>
         </is>
       </c>
       <c r="B24" s="24" t="inlineStr">
         <is>
-          <t>2026-07-28T16:31:42.216046Z</t>
+          <t>2026-07-28T20:32:52.305699Z</t>
         </is>
       </c>
       <c r="C24" s="24" t="inlineStr">
@@ -8176,23 +8236,23 @@
         </is>
       </c>
       <c r="L24" s="26" t="n">
-        <v>-104</v>
+        <v>-125</v>
       </c>
       <c r="M24" s="27" t="n">
-        <v>1.961538</v>
+        <v>1.8</v>
       </c>
       <c r="N24" s="28" t="n">
-        <v>0.509804</v>
+        <v>0.555556</v>
       </c>
       <c r="O24" s="28" t="n">
         <v>0.660233</v>
       </c>
       <c r="P24" s="28" t="n"/>
       <c r="Q24" s="28" t="n">
-        <v>0.150429</v>
+        <v>0.104677</v>
       </c>
       <c r="R24" s="26" t="n">
-        <v>96</v>
+        <v>74</v>
       </c>
       <c r="S24" s="29" t="n">
         <v>2</v>
@@ -8204,21 +8264,41 @@
       </c>
       <c r="U24" s="24" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V24" s="24" t="n"/>
-      <c r="W24" s="26" t="n"/>
-      <c r="X24" s="26" t="n"/>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V24" s="24" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="W24" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="X24" s="26" t="n">
+        <v>1</v>
+      </c>
       <c r="Y24" s="25" t="n"/>
-      <c r="Z24" s="26" t="n"/>
-      <c r="AA24" s="28" t="n"/>
-      <c r="AB24" s="28" t="n"/>
-      <c r="AC24" s="30" t="n"/>
-      <c r="AD24" s="24" t="n"/>
+      <c r="Z24" s="26" t="n">
+        <v>-125</v>
+      </c>
+      <c r="AA24" s="28" t="n">
+        <v>0.555</v>
+      </c>
+      <c r="AB24" s="28" t="n">
+        <v>-0.000556</v>
+      </c>
+      <c r="AC24" s="30" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="AD24" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-29T02:41:26.407776Z</t>
+        </is>
+      </c>
       <c r="AE24" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.5690; executable ask 0.5100 (aec-mlb-phi-mia-2026-07-28).</t>
+          <t>Learned LR call at threshold 0.5690; executable ask 0.5550 (aec-mlb-phi-mia-2026-07-28).</t>
         </is>
       </c>
       <c r="AF24" s="31" t="inlineStr">
@@ -8337,7 +8417,7 @@
       </c>
       <c r="BH24" s="24" t="inlineStr">
         <is>
-          <t>2026-07-28T16:30:29.442714Z</t>
+          <t>2026-07-28T20:32:06.628497Z</t>
         </is>
       </c>
       <c r="BI24" s="24" t="inlineStr">
@@ -8347,21 +8427,25 @@
       </c>
       <c r="BJ24" s="25" t="n"/>
       <c r="BK24" s="26" t="n">
-        <v>-104</v>
+        <v>-125</v>
       </c>
       <c r="BL24" s="27" t="n">
-        <v>1.961538</v>
+        <v>1.8</v>
       </c>
       <c r="BM24" s="28" t="n">
-        <v>0.509804</v>
+        <v>0.555556</v>
       </c>
       <c r="BN24" s="28" t="n">
-        <v>0.507463</v>
+        <v>0.552239</v>
       </c>
       <c r="BO24" s="28" t="n"/>
       <c r="BP24" s="25" t="n"/>
-      <c r="BQ24" s="27" t="n"/>
-      <c r="BR24" s="28" t="n"/>
+      <c r="BQ24" s="27" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="BR24" s="28" t="n">
+        <v>0.555</v>
+      </c>
       <c r="BS24" s="28" t="n"/>
       <c r="BT24" s="28" t="n"/>
       <c r="BU24" s="25" t="n"/>
@@ -8405,12 +8489,12 @@
     <row r="25" ht="36" customHeight="1">
       <c r="A25" s="24" t="inlineStr">
         <is>
-          <t>577a98793e874f7b</t>
+          <t>30a1c6ea7aa44b4c</t>
         </is>
       </c>
       <c r="B25" s="24" t="inlineStr">
         <is>
-          <t>2026-07-28T16:31:42.216046Z</t>
+          <t>2026-07-28T23:38:20.366083Z</t>
         </is>
       </c>
       <c r="C25" s="24" t="inlineStr">
@@ -8455,20 +8539,20 @@
         </is>
       </c>
       <c r="L25" s="26" t="n">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="M25" s="27" t="n">
-        <v>2.04</v>
+        <v>2</v>
       </c>
       <c r="N25" s="28" t="n">
-        <v>0.490196</v>
+        <v>0.5</v>
       </c>
       <c r="O25" s="28" t="n">
         <v>0.658691</v>
       </c>
       <c r="P25" s="28" t="n"/>
       <c r="Q25" s="28" t="n">
-        <v>0.168495</v>
+        <v>0.158691</v>
       </c>
       <c r="R25" s="26" t="n">
         <v>100</v>
@@ -8497,7 +8581,7 @@
       <c r="AD25" s="24" t="n"/>
       <c r="AE25" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.5690; executable ask 0.4900 (aec-mlb-chc-stl-2026-07-28).</t>
+          <t>Learned LR call at threshold 0.5690; executable ask 0.5000 (aec-mlb-chc-stl-2026-07-28).</t>
         </is>
       </c>
       <c r="AF25" s="31" t="inlineStr">
@@ -8616,7 +8700,7 @@
       </c>
       <c r="BH25" s="24" t="inlineStr">
         <is>
-          <t>2026-07-28T16:30:36.724208Z</t>
+          <t>2026-07-28T23:37:48.025116Z</t>
         </is>
       </c>
       <c r="BI25" s="24" t="inlineStr">
@@ -8626,16 +8710,16 @@
       </c>
       <c r="BJ25" s="25" t="n"/>
       <c r="BK25" s="26" t="n">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="BL25" s="27" t="n">
-        <v>2.04</v>
+        <v>2</v>
       </c>
       <c r="BM25" s="28" t="n">
-        <v>0.490196</v>
+        <v>0.5</v>
       </c>
       <c r="BN25" s="28" t="n">
-        <v>0.487562</v>
+        <v>0.497512</v>
       </c>
       <c r="BO25" s="28" t="n"/>
       <c r="BP25" s="25" t="n"/>
@@ -8684,12 +8768,12 @@
     <row r="26" ht="36" customHeight="1">
       <c r="A26" s="24" t="inlineStr">
         <is>
-          <t>fe6ee8e5eb324995</t>
+          <t>96cb1cd6e3b045e9</t>
         </is>
       </c>
       <c r="B26" s="24" t="inlineStr">
         <is>
-          <t>2026-07-28T16:31:42.216046Z</t>
+          <t>2026-07-28T23:38:20.366083Z</t>
         </is>
       </c>
       <c r="C26" s="24" t="inlineStr">
@@ -8734,23 +8818,23 @@
         </is>
       </c>
       <c r="L26" s="26" t="n">
-        <v>-194</v>
+        <v>-213</v>
       </c>
       <c r="M26" s="27" t="n">
-        <v>1.515464</v>
+        <v>1.469484</v>
       </c>
       <c r="N26" s="28" t="n">
-        <v>0.659864</v>
+        <v>0.680511</v>
       </c>
       <c r="O26" s="28" t="n">
         <v>0.7310950000000001</v>
       </c>
       <c r="P26" s="28" t="n"/>
       <c r="Q26" s="28" t="n">
-        <v>0.071231</v>
+        <v>0.050584</v>
       </c>
       <c r="R26" s="26" t="n">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="S26" s="29" t="n">
         <v>2</v>
@@ -8776,7 +8860,7 @@
       <c r="AD26" s="24" t="n"/>
       <c r="AE26" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.5690; executable ask 0.6600 (aec-mlb-col-sd-2026-07-28).</t>
+          <t>Learned LR call at threshold 0.5690; executable ask 0.6800 (aec-mlb-col-sd-2026-07-28).</t>
         </is>
       </c>
       <c r="AF26" s="31" t="inlineStr">
@@ -8895,7 +8979,7 @@
       </c>
       <c r="BH26" s="24" t="inlineStr">
         <is>
-          <t>2026-07-28T16:30:39.820826Z</t>
+          <t>2026-07-28T23:37:49.975579Z</t>
         </is>
       </c>
       <c r="BI26" s="24" t="inlineStr">
@@ -8905,16 +8989,16 @@
       </c>
       <c r="BJ26" s="25" t="n"/>
       <c r="BK26" s="26" t="n">
-        <v>-194</v>
+        <v>-213</v>
       </c>
       <c r="BL26" s="27" t="n">
-        <v>1.515464</v>
+        <v>1.469484</v>
       </c>
       <c r="BM26" s="28" t="n">
-        <v>0.659864</v>
+        <v>0.680511</v>
       </c>
       <c r="BN26" s="28" t="n">
-        <v>0.656716</v>
+        <v>0.676617</v>
       </c>
       <c r="BO26" s="28" t="n"/>
       <c r="BP26" s="25" t="n"/>
@@ -8963,22 +9047,22 @@
     <row r="27" ht="36" customHeight="1">
       <c r="A27" s="24" t="inlineStr">
         <is>
-          <t>0a69661ad0a74ee5</t>
+          <t>4530e411e7664557</t>
         </is>
       </c>
       <c r="B27" s="24" t="inlineStr">
         <is>
-          <t>2026-07-28T16:31:42.216046Z</t>
+          <t>2026-07-29T05:19:46.912744Z</t>
         </is>
       </c>
       <c r="C27" s="24" t="inlineStr">
         <is>
-          <t>2026-07-28T22:10:00-0400</t>
+          <t>2026-07-29T13:10:00-0400</t>
         </is>
       </c>
       <c r="D27" s="24" t="inlineStr">
         <is>
-          <t>401816306</t>
+          <t>401816309</t>
         </is>
       </c>
       <c r="E27" s="24" t="inlineStr">
@@ -8988,12 +9072,12 @@
       </c>
       <c r="F27" s="24" t="inlineStr">
         <is>
-          <t>Seattle Mariners</t>
+          <t>Baltimore Orioles</t>
         </is>
       </c>
       <c r="G27" s="24" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers</t>
+          <t>Detroit Tigers</t>
         </is>
       </c>
       <c r="H27" s="24" t="inlineStr">
@@ -9009,30 +9093,30 @@
       <c r="J27" s="25" t="n"/>
       <c r="K27" s="24" t="inlineStr">
         <is>
-          <t>polymarket_us</t>
+          <t>model_opinion_no_executable_quote</t>
         </is>
       </c>
       <c r="L27" s="26" t="n">
-        <v>-178</v>
+        <v>-110</v>
       </c>
       <c r="M27" s="27" t="n">
-        <v>1.561798</v>
+        <v>1.909091</v>
       </c>
       <c r="N27" s="28" t="n">
-        <v>0.640288</v>
+        <v>0.52381</v>
       </c>
       <c r="O27" s="28" t="n">
-        <v>0.690607</v>
+        <v>0.642577</v>
       </c>
       <c r="P27" s="28" t="n"/>
       <c r="Q27" s="28" t="n">
-        <v>0.050319</v>
+        <v>0.118767</v>
       </c>
       <c r="R27" s="26" t="n">
-        <v>47</v>
+        <v>79</v>
       </c>
       <c r="S27" s="29" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="T27" s="24" t="inlineStr">
         <is>
@@ -9055,7 +9139,7 @@
       <c r="AD27" s="24" t="n"/>
       <c r="AE27" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.5690; executable ask 0.6400 (aec-mlb-sea-lad-2026-07-28).</t>
+          <t>Learned LR call at threshold 0.5690; no Polymarket quote available — using -110 default odds. WARNING: executable_quote_missing_or_unmatched; model opinion remains visible, but this row is not executable or price-qualified. NOTE: executable_quote_missing_or_unmatched unavailable for this game — defaulted to neutral, other features used normally.</t>
         </is>
       </c>
       <c r="AF27" s="31" t="inlineStr">
@@ -9073,7 +9157,7 @@
       <c r="AJ27" s="31" t="n"/>
       <c r="AK27" s="24" t="inlineStr">
         <is>
-          <t>model_qualified</t>
+          <t>research_observation</t>
         </is>
       </c>
       <c r="AL27" s="26" t="n">
@@ -9081,47 +9165,47 @@
       </c>
       <c r="AM27" s="24" t="inlineStr">
         <is>
-          <t>QUALIFIED_SHADOW_CALL</t>
+          <t>RESEARCH_OBSERVATION</t>
         </is>
       </c>
       <c r="AN27" s="24" t="inlineStr">
         <is>
-          <t>CALL</t>
+          <t>NO_CALL</t>
         </is>
       </c>
       <c r="AO27" s="24" t="inlineStr">
         <is>
-          <t>QUALIFIED</t>
+          <t>NO_CALL_MARKET_UNAVAILABLE</t>
         </is>
       </c>
       <c r="AP27" s="24" t="inlineStr">
         <is>
-          <t>mlb-sea</t>
+          <t>mlb-bal</t>
         </is>
       </c>
       <c r="AQ27" s="24" t="inlineStr">
         <is>
-          <t>Seattle Mariners</t>
+          <t>Baltimore Orioles</t>
         </is>
       </c>
       <c r="AR27" s="24" t="inlineStr">
         <is>
-          <t>Seattle Mariners</t>
+          <t>Baltimore Orioles</t>
         </is>
       </c>
       <c r="AS27" s="24" t="inlineStr">
         <is>
-          <t>mlb-lad</t>
+          <t>mlb-det</t>
         </is>
       </c>
       <c r="AT27" s="24" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers</t>
+          <t>Detroit Tigers</t>
         </is>
       </c>
       <c r="AU27" s="24" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers</t>
+          <t>Detroit Tigers</t>
         </is>
       </c>
       <c r="AV27" s="24" t="n"/>
@@ -9159,7 +9243,7 @@
       </c>
       <c r="BE27" s="24" t="inlineStr">
         <is>
-          <t>c0be61a1b000c85d</t>
+          <t>737a4d0bea1eb67e</t>
         </is>
       </c>
       <c r="BF27" s="24" t="inlineStr">
@@ -9174,7 +9258,7 @@
       </c>
       <c r="BH27" s="24" t="inlineStr">
         <is>
-          <t>2026-07-28T16:30:41.425716Z</t>
+          <t>2026-07-29T05:19:46.912744Z</t>
         </is>
       </c>
       <c r="BI27" s="24" t="inlineStr">
@@ -9184,17 +9268,15 @@
       </c>
       <c r="BJ27" s="25" t="n"/>
       <c r="BK27" s="26" t="n">
-        <v>-178</v>
+        <v>-110</v>
       </c>
       <c r="BL27" s="27" t="n">
-        <v>1.561798</v>
+        <v>1.909091</v>
       </c>
       <c r="BM27" s="28" t="n">
-        <v>0.640288</v>
-      </c>
-      <c r="BN27" s="28" t="n">
-        <v>0.636816</v>
-      </c>
+        <v>0.52381</v>
+      </c>
+      <c r="BN27" s="28" t="n"/>
       <c r="BO27" s="28" t="n"/>
       <c r="BP27" s="25" t="n"/>
       <c r="BQ27" s="27" t="n"/>
@@ -9211,33 +9293,2269 @@
       <c r="CB27" s="24" t="n"/>
       <c r="CC27" s="24" t="inlineStr">
         <is>
-          <t>0.6258863376</t>
+          <t>0.5578182793</t>
         </is>
       </c>
       <c r="CD27" s="24" t="inlineStr">
         <is>
-          <t>-0.186858</t>
+          <t>-0.528912</t>
         </is>
       </c>
       <c r="CE27" s="24" t="inlineStr">
         <is>
-          <t>0.99</t>
+          <t>0.98</t>
         </is>
       </c>
       <c r="CF27" s="24" t="n"/>
       <c r="CG27" s="24" t="n"/>
       <c r="CH27" s="24" t="inlineStr">
         <is>
-          <t>-2.23</t>
-        </is>
-      </c>
-      <c r="CI27" s="24" t="n"/>
+          <t>-1.47</t>
+        </is>
+      </c>
+      <c r="CI27" s="24" t="inlineStr">
+        <is>
+          <t>executable_quote_missing_or_unmatched</t>
+        </is>
+      </c>
       <c r="CJ27" s="24" t="n"/>
       <c r="CK27" s="24" t="n"/>
       <c r="CL27" s="24" t="n"/>
       <c r="CM27" s="24" t="n"/>
       <c r="CN27" s="24" t="n"/>
       <c r="CO27" s="24" t="n"/>
+    </row>
+    <row r="28" ht="36" customHeight="1">
+      <c r="A28" s="24" t="inlineStr">
+        <is>
+          <t>a4df93341b4c4840</t>
+        </is>
+      </c>
+      <c r="B28" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-29T05:19:46.912744Z</t>
+        </is>
+      </c>
+      <c r="C28" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-29T16:10:00-0400</t>
+        </is>
+      </c>
+      <c r="D28" s="24" t="inlineStr">
+        <is>
+          <t>401816318</t>
+        </is>
+      </c>
+      <c r="E28" s="24" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="F28" s="24" t="inlineStr">
+        <is>
+          <t>Colorado Rockies</t>
+        </is>
+      </c>
+      <c r="G28" s="24" t="inlineStr">
+        <is>
+          <t>San Diego Padres</t>
+        </is>
+      </c>
+      <c r="H28" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I28" s="24" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="J28" s="25" t="n"/>
+      <c r="K28" s="24" t="inlineStr">
+        <is>
+          <t>model_opinion_no_executable_quote</t>
+        </is>
+      </c>
+      <c r="L28" s="26" t="n">
+        <v>-110</v>
+      </c>
+      <c r="M28" s="27" t="n">
+        <v>1.909091</v>
+      </c>
+      <c r="N28" s="28" t="n">
+        <v>0.52381</v>
+      </c>
+      <c r="O28" s="28" t="n">
+        <v>0.758118</v>
+      </c>
+      <c r="P28" s="28" t="n"/>
+      <c r="Q28" s="28" t="n">
+        <v>0.234308</v>
+      </c>
+      <c r="R28" s="26" t="n">
+        <v>100</v>
+      </c>
+      <c r="S28" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="T28" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v6</t>
+        </is>
+      </c>
+      <c r="U28" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V28" s="24" t="n"/>
+      <c r="W28" s="26" t="n"/>
+      <c r="X28" s="26" t="n"/>
+      <c r="Y28" s="25" t="n"/>
+      <c r="Z28" s="26" t="n"/>
+      <c r="AA28" s="28" t="n"/>
+      <c r="AB28" s="28" t="n"/>
+      <c r="AC28" s="30" t="n"/>
+      <c r="AD28" s="24" t="n"/>
+      <c r="AE28" s="31" t="inlineStr">
+        <is>
+          <t>Learned LR call at threshold 0.5690; no Polymarket quote available — using -110 default odds. WARNING: executable_quote_missing_or_unmatched; model opinion remains visible, but this row is not executable or price-qualified. NOTE: executable_quote_missing_or_unmatched unavailable for this game — defaulted to neutral, other features used normally.</t>
+        </is>
+      </c>
+      <c r="AF28" s="31" t="inlineStr">
+        <is>
+          <t>Learned model; shadow-qualified via operator override.</t>
+        </is>
+      </c>
+      <c r="AG28" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH28" s="24" t="n"/>
+      <c r="AI28" s="31" t="n"/>
+      <c r="AJ28" s="31" t="n"/>
+      <c r="AK28" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL28" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM28" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN28" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO28" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_MARKET_UNAVAILABLE</t>
+        </is>
+      </c>
+      <c r="AP28" s="24" t="inlineStr">
+        <is>
+          <t>mlb-col</t>
+        </is>
+      </c>
+      <c r="AQ28" s="24" t="inlineStr">
+        <is>
+          <t>Colorado Rockies</t>
+        </is>
+      </c>
+      <c r="AR28" s="24" t="inlineStr">
+        <is>
+          <t>Colorado Rockies</t>
+        </is>
+      </c>
+      <c r="AS28" s="24" t="inlineStr">
+        <is>
+          <t>mlb-sd</t>
+        </is>
+      </c>
+      <c r="AT28" s="24" t="inlineStr">
+        <is>
+          <t>San Diego Padres</t>
+        </is>
+      </c>
+      <c r="AU28" s="24" t="inlineStr">
+        <is>
+          <t>San Diego Padres</t>
+        </is>
+      </c>
+      <c r="AV28" s="24" t="n"/>
+      <c r="AW28" s="24" t="n"/>
+      <c r="AX28" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY28" s="24" t="n"/>
+      <c r="AZ28" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA28" s="24" t="inlineStr">
+        <is>
+          <t>0633355b1144e4205ca6d08e3f328d99cab0970358846bd77228f3bcbfcd70ee</t>
+        </is>
+      </c>
+      <c r="BB28" s="24" t="inlineStr">
+        <is>
+          <t>learned_lr</t>
+        </is>
+      </c>
+      <c r="BC28" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v6</t>
+        </is>
+      </c>
+      <c r="BD28" s="24" t="inlineStr">
+        <is>
+          <t>0633355b1144e4205ca6d08e3f328d99cab0970358846bd77228f3bcbfcd70ee</t>
+        </is>
+      </c>
+      <c r="BE28" s="24" t="inlineStr">
+        <is>
+          <t>50faeb2db498d024</t>
+        </is>
+      </c>
+      <c r="BF28" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG28" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v6</t>
+        </is>
+      </c>
+      <c r="BH28" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-29T05:19:46.912744Z</t>
+        </is>
+      </c>
+      <c r="BI28" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ28" s="25" t="n"/>
+      <c r="BK28" s="26" t="n">
+        <v>-110</v>
+      </c>
+      <c r="BL28" s="27" t="n">
+        <v>1.909091</v>
+      </c>
+      <c r="BM28" s="28" t="n">
+        <v>0.52381</v>
+      </c>
+      <c r="BN28" s="28" t="n"/>
+      <c r="BO28" s="28" t="n"/>
+      <c r="BP28" s="25" t="n"/>
+      <c r="BQ28" s="27" t="n"/>
+      <c r="BR28" s="28" t="n"/>
+      <c r="BS28" s="28" t="n"/>
+      <c r="BT28" s="28" t="n"/>
+      <c r="BU28" s="25" t="n"/>
+      <c r="BV28" s="29" t="n"/>
+      <c r="BW28" s="24" t="n"/>
+      <c r="BX28" s="30" t="n"/>
+      <c r="BY28" s="27" t="n"/>
+      <c r="BZ28" s="24" t="n"/>
+      <c r="CA28" s="31" t="n"/>
+      <c r="CB28" s="24" t="n"/>
+      <c r="CC28" s="24" t="inlineStr">
+        <is>
+          <t>0.6881581363</t>
+        </is>
+      </c>
+      <c r="CD28" s="24" t="inlineStr">
+        <is>
+          <t>2.156212</t>
+        </is>
+      </c>
+      <c r="CE28" s="24" t="inlineStr">
+        <is>
+          <t>0.95</t>
+        </is>
+      </c>
+      <c r="CF28" s="24" t="n"/>
+      <c r="CG28" s="24" t="n"/>
+      <c r="CH28" s="24" t="inlineStr">
+        <is>
+          <t>4.18</t>
+        </is>
+      </c>
+      <c r="CI28" s="24" t="inlineStr">
+        <is>
+          <t>executable_quote_missing_or_unmatched</t>
+        </is>
+      </c>
+      <c r="CJ28" s="24" t="n"/>
+      <c r="CK28" s="24" t="n"/>
+      <c r="CL28" s="24" t="n"/>
+      <c r="CM28" s="24" t="n"/>
+      <c r="CN28" s="24" t="n"/>
+      <c r="CO28" s="24" t="n"/>
+    </row>
+    <row r="29" ht="36" customHeight="1">
+      <c r="A29" s="24" t="inlineStr">
+        <is>
+          <t>ecb593c89de14d16</t>
+        </is>
+      </c>
+      <c r="B29" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-29T05:19:46.912744Z</t>
+        </is>
+      </c>
+      <c r="C29" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-29T18:40:00-0400</t>
+        </is>
+      </c>
+      <c r="D29" s="24" t="inlineStr">
+        <is>
+          <t>401816312</t>
+        </is>
+      </c>
+      <c r="E29" s="24" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="F29" s="24" t="inlineStr">
+        <is>
+          <t>Texas Rangers</t>
+        </is>
+      </c>
+      <c r="G29" s="24" t="inlineStr">
+        <is>
+          <t>Tampa Bay Rays</t>
+        </is>
+      </c>
+      <c r="H29" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I29" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J29" s="25" t="n"/>
+      <c r="K29" s="24" t="inlineStr">
+        <is>
+          <t>model_opinion_no_executable_quote</t>
+        </is>
+      </c>
+      <c r="L29" s="26" t="n">
+        <v>-110</v>
+      </c>
+      <c r="M29" s="27" t="n">
+        <v>1.909091</v>
+      </c>
+      <c r="N29" s="28" t="n">
+        <v>0.52381</v>
+      </c>
+      <c r="O29" s="28" t="n">
+        <v>0.579954</v>
+      </c>
+      <c r="P29" s="28" t="n"/>
+      <c r="Q29" s="28" t="n">
+        <v>0.056144</v>
+      </c>
+      <c r="R29" s="26" t="n">
+        <v>48</v>
+      </c>
+      <c r="S29" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="T29" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v6</t>
+        </is>
+      </c>
+      <c r="U29" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V29" s="24" t="n"/>
+      <c r="W29" s="26" t="n"/>
+      <c r="X29" s="26" t="n"/>
+      <c r="Y29" s="25" t="n"/>
+      <c r="Z29" s="26" t="n"/>
+      <c r="AA29" s="28" t="n"/>
+      <c r="AB29" s="28" t="n"/>
+      <c r="AC29" s="30" t="n"/>
+      <c r="AD29" s="24" t="n"/>
+      <c r="AE29" s="31" t="inlineStr">
+        <is>
+          <t>Learned LR call at threshold 0.5690; no Polymarket quote available — using -110 default odds. WARNING: executable_quote_missing_or_unmatched; model opinion remains visible, but this row is not executable or price-qualified. NOTE: executable_quote_missing_or_unmatched unavailable for this game — defaulted to neutral, other features used normally.</t>
+        </is>
+      </c>
+      <c r="AF29" s="31" t="inlineStr">
+        <is>
+          <t>Learned model; shadow-qualified via operator override.</t>
+        </is>
+      </c>
+      <c r="AG29" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH29" s="24" t="n"/>
+      <c r="AI29" s="31" t="n"/>
+      <c r="AJ29" s="31" t="n"/>
+      <c r="AK29" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL29" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM29" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN29" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO29" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_MARKET_UNAVAILABLE</t>
+        </is>
+      </c>
+      <c r="AP29" s="24" t="inlineStr">
+        <is>
+          <t>mlb-tex</t>
+        </is>
+      </c>
+      <c r="AQ29" s="24" t="inlineStr">
+        <is>
+          <t>Texas Rangers</t>
+        </is>
+      </c>
+      <c r="AR29" s="24" t="inlineStr">
+        <is>
+          <t>Texas Rangers</t>
+        </is>
+      </c>
+      <c r="AS29" s="24" t="inlineStr">
+        <is>
+          <t>mlb-tb</t>
+        </is>
+      </c>
+      <c r="AT29" s="24" t="inlineStr">
+        <is>
+          <t>Tampa Bay Rays</t>
+        </is>
+      </c>
+      <c r="AU29" s="24" t="inlineStr">
+        <is>
+          <t>Tampa Bay Rays</t>
+        </is>
+      </c>
+      <c r="AV29" s="24" t="n"/>
+      <c r="AW29" s="24" t="n"/>
+      <c r="AX29" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY29" s="24" t="n"/>
+      <c r="AZ29" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA29" s="24" t="inlineStr">
+        <is>
+          <t>0633355b1144e4205ca6d08e3f328d99cab0970358846bd77228f3bcbfcd70ee</t>
+        </is>
+      </c>
+      <c r="BB29" s="24" t="inlineStr">
+        <is>
+          <t>learned_lr</t>
+        </is>
+      </c>
+      <c r="BC29" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v6</t>
+        </is>
+      </c>
+      <c r="BD29" s="24" t="inlineStr">
+        <is>
+          <t>0633355b1144e4205ca6d08e3f328d99cab0970358846bd77228f3bcbfcd70ee</t>
+        </is>
+      </c>
+      <c r="BE29" s="24" t="inlineStr">
+        <is>
+          <t>f28f46ef3960c6ac</t>
+        </is>
+      </c>
+      <c r="BF29" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG29" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v6</t>
+        </is>
+      </c>
+      <c r="BH29" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-29T05:19:46.912744Z</t>
+        </is>
+      </c>
+      <c r="BI29" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ29" s="25" t="n"/>
+      <c r="BK29" s="26" t="n">
+        <v>-110</v>
+      </c>
+      <c r="BL29" s="27" t="n">
+        <v>1.909091</v>
+      </c>
+      <c r="BM29" s="28" t="n">
+        <v>0.52381</v>
+      </c>
+      <c r="BN29" s="28" t="n"/>
+      <c r="BO29" s="28" t="n"/>
+      <c r="BP29" s="25" t="n"/>
+      <c r="BQ29" s="27" t="n"/>
+      <c r="BR29" s="28" t="n"/>
+      <c r="BS29" s="28" t="n"/>
+      <c r="BT29" s="28" t="n"/>
+      <c r="BU29" s="25" t="n"/>
+      <c r="BV29" s="29" t="n"/>
+      <c r="BW29" s="24" t="n"/>
+      <c r="BX29" s="30" t="n"/>
+      <c r="BY29" s="27" t="n"/>
+      <c r="BZ29" s="24" t="n"/>
+      <c r="CA29" s="31" t="n"/>
+      <c r="CB29" s="24" t="n"/>
+      <c r="CC29" s="24" t="inlineStr">
+        <is>
+          <t>0.5812862212</t>
+        </is>
+      </c>
+      <c r="CD29" s="24" t="inlineStr">
+        <is>
+          <t>1.271016</t>
+        </is>
+      </c>
+      <c r="CE29" s="24" t="inlineStr">
+        <is>
+          <t>0.96</t>
+        </is>
+      </c>
+      <c r="CF29" s="24" t="n"/>
+      <c r="CG29" s="24" t="n"/>
+      <c r="CH29" s="24" t="inlineStr">
+        <is>
+          <t>-0.87</t>
+        </is>
+      </c>
+      <c r="CI29" s="24" t="inlineStr">
+        <is>
+          <t>executable_quote_missing_or_unmatched</t>
+        </is>
+      </c>
+      <c r="CJ29" s="24" t="n"/>
+      <c r="CK29" s="24" t="n"/>
+      <c r="CL29" s="24" t="n"/>
+      <c r="CM29" s="24" t="n"/>
+      <c r="CN29" s="24" t="n"/>
+      <c r="CO29" s="24" t="n"/>
+    </row>
+    <row r="30" ht="36" customHeight="1">
+      <c r="A30" s="24" t="inlineStr">
+        <is>
+          <t>9cf1b29591de4274</t>
+        </is>
+      </c>
+      <c r="B30" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-29T05:19:46.912744Z</t>
+        </is>
+      </c>
+      <c r="C30" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-29T19:40:00-0400</t>
+        </is>
+      </c>
+      <c r="D30" s="24" t="inlineStr">
+        <is>
+          <t>401816315</t>
+        </is>
+      </c>
+      <c r="E30" s="24" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="F30" s="24" t="inlineStr">
+        <is>
+          <t>Kansas City Royals</t>
+        </is>
+      </c>
+      <c r="G30" s="24" t="inlineStr">
+        <is>
+          <t>Minnesota Twins</t>
+        </is>
+      </c>
+      <c r="H30" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I30" s="24" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="J30" s="25" t="n"/>
+      <c r="K30" s="24" t="inlineStr">
+        <is>
+          <t>model_opinion_no_executable_quote</t>
+        </is>
+      </c>
+      <c r="L30" s="26" t="n">
+        <v>-110</v>
+      </c>
+      <c r="M30" s="27" t="n">
+        <v>1.909091</v>
+      </c>
+      <c r="N30" s="28" t="n">
+        <v>0.52381</v>
+      </c>
+      <c r="O30" s="28" t="n">
+        <v>0.6076009999999999</v>
+      </c>
+      <c r="P30" s="28" t="n"/>
+      <c r="Q30" s="28" t="n">
+        <v>0.083791</v>
+      </c>
+      <c r="R30" s="26" t="n">
+        <v>62</v>
+      </c>
+      <c r="S30" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="T30" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v6</t>
+        </is>
+      </c>
+      <c r="U30" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V30" s="24" t="n"/>
+      <c r="W30" s="26" t="n"/>
+      <c r="X30" s="26" t="n"/>
+      <c r="Y30" s="25" t="n"/>
+      <c r="Z30" s="26" t="n"/>
+      <c r="AA30" s="28" t="n"/>
+      <c r="AB30" s="28" t="n"/>
+      <c r="AC30" s="30" t="n"/>
+      <c r="AD30" s="24" t="n"/>
+      <c r="AE30" s="31" t="inlineStr">
+        <is>
+          <t>Learned LR call at threshold 0.5690; no Polymarket quote available — using -110 default odds. WARNING: executable_quote_missing_or_unmatched; model opinion remains visible, but this row is not executable or price-qualified. NOTE: executable_quote_missing_or_unmatched unavailable for this game — defaulted to neutral, other features used normally.</t>
+        </is>
+      </c>
+      <c r="AF30" s="31" t="inlineStr">
+        <is>
+          <t>Learned model; shadow-qualified via operator override.</t>
+        </is>
+      </c>
+      <c r="AG30" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH30" s="24" t="n"/>
+      <c r="AI30" s="31" t="n"/>
+      <c r="AJ30" s="31" t="n"/>
+      <c r="AK30" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL30" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM30" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN30" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO30" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_MARKET_UNAVAILABLE</t>
+        </is>
+      </c>
+      <c r="AP30" s="24" t="inlineStr">
+        <is>
+          <t>mlb-kc</t>
+        </is>
+      </c>
+      <c r="AQ30" s="24" t="inlineStr">
+        <is>
+          <t>Kansas City Royals</t>
+        </is>
+      </c>
+      <c r="AR30" s="24" t="inlineStr">
+        <is>
+          <t>Kansas City Royals</t>
+        </is>
+      </c>
+      <c r="AS30" s="24" t="inlineStr">
+        <is>
+          <t>mlb-min</t>
+        </is>
+      </c>
+      <c r="AT30" s="24" t="inlineStr">
+        <is>
+          <t>Minnesota Twins</t>
+        </is>
+      </c>
+      <c r="AU30" s="24" t="inlineStr">
+        <is>
+          <t>Minnesota Twins</t>
+        </is>
+      </c>
+      <c r="AV30" s="24" t="n"/>
+      <c r="AW30" s="24" t="n"/>
+      <c r="AX30" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY30" s="24" t="n"/>
+      <c r="AZ30" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA30" s="24" t="inlineStr">
+        <is>
+          <t>0633355b1144e4205ca6d08e3f328d99cab0970358846bd77228f3bcbfcd70ee</t>
+        </is>
+      </c>
+      <c r="BB30" s="24" t="inlineStr">
+        <is>
+          <t>learned_lr</t>
+        </is>
+      </c>
+      <c r="BC30" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v6</t>
+        </is>
+      </c>
+      <c r="BD30" s="24" t="inlineStr">
+        <is>
+          <t>0633355b1144e4205ca6d08e3f328d99cab0970358846bd77228f3bcbfcd70ee</t>
+        </is>
+      </c>
+      <c r="BE30" s="24" t="inlineStr">
+        <is>
+          <t>fd890ce0158a231f</t>
+        </is>
+      </c>
+      <c r="BF30" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG30" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v6</t>
+        </is>
+      </c>
+      <c r="BH30" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-29T05:19:46.912744Z</t>
+        </is>
+      </c>
+      <c r="BI30" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ30" s="25" t="n"/>
+      <c r="BK30" s="26" t="n">
+        <v>-110</v>
+      </c>
+      <c r="BL30" s="27" t="n">
+        <v>1.909091</v>
+      </c>
+      <c r="BM30" s="28" t="n">
+        <v>0.52381</v>
+      </c>
+      <c r="BN30" s="28" t="n"/>
+      <c r="BO30" s="28" t="n"/>
+      <c r="BP30" s="25" t="n"/>
+      <c r="BQ30" s="27" t="n"/>
+      <c r="BR30" s="28" t="n"/>
+      <c r="BS30" s="28" t="n"/>
+      <c r="BT30" s="28" t="n"/>
+      <c r="BU30" s="25" t="n"/>
+      <c r="BV30" s="29" t="n"/>
+      <c r="BW30" s="24" t="n"/>
+      <c r="BX30" s="30" t="n"/>
+      <c r="BY30" s="27" t="n"/>
+      <c r="BZ30" s="24" t="n"/>
+      <c r="CA30" s="31" t="n"/>
+      <c r="CB30" s="24" t="n"/>
+      <c r="CC30" s="24" t="inlineStr">
+        <is>
+          <t>0.5494442227</t>
+        </is>
+      </c>
+      <c r="CD30" s="24" t="inlineStr">
+        <is>
+          <t>0.040618</t>
+        </is>
+      </c>
+      <c r="CE30" s="24" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="CF30" s="24" t="n"/>
+      <c r="CG30" s="24" t="n"/>
+      <c r="CH30" s="24" t="inlineStr">
+        <is>
+          <t>1.96</t>
+        </is>
+      </c>
+      <c r="CI30" s="24" t="inlineStr">
+        <is>
+          <t>executable_quote_missing_or_unmatched</t>
+        </is>
+      </c>
+      <c r="CJ30" s="24" t="n"/>
+      <c r="CK30" s="24" t="n"/>
+      <c r="CL30" s="24" t="n"/>
+      <c r="CM30" s="24" t="n"/>
+      <c r="CN30" s="24" t="n"/>
+      <c r="CO30" s="24" t="n"/>
+    </row>
+    <row r="31" ht="36" customHeight="1">
+      <c r="A31" s="24" t="inlineStr">
+        <is>
+          <t>208e8b124e534e6b</t>
+        </is>
+      </c>
+      <c r="B31" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-29T05:19:46.912744Z</t>
+        </is>
+      </c>
+      <c r="C31" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-29T19:40:00-0400</t>
+        </is>
+      </c>
+      <c r="D31" s="24" t="inlineStr">
+        <is>
+          <t>401816316</t>
+        </is>
+      </c>
+      <c r="E31" s="24" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="F31" s="24" t="inlineStr">
+        <is>
+          <t>New York Yankees</t>
+        </is>
+      </c>
+      <c r="G31" s="24" t="inlineStr">
+        <is>
+          <t>Chicago White Sox</t>
+        </is>
+      </c>
+      <c r="H31" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I31" s="24" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="J31" s="25" t="n"/>
+      <c r="K31" s="24" t="inlineStr">
+        <is>
+          <t>model_opinion_no_executable_quote</t>
+        </is>
+      </c>
+      <c r="L31" s="26" t="n">
+        <v>-110</v>
+      </c>
+      <c r="M31" s="27" t="n">
+        <v>1.909091</v>
+      </c>
+      <c r="N31" s="28" t="n">
+        <v>0.52381</v>
+      </c>
+      <c r="O31" s="28" t="n">
+        <v>0.595337</v>
+      </c>
+      <c r="P31" s="28" t="n"/>
+      <c r="Q31" s="28" t="n">
+        <v>0.07152699999999999</v>
+      </c>
+      <c r="R31" s="26" t="n">
+        <v>56</v>
+      </c>
+      <c r="S31" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="T31" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v6</t>
+        </is>
+      </c>
+      <c r="U31" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V31" s="24" t="n"/>
+      <c r="W31" s="26" t="n"/>
+      <c r="X31" s="26" t="n"/>
+      <c r="Y31" s="25" t="n"/>
+      <c r="Z31" s="26" t="n"/>
+      <c r="AA31" s="28" t="n"/>
+      <c r="AB31" s="28" t="n"/>
+      <c r="AC31" s="30" t="n"/>
+      <c r="AD31" s="24" t="n"/>
+      <c r="AE31" s="31" t="inlineStr">
+        <is>
+          <t>Learned LR call at threshold 0.5690; no Polymarket quote available — using -110 default odds. WARNING: executable_quote_missing_or_unmatched; model opinion remains visible, but this row is not executable or price-qualified. NOTE: executable_quote_missing_or_unmatched unavailable for this game — defaulted to neutral, other features used normally.</t>
+        </is>
+      </c>
+      <c r="AF31" s="31" t="inlineStr">
+        <is>
+          <t>Learned model; shadow-qualified via operator override.</t>
+        </is>
+      </c>
+      <c r="AG31" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH31" s="24" t="n"/>
+      <c r="AI31" s="31" t="n"/>
+      <c r="AJ31" s="31" t="n"/>
+      <c r="AK31" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL31" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM31" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN31" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO31" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_MARKET_UNAVAILABLE</t>
+        </is>
+      </c>
+      <c r="AP31" s="24" t="inlineStr">
+        <is>
+          <t>mlb-nyy</t>
+        </is>
+      </c>
+      <c r="AQ31" s="24" t="inlineStr">
+        <is>
+          <t>New York Yankees</t>
+        </is>
+      </c>
+      <c r="AR31" s="24" t="inlineStr">
+        <is>
+          <t>New York Yankees</t>
+        </is>
+      </c>
+      <c r="AS31" s="24" t="inlineStr">
+        <is>
+          <t>mlb-cws</t>
+        </is>
+      </c>
+      <c r="AT31" s="24" t="inlineStr">
+        <is>
+          <t>Chicago White Sox</t>
+        </is>
+      </c>
+      <c r="AU31" s="24" t="inlineStr">
+        <is>
+          <t>Chicago White Sox</t>
+        </is>
+      </c>
+      <c r="AV31" s="24" t="n"/>
+      <c r="AW31" s="24" t="n"/>
+      <c r="AX31" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY31" s="24" t="n"/>
+      <c r="AZ31" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA31" s="24" t="inlineStr">
+        <is>
+          <t>0633355b1144e4205ca6d08e3f328d99cab0970358846bd77228f3bcbfcd70ee</t>
+        </is>
+      </c>
+      <c r="BB31" s="24" t="inlineStr">
+        <is>
+          <t>learned_lr</t>
+        </is>
+      </c>
+      <c r="BC31" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v6</t>
+        </is>
+      </c>
+      <c r="BD31" s="24" t="inlineStr">
+        <is>
+          <t>0633355b1144e4205ca6d08e3f328d99cab0970358846bd77228f3bcbfcd70ee</t>
+        </is>
+      </c>
+      <c r="BE31" s="24" t="inlineStr">
+        <is>
+          <t>9fd872ad0f3e63a3</t>
+        </is>
+      </c>
+      <c r="BF31" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG31" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v6</t>
+        </is>
+      </c>
+      <c r="BH31" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-29T05:19:46.912744Z</t>
+        </is>
+      </c>
+      <c r="BI31" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ31" s="25" t="n"/>
+      <c r="BK31" s="26" t="n">
+        <v>-110</v>
+      </c>
+      <c r="BL31" s="27" t="n">
+        <v>1.909091</v>
+      </c>
+      <c r="BM31" s="28" t="n">
+        <v>0.52381</v>
+      </c>
+      <c r="BN31" s="28" t="n"/>
+      <c r="BO31" s="28" t="n"/>
+      <c r="BP31" s="25" t="n"/>
+      <c r="BQ31" s="27" t="n"/>
+      <c r="BR31" s="28" t="n"/>
+      <c r="BS31" s="28" t="n"/>
+      <c r="BT31" s="28" t="n"/>
+      <c r="BU31" s="25" t="n"/>
+      <c r="BV31" s="29" t="n"/>
+      <c r="BW31" s="24" t="n"/>
+      <c r="BX31" s="30" t="n"/>
+      <c r="BY31" s="27" t="n"/>
+      <c r="BZ31" s="24" t="n"/>
+      <c r="CA31" s="31" t="n"/>
+      <c r="CB31" s="24" t="n"/>
+      <c r="CC31" s="24" t="inlineStr">
+        <is>
+          <t>0.4761494151</t>
+        </is>
+      </c>
+      <c r="CD31" s="24" t="inlineStr">
+        <is>
+          <t>1.500354</t>
+        </is>
+      </c>
+      <c r="CE31" s="24" t="inlineStr">
+        <is>
+          <t>0.99</t>
+        </is>
+      </c>
+      <c r="CF31" s="24" t="n"/>
+      <c r="CG31" s="24" t="n"/>
+      <c r="CH31" s="24" t="inlineStr">
+        <is>
+          <t>1.42</t>
+        </is>
+      </c>
+      <c r="CI31" s="24" t="inlineStr">
+        <is>
+          <t>executable_quote_missing_or_unmatched</t>
+        </is>
+      </c>
+      <c r="CJ31" s="24" t="n"/>
+      <c r="CK31" s="24" t="n"/>
+      <c r="CL31" s="24" t="n"/>
+      <c r="CM31" s="24" t="n"/>
+      <c r="CN31" s="24" t="n"/>
+      <c r="CO31" s="24" t="n"/>
+    </row>
+    <row r="32" ht="36" customHeight="1">
+      <c r="A32" s="24" t="inlineStr">
+        <is>
+          <t>d536ae89b2e54ac1</t>
+        </is>
+      </c>
+      <c r="B32" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-29T05:19:46.912744Z</t>
+        </is>
+      </c>
+      <c r="C32" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-29T21:40:00-0400</t>
+        </is>
+      </c>
+      <c r="D32" s="24" t="inlineStr">
+        <is>
+          <t>401816317</t>
+        </is>
+      </c>
+      <c r="E32" s="24" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="F32" s="24" t="inlineStr">
+        <is>
+          <t>Boston Red Sox</t>
+        </is>
+      </c>
+      <c r="G32" s="24" t="inlineStr">
+        <is>
+          <t>Athletics</t>
+        </is>
+      </c>
+      <c r="H32" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I32" s="24" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="J32" s="25" t="n"/>
+      <c r="K32" s="24" t="inlineStr">
+        <is>
+          <t>model_opinion_no_executable_quote</t>
+        </is>
+      </c>
+      <c r="L32" s="26" t="n">
+        <v>-110</v>
+      </c>
+      <c r="M32" s="27" t="n">
+        <v>1.909091</v>
+      </c>
+      <c r="N32" s="28" t="n">
+        <v>0.52381</v>
+      </c>
+      <c r="O32" s="28" t="n">
+        <v>0.6658500000000001</v>
+      </c>
+      <c r="P32" s="28" t="n"/>
+      <c r="Q32" s="28" t="n">
+        <v>0.14204</v>
+      </c>
+      <c r="R32" s="26" t="n">
+        <v>91</v>
+      </c>
+      <c r="S32" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="T32" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v6</t>
+        </is>
+      </c>
+      <c r="U32" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V32" s="24" t="n"/>
+      <c r="W32" s="26" t="n"/>
+      <c r="X32" s="26" t="n"/>
+      <c r="Y32" s="25" t="n"/>
+      <c r="Z32" s="26" t="n"/>
+      <c r="AA32" s="28" t="n"/>
+      <c r="AB32" s="28" t="n"/>
+      <c r="AC32" s="30" t="n"/>
+      <c r="AD32" s="24" t="n"/>
+      <c r="AE32" s="31" t="inlineStr">
+        <is>
+          <t>Learned LR call at threshold 0.5690; no Polymarket quote available — using -110 default odds. WARNING: executable_quote_missing_or_unmatched; model opinion remains visible, but this row is not executable or price-qualified. NOTE: executable_quote_missing_or_unmatched unavailable for this game — defaulted to neutral, other features used normally.</t>
+        </is>
+      </c>
+      <c r="AF32" s="31" t="inlineStr">
+        <is>
+          <t>Learned model; shadow-qualified via operator override.</t>
+        </is>
+      </c>
+      <c r="AG32" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH32" s="24" t="n"/>
+      <c r="AI32" s="31" t="n"/>
+      <c r="AJ32" s="31" t="n"/>
+      <c r="AK32" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL32" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM32" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN32" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO32" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_MARKET_UNAVAILABLE</t>
+        </is>
+      </c>
+      <c r="AP32" s="24" t="inlineStr">
+        <is>
+          <t>mlb-bos</t>
+        </is>
+      </c>
+      <c r="AQ32" s="24" t="inlineStr">
+        <is>
+          <t>Boston Red Sox</t>
+        </is>
+      </c>
+      <c r="AR32" s="24" t="inlineStr">
+        <is>
+          <t>Boston Red Sox</t>
+        </is>
+      </c>
+      <c r="AS32" s="24" t="inlineStr">
+        <is>
+          <t>mlb-ath</t>
+        </is>
+      </c>
+      <c r="AT32" s="24" t="inlineStr">
+        <is>
+          <t>Athletics</t>
+        </is>
+      </c>
+      <c r="AU32" s="24" t="inlineStr">
+        <is>
+          <t>Athletics</t>
+        </is>
+      </c>
+      <c r="AV32" s="24" t="n"/>
+      <c r="AW32" s="24" t="n"/>
+      <c r="AX32" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY32" s="24" t="n"/>
+      <c r="AZ32" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA32" s="24" t="inlineStr">
+        <is>
+          <t>0633355b1144e4205ca6d08e3f328d99cab0970358846bd77228f3bcbfcd70ee</t>
+        </is>
+      </c>
+      <c r="BB32" s="24" t="inlineStr">
+        <is>
+          <t>learned_lr</t>
+        </is>
+      </c>
+      <c r="BC32" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v6</t>
+        </is>
+      </c>
+      <c r="BD32" s="24" t="inlineStr">
+        <is>
+          <t>0633355b1144e4205ca6d08e3f328d99cab0970358846bd77228f3bcbfcd70ee</t>
+        </is>
+      </c>
+      <c r="BE32" s="24" t="inlineStr">
+        <is>
+          <t>e8772ec77b881e9a</t>
+        </is>
+      </c>
+      <c r="BF32" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG32" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v6</t>
+        </is>
+      </c>
+      <c r="BH32" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-29T05:19:46.912744Z</t>
+        </is>
+      </c>
+      <c r="BI32" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ32" s="25" t="n"/>
+      <c r="BK32" s="26" t="n">
+        <v>-110</v>
+      </c>
+      <c r="BL32" s="27" t="n">
+        <v>1.909091</v>
+      </c>
+      <c r="BM32" s="28" t="n">
+        <v>0.52381</v>
+      </c>
+      <c r="BN32" s="28" t="n"/>
+      <c r="BO32" s="28" t="n"/>
+      <c r="BP32" s="25" t="n"/>
+      <c r="BQ32" s="27" t="n"/>
+      <c r="BR32" s="28" t="n"/>
+      <c r="BS32" s="28" t="n"/>
+      <c r="BT32" s="28" t="n"/>
+      <c r="BU32" s="25" t="n"/>
+      <c r="BV32" s="29" t="n"/>
+      <c r="BW32" s="24" t="n"/>
+      <c r="BX32" s="30" t="n"/>
+      <c r="BY32" s="27" t="n"/>
+      <c r="BZ32" s="24" t="n"/>
+      <c r="CA32" s="31" t="n"/>
+      <c r="CB32" s="24" t="n"/>
+      <c r="CC32" s="24" t="inlineStr">
+        <is>
+          <t>0.3891185316</t>
+        </is>
+      </c>
+      <c r="CD32" s="24" t="inlineStr">
+        <is>
+          <t>-1.066043</t>
+        </is>
+      </c>
+      <c r="CE32" s="24" t="inlineStr">
+        <is>
+          <t>0.98</t>
+        </is>
+      </c>
+      <c r="CF32" s="24" t="n"/>
+      <c r="CG32" s="24" t="n"/>
+      <c r="CH32" s="24" t="inlineStr">
+        <is>
+          <t>2.91</t>
+        </is>
+      </c>
+      <c r="CI32" s="24" t="inlineStr">
+        <is>
+          <t>executable_quote_missing_or_unmatched</t>
+        </is>
+      </c>
+      <c r="CJ32" s="24" t="n"/>
+      <c r="CK32" s="24" t="n"/>
+      <c r="CL32" s="24" t="n"/>
+      <c r="CM32" s="24" t="n"/>
+      <c r="CN32" s="24" t="n"/>
+      <c r="CO32" s="24" t="n"/>
+    </row>
+    <row r="33" ht="36" customHeight="1">
+      <c r="A33" s="24" t="inlineStr">
+        <is>
+          <t>0b44eef52d4c4880</t>
+        </is>
+      </c>
+      <c r="B33" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-29T05:19:46.912744Z</t>
+        </is>
+      </c>
+      <c r="C33" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-29T22:10:00-0400</t>
+        </is>
+      </c>
+      <c r="D33" s="24" t="inlineStr">
+        <is>
+          <t>401816321</t>
+        </is>
+      </c>
+      <c r="E33" s="24" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="F33" s="24" t="inlineStr">
+        <is>
+          <t>Seattle Mariners</t>
+        </is>
+      </c>
+      <c r="G33" s="24" t="inlineStr">
+        <is>
+          <t>Los Angeles Dodgers</t>
+        </is>
+      </c>
+      <c r="H33" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I33" s="24" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="J33" s="25" t="n"/>
+      <c r="K33" s="24" t="inlineStr">
+        <is>
+          <t>model_opinion_no_executable_quote</t>
+        </is>
+      </c>
+      <c r="L33" s="26" t="n">
+        <v>-110</v>
+      </c>
+      <c r="M33" s="27" t="n">
+        <v>1.909091</v>
+      </c>
+      <c r="N33" s="28" t="n">
+        <v>0.52381</v>
+      </c>
+      <c r="O33" s="28" t="n">
+        <v>0.578264</v>
+      </c>
+      <c r="P33" s="28" t="n"/>
+      <c r="Q33" s="28" t="n">
+        <v>0.054454</v>
+      </c>
+      <c r="R33" s="26" t="n">
+        <v>47</v>
+      </c>
+      <c r="S33" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="T33" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v6</t>
+        </is>
+      </c>
+      <c r="U33" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V33" s="24" t="n"/>
+      <c r="W33" s="26" t="n"/>
+      <c r="X33" s="26" t="n"/>
+      <c r="Y33" s="25" t="n"/>
+      <c r="Z33" s="26" t="n"/>
+      <c r="AA33" s="28" t="n"/>
+      <c r="AB33" s="28" t="n"/>
+      <c r="AC33" s="30" t="n"/>
+      <c r="AD33" s="24" t="n"/>
+      <c r="AE33" s="31" t="inlineStr">
+        <is>
+          <t>Learned LR call at threshold 0.5690; no Polymarket quote available — using -110 default odds. WARNING: executable_quote_missing_or_unmatched; model opinion remains visible, but this row is not executable or price-qualified. NOTE: executable_quote_missing_or_unmatched unavailable for this game — defaulted to neutral, other features used normally.</t>
+        </is>
+      </c>
+      <c r="AF33" s="31" t="inlineStr">
+        <is>
+          <t>Learned model; shadow-qualified via operator override.</t>
+        </is>
+      </c>
+      <c r="AG33" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH33" s="24" t="n"/>
+      <c r="AI33" s="31" t="n"/>
+      <c r="AJ33" s="31" t="n"/>
+      <c r="AK33" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL33" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM33" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN33" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO33" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_MARKET_UNAVAILABLE</t>
+        </is>
+      </c>
+      <c r="AP33" s="24" t="inlineStr">
+        <is>
+          <t>mlb-sea</t>
+        </is>
+      </c>
+      <c r="AQ33" s="24" t="inlineStr">
+        <is>
+          <t>Seattle Mariners</t>
+        </is>
+      </c>
+      <c r="AR33" s="24" t="inlineStr">
+        <is>
+          <t>Seattle Mariners</t>
+        </is>
+      </c>
+      <c r="AS33" s="24" t="inlineStr">
+        <is>
+          <t>mlb-lad</t>
+        </is>
+      </c>
+      <c r="AT33" s="24" t="inlineStr">
+        <is>
+          <t>Los Angeles Dodgers</t>
+        </is>
+      </c>
+      <c r="AU33" s="24" t="inlineStr">
+        <is>
+          <t>Los Angeles Dodgers</t>
+        </is>
+      </c>
+      <c r="AV33" s="24" t="n"/>
+      <c r="AW33" s="24" t="n"/>
+      <c r="AX33" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY33" s="24" t="n"/>
+      <c r="AZ33" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA33" s="24" t="inlineStr">
+        <is>
+          <t>0633355b1144e4205ca6d08e3f328d99cab0970358846bd77228f3bcbfcd70ee</t>
+        </is>
+      </c>
+      <c r="BB33" s="24" t="inlineStr">
+        <is>
+          <t>learned_lr</t>
+        </is>
+      </c>
+      <c r="BC33" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v6</t>
+        </is>
+      </c>
+      <c r="BD33" s="24" t="inlineStr">
+        <is>
+          <t>0633355b1144e4205ca6d08e3f328d99cab0970358846bd77228f3bcbfcd70ee</t>
+        </is>
+      </c>
+      <c r="BE33" s="24" t="inlineStr">
+        <is>
+          <t>48afb82b2455fcbf</t>
+        </is>
+      </c>
+      <c r="BF33" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG33" s="24" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v6</t>
+        </is>
+      </c>
+      <c r="BH33" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-29T05:19:46.912744Z</t>
+        </is>
+      </c>
+      <c r="BI33" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ33" s="25" t="n"/>
+      <c r="BK33" s="26" t="n">
+        <v>-110</v>
+      </c>
+      <c r="BL33" s="27" t="n">
+        <v>1.909091</v>
+      </c>
+      <c r="BM33" s="28" t="n">
+        <v>0.52381</v>
+      </c>
+      <c r="BN33" s="28" t="n"/>
+      <c r="BO33" s="28" t="n"/>
+      <c r="BP33" s="25" t="n"/>
+      <c r="BQ33" s="27" t="n"/>
+      <c r="BR33" s="28" t="n"/>
+      <c r="BS33" s="28" t="n"/>
+      <c r="BT33" s="28" t="n"/>
+      <c r="BU33" s="25" t="n"/>
+      <c r="BV33" s="29" t="n"/>
+      <c r="BW33" s="24" t="n"/>
+      <c r="BX33" s="30" t="n"/>
+      <c r="BY33" s="27" t="n"/>
+      <c r="BZ33" s="24" t="n"/>
+      <c r="CA33" s="31" t="n"/>
+      <c r="CB33" s="24" t="n"/>
+      <c r="CC33" s="24" t="inlineStr">
+        <is>
+          <t>0.6258863376</t>
+        </is>
+      </c>
+      <c r="CD33" s="24" t="inlineStr">
+        <is>
+          <t>-0.186858</t>
+        </is>
+      </c>
+      <c r="CE33" s="24" t="inlineStr">
+        <is>
+          <t>0.99</t>
+        </is>
+      </c>
+      <c r="CF33" s="24" t="n"/>
+      <c r="CG33" s="24" t="n"/>
+      <c r="CH33" s="24" t="inlineStr">
+        <is>
+          <t>1.67</t>
+        </is>
+      </c>
+      <c r="CI33" s="24" t="inlineStr">
+        <is>
+          <t>executable_quote_missing_or_unmatched</t>
+        </is>
+      </c>
+      <c r="CJ33" s="24" t="n"/>
+      <c r="CK33" s="24" t="n"/>
+      <c r="CL33" s="24" t="n"/>
+      <c r="CM33" s="24" t="n"/>
+      <c r="CN33" s="24" t="n"/>
+      <c r="CO33" s="24" t="n"/>
+    </row>
+    <row r="34" ht="36" customHeight="1">
+      <c r="A34" s="24" t="inlineStr">
+        <is>
+          <t>383f41591c534ef5</t>
+        </is>
+      </c>
+      <c r="B34" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-29T05:19:53.585877Z</t>
+        </is>
+      </c>
+      <c r="C34" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-29T20:00:00-0400</t>
+        </is>
+      </c>
+      <c r="D34" s="24" t="inlineStr">
+        <is>
+          <t>401857097</t>
+        </is>
+      </c>
+      <c r="E34" s="24" t="inlineStr">
+        <is>
+          <t>WNBA</t>
+        </is>
+      </c>
+      <c r="F34" s="24" t="inlineStr">
+        <is>
+          <t>Atlanta Dream</t>
+        </is>
+      </c>
+      <c r="G34" s="24" t="inlineStr">
+        <is>
+          <t>Dallas Wings</t>
+        </is>
+      </c>
+      <c r="H34" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I34" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J34" s="25" t="n"/>
+      <c r="K34" s="24" t="inlineStr">
+        <is>
+          <t>model_opinion_no_executable_quote</t>
+        </is>
+      </c>
+      <c r="L34" s="26" t="n">
+        <v>-110</v>
+      </c>
+      <c r="M34" s="27" t="n">
+        <v>1.909091</v>
+      </c>
+      <c r="N34" s="28" t="n">
+        <v>0.52381</v>
+      </c>
+      <c r="O34" s="28" t="n">
+        <v>0.66476</v>
+      </c>
+      <c r="P34" s="28" t="n"/>
+      <c r="Q34" s="28" t="n">
+        <v>0.14095</v>
+      </c>
+      <c r="R34" s="26" t="n">
+        <v>90</v>
+      </c>
+      <c r="S34" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="T34" s="24" t="inlineStr">
+        <is>
+          <t>wnba-elo-trend-lr-v4</t>
+        </is>
+      </c>
+      <c r="U34" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V34" s="24" t="n"/>
+      <c r="W34" s="26" t="n"/>
+      <c r="X34" s="26" t="n"/>
+      <c r="Y34" s="25" t="n"/>
+      <c r="Z34" s="26" t="n"/>
+      <c r="AA34" s="28" t="n"/>
+      <c r="AB34" s="28" t="n"/>
+      <c r="AC34" s="30" t="n"/>
+      <c r="AD34" s="24" t="n"/>
+      <c r="AE34" s="31" t="inlineStr">
+        <is>
+          <t>Learned LR call at threshold 0.5001; no Polymarket quote available — using -110 default odds. WARNING: executable_quote_missing_or_unmatched; model opinion remains visible, but this row is not executable or price-qualified. NOTE: NO_CALL_AVAILABILITY_UNAVAILABLE, executable_quote_missing_or_unmatched unavailable for this game — defaulted to neutral, other features used normally.</t>
+        </is>
+      </c>
+      <c r="AF34" s="31" t="inlineStr">
+        <is>
+          <t>Learned model; shadow-qualified via operator override.</t>
+        </is>
+      </c>
+      <c r="AG34" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH34" s="24" t="n"/>
+      <c r="AI34" s="31" t="n"/>
+      <c r="AJ34" s="31" t="n"/>
+      <c r="AK34" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL34" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM34" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN34" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO34" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_MARKET_UNAVAILABLE</t>
+        </is>
+      </c>
+      <c r="AP34" s="24" t="inlineStr">
+        <is>
+          <t>wnba-atl</t>
+        </is>
+      </c>
+      <c r="AQ34" s="24" t="inlineStr">
+        <is>
+          <t>Atlanta Dream</t>
+        </is>
+      </c>
+      <c r="AR34" s="24" t="inlineStr">
+        <is>
+          <t>Atlanta Dream</t>
+        </is>
+      </c>
+      <c r="AS34" s="24" t="inlineStr">
+        <is>
+          <t>wnba-dal</t>
+        </is>
+      </c>
+      <c r="AT34" s="24" t="inlineStr">
+        <is>
+          <t>Dallas Wings</t>
+        </is>
+      </c>
+      <c r="AU34" s="24" t="inlineStr">
+        <is>
+          <t>Dallas Wings</t>
+        </is>
+      </c>
+      <c r="AV34" s="24" t="n"/>
+      <c r="AW34" s="24" t="n"/>
+      <c r="AX34" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY34" s="24" t="n"/>
+      <c r="AZ34" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA34" s="24" t="inlineStr">
+        <is>
+          <t>7afd5274214b58b7efd7f7febc7be3ab33b92351cda5cc6403c0a39faea0cc8c</t>
+        </is>
+      </c>
+      <c r="BB34" s="24" t="inlineStr">
+        <is>
+          <t>learned_lr</t>
+        </is>
+      </c>
+      <c r="BC34" s="24" t="inlineStr">
+        <is>
+          <t>wnba-elo-trend-lr-v4</t>
+        </is>
+      </c>
+      <c r="BD34" s="24" t="inlineStr">
+        <is>
+          <t>7afd5274214b58b7efd7f7febc7be3ab33b92351cda5cc6403c0a39faea0cc8c</t>
+        </is>
+      </c>
+      <c r="BE34" s="24" t="inlineStr">
+        <is>
+          <t>f25936b561e6d355</t>
+        </is>
+      </c>
+      <c r="BF34" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG34" s="24" t="inlineStr">
+        <is>
+          <t>wnba-elo-trend-lr-v4</t>
+        </is>
+      </c>
+      <c r="BH34" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-29T05:19:53.585877Z</t>
+        </is>
+      </c>
+      <c r="BI34" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ34" s="25" t="n"/>
+      <c r="BK34" s="26" t="n">
+        <v>-110</v>
+      </c>
+      <c r="BL34" s="27" t="n">
+        <v>1.909091</v>
+      </c>
+      <c r="BM34" s="28" t="n">
+        <v>0.52381</v>
+      </c>
+      <c r="BN34" s="28" t="n"/>
+      <c r="BO34" s="28" t="n"/>
+      <c r="BP34" s="25" t="n"/>
+      <c r="BQ34" s="27" t="n"/>
+      <c r="BR34" s="28" t="n"/>
+      <c r="BS34" s="28" t="n"/>
+      <c r="BT34" s="28" t="n"/>
+      <c r="BU34" s="25" t="n"/>
+      <c r="BV34" s="29" t="n"/>
+      <c r="BW34" s="24" t="n"/>
+      <c r="BX34" s="30" t="n"/>
+      <c r="BY34" s="27" t="n"/>
+      <c r="BZ34" s="24" t="n"/>
+      <c r="CA34" s="31" t="n"/>
+      <c r="CB34" s="24" t="n"/>
+      <c r="CC34" s="24" t="inlineStr">
+        <is>
+          <t>0.7229749194</t>
+        </is>
+      </c>
+      <c r="CD34" s="24" t="inlineStr">
+        <is>
+          <t>-2.425932</t>
+        </is>
+      </c>
+      <c r="CE34" s="24" t="n"/>
+      <c r="CF34" s="24" t="n"/>
+      <c r="CG34" s="24" t="n"/>
+      <c r="CH34" s="24" t="n"/>
+      <c r="CI34" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_AVAILABILITY_UNAVAILABLE,executable_quote_missing_or_unmatched</t>
+        </is>
+      </c>
+      <c r="CJ34" s="24" t="n"/>
+      <c r="CK34" s="24" t="n"/>
+      <c r="CL34" s="24" t="n"/>
+      <c r="CM34" s="24" t="n"/>
+      <c r="CN34" s="24" t="n"/>
+      <c r="CO34" s="24" t="n"/>
+    </row>
+    <row r="35" ht="36" customHeight="1">
+      <c r="A35" s="24" t="inlineStr">
+        <is>
+          <t>df3672f8d9724eb8</t>
+        </is>
+      </c>
+      <c r="B35" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-29T05:19:53.585877Z</t>
+        </is>
+      </c>
+      <c r="C35" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-29T22:00:00-0400</t>
+        </is>
+      </c>
+      <c r="D35" s="24" t="inlineStr">
+        <is>
+          <t>401857098</t>
+        </is>
+      </c>
+      <c r="E35" s="24" t="inlineStr">
+        <is>
+          <t>WNBA</t>
+        </is>
+      </c>
+      <c r="F35" s="24" t="inlineStr">
+        <is>
+          <t>Golden State Valkyries</t>
+        </is>
+      </c>
+      <c r="G35" s="24" t="inlineStr">
+        <is>
+          <t>Phoenix Mercury</t>
+        </is>
+      </c>
+      <c r="H35" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I35" s="24" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="J35" s="25" t="n"/>
+      <c r="K35" s="24" t="inlineStr">
+        <is>
+          <t>model_opinion_no_executable_quote</t>
+        </is>
+      </c>
+      <c r="L35" s="26" t="n">
+        <v>-110</v>
+      </c>
+      <c r="M35" s="27" t="n">
+        <v>1.909091</v>
+      </c>
+      <c r="N35" s="28" t="n">
+        <v>0.52381</v>
+      </c>
+      <c r="O35" s="28" t="n">
+        <v>0.7219989999999999</v>
+      </c>
+      <c r="P35" s="28" t="n"/>
+      <c r="Q35" s="28" t="n">
+        <v>0.198189</v>
+      </c>
+      <c r="R35" s="26" t="n">
+        <v>100</v>
+      </c>
+      <c r="S35" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="T35" s="24" t="inlineStr">
+        <is>
+          <t>wnba-elo-trend-lr-v4</t>
+        </is>
+      </c>
+      <c r="U35" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V35" s="24" t="n"/>
+      <c r="W35" s="26" t="n"/>
+      <c r="X35" s="26" t="n"/>
+      <c r="Y35" s="25" t="n"/>
+      <c r="Z35" s="26" t="n"/>
+      <c r="AA35" s="28" t="n"/>
+      <c r="AB35" s="28" t="n"/>
+      <c r="AC35" s="30" t="n"/>
+      <c r="AD35" s="24" t="n"/>
+      <c r="AE35" s="31" t="inlineStr">
+        <is>
+          <t>Learned LR call at threshold 0.5001; no Polymarket quote available — using -110 default odds. WARNING: executable_quote_missing_or_unmatched; model opinion remains visible, but this row is not executable or price-qualified. NOTE: NO_CALL_AVAILABILITY_UNAVAILABLE, executable_quote_missing_or_unmatched unavailable for this game — defaulted to neutral, other features used normally.</t>
+        </is>
+      </c>
+      <c r="AF35" s="31" t="inlineStr">
+        <is>
+          <t>Learned model; shadow-qualified via operator override.</t>
+        </is>
+      </c>
+      <c r="AG35" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH35" s="24" t="n"/>
+      <c r="AI35" s="31" t="n"/>
+      <c r="AJ35" s="31" t="n"/>
+      <c r="AK35" s="24" t="inlineStr">
+        <is>
+          <t>research_observation</t>
+        </is>
+      </c>
+      <c r="AL35" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM35" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN35" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL</t>
+        </is>
+      </c>
+      <c r="AO35" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_MARKET_UNAVAILABLE</t>
+        </is>
+      </c>
+      <c r="AP35" s="24" t="inlineStr">
+        <is>
+          <t>wnba-gsv</t>
+        </is>
+      </c>
+      <c r="AQ35" s="24" t="inlineStr">
+        <is>
+          <t>Golden State Valkyries</t>
+        </is>
+      </c>
+      <c r="AR35" s="24" t="inlineStr">
+        <is>
+          <t>Golden State Valkyries</t>
+        </is>
+      </c>
+      <c r="AS35" s="24" t="inlineStr">
+        <is>
+          <t>wnba-phx</t>
+        </is>
+      </c>
+      <c r="AT35" s="24" t="inlineStr">
+        <is>
+          <t>Phoenix Mercury</t>
+        </is>
+      </c>
+      <c r="AU35" s="24" t="inlineStr">
+        <is>
+          <t>Phoenix Mercury</t>
+        </is>
+      </c>
+      <c r="AV35" s="24" t="n"/>
+      <c r="AW35" s="24" t="n"/>
+      <c r="AX35" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY35" s="24" t="n"/>
+      <c r="AZ35" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA35" s="24" t="inlineStr">
+        <is>
+          <t>7afd5274214b58b7efd7f7febc7be3ab33b92351cda5cc6403c0a39faea0cc8c</t>
+        </is>
+      </c>
+      <c r="BB35" s="24" t="inlineStr">
+        <is>
+          <t>learned_lr</t>
+        </is>
+      </c>
+      <c r="BC35" s="24" t="inlineStr">
+        <is>
+          <t>wnba-elo-trend-lr-v4</t>
+        </is>
+      </c>
+      <c r="BD35" s="24" t="inlineStr">
+        <is>
+          <t>7afd5274214b58b7efd7f7febc7be3ab33b92351cda5cc6403c0a39faea0cc8c</t>
+        </is>
+      </c>
+      <c r="BE35" s="24" t="inlineStr">
+        <is>
+          <t>5ba5847b783e4237</t>
+        </is>
+      </c>
+      <c r="BF35" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG35" s="24" t="inlineStr">
+        <is>
+          <t>wnba-elo-trend-lr-v4</t>
+        </is>
+      </c>
+      <c r="BH35" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-29T05:19:53.585877Z</t>
+        </is>
+      </c>
+      <c r="BI35" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ35" s="25" t="n"/>
+      <c r="BK35" s="26" t="n">
+        <v>-110</v>
+      </c>
+      <c r="BL35" s="27" t="n">
+        <v>1.909091</v>
+      </c>
+      <c r="BM35" s="28" t="n">
+        <v>0.52381</v>
+      </c>
+      <c r="BN35" s="28" t="n"/>
+      <c r="BO35" s="28" t="n"/>
+      <c r="BP35" s="25" t="n"/>
+      <c r="BQ35" s="27" t="n"/>
+      <c r="BR35" s="28" t="n"/>
+      <c r="BS35" s="28" t="n"/>
+      <c r="BT35" s="28" t="n"/>
+      <c r="BU35" s="25" t="n"/>
+      <c r="BV35" s="29" t="n"/>
+      <c r="BW35" s="24" t="n"/>
+      <c r="BX35" s="30" t="n"/>
+      <c r="BY35" s="27" t="n"/>
+      <c r="BZ35" s="24" t="n"/>
+      <c r="CA35" s="31" t="n"/>
+      <c r="CB35" s="24" t="n"/>
+      <c r="CC35" s="24" t="inlineStr">
+        <is>
+          <t>0.1902656067</t>
+        </is>
+      </c>
+      <c r="CD35" s="24" t="inlineStr">
+        <is>
+          <t>-0.399848</t>
+        </is>
+      </c>
+      <c r="CE35" s="24" t="n"/>
+      <c r="CF35" s="24" t="n"/>
+      <c r="CG35" s="24" t="n"/>
+      <c r="CH35" s="24" t="n"/>
+      <c r="CI35" s="24" t="inlineStr">
+        <is>
+          <t>NO_CALL_AVAILABILITY_UNAVAILABLE,executable_quote_missing_or_unmatched</t>
+        </is>
+      </c>
+      <c r="CJ35" s="24" t="n"/>
+      <c r="CK35" s="24" t="n"/>
+      <c r="CL35" s="24" t="n"/>
+      <c r="CM35" s="24" t="n"/>
+      <c r="CN35" s="24" t="n"/>
+      <c r="CO35" s="24" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Real daily forecast run under the fixed MLB model + baseline refresh state
Final end-to-end verification: real daily run logged 4 MLB moneyline and 22
MLB totals/spread picks under the newly-fixed/recalibrated Measured Edge
model, with the baseline-refresh throttle correctly skipping (ran manually
minutes earlier). 478/478 tests pass, verify-chain clean.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/picks.xlsx
+++ b/data/picks.xlsx
@@ -300,8 +300,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CO35" headerRowCount="1">
-  <autoFilter ref="A1:CO35"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CO32" headerRowCount="1">
+  <autoFilter ref="A1:CO32"/>
   <tableColumns count="93">
     <tableColumn id="1" name="pick_id"/>
     <tableColumn id="2" name="created_at_utc"/>
@@ -752,19 +752,19 @@
     </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="6">
-        <f>COUNTA('Picks'!$A$2:$A$35)</f>
+        <f>COUNTA('Picks'!$A$2:$A$32)</f>
         <v/>
       </c>
       <c r="C4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$35,"open")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$32,"open")</f>
         <v/>
       </c>
       <c r="E4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$35,"settled")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$32,"settled")</f>
         <v/>
       </c>
       <c r="G4" s="6">
-        <f>IF(COUNTIFS('Picks'!$U$2:$U$35,"settled",'Picks'!$V$2:$V$35,"win")+COUNTIFS('Picks'!$U$2:$U$35,"settled",'Picks'!$V$2:$V$35,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
+        <f>IF(COUNTIFS('Picks'!$U$2:$U$32,"settled",'Picks'!$V$2:$V$32,"win")+COUNTIFS('Picks'!$U$2:$U$32,"settled",'Picks'!$V$2:$V$32,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
         <v/>
       </c>
     </row>
@@ -792,19 +792,19 @@
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="6">
-        <f>COUNTIF('Picks'!$BX$2:$BX$35,"&gt;0")</f>
+        <f>COUNTIF('Picks'!$BX$2:$BX$32,"&gt;0")</f>
         <v/>
       </c>
       <c r="C7" s="6">
-        <f>COUNTIFS('Picks'!$BX$2:$BX$35,"&gt;0",'Picks'!$V$2:$V$35,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$35,"&gt;0",'Picks'!$V$2:$V$35,"loss")</f>
+        <f>COUNTIFS('Picks'!$BX$2:$BX$32,"&gt;0",'Picks'!$V$2:$V$32,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$32,"&gt;0",'Picks'!$V$2:$V$32,"loss")</f>
         <v/>
       </c>
       <c r="E7" s="7">
-        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$35,"&gt;0",'Picks'!$V$2:$V$35,"win")/(COUNTIFS('Picks'!$BX$2:$BX$35,"&gt;0",'Picks'!$V$2:$V$35,"win")+COUNTIFS('Picks'!$BX$2:$BX$35,"&gt;0",'Picks'!$V$2:$V$35,"loss")),0)</f>
+        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$32,"&gt;0",'Picks'!$V$2:$V$32,"win")/(COUNTIFS('Picks'!$BX$2:$BX$32,"&gt;0",'Picks'!$V$2:$V$32,"win")+COUNTIFS('Picks'!$BX$2:$BX$32,"&gt;0",'Picks'!$V$2:$V$32,"loss")),0)</f>
         <v/>
       </c>
       <c r="G7" s="7">
-        <f>IFERROR(SUM('Picks'!$BY$2:$BY$35)/SUM('Picks'!$BX$2:$BX$35),0)</f>
+        <f>IFERROR(SUM('Picks'!$BY$2:$BY$32)/SUM('Picks'!$BX$2:$BX$32),0)</f>
         <v/>
       </c>
     </row>
@@ -832,19 +832,19 @@
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="8">
-        <f>SUM('Picks'!$BY$2:$BY$35)</f>
+        <f>SUM('Picks'!$BY$2:$BY$32)</f>
         <v/>
       </c>
       <c r="C10" s="9">
-        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$35,"&lt;&gt;",'Picks'!$AB$2:$AB$35),0)</f>
+        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$32,"&lt;&gt;",'Picks'!$AB$2:$AB$32),0)</f>
         <v/>
       </c>
       <c r="E10" s="6">
-        <f>COUNTIFS('Picks'!$AM$2:$AM$35,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$35,"settled")</f>
+        <f>COUNTIFS('Picks'!$AM$2:$AM$32,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$32,"settled")</f>
         <v/>
       </c>
       <c r="G10" s="8">
-        <f>SUMIFS('Picks'!$AC$2:$AC$35,'Picks'!$AM$2:$AM$35,"QUALIFIED_SHADOW_CALL")</f>
+        <f>SUMIFS('Picks'!$AC$2:$AC$32,'Picks'!$AM$2:$AM$32,"QUALIFIED_SHADOW_CALL")</f>
         <v/>
       </c>
     </row>
@@ -899,15 +899,15 @@
         </is>
       </c>
       <c r="B14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$35,$A14,'Picks'!$U$2:$U$35,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$32,$A14,'Picks'!$U$2:$U$32,"settled")</f>
         <v/>
       </c>
       <c r="C14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$35,$A14,'Picks'!$U$2:$U$35,"settled",'Picks'!$V$2:$V$35,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$32,$A14,'Picks'!$U$2:$U$32,"settled",'Picks'!$V$2:$V$32,"win")</f>
         <v/>
       </c>
       <c r="D14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$35,$A14,'Picks'!$U$2:$U$35,"settled",'Picks'!$V$2:$V$35,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$32,$A14,'Picks'!$U$2:$U$32,"settled",'Picks'!$V$2:$V$32,"loss")</f>
         <v/>
       </c>
       <c r="E14" s="14">
@@ -915,11 +915,11 @@
         <v/>
       </c>
       <c r="F14" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$35,'Picks'!$H$2:$H$35,$A14)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$32,'Picks'!$H$2:$H$32,$A14)</f>
         <v/>
       </c>
       <c r="G14" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$35,'Picks'!$H$2:$H$35,$A14,'Picks'!$U$2:$U$35,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$32,'Picks'!$H$2:$H$32,$A14,'Picks'!$U$2:$U$32,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -930,15 +930,15 @@
         </is>
       </c>
       <c r="B15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$35,$A15,'Picks'!$U$2:$U$35,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$32,$A15,'Picks'!$U$2:$U$32,"settled")</f>
         <v/>
       </c>
       <c r="C15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$35,$A15,'Picks'!$U$2:$U$35,"settled",'Picks'!$V$2:$V$35,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$32,$A15,'Picks'!$U$2:$U$32,"settled",'Picks'!$V$2:$V$32,"win")</f>
         <v/>
       </c>
       <c r="D15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$35,$A15,'Picks'!$U$2:$U$35,"settled",'Picks'!$V$2:$V$35,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$32,$A15,'Picks'!$U$2:$U$32,"settled",'Picks'!$V$2:$V$32,"loss")</f>
         <v/>
       </c>
       <c r="E15" s="19">
@@ -946,11 +946,11 @@
         <v/>
       </c>
       <c r="F15" s="20">
-        <f>SUMIFS('Picks'!$BY$2:$BY$35,'Picks'!$H$2:$H$35,$A15)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$32,'Picks'!$H$2:$H$32,$A15)</f>
         <v/>
       </c>
       <c r="G15" s="21">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$35,'Picks'!$H$2:$H$35,$A15,'Picks'!$U$2:$U$35,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$32,'Picks'!$H$2:$H$32,$A15,'Picks'!$U$2:$U$32,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -961,15 +961,15 @@
         </is>
       </c>
       <c r="B16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$35,$A16,'Picks'!$U$2:$U$35,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$32,$A16,'Picks'!$U$2:$U$32,"settled")</f>
         <v/>
       </c>
       <c r="C16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$35,$A16,'Picks'!$U$2:$U$35,"settled",'Picks'!$V$2:$V$35,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$32,$A16,'Picks'!$U$2:$U$32,"settled",'Picks'!$V$2:$V$32,"win")</f>
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$35,$A16,'Picks'!$U$2:$U$35,"settled",'Picks'!$V$2:$V$35,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$32,$A16,'Picks'!$U$2:$U$32,"settled",'Picks'!$V$2:$V$32,"loss")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -977,11 +977,11 @@
         <v/>
       </c>
       <c r="F16" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$35,'Picks'!$H$2:$H$35,$A16)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$32,'Picks'!$H$2:$H$32,$A16)</f>
         <v/>
       </c>
       <c r="G16" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$35,'Picks'!$H$2:$H$35,$A16,'Picks'!$U$2:$U$35,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$32,'Picks'!$H$2:$H$32,$A16,'Picks'!$U$2:$U$32,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -1010,7 +1010,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:CO35"/>
+  <dimension ref="A1:CO32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -8567,18 +8567,38 @@
       </c>
       <c r="U25" s="24" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V25" s="24" t="n"/>
-      <c r="W25" s="26" t="n"/>
-      <c r="X25" s="26" t="n"/>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V25" s="24" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="W25" s="26" t="n">
+        <v>10</v>
+      </c>
+      <c r="X25" s="26" t="n">
+        <v>2</v>
+      </c>
       <c r="Y25" s="25" t="n"/>
-      <c r="Z25" s="26" t="n"/>
-      <c r="AA25" s="28" t="n"/>
-      <c r="AB25" s="28" t="n"/>
-      <c r="AC25" s="30" t="n"/>
-      <c r="AD25" s="24" t="n"/>
+      <c r="Z25" s="26" t="n">
+        <v>100</v>
+      </c>
+      <c r="AA25" s="28" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AB25" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC25" s="30" t="n">
+        <v>-2</v>
+      </c>
+      <c r="AD25" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-29T05:44:51.428715Z</t>
+        </is>
+      </c>
       <c r="AE25" s="31" t="inlineStr">
         <is>
           <t>Learned LR call at threshold 0.5690; executable ask 0.5000 (aec-mlb-chc-stl-2026-07-28).</t>
@@ -8591,7 +8611,7 @@
       </c>
       <c r="AG25" s="24" t="inlineStr">
         <is>
-          <t>not_applicable</t>
+          <t>review_required</t>
         </is>
       </c>
       <c r="AH25" s="24" t="n"/>
@@ -8723,8 +8743,12 @@
       </c>
       <c r="BO25" s="28" t="n"/>
       <c r="BP25" s="25" t="n"/>
-      <c r="BQ25" s="27" t="n"/>
-      <c r="BR25" s="28" t="n"/>
+      <c r="BQ25" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="BR25" s="28" t="n">
+        <v>0.5</v>
+      </c>
       <c r="BS25" s="28" t="n"/>
       <c r="BT25" s="28" t="n"/>
       <c r="BU25" s="25" t="n"/>
@@ -8846,18 +8870,38 @@
       </c>
       <c r="U26" s="24" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V26" s="24" t="n"/>
-      <c r="W26" s="26" t="n"/>
-      <c r="X26" s="26" t="n"/>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V26" s="24" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="W26" s="26" t="n">
+        <v>7</v>
+      </c>
+      <c r="X26" s="26" t="n">
+        <v>8</v>
+      </c>
       <c r="Y26" s="25" t="n"/>
-      <c r="Z26" s="26" t="n"/>
-      <c r="AA26" s="28" t="n"/>
-      <c r="AB26" s="28" t="n"/>
-      <c r="AC26" s="30" t="n"/>
-      <c r="AD26" s="24" t="n"/>
+      <c r="Z26" s="26" t="n">
+        <v>-213</v>
+      </c>
+      <c r="AA26" s="28" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="AB26" s="28" t="n">
+        <v>-0.000511</v>
+      </c>
+      <c r="AC26" s="30" t="n">
+        <v>0.9389999999999999</v>
+      </c>
+      <c r="AD26" s="24" t="inlineStr">
+        <is>
+          <t>2026-07-29T05:44:51.563870Z</t>
+        </is>
+      </c>
       <c r="AE26" s="31" t="inlineStr">
         <is>
           <t>Learned LR call at threshold 0.5690; executable ask 0.6800 (aec-mlb-col-sd-2026-07-28).</t>
@@ -9002,8 +9046,12 @@
       </c>
       <c r="BO26" s="28" t="n"/>
       <c r="BP26" s="25" t="n"/>
-      <c r="BQ26" s="27" t="n"/>
-      <c r="BR26" s="28" t="n"/>
+      <c r="BQ26" s="27" t="n">
+        <v>1.469484</v>
+      </c>
+      <c r="BR26" s="28" t="n">
+        <v>0.68</v>
+      </c>
       <c r="BS26" s="28" t="n"/>
       <c r="BT26" s="28" t="n"/>
       <c r="BU26" s="25" t="n"/>
@@ -9047,37 +9095,37 @@
     <row r="27" ht="36" customHeight="1">
       <c r="A27" s="24" t="inlineStr">
         <is>
-          <t>4530e411e7664557</t>
+          <t>4afbde32316849b6</t>
         </is>
       </c>
       <c r="B27" s="24" t="inlineStr">
         <is>
-          <t>2026-07-29T05:19:46.912744Z</t>
+          <t>2026-07-29T17:43:50.913671Z</t>
         </is>
       </c>
       <c r="C27" s="24" t="inlineStr">
         <is>
-          <t>2026-07-29T13:10:00-0400</t>
+          <t>2026-07-29T20:00:00-0400</t>
         </is>
       </c>
       <c r="D27" s="24" t="inlineStr">
         <is>
-          <t>401816309</t>
+          <t>401857097</t>
         </is>
       </c>
       <c r="E27" s="24" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>WNBA</t>
         </is>
       </c>
       <c r="F27" s="24" t="inlineStr">
         <is>
-          <t>Baltimore Orioles</t>
+          <t>Atlanta Dream</t>
         </is>
       </c>
       <c r="G27" s="24" t="inlineStr">
         <is>
-          <t>Detroit Tigers</t>
+          <t>Dallas Wings</t>
         </is>
       </c>
       <c r="H27" s="24" t="inlineStr">
@@ -9093,34 +9141,34 @@
       <c r="J27" s="25" t="n"/>
       <c r="K27" s="24" t="inlineStr">
         <is>
-          <t>model_opinion_no_executable_quote</t>
+          <t>polymarket_us</t>
         </is>
       </c>
       <c r="L27" s="26" t="n">
-        <v>-110</v>
+        <v>108</v>
       </c>
       <c r="M27" s="27" t="n">
-        <v>1.909091</v>
+        <v>2.08</v>
       </c>
       <c r="N27" s="28" t="n">
-        <v>0.52381</v>
+        <v>0.480769</v>
       </c>
       <c r="O27" s="28" t="n">
-        <v>0.642577</v>
+        <v>0.66476</v>
       </c>
       <c r="P27" s="28" t="n"/>
       <c r="Q27" s="28" t="n">
-        <v>0.118767</v>
+        <v>0.183991</v>
       </c>
       <c r="R27" s="26" t="n">
-        <v>79</v>
+        <v>100</v>
       </c>
       <c r="S27" s="29" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="T27" s="24" t="inlineStr">
         <is>
-          <t>mlb-elo-trend-lr-v6</t>
+          <t>wnba-elo-trend-lr-v4</t>
         </is>
       </c>
       <c r="U27" s="24" t="inlineStr">
@@ -9139,7 +9187,7 @@
       <c r="AD27" s="24" t="n"/>
       <c r="AE27" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.5690; no Polymarket quote available — using -110 default odds. WARNING: executable_quote_missing_or_unmatched; model opinion remains visible, but this row is not executable or price-qualified. NOTE: executable_quote_missing_or_unmatched unavailable for this game — defaulted to neutral, other features used normally.</t>
+          <t>Learned LR call at threshold 0.5001; executable ask 0.4800 (aec-wnba-atl-dal-2026-07-29). NOTE: wnba_availability_source_conflict unavailable for this game — defaulted to neutral, other features used normally.</t>
         </is>
       </c>
       <c r="AF27" s="31" t="inlineStr">
@@ -9157,7 +9205,7 @@
       <c r="AJ27" s="31" t="n"/>
       <c r="AK27" s="24" t="inlineStr">
         <is>
-          <t>research_observation</t>
+          <t>model_qualified</t>
         </is>
       </c>
       <c r="AL27" s="26" t="n">
@@ -9165,47 +9213,47 @@
       </c>
       <c r="AM27" s="24" t="inlineStr">
         <is>
-          <t>RESEARCH_OBSERVATION</t>
+          <t>QUALIFIED_SHADOW_CALL</t>
         </is>
       </c>
       <c r="AN27" s="24" t="inlineStr">
         <is>
-          <t>NO_CALL</t>
+          <t>CALL</t>
         </is>
       </c>
       <c r="AO27" s="24" t="inlineStr">
         <is>
-          <t>NO_CALL_MARKET_UNAVAILABLE</t>
+          <t>QUALIFIED</t>
         </is>
       </c>
       <c r="AP27" s="24" t="inlineStr">
         <is>
-          <t>mlb-bal</t>
+          <t>wnba-atl</t>
         </is>
       </c>
       <c r="AQ27" s="24" t="inlineStr">
         <is>
-          <t>Baltimore Orioles</t>
+          <t>Atlanta Dream</t>
         </is>
       </c>
       <c r="AR27" s="24" t="inlineStr">
         <is>
-          <t>Baltimore Orioles</t>
+          <t>Atlanta Dream</t>
         </is>
       </c>
       <c r="AS27" s="24" t="inlineStr">
         <is>
-          <t>mlb-det</t>
+          <t>wnba-dal</t>
         </is>
       </c>
       <c r="AT27" s="24" t="inlineStr">
         <is>
-          <t>Detroit Tigers</t>
+          <t>Dallas Wings</t>
         </is>
       </c>
       <c r="AU27" s="24" t="inlineStr">
         <is>
-          <t>Detroit Tigers</t>
+          <t>Dallas Wings</t>
         </is>
       </c>
       <c r="AV27" s="24" t="n"/>
@@ -9223,7 +9271,7 @@
       </c>
       <c r="BA27" s="24" t="inlineStr">
         <is>
-          <t>0633355b1144e4205ca6d08e3f328d99cab0970358846bd77228f3bcbfcd70ee</t>
+          <t>7afd5274214b58b7efd7f7febc7be3ab33b92351cda5cc6403c0a39faea0cc8c</t>
         </is>
       </c>
       <c r="BB27" s="24" t="inlineStr">
@@ -9233,17 +9281,17 @@
       </c>
       <c r="BC27" s="24" t="inlineStr">
         <is>
-          <t>mlb-elo-trend-lr-v6</t>
+          <t>wnba-elo-trend-lr-v4</t>
         </is>
       </c>
       <c r="BD27" s="24" t="inlineStr">
         <is>
-          <t>0633355b1144e4205ca6d08e3f328d99cab0970358846bd77228f3bcbfcd70ee</t>
+          <t>7afd5274214b58b7efd7f7febc7be3ab33b92351cda5cc6403c0a39faea0cc8c</t>
         </is>
       </c>
       <c r="BE27" s="24" t="inlineStr">
         <is>
-          <t>737a4d0bea1eb67e</t>
+          <t>f25936b561e6d355</t>
         </is>
       </c>
       <c r="BF27" s="24" t="inlineStr">
@@ -9253,12 +9301,12 @@
       </c>
       <c r="BG27" s="24" t="inlineStr">
         <is>
-          <t>mlb-elo-trend-lr-v6</t>
+          <t>wnba-elo-trend-lr-v4</t>
         </is>
       </c>
       <c r="BH27" s="24" t="inlineStr">
         <is>
-          <t>2026-07-29T05:19:46.912744Z</t>
+          <t>2026-07-29T17:43:12.551208Z</t>
         </is>
       </c>
       <c r="BI27" s="24" t="inlineStr">
@@ -9268,15 +9316,17 @@
       </c>
       <c r="BJ27" s="25" t="n"/>
       <c r="BK27" s="26" t="n">
-        <v>-110</v>
+        <v>108</v>
       </c>
       <c r="BL27" s="27" t="n">
-        <v>1.909091</v>
+        <v>2.08</v>
       </c>
       <c r="BM27" s="28" t="n">
-        <v>0.52381</v>
-      </c>
-      <c r="BN27" s="28" t="n"/>
+        <v>0.480769</v>
+      </c>
+      <c r="BN27" s="28" t="n">
+        <v>0.475248</v>
+      </c>
       <c r="BO27" s="28" t="n"/>
       <c r="BP27" s="25" t="n"/>
       <c r="BQ27" s="27" t="n"/>
@@ -9293,29 +9343,21 @@
       <c r="CB27" s="24" t="n"/>
       <c r="CC27" s="24" t="inlineStr">
         <is>
-          <t>0.5578182793</t>
+          <t>0.7229749194</t>
         </is>
       </c>
       <c r="CD27" s="24" t="inlineStr">
         <is>
-          <t>-0.528912</t>
-        </is>
-      </c>
-      <c r="CE27" s="24" t="inlineStr">
-        <is>
-          <t>0.98</t>
-        </is>
-      </c>
+          <t>-2.425932</t>
+        </is>
+      </c>
+      <c r="CE27" s="24" t="n"/>
       <c r="CF27" s="24" t="n"/>
       <c r="CG27" s="24" t="n"/>
-      <c r="CH27" s="24" t="inlineStr">
-        <is>
-          <t>-1.47</t>
-        </is>
-      </c>
+      <c r="CH27" s="24" t="n"/>
       <c r="CI27" s="24" t="inlineStr">
         <is>
-          <t>executable_quote_missing_or_unmatched</t>
+          <t>wnba_availability_source_conflict</t>
         </is>
       </c>
       <c r="CJ27" s="24" t="n"/>
@@ -9328,37 +9370,37 @@
     <row r="28" ht="36" customHeight="1">
       <c r="A28" s="24" t="inlineStr">
         <is>
-          <t>a4df93341b4c4840</t>
+          <t>0591969d590f4c4c</t>
         </is>
       </c>
       <c r="B28" s="24" t="inlineStr">
         <is>
-          <t>2026-07-29T05:19:46.912744Z</t>
+          <t>2026-07-29T17:43:50.913671Z</t>
         </is>
       </c>
       <c r="C28" s="24" t="inlineStr">
         <is>
-          <t>2026-07-29T16:10:00-0400</t>
+          <t>2026-07-29T22:00:00-0400</t>
         </is>
       </c>
       <c r="D28" s="24" t="inlineStr">
         <is>
-          <t>401816318</t>
+          <t>401857098</t>
         </is>
       </c>
       <c r="E28" s="24" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>WNBA</t>
         </is>
       </c>
       <c r="F28" s="24" t="inlineStr">
         <is>
-          <t>Colorado Rockies</t>
+          <t>Golden State Valkyries</t>
         </is>
       </c>
       <c r="G28" s="24" t="inlineStr">
         <is>
-          <t>San Diego Padres</t>
+          <t>Phoenix Mercury</t>
         </is>
       </c>
       <c r="H28" s="24" t="inlineStr">
@@ -9374,34 +9416,34 @@
       <c r="J28" s="25" t="n"/>
       <c r="K28" s="24" t="inlineStr">
         <is>
-          <t>model_opinion_no_executable_quote</t>
+          <t>polymarket_us</t>
         </is>
       </c>
       <c r="L28" s="26" t="n">
-        <v>-110</v>
+        <v>-156</v>
       </c>
       <c r="M28" s="27" t="n">
-        <v>1.909091</v>
+        <v>1.641026</v>
       </c>
       <c r="N28" s="28" t="n">
-        <v>0.52381</v>
+        <v>0.609375</v>
       </c>
       <c r="O28" s="28" t="n">
-        <v>0.758118</v>
+        <v>0.7219989999999999</v>
       </c>
       <c r="P28" s="28" t="n"/>
       <c r="Q28" s="28" t="n">
-        <v>0.234308</v>
+        <v>0.112624</v>
       </c>
       <c r="R28" s="26" t="n">
-        <v>100</v>
+        <v>79</v>
       </c>
       <c r="S28" s="29" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="T28" s="24" t="inlineStr">
         <is>
-          <t>mlb-elo-trend-lr-v6</t>
+          <t>wnba-elo-trend-lr-v4</t>
         </is>
       </c>
       <c r="U28" s="24" t="inlineStr">
@@ -9420,7 +9462,7 @@
       <c r="AD28" s="24" t="n"/>
       <c r="AE28" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.5690; no Polymarket quote available — using -110 default odds. WARNING: executable_quote_missing_or_unmatched; model opinion remains visible, but this row is not executable or price-qualified. NOTE: executable_quote_missing_or_unmatched unavailable for this game — defaulted to neutral, other features used normally.</t>
+          <t>Learned LR call at threshold 0.5001; executable ask 0.6100 (aec-wnba-gsv-phx-2026-07-29).</t>
         </is>
       </c>
       <c r="AF28" s="31" t="inlineStr">
@@ -9438,7 +9480,7 @@
       <c r="AJ28" s="31" t="n"/>
       <c r="AK28" s="24" t="inlineStr">
         <is>
-          <t>research_observation</t>
+          <t>model_qualified</t>
         </is>
       </c>
       <c r="AL28" s="26" t="n">
@@ -9446,47 +9488,47 @@
       </c>
       <c r="AM28" s="24" t="inlineStr">
         <is>
-          <t>RESEARCH_OBSERVATION</t>
+          <t>QUALIFIED_SHADOW_CALL</t>
         </is>
       </c>
       <c r="AN28" s="24" t="inlineStr">
         <is>
-          <t>NO_CALL</t>
+          <t>CALL</t>
         </is>
       </c>
       <c r="AO28" s="24" t="inlineStr">
         <is>
-          <t>NO_CALL_MARKET_UNAVAILABLE</t>
+          <t>QUALIFIED</t>
         </is>
       </c>
       <c r="AP28" s="24" t="inlineStr">
         <is>
-          <t>mlb-col</t>
+          <t>wnba-gsv</t>
         </is>
       </c>
       <c r="AQ28" s="24" t="inlineStr">
         <is>
-          <t>Colorado Rockies</t>
+          <t>Golden State Valkyries</t>
         </is>
       </c>
       <c r="AR28" s="24" t="inlineStr">
         <is>
-          <t>Colorado Rockies</t>
+          <t>Golden State Valkyries</t>
         </is>
       </c>
       <c r="AS28" s="24" t="inlineStr">
         <is>
-          <t>mlb-sd</t>
+          <t>wnba-phx</t>
         </is>
       </c>
       <c r="AT28" s="24" t="inlineStr">
         <is>
-          <t>San Diego Padres</t>
+          <t>Phoenix Mercury</t>
         </is>
       </c>
       <c r="AU28" s="24" t="inlineStr">
         <is>
-          <t>San Diego Padres</t>
+          <t>Phoenix Mercury</t>
         </is>
       </c>
       <c r="AV28" s="24" t="n"/>
@@ -9504,7 +9546,7 @@
       </c>
       <c r="BA28" s="24" t="inlineStr">
         <is>
-          <t>0633355b1144e4205ca6d08e3f328d99cab0970358846bd77228f3bcbfcd70ee</t>
+          <t>7afd5274214b58b7efd7f7febc7be3ab33b92351cda5cc6403c0a39faea0cc8c</t>
         </is>
       </c>
       <c r="BB28" s="24" t="inlineStr">
@@ -9514,17 +9556,17 @@
       </c>
       <c r="BC28" s="24" t="inlineStr">
         <is>
-          <t>mlb-elo-trend-lr-v6</t>
+          <t>wnba-elo-trend-lr-v4</t>
         </is>
       </c>
       <c r="BD28" s="24" t="inlineStr">
         <is>
-          <t>0633355b1144e4205ca6d08e3f328d99cab0970358846bd77228f3bcbfcd70ee</t>
+          <t>7afd5274214b58b7efd7f7febc7be3ab33b92351cda5cc6403c0a39faea0cc8c</t>
         </is>
       </c>
       <c r="BE28" s="24" t="inlineStr">
         <is>
-          <t>50faeb2db498d024</t>
+          <t>5ba5847b783e4237</t>
         </is>
       </c>
       <c r="BF28" s="24" t="inlineStr">
@@ -9534,12 +9576,12 @@
       </c>
       <c r="BG28" s="24" t="inlineStr">
         <is>
-          <t>mlb-elo-trend-lr-v6</t>
+          <t>wnba-elo-trend-lr-v4</t>
         </is>
       </c>
       <c r="BH28" s="24" t="inlineStr">
         <is>
-          <t>2026-07-29T05:19:46.912744Z</t>
+          <t>2026-07-29T17:43:13.575889Z</t>
         </is>
       </c>
       <c r="BI28" s="24" t="inlineStr">
@@ -9549,15 +9591,17 @@
       </c>
       <c r="BJ28" s="25" t="n"/>
       <c r="BK28" s="26" t="n">
-        <v>-110</v>
+        <v>-156</v>
       </c>
       <c r="BL28" s="27" t="n">
-        <v>1.909091</v>
+        <v>1.641026</v>
       </c>
       <c r="BM28" s="28" t="n">
-        <v>0.52381</v>
-      </c>
-      <c r="BN28" s="28" t="n"/>
+        <v>0.609375</v>
+      </c>
+      <c r="BN28" s="28" t="n">
+        <v>0.6039600000000001</v>
+      </c>
       <c r="BO28" s="28" t="n"/>
       <c r="BP28" s="25" t="n"/>
       <c r="BQ28" s="27" t="n"/>
@@ -9574,31 +9618,19 @@
       <c r="CB28" s="24" t="n"/>
       <c r="CC28" s="24" t="inlineStr">
         <is>
-          <t>0.6881581363</t>
+          <t>0.1902656067</t>
         </is>
       </c>
       <c r="CD28" s="24" t="inlineStr">
         <is>
-          <t>2.156212</t>
-        </is>
-      </c>
-      <c r="CE28" s="24" t="inlineStr">
-        <is>
-          <t>0.95</t>
-        </is>
-      </c>
+          <t>-0.399848</t>
+        </is>
+      </c>
+      <c r="CE28" s="24" t="n"/>
       <c r="CF28" s="24" t="n"/>
       <c r="CG28" s="24" t="n"/>
-      <c r="CH28" s="24" t="inlineStr">
-        <is>
-          <t>4.18</t>
-        </is>
-      </c>
-      <c r="CI28" s="24" t="inlineStr">
-        <is>
-          <t>executable_quote_missing_or_unmatched</t>
-        </is>
-      </c>
+      <c r="CH28" s="24" t="n"/>
+      <c r="CI28" s="24" t="n"/>
       <c r="CJ28" s="24" t="n"/>
       <c r="CK28" s="24" t="n"/>
       <c r="CL28" s="24" t="n"/>
@@ -9609,22 +9641,22 @@
     <row r="29" ht="36" customHeight="1">
       <c r="A29" s="24" t="inlineStr">
         <is>
-          <t>ecb593c89de14d16</t>
+          <t>0f9039db899f4453</t>
         </is>
       </c>
       <c r="B29" s="24" t="inlineStr">
         <is>
-          <t>2026-07-29T05:19:46.912744Z</t>
+          <t>2026-07-29T17:43:50.913671Z</t>
         </is>
       </c>
       <c r="C29" s="24" t="inlineStr">
         <is>
-          <t>2026-07-29T18:40:00-0400</t>
+          <t>2026-07-29T16:10:00-0400</t>
         </is>
       </c>
       <c r="D29" s="24" t="inlineStr">
         <is>
-          <t>401816312</t>
+          <t>401816318</t>
         </is>
       </c>
       <c r="E29" s="24" t="inlineStr">
@@ -9634,12 +9666,12 @@
       </c>
       <c r="F29" s="24" t="inlineStr">
         <is>
-          <t>Texas Rangers</t>
+          <t>Colorado Rockies</t>
         </is>
       </c>
       <c r="G29" s="24" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays</t>
+          <t>San Diego Padres</t>
         </is>
       </c>
       <c r="H29" s="24" t="inlineStr">
@@ -9649,36 +9681,36 @@
       </c>
       <c r="I29" s="24" t="inlineStr">
         <is>
-          <t>home</t>
+          <t>away</t>
         </is>
       </c>
       <c r="J29" s="25" t="n"/>
       <c r="K29" s="24" t="inlineStr">
         <is>
-          <t>model_opinion_no_executable_quote</t>
+          <t>polymarket_us</t>
         </is>
       </c>
       <c r="L29" s="26" t="n">
-        <v>-110</v>
+        <v>150</v>
       </c>
       <c r="M29" s="27" t="n">
-        <v>1.909091</v>
+        <v>2.5</v>
       </c>
       <c r="N29" s="28" t="n">
-        <v>0.52381</v>
+        <v>0.4</v>
       </c>
       <c r="O29" s="28" t="n">
-        <v>0.579954</v>
+        <v>0.65394</v>
       </c>
       <c r="P29" s="28" t="n"/>
       <c r="Q29" s="28" t="n">
-        <v>0.056144</v>
+        <v>0.25394</v>
       </c>
       <c r="R29" s="26" t="n">
-        <v>48</v>
+        <v>100</v>
       </c>
       <c r="S29" s="29" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="T29" s="24" t="inlineStr">
         <is>
@@ -9701,7 +9733,7 @@
       <c r="AD29" s="24" t="n"/>
       <c r="AE29" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.5690; no Polymarket quote available — using -110 default odds. WARNING: executable_quote_missing_or_unmatched; model opinion remains visible, but this row is not executable or price-qualified. NOTE: executable_quote_missing_or_unmatched unavailable for this game — defaulted to neutral, other features used normally.</t>
+          <t>Learned LR call at threshold 0.5690; executable ask 0.4000 (aec-mlb-col-sd-2026-07-29).</t>
         </is>
       </c>
       <c r="AF29" s="31" t="inlineStr">
@@ -9719,7 +9751,7 @@
       <c r="AJ29" s="31" t="n"/>
       <c r="AK29" s="24" t="inlineStr">
         <is>
-          <t>research_observation</t>
+          <t>model_qualified</t>
         </is>
       </c>
       <c r="AL29" s="26" t="n">
@@ -9727,47 +9759,47 @@
       </c>
       <c r="AM29" s="24" t="inlineStr">
         <is>
-          <t>RESEARCH_OBSERVATION</t>
+          <t>QUALIFIED_SHADOW_CALL</t>
         </is>
       </c>
       <c r="AN29" s="24" t="inlineStr">
         <is>
-          <t>NO_CALL</t>
+          <t>CALL</t>
         </is>
       </c>
       <c r="AO29" s="24" t="inlineStr">
         <is>
-          <t>NO_CALL_MARKET_UNAVAILABLE</t>
+          <t>QUALIFIED</t>
         </is>
       </c>
       <c r="AP29" s="24" t="inlineStr">
         <is>
-          <t>mlb-tex</t>
+          <t>mlb-col</t>
         </is>
       </c>
       <c r="AQ29" s="24" t="inlineStr">
         <is>
-          <t>Texas Rangers</t>
+          <t>Colorado Rockies</t>
         </is>
       </c>
       <c r="AR29" s="24" t="inlineStr">
         <is>
-          <t>Texas Rangers</t>
+          <t>Colorado Rockies</t>
         </is>
       </c>
       <c r="AS29" s="24" t="inlineStr">
         <is>
-          <t>mlb-tb</t>
+          <t>mlb-sd</t>
         </is>
       </c>
       <c r="AT29" s="24" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays</t>
+          <t>San Diego Padres</t>
         </is>
       </c>
       <c r="AU29" s="24" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays</t>
+          <t>San Diego Padres</t>
         </is>
       </c>
       <c r="AV29" s="24" t="n"/>
@@ -9805,7 +9837,7 @@
       </c>
       <c r="BE29" s="24" t="inlineStr">
         <is>
-          <t>f28f46ef3960c6ac</t>
+          <t>60e5bdc1faca52aa</t>
         </is>
       </c>
       <c r="BF29" s="24" t="inlineStr">
@@ -9820,7 +9852,7 @@
       </c>
       <c r="BH29" s="24" t="inlineStr">
         <is>
-          <t>2026-07-29T05:19:46.912744Z</t>
+          <t>2026-07-29T17:43:02.309112Z</t>
         </is>
       </c>
       <c r="BI29" s="24" t="inlineStr">
@@ -9830,15 +9862,17 @@
       </c>
       <c r="BJ29" s="25" t="n"/>
       <c r="BK29" s="26" t="n">
-        <v>-110</v>
+        <v>150</v>
       </c>
       <c r="BL29" s="27" t="n">
-        <v>1.909091</v>
+        <v>2.5</v>
       </c>
       <c r="BM29" s="28" t="n">
-        <v>0.52381</v>
-      </c>
-      <c r="BN29" s="28" t="n"/>
+        <v>0.4</v>
+      </c>
+      <c r="BN29" s="28" t="n">
+        <v>0.39801</v>
+      </c>
       <c r="BO29" s="28" t="n"/>
       <c r="BP29" s="25" t="n"/>
       <c r="BQ29" s="27" t="n"/>
@@ -9855,31 +9889,27 @@
       <c r="CB29" s="24" t="n"/>
       <c r="CC29" s="24" t="inlineStr">
         <is>
-          <t>0.5812862212</t>
+          <t>0.6881581363</t>
         </is>
       </c>
       <c r="CD29" s="24" t="inlineStr">
         <is>
-          <t>1.271016</t>
+          <t>2.156212</t>
         </is>
       </c>
       <c r="CE29" s="24" t="inlineStr">
         <is>
-          <t>0.96</t>
+          <t>0.945</t>
         </is>
       </c>
       <c r="CF29" s="24" t="n"/>
       <c r="CG29" s="24" t="n"/>
       <c r="CH29" s="24" t="inlineStr">
         <is>
-          <t>-0.87</t>
-        </is>
-      </c>
-      <c r="CI29" s="24" t="inlineStr">
-        <is>
-          <t>executable_quote_missing_or_unmatched</t>
-        </is>
-      </c>
+          <t>2.42</t>
+        </is>
+      </c>
+      <c r="CI29" s="24" t="n"/>
       <c r="CJ29" s="24" t="n"/>
       <c r="CK29" s="24" t="n"/>
       <c r="CL29" s="24" t="n"/>
@@ -9890,12 +9920,12 @@
     <row r="30" ht="36" customHeight="1">
       <c r="A30" s="24" t="inlineStr">
         <is>
-          <t>9cf1b29591de4274</t>
+          <t>d6e9854bef234238</t>
         </is>
       </c>
       <c r="B30" s="24" t="inlineStr">
         <is>
-          <t>2026-07-29T05:19:46.912744Z</t>
+          <t>2026-07-29T17:43:50.913671Z</t>
         </is>
       </c>
       <c r="C30" s="24" t="inlineStr">
@@ -9936,30 +9966,30 @@
       <c r="J30" s="25" t="n"/>
       <c r="K30" s="24" t="inlineStr">
         <is>
-          <t>model_opinion_no_executable_quote</t>
+          <t>polymarket_us</t>
         </is>
       </c>
       <c r="L30" s="26" t="n">
-        <v>-110</v>
+        <v>178</v>
       </c>
       <c r="M30" s="27" t="n">
-        <v>1.909091</v>
+        <v>2.78</v>
       </c>
       <c r="N30" s="28" t="n">
-        <v>0.52381</v>
+        <v>0.359712</v>
       </c>
       <c r="O30" s="28" t="n">
-        <v>0.6076009999999999</v>
+        <v>0.60967</v>
       </c>
       <c r="P30" s="28" t="n"/>
       <c r="Q30" s="28" t="n">
-        <v>0.083791</v>
+        <v>0.249958</v>
       </c>
       <c r="R30" s="26" t="n">
-        <v>62</v>
+        <v>100</v>
       </c>
       <c r="S30" s="29" t="n">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="T30" s="24" t="inlineStr">
         <is>
@@ -9982,7 +10012,7 @@
       <c r="AD30" s="24" t="n"/>
       <c r="AE30" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.5690; no Polymarket quote available — using -110 default odds. WARNING: executable_quote_missing_or_unmatched; model opinion remains visible, but this row is not executable or price-qualified. NOTE: executable_quote_missing_or_unmatched unavailable for this game — defaulted to neutral, other features used normally.</t>
+          <t>Learned LR call at threshold 0.5690; executable ask 0.3600 (aec-mlb-kc-min-2026-07-29).</t>
         </is>
       </c>
       <c r="AF30" s="31" t="inlineStr">
@@ -10000,7 +10030,7 @@
       <c r="AJ30" s="31" t="n"/>
       <c r="AK30" s="24" t="inlineStr">
         <is>
-          <t>research_observation</t>
+          <t>model_qualified</t>
         </is>
       </c>
       <c r="AL30" s="26" t="n">
@@ -10008,17 +10038,17 @@
       </c>
       <c r="AM30" s="24" t="inlineStr">
         <is>
-          <t>RESEARCH_OBSERVATION</t>
+          <t>QUALIFIED_SHADOW_CALL</t>
         </is>
       </c>
       <c r="AN30" s="24" t="inlineStr">
         <is>
-          <t>NO_CALL</t>
+          <t>CALL</t>
         </is>
       </c>
       <c r="AO30" s="24" t="inlineStr">
         <is>
-          <t>NO_CALL_MARKET_UNAVAILABLE</t>
+          <t>QUALIFIED</t>
         </is>
       </c>
       <c r="AP30" s="24" t="inlineStr">
@@ -10086,7 +10116,7 @@
       </c>
       <c r="BE30" s="24" t="inlineStr">
         <is>
-          <t>fd890ce0158a231f</t>
+          <t>b93a857ee5bf807e</t>
         </is>
       </c>
       <c r="BF30" s="24" t="inlineStr">
@@ -10101,7 +10131,7 @@
       </c>
       <c r="BH30" s="24" t="inlineStr">
         <is>
-          <t>2026-07-29T05:19:46.912744Z</t>
+          <t>2026-07-29T17:43:06.195384Z</t>
         </is>
       </c>
       <c r="BI30" s="24" t="inlineStr">
@@ -10111,15 +10141,17 @@
       </c>
       <c r="BJ30" s="25" t="n"/>
       <c r="BK30" s="26" t="n">
-        <v>-110</v>
+        <v>178</v>
       </c>
       <c r="BL30" s="27" t="n">
-        <v>1.909091</v>
+        <v>2.78</v>
       </c>
       <c r="BM30" s="28" t="n">
-        <v>0.52381</v>
-      </c>
-      <c r="BN30" s="28" t="n"/>
+        <v>0.359712</v>
+      </c>
+      <c r="BN30" s="28" t="n">
+        <v>0.358209</v>
+      </c>
       <c r="BO30" s="28" t="n"/>
       <c r="BP30" s="25" t="n"/>
       <c r="BQ30" s="27" t="n"/>
@@ -10146,7 +10178,7 @@
       </c>
       <c r="CE30" s="24" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>1.037</t>
         </is>
       </c>
       <c r="CF30" s="24" t="n"/>
@@ -10156,11 +10188,7 @@
           <t>1.96</t>
         </is>
       </c>
-      <c r="CI30" s="24" t="inlineStr">
-        <is>
-          <t>executable_quote_missing_or_unmatched</t>
-        </is>
-      </c>
+      <c r="CI30" s="24" t="n"/>
       <c r="CJ30" s="24" t="n"/>
       <c r="CK30" s="24" t="n"/>
       <c r="CL30" s="24" t="n"/>
@@ -10171,22 +10199,22 @@
     <row r="31" ht="36" customHeight="1">
       <c r="A31" s="24" t="inlineStr">
         <is>
-          <t>208e8b124e534e6b</t>
+          <t>94b3ad28ea444fba</t>
         </is>
       </c>
       <c r="B31" s="24" t="inlineStr">
         <is>
-          <t>2026-07-29T05:19:46.912744Z</t>
+          <t>2026-07-29T17:43:50.913671Z</t>
         </is>
       </c>
       <c r="C31" s="24" t="inlineStr">
         <is>
-          <t>2026-07-29T19:40:00-0400</t>
+          <t>2026-07-29T21:40:00-0400</t>
         </is>
       </c>
       <c r="D31" s="24" t="inlineStr">
         <is>
-          <t>401816316</t>
+          <t>401816317</t>
         </is>
       </c>
       <c r="E31" s="24" t="inlineStr">
@@ -10196,12 +10224,12 @@
       </c>
       <c r="F31" s="24" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>Boston Red Sox</t>
         </is>
       </c>
       <c r="G31" s="24" t="inlineStr">
         <is>
-          <t>Chicago White Sox</t>
+          <t>Athletics</t>
         </is>
       </c>
       <c r="H31" s="24" t="inlineStr">
@@ -10217,30 +10245,30 @@
       <c r="J31" s="25" t="n"/>
       <c r="K31" s="24" t="inlineStr">
         <is>
-          <t>model_opinion_no_executable_quote</t>
+          <t>polymarket_us</t>
         </is>
       </c>
       <c r="L31" s="26" t="n">
-        <v>-110</v>
+        <v>-141</v>
       </c>
       <c r="M31" s="27" t="n">
-        <v>1.909091</v>
+        <v>1.70922</v>
       </c>
       <c r="N31" s="28" t="n">
-        <v>0.52381</v>
+        <v>0.585062</v>
       </c>
       <c r="O31" s="28" t="n">
-        <v>0.595337</v>
+        <v>0.674823</v>
       </c>
       <c r="P31" s="28" t="n"/>
       <c r="Q31" s="28" t="n">
-        <v>0.07152699999999999</v>
+        <v>0.08976099999999999</v>
       </c>
       <c r="R31" s="26" t="n">
-        <v>56</v>
+        <v>66</v>
       </c>
       <c r="S31" s="29" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="T31" s="24" t="inlineStr">
         <is>
@@ -10263,7 +10291,7 @@
       <c r="AD31" s="24" t="n"/>
       <c r="AE31" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.5690; no Polymarket quote available — using -110 default odds. WARNING: executable_quote_missing_or_unmatched; model opinion remains visible, but this row is not executable or price-qualified. NOTE: executable_quote_missing_or_unmatched unavailable for this game — defaulted to neutral, other features used normally.</t>
+          <t>Learned LR call at threshold 0.5690; executable ask 0.5850 (aec-mlb-bos-ath-2026-07-29).</t>
         </is>
       </c>
       <c r="AF31" s="31" t="inlineStr">
@@ -10281,7 +10309,7 @@
       <c r="AJ31" s="31" t="n"/>
       <c r="AK31" s="24" t="inlineStr">
         <is>
-          <t>research_observation</t>
+          <t>model_qualified</t>
         </is>
       </c>
       <c r="AL31" s="26" t="n">
@@ -10289,47 +10317,47 @@
       </c>
       <c r="AM31" s="24" t="inlineStr">
         <is>
-          <t>RESEARCH_OBSERVATION</t>
+          <t>QUALIFIED_SHADOW_CALL</t>
         </is>
       </c>
       <c r="AN31" s="24" t="inlineStr">
         <is>
-          <t>NO_CALL</t>
+          <t>CALL</t>
         </is>
       </c>
       <c r="AO31" s="24" t="inlineStr">
         <is>
-          <t>NO_CALL_MARKET_UNAVAILABLE</t>
+          <t>QUALIFIED</t>
         </is>
       </c>
       <c r="AP31" s="24" t="inlineStr">
         <is>
-          <t>mlb-nyy</t>
+          <t>mlb-bos</t>
         </is>
       </c>
       <c r="AQ31" s="24" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>Boston Red Sox</t>
         </is>
       </c>
       <c r="AR31" s="24" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>Boston Red Sox</t>
         </is>
       </c>
       <c r="AS31" s="24" t="inlineStr">
         <is>
-          <t>mlb-cws</t>
+          <t>mlb-ath</t>
         </is>
       </c>
       <c r="AT31" s="24" t="inlineStr">
         <is>
-          <t>Chicago White Sox</t>
+          <t>Athletics</t>
         </is>
       </c>
       <c r="AU31" s="24" t="inlineStr">
         <is>
-          <t>Chicago White Sox</t>
+          <t>Athletics</t>
         </is>
       </c>
       <c r="AV31" s="24" t="n"/>
@@ -10367,7 +10395,7 @@
       </c>
       <c r="BE31" s="24" t="inlineStr">
         <is>
-          <t>9fd872ad0f3e63a3</t>
+          <t>93cfc12c40e6d755</t>
         </is>
       </c>
       <c r="BF31" s="24" t="inlineStr">
@@ -10382,7 +10410,7 @@
       </c>
       <c r="BH31" s="24" t="inlineStr">
         <is>
-          <t>2026-07-29T05:19:46.912744Z</t>
+          <t>2026-07-29T17:43:10.028043Z</t>
         </is>
       </c>
       <c r="BI31" s="24" t="inlineStr">
@@ -10392,15 +10420,17 @@
       </c>
       <c r="BJ31" s="25" t="n"/>
       <c r="BK31" s="26" t="n">
-        <v>-110</v>
+        <v>-141</v>
       </c>
       <c r="BL31" s="27" t="n">
-        <v>1.909091</v>
+        <v>1.70922</v>
       </c>
       <c r="BM31" s="28" t="n">
-        <v>0.52381</v>
-      </c>
-      <c r="BN31" s="28" t="n"/>
+        <v>0.585062</v>
+      </c>
+      <c r="BN31" s="28" t="n">
+        <v>0.58209</v>
+      </c>
       <c r="BO31" s="28" t="n"/>
       <c r="BP31" s="25" t="n"/>
       <c r="BQ31" s="27" t="n"/>
@@ -10417,31 +10447,27 @@
       <c r="CB31" s="24" t="n"/>
       <c r="CC31" s="24" t="inlineStr">
         <is>
-          <t>0.4761494151</t>
+          <t>0.3891185316</t>
         </is>
       </c>
       <c r="CD31" s="24" t="inlineStr">
         <is>
-          <t>1.500354</t>
+          <t>-1.066043</t>
         </is>
       </c>
       <c r="CE31" s="24" t="inlineStr">
         <is>
-          <t>0.99</t>
+          <t>1.153</t>
         </is>
       </c>
       <c r="CF31" s="24" t="n"/>
       <c r="CG31" s="24" t="n"/>
       <c r="CH31" s="24" t="inlineStr">
         <is>
-          <t>1.42</t>
-        </is>
-      </c>
-      <c r="CI31" s="24" t="inlineStr">
-        <is>
-          <t>executable_quote_missing_or_unmatched</t>
-        </is>
-      </c>
+          <t>2.91</t>
+        </is>
+      </c>
+      <c r="CI31" s="24" t="n"/>
       <c r="CJ31" s="24" t="n"/>
       <c r="CK31" s="24" t="n"/>
       <c r="CL31" s="24" t="n"/>
@@ -10452,22 +10478,22 @@
     <row r="32" ht="36" customHeight="1">
       <c r="A32" s="24" t="inlineStr">
         <is>
-          <t>d536ae89b2e54ac1</t>
+          <t>5c59fb610fc44d22</t>
         </is>
       </c>
       <c r="B32" s="24" t="inlineStr">
         <is>
-          <t>2026-07-29T05:19:46.912744Z</t>
+          <t>2026-07-29T17:43:50.913671Z</t>
         </is>
       </c>
       <c r="C32" s="24" t="inlineStr">
         <is>
-          <t>2026-07-29T21:40:00-0400</t>
+          <t>2026-07-29T22:10:00-0400</t>
         </is>
       </c>
       <c r="D32" s="24" t="inlineStr">
         <is>
-          <t>401816317</t>
+          <t>401816321</t>
         </is>
       </c>
       <c r="E32" s="24" t="inlineStr">
@@ -10477,12 +10503,12 @@
       </c>
       <c r="F32" s="24" t="inlineStr">
         <is>
-          <t>Boston Red Sox</t>
+          <t>Seattle Mariners</t>
         </is>
       </c>
       <c r="G32" s="24" t="inlineStr">
         <is>
-          <t>Athletics</t>
+          <t>Los Angeles Dodgers</t>
         </is>
       </c>
       <c r="H32" s="24" t="inlineStr">
@@ -10498,30 +10524,30 @@
       <c r="J32" s="25" t="n"/>
       <c r="K32" s="24" t="inlineStr">
         <is>
-          <t>model_opinion_no_executable_quote</t>
+          <t>polymarket_us</t>
         </is>
       </c>
       <c r="L32" s="26" t="n">
-        <v>-110</v>
+        <v>153</v>
       </c>
       <c r="M32" s="27" t="n">
-        <v>1.909091</v>
+        <v>2.53</v>
       </c>
       <c r="N32" s="28" t="n">
-        <v>0.52381</v>
+        <v>0.395257</v>
       </c>
       <c r="O32" s="28" t="n">
-        <v>0.6658500000000001</v>
+        <v>0.580323</v>
       </c>
       <c r="P32" s="28" t="n"/>
       <c r="Q32" s="28" t="n">
-        <v>0.14204</v>
+        <v>0.185066</v>
       </c>
       <c r="R32" s="26" t="n">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="S32" s="29" t="n">
-        <v>0</v>
+        <v>1.25</v>
       </c>
       <c r="T32" s="24" t="inlineStr">
         <is>
@@ -10544,7 +10570,7 @@
       <c r="AD32" s="24" t="n"/>
       <c r="AE32" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.5690; no Polymarket quote available — using -110 default odds. WARNING: executable_quote_missing_or_unmatched; model opinion remains visible, but this row is not executable or price-qualified. NOTE: executable_quote_missing_or_unmatched unavailable for this game — defaulted to neutral, other features used normally.</t>
+          <t>Learned LR call at threshold 0.5690; executable ask 0.3950 (aec-mlb-sea-lad-2026-07-29).</t>
         </is>
       </c>
       <c r="AF32" s="31" t="inlineStr">
@@ -10562,7 +10588,7 @@
       <c r="AJ32" s="31" t="n"/>
       <c r="AK32" s="24" t="inlineStr">
         <is>
-          <t>research_observation</t>
+          <t>model_qualified</t>
         </is>
       </c>
       <c r="AL32" s="26" t="n">
@@ -10570,47 +10596,47 @@
       </c>
       <c r="AM32" s="24" t="inlineStr">
         <is>
-          <t>RESEARCH_OBSERVATION</t>
+          <t>QUALIFIED_SHADOW_CALL</t>
         </is>
       </c>
       <c r="AN32" s="24" t="inlineStr">
         <is>
-          <t>NO_CALL</t>
+          <t>CALL</t>
         </is>
       </c>
       <c r="AO32" s="24" t="inlineStr">
         <is>
-          <t>NO_CALL_MARKET_UNAVAILABLE</t>
+          <t>QUALIFIED</t>
         </is>
       </c>
       <c r="AP32" s="24" t="inlineStr">
         <is>
-          <t>mlb-bos</t>
+          <t>mlb-sea</t>
         </is>
       </c>
       <c r="AQ32" s="24" t="inlineStr">
         <is>
-          <t>Boston Red Sox</t>
+          <t>Seattle Mariners</t>
         </is>
       </c>
       <c r="AR32" s="24" t="inlineStr">
         <is>
-          <t>Boston Red Sox</t>
+          <t>Seattle Mariners</t>
         </is>
       </c>
       <c r="AS32" s="24" t="inlineStr">
         <is>
-          <t>mlb-ath</t>
+          <t>mlb-lad</t>
         </is>
       </c>
       <c r="AT32" s="24" t="inlineStr">
         <is>
-          <t>Athletics</t>
+          <t>Los Angeles Dodgers</t>
         </is>
       </c>
       <c r="AU32" s="24" t="inlineStr">
         <is>
-          <t>Athletics</t>
+          <t>Los Angeles Dodgers</t>
         </is>
       </c>
       <c r="AV32" s="24" t="n"/>
@@ -10648,7 +10674,7 @@
       </c>
       <c r="BE32" s="24" t="inlineStr">
         <is>
-          <t>e8772ec77b881e9a</t>
+          <t>cef2fcdedc4d9995</t>
         </is>
       </c>
       <c r="BF32" s="24" t="inlineStr">
@@ -10663,7 +10689,7 @@
       </c>
       <c r="BH32" s="24" t="inlineStr">
         <is>
-          <t>2026-07-29T05:19:46.912744Z</t>
+          <t>2026-07-29T17:43:11.216934Z</t>
         </is>
       </c>
       <c r="BI32" s="24" t="inlineStr">
@@ -10673,15 +10699,17 @@
       </c>
       <c r="BJ32" s="25" t="n"/>
       <c r="BK32" s="26" t="n">
-        <v>-110</v>
+        <v>153</v>
       </c>
       <c r="BL32" s="27" t="n">
-        <v>1.909091</v>
+        <v>2.53</v>
       </c>
       <c r="BM32" s="28" t="n">
-        <v>0.52381</v>
-      </c>
-      <c r="BN32" s="28" t="n"/>
+        <v>0.395257</v>
+      </c>
+      <c r="BN32" s="28" t="n">
+        <v>0.393035</v>
+      </c>
       <c r="BO32" s="28" t="n"/>
       <c r="BP32" s="25" t="n"/>
       <c r="BQ32" s="27" t="n"/>
@@ -10698,864 +10726,33 @@
       <c r="CB32" s="24" t="n"/>
       <c r="CC32" s="24" t="inlineStr">
         <is>
-          <t>0.3891185316</t>
+          <t>0.6258863376</t>
         </is>
       </c>
       <c r="CD32" s="24" t="inlineStr">
         <is>
-          <t>-1.066043</t>
+          <t>-0.186858</t>
         </is>
       </c>
       <c r="CE32" s="24" t="inlineStr">
         <is>
-          <t>0.98</t>
+          <t>1.026</t>
         </is>
       </c>
       <c r="CF32" s="24" t="n"/>
       <c r="CG32" s="24" t="n"/>
       <c r="CH32" s="24" t="inlineStr">
         <is>
-          <t>2.91</t>
-        </is>
-      </c>
-      <c r="CI32" s="24" t="inlineStr">
-        <is>
-          <t>executable_quote_missing_or_unmatched</t>
-        </is>
-      </c>
+          <t>1.67</t>
+        </is>
+      </c>
+      <c r="CI32" s="24" t="n"/>
       <c r="CJ32" s="24" t="n"/>
       <c r="CK32" s="24" t="n"/>
       <c r="CL32" s="24" t="n"/>
       <c r="CM32" s="24" t="n"/>
       <c r="CN32" s="24" t="n"/>
       <c r="CO32" s="24" t="n"/>
-    </row>
-    <row r="33" ht="36" customHeight="1">
-      <c r="A33" s="24" t="inlineStr">
-        <is>
-          <t>0b44eef52d4c4880</t>
-        </is>
-      </c>
-      <c r="B33" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-29T05:19:46.912744Z</t>
-        </is>
-      </c>
-      <c r="C33" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-29T22:10:00-0400</t>
-        </is>
-      </c>
-      <c r="D33" s="24" t="inlineStr">
-        <is>
-          <t>401816321</t>
-        </is>
-      </c>
-      <c r="E33" s="24" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="F33" s="24" t="inlineStr">
-        <is>
-          <t>Seattle Mariners</t>
-        </is>
-      </c>
-      <c r="G33" s="24" t="inlineStr">
-        <is>
-          <t>Los Angeles Dodgers</t>
-        </is>
-      </c>
-      <c r="H33" s="24" t="inlineStr">
-        <is>
-          <t>moneyline</t>
-        </is>
-      </c>
-      <c r="I33" s="24" t="inlineStr">
-        <is>
-          <t>away</t>
-        </is>
-      </c>
-      <c r="J33" s="25" t="n"/>
-      <c r="K33" s="24" t="inlineStr">
-        <is>
-          <t>model_opinion_no_executable_quote</t>
-        </is>
-      </c>
-      <c r="L33" s="26" t="n">
-        <v>-110</v>
-      </c>
-      <c r="M33" s="27" t="n">
-        <v>1.909091</v>
-      </c>
-      <c r="N33" s="28" t="n">
-        <v>0.52381</v>
-      </c>
-      <c r="O33" s="28" t="n">
-        <v>0.578264</v>
-      </c>
-      <c r="P33" s="28" t="n"/>
-      <c r="Q33" s="28" t="n">
-        <v>0.054454</v>
-      </c>
-      <c r="R33" s="26" t="n">
-        <v>47</v>
-      </c>
-      <c r="S33" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="T33" s="24" t="inlineStr">
-        <is>
-          <t>mlb-elo-trend-lr-v6</t>
-        </is>
-      </c>
-      <c r="U33" s="24" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V33" s="24" t="n"/>
-      <c r="W33" s="26" t="n"/>
-      <c r="X33" s="26" t="n"/>
-      <c r="Y33" s="25" t="n"/>
-      <c r="Z33" s="26" t="n"/>
-      <c r="AA33" s="28" t="n"/>
-      <c r="AB33" s="28" t="n"/>
-      <c r="AC33" s="30" t="n"/>
-      <c r="AD33" s="24" t="n"/>
-      <c r="AE33" s="31" t="inlineStr">
-        <is>
-          <t>Learned LR call at threshold 0.5690; no Polymarket quote available — using -110 default odds. WARNING: executable_quote_missing_or_unmatched; model opinion remains visible, but this row is not executable or price-qualified. NOTE: executable_quote_missing_or_unmatched unavailable for this game — defaulted to neutral, other features used normally.</t>
-        </is>
-      </c>
-      <c r="AF33" s="31" t="inlineStr">
-        <is>
-          <t>Learned model; shadow-qualified via operator override.</t>
-        </is>
-      </c>
-      <c r="AG33" s="24" t="inlineStr">
-        <is>
-          <t>not_applicable</t>
-        </is>
-      </c>
-      <c r="AH33" s="24" t="n"/>
-      <c r="AI33" s="31" t="n"/>
-      <c r="AJ33" s="31" t="n"/>
-      <c r="AK33" s="24" t="inlineStr">
-        <is>
-          <t>research_observation</t>
-        </is>
-      </c>
-      <c r="AL33" s="26" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM33" s="24" t="inlineStr">
-        <is>
-          <t>RESEARCH_OBSERVATION</t>
-        </is>
-      </c>
-      <c r="AN33" s="24" t="inlineStr">
-        <is>
-          <t>NO_CALL</t>
-        </is>
-      </c>
-      <c r="AO33" s="24" t="inlineStr">
-        <is>
-          <t>NO_CALL_MARKET_UNAVAILABLE</t>
-        </is>
-      </c>
-      <c r="AP33" s="24" t="inlineStr">
-        <is>
-          <t>mlb-sea</t>
-        </is>
-      </c>
-      <c r="AQ33" s="24" t="inlineStr">
-        <is>
-          <t>Seattle Mariners</t>
-        </is>
-      </c>
-      <c r="AR33" s="24" t="inlineStr">
-        <is>
-          <t>Seattle Mariners</t>
-        </is>
-      </c>
-      <c r="AS33" s="24" t="inlineStr">
-        <is>
-          <t>mlb-lad</t>
-        </is>
-      </c>
-      <c r="AT33" s="24" t="inlineStr">
-        <is>
-          <t>Los Angeles Dodgers</t>
-        </is>
-      </c>
-      <c r="AU33" s="24" t="inlineStr">
-        <is>
-          <t>Los Angeles Dodgers</t>
-        </is>
-      </c>
-      <c r="AV33" s="24" t="n"/>
-      <c r="AW33" s="24" t="n"/>
-      <c r="AX33" s="24" t="inlineStr">
-        <is>
-          <t>statistical_model</t>
-        </is>
-      </c>
-      <c r="AY33" s="24" t="n"/>
-      <c r="AZ33" s="24" t="inlineStr">
-        <is>
-          <t>shadow_qualified</t>
-        </is>
-      </c>
-      <c r="BA33" s="24" t="inlineStr">
-        <is>
-          <t>0633355b1144e4205ca6d08e3f328d99cab0970358846bd77228f3bcbfcd70ee</t>
-        </is>
-      </c>
-      <c r="BB33" s="24" t="inlineStr">
-        <is>
-          <t>learned_lr</t>
-        </is>
-      </c>
-      <c r="BC33" s="24" t="inlineStr">
-        <is>
-          <t>mlb-elo-trend-lr-v6</t>
-        </is>
-      </c>
-      <c r="BD33" s="24" t="inlineStr">
-        <is>
-          <t>0633355b1144e4205ca6d08e3f328d99cab0970358846bd77228f3bcbfcd70ee</t>
-        </is>
-      </c>
-      <c r="BE33" s="24" t="inlineStr">
-        <is>
-          <t>48afb82b2455fcbf</t>
-        </is>
-      </c>
-      <c r="BF33" s="24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BG33" s="24" t="inlineStr">
-        <is>
-          <t>mlb-elo-trend-lr-v6</t>
-        </is>
-      </c>
-      <c r="BH33" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-29T05:19:46.912744Z</t>
-        </is>
-      </c>
-      <c r="BI33" s="24" t="inlineStr">
-        <is>
-          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
-        </is>
-      </c>
-      <c r="BJ33" s="25" t="n"/>
-      <c r="BK33" s="26" t="n">
-        <v>-110</v>
-      </c>
-      <c r="BL33" s="27" t="n">
-        <v>1.909091</v>
-      </c>
-      <c r="BM33" s="28" t="n">
-        <v>0.52381</v>
-      </c>
-      <c r="BN33" s="28" t="n"/>
-      <c r="BO33" s="28" t="n"/>
-      <c r="BP33" s="25" t="n"/>
-      <c r="BQ33" s="27" t="n"/>
-      <c r="BR33" s="28" t="n"/>
-      <c r="BS33" s="28" t="n"/>
-      <c r="BT33" s="28" t="n"/>
-      <c r="BU33" s="25" t="n"/>
-      <c r="BV33" s="29" t="n"/>
-      <c r="BW33" s="24" t="n"/>
-      <c r="BX33" s="30" t="n"/>
-      <c r="BY33" s="27" t="n"/>
-      <c r="BZ33" s="24" t="n"/>
-      <c r="CA33" s="31" t="n"/>
-      <c r="CB33" s="24" t="n"/>
-      <c r="CC33" s="24" t="inlineStr">
-        <is>
-          <t>0.6258863376</t>
-        </is>
-      </c>
-      <c r="CD33" s="24" t="inlineStr">
-        <is>
-          <t>-0.186858</t>
-        </is>
-      </c>
-      <c r="CE33" s="24" t="inlineStr">
-        <is>
-          <t>0.99</t>
-        </is>
-      </c>
-      <c r="CF33" s="24" t="n"/>
-      <c r="CG33" s="24" t="n"/>
-      <c r="CH33" s="24" t="inlineStr">
-        <is>
-          <t>1.67</t>
-        </is>
-      </c>
-      <c r="CI33" s="24" t="inlineStr">
-        <is>
-          <t>executable_quote_missing_or_unmatched</t>
-        </is>
-      </c>
-      <c r="CJ33" s="24" t="n"/>
-      <c r="CK33" s="24" t="n"/>
-      <c r="CL33" s="24" t="n"/>
-      <c r="CM33" s="24" t="n"/>
-      <c r="CN33" s="24" t="n"/>
-      <c r="CO33" s="24" t="n"/>
-    </row>
-    <row r="34" ht="36" customHeight="1">
-      <c r="A34" s="24" t="inlineStr">
-        <is>
-          <t>383f41591c534ef5</t>
-        </is>
-      </c>
-      <c r="B34" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-29T05:19:53.585877Z</t>
-        </is>
-      </c>
-      <c r="C34" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-29T20:00:00-0400</t>
-        </is>
-      </c>
-      <c r="D34" s="24" t="inlineStr">
-        <is>
-          <t>401857097</t>
-        </is>
-      </c>
-      <c r="E34" s="24" t="inlineStr">
-        <is>
-          <t>WNBA</t>
-        </is>
-      </c>
-      <c r="F34" s="24" t="inlineStr">
-        <is>
-          <t>Atlanta Dream</t>
-        </is>
-      </c>
-      <c r="G34" s="24" t="inlineStr">
-        <is>
-          <t>Dallas Wings</t>
-        </is>
-      </c>
-      <c r="H34" s="24" t="inlineStr">
-        <is>
-          <t>moneyline</t>
-        </is>
-      </c>
-      <c r="I34" s="24" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="J34" s="25" t="n"/>
-      <c r="K34" s="24" t="inlineStr">
-        <is>
-          <t>model_opinion_no_executable_quote</t>
-        </is>
-      </c>
-      <c r="L34" s="26" t="n">
-        <v>-110</v>
-      </c>
-      <c r="M34" s="27" t="n">
-        <v>1.909091</v>
-      </c>
-      <c r="N34" s="28" t="n">
-        <v>0.52381</v>
-      </c>
-      <c r="O34" s="28" t="n">
-        <v>0.66476</v>
-      </c>
-      <c r="P34" s="28" t="n"/>
-      <c r="Q34" s="28" t="n">
-        <v>0.14095</v>
-      </c>
-      <c r="R34" s="26" t="n">
-        <v>90</v>
-      </c>
-      <c r="S34" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="T34" s="24" t="inlineStr">
-        <is>
-          <t>wnba-elo-trend-lr-v4</t>
-        </is>
-      </c>
-      <c r="U34" s="24" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V34" s="24" t="n"/>
-      <c r="W34" s="26" t="n"/>
-      <c r="X34" s="26" t="n"/>
-      <c r="Y34" s="25" t="n"/>
-      <c r="Z34" s="26" t="n"/>
-      <c r="AA34" s="28" t="n"/>
-      <c r="AB34" s="28" t="n"/>
-      <c r="AC34" s="30" t="n"/>
-      <c r="AD34" s="24" t="n"/>
-      <c r="AE34" s="31" t="inlineStr">
-        <is>
-          <t>Learned LR call at threshold 0.5001; no Polymarket quote available — using -110 default odds. WARNING: executable_quote_missing_or_unmatched; model opinion remains visible, but this row is not executable or price-qualified. NOTE: NO_CALL_AVAILABILITY_UNAVAILABLE, executable_quote_missing_or_unmatched unavailable for this game — defaulted to neutral, other features used normally.</t>
-        </is>
-      </c>
-      <c r="AF34" s="31" t="inlineStr">
-        <is>
-          <t>Learned model; shadow-qualified via operator override.</t>
-        </is>
-      </c>
-      <c r="AG34" s="24" t="inlineStr">
-        <is>
-          <t>not_applicable</t>
-        </is>
-      </c>
-      <c r="AH34" s="24" t="n"/>
-      <c r="AI34" s="31" t="n"/>
-      <c r="AJ34" s="31" t="n"/>
-      <c r="AK34" s="24" t="inlineStr">
-        <is>
-          <t>research_observation</t>
-        </is>
-      </c>
-      <c r="AL34" s="26" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM34" s="24" t="inlineStr">
-        <is>
-          <t>RESEARCH_OBSERVATION</t>
-        </is>
-      </c>
-      <c r="AN34" s="24" t="inlineStr">
-        <is>
-          <t>NO_CALL</t>
-        </is>
-      </c>
-      <c r="AO34" s="24" t="inlineStr">
-        <is>
-          <t>NO_CALL_MARKET_UNAVAILABLE</t>
-        </is>
-      </c>
-      <c r="AP34" s="24" t="inlineStr">
-        <is>
-          <t>wnba-atl</t>
-        </is>
-      </c>
-      <c r="AQ34" s="24" t="inlineStr">
-        <is>
-          <t>Atlanta Dream</t>
-        </is>
-      </c>
-      <c r="AR34" s="24" t="inlineStr">
-        <is>
-          <t>Atlanta Dream</t>
-        </is>
-      </c>
-      <c r="AS34" s="24" t="inlineStr">
-        <is>
-          <t>wnba-dal</t>
-        </is>
-      </c>
-      <c r="AT34" s="24" t="inlineStr">
-        <is>
-          <t>Dallas Wings</t>
-        </is>
-      </c>
-      <c r="AU34" s="24" t="inlineStr">
-        <is>
-          <t>Dallas Wings</t>
-        </is>
-      </c>
-      <c r="AV34" s="24" t="n"/>
-      <c r="AW34" s="24" t="n"/>
-      <c r="AX34" s="24" t="inlineStr">
-        <is>
-          <t>statistical_model</t>
-        </is>
-      </c>
-      <c r="AY34" s="24" t="n"/>
-      <c r="AZ34" s="24" t="inlineStr">
-        <is>
-          <t>shadow_qualified</t>
-        </is>
-      </c>
-      <c r="BA34" s="24" t="inlineStr">
-        <is>
-          <t>7afd5274214b58b7efd7f7febc7be3ab33b92351cda5cc6403c0a39faea0cc8c</t>
-        </is>
-      </c>
-      <c r="BB34" s="24" t="inlineStr">
-        <is>
-          <t>learned_lr</t>
-        </is>
-      </c>
-      <c r="BC34" s="24" t="inlineStr">
-        <is>
-          <t>wnba-elo-trend-lr-v4</t>
-        </is>
-      </c>
-      <c r="BD34" s="24" t="inlineStr">
-        <is>
-          <t>7afd5274214b58b7efd7f7febc7be3ab33b92351cda5cc6403c0a39faea0cc8c</t>
-        </is>
-      </c>
-      <c r="BE34" s="24" t="inlineStr">
-        <is>
-          <t>f25936b561e6d355</t>
-        </is>
-      </c>
-      <c r="BF34" s="24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BG34" s="24" t="inlineStr">
-        <is>
-          <t>wnba-elo-trend-lr-v4</t>
-        </is>
-      </c>
-      <c r="BH34" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-29T05:19:53.585877Z</t>
-        </is>
-      </c>
-      <c r="BI34" s="24" t="inlineStr">
-        <is>
-          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
-        </is>
-      </c>
-      <c r="BJ34" s="25" t="n"/>
-      <c r="BK34" s="26" t="n">
-        <v>-110</v>
-      </c>
-      <c r="BL34" s="27" t="n">
-        <v>1.909091</v>
-      </c>
-      <c r="BM34" s="28" t="n">
-        <v>0.52381</v>
-      </c>
-      <c r="BN34" s="28" t="n"/>
-      <c r="BO34" s="28" t="n"/>
-      <c r="BP34" s="25" t="n"/>
-      <c r="BQ34" s="27" t="n"/>
-      <c r="BR34" s="28" t="n"/>
-      <c r="BS34" s="28" t="n"/>
-      <c r="BT34" s="28" t="n"/>
-      <c r="BU34" s="25" t="n"/>
-      <c r="BV34" s="29" t="n"/>
-      <c r="BW34" s="24" t="n"/>
-      <c r="BX34" s="30" t="n"/>
-      <c r="BY34" s="27" t="n"/>
-      <c r="BZ34" s="24" t="n"/>
-      <c r="CA34" s="31" t="n"/>
-      <c r="CB34" s="24" t="n"/>
-      <c r="CC34" s="24" t="inlineStr">
-        <is>
-          <t>0.7229749194</t>
-        </is>
-      </c>
-      <c r="CD34" s="24" t="inlineStr">
-        <is>
-          <t>-2.425932</t>
-        </is>
-      </c>
-      <c r="CE34" s="24" t="n"/>
-      <c r="CF34" s="24" t="n"/>
-      <c r="CG34" s="24" t="n"/>
-      <c r="CH34" s="24" t="n"/>
-      <c r="CI34" s="24" t="inlineStr">
-        <is>
-          <t>NO_CALL_AVAILABILITY_UNAVAILABLE,executable_quote_missing_or_unmatched</t>
-        </is>
-      </c>
-      <c r="CJ34" s="24" t="n"/>
-      <c r="CK34" s="24" t="n"/>
-      <c r="CL34" s="24" t="n"/>
-      <c r="CM34" s="24" t="n"/>
-      <c r="CN34" s="24" t="n"/>
-      <c r="CO34" s="24" t="n"/>
-    </row>
-    <row r="35" ht="36" customHeight="1">
-      <c r="A35" s="24" t="inlineStr">
-        <is>
-          <t>df3672f8d9724eb8</t>
-        </is>
-      </c>
-      <c r="B35" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-29T05:19:53.585877Z</t>
-        </is>
-      </c>
-      <c r="C35" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-29T22:00:00-0400</t>
-        </is>
-      </c>
-      <c r="D35" s="24" t="inlineStr">
-        <is>
-          <t>401857098</t>
-        </is>
-      </c>
-      <c r="E35" s="24" t="inlineStr">
-        <is>
-          <t>WNBA</t>
-        </is>
-      </c>
-      <c r="F35" s="24" t="inlineStr">
-        <is>
-          <t>Golden State Valkyries</t>
-        </is>
-      </c>
-      <c r="G35" s="24" t="inlineStr">
-        <is>
-          <t>Phoenix Mercury</t>
-        </is>
-      </c>
-      <c r="H35" s="24" t="inlineStr">
-        <is>
-          <t>moneyline</t>
-        </is>
-      </c>
-      <c r="I35" s="24" t="inlineStr">
-        <is>
-          <t>away</t>
-        </is>
-      </c>
-      <c r="J35" s="25" t="n"/>
-      <c r="K35" s="24" t="inlineStr">
-        <is>
-          <t>model_opinion_no_executable_quote</t>
-        </is>
-      </c>
-      <c r="L35" s="26" t="n">
-        <v>-110</v>
-      </c>
-      <c r="M35" s="27" t="n">
-        <v>1.909091</v>
-      </c>
-      <c r="N35" s="28" t="n">
-        <v>0.52381</v>
-      </c>
-      <c r="O35" s="28" t="n">
-        <v>0.7219989999999999</v>
-      </c>
-      <c r="P35" s="28" t="n"/>
-      <c r="Q35" s="28" t="n">
-        <v>0.198189</v>
-      </c>
-      <c r="R35" s="26" t="n">
-        <v>100</v>
-      </c>
-      <c r="S35" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="T35" s="24" t="inlineStr">
-        <is>
-          <t>wnba-elo-trend-lr-v4</t>
-        </is>
-      </c>
-      <c r="U35" s="24" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V35" s="24" t="n"/>
-      <c r="W35" s="26" t="n"/>
-      <c r="X35" s="26" t="n"/>
-      <c r="Y35" s="25" t="n"/>
-      <c r="Z35" s="26" t="n"/>
-      <c r="AA35" s="28" t="n"/>
-      <c r="AB35" s="28" t="n"/>
-      <c r="AC35" s="30" t="n"/>
-      <c r="AD35" s="24" t="n"/>
-      <c r="AE35" s="31" t="inlineStr">
-        <is>
-          <t>Learned LR call at threshold 0.5001; no Polymarket quote available — using -110 default odds. WARNING: executable_quote_missing_or_unmatched; model opinion remains visible, but this row is not executable or price-qualified. NOTE: NO_CALL_AVAILABILITY_UNAVAILABLE, executable_quote_missing_or_unmatched unavailable for this game — defaulted to neutral, other features used normally.</t>
-        </is>
-      </c>
-      <c r="AF35" s="31" t="inlineStr">
-        <is>
-          <t>Learned model; shadow-qualified via operator override.</t>
-        </is>
-      </c>
-      <c r="AG35" s="24" t="inlineStr">
-        <is>
-          <t>not_applicable</t>
-        </is>
-      </c>
-      <c r="AH35" s="24" t="n"/>
-      <c r="AI35" s="31" t="n"/>
-      <c r="AJ35" s="31" t="n"/>
-      <c r="AK35" s="24" t="inlineStr">
-        <is>
-          <t>research_observation</t>
-        </is>
-      </c>
-      <c r="AL35" s="26" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM35" s="24" t="inlineStr">
-        <is>
-          <t>RESEARCH_OBSERVATION</t>
-        </is>
-      </c>
-      <c r="AN35" s="24" t="inlineStr">
-        <is>
-          <t>NO_CALL</t>
-        </is>
-      </c>
-      <c r="AO35" s="24" t="inlineStr">
-        <is>
-          <t>NO_CALL_MARKET_UNAVAILABLE</t>
-        </is>
-      </c>
-      <c r="AP35" s="24" t="inlineStr">
-        <is>
-          <t>wnba-gsv</t>
-        </is>
-      </c>
-      <c r="AQ35" s="24" t="inlineStr">
-        <is>
-          <t>Golden State Valkyries</t>
-        </is>
-      </c>
-      <c r="AR35" s="24" t="inlineStr">
-        <is>
-          <t>Golden State Valkyries</t>
-        </is>
-      </c>
-      <c r="AS35" s="24" t="inlineStr">
-        <is>
-          <t>wnba-phx</t>
-        </is>
-      </c>
-      <c r="AT35" s="24" t="inlineStr">
-        <is>
-          <t>Phoenix Mercury</t>
-        </is>
-      </c>
-      <c r="AU35" s="24" t="inlineStr">
-        <is>
-          <t>Phoenix Mercury</t>
-        </is>
-      </c>
-      <c r="AV35" s="24" t="n"/>
-      <c r="AW35" s="24" t="n"/>
-      <c r="AX35" s="24" t="inlineStr">
-        <is>
-          <t>statistical_model</t>
-        </is>
-      </c>
-      <c r="AY35" s="24" t="n"/>
-      <c r="AZ35" s="24" t="inlineStr">
-        <is>
-          <t>shadow_qualified</t>
-        </is>
-      </c>
-      <c r="BA35" s="24" t="inlineStr">
-        <is>
-          <t>7afd5274214b58b7efd7f7febc7be3ab33b92351cda5cc6403c0a39faea0cc8c</t>
-        </is>
-      </c>
-      <c r="BB35" s="24" t="inlineStr">
-        <is>
-          <t>learned_lr</t>
-        </is>
-      </c>
-      <c r="BC35" s="24" t="inlineStr">
-        <is>
-          <t>wnba-elo-trend-lr-v4</t>
-        </is>
-      </c>
-      <c r="BD35" s="24" t="inlineStr">
-        <is>
-          <t>7afd5274214b58b7efd7f7febc7be3ab33b92351cda5cc6403c0a39faea0cc8c</t>
-        </is>
-      </c>
-      <c r="BE35" s="24" t="inlineStr">
-        <is>
-          <t>5ba5847b783e4237</t>
-        </is>
-      </c>
-      <c r="BF35" s="24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BG35" s="24" t="inlineStr">
-        <is>
-          <t>wnba-elo-trend-lr-v4</t>
-        </is>
-      </c>
-      <c r="BH35" s="24" t="inlineStr">
-        <is>
-          <t>2026-07-29T05:19:53.585877Z</t>
-        </is>
-      </c>
-      <c r="BI35" s="24" t="inlineStr">
-        <is>
-          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
-        </is>
-      </c>
-      <c r="BJ35" s="25" t="n"/>
-      <c r="BK35" s="26" t="n">
-        <v>-110</v>
-      </c>
-      <c r="BL35" s="27" t="n">
-        <v>1.909091</v>
-      </c>
-      <c r="BM35" s="28" t="n">
-        <v>0.52381</v>
-      </c>
-      <c r="BN35" s="28" t="n"/>
-      <c r="BO35" s="28" t="n"/>
-      <c r="BP35" s="25" t="n"/>
-      <c r="BQ35" s="27" t="n"/>
-      <c r="BR35" s="28" t="n"/>
-      <c r="BS35" s="28" t="n"/>
-      <c r="BT35" s="28" t="n"/>
-      <c r="BU35" s="25" t="n"/>
-      <c r="BV35" s="29" t="n"/>
-      <c r="BW35" s="24" t="n"/>
-      <c r="BX35" s="30" t="n"/>
-      <c r="BY35" s="27" t="n"/>
-      <c r="BZ35" s="24" t="n"/>
-      <c r="CA35" s="31" t="n"/>
-      <c r="CB35" s="24" t="n"/>
-      <c r="CC35" s="24" t="inlineStr">
-        <is>
-          <t>0.1902656067</t>
-        </is>
-      </c>
-      <c r="CD35" s="24" t="inlineStr">
-        <is>
-          <t>-0.399848</t>
-        </is>
-      </c>
-      <c r="CE35" s="24" t="n"/>
-      <c r="CF35" s="24" t="n"/>
-      <c r="CG35" s="24" t="n"/>
-      <c r="CH35" s="24" t="n"/>
-      <c r="CI35" s="24" t="inlineStr">
-        <is>
-          <t>NO_CALL_AVAILABILITY_UNAVAILABLE,executable_quote_missing_or_unmatched</t>
-        </is>
-      </c>
-      <c r="CJ35" s="24" t="n"/>
-      <c r="CK35" s="24" t="n"/>
-      <c r="CL35" s="24" t="n"/>
-      <c r="CM35" s="24" t="n"/>
-      <c r="CN35" s="24" t="n"/>
-      <c r="CO35" s="24" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>